<commit_message>
feat: Package Types merged header + dropdown fixes + blue outlines + replay cleanup + activities link
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -96,8 +96,23 @@
       <color rgb="00D4AF37"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A3450"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -152,8 +167,38 @@
         <bgColor rgb="00DCE6F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD4AF37"/>
+        <bgColor rgb="FFD4AF37"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A3450"/>
+        <bgColor rgb="FF1A3450"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDAEEF3"/>
+        <bgColor rgb="FFDAEEF3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -226,11 +271,81 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF333333"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF333333"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF333333"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF333333"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF4472C4"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF4472C4"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF4472C4"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF4472C4"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -411,6 +526,60 @@
     <xf numFmtId="164" fontId="10" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="7" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="7" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="15" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -812,7 +981,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="31" t="inlineStr">
         <is>
@@ -860,15 +1028,15 @@
       <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="40" t="inlineStr">
+      <c r="A7" s="70" t="inlineStr">
         <is>
           <t>Trump National LA</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="71" t="n">
         <v>210</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="71" t="n">
         <v>210</v>
       </c>
       <c r="D7" s="5">
@@ -885,15 +1053,15 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="40" t="inlineStr">
+      <c r="A8" s="70" t="inlineStr">
         <is>
           <t>Sandpiper GC</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="71" t="n">
         <v>130</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="71" t="n">
         <v>130</v>
       </c>
       <c r="D8" s="5">
@@ -910,15 +1078,15 @@
       </c>
     </row>
     <row r="9" ht="30.75" customHeight="1" s="42">
-      <c r="A9" s="40" t="inlineStr">
+      <c r="A9" s="70" t="inlineStr">
         <is>
           <t>Hidden Valley GC</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="71" t="n">
         <v>109</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="71" t="n">
         <v>109</v>
       </c>
       <c r="D9" s="5">
@@ -989,8 +1157,6 @@
       <c r="E14" s="4" t="n"/>
       <c r="F14" s="6" t="n"/>
     </row>
-    <row r="15"/>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="31" t="inlineStr">
         <is>
@@ -1034,15 +1200,15 @@
       <c r="G18" s="2" t="n"/>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="42">
-      <c r="A19" s="40" t="inlineStr">
+      <c r="A19" s="70" t="inlineStr">
         <is>
           <t>Beverly Wilshire (5★) / Same Tier</t>
         </is>
       </c>
-      <c r="B19" s="4" t="n">
+      <c r="B19" s="71" t="n">
         <v>275</v>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="71" t="n">
         <v>375</v>
       </c>
       <c r="D19" s="5">
@@ -1105,7 +1271,6 @@
       </c>
       <c r="F24" s="6" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="31" t="inlineStr">
         <is>
@@ -1149,15 +1314,15 @@
       <c r="G27" s="2" t="n"/>
     </row>
     <row r="28" ht="16.5" customHeight="1" s="42">
-      <c r="A28" s="40" t="inlineStr">
+      <c r="A28" s="70" t="inlineStr">
         <is>
           <t>Driver/Guide + Van (일당)</t>
         </is>
       </c>
-      <c r="B28" s="4" t="n">
+      <c r="B28" s="71" t="n">
         <v>125</v>
       </c>
-      <c r="C28" s="4" t="n">
+      <c r="C28" s="71" t="n">
         <v>175</v>
       </c>
       <c r="D28" s="5">
@@ -1171,15 +1336,15 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="40" t="inlineStr">
+      <c r="A29" s="70" t="inlineStr">
         <is>
           <t>Airport Roundtrip Pickup</t>
         </is>
       </c>
-      <c r="B29" s="4" t="n">
+      <c r="B29" s="71" t="n">
         <v>75</v>
       </c>
-      <c r="C29" s="4" t="n">
+      <c r="C29" s="71" t="n">
         <v>120</v>
       </c>
       <c r="D29" s="5">
@@ -1242,7 +1407,6 @@
       </c>
       <c r="F34" s="6" t="n"/>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="31" t="inlineStr">
         <is>
@@ -1286,15 +1450,15 @@
       <c r="G37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="40" t="inlineStr">
+      <c r="A38" s="70" t="inlineStr">
         <is>
           <t>Breakfast (Hotel)</t>
         </is>
       </c>
-      <c r="B38" s="4" t="n">
+      <c r="B38" s="71" t="n">
         <v>30</v>
       </c>
-      <c r="C38" s="4" t="n">
+      <c r="C38" s="71" t="n">
         <v>45</v>
       </c>
       <c r="D38" s="5">
@@ -1308,15 +1472,15 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="40" t="inlineStr">
+      <c r="A39" s="70" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="B39" s="4" t="n">
+      <c r="B39" s="71" t="n">
         <v>40</v>
       </c>
-      <c r="C39" s="4" t="n">
+      <c r="C39" s="71" t="n">
         <v>60</v>
       </c>
       <c r="D39" s="5">
@@ -1330,15 +1494,15 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="40" t="inlineStr">
+      <c r="A40" s="70" t="inlineStr">
         <is>
           <t>Dinner (Regular)</t>
         </is>
       </c>
-      <c r="B40" s="4" t="n">
+      <c r="B40" s="71" t="n">
         <v>80</v>
       </c>
-      <c r="C40" s="4" t="n">
+      <c r="C40" s="71" t="n">
         <v>120</v>
       </c>
       <c r="D40" s="5">
@@ -1352,15 +1516,15 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="40" t="inlineStr">
+      <c r="A41" s="70" t="inlineStr">
         <is>
           <t>Exclusive Dinner (Michelin/Fine)</t>
         </is>
       </c>
-      <c r="B41" s="4" t="n">
+      <c r="B41" s="71" t="n">
         <v>120</v>
       </c>
-      <c r="C41" s="4" t="n">
+      <c r="C41" s="71" t="n">
         <v>180</v>
       </c>
       <c r="D41" s="5">
@@ -1423,7 +1587,6 @@
       </c>
       <c r="F46" s="6" t="n"/>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="31" t="inlineStr">
         <is>
@@ -1467,15 +1630,15 @@
       <c r="G49" s="2" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="40" t="inlineStr">
+      <c r="A50" s="70" t="inlineStr">
         <is>
           <t>Insurance / Tips / Contingency</t>
         </is>
       </c>
-      <c r="B50" s="4" t="n">
+      <c r="B50" s="71" t="n">
         <v>50</v>
       </c>
-      <c r="C50" s="4" t="n">
+      <c r="C50" s="71" t="n">
         <v>75</v>
       </c>
       <c r="D50" s="5">
@@ -1539,7 +1702,6 @@
       <c r="F55" s="6" t="n"/>
     </row>
     <row r="56"/>
-    <row r="57"/>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
         <is>
@@ -1601,188 +1763,188 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="40" t="inlineStr">
+      <c r="A60" s="70" t="inlineStr">
         <is>
           <t>KE011</t>
         </is>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B60" s="72" t="inlineStr">
         <is>
           <t>Korean Air</t>
         </is>
       </c>
-      <c r="C60" s="6" t="inlineStr">
+      <c r="C60" s="72" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="D60" s="6" t="inlineStr">
+      <c r="D60" s="72" t="inlineStr">
         <is>
           <t>14:30</t>
         </is>
       </c>
-      <c r="E60" s="6" t="inlineStr">
+      <c r="E60" s="72" t="inlineStr">
         <is>
           <t>ICN→LAX</t>
         </is>
       </c>
-      <c r="F60" s="6" t="inlineStr">
+      <c r="F60" s="72" t="inlineStr">
         <is>
           <t>Daily B747-8</t>
         </is>
       </c>
-      <c r="G60" s="47" t="inlineStr">
+      <c r="G60" s="73" t="inlineStr">
         <is>
           <t>First | Prestige | Economy</t>
         </is>
       </c>
-      <c r="H60" s="47" t="inlineStr">
+      <c r="H60" s="73" t="inlineStr">
         <is>
           <t>~11.5</t>
         </is>
       </c>
-      <c r="I60" s="47" t="inlineStr">
+      <c r="I60" s="73" t="inlineStr">
         <is>
           <t>B747-8</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="40" t="inlineStr">
+      <c r="A61" s="70" t="inlineStr">
         <is>
           <t>KE017</t>
         </is>
       </c>
-      <c r="B61" s="6" t="inlineStr">
+      <c r="B61" s="72" t="inlineStr">
         <is>
           <t>Korean Air</t>
         </is>
       </c>
-      <c r="C61" s="6" t="inlineStr">
+      <c r="C61" s="72" t="inlineStr">
         <is>
           <t>14:30</t>
         </is>
       </c>
-      <c r="D61" s="6" t="inlineStr">
+      <c r="D61" s="72" t="inlineStr">
         <is>
           <t>09:20</t>
         </is>
       </c>
-      <c r="E61" s="6" t="inlineStr">
+      <c r="E61" s="72" t="inlineStr">
         <is>
           <t>ICN→LAX</t>
         </is>
       </c>
-      <c r="F61" s="6" t="inlineStr">
+      <c r="F61" s="72" t="inlineStr">
         <is>
           <t>Daily B777</t>
         </is>
       </c>
-      <c r="G61" s="47" t="inlineStr">
+      <c r="G61" s="73" t="inlineStr">
         <is>
           <t>Prestige | Economy</t>
         </is>
       </c>
-      <c r="H61" s="47" t="inlineStr">
+      <c r="H61" s="73" t="inlineStr">
         <is>
           <t>~11.5</t>
         </is>
       </c>
-      <c r="I61" s="47" t="inlineStr">
+      <c r="I61" s="73" t="inlineStr">
         <is>
           <t>B777-300ER</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="40" t="inlineStr">
+      <c r="A62" s="70" t="inlineStr">
         <is>
           <t>OZ202</t>
         </is>
       </c>
-      <c r="B62" s="6" t="inlineStr">
+      <c r="B62" s="72" t="inlineStr">
         <is>
           <t>Asiana</t>
         </is>
       </c>
-      <c r="C62" s="6" t="inlineStr">
+      <c r="C62" s="72" t="inlineStr">
         <is>
           <t>14:40</t>
         </is>
       </c>
-      <c r="D62" s="6" t="inlineStr">
+      <c r="D62" s="72" t="inlineStr">
         <is>
           <t>09:30</t>
         </is>
       </c>
-      <c r="E62" s="6" t="inlineStr">
+      <c r="E62" s="72" t="inlineStr">
         <is>
           <t>ICN→LAX</t>
         </is>
       </c>
-      <c r="F62" s="6" t="inlineStr">
+      <c r="F62" s="72" t="inlineStr">
         <is>
           <t>Daily A380</t>
         </is>
       </c>
-      <c r="G62" s="47" t="inlineStr">
+      <c r="G62" s="73" t="inlineStr">
         <is>
           <t>First Suite | Business | Economy</t>
         </is>
       </c>
-      <c r="H62" s="47" t="inlineStr">
+      <c r="H62" s="73" t="inlineStr">
         <is>
           <t>~11.5</t>
         </is>
       </c>
-      <c r="I62" s="47" t="inlineStr">
+      <c r="I62" s="73" t="inlineStr">
         <is>
           <t>A380-800</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="40" t="inlineStr">
+      <c r="A63" s="70" t="inlineStr">
         <is>
           <t>OZ204</t>
         </is>
       </c>
-      <c r="B63" s="6" t="inlineStr">
+      <c r="B63" s="72" t="inlineStr">
         <is>
           <t>Asiana</t>
         </is>
       </c>
-      <c r="C63" s="6" t="inlineStr">
+      <c r="C63" s="72" t="inlineStr">
         <is>
           <t>20:40</t>
         </is>
       </c>
-      <c r="D63" s="6" t="inlineStr">
+      <c r="D63" s="72" t="inlineStr">
         <is>
           <t>15:30</t>
         </is>
       </c>
-      <c r="E63" s="6" t="inlineStr">
+      <c r="E63" s="72" t="inlineStr">
         <is>
           <t>ICN→LAX</t>
         </is>
       </c>
-      <c r="F63" s="6" t="inlineStr">
+      <c r="F63" s="72" t="inlineStr">
         <is>
           <t>Daily A350</t>
         </is>
       </c>
-      <c r="G63" s="47" t="inlineStr">
+      <c r="G63" s="73" t="inlineStr">
         <is>
           <t>Business | Economy</t>
         </is>
       </c>
-      <c r="H63" s="47" t="inlineStr">
+      <c r="H63" s="73" t="inlineStr">
         <is>
           <t>~11.5</t>
         </is>
       </c>
-      <c r="I63" s="47" t="inlineStr">
+      <c r="I63" s="73" t="inlineStr">
         <is>
           <t>A350-900</t>
         </is>
@@ -1828,9 +1990,6 @@
       <c r="E68" s="6" t="n"/>
       <c r="F68" s="6" t="n"/>
     </row>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="31" t="inlineStr">
         <is>
@@ -1892,188 +2051,188 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="40" t="inlineStr">
+      <c r="A74" s="70" t="inlineStr">
         <is>
           <t>KE012</t>
         </is>
       </c>
-      <c r="B74" s="6" t="inlineStr">
+      <c r="B74" s="72" t="inlineStr">
         <is>
           <t>Korean Air</t>
         </is>
       </c>
-      <c r="C74" s="6" t="inlineStr">
+      <c r="C74" s="72" t="inlineStr">
         <is>
           <t>23:50</t>
         </is>
       </c>
-      <c r="D74" s="6" t="inlineStr">
+      <c r="D74" s="72" t="inlineStr">
         <is>
           <t>05:00+2</t>
         </is>
       </c>
-      <c r="E74" s="6" t="inlineStr">
+      <c r="E74" s="72" t="inlineStr">
         <is>
           <t>LAX→ICN</t>
         </is>
       </c>
-      <c r="F74" s="6" t="inlineStr">
+      <c r="F74" s="72" t="inlineStr">
         <is>
           <t xml:space="preserve">Daily B747-8 </t>
         </is>
       </c>
-      <c r="G74" s="47" t="inlineStr">
+      <c r="G74" s="73" t="inlineStr">
         <is>
           <t>First | Prestige | Economy</t>
         </is>
       </c>
-      <c r="H74" s="47" t="inlineStr">
+      <c r="H74" s="73" t="inlineStr">
         <is>
           <t>~13</t>
         </is>
       </c>
-      <c r="I74" s="47" t="inlineStr">
+      <c r="I74" s="73" t="inlineStr">
         <is>
           <t>B747-8</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="40" t="inlineStr">
+      <c r="A75" s="70" t="inlineStr">
         <is>
           <t>KE018</t>
         </is>
       </c>
-      <c r="B75" s="6" t="inlineStr">
+      <c r="B75" s="72" t="inlineStr">
         <is>
           <t>Korean Air</t>
         </is>
       </c>
-      <c r="C75" s="6" t="inlineStr">
+      <c r="C75" s="72" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="D75" s="6" t="inlineStr">
+      <c r="D75" s="72" t="inlineStr">
         <is>
           <t>18:40+1</t>
         </is>
       </c>
-      <c r="E75" s="6" t="inlineStr">
+      <c r="E75" s="72" t="inlineStr">
         <is>
           <t>LAX→ICN</t>
         </is>
       </c>
-      <c r="F75" s="6" t="inlineStr">
+      <c r="F75" s="72" t="inlineStr">
         <is>
           <t>Daily B777</t>
         </is>
       </c>
-      <c r="G75" s="47" t="inlineStr">
+      <c r="G75" s="73" t="inlineStr">
         <is>
           <t>Prestige | Economy</t>
         </is>
       </c>
-      <c r="H75" s="47" t="inlineStr">
+      <c r="H75" s="73" t="inlineStr">
         <is>
           <t>~13</t>
         </is>
       </c>
-      <c r="I75" s="47" t="inlineStr">
+      <c r="I75" s="73" t="inlineStr">
         <is>
           <t>B777-300ER</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="40" t="inlineStr">
+      <c r="A76" s="70" t="inlineStr">
         <is>
           <t>OZ201</t>
         </is>
       </c>
-      <c r="B76" s="6" t="inlineStr">
+      <c r="B76" s="72" t="inlineStr">
         <is>
           <t>Asiana</t>
         </is>
       </c>
-      <c r="C76" s="6" t="inlineStr">
+      <c r="C76" s="72" t="inlineStr">
         <is>
           <t>23:30</t>
         </is>
       </c>
-      <c r="D76" s="6" t="inlineStr">
+      <c r="D76" s="72" t="inlineStr">
         <is>
           <t>04:30+2</t>
         </is>
       </c>
-      <c r="E76" s="6" t="inlineStr">
+      <c r="E76" s="72" t="inlineStr">
         <is>
           <t>LAX→ICN</t>
         </is>
       </c>
-      <c r="F76" s="6" t="inlineStr">
+      <c r="F76" s="72" t="inlineStr">
         <is>
           <t>Daily A380</t>
         </is>
       </c>
-      <c r="G76" s="47" t="inlineStr">
+      <c r="G76" s="73" t="inlineStr">
         <is>
           <t>First Suite | Business | Economy</t>
         </is>
       </c>
-      <c r="H76" s="47" t="inlineStr">
+      <c r="H76" s="73" t="inlineStr">
         <is>
           <t>~13</t>
         </is>
       </c>
-      <c r="I76" s="47" t="inlineStr">
+      <c r="I76" s="73" t="inlineStr">
         <is>
           <t>A380-800</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="40" t="inlineStr">
+      <c r="A77" s="70" t="inlineStr">
         <is>
           <t>OZ203</t>
         </is>
       </c>
-      <c r="B77" s="6" t="inlineStr">
+      <c r="B77" s="72" t="inlineStr">
         <is>
           <t>Asiana</t>
         </is>
       </c>
-      <c r="C77" s="6" t="inlineStr">
+      <c r="C77" s="72" t="inlineStr">
         <is>
           <t>13:00</t>
         </is>
       </c>
-      <c r="D77" s="6" t="inlineStr">
+      <c r="D77" s="72" t="inlineStr">
         <is>
           <t>18:10+1</t>
         </is>
       </c>
-      <c r="E77" s="6" t="inlineStr">
+      <c r="E77" s="72" t="inlineStr">
         <is>
           <t>LAX→ICN</t>
         </is>
       </c>
-      <c r="F77" s="6" t="inlineStr">
+      <c r="F77" s="72" t="inlineStr">
         <is>
           <t>Daily A350</t>
         </is>
       </c>
-      <c r="G77" s="47" t="inlineStr">
+      <c r="G77" s="73" t="inlineStr">
         <is>
           <t>Business | Economy</t>
         </is>
       </c>
-      <c r="H77" s="47" t="inlineStr">
+      <c r="H77" s="73" t="inlineStr">
         <is>
           <t>~13</t>
         </is>
       </c>
-      <c r="I77" s="47" t="inlineStr">
+      <c r="I77" s="73" t="inlineStr">
         <is>
           <t>A350-900</t>
         </is>
@@ -2119,7 +2278,6 @@
       <c r="E82" s="6" t="n"/>
       <c r="F82" s="6" t="n"/>
     </row>
-    <row r="83"/>
     <row r="84">
       <c r="A84" s="48" t="inlineStr">
         <is>
@@ -2160,15 +2318,15 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="49" t="inlineStr">
+      <c r="A86" s="74" t="inlineStr">
         <is>
           <t>NBA/MLB Game (Ticket)</t>
         </is>
       </c>
-      <c r="B86" s="50" t="n">
+      <c r="B86" s="75" t="n">
         <v>120</v>
       </c>
-      <c r="C86" s="50" t="n">
+      <c r="C86" s="75" t="n">
         <v>180</v>
       </c>
       <c r="D86" s="51">
@@ -2188,15 +2346,15 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="49" t="inlineStr">
+      <c r="A87" s="74" t="inlineStr">
         <is>
           <t>Sports Bar Experience</t>
         </is>
       </c>
-      <c r="B87" s="50" t="n">
+      <c r="B87" s="75" t="n">
         <v>60</v>
       </c>
-      <c r="C87" s="50" t="n">
+      <c r="C87" s="75" t="n">
         <v>90</v>
       </c>
       <c r="D87" s="51">
@@ -2216,15 +2374,15 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="49" t="inlineStr">
+      <c r="A88" s="74" t="inlineStr">
         <is>
           <t>Local Hiking (Griffith/Runyon)</t>
         </is>
       </c>
-      <c r="B88" s="50" t="n">
+      <c r="B88" s="75" t="n">
         <v>0</v>
       </c>
-      <c r="C88" s="50" t="n">
+      <c r="C88" s="75" t="n">
         <v>30</v>
       </c>
       <c r="D88" s="51">
@@ -2244,15 +2402,15 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="49" t="inlineStr">
+      <c r="A89" s="74" t="inlineStr">
         <is>
           <t>Beach/Surf Lesson</t>
         </is>
       </c>
-      <c r="B89" s="50" t="n">
+      <c r="B89" s="75" t="n">
         <v>60</v>
       </c>
-      <c r="C89" s="50" t="n">
+      <c r="C89" s="75" t="n">
         <v>100</v>
       </c>
       <c r="D89" s="51">
@@ -2272,7 +2430,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="49" t="inlineStr">
+      <c r="A90" s="74" t="inlineStr">
         <is>
           <t>(New Activity 5)</t>
         </is>
@@ -2288,7 +2446,7 @@
       <c r="G90" s="49" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="49" t="inlineStr">
+      <c r="A91" s="74" t="inlineStr">
         <is>
           <t>(New Activity 6)</t>
         </is>
@@ -2304,7 +2462,7 @@
       <c r="G91" s="49" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="49" t="inlineStr">
+      <c r="A92" s="74" t="inlineStr">
         <is>
           <t>(New Activity 7)</t>
         </is>
@@ -2320,7 +2478,7 @@
       <c r="G92" s="49" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="49" t="inlineStr">
+      <c r="A93" s="74" t="inlineStr">
         <is>
           <t>(New Activity 8)</t>
         </is>
@@ -2336,7 +2494,7 @@
       <c r="G93" s="49" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="49" t="inlineStr">
+      <c r="A94" s="74" t="inlineStr">
         <is>
           <t>(New Activity 9)</t>
         </is>
@@ -2374,7 +2532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="42" min="1" max="1"/>
@@ -2407,311 +2565,337 @@
       </c>
     </row>
     <row r="4" ht="16.5" customHeight="1" s="42">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="76" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="76" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="76" t="inlineStr">
         <is>
           <t>일정</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="76" t="inlineStr">
         <is>
           <t>패키지명</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="76" t="inlineStr">
         <is>
           <t>박</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="76" t="inlineStr">
         <is>
           <t>일</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="76" t="inlineStr">
         <is>
           <t>Rds</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="76" t="inlineStr">
         <is>
           <t>코스구성</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>골프C</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>골프S</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>호텔C</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>호텔S</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="I4" s="77" t="inlineStr">
+        <is>
+          <t>⛳ 골프</t>
+        </is>
+      </c>
+      <c r="J4" s="78" t="n"/>
+      <c r="K4" s="77" t="inlineStr">
+        <is>
+          <t>🏨 호텔</t>
+        </is>
+      </c>
+      <c r="L4" s="78" t="n"/>
+      <c r="M4" s="76" t="inlineStr">
         <is>
           <t>마진</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="N4" s="76" t="inlineStr">
         <is>
           <t>마진율</t>
         </is>
       </c>
     </row>
     <row r="5" ht="51" customHeight="1" s="42">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="79" t="n"/>
+      <c r="B5" s="79" t="n"/>
+      <c r="C5" s="79" t="n"/>
+      <c r="D5" s="79" t="n"/>
+      <c r="E5" s="79" t="n"/>
+      <c r="F5" s="79" t="n"/>
+      <c r="G5" s="79" t="n"/>
+      <c r="H5" s="79" t="n"/>
+      <c r="I5" s="79" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="J5" s="79" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="K5" s="79" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="L5" s="79" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="M5" s="79" t="n"/>
+      <c r="N5" s="79" t="n"/>
+    </row>
+    <row r="6" ht="51" customHeight="1" s="42">
+      <c r="A6" s="80" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="81" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C6" s="80" t="inlineStr">
         <is>
           <t>3N4D</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D6" s="80" t="inlineStr">
         <is>
           <t>트럼프 + 샌드파이퍼 오션뷰</t>
         </is>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E6" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F6" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G6" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H6" s="80" t="inlineStr">
         <is>
           <t>Trump×1 + Sand×1</t>
         </is>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="I6" s="82" t="n">
         <v>340</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="J6" s="82" t="n">
         <v>745</v>
       </c>
-      <c r="K5" s="5" t="n">
+      <c r="K6" s="82" t="n">
         <v>825</v>
       </c>
-      <c r="L5" s="5" t="n">
+      <c r="L6" s="82" t="n">
         <v>1125</v>
       </c>
-      <c r="M5" s="8">
-        <f>J5+L5-I5-K5</f>
-        <v/>
-      </c>
-      <c r="N5" s="9">
-        <f>IF(J5+L5&gt;0,(J5+L5-I5-K5)/(J5+L5),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" ht="51" customHeight="1" s="42">
-      <c r="A6" s="6" t="n">
+      <c r="M6" s="83">
+        <f>J6+L6-I6-K6</f>
+        <v/>
+      </c>
+      <c r="N6" s="84">
+        <f>IF(J6+L6&gt;0,(J6+L6-I6-K6)/(J6+L6),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="34.5" customHeight="1" s="42">
+      <c r="A7" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B7" s="81" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C7" s="80" t="inlineStr">
         <is>
           <t>3N4D</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="80" t="inlineStr">
         <is>
           <t>트럼프 + 히든밸리 밸리뷰</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E7" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F7" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G7" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H7" s="80" t="inlineStr">
         <is>
           <t>Trump×1 + HV×1</t>
         </is>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="I7" s="82" t="n">
         <v>319</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="J7" s="82" t="n">
         <v>609</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="K7" s="82" t="n">
         <v>825</v>
       </c>
-      <c r="L6" s="5" t="n">
+      <c r="L7" s="82" t="n">
         <v>1125</v>
       </c>
-      <c r="M6" s="8">
-        <f>J6+L6-I6-K6</f>
-        <v/>
-      </c>
-      <c r="N6" s="9">
-        <f>IF(J6+L6&gt;0,(J6+L6-I6-K6)/(J6+L6),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="34.5" customHeight="1" s="42">
-      <c r="A7" s="6" t="n">
+      <c r="M7" s="83">
+        <f>J7+L7-I7-K7</f>
+        <v/>
+      </c>
+      <c r="N7" s="84">
+        <f>IF(J7+L7&gt;0,(J7+L7-I7-K7)/(J7+L7),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B8" s="81" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C8" s="80" t="inlineStr">
         <is>
           <t>3N4D</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D8" s="80" t="inlineStr">
         <is>
           <t>샌드파이퍼 + 히든밸리</t>
         </is>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E8" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F8" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="G8" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H8" s="80" t="inlineStr">
         <is>
           <t>Sand×1 + HV×1</t>
         </is>
       </c>
-      <c r="I7" s="5" t="n">
+      <c r="I8" s="82" t="n">
         <v>239</v>
       </c>
-      <c r="J7" s="5" t="n">
+      <c r="J8" s="82" t="n">
         <v>354</v>
       </c>
-      <c r="K7" s="5" t="n">
+      <c r="K8" s="82" t="n">
         <v>825</v>
       </c>
-      <c r="L7" s="5" t="n">
+      <c r="L8" s="82" t="n">
         <v>1125</v>
       </c>
-      <c r="M7" s="8">
-        <f>J7+L7-I7-K7</f>
-        <v/>
-      </c>
-      <c r="N7" s="9">
-        <f>IF(J7+L7&gt;0,(J7+L7-I7-K7)/(J7+L7),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="n"/>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="10" t="n"/>
-      <c r="I8" s="10" t="n"/>
-      <c r="J8" s="10" t="n"/>
-      <c r="K8" s="10" t="n"/>
-      <c r="L8" s="10" t="n"/>
-      <c r="M8" s="10" t="n"/>
-      <c r="N8" s="10" t="n"/>
+      <c r="M8" s="83">
+        <f>J8+L8-I8-K8</f>
+        <v/>
+      </c>
+      <c r="N8" s="84">
+        <f>IF(J8+L8&gt;0,(J8+L8-I8-K8)/(J8+L8),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="51" customHeight="1" s="42">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
+      <c r="H9" s="10" t="n"/>
+      <c r="I9" s="10" t="n"/>
+      <c r="J9" s="10" t="n"/>
+      <c r="K9" s="10" t="n"/>
+      <c r="L9" s="10" t="n"/>
+      <c r="M9" s="10" t="n"/>
+      <c r="N9" s="10" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B10" s="81" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C10" s="80" t="inlineStr">
         <is>
           <t>5N7D</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D10" s="80" t="inlineStr">
         <is>
           <t>트럼프+샌드+히든 3色 시그니처</t>
         </is>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="E10" s="80" t="n">
         <v>5</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F10" s="80" t="n">
         <v>7</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="G10" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H10" s="80" t="inlineStr">
         <is>
           <t>Trump×1+Sand×1+HV×1</t>
         </is>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="I10" s="82" t="n">
         <v>449</v>
       </c>
-      <c r="J9" s="5" t="n">
+      <c r="J10" s="82" t="n">
         <v>854</v>
       </c>
-      <c r="K9" s="5" t="n">
+      <c r="K10" s="82" t="n">
         <v>1375</v>
       </c>
-      <c r="L9" s="5" t="n">
+      <c r="L10" s="82" t="n">
         <v>1875</v>
       </c>
-      <c r="M9" s="8">
-        <f>J9+L9-I9-K9</f>
-        <v/>
-      </c>
-      <c r="N9" s="9">
-        <f>IF(J9+L9&gt;0,(J9+L9-I9-K9)/(J9+L9),0)</f>
+      <c r="M10" s="83">
+        <f>J10+L10-I10-K10</f>
+        <v/>
+      </c>
+      <c r="N10" s="84">
+        <f>IF(J10+L10&gt;0,(J10+L10-I10-K10)/(J10+L10),0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="I4:J4"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2750,8 +2934,6 @@
           <t>🎯 결 TOUR — Package Selector &amp; Estimator</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr"/>
-      <c r="N1" t="inlineStr"/>
     </row>
     <row r="2" s="42">
       <c r="A2" s="37" t="inlineStr">
@@ -2759,17 +2941,8 @@
           <t>⬇️ 드롭다운 선택 → 가격 자동계산 → 항공편 연동 → 나만의 견적 완성!</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -2787,8 +2960,6 @@
       <c r="J4" s="44" t="n"/>
       <c r="K4" s="44" t="n"/>
       <c r="L4" s="45" t="n"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5" ht="30.75" customHeight="1" s="42">
       <c r="A5" s="11" t="inlineStr">
@@ -2813,17 +2984,8 @@
           <t>persons</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="31" t="inlineStr">
         <is>
@@ -2841,8 +3003,6 @@
       <c r="J7" s="44" t="n"/>
       <c r="K7" s="44" t="n"/>
       <c r="L7" s="45" t="n"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8" ht="32.25" customHeight="1" s="42">
       <c r="A8" s="11" t="inlineStr">
@@ -2987,8 +3147,6 @@
       <c r="J10" s="19" t="n"/>
       <c r="K10" s="19" t="inlineStr"/>
       <c r="L10" s="19" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11" ht="32.25" customHeight="1" s="42">
       <c r="A11" s="11" t="inlineStr">
@@ -3033,17 +3191,8 @@
         <f>IF(C11&lt;&gt;"",C11&amp;"N"&amp;F11&amp;"D","Select flights ↑")</f>
         <v/>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="31" t="inlineStr">
         <is>
@@ -3061,8 +3210,6 @@
       <c r="J13" s="44" t="n"/>
       <c r="K13" s="44" t="n"/>
       <c r="L13" s="45" t="n"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14" ht="32.25" customHeight="1" s="42">
       <c r="A14" s="2" t="inlineStr">
@@ -3117,221 +3264,204 @@
       </c>
       <c r="K14" s="2" t="inlineStr"/>
       <c r="L14" s="2" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15" ht="30.75" customHeight="1" s="42">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="80" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="34" t="inlineStr">
+      <c r="B15" s="85" t="inlineStr">
         <is>
           <t>Trump National LA</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="86" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="5">
-        <f>IF(B15="","",VLOOKUP(B15,'Master Data'!$A$7:$E$15,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E15" s="5">
-        <f>IF(B15="","",VLOOKUP(B15,'Master Data'!$A$7:$E$15,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F15" s="5">
+      <c r="D15" s="87">
+        <f>IF(B15="","",VLOOKUP(B15,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E15" s="87">
+        <f>IF(B15="","",VLOOKUP(B15,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F15" s="87">
         <f>IF(E15&lt;&gt;"",E15-D15,"")</f>
         <v/>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="87">
         <f>IF(B15="","",C15*D15)</f>
         <v/>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="87">
         <f>IF(B15="","",C15*E15)</f>
         <v/>
       </c>
-      <c r="I15" s="5">
+      <c r="I15" s="87">
         <f>IF(H15&lt;&gt;"",H15-G15,"")</f>
         <v/>
       </c>
-      <c r="J15" s="5">
-        <f>IF(B15="","",IF(C15&gt;1,(C15-1)*VLOOKUP(B15,'Master Data'!$A$7:$E$15,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="J15" s="87">
+        <f>IF(B15="","",IF(C15&gt;1,(C15-1)*VLOOKUP(B15,'Master Data'!$A$7:$E$14,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L15" s="6" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16" ht="30.75" customHeight="1" s="42">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="B16" s="34" t="inlineStr">
+      <c r="B16" s="85" t="inlineStr">
         <is>
           <t>Sandpiper GC</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" s="86" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="5">
-        <f>IF(B16="","",VLOOKUP(B16,'Master Data'!$A$7:$E$15,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E16" s="5">
-        <f>IF(B16="","",VLOOKUP(B16,'Master Data'!$A$7:$E$15,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F16" s="5">
+      <c r="D16" s="87">
+        <f>IF(B16="","",VLOOKUP(B16,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E16" s="87">
+        <f>IF(B16="","",VLOOKUP(B16,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F16" s="87">
         <f>IF(E16&lt;&gt;"",E16-D16,"")</f>
         <v/>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="87">
         <f>IF(B16="","",C16*D16)</f>
         <v/>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="87">
         <f>IF(B16="","",C16*E16)</f>
         <v/>
       </c>
-      <c r="I16" s="5">
+      <c r="I16" s="87">
         <f>IF(H16&lt;&gt;"",H16-G16,"")</f>
         <v/>
       </c>
-      <c r="J16" s="5">
-        <f>IF(B16="","",IF(C16&gt;1,(C16-1)*VLOOKUP(B16,'Master Data'!$A$7:$E$15,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="J16" s="87">
+        <f>IF(B16="","",IF(C16&gt;1,(C16-1)*VLOOKUP(B16,'Master Data'!$A$7:$E$14,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L16" s="6" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17" ht="30.75" customHeight="1" s="42">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="B17" s="34" t="inlineStr">
+      <c r="B17" s="85" t="inlineStr">
         <is>
           <t>Hidden Valley GC</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="86" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="5">
-        <f>IF(B17="","",VLOOKUP(B17,'Master Data'!$A$7:$E$15,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E17" s="5">
-        <f>IF(B17="","",VLOOKUP(B17,'Master Data'!$A$7:$E$15,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F17" s="5">
+      <c r="D17" s="87">
+        <f>IF(B17="","",VLOOKUP(B17,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E17" s="87">
+        <f>IF(B17="","",VLOOKUP(B17,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F17" s="87">
         <f>IF(E17&lt;&gt;"",E17-D17,"")</f>
         <v/>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="87">
         <f>IF(B17="","",C17*D17)</f>
         <v/>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="87">
         <f>IF(B17="","",C17*E17)</f>
         <v/>
       </c>
-      <c r="I17" s="5">
+      <c r="I17" s="87">
         <f>IF(H17&lt;&gt;"",H17-G17,"")</f>
         <v/>
       </c>
-      <c r="J17" s="5">
-        <f>IF(B17="","",IF(C17&gt;1,(C17-1)*VLOOKUP(B17,'Master Data'!$A$7:$E$15,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K17" t="inlineStr"/>
+      <c r="J17" s="87">
+        <f>IF(B17="","",IF(C17&gt;1,(C17-1)*VLOOKUP(B17,'Master Data'!$A$7:$E$14,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L17" s="6" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="B18" s="34" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="5">
-        <f>IF(B18="","",VLOOKUP(B18,'Master Data'!$A$7:$E$15,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E18" s="5">
-        <f>IF(B18="","",VLOOKUP(B18,'Master Data'!$A$7:$E$15,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F18" s="5">
+      <c r="B18" s="85" t="n"/>
+      <c r="C18" s="86" t="n"/>
+      <c r="D18" s="87">
+        <f>IF(B18="","",VLOOKUP(B18,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E18" s="87">
+        <f>IF(B18="","",VLOOKUP(B18,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F18" s="87">
         <f>IF(E18&lt;&gt;"",E18-D18,"")</f>
         <v/>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="87">
         <f>IF(B18="","",C18*D18)</f>
         <v/>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="87">
         <f>IF(B18="","",C18*E18)</f>
         <v/>
       </c>
-      <c r="I18" s="5">
+      <c r="I18" s="87">
         <f>IF(H18&lt;&gt;"",H18-G18,"")</f>
         <v/>
       </c>
-      <c r="J18" s="5">
-        <f>IF(B18="","",IF(C18&gt;1,(C18-1)*VLOOKUP(B18,'Master Data'!$A$7:$E$15,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K18" t="inlineStr"/>
+      <c r="J18" s="87">
+        <f>IF(B18="","",IF(C18&gt;1,(C18-1)*VLOOKUP(B18,'Master Data'!$A$7:$E$14,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L18" s="6" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n">
+      <c r="A19" s="80" t="n">
         <v>5</v>
       </c>
-      <c r="B19" s="34" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="5">
-        <f>IF(B19="","",VLOOKUP(B19,'Master Data'!$A$7:$E$15,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E19" s="5">
-        <f>IF(B19="","",VLOOKUP(B19,'Master Data'!$A$7:$E$15,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F19" s="5">
+      <c r="B19" s="85" t="n"/>
+      <c r="C19" s="86" t="n"/>
+      <c r="D19" s="87">
+        <f>IF(B19="","",VLOOKUP(B19,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E19" s="87">
+        <f>IF(B19="","",VLOOKUP(B19,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F19" s="87">
         <f>IF(E19&lt;&gt;"",E19-D19,"")</f>
         <v/>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="87">
         <f>IF(B19="","",C19*D19)</f>
         <v/>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="87">
         <f>IF(B19="","",C19*E19)</f>
         <v/>
       </c>
-      <c r="I19" s="5">
+      <c r="I19" s="87">
         <f>IF(H19&lt;&gt;"",H19-G19,"")</f>
         <v/>
       </c>
-      <c r="J19" s="5">
-        <f>IF(B19="","",IF(C19&gt;1,(C19-1)*VLOOKUP(B19,'Master Data'!$A$7:$E$15,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="J19" s="87">
+        <f>IF(B19="","",IF(C19&gt;1,(C19-1)*VLOOKUP(B19,'Master Data'!$A$7:$E$14,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L19" s="6" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="33" t="inlineStr">
@@ -3360,17 +3490,9 @@
         <f>SUM(J15:J19)</f>
         <v/>
       </c>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" s="6" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="31" t="inlineStr">
         <is>
@@ -3388,8 +3510,6 @@
       <c r="J22" s="44" t="n"/>
       <c r="K22" s="44" t="n"/>
       <c r="L22" s="45" t="n"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23" ht="32.25" customHeight="1" s="42">
       <c r="A23" s="2" t="inlineStr">
@@ -3437,11 +3557,7 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Replay</t>
-        </is>
-      </c>
+      <c r="J23" s="2" t="n"/>
       <c r="K23" s="52" t="inlineStr">
         <is>
           <t>Room Type</t>
@@ -3452,43 +3568,38 @@
           <t>Beds/Room</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n">
+      <c r="A24" s="80" t="n">
         <v>1</v>
       </c>
-      <c r="B24" s="34" t="n"/>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="5">
-        <f>IF(B24="","",VLOOKUP(B24,'Master Data'!$A$19:$D$25,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E24" s="5">
-        <f>IF(B24="","",VLOOKUP(B24,'Master Data'!$A$19:$D$25,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F24" s="5">
+      <c r="B24" s="85" t="n"/>
+      <c r="C24" s="86" t="n"/>
+      <c r="D24" s="87">
+        <f>IF(B24="","",VLOOKUP(B24,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E24" s="87">
+        <f>IF(B24="","",VLOOKUP(B24,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F24" s="87">
         <f>IF(E24&lt;&gt;"",E24-D24,"")</f>
         <v/>
       </c>
-      <c r="G24" s="5">
+      <c r="G24" s="87">
         <f>IF(B24="","",C24*D24)</f>
         <v/>
       </c>
-      <c r="H24" s="5">
+      <c r="H24" s="87">
         <f>IF(B24="","",C24*E24)</f>
         <v/>
       </c>
-      <c r="I24" s="5">
+      <c r="I24" s="87">
         <f>IF(H24&lt;&gt;"",H24-G24,"")</f>
         <v/>
       </c>
-      <c r="J24" s="5">
-        <f>IF(B24="","",IF(C24&gt;1,(C24-1)*VLOOKUP(B24,'Master Data'!$A$19:$D$25,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J24" s="82" t="n"/>
       <c r="K24" s="50" t="inlineStr">
         <is>
           <t>2인1실</t>
@@ -3497,43 +3608,38 @@
       <c r="L24" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="n">
+      <c r="A25" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="B25" s="34" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="5">
-        <f>IF(B25="","",VLOOKUP(B25,'Master Data'!$A$19:$D$25,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E25" s="5">
-        <f>IF(B25="","",VLOOKUP(B25,'Master Data'!$A$19:$D$25,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F25" s="5">
+      <c r="B25" s="85" t="n"/>
+      <c r="C25" s="86" t="n"/>
+      <c r="D25" s="87">
+        <f>IF(B25="","",VLOOKUP(B25,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E25" s="87">
+        <f>IF(B25="","",VLOOKUP(B25,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F25" s="87">
         <f>IF(E25&lt;&gt;"",E25-D25,"")</f>
         <v/>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="87">
         <f>IF(B25="","",C25*D25)</f>
         <v/>
       </c>
-      <c r="H25" s="5">
+      <c r="H25" s="87">
         <f>IF(B25="","",C25*E25)</f>
         <v/>
       </c>
-      <c r="I25" s="5">
+      <c r="I25" s="87">
         <f>IF(H25&lt;&gt;"",H25-G25,"")</f>
         <v/>
       </c>
-      <c r="J25" s="5">
-        <f>IF(B25="","",IF(C25&gt;1,(C25-1)*VLOOKUP(B25,'Master Data'!$A$19:$D$25,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J25" s="82" t="n"/>
       <c r="K25" s="50" t="inlineStr">
         <is>
           <t>2인1실</t>
@@ -3542,43 +3648,38 @@
       <c r="L25" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="n">
+      <c r="A26" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="B26" s="34" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="5">
-        <f>IF(B26="","",VLOOKUP(B26,'Master Data'!$A$19:$D$25,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E26" s="5">
-        <f>IF(B26="","",VLOOKUP(B26,'Master Data'!$A$19:$D$25,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F26" s="5">
+      <c r="B26" s="85" t="n"/>
+      <c r="C26" s="86" t="n"/>
+      <c r="D26" s="87">
+        <f>IF(B26="","",VLOOKUP(B26,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E26" s="87">
+        <f>IF(B26="","",VLOOKUP(B26,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F26" s="87">
         <f>IF(E26&lt;&gt;"",E26-D26,"")</f>
         <v/>
       </c>
-      <c r="G26" s="5">
+      <c r="G26" s="87">
         <f>IF(B26="","",C26*D26)</f>
         <v/>
       </c>
-      <c r="H26" s="5">
+      <c r="H26" s="87">
         <f>IF(B26="","",C26*E26)</f>
         <v/>
       </c>
-      <c r="I26" s="5">
+      <c r="I26" s="87">
         <f>IF(H26&lt;&gt;"",H26-G26,"")</f>
         <v/>
       </c>
-      <c r="J26" s="5">
-        <f>IF(B26="","",IF(C26&gt;1,(C26-1)*VLOOKUP(B26,'Master Data'!$A$19:$D$25,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J26" s="82" t="n"/>
       <c r="K26" s="50" t="inlineStr">
         <is>
           <t>2인1실</t>
@@ -3587,8 +3688,6 @@
       <c r="L26" s="54" t="n">
         <v>2</v>
       </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="33" t="inlineStr">
@@ -3613,21 +3712,10 @@
         <f>SUM(I24:I26)</f>
         <v/>
       </c>
-      <c r="J27" s="8">
-        <f>SUM(J24:J26)</f>
-        <v/>
-      </c>
-      <c r="K27" t="inlineStr"/>
+      <c r="J27" s="8" t="n"/>
       <c r="L27" s="6" t="inlineStr"/>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="K28" t="inlineStr"/>
-      <c r="L28" t="inlineStr"/>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="31" t="inlineStr">
         <is>
@@ -3645,8 +3733,6 @@
       <c r="J29" s="44" t="n"/>
       <c r="K29" s="44" t="n"/>
       <c r="L29" s="45" t="n"/>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30" ht="32.25" customHeight="1" s="42">
       <c r="A30" s="2" t="inlineStr">
@@ -3694,11 +3780,7 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>Replay</t>
-        </is>
-      </c>
+      <c r="J30" s="2" t="n"/>
       <c r="K30" s="52" t="inlineStr">
         <is>
           <t>Vehicle Type</t>
@@ -3709,47 +3791,42 @@
           <t>Pax Capacity</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31" ht="47.25" customHeight="1" s="42">
-      <c r="A31" s="6" t="n">
+      <c r="A31" s="80" t="n">
         <v>1</v>
       </c>
-      <c r="B31" s="34" t="inlineStr">
+      <c r="B31" s="85" t="inlineStr">
         <is>
           <t>Driver/Guide + Van (일당)</t>
         </is>
       </c>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="5">
-        <f>IF(B31="","",VLOOKUP(B31,'Master Data'!$A$28:$D$34,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E31" s="5">
-        <f>IF(B31="","",VLOOKUP(B31,'Master Data'!$A$28:$D$34,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F31" s="5">
+      <c r="C31" s="86" t="n"/>
+      <c r="D31" s="87">
+        <f>IF(B31="","",VLOOKUP(B31,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E31" s="87">
+        <f>IF(B31="","",VLOOKUP(B31,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F31" s="87">
         <f>IF(E31&lt;&gt;"",E31-D31,"")</f>
         <v/>
       </c>
-      <c r="G31" s="5">
+      <c r="G31" s="87">
         <f>IF(B31="","",C31*D31)</f>
         <v/>
       </c>
-      <c r="H31" s="5">
+      <c r="H31" s="87">
         <f>IF(B31="","",C31*E31)</f>
         <v/>
       </c>
-      <c r="I31" s="5">
+      <c r="I31" s="87">
         <f>IF(H31&lt;&gt;"",H31-G31,"")</f>
         <v/>
       </c>
-      <c r="J31" s="5">
-        <f>IF(B31="","",IF(C31&gt;1,(C31-1)*VLOOKUP(B31,'Master Data'!$A$28:$D$34,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J31" s="82" t="n"/>
       <c r="K31" s="50" t="inlineStr">
         <is>
           <t>Full-size Van</t>
@@ -3760,86 +3837,74 @@
           <t>7-8</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="n">
+      <c r="A32" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="B32" s="34" t="n"/>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="5">
-        <f>IF(B32="","",VLOOKUP(B32,'Master Data'!$A$28:$D$34,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E32" s="5">
-        <f>IF(B32="","",VLOOKUP(B32,'Master Data'!$A$28:$D$34,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F32" s="5">
+      <c r="B32" s="85" t="n"/>
+      <c r="C32" s="86" t="n"/>
+      <c r="D32" s="87">
+        <f>IF(B32="","",VLOOKUP(B32,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E32" s="87">
+        <f>IF(B32="","",VLOOKUP(B32,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F32" s="87">
         <f>IF(E32&lt;&gt;"",E32-D32,"")</f>
         <v/>
       </c>
-      <c r="G32" s="5">
+      <c r="G32" s="87">
         <f>IF(B32="","",C32*D32)</f>
         <v/>
       </c>
-      <c r="H32" s="5">
+      <c r="H32" s="87">
         <f>IF(B32="","",C32*E32)</f>
         <v/>
       </c>
-      <c r="I32" s="5">
+      <c r="I32" s="87">
         <f>IF(H32&lt;&gt;"",H32-G32,"")</f>
         <v/>
       </c>
-      <c r="J32" s="5">
-        <f>IF(B32="","",IF(C32&gt;1,(C32-1)*VLOOKUP(B32,'Master Data'!$A$28:$D$34,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J32" s="82" t="n"/>
       <c r="K32" s="50" t="inlineStr"/>
       <c r="L32" s="55" t="inlineStr"/>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n">
+      <c r="A33" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="B33" s="34" t="n"/>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="5">
-        <f>IF(B33="","",VLOOKUP(B33,'Master Data'!$A$28:$D$34,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E33" s="5">
-        <f>IF(B33="","",VLOOKUP(B33,'Master Data'!$A$28:$D$34,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F33" s="5">
+      <c r="B33" s="85" t="n"/>
+      <c r="C33" s="86" t="n"/>
+      <c r="D33" s="87">
+        <f>IF(B33="","",VLOOKUP(B33,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E33" s="87">
+        <f>IF(B33="","",VLOOKUP(B33,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F33" s="87">
         <f>IF(E33&lt;&gt;"",E33-D33,"")</f>
         <v/>
       </c>
-      <c r="G33" s="5">
+      <c r="G33" s="87">
         <f>IF(B33="","",C33*D33)</f>
         <v/>
       </c>
-      <c r="H33" s="5">
+      <c r="H33" s="87">
         <f>IF(B33="","",C33*E33)</f>
         <v/>
       </c>
-      <c r="I33" s="5">
+      <c r="I33" s="87">
         <f>IF(H33&lt;&gt;"",H33-G33,"")</f>
         <v/>
       </c>
-      <c r="J33" s="5">
-        <f>IF(B33="","",IF(C33&gt;1,(C33-1)*VLOOKUP(B33,'Master Data'!$A$28:$D$34,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J33" s="82" t="n"/>
       <c r="K33" s="50" t="inlineStr"/>
       <c r="L33" s="55" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="33" t="inlineStr">
@@ -3864,21 +3929,11 @@
         <f>SUM(I31:I33)</f>
         <v/>
       </c>
-      <c r="J34" s="8">
-        <f>SUM(J31:J33)</f>
-        <v/>
-      </c>
+      <c r="J34" s="8" t="n"/>
       <c r="K34" s="50" t="inlineStr"/>
       <c r="L34" s="55" t="inlineStr"/>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="K35" t="inlineStr"/>
-      <c r="L35" t="inlineStr"/>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="31" t="inlineStr">
         <is>
@@ -3896,8 +3951,6 @@
       <c r="J36" s="44" t="n"/>
       <c r="K36" s="44" t="n"/>
       <c r="L36" s="45" t="n"/>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37" ht="32.25" customHeight="1" s="42">
       <c r="A37" s="2" t="inlineStr">
@@ -3945,210 +3998,174 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>Replay</t>
-        </is>
-      </c>
+      <c r="J37" s="2" t="n"/>
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr"/>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="n">
+      <c r="A38" s="80" t="n">
         <v>1</v>
       </c>
-      <c r="B38" s="34" t="n"/>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="5">
-        <f>IF(B38="","",VLOOKUP(B38,'Master Data'!$A$38:$D$46,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E38" s="5">
-        <f>IF(B38="","",VLOOKUP(B38,'Master Data'!$A$38:$D$46,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F38" s="5">
+      <c r="B38" s="85" t="n"/>
+      <c r="C38" s="86" t="n"/>
+      <c r="D38" s="87">
+        <f>IF(B38="","",VLOOKUP(B38,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E38" s="87">
+        <f>IF(B38="","",VLOOKUP(B38,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F38" s="87">
         <f>IF(E38&lt;&gt;"",E38-D38,"")</f>
         <v/>
       </c>
-      <c r="G38" s="5">
+      <c r="G38" s="87">
         <f>IF(B38="","",C38*D38)</f>
         <v/>
       </c>
-      <c r="H38" s="5">
+      <c r="H38" s="87">
         <f>IF(B38="","",C38*E38)</f>
         <v/>
       </c>
-      <c r="I38" s="5">
+      <c r="I38" s="87">
         <f>IF(H38&lt;&gt;"",H38-G38,"")</f>
         <v/>
       </c>
-      <c r="J38" s="5">
-        <f>IF(B38="","",IF(C38&gt;1,(C38-1)*VLOOKUP(B38,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K38" t="inlineStr"/>
+      <c r="J38" s="82" t="n"/>
       <c r="L38" s="6" t="inlineStr"/>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="n">
+      <c r="A39" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="B39" s="34" t="n"/>
-      <c r="C39" s="4" t="n"/>
-      <c r="D39" s="5">
-        <f>IF(B39="","",VLOOKUP(B39,'Master Data'!$A$38:$D$46,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E39" s="5">
-        <f>IF(B39="","",VLOOKUP(B39,'Master Data'!$A$38:$D$46,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F39" s="5">
+      <c r="B39" s="85" t="n"/>
+      <c r="C39" s="86" t="n"/>
+      <c r="D39" s="87">
+        <f>IF(B39="","",VLOOKUP(B39,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E39" s="87">
+        <f>IF(B39="","",VLOOKUP(B39,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F39" s="87">
         <f>IF(E39&lt;&gt;"",E39-D39,"")</f>
         <v/>
       </c>
-      <c r="G39" s="5">
+      <c r="G39" s="87">
         <f>IF(B39="","",C39*D39)</f>
         <v/>
       </c>
-      <c r="H39" s="5">
+      <c r="H39" s="87">
         <f>IF(B39="","",C39*E39)</f>
         <v/>
       </c>
-      <c r="I39" s="5">
+      <c r="I39" s="87">
         <f>IF(H39&lt;&gt;"",H39-G39,"")</f>
         <v/>
       </c>
-      <c r="J39" s="5">
-        <f>IF(B39="","",IF(C39&gt;1,(C39-1)*VLOOKUP(B39,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K39" t="inlineStr"/>
+      <c r="J39" s="82" t="n"/>
       <c r="L39" s="6" t="inlineStr"/>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="n">
+      <c r="A40" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="B40" s="34" t="n"/>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="5">
-        <f>IF(B40="","",VLOOKUP(B40,'Master Data'!$A$38:$D$46,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E40" s="5">
-        <f>IF(B40="","",VLOOKUP(B40,'Master Data'!$A$38:$D$46,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F40" s="5">
+      <c r="B40" s="85" t="n"/>
+      <c r="C40" s="86" t="n"/>
+      <c r="D40" s="87">
+        <f>IF(B40="","",VLOOKUP(B40,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E40" s="87">
+        <f>IF(B40="","",VLOOKUP(B40,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F40" s="87">
         <f>IF(E40&lt;&gt;"",E40-D40,"")</f>
         <v/>
       </c>
-      <c r="G40" s="5">
+      <c r="G40" s="87">
         <f>IF(B40="","",C40*D40)</f>
         <v/>
       </c>
-      <c r="H40" s="5">
+      <c r="H40" s="87">
         <f>IF(B40="","",C40*E40)</f>
         <v/>
       </c>
-      <c r="I40" s="5">
+      <c r="I40" s="87">
         <f>IF(H40&lt;&gt;"",H40-G40,"")</f>
         <v/>
       </c>
-      <c r="J40" s="5">
-        <f>IF(B40="","",IF(C40&gt;1,(C40-1)*VLOOKUP(B40,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K40" t="inlineStr"/>
+      <c r="J40" s="82" t="n"/>
       <c r="L40" s="6" t="inlineStr"/>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="n">
+      <c r="A41" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="B41" s="34" t="n"/>
-      <c r="C41" s="4" t="n"/>
-      <c r="D41" s="5">
-        <f>IF(B41="","",VLOOKUP(B41,'Master Data'!$A$38:$D$46,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E41" s="5">
-        <f>IF(B41="","",VLOOKUP(B41,'Master Data'!$A$38:$D$46,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F41" s="5">
+      <c r="B41" s="85" t="n"/>
+      <c r="C41" s="86" t="n"/>
+      <c r="D41" s="87">
+        <f>IF(B41="","",VLOOKUP(B41,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E41" s="87">
+        <f>IF(B41="","",VLOOKUP(B41,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F41" s="87">
         <f>IF(E41&lt;&gt;"",E41-D41,"")</f>
         <v/>
       </c>
-      <c r="G41" s="5">
+      <c r="G41" s="87">
         <f>IF(B41="","",C41*D41)</f>
         <v/>
       </c>
-      <c r="H41" s="5">
+      <c r="H41" s="87">
         <f>IF(B41="","",C41*E41)</f>
         <v/>
       </c>
-      <c r="I41" s="5">
+      <c r="I41" s="87">
         <f>IF(H41&lt;&gt;"",H41-G41,"")</f>
         <v/>
       </c>
-      <c r="J41" s="5">
-        <f>IF(B41="","",IF(C41&gt;1,(C41-1)*VLOOKUP(B41,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K41" t="inlineStr"/>
+      <c r="J41" s="82" t="n"/>
       <c r="L41" s="6" t="inlineStr"/>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="n">
+      <c r="A42" s="80" t="n">
         <v>5</v>
       </c>
-      <c r="B42" s="34" t="n"/>
-      <c r="C42" s="4" t="n"/>
-      <c r="D42" s="5">
-        <f>IF(B42="","",VLOOKUP(B42,'Master Data'!$A$38:$D$46,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E42" s="5">
-        <f>IF(B42="","",VLOOKUP(B42,'Master Data'!$A$38:$D$46,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F42" s="5">
+      <c r="B42" s="85" t="n"/>
+      <c r="C42" s="86" t="n"/>
+      <c r="D42" s="87">
+        <f>IF(B42="","",VLOOKUP(B42,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E42" s="87">
+        <f>IF(B42="","",VLOOKUP(B42,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F42" s="87">
         <f>IF(E42&lt;&gt;"",E42-D42,"")</f>
         <v/>
       </c>
-      <c r="G42" s="5">
+      <c r="G42" s="87">
         <f>IF(B42="","",C42*D42)</f>
         <v/>
       </c>
-      <c r="H42" s="5">
+      <c r="H42" s="87">
         <f>IF(B42="","",C42*E42)</f>
         <v/>
       </c>
-      <c r="I42" s="5">
+      <c r="I42" s="87">
         <f>IF(H42&lt;&gt;"",H42-G42,"")</f>
         <v/>
       </c>
-      <c r="J42" s="5">
-        <f>IF(B42="","",IF(C42&gt;1,(C42-1)*VLOOKUP(B42,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K42" t="inlineStr"/>
+      <c r="J42" s="82" t="n"/>
       <c r="L42" s="6" t="inlineStr"/>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="33" t="inlineStr">
@@ -4173,21 +4190,10 @@
         <f>SUM(I38:I42)</f>
         <v/>
       </c>
-      <c r="J43" s="8">
-        <f>SUM(J38:J42)</f>
-        <v/>
-      </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="J43" s="8" t="n"/>
       <c r="L43" s="6" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="31" t="inlineStr">
         <is>
@@ -4205,8 +4211,6 @@
       <c r="J45" s="44" t="n"/>
       <c r="K45" s="44" t="n"/>
       <c r="L45" s="45" t="n"/>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
     </row>
     <row r="46" ht="32.25" customHeight="1" s="42">
       <c r="A46" s="2" t="inlineStr">
@@ -4254,132 +4258,108 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>Replay</t>
-        </is>
-      </c>
+      <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n">
+      <c r="A47" s="80" t="n">
         <v>1</v>
       </c>
-      <c r="B47" s="34" t="n"/>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="5">
-        <f>IF(B47="","",VLOOKUP(B47,'Master Data'!$A$50:$D$56,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E47" s="5">
-        <f>IF(B47="","",VLOOKUP(B47,'Master Data'!$A$50:$D$56,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F47" s="5">
+      <c r="B47" s="85" t="n"/>
+      <c r="C47" s="86" t="n"/>
+      <c r="D47" s="87">
+        <f>IF(B47="","",VLOOKUP(B47,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E47" s="87">
+        <f>IF(B47="","",VLOOKUP(B47,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F47" s="87">
         <f>IF(E47&lt;&gt;"",E47-D47,"")</f>
         <v/>
       </c>
-      <c r="G47" s="5">
+      <c r="G47" s="87">
         <f>IF(B47="","",C47*D47)</f>
         <v/>
       </c>
-      <c r="H47" s="5">
+      <c r="H47" s="87">
         <f>IF(B47="","",C47*E47)</f>
         <v/>
       </c>
-      <c r="I47" s="5">
+      <c r="I47" s="87">
         <f>IF(H47&lt;&gt;"",H47-G47,"")</f>
         <v/>
       </c>
-      <c r="J47" s="5">
-        <f>IF(B47="","",IF(C47&gt;1,(C47-1)*VLOOKUP(B47,'Master Data'!$A$50:$D$56,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K47" t="inlineStr"/>
+      <c r="J47" s="82" t="n"/>
       <c r="L47" s="6" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="n">
+      <c r="A48" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="B48" s="34" t="n"/>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="5">
-        <f>IF(B48="","",VLOOKUP(B48,'Master Data'!$A$50:$D$56,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E48" s="5">
-        <f>IF(B48="","",VLOOKUP(B48,'Master Data'!$A$50:$D$56,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F48" s="5">
+      <c r="B48" s="85" t="n"/>
+      <c r="C48" s="86" t="n"/>
+      <c r="D48" s="87">
+        <f>IF(B48="","",VLOOKUP(B48,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E48" s="87">
+        <f>IF(B48="","",VLOOKUP(B48,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F48" s="87">
         <f>IF(E48&lt;&gt;"",E48-D48,"")</f>
         <v/>
       </c>
-      <c r="G48" s="5">
+      <c r="G48" s="87">
         <f>IF(B48="","",C48*D48)</f>
         <v/>
       </c>
-      <c r="H48" s="5">
+      <c r="H48" s="87">
         <f>IF(B48="","",C48*E48)</f>
         <v/>
       </c>
-      <c r="I48" s="5">
+      <c r="I48" s="87">
         <f>IF(H48&lt;&gt;"",H48-G48,"")</f>
         <v/>
       </c>
-      <c r="J48" s="5">
-        <f>IF(B48="","",IF(C48&gt;1,(C48-1)*VLOOKUP(B48,'Master Data'!$A$50:$D$56,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K48" t="inlineStr"/>
+      <c r="J48" s="82" t="n"/>
       <c r="L48" s="6" t="inlineStr"/>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="n">
+      <c r="A49" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="B49" s="34" t="n"/>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="5">
-        <f>IF(B49="","",VLOOKUP(B49,'Master Data'!$A$50:$D$56,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E49" s="5">
-        <f>IF(B49="","",VLOOKUP(B49,'Master Data'!$A$50:$D$56,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F49" s="5">
+      <c r="B49" s="85" t="n"/>
+      <c r="C49" s="86" t="n"/>
+      <c r="D49" s="87">
+        <f>IF(B49="","",VLOOKUP(B49,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E49" s="87">
+        <f>IF(B49="","",VLOOKUP(B49,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F49" s="87">
         <f>IF(E49&lt;&gt;"",E49-D49,"")</f>
         <v/>
       </c>
-      <c r="G49" s="5">
+      <c r="G49" s="87">
         <f>IF(B49="","",C49*D49)</f>
         <v/>
       </c>
-      <c r="H49" s="5">
+      <c r="H49" s="87">
         <f>IF(B49="","",C49*E49)</f>
         <v/>
       </c>
-      <c r="I49" s="5">
+      <c r="I49" s="87">
         <f>IF(H49&lt;&gt;"",H49-G49,"")</f>
         <v/>
       </c>
-      <c r="J49" s="5">
-        <f>IF(B49="","",IF(C49&gt;1,(C49-1)*VLOOKUP(B49,'Master Data'!$A$50:$D$56,5,FALSE),0))</f>
-        <v/>
-      </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="J49" s="82" t="n"/>
       <c r="L49" s="6" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="33" t="inlineStr">
@@ -4404,21 +4384,10 @@
         <f>SUM(I47:I49)</f>
         <v/>
       </c>
-      <c r="J50" s="8">
-        <f>SUM(J47:J49)</f>
-        <v/>
-      </c>
-      <c r="K50" t="inlineStr"/>
+      <c r="J50" s="8" t="n"/>
       <c r="L50" s="6" t="inlineStr"/>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="K51" t="inlineStr"/>
-      <c r="L51" t="inlineStr"/>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="48" t="inlineStr">
         <is>
@@ -4489,292 +4458,276 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="47" t="n">
+      <c r="A54" s="80" t="n">
         <v>1</v>
       </c>
-      <c r="B54" s="56" t="n"/>
-      <c r="C54" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D54" s="51">
-        <f>IF(B54="","",VLOOKUP(B54,'Master Data'!$A$86:$D$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E54" s="51">
-        <f>IF(B54="","",VLOOKUP(B54,'Master Data'!$A$86:$D$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F54" s="51">
+      <c r="B54" s="85" t="n"/>
+      <c r="C54" s="86" t="n"/>
+      <c r="D54" s="87">
+        <f>IF(B54="","",VLOOKUP(B54,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E54" s="87">
+        <f>IF(B54="","",VLOOKUP(B54,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F54" s="87">
         <f>IF(E54&lt;&gt;"",E54-D54,"")</f>
         <v/>
       </c>
-      <c r="G54" s="51">
+      <c r="G54" s="87">
         <f>IF(B54="","",C54*D54)</f>
         <v/>
       </c>
-      <c r="H54" s="51">
+      <c r="H54" s="87">
         <f>IF(B54="","",C54*E54)</f>
         <v/>
       </c>
-      <c r="I54" s="51">
+      <c r="I54" s="87">
         <f>IF(H54&lt;&gt;"",H54-G54,"")</f>
         <v/>
       </c>
-      <c r="J54" s="50" t="n"/>
+      <c r="J54" s="85" t="n"/>
       <c r="K54" s="50" t="n"/>
       <c r="L54" s="49" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="47" t="n">
+      <c r="A55" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="B55" s="56" t="n"/>
-      <c r="C55" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" s="51">
-        <f>IF(B55="","",VLOOKUP(B55,'Master Data'!$A$86:$D$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E55" s="51">
-        <f>IF(B55="","",VLOOKUP(B55,'Master Data'!$A$86:$D$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F55" s="51">
+      <c r="B55" s="85" t="n"/>
+      <c r="C55" s="86" t="n"/>
+      <c r="D55" s="87">
+        <f>IF(B55="","",VLOOKUP(B55,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E55" s="87">
+        <f>IF(B55="","",VLOOKUP(B55,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F55" s="87">
         <f>IF(E55&lt;&gt;"",E55-D55,"")</f>
         <v/>
       </c>
-      <c r="G55" s="51">
+      <c r="G55" s="87">
         <f>IF(B55="","",C55*D55)</f>
         <v/>
       </c>
-      <c r="H55" s="51">
+      <c r="H55" s="87">
         <f>IF(B55="","",C55*E55)</f>
         <v/>
       </c>
-      <c r="I55" s="51">
+      <c r="I55" s="87">
         <f>IF(H55&lt;&gt;"",H55-G55,"")</f>
         <v/>
       </c>
-      <c r="J55" s="50" t="n"/>
+      <c r="J55" s="85" t="n"/>
       <c r="K55" s="50" t="n"/>
       <c r="L55" s="49" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="47" t="n">
+      <c r="A56" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="B56" s="56" t="n"/>
-      <c r="C56" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" s="51">
-        <f>IF(B56="","",VLOOKUP(B56,'Master Data'!$A$86:$D$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E56" s="51">
-        <f>IF(B56="","",VLOOKUP(B56,'Master Data'!$A$86:$D$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F56" s="51">
+      <c r="B56" s="85" t="n"/>
+      <c r="C56" s="86" t="n"/>
+      <c r="D56" s="87">
+        <f>IF(B56="","",VLOOKUP(B56,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E56" s="87">
+        <f>IF(B56="","",VLOOKUP(B56,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F56" s="87">
         <f>IF(E56&lt;&gt;"",E56-D56,"")</f>
         <v/>
       </c>
-      <c r="G56" s="51">
+      <c r="G56" s="87">
         <f>IF(B56="","",C56*D56)</f>
         <v/>
       </c>
-      <c r="H56" s="51">
+      <c r="H56" s="87">
         <f>IF(B56="","",C56*E56)</f>
         <v/>
       </c>
-      <c r="I56" s="51">
+      <c r="I56" s="87">
         <f>IF(H56&lt;&gt;"",H56-G56,"")</f>
         <v/>
       </c>
-      <c r="J56" s="50" t="n"/>
+      <c r="J56" s="85" t="n"/>
       <c r="K56" s="50" t="n"/>
       <c r="L56" s="49" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="47" t="n">
+      <c r="A57" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="B57" s="56" t="n"/>
-      <c r="C57" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D57" s="51">
-        <f>IF(B57="","",VLOOKUP(B57,'Master Data'!$A$86:$D$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E57" s="51">
-        <f>IF(B57="","",VLOOKUP(B57,'Master Data'!$A$86:$D$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F57" s="51">
+      <c r="B57" s="85" t="n"/>
+      <c r="C57" s="86" t="n"/>
+      <c r="D57" s="87">
+        <f>IF(B57="","",VLOOKUP(B57,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E57" s="87">
+        <f>IF(B57="","",VLOOKUP(B57,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F57" s="87">
         <f>IF(E57&lt;&gt;"",E57-D57,"")</f>
         <v/>
       </c>
-      <c r="G57" s="51">
+      <c r="G57" s="87">
         <f>IF(B57="","",C57*D57)</f>
         <v/>
       </c>
-      <c r="H57" s="51">
+      <c r="H57" s="87">
         <f>IF(B57="","",C57*E57)</f>
         <v/>
       </c>
-      <c r="I57" s="51">
+      <c r="I57" s="87">
         <f>IF(H57&lt;&gt;"",H57-G57,"")</f>
         <v/>
       </c>
-      <c r="J57" s="50" t="n"/>
+      <c r="J57" s="85" t="n"/>
       <c r="K57" s="50" t="n"/>
       <c r="L57" s="49" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="47" t="n">
+      <c r="A58" s="80" t="n">
         <v>5</v>
       </c>
-      <c r="B58" s="56" t="n"/>
-      <c r="C58" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" s="51">
-        <f>IF(B58="","",VLOOKUP(B58,'Master Data'!$A$86:$D$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E58" s="51">
-        <f>IF(B58="","",VLOOKUP(B58,'Master Data'!$A$86:$D$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F58" s="51">
+      <c r="B58" s="85" t="n"/>
+      <c r="C58" s="86" t="n"/>
+      <c r="D58" s="87">
+        <f>IF(B58="","",VLOOKUP(B58,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E58" s="87">
+        <f>IF(B58="","",VLOOKUP(B58,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F58" s="87">
         <f>IF(E58&lt;&gt;"",E58-D58,"")</f>
         <v/>
       </c>
-      <c r="G58" s="51">
+      <c r="G58" s="87">
         <f>IF(B58="","",C58*D58)</f>
         <v/>
       </c>
-      <c r="H58" s="51">
+      <c r="H58" s="87">
         <f>IF(B58="","",C58*E58)</f>
         <v/>
       </c>
-      <c r="I58" s="51">
+      <c r="I58" s="87">
         <f>IF(H58&lt;&gt;"",H58-G58,"")</f>
         <v/>
       </c>
-      <c r="J58" s="50" t="n"/>
+      <c r="J58" s="85" t="n"/>
       <c r="K58" s="50" t="n"/>
       <c r="L58" s="49" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="47" t="n">
+      <c r="A59" s="80" t="n">
         <v>6</v>
       </c>
-      <c r="B59" s="56" t="n"/>
-      <c r="C59" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" s="51">
-        <f>IF(B59="","",VLOOKUP(B59,'Master Data'!$A$86:$D$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E59" s="51">
-        <f>IF(B59="","",VLOOKUP(B59,'Master Data'!$A$86:$D$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F59" s="51">
+      <c r="B59" s="85" t="n"/>
+      <c r="C59" s="86" t="n"/>
+      <c r="D59" s="87">
+        <f>IF(B59="","",VLOOKUP(B59,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E59" s="87">
+        <f>IF(B59="","",VLOOKUP(B59,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F59" s="87">
         <f>IF(E59&lt;&gt;"",E59-D59,"")</f>
         <v/>
       </c>
-      <c r="G59" s="51">
+      <c r="G59" s="87">
         <f>IF(B59="","",C59*D59)</f>
         <v/>
       </c>
-      <c r="H59" s="51">
+      <c r="H59" s="87">
         <f>IF(B59="","",C59*E59)</f>
         <v/>
       </c>
-      <c r="I59" s="51">
+      <c r="I59" s="87">
         <f>IF(H59&lt;&gt;"",H59-G59,"")</f>
         <v/>
       </c>
-      <c r="J59" s="50" t="n"/>
+      <c r="J59" s="85" t="n"/>
       <c r="K59" s="50" t="n"/>
       <c r="L59" s="49" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="47" t="n">
+      <c r="A60" s="80" t="n">
         <v>7</v>
       </c>
-      <c r="B60" s="56" t="n"/>
-      <c r="C60" s="50" t="n">
+      <c r="B60" s="85" t="n"/>
+      <c r="C60" s="86" t="n">
         <v>1</v>
       </c>
-      <c r="D60" s="51">
-        <f>IF(B60="","",VLOOKUP(B60,'Master Data'!$A$86:$D$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E60" s="51">
-        <f>IF(B60="","",VLOOKUP(B60,'Master Data'!$A$86:$D$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F60" s="51">
+      <c r="D60" s="87">
+        <f>IF(B60="","",VLOOKUP(B60,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E60" s="87">
+        <f>IF(B60="","",VLOOKUP(B60,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F60" s="87">
         <f>IF(E60&lt;&gt;"",E60-D60,"")</f>
         <v/>
       </c>
-      <c r="G60" s="51">
+      <c r="G60" s="87">
         <f>IF(B60="","",C60*D60)</f>
         <v/>
       </c>
-      <c r="H60" s="51">
+      <c r="H60" s="87">
         <f>IF(B60="","",C60*E60)</f>
         <v/>
       </c>
-      <c r="I60" s="51">
+      <c r="I60" s="87">
         <f>IF(H60&lt;&gt;"",H60-G60,"")</f>
         <v/>
       </c>
-      <c r="J60" s="50" t="n"/>
+      <c r="J60" s="85" t="n"/>
       <c r="K60" s="50" t="n"/>
       <c r="L60" s="49" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="47" t="n">
+      <c r="A61" s="80" t="n">
         <v>8</v>
       </c>
-      <c r="B61" s="56" t="n"/>
-      <c r="C61" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="51">
-        <f>IF(B61="","",VLOOKUP(B61,'Master Data'!$A$86:$D$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E61" s="51">
-        <f>IF(B61="","",VLOOKUP(B61,'Master Data'!$A$86:$D$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F61" s="51">
+      <c r="B61" s="85" t="n"/>
+      <c r="C61" s="86" t="n"/>
+      <c r="D61" s="87">
+        <f>IF(B61="","",VLOOKUP(B61,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E61" s="87">
+        <f>IF(B61="","",VLOOKUP(B61,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F61" s="87">
         <f>IF(E61&lt;&gt;"",E61-D61,"")</f>
         <v/>
       </c>
-      <c r="G61" s="51">
+      <c r="G61" s="87">
         <f>IF(B61="","",C61*D61)</f>
         <v/>
       </c>
-      <c r="H61" s="51">
+      <c r="H61" s="87">
         <f>IF(B61="","",C61*E61)</f>
         <v/>
       </c>
-      <c r="I61" s="51">
+      <c r="I61" s="87">
         <f>IF(H61&lt;&gt;"",H61-G61,"")</f>
         <v/>
       </c>
-      <c r="J61" s="50" t="n"/>
-      <c r="K61" s="50" t="n"/>
-      <c r="L61" s="49" t="n"/>
+      <c r="J61" s="85" t="n"/>
     </row>
     <row r="62" ht="16.5" customHeight="1" s="42">
       <c r="A62" s="57" t="inlineStr">
@@ -4782,6 +4735,11 @@
           <t>SUBTOTAL</t>
         </is>
       </c>
+      <c r="B62" s="88" t="n"/>
+      <c r="C62" s="88" t="n"/>
+      <c r="D62" s="88" t="n"/>
+      <c r="E62" s="88" t="n"/>
+      <c r="F62" s="89" t="n"/>
       <c r="G62" s="58">
         <f>SUM(G54:G61)</f>
         <v/>
@@ -4795,7 +4753,6 @@
         <v/>
       </c>
     </row>
-    <row r="63"/>
     <row r="64">
       <c r="A64" s="59" t="inlineStr">
         <is>
@@ -4905,19 +4862,19 @@
           <t>MEALS</t>
         </is>
       </c>
-      <c r="G69" s="47">
+      <c r="G69">
         <f>G43</f>
         <v/>
       </c>
-      <c r="H69" s="47">
+      <c r="H69">
         <f>H43</f>
         <v/>
       </c>
-      <c r="I69" s="47">
+      <c r="I69">
         <f>I43</f>
         <v/>
       </c>
-      <c r="K69" s="60">
+      <c r="K69">
         <f>IF(H69&gt;0,I69/H69,0)</f>
         <v/>
       </c>
@@ -4928,19 +4885,19 @@
           <t>ACTIVITIES</t>
         </is>
       </c>
-      <c r="G70" s="47">
+      <c r="G70">
         <f>G62</f>
         <v/>
       </c>
-      <c r="H70" s="47">
+      <c r="H70">
         <f>H62</f>
         <v/>
       </c>
-      <c r="I70" s="47">
+      <c r="I70">
         <f>I62</f>
         <v/>
       </c>
-      <c r="K70" s="60">
+      <c r="K70">
         <f>IF(H70&gt;0,I70/H70,0)</f>
         <v/>
       </c>
@@ -4974,22 +4931,17 @@
           <t>📌 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="G72" s="62">
-        <f>SUM(G66:G71)</f>
-        <v/>
-      </c>
-      <c r="H72" s="62">
-        <f>SUM(H66:H71)</f>
-        <v/>
-      </c>
-      <c r="I72" s="62">
-        <f>SUM(I66:I71)</f>
-        <v/>
-      </c>
-      <c r="K72" s="63">
-        <f>IF(H72&gt;0,I72/H72,0)</f>
-        <v/>
-      </c>
+      <c r="B72" s="88" t="n"/>
+      <c r="C72" s="88" t="n"/>
+      <c r="D72" s="88" t="n"/>
+      <c r="E72" s="88" t="n"/>
+      <c r="F72" s="88" t="n"/>
+      <c r="G72" s="88" t="n"/>
+      <c r="H72" s="88" t="n"/>
+      <c r="I72" s="88" t="n"/>
+      <c r="J72" s="88" t="n"/>
+      <c r="K72" s="88" t="n"/>
+      <c r="L72" s="89" t="n"/>
     </row>
     <row r="73" ht="30.75" customHeight="1" s="42"/>
     <row r="74" ht="30.75" customHeight="1" s="42">
@@ -5432,7 +5384,6 @@
         </is>
       </c>
     </row>
-    <row r="85"/>
     <row r="86">
       <c r="A86" s="48" t="inlineStr">
         <is>
@@ -5499,65 +5450,123 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
-    <mergeCell ref="A54:F54"/>
+  <mergeCells count="19">
     <mergeCell ref="A7:L7"/>
     <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A50:F50"/>
     <mergeCell ref="A74:L74"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A50:F50"/>
     <mergeCell ref="B5:E5"/>
-    <mergeCell ref="A68"/>
-    <mergeCell ref="A55:F55"/>
-    <mergeCell ref="A57:F57"/>
     <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A62:F62"/>
     <mergeCell ref="A20:F20"/>
     <mergeCell ref="A4:L4"/>
     <mergeCell ref="A43:F43"/>
-    <mergeCell ref="A72:L72"/>
     <mergeCell ref="A29:L29"/>
     <mergeCell ref="A52:L52"/>
+    <mergeCell ref="A72:L72"/>
     <mergeCell ref="A13:L13"/>
-    <mergeCell ref="A58:F58"/>
     <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A59:F59"/>
-    <mergeCell ref="A45:L45"/>
+    <mergeCell ref="A64:L64"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A36:L36"/>
-    <mergeCell ref="A61:L61"/>
-    <mergeCell ref="A70:L70"/>
-    <mergeCell ref="A69:L69"/>
+    <mergeCell ref="A45:L45"/>
   </mergeCells>
-  <dataValidations count="10">
-    <dataValidation sqref="G5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="32">
+    <dataValidation sqref="B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$7:$A$14</formula1>
+    </dataValidation>
+    <dataValidation sqref="B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$7:$A$14</formula1>
+    </dataValidation>
+    <dataValidation sqref="B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$7:$A$14</formula1>
+    </dataValidation>
+    <dataValidation sqref="B18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$7:$A$14</formula1>
+    </dataValidation>
+    <dataValidation sqref="B19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$7:$A$14</formula1>
+    </dataValidation>
+    <dataValidation sqref="B24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$19:$A$24</formula1>
+    </dataValidation>
+    <dataValidation sqref="B25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$19:$A$24</formula1>
+    </dataValidation>
+    <dataValidation sqref="B26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$19:$A$24</formula1>
+    </dataValidation>
+    <dataValidation sqref="K24 K25 K26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>"1인1실, 2인1실, 3인1실, 4인1실"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L24 L25 L26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>"1, 2, 3, 4"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$28:$A$34</formula1>
+    </dataValidation>
+    <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$28:$A$34</formula1>
+    </dataValidation>
+    <dataValidation sqref="B33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$28:$A$34</formula1>
+    </dataValidation>
+    <dataValidation sqref="K31 K32 K33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>"Full-size Van, Mini Van, SUV, Sedan, Limo, Mini Bus (15p), Charter Bus (40p)"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$38:$A$46</formula1>
+    </dataValidation>
+    <dataValidation sqref="B39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$38:$A$46</formula1>
+    </dataValidation>
+    <dataValidation sqref="B40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$38:$A$46</formula1>
+    </dataValidation>
+    <dataValidation sqref="B41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$38:$A$46</formula1>
+    </dataValidation>
+    <dataValidation sqref="B42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$38:$A$46</formula1>
+    </dataValidation>
+    <dataValidation sqref="B47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$50:$A$56</formula1>
+    </dataValidation>
+    <dataValidation sqref="B48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$50:$A$56</formula1>
+    </dataValidation>
+    <dataValidation sqref="B49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$50:$A$56</formula1>
+    </dataValidation>
+    <dataValidation sqref="B54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$86:$A$94</formula1>
+    </dataValidation>
+    <dataValidation sqref="B55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$86:$A$94</formula1>
+    </dataValidation>
+    <dataValidation sqref="B56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$86:$A$94</formula1>
+    </dataValidation>
+    <dataValidation sqref="B57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$86:$A$94</formula1>
+    </dataValidation>
+    <dataValidation sqref="B58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$86:$A$94</formula1>
+    </dataValidation>
+    <dataValidation sqref="B59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$86:$A$94</formula1>
+    </dataValidation>
+    <dataValidation sqref="B60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$86:$A$94</formula1>
+    </dataValidation>
+    <dataValidation sqref="B61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$86:$A$94</formula1>
+    </dataValidation>
+    <dataValidation sqref="G5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
       <formula1>"2,4,6,8"</formula1>
     </dataValidation>
-    <dataValidation sqref="L8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L8 L9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
       <formula1>"First, Business, Premium Economy, Economy"</formula1>
-    </dataValidation>
-    <dataValidation sqref="L9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"First, Business, Premium Economy, Economy"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1인1실, 2인1실, 3인1실, 4인1실"</formula1>
-    </dataValidation>
-    <dataValidation sqref="L24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1, 2, 3, 4"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1인1실, 2인1실, 3인1실, 4인1실"</formula1>
-    </dataValidation>
-    <dataValidation sqref="L25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1, 2, 3, 4"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1인1실, 2인1실, 3인1실, 4인1실"</formula1>
-    </dataValidation>
-    <dataValidation sqref="L26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1, 2, 3, 4"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Full-size Van, Mini Van, SUV, Sedan, Limo, Mini Bus (15p), Charter Bus (40p)"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: complete v3 rebuild - merged headers, dropdowns fixed, blue outlines, replay cleanup, activities link, grand total formulas
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -104,6 +104,8 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -111,8 +113,12 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -175,14 +181,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF1A3450"/>
+        <bgColor rgb="FF1A3450"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1A3450"/>
-        <bgColor rgb="FF1A3450"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -193,12 +205,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFD9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -328,6 +346,50 @@
       </bottom>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color rgb="FF4472C4"/>
       </left>
@@ -341,11 +403,44 @@
         <color rgb="FF4472C4"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF333333"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF333333"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF333333"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF333333"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF333333"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF333333"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -526,60 +621,63 @@
     <xf numFmtId="164" fontId="10" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="13" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="17" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="15" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="17" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="15" fillId="7" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="7" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="16" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="16" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1701,7 +1799,6 @@
       </c>
       <c r="F55" s="6" t="n"/>
     </row>
-    <row r="56"/>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
         <is>
@@ -2610,13 +2707,13 @@
           <t>⛳ 골프</t>
         </is>
       </c>
-      <c r="J4" s="78" t="n"/>
+      <c r="J4" s="92" t="n"/>
       <c r="K4" s="77" t="inlineStr">
         <is>
           <t>🏨 호텔</t>
         </is>
       </c>
-      <c r="L4" s="78" t="n"/>
+      <c r="L4" s="92" t="n"/>
       <c r="M4" s="76" t="inlineStr">
         <is>
           <t>마진</t>
@@ -2629,195 +2726,195 @@
       </c>
     </row>
     <row r="5" ht="51" customHeight="1" s="42">
-      <c r="A5" s="79" t="n"/>
-      <c r="B5" s="79" t="n"/>
-      <c r="C5" s="79" t="n"/>
-      <c r="D5" s="79" t="n"/>
-      <c r="E5" s="79" t="n"/>
-      <c r="F5" s="79" t="n"/>
-      <c r="G5" s="79" t="n"/>
-      <c r="H5" s="79" t="n"/>
-      <c r="I5" s="79" t="inlineStr">
+      <c r="A5" s="78" t="n"/>
+      <c r="B5" s="78" t="n"/>
+      <c r="C5" s="78" t="n"/>
+      <c r="D5" s="78" t="n"/>
+      <c r="E5" s="78" t="n"/>
+      <c r="F5" s="78" t="n"/>
+      <c r="G5" s="78" t="n"/>
+      <c r="H5" s="78" t="n"/>
+      <c r="I5" s="78" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="J5" s="79" t="inlineStr">
+      <c r="J5" s="78" t="inlineStr">
         <is>
           <t>Sell</t>
         </is>
       </c>
-      <c r="K5" s="79" t="inlineStr">
+      <c r="K5" s="78" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="L5" s="79" t="inlineStr">
+      <c r="L5" s="78" t="inlineStr">
         <is>
           <t>Sell</t>
         </is>
       </c>
-      <c r="M5" s="79" t="n"/>
-      <c r="N5" s="79" t="n"/>
+      <c r="M5" s="78" t="n"/>
+      <c r="N5" s="78" t="n"/>
     </row>
     <row r="6" ht="51" customHeight="1" s="42">
-      <c r="A6" s="80" t="n">
+      <c r="A6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="81" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="C6" s="80" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>3N4D</t>
         </is>
       </c>
-      <c r="D6" s="80" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>트럼프 + 샌드파이퍼 오션뷰</t>
         </is>
       </c>
-      <c r="E6" s="80" t="n">
+      <c r="E6" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="80" t="n">
+      <c r="F6" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="G6" s="80" t="n">
+      <c r="G6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="80" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Trump×1 + Sand×1</t>
         </is>
       </c>
-      <c r="I6" s="82" t="n">
+      <c r="I6" s="5" t="n">
         <v>340</v>
       </c>
-      <c r="J6" s="82" t="n">
+      <c r="J6" s="5" t="n">
         <v>745</v>
       </c>
-      <c r="K6" s="82" t="n">
+      <c r="K6" s="5" t="n">
         <v>825</v>
       </c>
-      <c r="L6" s="82" t="n">
+      <c r="L6" s="5" t="n">
         <v>1125</v>
       </c>
-      <c r="M6" s="83">
+      <c r="M6" s="79">
         <f>J6+L6-I6-K6</f>
         <v/>
       </c>
-      <c r="N6" s="84">
+      <c r="N6" s="80">
         <f>IF(J6+L6&gt;0,(J6+L6-I6-K6)/(J6+L6),0)</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="34.5" customHeight="1" s="42">
-      <c r="A7" s="80" t="n">
+      <c r="A7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="81" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="C7" s="80" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>3N4D</t>
         </is>
       </c>
-      <c r="D7" s="80" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>트럼프 + 히든밸리 밸리뷰</t>
         </is>
       </c>
-      <c r="E7" s="80" t="n">
+      <c r="E7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="80" t="n">
+      <c r="F7" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="G7" s="80" t="n">
+      <c r="G7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="80" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Trump×1 + HV×1</t>
         </is>
       </c>
-      <c r="I7" s="82" t="n">
+      <c r="I7" s="5" t="n">
         <v>319</v>
       </c>
-      <c r="J7" s="82" t="n">
+      <c r="J7" s="5" t="n">
         <v>609</v>
       </c>
-      <c r="K7" s="82" t="n">
+      <c r="K7" s="5" t="n">
         <v>825</v>
       </c>
-      <c r="L7" s="82" t="n">
+      <c r="L7" s="5" t="n">
         <v>1125</v>
       </c>
-      <c r="M7" s="83">
+      <c r="M7" s="79">
         <f>J7+L7-I7-K7</f>
         <v/>
       </c>
-      <c r="N7" s="84">
+      <c r="N7" s="80">
         <f>IF(J7+L7&gt;0,(J7+L7-I7-K7)/(J7+L7),0)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="80" t="n">
+      <c r="A8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="81" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="C8" s="80" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>3N4D</t>
         </is>
       </c>
-      <c r="D8" s="80" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>샌드파이퍼 + 히든밸리</t>
         </is>
       </c>
-      <c r="E8" s="80" t="n">
+      <c r="E8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="80" t="n">
+      <c r="F8" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="G8" s="80" t="n">
+      <c r="G8" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H8" s="80" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Sand×1 + HV×1</t>
         </is>
       </c>
-      <c r="I8" s="82" t="n">
+      <c r="I8" s="5" t="n">
         <v>239</v>
       </c>
-      <c r="J8" s="82" t="n">
+      <c r="J8" s="5" t="n">
         <v>354</v>
       </c>
-      <c r="K8" s="82" t="n">
+      <c r="K8" s="5" t="n">
         <v>825</v>
       </c>
-      <c r="L8" s="82" t="n">
+      <c r="L8" s="5" t="n">
         <v>1125</v>
       </c>
-      <c r="M8" s="83">
+      <c r="M8" s="79">
         <f>J8+L8-I8-K8</f>
         <v/>
       </c>
-      <c r="N8" s="84">
+      <c r="N8" s="80">
         <f>IF(J8+L8&gt;0,(J8+L8-I8-K8)/(J8+L8),0)</f>
         <v/>
       </c>
@@ -2839,55 +2936,55 @@
       <c r="N9" s="10" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="80" t="n">
+      <c r="A10" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="81" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>M1</t>
         </is>
       </c>
-      <c r="C10" s="80" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>5N7D</t>
         </is>
       </c>
-      <c r="D10" s="80" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>트럼프+샌드+히든 3色 시그니처</t>
         </is>
       </c>
-      <c r="E10" s="80" t="n">
+      <c r="E10" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="80" t="n">
+      <c r="F10" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="G10" s="80" t="n">
+      <c r="G10" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H10" s="80" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Trump×1+Sand×1+HV×1</t>
         </is>
       </c>
-      <c r="I10" s="82" t="n">
+      <c r="I10" s="5" t="n">
         <v>449</v>
       </c>
-      <c r="J10" s="82" t="n">
+      <c r="J10" s="5" t="n">
         <v>854</v>
       </c>
-      <c r="K10" s="82" t="n">
+      <c r="K10" s="5" t="n">
         <v>1375</v>
       </c>
-      <c r="L10" s="82" t="n">
+      <c r="L10" s="5" t="n">
         <v>1875</v>
       </c>
-      <c r="M10" s="83">
+      <c r="M10" s="79">
         <f>J10+L10-I10-K10</f>
         <v/>
       </c>
-      <c r="N10" s="84">
+      <c r="N10" s="80">
         <f>IF(J10+L10&gt;0,(J10+L10-I10-K10)/(J10+L10),0)</f>
         <v/>
       </c>
@@ -2942,7 +3039,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -2985,7 +3081,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="31" t="inlineStr">
         <is>
@@ -3192,7 +3287,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="31" t="inlineStr">
         <is>
@@ -3266,233 +3360,232 @@
       <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="30.75" customHeight="1" s="42">
-      <c r="A15" s="80" t="n">
+      <c r="A15" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="85" t="inlineStr">
+      <c r="B15" s="82" t="inlineStr">
         <is>
           <t>Trump National LA</t>
         </is>
       </c>
-      <c r="C15" s="86" t="n">
+      <c r="C15" s="83" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="87">
+      <c r="D15" s="84">
         <f>IF(B15="","",VLOOKUP(B15,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E15" s="87">
+      <c r="E15" s="84">
         <f>IF(B15="","",VLOOKUP(B15,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F15" s="87">
+      <c r="F15" s="84">
         <f>IF(E15&lt;&gt;"",E15-D15,"")</f>
         <v/>
       </c>
-      <c r="G15" s="87">
+      <c r="G15" s="84">
         <f>IF(B15="","",C15*D15)</f>
         <v/>
       </c>
-      <c r="H15" s="87">
+      <c r="H15" s="84">
         <f>IF(B15="","",C15*E15)</f>
         <v/>
       </c>
-      <c r="I15" s="87">
+      <c r="I15" s="84">
         <f>IF(H15&lt;&gt;"",H15-G15,"")</f>
         <v/>
       </c>
-      <c r="J15" s="87">
+      <c r="J15" s="84">
         <f>IF(B15="","",IF(C15&gt;1,(C15-1)*VLOOKUP(B15,'Master Data'!$A$7:$E$14,5,FALSE),0))</f>
         <v/>
       </c>
       <c r="L15" s="6" t="inlineStr"/>
     </row>
     <row r="16" ht="30.75" customHeight="1" s="42">
-      <c r="A16" s="80" t="n">
+      <c r="A16" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="B16" s="85" t="inlineStr">
+      <c r="B16" s="82" t="inlineStr">
         <is>
           <t>Sandpiper GC</t>
         </is>
       </c>
-      <c r="C16" s="86" t="n">
+      <c r="C16" s="83" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="87">
+      <c r="D16" s="84">
         <f>IF(B16="","",VLOOKUP(B16,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E16" s="87">
+      <c r="E16" s="84">
         <f>IF(B16="","",VLOOKUP(B16,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F16" s="87">
+      <c r="F16" s="84">
         <f>IF(E16&lt;&gt;"",E16-D16,"")</f>
         <v/>
       </c>
-      <c r="G16" s="87">
+      <c r="G16" s="84">
         <f>IF(B16="","",C16*D16)</f>
         <v/>
       </c>
-      <c r="H16" s="87">
+      <c r="H16" s="84">
         <f>IF(B16="","",C16*E16)</f>
         <v/>
       </c>
-      <c r="I16" s="87">
+      <c r="I16" s="84">
         <f>IF(H16&lt;&gt;"",H16-G16,"")</f>
         <v/>
       </c>
-      <c r="J16" s="87">
+      <c r="J16" s="84">
         <f>IF(B16="","",IF(C16&gt;1,(C16-1)*VLOOKUP(B16,'Master Data'!$A$7:$E$14,5,FALSE),0))</f>
         <v/>
       </c>
       <c r="L16" s="6" t="inlineStr"/>
     </row>
     <row r="17" ht="30.75" customHeight="1" s="42">
-      <c r="A17" s="80" t="n">
+      <c r="A17" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="B17" s="85" t="inlineStr">
+      <c r="B17" s="82" t="inlineStr">
         <is>
           <t>Hidden Valley GC</t>
         </is>
       </c>
-      <c r="C17" s="86" t="n">
+      <c r="C17" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="87">
+      <c r="D17" s="84">
         <f>IF(B17="","",VLOOKUP(B17,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E17" s="87">
+      <c r="E17" s="84">
         <f>IF(B17="","",VLOOKUP(B17,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F17" s="87">
+      <c r="F17" s="84">
         <f>IF(E17&lt;&gt;"",E17-D17,"")</f>
         <v/>
       </c>
-      <c r="G17" s="87">
+      <c r="G17" s="84">
         <f>IF(B17="","",C17*D17)</f>
         <v/>
       </c>
-      <c r="H17" s="87">
+      <c r="H17" s="84">
         <f>IF(B17="","",C17*E17)</f>
         <v/>
       </c>
-      <c r="I17" s="87">
+      <c r="I17" s="84">
         <f>IF(H17&lt;&gt;"",H17-G17,"")</f>
         <v/>
       </c>
-      <c r="J17" s="87">
+      <c r="J17" s="84">
         <f>IF(B17="","",IF(C17&gt;1,(C17-1)*VLOOKUP(B17,'Master Data'!$A$7:$E$14,5,FALSE),0))</f>
         <v/>
       </c>
       <c r="L17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="80" t="n">
+      <c r="A18" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="B18" s="85" t="n"/>
-      <c r="C18" s="86" t="n"/>
-      <c r="D18" s="87">
+      <c r="B18" s="82" t="n"/>
+      <c r="C18" s="83" t="n"/>
+      <c r="D18" s="84">
         <f>IF(B18="","",VLOOKUP(B18,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E18" s="87">
+      <c r="E18" s="84">
         <f>IF(B18="","",VLOOKUP(B18,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F18" s="87">
+      <c r="F18" s="84">
         <f>IF(E18&lt;&gt;"",E18-D18,"")</f>
         <v/>
       </c>
-      <c r="G18" s="87">
+      <c r="G18" s="84">
         <f>IF(B18="","",C18*D18)</f>
         <v/>
       </c>
-      <c r="H18" s="87">
+      <c r="H18" s="84">
         <f>IF(B18="","",C18*E18)</f>
         <v/>
       </c>
-      <c r="I18" s="87">
+      <c r="I18" s="84">
         <f>IF(H18&lt;&gt;"",H18-G18,"")</f>
         <v/>
       </c>
-      <c r="J18" s="87">
+      <c r="J18" s="84">
         <f>IF(B18="","",IF(C18&gt;1,(C18-1)*VLOOKUP(B18,'Master Data'!$A$7:$E$14,5,FALSE),0))</f>
         <v/>
       </c>
       <c r="L18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="80" t="n">
+      <c r="A19" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="B19" s="85" t="n"/>
-      <c r="C19" s="86" t="n"/>
-      <c r="D19" s="87">
+      <c r="B19" s="82" t="n"/>
+      <c r="C19" s="83" t="n"/>
+      <c r="D19" s="84">
         <f>IF(B19="","",VLOOKUP(B19,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E19" s="87">
+      <c r="E19" s="84">
         <f>IF(B19="","",VLOOKUP(B19,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F19" s="87">
+      <c r="F19" s="84">
         <f>IF(E19&lt;&gt;"",E19-D19,"")</f>
         <v/>
       </c>
-      <c r="G19" s="87">
+      <c r="G19" s="84">
         <f>IF(B19="","",C19*D19)</f>
         <v/>
       </c>
-      <c r="H19" s="87">
+      <c r="H19" s="84">
         <f>IF(B19="","",C19*E19)</f>
         <v/>
       </c>
-      <c r="I19" s="87">
+      <c r="I19" s="84">
         <f>IF(H19&lt;&gt;"",H19-G19,"")</f>
         <v/>
       </c>
-      <c r="J19" s="87">
+      <c r="J19" s="84">
         <f>IF(B19="","",IF(C19&gt;1,(C19-1)*VLOOKUP(B19,'Master Data'!$A$7:$E$14,5,FALSE),0))</f>
         <v/>
       </c>
       <c r="L19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="33" t="inlineStr">
+      <c r="A20" s="85" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B20" s="44" t="n"/>
-      <c r="C20" s="44" t="n"/>
-      <c r="D20" s="44" t="n"/>
-      <c r="E20" s="44" t="n"/>
-      <c r="F20" s="45" t="n"/>
-      <c r="G20" s="8">
+      <c r="B20" s="86" t="n"/>
+      <c r="C20" s="86" t="n"/>
+      <c r="D20" s="86" t="n"/>
+      <c r="E20" s="86" t="n"/>
+      <c r="F20" s="87" t="n"/>
+      <c r="G20" s="88">
         <f>SUM(G15:G19)</f>
         <v/>
       </c>
-      <c r="H20" s="8">
+      <c r="H20" s="88">
         <f>SUM(H15:H19)</f>
         <v/>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="88">
         <f>SUM(I15:I19)</f>
         <v/>
       </c>
-      <c r="J20" s="8">
+      <c r="J20" s="88">
         <f>SUM(J15:J19)</f>
         <v/>
       </c>
       <c r="L20" s="6" t="inlineStr"/>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="31" t="inlineStr">
         <is>
@@ -3557,7 +3650,11 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J23" s="2" t="n"/>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Replay</t>
+        </is>
+      </c>
       <c r="K23" s="52" t="inlineStr">
         <is>
           <t>Room Type</t>
@@ -3570,36 +3667,45 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="80" t="n">
+      <c r="A24" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="B24" s="85" t="n"/>
-      <c r="C24" s="86" t="n"/>
-      <c r="D24" s="87">
+      <c r="B24" s="82" t="inlineStr">
+        <is>
+          <t>Beverly Wilshire (5★) / Same Tier</t>
+        </is>
+      </c>
+      <c r="C24" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" s="84">
         <f>IF(B24="","",VLOOKUP(B24,'Master Data'!$A$19:$C$24,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E24" s="87">
+      <c r="E24" s="84">
         <f>IF(B24="","",VLOOKUP(B24,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F24" s="87">
+      <c r="F24" s="84">
         <f>IF(E24&lt;&gt;"",E24-D24,"")</f>
         <v/>
       </c>
-      <c r="G24" s="87">
+      <c r="G24" s="84">
         <f>IF(B24="","",C24*D24)</f>
         <v/>
       </c>
-      <c r="H24" s="87">
+      <c r="H24" s="84">
         <f>IF(B24="","",C24*E24)</f>
         <v/>
       </c>
-      <c r="I24" s="87">
+      <c r="I24" s="84">
         <f>IF(H24&lt;&gt;"",H24-G24,"")</f>
         <v/>
       </c>
-      <c r="J24" s="82" t="n"/>
+      <c r="J24" s="79">
+        <f>IF(B24="","",IF(C24&gt;1,(C24-1)*VLOOKUP(B24,'Master Data'!$A$19:$D$25,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="K24" s="50" t="inlineStr">
         <is>
           <t>2인1실</t>
@@ -3610,36 +3716,39 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="80" t="n">
+      <c r="A25" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="B25" s="85" t="n"/>
-      <c r="C25" s="86" t="n"/>
-      <c r="D25" s="87">
+      <c r="B25" s="82" t="n"/>
+      <c r="C25" s="83" t="n"/>
+      <c r="D25" s="84">
         <f>IF(B25="","",VLOOKUP(B25,'Master Data'!$A$19:$C$24,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E25" s="87">
+      <c r="E25" s="84">
         <f>IF(B25="","",VLOOKUP(B25,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F25" s="87">
+      <c r="F25" s="84">
         <f>IF(E25&lt;&gt;"",E25-D25,"")</f>
         <v/>
       </c>
-      <c r="G25" s="87">
+      <c r="G25" s="84">
         <f>IF(B25="","",C25*D25)</f>
         <v/>
       </c>
-      <c r="H25" s="87">
+      <c r="H25" s="84">
         <f>IF(B25="","",C25*E25)</f>
         <v/>
       </c>
-      <c r="I25" s="87">
+      <c r="I25" s="84">
         <f>IF(H25&lt;&gt;"",H25-G25,"")</f>
         <v/>
       </c>
-      <c r="J25" s="82" t="n"/>
+      <c r="J25" s="79">
+        <f>IF(B25="","",IF(C25&gt;1,(C25-1)*VLOOKUP(B25,'Master Data'!$A$19:$D$25,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="K25" s="50" t="inlineStr">
         <is>
           <t>2인1실</t>
@@ -3650,36 +3759,39 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="80" t="n">
+      <c r="A26" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="B26" s="85" t="n"/>
-      <c r="C26" s="86" t="n"/>
-      <c r="D26" s="87">
+      <c r="B26" s="82" t="n"/>
+      <c r="C26" s="83" t="n"/>
+      <c r="D26" s="84">
         <f>IF(B26="","",VLOOKUP(B26,'Master Data'!$A$19:$C$24,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E26" s="87">
+      <c r="E26" s="84">
         <f>IF(B26="","",VLOOKUP(B26,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F26" s="87">
+      <c r="F26" s="84">
         <f>IF(E26&lt;&gt;"",E26-D26,"")</f>
         <v/>
       </c>
-      <c r="G26" s="87">
+      <c r="G26" s="84">
         <f>IF(B26="","",C26*D26)</f>
         <v/>
       </c>
-      <c r="H26" s="87">
+      <c r="H26" s="84">
         <f>IF(B26="","",C26*E26)</f>
         <v/>
       </c>
-      <c r="I26" s="87">
+      <c r="I26" s="84">
         <f>IF(H26&lt;&gt;"",H26-G26,"")</f>
         <v/>
       </c>
-      <c r="J26" s="82" t="n"/>
+      <c r="J26" s="79">
+        <f>IF(B26="","",IF(C26&gt;1,(C26-1)*VLOOKUP(B26,'Master Data'!$A$19:$D$25,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="K26" s="50" t="inlineStr">
         <is>
           <t>2인1실</t>
@@ -3690,32 +3802,34 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="33" t="inlineStr">
+      <c r="A27" s="85" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B27" s="44" t="n"/>
-      <c r="C27" s="44" t="n"/>
-      <c r="D27" s="44" t="n"/>
-      <c r="E27" s="44" t="n"/>
-      <c r="F27" s="45" t="n"/>
-      <c r="G27" s="8">
+      <c r="B27" s="86" t="n"/>
+      <c r="C27" s="86" t="n"/>
+      <c r="D27" s="86" t="n"/>
+      <c r="E27" s="86" t="n"/>
+      <c r="F27" s="87" t="n"/>
+      <c r="G27" s="88">
         <f>SUM(G24:G26)</f>
         <v/>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="88">
         <f>SUM(H24:H26)</f>
         <v/>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="88">
         <f>SUM(I24:I26)</f>
         <v/>
       </c>
-      <c r="J27" s="8" t="n"/>
+      <c r="J27" s="8">
+        <f>SUM(J24:J26)</f>
+        <v/>
+      </c>
       <c r="L27" s="6" t="inlineStr"/>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="31" t="inlineStr">
         <is>
@@ -3780,7 +3894,11 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J30" s="2" t="n"/>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Replay</t>
+        </is>
+      </c>
       <c r="K30" s="52" t="inlineStr">
         <is>
           <t>Vehicle Type</t>
@@ -3793,40 +3911,45 @@
       </c>
     </row>
     <row r="31" ht="47.25" customHeight="1" s="42">
-      <c r="A31" s="80" t="n">
+      <c r="A31" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="B31" s="85" t="inlineStr">
+      <c r="B31" s="82" t="inlineStr">
         <is>
           <t>Driver/Guide + Van (일당)</t>
         </is>
       </c>
-      <c r="C31" s="86" t="n"/>
-      <c r="D31" s="87">
+      <c r="C31" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="84">
         <f>IF(B31="","",VLOOKUP(B31,'Master Data'!$A$28:$C$34,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E31" s="87">
+      <c r="E31" s="84">
         <f>IF(B31="","",VLOOKUP(B31,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F31" s="87">
+      <c r="F31" s="84">
         <f>IF(E31&lt;&gt;"",E31-D31,"")</f>
         <v/>
       </c>
-      <c r="G31" s="87">
+      <c r="G31" s="84">
         <f>IF(B31="","",C31*D31)</f>
         <v/>
       </c>
-      <c r="H31" s="87">
+      <c r="H31" s="84">
         <f>IF(B31="","",C31*E31)</f>
         <v/>
       </c>
-      <c r="I31" s="87">
+      <c r="I31" s="84">
         <f>IF(H31&lt;&gt;"",H31-G31,"")</f>
         <v/>
       </c>
-      <c r="J31" s="82" t="n"/>
+      <c r="J31" s="79">
+        <f>IF(B31="","",IF(C31&gt;1,(C31-1)*VLOOKUP(B31,'Master Data'!$A$28:$D$34,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="K31" s="50" t="inlineStr">
         <is>
           <t>Full-size Van</t>
@@ -3839,101 +3962,109 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="80" t="n">
+      <c r="A32" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="B32" s="85" t="n"/>
-      <c r="C32" s="86" t="n"/>
-      <c r="D32" s="87">
+      <c r="B32" s="82" t="n"/>
+      <c r="C32" s="83" t="n"/>
+      <c r="D32" s="84">
         <f>IF(B32="","",VLOOKUP(B32,'Master Data'!$A$28:$C$34,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E32" s="87">
+      <c r="E32" s="84">
         <f>IF(B32="","",VLOOKUP(B32,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F32" s="87">
+      <c r="F32" s="84">
         <f>IF(E32&lt;&gt;"",E32-D32,"")</f>
         <v/>
       </c>
-      <c r="G32" s="87">
+      <c r="G32" s="84">
         <f>IF(B32="","",C32*D32)</f>
         <v/>
       </c>
-      <c r="H32" s="87">
+      <c r="H32" s="84">
         <f>IF(B32="","",C32*E32)</f>
         <v/>
       </c>
-      <c r="I32" s="87">
+      <c r="I32" s="84">
         <f>IF(H32&lt;&gt;"",H32-G32,"")</f>
         <v/>
       </c>
-      <c r="J32" s="82" t="n"/>
+      <c r="J32" s="79">
+        <f>IF(B32="","",IF(C32&gt;1,(C32-1)*VLOOKUP(B32,'Master Data'!$A$28:$D$34,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="K32" s="50" t="inlineStr"/>
       <c r="L32" s="55" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="80" t="n">
+      <c r="A33" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="B33" s="85" t="n"/>
-      <c r="C33" s="86" t="n"/>
-      <c r="D33" s="87">
+      <c r="B33" s="82" t="n"/>
+      <c r="C33" s="83" t="n"/>
+      <c r="D33" s="84">
         <f>IF(B33="","",VLOOKUP(B33,'Master Data'!$A$28:$C$34,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E33" s="87">
+      <c r="E33" s="84">
         <f>IF(B33="","",VLOOKUP(B33,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F33" s="87">
+      <c r="F33" s="84">
         <f>IF(E33&lt;&gt;"",E33-D33,"")</f>
         <v/>
       </c>
-      <c r="G33" s="87">
+      <c r="G33" s="84">
         <f>IF(B33="","",C33*D33)</f>
         <v/>
       </c>
-      <c r="H33" s="87">
+      <c r="H33" s="84">
         <f>IF(B33="","",C33*E33)</f>
         <v/>
       </c>
-      <c r="I33" s="87">
+      <c r="I33" s="84">
         <f>IF(H33&lt;&gt;"",H33-G33,"")</f>
         <v/>
       </c>
-      <c r="J33" s="82" t="n"/>
+      <c r="J33" s="79">
+        <f>IF(B33="","",IF(C33&gt;1,(C33-1)*VLOOKUP(B33,'Master Data'!$A$28:$D$34,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="K33" s="50" t="inlineStr"/>
       <c r="L33" s="55" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="33" t="inlineStr">
+      <c r="A34" s="85" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B34" s="44" t="n"/>
-      <c r="C34" s="44" t="n"/>
-      <c r="D34" s="44" t="n"/>
-      <c r="E34" s="44" t="n"/>
-      <c r="F34" s="45" t="n"/>
-      <c r="G34" s="8">
+      <c r="B34" s="86" t="n"/>
+      <c r="C34" s="86" t="n"/>
+      <c r="D34" s="86" t="n"/>
+      <c r="E34" s="86" t="n"/>
+      <c r="F34" s="87" t="n"/>
+      <c r="G34" s="88">
         <f>SUM(G31:G33)</f>
         <v/>
       </c>
-      <c r="H34" s="8">
+      <c r="H34" s="88">
         <f>SUM(H31:H33)</f>
         <v/>
       </c>
-      <c r="I34" s="8">
+      <c r="I34" s="88">
         <f>SUM(I31:I33)</f>
         <v/>
       </c>
-      <c r="J34" s="8" t="n"/>
+      <c r="J34" s="8">
+        <f>SUM(J31:J33)</f>
+        <v/>
+      </c>
       <c r="K34" s="50" t="inlineStr"/>
       <c r="L34" s="55" t="inlineStr"/>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="31" t="inlineStr">
         <is>
@@ -3998,202 +4129,247 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J37" s="2" t="n"/>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Replay</t>
+        </is>
+      </c>
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="80" t="n">
+      <c r="A38" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="B38" s="85" t="n"/>
-      <c r="C38" s="86" t="n"/>
-      <c r="D38" s="87">
+      <c r="B38" s="82" t="inlineStr">
+        <is>
+          <t>Breakfast (Hotel)</t>
+        </is>
+      </c>
+      <c r="C38" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" s="84">
         <f>IF(B38="","",VLOOKUP(B38,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E38" s="87">
+      <c r="E38" s="84">
         <f>IF(B38="","",VLOOKUP(B38,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F38" s="87">
+      <c r="F38" s="84">
         <f>IF(E38&lt;&gt;"",E38-D38,"")</f>
         <v/>
       </c>
-      <c r="G38" s="87">
+      <c r="G38" s="84">
         <f>IF(B38="","",C38*D38)</f>
         <v/>
       </c>
-      <c r="H38" s="87">
+      <c r="H38" s="84">
         <f>IF(B38="","",C38*E38)</f>
         <v/>
       </c>
-      <c r="I38" s="87">
+      <c r="I38" s="84">
         <f>IF(H38&lt;&gt;"",H38-G38,"")</f>
         <v/>
       </c>
-      <c r="J38" s="82" t="n"/>
+      <c r="J38" s="79">
+        <f>IF(B38="","",IF(C38&gt;1,(C38-1)*VLOOKUP(B38,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="80" t="n">
+      <c r="A39" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="B39" s="85" t="n"/>
-      <c r="C39" s="86" t="n"/>
-      <c r="D39" s="87">
+      <c r="B39" s="82" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C39" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="D39" s="84">
         <f>IF(B39="","",VLOOKUP(B39,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E39" s="87">
+      <c r="E39" s="84">
         <f>IF(B39="","",VLOOKUP(B39,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F39" s="87">
+      <c r="F39" s="84">
         <f>IF(E39&lt;&gt;"",E39-D39,"")</f>
         <v/>
       </c>
-      <c r="G39" s="87">
+      <c r="G39" s="84">
         <f>IF(B39="","",C39*D39)</f>
         <v/>
       </c>
-      <c r="H39" s="87">
+      <c r="H39" s="84">
         <f>IF(B39="","",C39*E39)</f>
         <v/>
       </c>
-      <c r="I39" s="87">
+      <c r="I39" s="84">
         <f>IF(H39&lt;&gt;"",H39-G39,"")</f>
         <v/>
       </c>
-      <c r="J39" s="82" t="n"/>
+      <c r="J39" s="79">
+        <f>IF(B39="","",IF(C39&gt;1,(C39-1)*VLOOKUP(B39,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="80" t="n">
+      <c r="A40" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="B40" s="85" t="n"/>
-      <c r="C40" s="86" t="n"/>
-      <c r="D40" s="87">
+      <c r="B40" s="82" t="inlineStr">
+        <is>
+          <t>Dinner (Regular)</t>
+        </is>
+      </c>
+      <c r="C40" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="D40" s="84">
         <f>IF(B40="","",VLOOKUP(B40,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E40" s="87">
+      <c r="E40" s="84">
         <f>IF(B40="","",VLOOKUP(B40,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F40" s="87">
+      <c r="F40" s="84">
         <f>IF(E40&lt;&gt;"",E40-D40,"")</f>
         <v/>
       </c>
-      <c r="G40" s="87">
+      <c r="G40" s="84">
         <f>IF(B40="","",C40*D40)</f>
         <v/>
       </c>
-      <c r="H40" s="87">
+      <c r="H40" s="84">
         <f>IF(B40="","",C40*E40)</f>
         <v/>
       </c>
-      <c r="I40" s="87">
+      <c r="I40" s="84">
         <f>IF(H40&lt;&gt;"",H40-G40,"")</f>
         <v/>
       </c>
-      <c r="J40" s="82" t="n"/>
+      <c r="J40" s="79">
+        <f>IF(B40="","",IF(C40&gt;1,(C40-1)*VLOOKUP(B40,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="80" t="n">
+      <c r="A41" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="B41" s="85" t="n"/>
-      <c r="C41" s="86" t="n"/>
-      <c r="D41" s="87">
+      <c r="B41" s="82" t="inlineStr">
+        <is>
+          <t>Exclusive Dinner (Michelin/Fine)</t>
+        </is>
+      </c>
+      <c r="C41" s="83" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" s="84">
         <f>IF(B41="","",VLOOKUP(B41,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E41" s="87">
+      <c r="E41" s="84">
         <f>IF(B41="","",VLOOKUP(B41,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F41" s="87">
+      <c r="F41" s="84">
         <f>IF(E41&lt;&gt;"",E41-D41,"")</f>
         <v/>
       </c>
-      <c r="G41" s="87">
+      <c r="G41" s="84">
         <f>IF(B41="","",C41*D41)</f>
         <v/>
       </c>
-      <c r="H41" s="87">
+      <c r="H41" s="84">
         <f>IF(B41="","",C41*E41)</f>
         <v/>
       </c>
-      <c r="I41" s="87">
+      <c r="I41" s="84">
         <f>IF(H41&lt;&gt;"",H41-G41,"")</f>
         <v/>
       </c>
-      <c r="J41" s="82" t="n"/>
+      <c r="J41" s="79">
+        <f>IF(B41="","",IF(C41&gt;1,(C41-1)*VLOOKUP(B41,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="80" t="n">
+      <c r="A42" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="B42" s="85" t="n"/>
-      <c r="C42" s="86" t="n"/>
-      <c r="D42" s="87">
+      <c r="B42" s="82" t="n"/>
+      <c r="C42" s="83" t="n"/>
+      <c r="D42" s="84">
         <f>IF(B42="","",VLOOKUP(B42,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E42" s="87">
+      <c r="E42" s="84">
         <f>IF(B42="","",VLOOKUP(B42,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F42" s="87">
+      <c r="F42" s="84">
         <f>IF(E42&lt;&gt;"",E42-D42,"")</f>
         <v/>
       </c>
-      <c r="G42" s="87">
+      <c r="G42" s="84">
         <f>IF(B42="","",C42*D42)</f>
         <v/>
       </c>
-      <c r="H42" s="87">
+      <c r="H42" s="84">
         <f>IF(B42="","",C42*E42)</f>
         <v/>
       </c>
-      <c r="I42" s="87">
+      <c r="I42" s="84">
         <f>IF(H42&lt;&gt;"",H42-G42,"")</f>
         <v/>
       </c>
-      <c r="J42" s="82" t="n"/>
+      <c r="J42" s="79">
+        <f>IF(B42="","",IF(C42&gt;1,(C42-1)*VLOOKUP(B42,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="33" t="inlineStr">
+      <c r="A43" s="85" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B43" s="44" t="n"/>
-      <c r="C43" s="44" t="n"/>
-      <c r="D43" s="44" t="n"/>
-      <c r="E43" s="44" t="n"/>
-      <c r="F43" s="45" t="n"/>
-      <c r="G43" s="8">
+      <c r="B43" s="86" t="n"/>
+      <c r="C43" s="86" t="n"/>
+      <c r="D43" s="86" t="n"/>
+      <c r="E43" s="86" t="n"/>
+      <c r="F43" s="87" t="n"/>
+      <c r="G43" s="88">
         <f>SUM(G38:G42)</f>
         <v/>
       </c>
-      <c r="H43" s="8">
+      <c r="H43" s="88">
         <f>SUM(H38:H42)</f>
         <v/>
       </c>
-      <c r="I43" s="8">
+      <c r="I43" s="88">
         <f>SUM(I38:I42)</f>
         <v/>
       </c>
-      <c r="J43" s="8" t="n"/>
+      <c r="J43" s="8">
+        <f>SUM(J38:J42)</f>
+        <v/>
+      </c>
       <c r="L43" s="6" t="inlineStr"/>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="31" t="inlineStr">
         <is>
@@ -4258,136 +4434,157 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J46" s="2" t="n"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Replay</t>
+        </is>
+      </c>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="80" t="n">
+      <c r="A47" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="B47" s="85" t="n"/>
-      <c r="C47" s="86" t="n"/>
-      <c r="D47" s="87">
+      <c r="B47" s="82" t="inlineStr">
+        <is>
+          <t>Insurance / Tips / Contingency</t>
+        </is>
+      </c>
+      <c r="C47" s="83" t="n">
+        <v>4</v>
+      </c>
+      <c r="D47" s="84">
         <f>IF(B47="","",VLOOKUP(B47,'Master Data'!$A$50:$C$56,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E47" s="87">
+      <c r="E47" s="84">
         <f>IF(B47="","",VLOOKUP(B47,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F47" s="87">
+      <c r="F47" s="84">
         <f>IF(E47&lt;&gt;"",E47-D47,"")</f>
         <v/>
       </c>
-      <c r="G47" s="87">
+      <c r="G47" s="84">
         <f>IF(B47="","",C47*D47)</f>
         <v/>
       </c>
-      <c r="H47" s="87">
+      <c r="H47" s="84">
         <f>IF(B47="","",C47*E47)</f>
         <v/>
       </c>
-      <c r="I47" s="87">
+      <c r="I47" s="84">
         <f>IF(H47&lt;&gt;"",H47-G47,"")</f>
         <v/>
       </c>
-      <c r="J47" s="82" t="n"/>
+      <c r="J47" s="79">
+        <f>IF(B47="","",IF(C47&gt;1,(C47-1)*VLOOKUP(B47,'Master Data'!$A$50:$D$56,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L47" s="6" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="80" t="n">
+      <c r="A48" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="B48" s="85" t="n"/>
-      <c r="C48" s="86" t="n"/>
-      <c r="D48" s="87">
+      <c r="B48" s="82" t="n"/>
+      <c r="C48" s="83" t="n"/>
+      <c r="D48" s="84">
         <f>IF(B48="","",VLOOKUP(B48,'Master Data'!$A$50:$C$56,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E48" s="87">
+      <c r="E48" s="84">
         <f>IF(B48="","",VLOOKUP(B48,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F48" s="87">
+      <c r="F48" s="84">
         <f>IF(E48&lt;&gt;"",E48-D48,"")</f>
         <v/>
       </c>
-      <c r="G48" s="87">
+      <c r="G48" s="84">
         <f>IF(B48="","",C48*D48)</f>
         <v/>
       </c>
-      <c r="H48" s="87">
+      <c r="H48" s="84">
         <f>IF(B48="","",C48*E48)</f>
         <v/>
       </c>
-      <c r="I48" s="87">
+      <c r="I48" s="84">
         <f>IF(H48&lt;&gt;"",H48-G48,"")</f>
         <v/>
       </c>
-      <c r="J48" s="82" t="n"/>
+      <c r="J48" s="79">
+        <f>IF(B48="","",IF(C48&gt;1,(C48-1)*VLOOKUP(B48,'Master Data'!$A$50:$D$56,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L48" s="6" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="80" t="n">
+      <c r="A49" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="B49" s="85" t="n"/>
-      <c r="C49" s="86" t="n"/>
-      <c r="D49" s="87">
+      <c r="B49" s="82" t="n"/>
+      <c r="C49" s="83" t="n"/>
+      <c r="D49" s="84">
         <f>IF(B49="","",VLOOKUP(B49,'Master Data'!$A$50:$C$56,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E49" s="87">
+      <c r="E49" s="84">
         <f>IF(B49="","",VLOOKUP(B49,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F49" s="87">
+      <c r="F49" s="84">
         <f>IF(E49&lt;&gt;"",E49-D49,"")</f>
         <v/>
       </c>
-      <c r="G49" s="87">
+      <c r="G49" s="84">
         <f>IF(B49="","",C49*D49)</f>
         <v/>
       </c>
-      <c r="H49" s="87">
+      <c r="H49" s="84">
         <f>IF(B49="","",C49*E49)</f>
         <v/>
       </c>
-      <c r="I49" s="87">
+      <c r="I49" s="84">
         <f>IF(H49&lt;&gt;"",H49-G49,"")</f>
         <v/>
       </c>
-      <c r="J49" s="82" t="n"/>
+      <c r="J49" s="79">
+        <f>IF(B49="","",IF(C49&gt;1,(C49-1)*VLOOKUP(B49,'Master Data'!$A$50:$D$56,5,FALSE),0))</f>
+        <v/>
+      </c>
       <c r="L49" s="6" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="33" t="inlineStr">
+      <c r="A50" s="85" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B50" s="44" t="n"/>
-      <c r="C50" s="44" t="n"/>
-      <c r="D50" s="44" t="n"/>
-      <c r="E50" s="44" t="n"/>
-      <c r="F50" s="45" t="n"/>
-      <c r="G50" s="8">
+      <c r="B50" s="86" t="n"/>
+      <c r="C50" s="86" t="n"/>
+      <c r="D50" s="86" t="n"/>
+      <c r="E50" s="86" t="n"/>
+      <c r="F50" s="87" t="n"/>
+      <c r="G50" s="88">
         <f>SUM(G47:G49)</f>
         <v/>
       </c>
-      <c r="H50" s="8">
+      <c r="H50" s="88">
         <f>SUM(H47:H49)</f>
         <v/>
       </c>
-      <c r="I50" s="8">
+      <c r="I50" s="88">
         <f>SUM(I47:I49)</f>
         <v/>
       </c>
-      <c r="J50" s="8" t="n"/>
+      <c r="J50" s="8">
+        <f>SUM(J47:J49)</f>
+        <v/>
+      </c>
       <c r="L50" s="6" t="inlineStr"/>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="A52" s="48" t="inlineStr">
         <is>
@@ -4458,297 +4655,309 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="80" t="n">
+      <c r="A54" s="81" t="n">
         <v>1</v>
       </c>
-      <c r="B54" s="85" t="n"/>
-      <c r="C54" s="86" t="n"/>
-      <c r="D54" s="87">
+      <c r="B54" s="82" t="inlineStr">
+        <is>
+          <t>NBA/MLB Game (Ticket)</t>
+        </is>
+      </c>
+      <c r="C54" s="83" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="84">
         <f>IF(B54="","",VLOOKUP(B54,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E54" s="87">
+      <c r="E54" s="84">
         <f>IF(B54="","",VLOOKUP(B54,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F54" s="87">
+      <c r="F54" s="84">
         <f>IF(E54&lt;&gt;"",E54-D54,"")</f>
         <v/>
       </c>
-      <c r="G54" s="87">
+      <c r="G54" s="84">
         <f>IF(B54="","",C54*D54)</f>
         <v/>
       </c>
-      <c r="H54" s="87">
+      <c r="H54" s="84">
         <f>IF(B54="","",C54*E54)</f>
         <v/>
       </c>
-      <c r="I54" s="87">
+      <c r="I54" s="84">
         <f>IF(H54&lt;&gt;"",H54-G54,"")</f>
         <v/>
       </c>
-      <c r="J54" s="85" t="n"/>
+      <c r="J54" s="81" t="n"/>
       <c r="K54" s="50" t="n"/>
       <c r="L54" s="49" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="80" t="n">
+      <c r="A55" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="B55" s="85" t="n"/>
-      <c r="C55" s="86" t="n"/>
-      <c r="D55" s="87">
+      <c r="B55" s="82" t="inlineStr">
+        <is>
+          <t>Sports Bar Experience</t>
+        </is>
+      </c>
+      <c r="C55" s="83" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" s="84">
         <f>IF(B55="","",VLOOKUP(B55,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E55" s="87">
+      <c r="E55" s="84">
         <f>IF(B55="","",VLOOKUP(B55,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F55" s="87">
+      <c r="F55" s="84">
         <f>IF(E55&lt;&gt;"",E55-D55,"")</f>
         <v/>
       </c>
-      <c r="G55" s="87">
+      <c r="G55" s="84">
         <f>IF(B55="","",C55*D55)</f>
         <v/>
       </c>
-      <c r="H55" s="87">
+      <c r="H55" s="84">
         <f>IF(B55="","",C55*E55)</f>
         <v/>
       </c>
-      <c r="I55" s="87">
+      <c r="I55" s="84">
         <f>IF(H55&lt;&gt;"",H55-G55,"")</f>
         <v/>
       </c>
-      <c r="J55" s="85" t="n"/>
+      <c r="J55" s="81" t="n"/>
       <c r="K55" s="50" t="n"/>
       <c r="L55" s="49" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="80" t="n">
+      <c r="A56" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="B56" s="85" t="n"/>
-      <c r="C56" s="86" t="n"/>
-      <c r="D56" s="87">
+      <c r="B56" s="82" t="n"/>
+      <c r="C56" s="83" t="n"/>
+      <c r="D56" s="84">
         <f>IF(B56="","",VLOOKUP(B56,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E56" s="87">
+      <c r="E56" s="84">
         <f>IF(B56="","",VLOOKUP(B56,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F56" s="87">
+      <c r="F56" s="84">
         <f>IF(E56&lt;&gt;"",E56-D56,"")</f>
         <v/>
       </c>
-      <c r="G56" s="87">
+      <c r="G56" s="84">
         <f>IF(B56="","",C56*D56)</f>
         <v/>
       </c>
-      <c r="H56" s="87">
+      <c r="H56" s="84">
         <f>IF(B56="","",C56*E56)</f>
         <v/>
       </c>
-      <c r="I56" s="87">
+      <c r="I56" s="84">
         <f>IF(H56&lt;&gt;"",H56-G56,"")</f>
         <v/>
       </c>
-      <c r="J56" s="85" t="n"/>
+      <c r="J56" s="81" t="n"/>
       <c r="K56" s="50" t="n"/>
       <c r="L56" s="49" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="80" t="n">
+      <c r="A57" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="B57" s="85" t="n"/>
-      <c r="C57" s="86" t="n"/>
-      <c r="D57" s="87">
+      <c r="B57" s="82" t="n"/>
+      <c r="C57" s="83" t="n"/>
+      <c r="D57" s="84">
         <f>IF(B57="","",VLOOKUP(B57,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E57" s="87">
+      <c r="E57" s="84">
         <f>IF(B57="","",VLOOKUP(B57,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F57" s="87">
+      <c r="F57" s="84">
         <f>IF(E57&lt;&gt;"",E57-D57,"")</f>
         <v/>
       </c>
-      <c r="G57" s="87">
+      <c r="G57" s="84">
         <f>IF(B57="","",C57*D57)</f>
         <v/>
       </c>
-      <c r="H57" s="87">
+      <c r="H57" s="84">
         <f>IF(B57="","",C57*E57)</f>
         <v/>
       </c>
-      <c r="I57" s="87">
+      <c r="I57" s="84">
         <f>IF(H57&lt;&gt;"",H57-G57,"")</f>
         <v/>
       </c>
-      <c r="J57" s="85" t="n"/>
+      <c r="J57" s="81" t="n"/>
       <c r="K57" s="50" t="n"/>
       <c r="L57" s="49" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="80" t="n">
+      <c r="A58" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="B58" s="85" t="n"/>
-      <c r="C58" s="86" t="n"/>
-      <c r="D58" s="87">
+      <c r="B58" s="82" t="n"/>
+      <c r="C58" s="83" t="n"/>
+      <c r="D58" s="84">
         <f>IF(B58="","",VLOOKUP(B58,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E58" s="87">
+      <c r="E58" s="84">
         <f>IF(B58="","",VLOOKUP(B58,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F58" s="87">
+      <c r="F58" s="84">
         <f>IF(E58&lt;&gt;"",E58-D58,"")</f>
         <v/>
       </c>
-      <c r="G58" s="87">
+      <c r="G58" s="84">
         <f>IF(B58="","",C58*D58)</f>
         <v/>
       </c>
-      <c r="H58" s="87">
+      <c r="H58" s="84">
         <f>IF(B58="","",C58*E58)</f>
         <v/>
       </c>
-      <c r="I58" s="87">
+      <c r="I58" s="84">
         <f>IF(H58&lt;&gt;"",H58-G58,"")</f>
         <v/>
       </c>
-      <c r="J58" s="85" t="n"/>
+      <c r="J58" s="81" t="n"/>
       <c r="K58" s="50" t="n"/>
       <c r="L58" s="49" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="80" t="n">
+      <c r="A59" s="81" t="n">
         <v>6</v>
       </c>
-      <c r="B59" s="85" t="n"/>
-      <c r="C59" s="86" t="n"/>
-      <c r="D59" s="87">
+      <c r="B59" s="82" t="n"/>
+      <c r="C59" s="83" t="n"/>
+      <c r="D59" s="84">
         <f>IF(B59="","",VLOOKUP(B59,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E59" s="87">
+      <c r="E59" s="84">
         <f>IF(B59="","",VLOOKUP(B59,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F59" s="87">
+      <c r="F59" s="84">
         <f>IF(E59&lt;&gt;"",E59-D59,"")</f>
         <v/>
       </c>
-      <c r="G59" s="87">
+      <c r="G59" s="84">
         <f>IF(B59="","",C59*D59)</f>
         <v/>
       </c>
-      <c r="H59" s="87">
+      <c r="H59" s="84">
         <f>IF(B59="","",C59*E59)</f>
         <v/>
       </c>
-      <c r="I59" s="87">
+      <c r="I59" s="84">
         <f>IF(H59&lt;&gt;"",H59-G59,"")</f>
         <v/>
       </c>
-      <c r="J59" s="85" t="n"/>
+      <c r="J59" s="81" t="n"/>
       <c r="K59" s="50" t="n"/>
       <c r="L59" s="49" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="80" t="n">
+      <c r="A60" s="81" t="n">
         <v>7</v>
       </c>
-      <c r="B60" s="85" t="n"/>
-      <c r="C60" s="86" t="n">
+      <c r="B60" s="82" t="n"/>
+      <c r="C60" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="D60" s="87">
+      <c r="D60" s="84">
         <f>IF(B60="","",VLOOKUP(B60,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E60" s="87">
+      <c r="E60" s="84">
         <f>IF(B60="","",VLOOKUP(B60,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F60" s="87">
+      <c r="F60" s="84">
         <f>IF(E60&lt;&gt;"",E60-D60,"")</f>
         <v/>
       </c>
-      <c r="G60" s="87">
+      <c r="G60" s="84">
         <f>IF(B60="","",C60*D60)</f>
         <v/>
       </c>
-      <c r="H60" s="87">
+      <c r="H60" s="84">
         <f>IF(B60="","",C60*E60)</f>
         <v/>
       </c>
-      <c r="I60" s="87">
+      <c r="I60" s="84">
         <f>IF(H60&lt;&gt;"",H60-G60,"")</f>
         <v/>
       </c>
-      <c r="J60" s="85" t="n"/>
+      <c r="J60" s="81" t="n"/>
       <c r="K60" s="50" t="n"/>
       <c r="L60" s="49" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="80" t="n">
+      <c r="A61" s="81" t="n">
         <v>8</v>
       </c>
-      <c r="B61" s="85" t="n"/>
-      <c r="C61" s="86" t="n"/>
-      <c r="D61" s="87">
+      <c r="B61" s="82" t="n"/>
+      <c r="C61" s="83" t="n"/>
+      <c r="D61" s="84">
         <f>IF(B61="","",VLOOKUP(B61,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
-      <c r="E61" s="87">
+      <c r="E61" s="84">
         <f>IF(B61="","",VLOOKUP(B61,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="F61" s="87">
+      <c r="F61" s="84">
         <f>IF(E61&lt;&gt;"",E61-D61,"")</f>
         <v/>
       </c>
-      <c r="G61" s="87">
+      <c r="G61" s="84">
         <f>IF(B61="","",C61*D61)</f>
         <v/>
       </c>
-      <c r="H61" s="87">
+      <c r="H61" s="84">
         <f>IF(B61="","",C61*E61)</f>
         <v/>
       </c>
-      <c r="I61" s="87">
+      <c r="I61" s="84">
         <f>IF(H61&lt;&gt;"",H61-G61,"")</f>
         <v/>
       </c>
-      <c r="J61" s="85" t="n"/>
+      <c r="J61" s="81" t="n"/>
     </row>
     <row r="62" ht="16.5" customHeight="1" s="42">
-      <c r="A62" s="57" t="inlineStr">
+      <c r="A62" s="85" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B62" s="88" t="n"/>
-      <c r="C62" s="88" t="n"/>
-      <c r="D62" s="88" t="n"/>
-      <c r="E62" s="88" t="n"/>
-      <c r="F62" s="89" t="n"/>
-      <c r="G62" s="58">
+      <c r="B62" s="86" t="n"/>
+      <c r="C62" s="86" t="n"/>
+      <c r="D62" s="86" t="n"/>
+      <c r="E62" s="86" t="n"/>
+      <c r="F62" s="87" t="n"/>
+      <c r="G62" s="88">
         <f>SUM(G54:G61)</f>
         <v/>
       </c>
-      <c r="H62" s="58">
+      <c r="H62" s="88">
         <f>SUM(H54:H61)</f>
         <v/>
       </c>
-      <c r="I62" s="58">
+      <c r="I62" s="88">
         <f>SUM(I54:I61)</f>
         <v/>
       </c>
@@ -4862,19 +5071,19 @@
           <t>MEALS</t>
         </is>
       </c>
-      <c r="G69">
+      <c r="G69" s="88">
         <f>G43</f>
         <v/>
       </c>
-      <c r="H69">
+      <c r="H69" s="88">
         <f>H43</f>
         <v/>
       </c>
-      <c r="I69">
+      <c r="I69" s="88">
         <f>I43</f>
         <v/>
       </c>
-      <c r="K69">
+      <c r="K69" s="91">
         <f>IF(H69&gt;0,I69/H69,0)</f>
         <v/>
       </c>
@@ -4931,17 +5140,27 @@
           <t>📌 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B72" s="88" t="n"/>
-      <c r="C72" s="88" t="n"/>
-      <c r="D72" s="88" t="n"/>
-      <c r="E72" s="88" t="n"/>
-      <c r="F72" s="88" t="n"/>
-      <c r="G72" s="88" t="n"/>
-      <c r="H72" s="88" t="n"/>
-      <c r="I72" s="88" t="n"/>
-      <c r="J72" s="88" t="n"/>
-      <c r="K72" s="88" t="n"/>
-      <c r="L72" s="89" t="n"/>
+      <c r="B72" s="89" t="n"/>
+      <c r="C72" s="89" t="n"/>
+      <c r="D72" s="89" t="n"/>
+      <c r="E72" s="89" t="n"/>
+      <c r="F72" s="90" t="n"/>
+      <c r="G72" s="88">
+        <f>SUM(G66:G71)</f>
+        <v/>
+      </c>
+      <c r="H72" s="88">
+        <f>SUM(H66:H71)</f>
+        <v/>
+      </c>
+      <c r="I72" s="88">
+        <f>SUM(I66:I71)</f>
+        <v/>
+      </c>
+      <c r="K72" s="91">
+        <f>IF(H72&gt;0,I72/H72,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="73" ht="30.75" customHeight="1" s="42"/>
     <row r="74" ht="30.75" customHeight="1" s="42">
@@ -5453,119 +5672,56 @@
   <mergeCells count="19">
     <mergeCell ref="A7:L7"/>
     <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A74:L74"/>
     <mergeCell ref="A50:F50"/>
-    <mergeCell ref="A74:L74"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="A22:L22"/>
     <mergeCell ref="A62:F62"/>
     <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A72:F72"/>
     <mergeCell ref="A4:L4"/>
     <mergeCell ref="A43:F43"/>
     <mergeCell ref="A29:L29"/>
     <mergeCell ref="A52:L52"/>
-    <mergeCell ref="A72:L72"/>
     <mergeCell ref="A13:L13"/>
     <mergeCell ref="A34:F34"/>
     <mergeCell ref="A64:L64"/>
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A45:L45"/>
     <mergeCell ref="A36:L36"/>
-    <mergeCell ref="A45:L45"/>
   </mergeCells>
-  <dataValidations count="32">
-    <dataValidation sqref="B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+  <dataValidations count="11">
+    <dataValidation sqref="B15 B16 B17 B18 B19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
       <formula1>'Master Data'!$A$7:$A$14</formula1>
     </dataValidation>
-    <dataValidation sqref="B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$7:$A$14</formula1>
-    </dataValidation>
-    <dataValidation sqref="B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$7:$A$14</formula1>
-    </dataValidation>
-    <dataValidation sqref="B18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$7:$A$14</formula1>
-    </dataValidation>
-    <dataValidation sqref="B19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$7:$A$14</formula1>
-    </dataValidation>
-    <dataValidation sqref="B24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+    <dataValidation sqref="B24 B25 B26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
       <formula1>'Master Data'!$A$19:$A$24</formula1>
     </dataValidation>
-    <dataValidation sqref="B25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$19:$A$24</formula1>
-    </dataValidation>
-    <dataValidation sqref="B26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$19:$A$24</formula1>
-    </dataValidation>
-    <dataValidation sqref="K24 K25 K26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+    <dataValidation sqref="K24 K25 K26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"1인1실, 2인1실, 3인1실, 4인1실"</formula1>
     </dataValidation>
-    <dataValidation sqref="L24 L25 L26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+    <dataValidation sqref="L24 L25 L26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"1, 2, 3, 4"</formula1>
     </dataValidation>
-    <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+    <dataValidation sqref="B31 B32 B33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
       <formula1>'Master Data'!$A$28:$A$34</formula1>
     </dataValidation>
-    <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$28:$A$34</formula1>
-    </dataValidation>
-    <dataValidation sqref="B33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$28:$A$34</formula1>
-    </dataValidation>
-    <dataValidation sqref="K31 K32 K33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+    <dataValidation sqref="K31 K32 K33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Full-size Van, Mini Van, SUV, Sedan, Limo, Mini Bus (15p), Charter Bus (40p)"</formula1>
     </dataValidation>
-    <dataValidation sqref="B38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+    <dataValidation sqref="B38 B39 B40 B41 B42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
       <formula1>'Master Data'!$A$38:$A$46</formula1>
     </dataValidation>
-    <dataValidation sqref="B39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$38:$A$46</formula1>
-    </dataValidation>
-    <dataValidation sqref="B40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$38:$A$46</formula1>
-    </dataValidation>
-    <dataValidation sqref="B41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$38:$A$46</formula1>
-    </dataValidation>
-    <dataValidation sqref="B42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$38:$A$46</formula1>
-    </dataValidation>
-    <dataValidation sqref="B47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+    <dataValidation sqref="B47 B48 B49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
       <formula1>'Master Data'!$A$50:$A$56</formula1>
     </dataValidation>
-    <dataValidation sqref="B48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$50:$A$56</formula1>
-    </dataValidation>
-    <dataValidation sqref="B49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$50:$A$56</formula1>
-    </dataValidation>
-    <dataValidation sqref="B54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+    <dataValidation sqref="B54 B55 B56 B57 B58 B59 B60 B61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
       <formula1>'Master Data'!$A$86:$A$94</formula1>
     </dataValidation>
-    <dataValidation sqref="B55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$86:$A$94</formula1>
-    </dataValidation>
-    <dataValidation sqref="B56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$86:$A$94</formula1>
-    </dataValidation>
-    <dataValidation sqref="B57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$86:$A$94</formula1>
-    </dataValidation>
-    <dataValidation sqref="B58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$86:$A$94</formula1>
-    </dataValidation>
-    <dataValidation sqref="B59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$86:$A$94</formula1>
-    </dataValidation>
-    <dataValidation sqref="B60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$86:$A$94</formula1>
-    </dataValidation>
-    <dataValidation sqref="B61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
-      <formula1>'Master Data'!$A$86:$A$94</formula1>
-    </dataValidation>
-    <dataValidation sqref="G5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+    <dataValidation sqref="G5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"2,4,6,8"</formula1>
     </dataValidation>
-    <dataValidation sqref="L8 L9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="입력 오류" error="올바른 항목을 선택하세요" type="list">
+    <dataValidation sqref="L8 L9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"First, Business, Premium Economy, Economy"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5854,19 +6010,19 @@
         <v/>
       </c>
       <c r="E11" s="22">
-        <f>IF(C10&gt;0,D10/C10,0)</f>
+        <f>IF(C11&gt;0,D11/C11,0)</f>
         <v/>
       </c>
       <c r="F11" s="5">
-        <f>IF('Package Selector'!G5&gt;0,B10/'Package Selector'!G5,0)</f>
+        <f>IF('Package Selector'!G5&gt;0,B11/'Package Selector'!G5,0)</f>
         <v/>
       </c>
       <c r="G11" s="5">
-        <f>IF('Package Selector'!G5&gt;0,C10/'Package Selector'!G5,0)</f>
+        <f>IF('Package Selector'!G5&gt;0,C11/'Package Selector'!G5,0)</f>
         <v/>
       </c>
       <c r="H11" s="5">
-        <f>IF('Package Selector'!G5&gt;0,D10/'Package Selector'!G5,0)</f>
+        <f>IF('Package Selector'!G5&gt;0,D11/'Package Selector'!G5,0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: clear replay from non-golf sections, add qty dropdowns 1-20, add golf replay columns to Package Types
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -118,7 +118,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -213,6 +213,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4B183"/>
+        <bgColor rgb="FFF4B183"/>
       </patternFill>
     </fill>
   </fills>
@@ -440,7 +446,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -678,6 +684,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2629,7 +2643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="42" min="1" max="1"/>
@@ -2661,6 +2675,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="16.5" customHeight="1" s="42">
       <c r="A4" s="76" t="inlineStr">
         <is>
@@ -2708,18 +2723,24 @@
         </is>
       </c>
       <c r="J4" s="92" t="n"/>
-      <c r="K4" s="77" t="inlineStr">
+      <c r="K4" s="93" t="inlineStr">
+        <is>
+          <t>🔄 리플레이</t>
+        </is>
+      </c>
+      <c r="L4" s="94" t="n"/>
+      <c r="M4" s="77" t="inlineStr">
         <is>
           <t>🏨 호텔</t>
         </is>
       </c>
-      <c r="L4" s="92" t="n"/>
-      <c r="M4" s="76" t="inlineStr">
+      <c r="N4" s="95" t="n"/>
+      <c r="O4" s="76" t="inlineStr">
         <is>
           <t>마진</t>
         </is>
       </c>
-      <c r="N4" s="76" t="inlineStr">
+      <c r="P4" s="76" t="inlineStr">
         <is>
           <t>마진율</t>
         </is>
@@ -2744,18 +2765,28 @@
           <t>Sell</t>
         </is>
       </c>
-      <c r="K5" s="78" t="inlineStr">
+      <c r="K5" s="96" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="L5" s="78" t="inlineStr">
+      <c r="L5" s="96" t="inlineStr">
         <is>
           <t>Sell</t>
         </is>
       </c>
-      <c r="M5" s="78" t="n"/>
-      <c r="N5" s="78" t="n"/>
+      <c r="M5" s="78" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="N5" s="78" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="O5" s="78" t="n"/>
+      <c r="P5" s="78" t="n"/>
     </row>
     <row r="6" ht="51" customHeight="1" s="42">
       <c r="A6" s="6" t="n">
@@ -2796,18 +2827,24 @@
       <c r="J6" s="5" t="n">
         <v>745</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="K6" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="79" t="n">
+        <v>120</v>
+      </c>
+      <c r="M6" s="5" t="n">
         <v>825</v>
       </c>
-      <c r="L6" s="5" t="n">
+      <c r="N6" s="5" t="n">
         <v>1125</v>
       </c>
-      <c r="M6" s="79">
-        <f>J6+L6-I6-K6</f>
-        <v/>
-      </c>
-      <c r="N6" s="80">
-        <f>IF(J6+L6&gt;0,(J6+L6-I6-K6)/(J6+L6),0)</f>
+      <c r="O6" s="79">
+        <f>(J6+L6+N6)-(I6+K6+M6)</f>
+        <v/>
+      </c>
+      <c r="P6" s="80">
+        <f>IF(J6+L6+N6&gt;0,(J6+L6+N6-I6-K6-M6)/(J6+L6+N6),0)</f>
         <v/>
       </c>
     </row>
@@ -2850,18 +2887,24 @@
       <c r="J7" s="5" t="n">
         <v>609</v>
       </c>
-      <c r="K7" s="5" t="n">
+      <c r="K7" s="79" t="n">
+        <v>45</v>
+      </c>
+      <c r="L7" s="79" t="n">
+        <v>45</v>
+      </c>
+      <c r="M7" s="5" t="n">
         <v>825</v>
       </c>
-      <c r="L7" s="5" t="n">
+      <c r="N7" s="5" t="n">
         <v>1125</v>
       </c>
-      <c r="M7" s="79">
-        <f>J7+L7-I7-K7</f>
-        <v/>
-      </c>
-      <c r="N7" s="80">
-        <f>IF(J7+L7&gt;0,(J7+L7-I7-K7)/(J7+L7),0)</f>
+      <c r="O7" s="79">
+        <f>(J7+L7+N7)-(I7+K7+M7)</f>
+        <v/>
+      </c>
+      <c r="P7" s="80">
+        <f>IF(J7+L7+N7&gt;0,(J7+L7+N7-I7-K7-M7)/(J7+L7+N7),0)</f>
         <v/>
       </c>
     </row>
@@ -2904,18 +2947,24 @@
       <c r="J8" s="5" t="n">
         <v>354</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="K8" s="79" t="n">
+        <v>45</v>
+      </c>
+      <c r="L8" s="79" t="n">
+        <v>45</v>
+      </c>
+      <c r="M8" s="5" t="n">
         <v>825</v>
       </c>
-      <c r="L8" s="5" t="n">
+      <c r="N8" s="5" t="n">
         <v>1125</v>
       </c>
-      <c r="M8" s="79">
-        <f>J8+L8-I8-K8</f>
-        <v/>
-      </c>
-      <c r="N8" s="80">
-        <f>IF(J8+L8&gt;0,(J8+L8-I8-K8)/(J8+L8),0)</f>
+      <c r="O8" s="79">
+        <f>(J8+L8+N8)-(I8+K8+M8)</f>
+        <v/>
+      </c>
+      <c r="P8" s="80">
+        <f>IF(J8+L8+N8&gt;0,(J8+L8+N8-I8-K8-M8)/(J8+L8+N8),0)</f>
         <v/>
       </c>
     </row>
@@ -2930,10 +2979,10 @@
       <c r="H9" s="10" t="n"/>
       <c r="I9" s="10" t="n"/>
       <c r="J9" s="10" t="n"/>
-      <c r="K9" s="10" t="n"/>
-      <c r="L9" s="10" t="n"/>
       <c r="M9" s="10" t="n"/>
       <c r="N9" s="10" t="n"/>
+      <c r="O9" s="10" t="n"/>
+      <c r="P9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
@@ -2974,25 +3023,33 @@
       <c r="J10" s="5" t="n">
         <v>854</v>
       </c>
-      <c r="K10" s="5" t="n">
+      <c r="K10" s="79" t="n">
+        <v>45</v>
+      </c>
+      <c r="L10" s="79" t="n">
+        <v>165</v>
+      </c>
+      <c r="M10" s="5" t="n">
         <v>1375</v>
       </c>
-      <c r="L10" s="5" t="n">
+      <c r="N10" s="5" t="n">
         <v>1875</v>
       </c>
-      <c r="M10" s="79">
-        <f>J10+L10-I10-K10</f>
-        <v/>
-      </c>
-      <c r="N10" s="80">
-        <f>IF(J10+L10&gt;0,(J10+L10-I10-K10)/(J10+L10),0)</f>
+      <c r="O10" s="79">
+        <f>(J10+L10+N10)-(I10+K10+M10)</f>
+        <v/>
+      </c>
+      <c r="P10" s="80">
+        <f>IF(J10+L10+N10&gt;0,(J10+L10+N10-I10-K10-M10)/(J10+L10+N10),0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="A1:P1"/>
     <mergeCell ref="K4:L4"/>
-    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3650,11 +3707,7 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Replay</t>
-        </is>
-      </c>
+      <c r="J23" s="2" t="n"/>
       <c r="K23" s="52" t="inlineStr">
         <is>
           <t>Room Type</t>
@@ -3702,10 +3755,7 @@
         <f>IF(H24&lt;&gt;"",H24-G24,"")</f>
         <v/>
       </c>
-      <c r="J24" s="79">
-        <f>IF(B24="","",IF(C24&gt;1,(C24-1)*VLOOKUP(B24,'Master Data'!$A$19:$D$25,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J24" s="79" t="n"/>
       <c r="K24" s="50" t="inlineStr">
         <is>
           <t>2인1실</t>
@@ -3745,10 +3795,7 @@
         <f>IF(H25&lt;&gt;"",H25-G25,"")</f>
         <v/>
       </c>
-      <c r="J25" s="79">
-        <f>IF(B25="","",IF(C25&gt;1,(C25-1)*VLOOKUP(B25,'Master Data'!$A$19:$D$25,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J25" s="79" t="n"/>
       <c r="K25" s="50" t="inlineStr">
         <is>
           <t>2인1실</t>
@@ -3788,10 +3835,7 @@
         <f>IF(H26&lt;&gt;"",H26-G26,"")</f>
         <v/>
       </c>
-      <c r="J26" s="79">
-        <f>IF(B26="","",IF(C26&gt;1,(C26-1)*VLOOKUP(B26,'Master Data'!$A$19:$D$25,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J26" s="79" t="n"/>
       <c r="K26" s="50" t="inlineStr">
         <is>
           <t>2인1실</t>
@@ -3824,10 +3868,7 @@
         <f>SUM(I24:I26)</f>
         <v/>
       </c>
-      <c r="J27" s="8">
-        <f>SUM(J24:J26)</f>
-        <v/>
-      </c>
+      <c r="J27" s="8" t="n"/>
       <c r="L27" s="6" t="inlineStr"/>
     </row>
     <row r="29">
@@ -3894,11 +3935,7 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>Replay</t>
-        </is>
-      </c>
+      <c r="J30" s="2" t="n"/>
       <c r="K30" s="52" t="inlineStr">
         <is>
           <t>Vehicle Type</t>
@@ -3946,10 +3983,7 @@
         <f>IF(H31&lt;&gt;"",H31-G31,"")</f>
         <v/>
       </c>
-      <c r="J31" s="79">
-        <f>IF(B31="","",IF(C31&gt;1,(C31-1)*VLOOKUP(B31,'Master Data'!$A$28:$D$34,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J31" s="79" t="n"/>
       <c r="K31" s="50" t="inlineStr">
         <is>
           <t>Full-size Van</t>
@@ -3991,10 +4025,7 @@
         <f>IF(H32&lt;&gt;"",H32-G32,"")</f>
         <v/>
       </c>
-      <c r="J32" s="79">
-        <f>IF(B32="","",IF(C32&gt;1,(C32-1)*VLOOKUP(B32,'Master Data'!$A$28:$D$34,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J32" s="79" t="n"/>
       <c r="K32" s="50" t="inlineStr"/>
       <c r="L32" s="55" t="inlineStr"/>
     </row>
@@ -4028,10 +4059,7 @@
         <f>IF(H33&lt;&gt;"",H33-G33,"")</f>
         <v/>
       </c>
-      <c r="J33" s="79">
-        <f>IF(B33="","",IF(C33&gt;1,(C33-1)*VLOOKUP(B33,'Master Data'!$A$28:$D$34,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J33" s="79" t="n"/>
       <c r="K33" s="50" t="inlineStr"/>
       <c r="L33" s="55" t="inlineStr"/>
     </row>
@@ -4058,10 +4086,7 @@
         <f>SUM(I31:I33)</f>
         <v/>
       </c>
-      <c r="J34" s="8">
-        <f>SUM(J31:J33)</f>
-        <v/>
-      </c>
+      <c r="J34" s="8" t="n"/>
       <c r="K34" s="50" t="inlineStr"/>
       <c r="L34" s="55" t="inlineStr"/>
     </row>
@@ -4129,11 +4154,7 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>Replay</t>
-        </is>
-      </c>
+      <c r="J37" s="2" t="n"/>
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr"/>
     </row>
@@ -4173,10 +4194,7 @@
         <f>IF(H38&lt;&gt;"",H38-G38,"")</f>
         <v/>
       </c>
-      <c r="J38" s="79">
-        <f>IF(B38="","",IF(C38&gt;1,(C38-1)*VLOOKUP(B38,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J38" s="79" t="n"/>
       <c r="L38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
@@ -4215,10 +4233,7 @@
         <f>IF(H39&lt;&gt;"",H39-G39,"")</f>
         <v/>
       </c>
-      <c r="J39" s="79">
-        <f>IF(B39="","",IF(C39&gt;1,(C39-1)*VLOOKUP(B39,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J39" s="79" t="n"/>
       <c r="L39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
@@ -4257,10 +4272,7 @@
         <f>IF(H40&lt;&gt;"",H40-G40,"")</f>
         <v/>
       </c>
-      <c r="J40" s="79">
-        <f>IF(B40="","",IF(C40&gt;1,(C40-1)*VLOOKUP(B40,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J40" s="79" t="n"/>
       <c r="L40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
@@ -4299,10 +4311,7 @@
         <f>IF(H41&lt;&gt;"",H41-G41,"")</f>
         <v/>
       </c>
-      <c r="J41" s="79">
-        <f>IF(B41="","",IF(C41&gt;1,(C41-1)*VLOOKUP(B41,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J41" s="79" t="n"/>
       <c r="L41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
@@ -4335,10 +4344,7 @@
         <f>IF(H42&lt;&gt;"",H42-G42,"")</f>
         <v/>
       </c>
-      <c r="J42" s="79">
-        <f>IF(B42="","",IF(C42&gt;1,(C42-1)*VLOOKUP(B42,'Master Data'!$A$38:$D$46,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J42" s="79" t="n"/>
       <c r="L42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
@@ -4364,10 +4370,7 @@
         <f>SUM(I38:I42)</f>
         <v/>
       </c>
-      <c r="J43" s="8">
-        <f>SUM(J38:J42)</f>
-        <v/>
-      </c>
+      <c r="J43" s="8" t="n"/>
       <c r="L43" s="6" t="inlineStr"/>
     </row>
     <row r="45">
@@ -4434,11 +4437,7 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>Replay</t>
-        </is>
-      </c>
+      <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
     </row>
@@ -4478,10 +4477,7 @@
         <f>IF(H47&lt;&gt;"",H47-G47,"")</f>
         <v/>
       </c>
-      <c r="J47" s="79">
-        <f>IF(B47="","",IF(C47&gt;1,(C47-1)*VLOOKUP(B47,'Master Data'!$A$50:$D$56,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J47" s="79" t="n"/>
       <c r="L47" s="6" t="inlineStr"/>
     </row>
     <row r="48">
@@ -4514,10 +4510,7 @@
         <f>IF(H48&lt;&gt;"",H48-G48,"")</f>
         <v/>
       </c>
-      <c r="J48" s="79">
-        <f>IF(B48="","",IF(C48&gt;1,(C48-1)*VLOOKUP(B48,'Master Data'!$A$50:$D$56,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J48" s="79" t="n"/>
       <c r="L48" s="6" t="inlineStr"/>
     </row>
     <row r="49">
@@ -4550,10 +4543,7 @@
         <f>IF(H49&lt;&gt;"",H49-G49,"")</f>
         <v/>
       </c>
-      <c r="J49" s="79">
-        <f>IF(B49="","",IF(C49&gt;1,(C49-1)*VLOOKUP(B49,'Master Data'!$A$50:$D$56,5,FALSE),0))</f>
-        <v/>
-      </c>
+      <c r="J49" s="79" t="n"/>
       <c r="L49" s="6" t="inlineStr"/>
     </row>
     <row r="50">
@@ -4579,10 +4569,7 @@
         <f>SUM(I47:I49)</f>
         <v/>
       </c>
-      <c r="J50" s="8">
-        <f>SUM(J47:J49)</f>
-        <v/>
-      </c>
+      <c r="J50" s="8" t="n"/>
       <c r="L50" s="6" t="inlineStr"/>
     </row>
     <row r="52">
@@ -5690,7 +5677,7 @@
     <mergeCell ref="A45:L45"/>
     <mergeCell ref="A36:L36"/>
   </mergeCells>
-  <dataValidations count="11">
+  <dataValidations count="12">
     <dataValidation sqref="B15 B16 B17 B18 B19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
       <formula1>'Master Data'!$A$7:$A$14</formula1>
     </dataValidation>
@@ -5724,6 +5711,9 @@
     <dataValidation sqref="L8 L9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"First, Business, Premium Economy, Economy"</formula1>
     </dataValidation>
+    <dataValidation sqref="C15 C16 C17 C18 C19 C24 C25 C26 C31 C32 C33 C38 C39 C40 C41 C42 C47 C48 C49 C54 C55 C56 C57 C58 C59 C60 C61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="1-20 사이 값을 선택하세요" type="list">
+      <formula1>"1,2,3,4,5,6,7,8,9,10,11,12,13,14,15,16,17,18,19,20"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: visual cleanup - remove duplicate merges, fix header fills, add missing sub-headers
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -446,7 +446,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -690,6 +690,18 @@
     <xf numFmtId="0" fontId="0" fillId="18" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="18" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2675,7 +2687,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="16.5" customHeight="1" s="42">
       <c r="A4" s="76" t="inlineStr">
         <is>
@@ -2728,13 +2739,13 @@
           <t>🔄 리플레이</t>
         </is>
       </c>
-      <c r="L4" s="94" t="n"/>
+      <c r="L4" s="92" t="n"/>
       <c r="M4" s="77" t="inlineStr">
         <is>
           <t>🏨 호텔</t>
         </is>
       </c>
-      <c r="N4" s="95" t="n"/>
+      <c r="N4" s="92" t="n"/>
       <c r="O4" s="76" t="inlineStr">
         <is>
           <t>마진</t>
@@ -2785,8 +2796,16 @@
           <t>Sell</t>
         </is>
       </c>
-      <c r="O5" s="78" t="n"/>
-      <c r="P5" s="78" t="n"/>
+      <c r="O5" s="76" t="inlineStr">
+        <is>
+          <t>마진</t>
+        </is>
+      </c>
+      <c r="P5" s="76" t="inlineStr">
+        <is>
+          <t>마진율</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="51" customHeight="1" s="42">
       <c r="A6" s="6" t="n">
@@ -3045,12 +3064,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="I4:J4"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3707,13 +3725,13 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J23" s="2" t="n"/>
-      <c r="K23" s="52" t="inlineStr">
+      <c r="J23" s="97" t="n"/>
+      <c r="K23" s="98" t="inlineStr">
         <is>
           <t>Room Type</t>
         </is>
       </c>
-      <c r="L23" s="53" t="inlineStr">
+      <c r="L23" s="98" t="inlineStr">
         <is>
           <t>Beds/Room</t>
         </is>
@@ -3868,7 +3886,7 @@
         <f>SUM(I24:I26)</f>
         <v/>
       </c>
-      <c r="J27" s="8" t="n"/>
+      <c r="J27" s="99" t="n"/>
       <c r="L27" s="6" t="inlineStr"/>
     </row>
     <row r="29">
@@ -3935,13 +3953,13 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J30" s="2" t="n"/>
-      <c r="K30" s="52" t="inlineStr">
+      <c r="J30" s="97" t="n"/>
+      <c r="K30" s="98" t="inlineStr">
         <is>
           <t>Vehicle Type</t>
         </is>
       </c>
-      <c r="L30" s="53" t="inlineStr">
+      <c r="L30" s="98" t="inlineStr">
         <is>
           <t>Pax Capacity</t>
         </is>
@@ -4086,7 +4104,7 @@
         <f>SUM(I31:I33)</f>
         <v/>
       </c>
-      <c r="J34" s="8" t="n"/>
+      <c r="J34" s="99" t="n"/>
       <c r="K34" s="50" t="inlineStr"/>
       <c r="L34" s="55" t="inlineStr"/>
     </row>
@@ -4154,7 +4172,7 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J37" s="2" t="n"/>
+      <c r="J37" s="100" t="n"/>
       <c r="K37" s="2" t="inlineStr"/>
       <c r="L37" s="2" t="inlineStr"/>
     </row>
@@ -4370,7 +4388,7 @@
         <f>SUM(I38:I42)</f>
         <v/>
       </c>
-      <c r="J43" s="8" t="n"/>
+      <c r="J43" s="99" t="n"/>
       <c r="L43" s="6" t="inlineStr"/>
     </row>
     <row r="45">
@@ -4437,7 +4455,7 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J46" s="2" t="n"/>
+      <c r="J46" s="100" t="n"/>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
     </row>
@@ -4569,7 +4587,7 @@
         <f>SUM(I47:I49)</f>
         <v/>
       </c>
-      <c r="J50" s="8" t="n"/>
+      <c r="J50" s="99" t="n"/>
       <c r="L50" s="6" t="inlineStr"/>
     </row>
     <row r="52">
@@ -4625,17 +4643,17 @@
           <t>Total Margin</t>
         </is>
       </c>
-      <c r="J53" s="52" t="inlineStr">
+      <c r="J53" s="98" t="inlineStr">
         <is>
           <t>Per Group</t>
         </is>
       </c>
-      <c r="K53" s="52" t="inlineStr">
+      <c r="K53" s="98" t="inlineStr">
         <is>
           <t>Group Size</t>
         </is>
       </c>
-      <c r="L53" s="52" t="inlineStr">
+      <c r="L53" s="98" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>

</xml_diff>

<commit_message>
feat: v4 - Master Data sub-categories, Package Selector 2 (activity checkmarks), Profit Summary 2, error-proof features
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -10,6 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Types" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Selector" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profit Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Selector 2" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profit Summary 2" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -23,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -117,8 +119,19 @@
       <name val="Calibri"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -221,8 +234,26 @@
         <bgColor rgb="FFF4B183"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F0FE"/>
+        <bgColor rgb="FFE8F0FE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="21">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -442,11 +473,66 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF333333"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF333333"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF4472C4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF4472C4"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF4472C4"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF4472C4"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF4472C4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF4472C4"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF4472C4"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF4472C4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="139">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -704,10 +790,141 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="16" fillId="21" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="19" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="20" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="20" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="20" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -1099,82 +1316,80 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    새 코스·호텔·편명 추가는 빈칸에 직접 입력 → 자동으로 드롭다운에 반영</t>
-        </is>
-      </c>
+      <c r="A3" s="98" t="inlineStr"/>
+      <c r="B3" s="98" t="inlineStr">
+        <is>
+          <t>Cost ($)</t>
+        </is>
+      </c>
+      <c r="C3" s="98" t="inlineStr">
+        <is>
+          <t>Sell ($)</t>
+        </is>
+      </c>
+      <c r="D3" s="98" t="inlineStr">
+        <is>
+          <t>Margin ($)</t>
+        </is>
+      </c>
+      <c r="E3" s="98" t="inlineStr">
+        <is>
+          <t>+Info</t>
+        </is>
+      </c>
+      <c r="F3" s="98" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G3" s="98" t="inlineStr"/>
+      <c r="H3" s="98" t="inlineStr"/>
+      <c r="I3" s="98" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="31" t="inlineStr">
+      <c r="A5" s="101" t="inlineStr">
         <is>
           <t>⛳ GOLF COURSES (1인 1라운드, USD)</t>
         </is>
       </c>
-      <c r="B5" s="44" t="n"/>
-      <c r="C5" s="44" t="n"/>
-      <c r="D5" s="44" t="n"/>
-      <c r="E5" s="44" t="n"/>
-      <c r="F5" s="44" t="n"/>
-      <c r="G5" s="45" t="n"/>
+      <c r="B5" s="102" t="n"/>
+      <c r="C5" s="102" t="n"/>
+      <c r="D5" s="102" t="n"/>
+      <c r="E5" s="102" t="n"/>
+      <c r="F5" s="102" t="n"/>
+      <c r="G5" s="102" t="n"/>
+      <c r="H5" s="102" t="n"/>
+      <c r="I5" s="102" t="n"/>
     </row>
     <row r="6" ht="30.75" customHeight="1" s="42">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Course</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Cost ($)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sell ($)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Margin ($)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Replay Rate ($)</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="n"/>
+      <c r="A6" s="103" t="inlineStr">
+        <is>
+          <t>↳</t>
+        </is>
+      </c>
+      <c r="B6" s="104" t="n"/>
+      <c r="C6" s="104" t="n"/>
+      <c r="D6" s="104" t="n"/>
+      <c r="E6" s="104" t="n"/>
+      <c r="F6" s="104" t="n"/>
+      <c r="G6" s="104" t="n"/>
+      <c r="H6" s="105" t="n"/>
+      <c r="I6" s="105" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="70" t="inlineStr">
-        <is>
-          <t>Trump National LA</t>
-        </is>
-      </c>
-      <c r="B7" s="71" t="n">
-        <v>210</v>
-      </c>
-      <c r="C7" s="71" t="n">
-        <v>210</v>
-      </c>
-      <c r="D7" s="5">
-        <f>IF(A7="","",C7-B7)</f>
-        <v/>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>111</v>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Member guest | Cart incl. | Replay ~50%</t>
-        </is>
-      </c>
+      <c r="A7" s="106" t="inlineStr">
+        <is>
+          <t>🏆 PREMIUM COURSES</t>
+        </is>
+      </c>
+      <c r="B7" s="107" t="n"/>
+      <c r="C7" s="107" t="n"/>
+      <c r="D7" s="107" t="n"/>
+      <c r="E7" s="107" t="n"/>
+      <c r="F7" s="107" t="n"/>
+      <c r="G7" s="107" t="n"/>
+      <c r="H7" s="107" t="n"/>
+      <c r="I7" s="107" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="70" t="inlineStr">
@@ -1249,15 +1464,19 @@
       <c r="F11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="40" t="n"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="5">
-        <f>IF(A12="","",C12-B12)</f>
-        <v/>
-      </c>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="6" t="n"/>
+      <c r="A12" s="106" t="inlineStr">
+        <is>
+          <t>📋 ADDITIONAL COURSES (추가 가능)</t>
+        </is>
+      </c>
+      <c r="B12" s="107" t="n"/>
+      <c r="C12" s="107" t="n"/>
+      <c r="D12" s="107" t="n"/>
+      <c r="E12" s="107" t="n"/>
+      <c r="F12" s="107" t="n"/>
+      <c r="G12" s="107" t="n"/>
+      <c r="H12" s="107" t="n"/>
+      <c r="I12" s="107" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="40" t="n"/>
@@ -1282,46 +1501,34 @@
       <c r="F14" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="31" t="inlineStr">
-        <is>
-          <t>🏨 HOTEL (1인 1박, Double Occupancy, USD)</t>
-        </is>
-      </c>
-      <c r="B17" s="44" t="n"/>
-      <c r="C17" s="44" t="n"/>
-      <c r="D17" s="44" t="n"/>
-      <c r="E17" s="44" t="n"/>
-      <c r="F17" s="44" t="n"/>
-      <c r="G17" s="45" t="n"/>
+      <c r="A17" s="101" t="inlineStr">
+        <is>
+          <t>🏨 HOTELS (1인 1박, Double Occ., USD)</t>
+        </is>
+      </c>
+      <c r="B17" s="102" t="n"/>
+      <c r="C17" s="102" t="n"/>
+      <c r="D17" s="102" t="n"/>
+      <c r="E17" s="102" t="n"/>
+      <c r="F17" s="102" t="n"/>
+      <c r="G17" s="102" t="n"/>
+      <c r="H17" s="102" t="n"/>
+      <c r="I17" s="102" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Hotel</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Cost/night</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Sell/night</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Margin</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="n"/>
+      <c r="A18" s="103" t="inlineStr">
+        <is>
+          <t>↳</t>
+        </is>
+      </c>
+      <c r="B18" s="104" t="n"/>
+      <c r="C18" s="104" t="n"/>
+      <c r="D18" s="104" t="n"/>
+      <c r="E18" s="104" t="n"/>
+      <c r="F18" s="104" t="n"/>
+      <c r="G18" s="104" t="n"/>
+      <c r="H18" s="105" t="n"/>
+      <c r="I18" s="105" t="n"/>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="42">
       <c r="A19" s="70" t="inlineStr">
@@ -1396,46 +1603,34 @@
       <c r="F24" s="6" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="31" t="inlineStr">
-        <is>
-          <t>🚐 TRANSPORT (1인 기준, 4인 1조, USD)</t>
-        </is>
-      </c>
-      <c r="B26" s="44" t="n"/>
-      <c r="C26" s="44" t="n"/>
-      <c r="D26" s="44" t="n"/>
-      <c r="E26" s="44" t="n"/>
-      <c r="F26" s="44" t="n"/>
-      <c r="G26" s="45" t="n"/>
+      <c r="A26" s="101" t="inlineStr">
+        <is>
+          <t>🚐 TRANSPORT (1인 기준, 4인1조, USD)</t>
+        </is>
+      </c>
+      <c r="B26" s="102" t="n"/>
+      <c r="C26" s="102" t="n"/>
+      <c r="D26" s="102" t="n"/>
+      <c r="E26" s="102" t="n"/>
+      <c r="F26" s="102" t="n"/>
+      <c r="G26" s="102" t="n"/>
+      <c r="H26" s="102" t="n"/>
+      <c r="I26" s="102" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Cost/p</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Sell/p</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Margin</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="n"/>
+      <c r="A27" s="103" t="inlineStr">
+        <is>
+          <t>↳</t>
+        </is>
+      </c>
+      <c r="B27" s="104" t="n"/>
+      <c r="C27" s="104" t="n"/>
+      <c r="D27" s="104" t="n"/>
+      <c r="E27" s="104" t="n"/>
+      <c r="F27" s="104" t="n"/>
+      <c r="G27" s="104" t="n"/>
+      <c r="H27" s="105" t="n"/>
+      <c r="I27" s="105" t="n"/>
     </row>
     <row r="28" ht="16.5" customHeight="1" s="42">
       <c r="A28" s="70" t="inlineStr">
@@ -1532,68 +1727,49 @@
       <c r="F34" s="6" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="31" t="inlineStr">
+      <c r="A36" s="101" t="inlineStr">
         <is>
           <t>🍽️ MEALS (1인 1끼, USD)</t>
         </is>
       </c>
-      <c r="B36" s="44" t="n"/>
-      <c r="C36" s="44" t="n"/>
-      <c r="D36" s="44" t="n"/>
-      <c r="E36" s="44" t="n"/>
-      <c r="F36" s="44" t="n"/>
-      <c r="G36" s="45" t="n"/>
+      <c r="B36" s="102" t="n"/>
+      <c r="C36" s="102" t="n"/>
+      <c r="D36" s="102" t="n"/>
+      <c r="E36" s="102" t="n"/>
+      <c r="F36" s="102" t="n"/>
+      <c r="G36" s="102" t="n"/>
+      <c r="H36" s="102" t="n"/>
+      <c r="I36" s="102" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Meal</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>Margin</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="n"/>
+      <c r="A37" s="103" t="inlineStr">
+        <is>
+          <t>↳</t>
+        </is>
+      </c>
+      <c r="B37" s="104" t="n"/>
+      <c r="C37" s="104" t="n"/>
+      <c r="D37" s="104" t="n"/>
+      <c r="E37" s="104" t="n"/>
+      <c r="F37" s="104" t="n"/>
+      <c r="G37" s="104" t="n"/>
+      <c r="H37" s="105" t="n"/>
+      <c r="I37" s="105" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="70" t="inlineStr">
-        <is>
-          <t>Breakfast (Hotel)</t>
-        </is>
-      </c>
-      <c r="B38" s="71" t="n">
-        <v>30</v>
-      </c>
-      <c r="C38" s="71" t="n">
-        <v>45</v>
-      </c>
-      <c r="D38" s="5">
-        <f>IF(A38="","",C38-B38)</f>
-        <v/>
-      </c>
-      <c r="F38" s="6" t="inlineStr">
-        <is>
-          <t>Daily included</t>
-        </is>
-      </c>
+      <c r="A38" s="106" t="inlineStr">
+        <is>
+          <t>🍳 REGULAR MEALS</t>
+        </is>
+      </c>
+      <c r="B38" s="107" t="n"/>
+      <c r="C38" s="107" t="n"/>
+      <c r="D38" s="107" t="n"/>
+      <c r="E38" s="107" t="n"/>
+      <c r="F38" s="107" t="n"/>
+      <c r="G38" s="107" t="n"/>
+      <c r="H38" s="107" t="n"/>
+      <c r="I38" s="107" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="70" t="inlineStr">
@@ -1640,26 +1816,19 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="70" t="inlineStr">
-        <is>
-          <t>Exclusive Dinner (Michelin/Fine)</t>
-        </is>
-      </c>
-      <c r="B41" s="71" t="n">
-        <v>120</v>
-      </c>
-      <c r="C41" s="71" t="n">
-        <v>180</v>
-      </c>
-      <c r="D41" s="5">
-        <f>IF(A41="","",C41-B41)</f>
-        <v/>
-      </c>
-      <c r="F41" s="6" t="inlineStr">
-        <is>
-          <t>2x per trip</t>
-        </is>
-      </c>
+      <c r="A41" s="106" t="inlineStr">
+        <is>
+          <t>🍽️ PREMIUM DINING</t>
+        </is>
+      </c>
+      <c r="B41" s="107" t="n"/>
+      <c r="C41" s="107" t="n"/>
+      <c r="D41" s="107" t="n"/>
+      <c r="E41" s="107" t="n"/>
+      <c r="F41" s="107" t="n"/>
+      <c r="G41" s="107" t="n"/>
+      <c r="H41" s="107" t="n"/>
+      <c r="I41" s="107" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="40" t="n"/>
@@ -1712,46 +1881,34 @@
       <c r="F46" s="6" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="31" t="inlineStr">
+      <c r="A48" s="101" t="inlineStr">
         <is>
           <t>📦 OTHER (1인 1일, USD)</t>
         </is>
       </c>
-      <c r="B48" s="44" t="n"/>
-      <c r="C48" s="44" t="n"/>
-      <c r="D48" s="44" t="n"/>
-      <c r="E48" s="44" t="n"/>
-      <c r="F48" s="44" t="n"/>
-      <c r="G48" s="45" t="n"/>
+      <c r="B48" s="102" t="n"/>
+      <c r="C48" s="102" t="n"/>
+      <c r="D48" s="102" t="n"/>
+      <c r="E48" s="102" t="n"/>
+      <c r="F48" s="102" t="n"/>
+      <c r="G48" s="102" t="n"/>
+      <c r="H48" s="102" t="n"/>
+      <c r="I48" s="102" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Margin</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="n"/>
+      <c r="A49" s="103" t="inlineStr">
+        <is>
+          <t>↳</t>
+        </is>
+      </c>
+      <c r="B49" s="104" t="n"/>
+      <c r="C49" s="104" t="n"/>
+      <c r="D49" s="104" t="n"/>
+      <c r="E49" s="104" t="n"/>
+      <c r="F49" s="104" t="n"/>
+      <c r="G49" s="104" t="n"/>
+      <c r="H49" s="105" t="n"/>
+      <c r="I49" s="105" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="70" t="inlineStr">
@@ -1825,65 +1982,36 @@
       </c>
       <c r="F55" s="6" t="n"/>
     </row>
+    <row r="56"/>
     <row r="58">
-      <c r="A58" s="31" t="inlineStr">
-        <is>
-          <t>✈️ FLIGHT SCHEDULE — ICN ↔ LAX (현지시간 기준)</t>
-        </is>
-      </c>
-      <c r="B58" s="44" t="n"/>
-      <c r="C58" s="44" t="n"/>
-      <c r="D58" s="44" t="n"/>
-      <c r="E58" s="44" t="n"/>
-      <c r="F58" s="44" t="n"/>
-      <c r="G58" s="45" t="n"/>
+      <c r="A58" s="101" t="inlineStr">
+        <is>
+          <t>✈️ OUTBOUND FLIGHTS (ICN → LAX)</t>
+        </is>
+      </c>
+      <c r="B58" s="102" t="n"/>
+      <c r="C58" s="102" t="n"/>
+      <c r="D58" s="102" t="n"/>
+      <c r="E58" s="102" t="n"/>
+      <c r="F58" s="102" t="n"/>
+      <c r="G58" s="102" t="n"/>
+      <c r="H58" s="102" t="n"/>
+      <c r="I58" s="102" t="n"/>
     </row>
     <row r="59" ht="34.5" customHeight="1" s="42">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Flight#</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Airline</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Dep Time (출발)</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>Arr Time (도착)</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G59" s="46" t="inlineStr">
-        <is>
-          <t>Seat Class</t>
-        </is>
-      </c>
-      <c r="H59" s="46" t="inlineStr">
-        <is>
-          <t>Duration (hrs)</t>
-        </is>
-      </c>
-      <c r="I59" s="46" t="inlineStr">
-        <is>
-          <t>Aircraft</t>
-        </is>
-      </c>
+      <c r="A59" s="103" t="inlineStr">
+        <is>
+          <t>↳</t>
+        </is>
+      </c>
+      <c r="B59" s="104" t="n"/>
+      <c r="C59" s="104" t="n"/>
+      <c r="D59" s="104" t="n"/>
+      <c r="E59" s="104" t="n"/>
+      <c r="F59" s="104" t="n"/>
+      <c r="G59" s="108" t="n"/>
+      <c r="H59" s="108" t="n"/>
+      <c r="I59" s="108" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="70" t="inlineStr">
@@ -2114,64 +2242,34 @@
       <c r="F68" s="6" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="31" t="inlineStr">
+      <c r="A72" s="101" t="inlineStr">
         <is>
           <t>✈️ RETURN FLIGHTS (LAX → ICN)</t>
         </is>
       </c>
-      <c r="B72" s="44" t="n"/>
-      <c r="C72" s="44" t="n"/>
-      <c r="D72" s="44" t="n"/>
-      <c r="E72" s="44" t="n"/>
-      <c r="F72" s="44" t="n"/>
-      <c r="G72" s="45" t="n"/>
+      <c r="B72" s="102" t="n"/>
+      <c r="C72" s="102" t="n"/>
+      <c r="D72" s="102" t="n"/>
+      <c r="E72" s="102" t="n"/>
+      <c r="F72" s="102" t="n"/>
+      <c r="G72" s="102" t="n"/>
+      <c r="H72" s="102" t="n"/>
+      <c r="I72" s="102" t="n"/>
     </row>
     <row r="73" ht="34.5" customHeight="1" s="42">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>Flight#</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>Airline</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>Dep Time (출발)</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>Arr Time (도착)</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="G73" s="46" t="inlineStr">
-        <is>
-          <t>Seat Class</t>
-        </is>
-      </c>
-      <c r="H73" s="46" t="inlineStr">
-        <is>
-          <t>Duration (hrs)</t>
-        </is>
-      </c>
-      <c r="I73" s="46" t="inlineStr">
-        <is>
-          <t>Aircraft</t>
-        </is>
-      </c>
+      <c r="A73" s="103" t="inlineStr">
+        <is>
+          <t>↳</t>
+        </is>
+      </c>
+      <c r="B73" s="104" t="n"/>
+      <c r="C73" s="104" t="n"/>
+      <c r="D73" s="104" t="n"/>
+      <c r="E73" s="104" t="n"/>
+      <c r="F73" s="104" t="n"/>
+      <c r="G73" s="108" t="n"/>
+      <c r="H73" s="108" t="n"/>
+      <c r="I73" s="108" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="70" t="inlineStr">
@@ -2402,71 +2500,49 @@
       <c r="F82" s="6" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="48" t="inlineStr">
+      <c r="A84" s="101" t="inlineStr">
         <is>
           <t>🎯 ACTIVITIES &amp; EXPERIENCES (1인 1회, USD)</t>
         </is>
       </c>
+      <c r="B84" s="109" t="n"/>
+      <c r="C84" s="109" t="n"/>
+      <c r="D84" s="109" t="n"/>
+      <c r="E84" s="109" t="n"/>
+      <c r="F84" s="109" t="n"/>
+      <c r="G84" s="109" t="n"/>
+      <c r="H84" s="109" t="n"/>
+      <c r="I84" s="92" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="46" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="B85" s="46" t="inlineStr">
-        <is>
-          <t>Cost ($)</t>
-        </is>
-      </c>
-      <c r="C85" s="46" t="inlineStr">
-        <is>
-          <t>Sell ($)</t>
-        </is>
-      </c>
-      <c r="D85" s="46" t="inlineStr">
-        <is>
-          <t>Margin ($)</t>
-        </is>
-      </c>
-      <c r="F85" s="46" t="inlineStr">
-        <is>
-          <t>Per Group?</t>
-        </is>
-      </c>
-      <c r="G85" s="46" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="A85" s="103" t="inlineStr">
+        <is>
+          <t>↳</t>
+        </is>
+      </c>
+      <c r="B85" s="108" t="n"/>
+      <c r="C85" s="108" t="n"/>
+      <c r="D85" s="108" t="n"/>
+      <c r="E85" s="105" t="n"/>
+      <c r="F85" s="108" t="n"/>
+      <c r="G85" s="108" t="n"/>
+      <c r="H85" s="105" t="n"/>
+      <c r="I85" s="105" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="74" t="inlineStr">
-        <is>
-          <t>NBA/MLB Game (Ticket)</t>
-        </is>
-      </c>
-      <c r="B86" s="75" t="n">
-        <v>120</v>
-      </c>
-      <c r="C86" s="75" t="n">
-        <v>180</v>
-      </c>
-      <c r="D86" s="51">
-        <f>IF(A86="","",C86-B86)</f>
-        <v/>
-      </c>
-      <c r="E86" s="49" t="n"/>
-      <c r="F86" s="49" t="inlineStr">
-        <is>
-          <t>1p</t>
-        </is>
-      </c>
-      <c r="G86" s="49" t="inlineStr">
-        <is>
-          <t>Seasonal; group rates available</t>
-        </is>
-      </c>
+      <c r="A86" s="106" t="inlineStr">
+        <is>
+          <t>🎫 SPORTS &amp; EVENTS</t>
+        </is>
+      </c>
+      <c r="B86" s="107" t="n"/>
+      <c r="C86" s="107" t="n"/>
+      <c r="D86" s="107" t="n"/>
+      <c r="E86" s="107" t="n"/>
+      <c r="F86" s="107" t="n"/>
+      <c r="G86" s="107" t="n"/>
+      <c r="H86" s="107" t="n"/>
+      <c r="I86" s="107" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="74" t="inlineStr">
@@ -2497,32 +2573,19 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="74" t="inlineStr">
-        <is>
-          <t>Local Hiking (Griffith/Runyon)</t>
-        </is>
-      </c>
-      <c r="B88" s="75" t="n">
-        <v>0</v>
-      </c>
-      <c r="C88" s="75" t="n">
-        <v>30</v>
-      </c>
-      <c r="D88" s="51">
-        <f>IF(A88="","",C88-B88)</f>
-        <v/>
-      </c>
-      <c r="E88" s="49" t="n"/>
-      <c r="F88" s="49" t="inlineStr">
-        <is>
-          <t>1p</t>
-        </is>
-      </c>
-      <c r="G88" s="49" t="inlineStr">
-        <is>
-          <t>Guided tour included</t>
-        </is>
-      </c>
+      <c r="A88" s="106" t="inlineStr">
+        <is>
+          <t>🌿 OUTDOOR &amp; NATURE</t>
+        </is>
+      </c>
+      <c r="B88" s="107" t="n"/>
+      <c r="C88" s="107" t="n"/>
+      <c r="D88" s="107" t="n"/>
+      <c r="E88" s="107" t="n"/>
+      <c r="F88" s="107" t="n"/>
+      <c r="G88" s="107" t="n"/>
+      <c r="H88" s="107" t="n"/>
+      <c r="I88" s="107" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="74" t="inlineStr">
@@ -2633,15 +2696,29 @@
       <c r="G94" s="49" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="23">
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A84:I84"/>
+    <mergeCell ref="A72:G72"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A86:I86"/>
+    <mergeCell ref="A58:G58"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A38:I38"/>
+    <mergeCell ref="A72:I72"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A58:I58"/>
+    <mergeCell ref="A48:I48"/>
     <mergeCell ref="A84:G84"/>
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A58:G58"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="A88:I88"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A72:G72"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3065,10 +3142,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="I4:J4"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3081,7 +3158,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N90"/>
+  <dimension ref="A1:N94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="42" min="1" max="1"/>
@@ -5169,11 +5246,22 @@
     </row>
     <row r="73" ht="30.75" customHeight="1" s="42"/>
     <row r="74" ht="30.75" customHeight="1" s="42">
-      <c r="A74" s="48" t="inlineStr">
-        <is>
-          <t>👤 MULTI-DIRECTIONAL COST ALLOCATION (per person — override any yellow cell)</t>
-        </is>
-      </c>
+      <c r="A74" s="101" t="inlineStr">
+        <is>
+          <t>👤 COST ALLOCATION (노란색 이름 셀을 실제 이름으로 변경 가능)</t>
+        </is>
+      </c>
+      <c r="B74" s="102" t="n"/>
+      <c r="C74" s="102" t="n"/>
+      <c r="D74" s="102" t="n"/>
+      <c r="E74" s="102" t="n"/>
+      <c r="F74" s="102" t="n"/>
+      <c r="G74" s="102" t="n"/>
+      <c r="H74" s="102" t="n"/>
+      <c r="I74" s="102" t="n"/>
+      <c r="J74" s="102" t="n"/>
+      <c r="K74" s="102" t="n"/>
+      <c r="L74" s="102" t="n"/>
     </row>
     <row r="75" ht="30.75" customHeight="1" s="42">
       <c r="A75" s="52" t="inlineStr">
@@ -5181,44 +5269,44 @@
           <t>Category</t>
         </is>
       </c>
-      <c r="B75" s="52" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C75" s="52" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="D75" s="52" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="E75" s="52" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="F75" s="52" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="G75" s="52" t="inlineStr">
-        <is>
-          <t>P6</t>
-        </is>
-      </c>
-      <c r="H75" s="52" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="I75" s="52" t="inlineStr">
-        <is>
-          <t>P8</t>
+      <c r="B75" s="82" t="inlineStr">
+        <is>
+          <t>참가자1</t>
+        </is>
+      </c>
+      <c r="C75" s="82" t="inlineStr">
+        <is>
+          <t>참가자2</t>
+        </is>
+      </c>
+      <c r="D75" s="82" t="inlineStr">
+        <is>
+          <t>참가자3</t>
+        </is>
+      </c>
+      <c r="E75" s="82" t="inlineStr">
+        <is>
+          <t>참가자4</t>
+        </is>
+      </c>
+      <c r="F75" s="82" t="inlineStr">
+        <is>
+          <t>참가자5</t>
+        </is>
+      </c>
+      <c r="G75" s="82" t="inlineStr">
+        <is>
+          <t>참가자6</t>
+        </is>
+      </c>
+      <c r="H75" s="82" t="inlineStr">
+        <is>
+          <t>참가자7</t>
+        </is>
+      </c>
+      <c r="I75" s="82" t="inlineStr">
+        <is>
+          <t>참가자8</t>
         </is>
       </c>
       <c r="J75" s="52" t="inlineStr">
@@ -5608,70 +5696,203 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" s="101" t="inlineStr">
+        <is>
+          <t>🛡️ CONSISTENCY CHECKS</t>
+        </is>
+      </c>
+      <c r="B85" s="102" t="n"/>
+      <c r="C85" s="102" t="n"/>
+      <c r="D85" s="102" t="n"/>
+      <c r="E85" s="102" t="n"/>
+      <c r="F85" s="102" t="n"/>
+      <c r="G85" s="102" t="n"/>
+      <c r="H85" s="102" t="n"/>
+      <c r="I85" s="102" t="n"/>
+      <c r="J85" s="102" t="n"/>
+      <c r="K85" s="102" t="n"/>
+      <c r="L85" s="102" t="n"/>
+    </row>
     <row r="86">
-      <c r="A86" s="48" t="inlineStr">
-        <is>
-          <t>👤 PER PERSON QUICK SUMMARY</t>
-        </is>
-      </c>
+      <c r="A86" s="110" t="inlineStr">
+        <is>
+          <t>Allocation accuracy (0=perfect):</t>
+        </is>
+      </c>
+      <c r="B86" s="111" t="n"/>
+      <c r="C86" s="111" t="n"/>
+      <c r="D86" s="111" t="n"/>
+      <c r="E86" s="111" t="n"/>
+      <c r="F86" s="111" t="n"/>
+      <c r="G86" s="112">
+        <f>SUM(L76:L82)</f>
+        <v/>
+      </c>
+      <c r="H86" s="113">
+        <f>IF(G86=0,"✅ All OK","❌ Fix allocation")</f>
+        <v/>
+      </c>
+      <c r="I86" s="111" t="n"/>
+      <c r="J86" s="111" t="n"/>
+      <c r="K86" s="111" t="n"/>
+      <c r="L86" s="111" t="n"/>
+      <c r="M86" s="111" t="n"/>
+      <c r="N86" s="111" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>Golfers:</t>
-        </is>
-      </c>
-      <c r="B87">
-        <f>G5</f>
-        <v/>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>persons</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Duration:</t>
-        </is>
-      </c>
-      <c r="F87">
-        <f>I11</f>
-        <v/>
-      </c>
+      <c r="A87" s="110" t="inlineStr">
+        <is>
+          <t>Grand Total vs P1-P8 sum:</t>
+        </is>
+      </c>
+      <c r="B87" s="111" t="n"/>
+      <c r="C87" s="111" t="n"/>
+      <c r="D87" s="111" t="n"/>
+      <c r="E87" s="111" t="n"/>
+      <c r="F87" s="111" t="n"/>
+      <c r="G87" s="112">
+        <f>H72-J82</f>
+        <v/>
+      </c>
+      <c r="H87" s="113">
+        <f>IF(G87=0,"✅ All OK","❌ Mismatch")</f>
+        <v/>
+      </c>
+      <c r="I87" s="111" t="n"/>
+      <c r="J87" s="111" t="n"/>
+      <c r="K87" s="111" t="n"/>
+      <c r="L87" s="111" t="n"/>
+      <c r="M87" s="111" t="n"/>
+      <c r="N87" s="111" t="n"/>
     </row>
     <row r="88">
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Per Person Total:</t>
-        </is>
-      </c>
-      <c r="F88" s="66">
-        <f>IF(G5&gt;0,H72/G5,0)</f>
-        <v/>
-      </c>
+      <c r="A88" s="111" t="n"/>
+      <c r="B88" s="111" t="n"/>
+      <c r="C88" s="111" t="n"/>
+      <c r="D88" s="111" t="n"/>
+      <c r="E88" s="111" t="n"/>
+      <c r="F88" s="114" t="n"/>
+      <c r="G88" s="111" t="n"/>
+      <c r="H88" s="111" t="n"/>
+      <c r="I88" s="111" t="n"/>
+      <c r="J88" s="111" t="n"/>
+      <c r="K88" s="111" t="n"/>
+      <c r="L88" s="111" t="n"/>
+      <c r="M88" s="111" t="n"/>
+      <c r="N88" s="111" t="n"/>
     </row>
     <row r="89">
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Per Person Cost:</t>
-        </is>
-      </c>
-      <c r="F89" s="66">
-        <f>IF(G5&gt;0,G72/G5,0)</f>
-        <v/>
-      </c>
+      <c r="A89" s="115" t="inlineStr">
+        <is>
+          <t>💡 ERROR-PROOF TIPS</t>
+        </is>
+      </c>
+      <c r="B89" s="116" t="n"/>
+      <c r="C89" s="116" t="n"/>
+      <c r="D89" s="116" t="n"/>
+      <c r="E89" s="116" t="n"/>
+      <c r="F89" s="117" t="n"/>
+      <c r="G89" s="116" t="n"/>
+      <c r="H89" s="116" t="n"/>
+      <c r="I89" s="116" t="n"/>
+      <c r="J89" s="116" t="n"/>
+      <c r="K89" s="116" t="n"/>
+      <c r="L89" s="116" t="n"/>
+      <c r="M89" s="111" t="n"/>
+      <c r="N89" s="111" t="n"/>
     </row>
     <row r="90">
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Per Person Margin:</t>
-        </is>
-      </c>
-      <c r="F90" s="66">
-        <f>IF(G5&gt;0,I72/G5,0)</f>
-        <v/>
-      </c>
+      <c r="A90" s="118" t="inlineStr">
+        <is>
+          <t>① 빨간색 하이라이트 = 불일치 감지 (수정 필요)</t>
+        </is>
+      </c>
+      <c r="B90" s="81" t="n"/>
+      <c r="C90" s="81" t="n"/>
+      <c r="D90" s="81" t="n"/>
+      <c r="E90" s="81" t="n"/>
+      <c r="F90" s="119" t="n"/>
+      <c r="G90" s="81" t="n"/>
+      <c r="H90" s="81" t="n"/>
+      <c r="I90" s="81" t="n"/>
+      <c r="J90" s="81" t="n"/>
+      <c r="K90" s="81" t="n"/>
+      <c r="L90" s="81" t="n"/>
+      <c r="M90" s="111" t="n"/>
+      <c r="N90" s="111" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="118" t="inlineStr">
+        <is>
+          <t>② ✓Check=0 인지 항상 확인 → 0이면 완벽분배</t>
+        </is>
+      </c>
+      <c r="B91" s="81" t="n"/>
+      <c r="C91" s="81" t="n"/>
+      <c r="D91" s="81" t="n"/>
+      <c r="E91" s="81" t="n"/>
+      <c r="F91" s="81" t="n"/>
+      <c r="G91" s="81" t="n"/>
+      <c r="H91" s="81" t="n"/>
+      <c r="I91" s="81" t="n"/>
+      <c r="J91" s="81" t="n"/>
+      <c r="K91" s="81" t="n"/>
+      <c r="L91" s="81" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="118" t="inlineStr">
+        <is>
+          <t>③ Grand Total = P1~P8 합계 일치 확인</t>
+        </is>
+      </c>
+      <c r="B92" s="81" t="n"/>
+      <c r="C92" s="81" t="n"/>
+      <c r="D92" s="81" t="n"/>
+      <c r="E92" s="81" t="n"/>
+      <c r="F92" s="81" t="n"/>
+      <c r="G92" s="81" t="n"/>
+      <c r="H92" s="81" t="n"/>
+      <c r="I92" s="81" t="n"/>
+      <c r="J92" s="81" t="n"/>
+      <c r="K92" s="81" t="n"/>
+      <c r="L92" s="81" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="118" t="inlineStr">
+        <is>
+          <t>④ Package Selector 2 액티비티 총액 = Package Selector 액티비티 총액 교차검증</t>
+        </is>
+      </c>
+      <c r="B93" s="81" t="n"/>
+      <c r="C93" s="81" t="n"/>
+      <c r="D93" s="81" t="n"/>
+      <c r="E93" s="81" t="n"/>
+      <c r="F93" s="81" t="n"/>
+      <c r="G93" s="81" t="n"/>
+      <c r="H93" s="81" t="n"/>
+      <c r="I93" s="81" t="n"/>
+      <c r="J93" s="81" t="n"/>
+      <c r="K93" s="81" t="n"/>
+      <c r="L93" s="81" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="118" t="inlineStr">
+        <is>
+          <t>⑤ 드롭다운 외 값 입력 시 #N/A → 드롭다운에서만 선택</t>
+        </is>
+      </c>
+      <c r="B94" s="81" t="n"/>
+      <c r="C94" s="81" t="n"/>
+      <c r="D94" s="81" t="n"/>
+      <c r="E94" s="81" t="n"/>
+      <c r="F94" s="81" t="n"/>
+      <c r="G94" s="81" t="n"/>
+      <c r="H94" s="81" t="n"/>
+      <c r="I94" s="81" t="n"/>
+      <c r="J94" s="81" t="n"/>
+      <c r="K94" s="81" t="n"/>
+      <c r="L94" s="81" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="19">
@@ -5695,6 +5916,41 @@
     <mergeCell ref="A45:L45"/>
     <mergeCell ref="A36:L36"/>
   </mergeCells>
+  <conditionalFormatting sqref="L76">
+    <cfRule type="cellIs" priority="1" operator="notEqual" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L77">
+    <cfRule type="cellIs" priority="2" operator="notEqual" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L78">
+    <cfRule type="cellIs" priority="3" operator="notEqual" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L79">
+    <cfRule type="cellIs" priority="4" operator="notEqual" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L80">
+    <cfRule type="cellIs" priority="5" operator="notEqual" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L81">
+    <cfRule type="cellIs" priority="6" operator="notEqual" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L82">
+    <cfRule type="cellIs" priority="7" operator="notEqual" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="12">
     <dataValidation sqref="B15 B16 B17 B18 B19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
       <formula1>'Master Data'!$A$7:$A$14</formula1>
@@ -6093,4 +6349,976 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" style="42" min="1" max="1"/>
+    <col width="12" customWidth="1" style="42" min="2" max="2"/>
+    <col width="12" customWidth="1" style="42" min="3" max="3"/>
+    <col width="12" customWidth="1" style="42" min="4" max="4"/>
+    <col width="12" customWidth="1" style="42" min="5" max="5"/>
+    <col width="12" customWidth="1" style="42" min="6" max="6"/>
+    <col width="12" customWidth="1" style="42" min="7" max="7"/>
+    <col width="12" customWidth="1" style="42" min="8" max="8"/>
+    <col width="12" customWidth="1" style="42" min="9" max="9"/>
+    <col width="14" customWidth="1" style="42" min="10" max="10"/>
+    <col width="14" customWidth="1" style="42" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="101" t="inlineStr">
+        <is>
+          <t>🎯 ACTIVITY SELECTOR — Per Person (참가자별 액티비티 선택)</t>
+        </is>
+      </c>
+      <c r="B1" s="102" t="n"/>
+      <c r="C1" s="102" t="n"/>
+      <c r="D1" s="102" t="n"/>
+      <c r="E1" s="102" t="n"/>
+      <c r="F1" s="102" t="n"/>
+      <c r="G1" s="102" t="n"/>
+      <c r="H1" s="102" t="n"/>
+      <c r="I1" s="102" t="n"/>
+      <c r="J1" s="102" t="n"/>
+      <c r="K1" s="102" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="120" t="inlineStr">
+        <is>
+          <t>각 참가자가 원하는 액티비티에 ✓ 체크 → 자동 비용계산 → Profit Summary 2에 반영</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="110" t="inlineStr">
+        <is>
+          <t>Group Size:</t>
+        </is>
+      </c>
+      <c r="B4" s="121">
+        <f>'Package Selector'!G5</f>
+        <v/>
+      </c>
+      <c r="C4" s="118" t="inlineStr">
+        <is>
+          <t>persons</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="98" t="inlineStr">
+        <is>
+          <t>Activity \ Person</t>
+        </is>
+      </c>
+      <c r="B6" s="98" t="inlineStr">
+        <is>
+          <t>참가자1</t>
+        </is>
+      </c>
+      <c r="C6" s="98" t="inlineStr">
+        <is>
+          <t>참가자2</t>
+        </is>
+      </c>
+      <c r="D6" s="98" t="inlineStr">
+        <is>
+          <t>참가자3</t>
+        </is>
+      </c>
+      <c r="E6" s="98" t="inlineStr">
+        <is>
+          <t>참가자4</t>
+        </is>
+      </c>
+      <c r="F6" s="98" t="inlineStr">
+        <is>
+          <t>참가자5</t>
+        </is>
+      </c>
+      <c r="G6" s="98" t="inlineStr">
+        <is>
+          <t>참가자6</t>
+        </is>
+      </c>
+      <c r="H6" s="98" t="inlineStr">
+        <is>
+          <t>참가자7</t>
+        </is>
+      </c>
+      <c r="I6" s="98" t="inlineStr">
+        <is>
+          <t>참가자8</t>
+        </is>
+      </c>
+      <c r="J6" s="98" t="inlineStr">
+        <is>
+          <t>✓ Count</t>
+        </is>
+      </c>
+      <c r="K6" s="98" t="inlineStr">
+        <is>
+          <t>Cost/Person</t>
+        </is>
+      </c>
+      <c r="L6" s="98" t="inlineStr">
+        <is>
+          <t>Sell/Person</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="122" t="inlineStr">
+        <is>
+          <t>NBA/MLB Game (Ticket)</t>
+        </is>
+      </c>
+      <c r="B7" s="123" t="inlineStr"/>
+      <c r="C7" s="123" t="inlineStr"/>
+      <c r="D7" s="123" t="inlineStr"/>
+      <c r="E7" s="123" t="inlineStr"/>
+      <c r="F7" s="123" t="inlineStr"/>
+      <c r="G7" s="123" t="inlineStr"/>
+      <c r="H7" s="123" t="inlineStr"/>
+      <c r="I7" s="123" t="inlineStr"/>
+      <c r="J7" s="121">
+        <f>COUNTIF(B7:I7,"✓")</f>
+        <v/>
+      </c>
+      <c r="K7" s="124">
+        <f>IF(J7&gt;0,VLOOKUP(A7,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="L7" s="124">
+        <f>IF(J7&gt;0,VLOOKUP(A7,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="118" t="inlineStr">
+        <is>
+          <t>Sports Bar Experience</t>
+        </is>
+      </c>
+      <c r="B8" s="81" t="inlineStr"/>
+      <c r="C8" s="81" t="inlineStr"/>
+      <c r="D8" s="81" t="inlineStr"/>
+      <c r="E8" s="81" t="inlineStr"/>
+      <c r="F8" s="81" t="inlineStr"/>
+      <c r="G8" s="81" t="inlineStr"/>
+      <c r="H8" s="81" t="inlineStr"/>
+      <c r="I8" s="81" t="inlineStr"/>
+      <c r="J8" s="121">
+        <f>COUNTIF(B8:I8,"✓")</f>
+        <v/>
+      </c>
+      <c r="K8" s="124">
+        <f>IF(J8&gt;0,VLOOKUP(A8,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="L8" s="124">
+        <f>IF(J8&gt;0,VLOOKUP(A8,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="122" t="inlineStr">
+        <is>
+          <t>Local Hiking (Griffith)</t>
+        </is>
+      </c>
+      <c r="B9" s="123" t="inlineStr"/>
+      <c r="C9" s="123" t="inlineStr"/>
+      <c r="D9" s="123" t="inlineStr"/>
+      <c r="E9" s="123" t="inlineStr"/>
+      <c r="F9" s="123" t="inlineStr"/>
+      <c r="G9" s="123" t="inlineStr"/>
+      <c r="H9" s="123" t="inlineStr"/>
+      <c r="I9" s="123" t="inlineStr"/>
+      <c r="J9" s="121">
+        <f>COUNTIF(B9:I9,"✓")</f>
+        <v/>
+      </c>
+      <c r="K9" s="124">
+        <f>IF(J9&gt;0,VLOOKUP(A9,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="L9" s="124">
+        <f>IF(J9&gt;0,VLOOKUP(A9,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="118" t="inlineStr">
+        <is>
+          <t>Beach/Surf Lesson</t>
+        </is>
+      </c>
+      <c r="B10" s="81" t="inlineStr"/>
+      <c r="C10" s="81" t="inlineStr"/>
+      <c r="D10" s="81" t="inlineStr"/>
+      <c r="E10" s="81" t="inlineStr"/>
+      <c r="F10" s="81" t="inlineStr"/>
+      <c r="G10" s="81" t="inlineStr"/>
+      <c r="H10" s="81" t="inlineStr"/>
+      <c r="I10" s="81" t="inlineStr"/>
+      <c r="J10" s="121">
+        <f>COUNTIF(B10:I10,"✓")</f>
+        <v/>
+      </c>
+      <c r="K10" s="124">
+        <f>IF(J10&gt;0,VLOOKUP(A10,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="L10" s="124">
+        <f>IF(J10&gt;0,VLOOKUP(A10,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="125" t="inlineStr">
+        <is>
+          <t>(New Activity 5)</t>
+        </is>
+      </c>
+      <c r="B11" s="123" t="inlineStr"/>
+      <c r="C11" s="123" t="inlineStr"/>
+      <c r="D11" s="123" t="inlineStr"/>
+      <c r="E11" s="123" t="inlineStr"/>
+      <c r="F11" s="123" t="inlineStr"/>
+      <c r="G11" s="123" t="inlineStr"/>
+      <c r="H11" s="123" t="inlineStr"/>
+      <c r="I11" s="123" t="inlineStr"/>
+      <c r="J11" s="121">
+        <f>COUNTIF(B11:I11,"✓")</f>
+        <v/>
+      </c>
+      <c r="K11" s="126">
+        <f>IF(J11&gt;0,VLOOKUP(A11,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="L11" s="126">
+        <f>IF(J11&gt;0,VLOOKUP(A11,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="120" t="inlineStr">
+        <is>
+          <t>(New Activity 6)</t>
+        </is>
+      </c>
+      <c r="B12" s="81" t="inlineStr"/>
+      <c r="C12" s="81" t="inlineStr"/>
+      <c r="D12" s="81" t="inlineStr"/>
+      <c r="E12" s="81" t="inlineStr"/>
+      <c r="F12" s="81" t="inlineStr"/>
+      <c r="G12" s="81" t="inlineStr"/>
+      <c r="H12" s="81" t="inlineStr"/>
+      <c r="I12" s="81" t="inlineStr"/>
+      <c r="J12" s="121">
+        <f>COUNTIF(B12:I12,"✓")</f>
+        <v/>
+      </c>
+      <c r="K12" s="126">
+        <f>IF(J12&gt;0,VLOOKUP(A12,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="L12" s="126">
+        <f>IF(J12&gt;0,VLOOKUP(A12,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="125" t="inlineStr">
+        <is>
+          <t>(New Activity 7)</t>
+        </is>
+      </c>
+      <c r="B13" s="123" t="inlineStr"/>
+      <c r="C13" s="123" t="inlineStr"/>
+      <c r="D13" s="123" t="inlineStr"/>
+      <c r="E13" s="123" t="inlineStr"/>
+      <c r="F13" s="123" t="inlineStr"/>
+      <c r="G13" s="123" t="inlineStr"/>
+      <c r="H13" s="123" t="inlineStr"/>
+      <c r="I13" s="123" t="inlineStr"/>
+      <c r="J13" s="121">
+        <f>COUNTIF(B13:I13,"✓")</f>
+        <v/>
+      </c>
+      <c r="K13" s="126">
+        <f>IF(J13&gt;0,VLOOKUP(A13,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="L13" s="126">
+        <f>IF(J13&gt;0,VLOOKUP(A13,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="120" t="inlineStr">
+        <is>
+          <t>(New Activity 8)</t>
+        </is>
+      </c>
+      <c r="B14" s="81" t="inlineStr"/>
+      <c r="C14" s="81" t="inlineStr"/>
+      <c r="D14" s="81" t="inlineStr"/>
+      <c r="E14" s="81" t="inlineStr"/>
+      <c r="F14" s="81" t="inlineStr"/>
+      <c r="G14" s="81" t="inlineStr"/>
+      <c r="H14" s="81" t="inlineStr"/>
+      <c r="I14" s="81" t="inlineStr"/>
+      <c r="J14" s="121">
+        <f>COUNTIF(B14:I14,"✓")</f>
+        <v/>
+      </c>
+      <c r="K14" s="126">
+        <f>IF(J14&gt;0,VLOOKUP(A14,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="L14" s="126">
+        <f>IF(J14&gt;0,VLOOKUP(A14,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="125" t="inlineStr">
+        <is>
+          <t>(New Activity 9)</t>
+        </is>
+      </c>
+      <c r="B15" s="123" t="inlineStr"/>
+      <c r="C15" s="123" t="inlineStr"/>
+      <c r="D15" s="123" t="inlineStr"/>
+      <c r="E15" s="123" t="inlineStr"/>
+      <c r="F15" s="123" t="inlineStr"/>
+      <c r="G15" s="123" t="inlineStr"/>
+      <c r="H15" s="123" t="inlineStr"/>
+      <c r="I15" s="123" t="inlineStr"/>
+      <c r="J15" s="121">
+        <f>COUNTIF(B15:I15,"✓")</f>
+        <v/>
+      </c>
+      <c r="K15" s="126">
+        <f>IF(J15&gt;0,VLOOKUP(A15,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="L15" s="126">
+        <f>IF(J15&gt;0,VLOOKUP(A15,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="127" t="inlineStr">
+        <is>
+          <t>📌 TOTALS</t>
+        </is>
+      </c>
+      <c r="B16" s="128" t="inlineStr"/>
+      <c r="C16" s="128" t="inlineStr"/>
+      <c r="D16" s="128" t="inlineStr"/>
+      <c r="E16" s="128" t="inlineStr"/>
+      <c r="F16" s="128" t="inlineStr"/>
+      <c r="G16" s="128" t="inlineStr"/>
+      <c r="H16" s="128" t="inlineStr"/>
+      <c r="I16" s="128" t="inlineStr"/>
+      <c r="J16" s="129">
+        <f>SUM(J7:J15)</f>
+        <v/>
+      </c>
+      <c r="K16" s="88">
+        <f>SUM(K7:K15)</f>
+        <v/>
+      </c>
+      <c r="L16" s="88">
+        <f>SUM(L7:L15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="101" t="inlineStr">
+        <is>
+          <t>👤 PER-PERSON ACTIVITY COST</t>
+        </is>
+      </c>
+      <c r="B18" s="102" t="n"/>
+      <c r="C18" s="102" t="n"/>
+      <c r="D18" s="102" t="n"/>
+      <c r="E18" s="102" t="n"/>
+      <c r="F18" s="102" t="n"/>
+      <c r="G18" s="102" t="n"/>
+      <c r="H18" s="102" t="n"/>
+      <c r="I18" s="102" t="n"/>
+      <c r="J18" s="102" t="n"/>
+      <c r="K18" s="102" t="n"/>
+      <c r="L18" s="102" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="98" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="B19" s="98" t="inlineStr">
+        <is>
+          <t>Activity Cost</t>
+        </is>
+      </c>
+      <c r="C19" s="98" t="inlineStr">
+        <is>
+          <t>Activity Sell</t>
+        </is>
+      </c>
+      <c r="D19" s="98" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="118" t="inlineStr">
+        <is>
+          <t>참가자1</t>
+        </is>
+      </c>
+      <c r="B20" s="124">
+        <f>SUMPRODUCT((B7:B15="✓")*1,K7:K15)</f>
+        <v/>
+      </c>
+      <c r="C20" s="124">
+        <f>SUMPRODUCT((B7:B15="✓")*1,L7:L15)</f>
+        <v/>
+      </c>
+      <c r="D20" s="124">
+        <f>C20-B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="118" t="inlineStr">
+        <is>
+          <t>참가자2</t>
+        </is>
+      </c>
+      <c r="B21" s="124">
+        <f>SUMPRODUCT((C7:C15="✓")*1,K7:K15)</f>
+        <v/>
+      </c>
+      <c r="C21" s="124">
+        <f>SUMPRODUCT((C7:C15="✓")*1,L7:L15)</f>
+        <v/>
+      </c>
+      <c r="D21" s="124">
+        <f>C21-B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="118" t="inlineStr">
+        <is>
+          <t>참가자3</t>
+        </is>
+      </c>
+      <c r="B22" s="124">
+        <f>SUMPRODUCT((D7:D15="✓")*1,K7:K15)</f>
+        <v/>
+      </c>
+      <c r="C22" s="124">
+        <f>SUMPRODUCT((D7:D15="✓")*1,L7:L15)</f>
+        <v/>
+      </c>
+      <c r="D22" s="124">
+        <f>C22-B22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="118" t="inlineStr">
+        <is>
+          <t>참가자4</t>
+        </is>
+      </c>
+      <c r="B23" s="124">
+        <f>SUMPRODUCT((E7:E15="✓")*1,K7:K15)</f>
+        <v/>
+      </c>
+      <c r="C23" s="124">
+        <f>SUMPRODUCT((E7:E15="✓")*1,L7:L15)</f>
+        <v/>
+      </c>
+      <c r="D23" s="124">
+        <f>C23-B23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="118" t="inlineStr">
+        <is>
+          <t>참가자5</t>
+        </is>
+      </c>
+      <c r="B24" s="124">
+        <f>SUMPRODUCT((F7:F15="✓")*1,K7:K15)</f>
+        <v/>
+      </c>
+      <c r="C24" s="124">
+        <f>SUMPRODUCT((F7:F15="✓")*1,L7:L15)</f>
+        <v/>
+      </c>
+      <c r="D24" s="124">
+        <f>C24-B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="118" t="inlineStr">
+        <is>
+          <t>참가자6</t>
+        </is>
+      </c>
+      <c r="B25" s="124">
+        <f>SUMPRODUCT((G7:G15="✓")*1,K7:K15)</f>
+        <v/>
+      </c>
+      <c r="C25" s="124">
+        <f>SUMPRODUCT((G7:G15="✓")*1,L7:L15)</f>
+        <v/>
+      </c>
+      <c r="D25" s="124">
+        <f>C25-B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="118" t="inlineStr">
+        <is>
+          <t>참가자7</t>
+        </is>
+      </c>
+      <c r="B26" s="124">
+        <f>SUMPRODUCT((H7:H15="✓")*1,K7:K15)</f>
+        <v/>
+      </c>
+      <c r="C26" s="124">
+        <f>SUMPRODUCT((H7:H15="✓")*1,L7:L15)</f>
+        <v/>
+      </c>
+      <c r="D26" s="124">
+        <f>C26-B26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="118" t="inlineStr">
+        <is>
+          <t>참가자8</t>
+        </is>
+      </c>
+      <c r="B27" s="124">
+        <f>SUMPRODUCT((I7:I15="✓")*1,K7:K15)</f>
+        <v/>
+      </c>
+      <c r="C27" s="124">
+        <f>SUMPRODUCT((I7:I15="✓")*1,L7:L15)</f>
+        <v/>
+      </c>
+      <c r="D27" s="124">
+        <f>C27-B27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="130" t="inlineStr">
+        <is>
+          <t>📌 TOTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="88">
+        <f>SUM(B20:B27)</f>
+        <v/>
+      </c>
+      <c r="C28" s="88">
+        <f>SUM(C20:C27)</f>
+        <v/>
+      </c>
+      <c r="D28" s="88">
+        <f>SUM(D20:D27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="131" t="inlineStr">
+        <is>
+          <t>✓Check (0=OK):</t>
+        </is>
+      </c>
+      <c r="B29" s="112">
+        <f>B28-K16</f>
+        <v/>
+      </c>
+      <c r="C29" s="113" t="inlineStr"/>
+      <c r="D29" s="113">
+        <f>IF(B29=0,"✅ 정확","❌ 불일치")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A18:L18"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B29">
+    <cfRule type="cellIs" priority="1" operator="notEqual" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" style="42" min="1" max="1"/>
+    <col width="14" customWidth="1" style="42" min="2" max="2"/>
+    <col width="14" customWidth="1" style="42" min="3" max="3"/>
+    <col width="14" customWidth="1" style="42" min="4" max="4"/>
+    <col width="14" customWidth="1" style="42" min="5" max="5"/>
+    <col width="14" customWidth="1" style="42" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="101" t="inlineStr">
+        <is>
+          <t>📊 PROFIT SUMMARY 2 — Activity Sub-Category Breakdown</t>
+        </is>
+      </c>
+      <c r="B1" s="102" t="n"/>
+      <c r="C1" s="102" t="n"/>
+      <c r="D1" s="102" t="n"/>
+      <c r="E1" s="102" t="n"/>
+      <c r="F1" s="102" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="120" t="inlineStr">
+        <is>
+          <t>⬇️ 'Package Selector 2' 체크마크 기반 → 활동별·참가자별 자동 분석</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="132" t="inlineStr">
+        <is>
+          <t>Category / Activity</t>
+        </is>
+      </c>
+      <c r="B4" s="98" t="inlineStr">
+        <is>
+          <t>Participants</t>
+        </is>
+      </c>
+      <c r="C4" s="98" t="inlineStr">
+        <is>
+          <t>Cost/Person</t>
+        </is>
+      </c>
+      <c r="D4" s="98" t="inlineStr">
+        <is>
+          <t>Total Cost</t>
+        </is>
+      </c>
+      <c r="E4" s="98" t="inlineStr">
+        <is>
+          <t>Total Sell</t>
+        </is>
+      </c>
+      <c r="F4" s="98" t="inlineStr">
+        <is>
+          <t>Total Margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="133" t="inlineStr">
+        <is>
+          <t>🎫 SPORTS &amp; EVENTS</t>
+        </is>
+      </c>
+      <c r="B5" s="134" t="n"/>
+      <c r="C5" s="134" t="n"/>
+      <c r="D5" s="134" t="n"/>
+      <c r="E5" s="134" t="n"/>
+      <c r="F5" s="134" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NBA/MLB Game (Ticket)</t>
+        </is>
+      </c>
+      <c r="B6" s="135">
+        <f>'Package Selector 2'!J7</f>
+        <v/>
+      </c>
+      <c r="C6" s="84">
+        <f>'Package Selector 2'!K7</f>
+        <v/>
+      </c>
+      <c r="D6" s="84">
+        <f>B6*C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="84">
+        <f>B6*'Package Selector 2'!L7</f>
+        <v/>
+      </c>
+      <c r="F6" s="84">
+        <f>E6-D6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sports Bar Experience</t>
+        </is>
+      </c>
+      <c r="B7" s="135">
+        <f>'Package Selector 2'!J8</f>
+        <v/>
+      </c>
+      <c r="C7" s="84">
+        <f>'Package Selector 2'!K8</f>
+        <v/>
+      </c>
+      <c r="D7" s="84">
+        <f>B7*C7</f>
+        <v/>
+      </c>
+      <c r="E7" s="84">
+        <f>B7*'Package Selector 2'!L8</f>
+        <v/>
+      </c>
+      <c r="F7" s="84">
+        <f>E7-D7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SPORTS SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="D8" s="88">
+        <f>SUM(D6:D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="88">
+        <f>SUM(E6:E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="88">
+        <f>SUM(F6:F7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="133" t="inlineStr">
+        <is>
+          <t>🌿 OUTDOOR &amp; NATURE</t>
+        </is>
+      </c>
+      <c r="B10" s="134" t="n"/>
+      <c r="C10" s="134" t="n"/>
+      <c r="D10" s="134" t="n"/>
+      <c r="E10" s="134" t="n"/>
+      <c r="F10" s="134" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Local Hiking (Griffith)</t>
+        </is>
+      </c>
+      <c r="B11" s="135">
+        <f>'Package Selector 2'!J9</f>
+        <v/>
+      </c>
+      <c r="C11" s="84">
+        <f>'Package Selector 2'!K9</f>
+        <v/>
+      </c>
+      <c r="D11" s="84">
+        <f>B11*C11</f>
+        <v/>
+      </c>
+      <c r="E11" s="84">
+        <f>B11*'Package Selector 2'!L9</f>
+        <v/>
+      </c>
+      <c r="F11" s="84">
+        <f>E11-D11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Beach/Surf Lesson</t>
+        </is>
+      </c>
+      <c r="B12" s="135">
+        <f>'Package Selector 2'!J10</f>
+        <v/>
+      </c>
+      <c r="C12" s="84">
+        <f>'Package Selector 2'!K10</f>
+        <v/>
+      </c>
+      <c r="D12" s="84">
+        <f>B12*C12</f>
+        <v/>
+      </c>
+      <c r="E12" s="84">
+        <f>B12*'Package Selector 2'!L10</f>
+        <v/>
+      </c>
+      <c r="F12" s="84">
+        <f>E12-D12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  OUTDOOR SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="D13" s="88">
+        <f>SUM(D11:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="88">
+        <f>SUM(E11:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="88">
+        <f>SUM(F11:F12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="101" t="inlineStr">
+        <is>
+          <t>🏆 ACTIVITIES GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="B15" s="102" t="n"/>
+      <c r="C15" s="102" t="n"/>
+      <c r="D15" s="102" t="n"/>
+      <c r="E15" s="102" t="n"/>
+      <c r="F15" s="102" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="110" t="inlineStr">
+        <is>
+          <t>📌 TOTAL ALL ACTIVITIES</t>
+        </is>
+      </c>
+      <c r="D16" s="88">
+        <f>D8+D13</f>
+        <v/>
+      </c>
+      <c r="E16" s="88">
+        <f>E8+E13</f>
+        <v/>
+      </c>
+      <c r="F16" s="88">
+        <f>F8+F13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="115" t="inlineStr">
+        <is>
+          <t>🔍 CROSS-CHECK vs Package Selector</t>
+        </is>
+      </c>
+      <c r="B18" s="116" t="n"/>
+      <c r="C18" s="116" t="n"/>
+      <c r="D18" s="116" t="n"/>
+      <c r="E18" s="116" t="n"/>
+      <c r="F18" s="116" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="137" t="inlineStr">
+        <is>
+          <t>Package Selector Activities Cost:</t>
+        </is>
+      </c>
+      <c r="D19" s="84">
+        <f>'Package Selector'!G62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="137" t="inlineStr">
+        <is>
+          <t>Package Selector 2 Activities Cost:</t>
+        </is>
+      </c>
+      <c r="D20" s="84">
+        <f>D16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="131" t="inlineStr">
+        <is>
+          <t>Difference:</t>
+        </is>
+      </c>
+      <c r="D21" s="138">
+        <f>D20-D19</f>
+        <v/>
+      </c>
+      <c r="E21" s="113">
+        <f>IF(D21=0,"✅ MATCH","❌ MISMATCH — check selections")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D21">
+    <cfRule type="cellIs" priority="1" operator="notEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: restore from bak5, keep Master Data intact, add PS2+PF2 tabs, duplicate detection
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -121,14 +121,14 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00666666"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <color rgb="00888888"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="22">
@@ -236,14 +236,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFE8F0FE"/>
+        <bgColor rgb="FFE8F0FE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8F0FE"/>
-        <bgColor rgb="FFE8F0FE"/>
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -253,7 +253,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -473,66 +473,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF333333"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF333333"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF4472C4"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF4472C4"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF4472C4"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF4472C4"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF4472C4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF4472C4"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF4472C4"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF4472C4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -790,98 +735,63 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="20" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="20" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="16" fillId="21" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="20" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="19" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="17" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="19" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="20" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="20" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="18" fillId="20" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="12" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="20" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -890,11 +800,14 @@
     <xf numFmtId="0" fontId="16" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -903,6 +816,7 @@
   <dxfs count="2">
     <dxf>
       <font>
+        <b val="1"/>
         <color rgb="009C0006"/>
       </font>
       <fill>
@@ -914,7 +828,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
         <color rgb="009C0006"/>
       </font>
       <fill>
@@ -1316,80 +1229,82 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="98" t="inlineStr"/>
-      <c r="B3" s="98" t="inlineStr">
+      <c r="A3" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    새 코스·호텔·편명 추가는 빈칸에 직접 입력 → 자동으로 드롭다운에 반영</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>⛳ GOLF COURSES (1인 1라운드, USD)</t>
+        </is>
+      </c>
+      <c r="B5" s="44" t="n"/>
+      <c r="C5" s="44" t="n"/>
+      <c r="D5" s="44" t="n"/>
+      <c r="E5" s="44" t="n"/>
+      <c r="F5" s="44" t="n"/>
+      <c r="G5" s="45" t="n"/>
+    </row>
+    <row r="6" ht="30.75" customHeight="1" s="42">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Course</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Cost ($)</t>
         </is>
       </c>
-      <c r="C3" s="98" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sell ($)</t>
         </is>
       </c>
-      <c r="D3" s="98" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Margin ($)</t>
         </is>
       </c>
-      <c r="E3" s="98" t="inlineStr">
-        <is>
-          <t>+Info</t>
-        </is>
-      </c>
-      <c r="F3" s="98" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Replay Rate ($)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="G3" s="98" t="inlineStr"/>
-      <c r="H3" s="98" t="inlineStr"/>
-      <c r="I3" s="98" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="101" t="inlineStr">
-        <is>
-          <t>⛳ GOLF COURSES (1인 1라운드, USD)</t>
-        </is>
-      </c>
-      <c r="B5" s="102" t="n"/>
-      <c r="C5" s="102" t="n"/>
-      <c r="D5" s="102" t="n"/>
-      <c r="E5" s="102" t="n"/>
-      <c r="F5" s="102" t="n"/>
-      <c r="G5" s="102" t="n"/>
-      <c r="H5" s="102" t="n"/>
-      <c r="I5" s="102" t="n"/>
-    </row>
-    <row r="6" ht="30.75" customHeight="1" s="42">
-      <c r="A6" s="103" t="inlineStr">
-        <is>
-          <t>↳</t>
-        </is>
-      </c>
-      <c r="B6" s="104" t="n"/>
-      <c r="C6" s="104" t="n"/>
-      <c r="D6" s="104" t="n"/>
-      <c r="E6" s="104" t="n"/>
-      <c r="F6" s="104" t="n"/>
-      <c r="G6" s="104" t="n"/>
-      <c r="H6" s="105" t="n"/>
-      <c r="I6" s="105" t="n"/>
+      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="106" t="inlineStr">
-        <is>
-          <t>🏆 PREMIUM COURSES</t>
-        </is>
-      </c>
-      <c r="B7" s="107" t="n"/>
-      <c r="C7" s="107" t="n"/>
-      <c r="D7" s="107" t="n"/>
-      <c r="E7" s="107" t="n"/>
-      <c r="F7" s="107" t="n"/>
-      <c r="G7" s="107" t="n"/>
-      <c r="H7" s="107" t="n"/>
-      <c r="I7" s="107" t="n"/>
+      <c r="A7" s="70" t="inlineStr">
+        <is>
+          <t>Trump National LA</t>
+        </is>
+      </c>
+      <c r="B7" s="71" t="n">
+        <v>210</v>
+      </c>
+      <c r="C7" s="71" t="n">
+        <v>210</v>
+      </c>
+      <c r="D7" s="5">
+        <f>IF(A7="","",C7-B7)</f>
+        <v/>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>111</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Member guest | Cart incl. | Replay ~50%</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="70" t="inlineStr">
@@ -1464,19 +1379,15 @@
       <c r="F11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="106" t="inlineStr">
-        <is>
-          <t>📋 ADDITIONAL COURSES (추가 가능)</t>
-        </is>
-      </c>
-      <c r="B12" s="107" t="n"/>
-      <c r="C12" s="107" t="n"/>
-      <c r="D12" s="107" t="n"/>
-      <c r="E12" s="107" t="n"/>
-      <c r="F12" s="107" t="n"/>
-      <c r="G12" s="107" t="n"/>
-      <c r="H12" s="107" t="n"/>
-      <c r="I12" s="107" t="n"/>
+      <c r="A12" s="40" t="n"/>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="5">
+        <f>IF(A12="","",C12-B12)</f>
+        <v/>
+      </c>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="40" t="n"/>
@@ -1501,34 +1412,46 @@
       <c r="F14" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="101" t="inlineStr">
-        <is>
-          <t>🏨 HOTELS (1인 1박, Double Occ., USD)</t>
-        </is>
-      </c>
-      <c r="B17" s="102" t="n"/>
-      <c r="C17" s="102" t="n"/>
-      <c r="D17" s="102" t="n"/>
-      <c r="E17" s="102" t="n"/>
-      <c r="F17" s="102" t="n"/>
-      <c r="G17" s="102" t="n"/>
-      <c r="H17" s="102" t="n"/>
-      <c r="I17" s="102" t="n"/>
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>🏨 HOTEL (1인 1박, Double Occupancy, USD)</t>
+        </is>
+      </c>
+      <c r="B17" s="44" t="n"/>
+      <c r="C17" s="44" t="n"/>
+      <c r="D17" s="44" t="n"/>
+      <c r="E17" s="44" t="n"/>
+      <c r="F17" s="44" t="n"/>
+      <c r="G17" s="45" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="103" t="inlineStr">
-        <is>
-          <t>↳</t>
-        </is>
-      </c>
-      <c r="B18" s="104" t="n"/>
-      <c r="C18" s="104" t="n"/>
-      <c r="D18" s="104" t="n"/>
-      <c r="E18" s="104" t="n"/>
-      <c r="F18" s="104" t="n"/>
-      <c r="G18" s="104" t="n"/>
-      <c r="H18" s="105" t="n"/>
-      <c r="I18" s="105" t="n"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Cost/night</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Sell/night</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n"/>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="42">
       <c r="A19" s="70" t="inlineStr">
@@ -1603,34 +1526,46 @@
       <c r="F24" s="6" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="101" t="inlineStr">
-        <is>
-          <t>🚐 TRANSPORT (1인 기준, 4인1조, USD)</t>
-        </is>
-      </c>
-      <c r="B26" s="102" t="n"/>
-      <c r="C26" s="102" t="n"/>
-      <c r="D26" s="102" t="n"/>
-      <c r="E26" s="102" t="n"/>
-      <c r="F26" s="102" t="n"/>
-      <c r="G26" s="102" t="n"/>
-      <c r="H26" s="102" t="n"/>
-      <c r="I26" s="102" t="n"/>
+      <c r="A26" s="31" t="inlineStr">
+        <is>
+          <t>🚐 TRANSPORT (1인 기준, 4인 1조, USD)</t>
+        </is>
+      </c>
+      <c r="B26" s="44" t="n"/>
+      <c r="C26" s="44" t="n"/>
+      <c r="D26" s="44" t="n"/>
+      <c r="E26" s="44" t="n"/>
+      <c r="F26" s="44" t="n"/>
+      <c r="G26" s="45" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="103" t="inlineStr">
-        <is>
-          <t>↳</t>
-        </is>
-      </c>
-      <c r="B27" s="104" t="n"/>
-      <c r="C27" s="104" t="n"/>
-      <c r="D27" s="104" t="n"/>
-      <c r="E27" s="104" t="n"/>
-      <c r="F27" s="104" t="n"/>
-      <c r="G27" s="104" t="n"/>
-      <c r="H27" s="105" t="n"/>
-      <c r="I27" s="105" t="n"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Cost/p</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Sell/p</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n"/>
     </row>
     <row r="28" ht="16.5" customHeight="1" s="42">
       <c r="A28" s="70" t="inlineStr">
@@ -1727,49 +1662,68 @@
       <c r="F34" s="6" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="101" t="inlineStr">
+      <c r="A36" s="31" t="inlineStr">
         <is>
           <t>🍽️ MEALS (1인 1끼, USD)</t>
         </is>
       </c>
-      <c r="B36" s="102" t="n"/>
-      <c r="C36" s="102" t="n"/>
-      <c r="D36" s="102" t="n"/>
-      <c r="E36" s="102" t="n"/>
-      <c r="F36" s="102" t="n"/>
-      <c r="G36" s="102" t="n"/>
-      <c r="H36" s="102" t="n"/>
-      <c r="I36" s="102" t="n"/>
+      <c r="B36" s="44" t="n"/>
+      <c r="C36" s="44" t="n"/>
+      <c r="D36" s="44" t="n"/>
+      <c r="E36" s="44" t="n"/>
+      <c r="F36" s="44" t="n"/>
+      <c r="G36" s="45" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="103" t="inlineStr">
-        <is>
-          <t>↳</t>
-        </is>
-      </c>
-      <c r="B37" s="104" t="n"/>
-      <c r="C37" s="104" t="n"/>
-      <c r="D37" s="104" t="n"/>
-      <c r="E37" s="104" t="n"/>
-      <c r="F37" s="104" t="n"/>
-      <c r="G37" s="104" t="n"/>
-      <c r="H37" s="105" t="n"/>
-      <c r="I37" s="105" t="n"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Meal</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="106" t="inlineStr">
-        <is>
-          <t>🍳 REGULAR MEALS</t>
-        </is>
-      </c>
-      <c r="B38" s="107" t="n"/>
-      <c r="C38" s="107" t="n"/>
-      <c r="D38" s="107" t="n"/>
-      <c r="E38" s="107" t="n"/>
-      <c r="F38" s="107" t="n"/>
-      <c r="G38" s="107" t="n"/>
-      <c r="H38" s="107" t="n"/>
-      <c r="I38" s="107" t="n"/>
+      <c r="A38" s="70" t="inlineStr">
+        <is>
+          <t>Breakfast (Hotel)</t>
+        </is>
+      </c>
+      <c r="B38" s="71" t="n">
+        <v>30</v>
+      </c>
+      <c r="C38" s="71" t="n">
+        <v>45</v>
+      </c>
+      <c r="D38" s="5">
+        <f>IF(A38="","",C38-B38)</f>
+        <v/>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Daily included</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="70" t="inlineStr">
@@ -1816,19 +1770,26 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="106" t="inlineStr">
-        <is>
-          <t>🍽️ PREMIUM DINING</t>
-        </is>
-      </c>
-      <c r="B41" s="107" t="n"/>
-      <c r="C41" s="107" t="n"/>
-      <c r="D41" s="107" t="n"/>
-      <c r="E41" s="107" t="n"/>
-      <c r="F41" s="107" t="n"/>
-      <c r="G41" s="107" t="n"/>
-      <c r="H41" s="107" t="n"/>
-      <c r="I41" s="107" t="n"/>
+      <c r="A41" s="70" t="inlineStr">
+        <is>
+          <t>Exclusive Dinner (Michelin/Fine)</t>
+        </is>
+      </c>
+      <c r="B41" s="71" t="n">
+        <v>120</v>
+      </c>
+      <c r="C41" s="71" t="n">
+        <v>180</v>
+      </c>
+      <c r="D41" s="5">
+        <f>IF(A41="","",C41-B41)</f>
+        <v/>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>2x per trip</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="40" t="n"/>
@@ -1881,34 +1842,46 @@
       <c r="F46" s="6" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="101" t="inlineStr">
+      <c r="A48" s="31" t="inlineStr">
         <is>
           <t>📦 OTHER (1인 1일, USD)</t>
         </is>
       </c>
-      <c r="B48" s="102" t="n"/>
-      <c r="C48" s="102" t="n"/>
-      <c r="D48" s="102" t="n"/>
-      <c r="E48" s="102" t="n"/>
-      <c r="F48" s="102" t="n"/>
-      <c r="G48" s="102" t="n"/>
-      <c r="H48" s="102" t="n"/>
-      <c r="I48" s="102" t="n"/>
+      <c r="B48" s="44" t="n"/>
+      <c r="C48" s="44" t="n"/>
+      <c r="D48" s="44" t="n"/>
+      <c r="E48" s="44" t="n"/>
+      <c r="F48" s="44" t="n"/>
+      <c r="G48" s="45" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="103" t="inlineStr">
-        <is>
-          <t>↳</t>
-        </is>
-      </c>
-      <c r="B49" s="104" t="n"/>
-      <c r="C49" s="104" t="n"/>
-      <c r="D49" s="104" t="n"/>
-      <c r="E49" s="104" t="n"/>
-      <c r="F49" s="104" t="n"/>
-      <c r="G49" s="104" t="n"/>
-      <c r="H49" s="105" t="n"/>
-      <c r="I49" s="105" t="n"/>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="70" t="inlineStr">
@@ -1982,36 +1955,65 @@
       </c>
       <c r="F55" s="6" t="n"/>
     </row>
-    <row r="56"/>
     <row r="58">
-      <c r="A58" s="101" t="inlineStr">
-        <is>
-          <t>✈️ OUTBOUND FLIGHTS (ICN → LAX)</t>
-        </is>
-      </c>
-      <c r="B58" s="102" t="n"/>
-      <c r="C58" s="102" t="n"/>
-      <c r="D58" s="102" t="n"/>
-      <c r="E58" s="102" t="n"/>
-      <c r="F58" s="102" t="n"/>
-      <c r="G58" s="102" t="n"/>
-      <c r="H58" s="102" t="n"/>
-      <c r="I58" s="102" t="n"/>
+      <c r="A58" s="31" t="inlineStr">
+        <is>
+          <t>✈️ FLIGHT SCHEDULE — ICN ↔ LAX (현지시간 기준)</t>
+        </is>
+      </c>
+      <c r="B58" s="44" t="n"/>
+      <c r="C58" s="44" t="n"/>
+      <c r="D58" s="44" t="n"/>
+      <c r="E58" s="44" t="n"/>
+      <c r="F58" s="44" t="n"/>
+      <c r="G58" s="45" t="n"/>
     </row>
     <row r="59" ht="34.5" customHeight="1" s="42">
-      <c r="A59" s="103" t="inlineStr">
-        <is>
-          <t>↳</t>
-        </is>
-      </c>
-      <c r="B59" s="104" t="n"/>
-      <c r="C59" s="104" t="n"/>
-      <c r="D59" s="104" t="n"/>
-      <c r="E59" s="104" t="n"/>
-      <c r="F59" s="104" t="n"/>
-      <c r="G59" s="108" t="n"/>
-      <c r="H59" s="108" t="n"/>
-      <c r="I59" s="108" t="n"/>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Flight#</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Dep Time (출발)</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Arr Time (도착)</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G59" s="46" t="inlineStr">
+        <is>
+          <t>Seat Class</t>
+        </is>
+      </c>
+      <c r="H59" s="46" t="inlineStr">
+        <is>
+          <t>Duration (hrs)</t>
+        </is>
+      </c>
+      <c r="I59" s="46" t="inlineStr">
+        <is>
+          <t>Aircraft</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="70" t="inlineStr">
@@ -2242,34 +2244,64 @@
       <c r="F68" s="6" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="101" t="inlineStr">
+      <c r="A72" s="31" t="inlineStr">
         <is>
           <t>✈️ RETURN FLIGHTS (LAX → ICN)</t>
         </is>
       </c>
-      <c r="B72" s="102" t="n"/>
-      <c r="C72" s="102" t="n"/>
-      <c r="D72" s="102" t="n"/>
-      <c r="E72" s="102" t="n"/>
-      <c r="F72" s="102" t="n"/>
-      <c r="G72" s="102" t="n"/>
-      <c r="H72" s="102" t="n"/>
-      <c r="I72" s="102" t="n"/>
+      <c r="B72" s="44" t="n"/>
+      <c r="C72" s="44" t="n"/>
+      <c r="D72" s="44" t="n"/>
+      <c r="E72" s="44" t="n"/>
+      <c r="F72" s="44" t="n"/>
+      <c r="G72" s="45" t="n"/>
     </row>
     <row r="73" ht="34.5" customHeight="1" s="42">
-      <c r="A73" s="103" t="inlineStr">
-        <is>
-          <t>↳</t>
-        </is>
-      </c>
-      <c r="B73" s="104" t="n"/>
-      <c r="C73" s="104" t="n"/>
-      <c r="D73" s="104" t="n"/>
-      <c r="E73" s="104" t="n"/>
-      <c r="F73" s="104" t="n"/>
-      <c r="G73" s="108" t="n"/>
-      <c r="H73" s="108" t="n"/>
-      <c r="I73" s="108" t="n"/>
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Flight#</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Airline</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Dep Time (출발)</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Arr Time (도착)</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G73" s="46" t="inlineStr">
+        <is>
+          <t>Seat Class</t>
+        </is>
+      </c>
+      <c r="H73" s="46" t="inlineStr">
+        <is>
+          <t>Duration (hrs)</t>
+        </is>
+      </c>
+      <c r="I73" s="46" t="inlineStr">
+        <is>
+          <t>Aircraft</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="70" t="inlineStr">
@@ -2500,49 +2532,71 @@
       <c r="F82" s="6" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="101" t="inlineStr">
+      <c r="A84" s="48" t="inlineStr">
         <is>
           <t>🎯 ACTIVITIES &amp; EXPERIENCES (1인 1회, USD)</t>
         </is>
       </c>
-      <c r="B84" s="109" t="n"/>
-      <c r="C84" s="109" t="n"/>
-      <c r="D84" s="109" t="n"/>
-      <c r="E84" s="109" t="n"/>
-      <c r="F84" s="109" t="n"/>
-      <c r="G84" s="109" t="n"/>
-      <c r="H84" s="109" t="n"/>
-      <c r="I84" s="92" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="103" t="inlineStr">
-        <is>
-          <t>↳</t>
-        </is>
-      </c>
-      <c r="B85" s="108" t="n"/>
-      <c r="C85" s="108" t="n"/>
-      <c r="D85" s="108" t="n"/>
-      <c r="E85" s="105" t="n"/>
-      <c r="F85" s="108" t="n"/>
-      <c r="G85" s="108" t="n"/>
-      <c r="H85" s="105" t="n"/>
-      <c r="I85" s="105" t="n"/>
+      <c r="A85" s="46" t="inlineStr">
+        <is>
+          <t>Activity</t>
+        </is>
+      </c>
+      <c r="B85" s="46" t="inlineStr">
+        <is>
+          <t>Cost ($)</t>
+        </is>
+      </c>
+      <c r="C85" s="46" t="inlineStr">
+        <is>
+          <t>Sell ($)</t>
+        </is>
+      </c>
+      <c r="D85" s="46" t="inlineStr">
+        <is>
+          <t>Margin ($)</t>
+        </is>
+      </c>
+      <c r="F85" s="46" t="inlineStr">
+        <is>
+          <t>Per Group?</t>
+        </is>
+      </c>
+      <c r="G85" s="46" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="106" t="inlineStr">
-        <is>
-          <t>🎫 SPORTS &amp; EVENTS</t>
-        </is>
-      </c>
-      <c r="B86" s="107" t="n"/>
-      <c r="C86" s="107" t="n"/>
-      <c r="D86" s="107" t="n"/>
-      <c r="E86" s="107" t="n"/>
-      <c r="F86" s="107" t="n"/>
-      <c r="G86" s="107" t="n"/>
-      <c r="H86" s="107" t="n"/>
-      <c r="I86" s="107" t="n"/>
+      <c r="A86" s="74" t="inlineStr">
+        <is>
+          <t>NBA/MLB Game (Ticket)</t>
+        </is>
+      </c>
+      <c r="B86" s="75" t="n">
+        <v>120</v>
+      </c>
+      <c r="C86" s="75" t="n">
+        <v>180</v>
+      </c>
+      <c r="D86" s="51">
+        <f>IF(A86="","",C86-B86)</f>
+        <v/>
+      </c>
+      <c r="E86" s="49" t="n"/>
+      <c r="F86" s="49" t="inlineStr">
+        <is>
+          <t>1p</t>
+        </is>
+      </c>
+      <c r="G86" s="49" t="inlineStr">
+        <is>
+          <t>Seasonal; group rates available</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="74" t="inlineStr">
@@ -2573,19 +2627,32 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="106" t="inlineStr">
-        <is>
-          <t>🌿 OUTDOOR &amp; NATURE</t>
-        </is>
-      </c>
-      <c r="B88" s="107" t="n"/>
-      <c r="C88" s="107" t="n"/>
-      <c r="D88" s="107" t="n"/>
-      <c r="E88" s="107" t="n"/>
-      <c r="F88" s="107" t="n"/>
-      <c r="G88" s="107" t="n"/>
-      <c r="H88" s="107" t="n"/>
-      <c r="I88" s="107" t="n"/>
+      <c r="A88" s="74" t="inlineStr">
+        <is>
+          <t>Local Hiking (Griffith/Runyon)</t>
+        </is>
+      </c>
+      <c r="B88" s="75" t="n">
+        <v>0</v>
+      </c>
+      <c r="C88" s="75" t="n">
+        <v>30</v>
+      </c>
+      <c r="D88" s="51">
+        <f>IF(A88="","",C88-B88)</f>
+        <v/>
+      </c>
+      <c r="E88" s="49" t="n"/>
+      <c r="F88" s="49" t="inlineStr">
+        <is>
+          <t>1p</t>
+        </is>
+      </c>
+      <c r="G88" s="49" t="inlineStr">
+        <is>
+          <t>Guided tour included</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="74" t="inlineStr">
@@ -2696,29 +2763,15 @@
       <c r="G94" s="49" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="A41:I41"/>
+  <mergeCells count="9">
+    <mergeCell ref="A84:G84"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A58:G58"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A84:I84"/>
+    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A26:G26"/>
     <mergeCell ref="A72:G72"/>
-    <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A86:I86"/>
-    <mergeCell ref="A58:G58"/>
-    <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A48:G48"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A38:I38"/>
-    <mergeCell ref="A72:I72"/>
-    <mergeCell ref="A36:G36"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A58:I58"/>
-    <mergeCell ref="A48:I48"/>
-    <mergeCell ref="A84:G84"/>
-    <mergeCell ref="A36:I36"/>
-    <mergeCell ref="A88:I88"/>
-    <mergeCell ref="A26:G26"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3158,7 +3211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N94"/>
+  <dimension ref="A1:N90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="42" min="1" max="1"/>
@@ -5246,22 +5299,11 @@
     </row>
     <row r="73" ht="30.75" customHeight="1" s="42"/>
     <row r="74" ht="30.75" customHeight="1" s="42">
-      <c r="A74" s="101" t="inlineStr">
-        <is>
-          <t>👤 COST ALLOCATION (노란색 이름 셀을 실제 이름으로 변경 가능)</t>
-        </is>
-      </c>
-      <c r="B74" s="102" t="n"/>
-      <c r="C74" s="102" t="n"/>
-      <c r="D74" s="102" t="n"/>
-      <c r="E74" s="102" t="n"/>
-      <c r="F74" s="102" t="n"/>
-      <c r="G74" s="102" t="n"/>
-      <c r="H74" s="102" t="n"/>
-      <c r="I74" s="102" t="n"/>
-      <c r="J74" s="102" t="n"/>
-      <c r="K74" s="102" t="n"/>
-      <c r="L74" s="102" t="n"/>
+      <c r="A74" s="48" t="inlineStr">
+        <is>
+          <t>👤 MULTI-DIRECTIONAL COST ALLOCATION (per person — override any yellow cell)</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="30.75" customHeight="1" s="42">
       <c r="A75" s="52" t="inlineStr">
@@ -5696,203 +5738,85 @@
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="101" t="inlineStr">
-        <is>
-          <t>🛡️ CONSISTENCY CHECKS</t>
-        </is>
-      </c>
-      <c r="B85" s="102" t="n"/>
-      <c r="C85" s="102" t="n"/>
-      <c r="D85" s="102" t="n"/>
-      <c r="E85" s="102" t="n"/>
-      <c r="F85" s="102" t="n"/>
-      <c r="G85" s="102" t="n"/>
-      <c r="H85" s="102" t="n"/>
-      <c r="I85" s="102" t="n"/>
-      <c r="J85" s="102" t="n"/>
-      <c r="K85" s="102" t="n"/>
-      <c r="L85" s="102" t="n"/>
-    </row>
     <row r="86">
-      <c r="A86" s="110" t="inlineStr">
-        <is>
-          <t>Allocation accuracy (0=perfect):</t>
-        </is>
-      </c>
-      <c r="B86" s="111" t="n"/>
-      <c r="C86" s="111" t="n"/>
-      <c r="D86" s="111" t="n"/>
-      <c r="E86" s="111" t="n"/>
-      <c r="F86" s="111" t="n"/>
-      <c r="G86" s="112">
-        <f>SUM(L76:L82)</f>
-        <v/>
-      </c>
-      <c r="H86" s="113">
-        <f>IF(G86=0,"✅ All OK","❌ Fix allocation")</f>
-        <v/>
-      </c>
-      <c r="I86" s="111" t="n"/>
-      <c r="J86" s="111" t="n"/>
-      <c r="K86" s="111" t="n"/>
-      <c r="L86" s="111" t="n"/>
-      <c r="M86" s="111" t="n"/>
-      <c r="N86" s="111" t="n"/>
+      <c r="A86" s="101" t="n"/>
+      <c r="B86" s="101" t="n"/>
+      <c r="C86" s="101" t="n"/>
+      <c r="D86" s="101" t="n"/>
+      <c r="E86" s="101" t="n"/>
+      <c r="F86" s="101" t="n"/>
+      <c r="G86" s="101" t="n"/>
+      <c r="H86" s="101" t="n"/>
+      <c r="I86" s="101" t="n"/>
+      <c r="J86" s="101" t="n"/>
+      <c r="K86" s="101" t="n"/>
+      <c r="L86" s="101" t="n"/>
+      <c r="M86" s="101" t="n"/>
+      <c r="N86" s="101" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="110" t="inlineStr">
-        <is>
-          <t>Grand Total vs P1-P8 sum:</t>
-        </is>
-      </c>
-      <c r="B87" s="111" t="n"/>
-      <c r="C87" s="111" t="n"/>
-      <c r="D87" s="111" t="n"/>
-      <c r="E87" s="111" t="n"/>
-      <c r="F87" s="111" t="n"/>
-      <c r="G87" s="112">
-        <f>H72-J82</f>
-        <v/>
-      </c>
-      <c r="H87" s="113">
-        <f>IF(G87=0,"✅ All OK","❌ Mismatch")</f>
-        <v/>
-      </c>
-      <c r="I87" s="111" t="n"/>
-      <c r="J87" s="111" t="n"/>
-      <c r="K87" s="111" t="n"/>
-      <c r="L87" s="111" t="n"/>
-      <c r="M87" s="111" t="n"/>
-      <c r="N87" s="111" t="n"/>
+      <c r="A87" s="101" t="n"/>
+      <c r="B87" s="101" t="n"/>
+      <c r="C87" s="101" t="n"/>
+      <c r="D87" s="101" t="n"/>
+      <c r="E87" s="101" t="n"/>
+      <c r="F87" s="101" t="n"/>
+      <c r="G87" s="101" t="n"/>
+      <c r="H87" s="101" t="n"/>
+      <c r="I87" s="101" t="n"/>
+      <c r="J87" s="101" t="n"/>
+      <c r="K87" s="101" t="n"/>
+      <c r="L87" s="101" t="n"/>
+      <c r="M87" s="101" t="n"/>
+      <c r="N87" s="101" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="111" t="n"/>
-      <c r="B88" s="111" t="n"/>
-      <c r="C88" s="111" t="n"/>
-      <c r="D88" s="111" t="n"/>
-      <c r="E88" s="111" t="n"/>
-      <c r="F88" s="114" t="n"/>
-      <c r="G88" s="111" t="n"/>
-      <c r="H88" s="111" t="n"/>
-      <c r="I88" s="111" t="n"/>
-      <c r="J88" s="111" t="n"/>
-      <c r="K88" s="111" t="n"/>
-      <c r="L88" s="111" t="n"/>
-      <c r="M88" s="111" t="n"/>
-      <c r="N88" s="111" t="n"/>
+      <c r="A88" s="101" t="n"/>
+      <c r="B88" s="101" t="n"/>
+      <c r="C88" s="101" t="n"/>
+      <c r="D88" s="101" t="n"/>
+      <c r="E88" s="101" t="n"/>
+      <c r="F88" s="102" t="n"/>
+      <c r="G88" s="101" t="n"/>
+      <c r="H88" s="101" t="n"/>
+      <c r="I88" s="101" t="n"/>
+      <c r="J88" s="101" t="n"/>
+      <c r="K88" s="101" t="n"/>
+      <c r="L88" s="101" t="n"/>
+      <c r="M88" s="101" t="n"/>
+      <c r="N88" s="101" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="115" t="inlineStr">
-        <is>
-          <t>💡 ERROR-PROOF TIPS</t>
-        </is>
-      </c>
-      <c r="B89" s="116" t="n"/>
-      <c r="C89" s="116" t="n"/>
-      <c r="D89" s="116" t="n"/>
-      <c r="E89" s="116" t="n"/>
-      <c r="F89" s="117" t="n"/>
-      <c r="G89" s="116" t="n"/>
-      <c r="H89" s="116" t="n"/>
-      <c r="I89" s="116" t="n"/>
-      <c r="J89" s="116" t="n"/>
-      <c r="K89" s="116" t="n"/>
-      <c r="L89" s="116" t="n"/>
-      <c r="M89" s="111" t="n"/>
-      <c r="N89" s="111" t="n"/>
+      <c r="A89" s="101" t="n"/>
+      <c r="B89" s="101" t="n"/>
+      <c r="C89" s="101" t="n"/>
+      <c r="D89" s="101" t="n"/>
+      <c r="E89" s="101" t="n"/>
+      <c r="F89" s="102" t="n"/>
+      <c r="G89" s="101" t="n"/>
+      <c r="H89" s="101" t="n"/>
+      <c r="I89" s="101" t="n"/>
+      <c r="J89" s="101" t="n"/>
+      <c r="K89" s="101" t="n"/>
+      <c r="L89" s="101" t="n"/>
+      <c r="M89" s="101" t="n"/>
+      <c r="N89" s="101" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="118" t="inlineStr">
-        <is>
-          <t>① 빨간색 하이라이트 = 불일치 감지 (수정 필요)</t>
-        </is>
-      </c>
-      <c r="B90" s="81" t="n"/>
-      <c r="C90" s="81" t="n"/>
-      <c r="D90" s="81" t="n"/>
-      <c r="E90" s="81" t="n"/>
-      <c r="F90" s="119" t="n"/>
-      <c r="G90" s="81" t="n"/>
-      <c r="H90" s="81" t="n"/>
-      <c r="I90" s="81" t="n"/>
-      <c r="J90" s="81" t="n"/>
-      <c r="K90" s="81" t="n"/>
-      <c r="L90" s="81" t="n"/>
-      <c r="M90" s="111" t="n"/>
-      <c r="N90" s="111" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="118" t="inlineStr">
-        <is>
-          <t>② ✓Check=0 인지 항상 확인 → 0이면 완벽분배</t>
-        </is>
-      </c>
-      <c r="B91" s="81" t="n"/>
-      <c r="C91" s="81" t="n"/>
-      <c r="D91" s="81" t="n"/>
-      <c r="E91" s="81" t="n"/>
-      <c r="F91" s="81" t="n"/>
-      <c r="G91" s="81" t="n"/>
-      <c r="H91" s="81" t="n"/>
-      <c r="I91" s="81" t="n"/>
-      <c r="J91" s="81" t="n"/>
-      <c r="K91" s="81" t="n"/>
-      <c r="L91" s="81" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="118" t="inlineStr">
-        <is>
-          <t>③ Grand Total = P1~P8 합계 일치 확인</t>
-        </is>
-      </c>
-      <c r="B92" s="81" t="n"/>
-      <c r="C92" s="81" t="n"/>
-      <c r="D92" s="81" t="n"/>
-      <c r="E92" s="81" t="n"/>
-      <c r="F92" s="81" t="n"/>
-      <c r="G92" s="81" t="n"/>
-      <c r="H92" s="81" t="n"/>
-      <c r="I92" s="81" t="n"/>
-      <c r="J92" s="81" t="n"/>
-      <c r="K92" s="81" t="n"/>
-      <c r="L92" s="81" t="n"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="118" t="inlineStr">
-        <is>
-          <t>④ Package Selector 2 액티비티 총액 = Package Selector 액티비티 총액 교차검증</t>
-        </is>
-      </c>
-      <c r="B93" s="81" t="n"/>
-      <c r="C93" s="81" t="n"/>
-      <c r="D93" s="81" t="n"/>
-      <c r="E93" s="81" t="n"/>
-      <c r="F93" s="81" t="n"/>
-      <c r="G93" s="81" t="n"/>
-      <c r="H93" s="81" t="n"/>
-      <c r="I93" s="81" t="n"/>
-      <c r="J93" s="81" t="n"/>
-      <c r="K93" s="81" t="n"/>
-      <c r="L93" s="81" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="118" t="inlineStr">
-        <is>
-          <t>⑤ 드롭다운 외 값 입력 시 #N/A → 드롭다운에서만 선택</t>
-        </is>
-      </c>
-      <c r="B94" s="81" t="n"/>
-      <c r="C94" s="81" t="n"/>
-      <c r="D94" s="81" t="n"/>
-      <c r="E94" s="81" t="n"/>
-      <c r="F94" s="81" t="n"/>
-      <c r="G94" s="81" t="n"/>
-      <c r="H94" s="81" t="n"/>
-      <c r="I94" s="81" t="n"/>
-      <c r="J94" s="81" t="n"/>
-      <c r="K94" s="81" t="n"/>
-      <c r="L94" s="81" t="n"/>
+      <c r="A90" s="101" t="n"/>
+      <c r="B90" s="101" t="n"/>
+      <c r="C90" s="101" t="n"/>
+      <c r="D90" s="101" t="n"/>
+      <c r="E90" s="101" t="n"/>
+      <c r="F90" s="102" t="n"/>
+      <c r="G90" s="101" t="n"/>
+      <c r="H90" s="101" t="n"/>
+      <c r="I90" s="101" t="n"/>
+      <c r="J90" s="101" t="n"/>
+      <c r="K90" s="101" t="n"/>
+      <c r="L90" s="101" t="n"/>
+      <c r="M90" s="101" t="n"/>
+      <c r="N90" s="101" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="19">
@@ -5916,41 +5840,6 @@
     <mergeCell ref="A45:L45"/>
     <mergeCell ref="A36:L36"/>
   </mergeCells>
-  <conditionalFormatting sqref="L76">
-    <cfRule type="cellIs" priority="1" operator="notEqual" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L77">
-    <cfRule type="cellIs" priority="2" operator="notEqual" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L78">
-    <cfRule type="cellIs" priority="3" operator="notEqual" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L79">
-    <cfRule type="cellIs" priority="4" operator="notEqual" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L80">
-    <cfRule type="cellIs" priority="5" operator="notEqual" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L81">
-    <cfRule type="cellIs" priority="6" operator="notEqual" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L82">
-    <cfRule type="cellIs" priority="7" operator="notEqual" dxfId="0">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="12">
     <dataValidation sqref="B15 B16 B17 B18 B19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
       <formula1>'Master Data'!$A$7:$A$14</formula1>
@@ -6357,57 +6246,59 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="42" min="1" max="1"/>
-    <col width="12" customWidth="1" style="42" min="2" max="2"/>
-    <col width="12" customWidth="1" style="42" min="3" max="3"/>
-    <col width="12" customWidth="1" style="42" min="4" max="4"/>
-    <col width="12" customWidth="1" style="42" min="5" max="5"/>
-    <col width="12" customWidth="1" style="42" min="6" max="6"/>
-    <col width="12" customWidth="1" style="42" min="7" max="7"/>
-    <col width="12" customWidth="1" style="42" min="8" max="8"/>
-    <col width="12" customWidth="1" style="42" min="9" max="9"/>
-    <col width="14" customWidth="1" style="42" min="10" max="10"/>
-    <col width="14" customWidth="1" style="42" min="11" max="11"/>
+    <col width="11" customWidth="1" style="42" min="2" max="2"/>
+    <col width="11" customWidth="1" style="42" min="3" max="3"/>
+    <col width="11" customWidth="1" style="42" min="4" max="4"/>
+    <col width="11" customWidth="1" style="42" min="5" max="5"/>
+    <col width="11" customWidth="1" style="42" min="6" max="6"/>
+    <col width="11" customWidth="1" style="42" min="7" max="7"/>
+    <col width="11" customWidth="1" style="42" min="8" max="8"/>
+    <col width="11" customWidth="1" style="42" min="9" max="9"/>
+    <col width="13" customWidth="1" style="42" min="10" max="10"/>
+    <col width="13" customWidth="1" style="42" min="11" max="11"/>
+    <col width="13" customWidth="1" style="42" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="101" t="inlineStr">
-        <is>
-          <t>🎯 ACTIVITY SELECTOR — Per Person (참가자별 액티비티 선택)</t>
-        </is>
-      </c>
-      <c r="B1" s="102" t="n"/>
-      <c r="C1" s="102" t="n"/>
-      <c r="D1" s="102" t="n"/>
-      <c r="E1" s="102" t="n"/>
-      <c r="F1" s="102" t="n"/>
-      <c r="G1" s="102" t="n"/>
-      <c r="H1" s="102" t="n"/>
-      <c r="I1" s="102" t="n"/>
-      <c r="J1" s="102" t="n"/>
-      <c r="K1" s="102" t="n"/>
+      <c r="A1" s="103" t="inlineStr">
+        <is>
+          <t>🎯 ACTIVITY SELECTOR — Per Person</t>
+        </is>
+      </c>
+      <c r="B1" s="104" t="n"/>
+      <c r="C1" s="104" t="n"/>
+      <c r="D1" s="104" t="n"/>
+      <c r="E1" s="104" t="n"/>
+      <c r="F1" s="104" t="n"/>
+      <c r="G1" s="104" t="n"/>
+      <c r="H1" s="104" t="n"/>
+      <c r="I1" s="104" t="n"/>
+      <c r="J1" s="104" t="n"/>
+      <c r="K1" s="104" t="n"/>
+      <c r="L1" s="104" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="120" t="inlineStr">
-        <is>
-          <t>각 참가자가 원하는 액티비티에 ✓ 체크 → 자동 비용계산 → Profit Summary 2에 반영</t>
+      <c r="A2" s="105" t="inlineStr">
+        <is>
+          <t>참가자 컬럼에 ✓ 체크 → 자동 비용계산 → Profit Summary 2 반영 | 중복선택 시 ⚠️ 표시</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="110" t="inlineStr">
+      <c r="A4" s="106" t="inlineStr">
         <is>
           <t>Group Size:</t>
         </is>
       </c>
-      <c r="B4" s="121">
+      <c r="B4" s="107">
         <f>'Package Selector'!G5</f>
         <v/>
       </c>
-      <c r="C4" s="118" t="inlineStr">
+      <c r="C4" s="108" t="inlineStr">
         <is>
           <t>persons</t>
         </is>
@@ -6466,44 +6357,58 @@
       </c>
       <c r="K6" s="98" t="inlineStr">
         <is>
-          <t>Cost/Person</t>
+          <t>Cost/P</t>
         </is>
       </c>
       <c r="L6" s="98" t="inlineStr">
         <is>
-          <t>Sell/Person</t>
+          <t>Sell/P</t>
+        </is>
+      </c>
+      <c r="M6" s="98" t="inlineStr">
+        <is>
+          <t>⚠️ Dup</t>
+        </is>
+      </c>
+      <c r="N6" s="98" t="inlineStr">
+        <is>
+          <t>Available Activities</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="122" t="inlineStr">
+      <c r="A7" s="109" t="inlineStr">
         <is>
           <t>NBA/MLB Game (Ticket)</t>
         </is>
       </c>
-      <c r="B7" s="123" t="inlineStr"/>
-      <c r="C7" s="123" t="inlineStr"/>
-      <c r="D7" s="123" t="inlineStr"/>
-      <c r="E7" s="123" t="inlineStr"/>
-      <c r="F7" s="123" t="inlineStr"/>
-      <c r="G7" s="123" t="inlineStr"/>
-      <c r="H7" s="123" t="inlineStr"/>
-      <c r="I7" s="123" t="inlineStr"/>
-      <c r="J7" s="121">
+      <c r="B7" s="81" t="inlineStr"/>
+      <c r="C7" s="81" t="inlineStr"/>
+      <c r="D7" s="81" t="inlineStr"/>
+      <c r="E7" s="81" t="inlineStr"/>
+      <c r="F7" s="81" t="inlineStr"/>
+      <c r="G7" s="81" t="inlineStr"/>
+      <c r="H7" s="81" t="inlineStr"/>
+      <c r="I7" s="81" t="inlineStr"/>
+      <c r="J7" s="107">
         <f>COUNTIF(B7:I7,"✓")</f>
         <v/>
       </c>
-      <c r="K7" s="124">
+      <c r="K7" s="110">
         <f>IF(J7&gt;0,VLOOKUP(A7,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
         <v/>
       </c>
-      <c r="L7" s="124">
+      <c r="L7" s="110">
         <f>IF(J7&gt;0,VLOOKUP(A7,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
         <v/>
       </c>
+      <c r="M7" s="111">
+        <f>IF(A7="","",COUNTIF($A$7:$A$6,A7)+COUNTIF($A$8:$A$15,A7))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="118" t="inlineStr">
+      <c r="A8" s="108" t="inlineStr">
         <is>
           <t>Sports Bar Experience</t>
         </is>
@@ -6516,48 +6421,56 @@
       <c r="G8" s="81" t="inlineStr"/>
       <c r="H8" s="81" t="inlineStr"/>
       <c r="I8" s="81" t="inlineStr"/>
-      <c r="J8" s="121">
+      <c r="J8" s="107">
         <f>COUNTIF(B8:I8,"✓")</f>
         <v/>
       </c>
-      <c r="K8" s="124">
+      <c r="K8" s="110">
         <f>IF(J8&gt;0,VLOOKUP(A8,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
         <v/>
       </c>
-      <c r="L8" s="124">
+      <c r="L8" s="110">
         <f>IF(J8&gt;0,VLOOKUP(A8,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
         <v/>
       </c>
+      <c r="M8" s="111">
+        <f>IF(A8="","",COUNTIF($A$7:$A$7,A8)+COUNTIF($A$9:$A$15,A8))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="122" t="inlineStr">
-        <is>
-          <t>Local Hiking (Griffith)</t>
-        </is>
-      </c>
-      <c r="B9" s="123" t="inlineStr"/>
-      <c r="C9" s="123" t="inlineStr"/>
-      <c r="D9" s="123" t="inlineStr"/>
-      <c r="E9" s="123" t="inlineStr"/>
-      <c r="F9" s="123" t="inlineStr"/>
-      <c r="G9" s="123" t="inlineStr"/>
-      <c r="H9" s="123" t="inlineStr"/>
-      <c r="I9" s="123" t="inlineStr"/>
-      <c r="J9" s="121">
+      <c r="A9" s="109" t="inlineStr">
+        <is>
+          <t>Local Hiking (Griffith/Runyon)</t>
+        </is>
+      </c>
+      <c r="B9" s="81" t="inlineStr"/>
+      <c r="C9" s="81" t="inlineStr"/>
+      <c r="D9" s="81" t="inlineStr"/>
+      <c r="E9" s="81" t="inlineStr"/>
+      <c r="F9" s="81" t="inlineStr"/>
+      <c r="G9" s="81" t="inlineStr"/>
+      <c r="H9" s="81" t="inlineStr"/>
+      <c r="I9" s="81" t="inlineStr"/>
+      <c r="J9" s="107">
         <f>COUNTIF(B9:I9,"✓")</f>
         <v/>
       </c>
-      <c r="K9" s="124">
+      <c r="K9" s="110">
         <f>IF(J9&gt;0,VLOOKUP(A9,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
         <v/>
       </c>
-      <c r="L9" s="124">
+      <c r="L9" s="110">
         <f>IF(J9&gt;0,VLOOKUP(A9,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
         <v/>
       </c>
+      <c r="M9" s="111">
+        <f>IF(A9="","",COUNTIF($A$7:$A$8,A9)+COUNTIF($A$10:$A$15,A9))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="118" t="inlineStr">
+      <c r="A10" s="108" t="inlineStr">
         <is>
           <t>Beach/Surf Lesson</t>
         </is>
@@ -6570,48 +6483,56 @@
       <c r="G10" s="81" t="inlineStr"/>
       <c r="H10" s="81" t="inlineStr"/>
       <c r="I10" s="81" t="inlineStr"/>
-      <c r="J10" s="121">
+      <c r="J10" s="107">
         <f>COUNTIF(B10:I10,"✓")</f>
         <v/>
       </c>
-      <c r="K10" s="124">
+      <c r="K10" s="110">
         <f>IF(J10&gt;0,VLOOKUP(A10,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
         <v/>
       </c>
-      <c r="L10" s="124">
+      <c r="L10" s="110">
         <f>IF(J10&gt;0,VLOOKUP(A10,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
         <v/>
       </c>
+      <c r="M10" s="111">
+        <f>IF(A10="","",COUNTIF($A$7:$A$9,A10)+COUNTIF($A$11:$A$15,A10))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="125" t="inlineStr">
+      <c r="A11" s="109" t="inlineStr">
         <is>
           <t>(New Activity 5)</t>
         </is>
       </c>
-      <c r="B11" s="123" t="inlineStr"/>
-      <c r="C11" s="123" t="inlineStr"/>
-      <c r="D11" s="123" t="inlineStr"/>
-      <c r="E11" s="123" t="inlineStr"/>
-      <c r="F11" s="123" t="inlineStr"/>
-      <c r="G11" s="123" t="inlineStr"/>
-      <c r="H11" s="123" t="inlineStr"/>
-      <c r="I11" s="123" t="inlineStr"/>
-      <c r="J11" s="121">
+      <c r="B11" s="81" t="inlineStr"/>
+      <c r="C11" s="81" t="inlineStr"/>
+      <c r="D11" s="81" t="inlineStr"/>
+      <c r="E11" s="81" t="inlineStr"/>
+      <c r="F11" s="81" t="inlineStr"/>
+      <c r="G11" s="81" t="inlineStr"/>
+      <c r="H11" s="81" t="inlineStr"/>
+      <c r="I11" s="81" t="inlineStr"/>
+      <c r="J11" s="107">
         <f>COUNTIF(B11:I11,"✓")</f>
         <v/>
       </c>
-      <c r="K11" s="126">
+      <c r="K11" s="112">
         <f>IF(J11&gt;0,VLOOKUP(A11,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
         <v/>
       </c>
-      <c r="L11" s="126">
+      <c r="L11" s="112">
         <f>IF(J11&gt;0,VLOOKUP(A11,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
         <v/>
       </c>
+      <c r="M11" s="111">
+        <f>IF(A11="","",COUNTIF($A$7:$A$10,A11)+COUNTIF($A$12:$A$15,A11))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="120" t="inlineStr">
+      <c r="A12" s="108" t="inlineStr">
         <is>
           <t>(New Activity 6)</t>
         </is>
@@ -6624,48 +6545,56 @@
       <c r="G12" s="81" t="inlineStr"/>
       <c r="H12" s="81" t="inlineStr"/>
       <c r="I12" s="81" t="inlineStr"/>
-      <c r="J12" s="121">
+      <c r="J12" s="107">
         <f>COUNTIF(B12:I12,"✓")</f>
         <v/>
       </c>
-      <c r="K12" s="126">
+      <c r="K12" s="112">
         <f>IF(J12&gt;0,VLOOKUP(A12,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
         <v/>
       </c>
-      <c r="L12" s="126">
+      <c r="L12" s="112">
         <f>IF(J12&gt;0,VLOOKUP(A12,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
         <v/>
       </c>
+      <c r="M12" s="111">
+        <f>IF(A12="","",COUNTIF($A$7:$A$11,A12)+COUNTIF($A$13:$A$15,A12))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="125" t="inlineStr">
+      <c r="A13" s="109" t="inlineStr">
         <is>
           <t>(New Activity 7)</t>
         </is>
       </c>
-      <c r="B13" s="123" t="inlineStr"/>
-      <c r="C13" s="123" t="inlineStr"/>
-      <c r="D13" s="123" t="inlineStr"/>
-      <c r="E13" s="123" t="inlineStr"/>
-      <c r="F13" s="123" t="inlineStr"/>
-      <c r="G13" s="123" t="inlineStr"/>
-      <c r="H13" s="123" t="inlineStr"/>
-      <c r="I13" s="123" t="inlineStr"/>
-      <c r="J13" s="121">
+      <c r="B13" s="81" t="inlineStr"/>
+      <c r="C13" s="81" t="inlineStr"/>
+      <c r="D13" s="81" t="inlineStr"/>
+      <c r="E13" s="81" t="inlineStr"/>
+      <c r="F13" s="81" t="inlineStr"/>
+      <c r="G13" s="81" t="inlineStr"/>
+      <c r="H13" s="81" t="inlineStr"/>
+      <c r="I13" s="81" t="inlineStr"/>
+      <c r="J13" s="107">
         <f>COUNTIF(B13:I13,"✓")</f>
         <v/>
       </c>
-      <c r="K13" s="126">
+      <c r="K13" s="112">
         <f>IF(J13&gt;0,VLOOKUP(A13,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
         <v/>
       </c>
-      <c r="L13" s="126">
+      <c r="L13" s="112">
         <f>IF(J13&gt;0,VLOOKUP(A13,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
         <v/>
       </c>
+      <c r="M13" s="111">
+        <f>IF(A13="","",COUNTIF($A$7:$A$12,A13)+COUNTIF($A$14:$A$15,A13))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="120" t="inlineStr">
+      <c r="A14" s="108" t="inlineStr">
         <is>
           <t>(New Activity 8)</t>
         </is>
@@ -6678,61 +6607,69 @@
       <c r="G14" s="81" t="inlineStr"/>
       <c r="H14" s="81" t="inlineStr"/>
       <c r="I14" s="81" t="inlineStr"/>
-      <c r="J14" s="121">
+      <c r="J14" s="107">
         <f>COUNTIF(B14:I14,"✓")</f>
         <v/>
       </c>
-      <c r="K14" s="126">
+      <c r="K14" s="112">
         <f>IF(J14&gt;0,VLOOKUP(A14,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
         <v/>
       </c>
-      <c r="L14" s="126">
+      <c r="L14" s="112">
         <f>IF(J14&gt;0,VLOOKUP(A14,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
         <v/>
       </c>
+      <c r="M14" s="111">
+        <f>IF(A14="","",COUNTIF($A$7:$A$13,A14)+COUNTIF($A$15:$A$15,A14))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="125" t="inlineStr">
+      <c r="A15" s="109" t="inlineStr">
         <is>
           <t>(New Activity 9)</t>
         </is>
       </c>
-      <c r="B15" s="123" t="inlineStr"/>
-      <c r="C15" s="123" t="inlineStr"/>
-      <c r="D15" s="123" t="inlineStr"/>
-      <c r="E15" s="123" t="inlineStr"/>
-      <c r="F15" s="123" t="inlineStr"/>
-      <c r="G15" s="123" t="inlineStr"/>
-      <c r="H15" s="123" t="inlineStr"/>
-      <c r="I15" s="123" t="inlineStr"/>
-      <c r="J15" s="121">
+      <c r="B15" s="81" t="inlineStr"/>
+      <c r="C15" s="81" t="inlineStr"/>
+      <c r="D15" s="81" t="inlineStr"/>
+      <c r="E15" s="81" t="inlineStr"/>
+      <c r="F15" s="81" t="inlineStr"/>
+      <c r="G15" s="81" t="inlineStr"/>
+      <c r="H15" s="81" t="inlineStr"/>
+      <c r="I15" s="81" t="inlineStr"/>
+      <c r="J15" s="107">
         <f>COUNTIF(B15:I15,"✓")</f>
         <v/>
       </c>
-      <c r="K15" s="126">
+      <c r="K15" s="112">
         <f>IF(J15&gt;0,VLOOKUP(A15,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
         <v/>
       </c>
-      <c r="L15" s="126">
+      <c r="L15" s="112">
         <f>IF(J15&gt;0,VLOOKUP(A15,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
         <v/>
       </c>
+      <c r="M15" s="111">
+        <f>IF(A15="","",COUNTIF($A$7:$A$14,A15)+COUNTIF($A$16:$A$15,A15))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="127" t="inlineStr">
+      <c r="A16" s="113" t="inlineStr">
         <is>
           <t>📌 TOTALS</t>
         </is>
       </c>
-      <c r="B16" s="128" t="inlineStr"/>
-      <c r="C16" s="128" t="inlineStr"/>
-      <c r="D16" s="128" t="inlineStr"/>
-      <c r="E16" s="128" t="inlineStr"/>
-      <c r="F16" s="128" t="inlineStr"/>
-      <c r="G16" s="128" t="inlineStr"/>
-      <c r="H16" s="128" t="inlineStr"/>
-      <c r="I16" s="128" t="inlineStr"/>
-      <c r="J16" s="129">
+      <c r="B16" s="114" t="inlineStr"/>
+      <c r="C16" s="114" t="inlineStr"/>
+      <c r="D16" s="114" t="inlineStr"/>
+      <c r="E16" s="114" t="inlineStr"/>
+      <c r="F16" s="114" t="inlineStr"/>
+      <c r="G16" s="114" t="inlineStr"/>
+      <c r="H16" s="114" t="inlineStr"/>
+      <c r="I16" s="114" t="inlineStr"/>
+      <c r="J16" s="88">
         <f>SUM(J7:J15)</f>
         <v/>
       </c>
@@ -6746,22 +6683,22 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="101" t="inlineStr">
+      <c r="A18" s="103" t="inlineStr">
         <is>
           <t>👤 PER-PERSON ACTIVITY COST</t>
         </is>
       </c>
-      <c r="B18" s="102" t="n"/>
-      <c r="C18" s="102" t="n"/>
-      <c r="D18" s="102" t="n"/>
-      <c r="E18" s="102" t="n"/>
-      <c r="F18" s="102" t="n"/>
-      <c r="G18" s="102" t="n"/>
-      <c r="H18" s="102" t="n"/>
-      <c r="I18" s="102" t="n"/>
-      <c r="J18" s="102" t="n"/>
-      <c r="K18" s="102" t="n"/>
-      <c r="L18" s="102" t="n"/>
+      <c r="B18" s="104" t="n"/>
+      <c r="C18" s="104" t="n"/>
+      <c r="D18" s="104" t="n"/>
+      <c r="E18" s="104" t="n"/>
+      <c r="F18" s="104" t="n"/>
+      <c r="G18" s="104" t="n"/>
+      <c r="H18" s="104" t="n"/>
+      <c r="I18" s="104" t="n"/>
+      <c r="J18" s="104" t="n"/>
+      <c r="K18" s="104" t="n"/>
+      <c r="L18" s="104" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="98" t="inlineStr">
@@ -6771,174 +6708,211 @@
       </c>
       <c r="B19" s="98" t="inlineStr">
         <is>
-          <t>Activity Cost</t>
+          <t># Activities</t>
         </is>
       </c>
       <c r="C19" s="98" t="inlineStr">
         <is>
-          <t>Activity Sell</t>
+          <t>Cost</t>
         </is>
       </c>
       <c r="D19" s="98" t="inlineStr">
         <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="E19" s="98" t="inlineStr">
+        <is>
           <t>Margin</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="118" t="inlineStr">
+      <c r="A20" s="108" t="inlineStr">
         <is>
           <t>참가자1</t>
         </is>
       </c>
-      <c r="B20" s="124">
+      <c r="B20" s="107">
+        <f>COUNTIF(B7:B15,"✓")</f>
+        <v/>
+      </c>
+      <c r="C20" s="110">
         <f>SUMPRODUCT((B7:B15="✓")*1,K7:K15)</f>
         <v/>
       </c>
-      <c r="C20" s="124">
+      <c r="D20" s="110">
         <f>SUMPRODUCT((B7:B15="✓")*1,L7:L15)</f>
         <v/>
       </c>
-      <c r="D20" s="124">
-        <f>C20-B20</f>
+      <c r="E20" s="110">
+        <f>D20-C20</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="118" t="inlineStr">
+      <c r="A21" s="108" t="inlineStr">
         <is>
           <t>참가자2</t>
         </is>
       </c>
-      <c r="B21" s="124">
+      <c r="B21" s="107">
+        <f>COUNTIF(C7:C15,"✓")</f>
+        <v/>
+      </c>
+      <c r="C21" s="110">
         <f>SUMPRODUCT((C7:C15="✓")*1,K7:K15)</f>
         <v/>
       </c>
-      <c r="C21" s="124">
+      <c r="D21" s="110">
         <f>SUMPRODUCT((C7:C15="✓")*1,L7:L15)</f>
         <v/>
       </c>
-      <c r="D21" s="124">
-        <f>C21-B21</f>
+      <c r="E21" s="110">
+        <f>D21-C21</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="118" t="inlineStr">
+      <c r="A22" s="108" t="inlineStr">
         <is>
           <t>참가자3</t>
         </is>
       </c>
-      <c r="B22" s="124">
+      <c r="B22" s="107">
+        <f>COUNTIF(D7:D15,"✓")</f>
+        <v/>
+      </c>
+      <c r="C22" s="110">
         <f>SUMPRODUCT((D7:D15="✓")*1,K7:K15)</f>
         <v/>
       </c>
-      <c r="C22" s="124">
+      <c r="D22" s="110">
         <f>SUMPRODUCT((D7:D15="✓")*1,L7:L15)</f>
         <v/>
       </c>
-      <c r="D22" s="124">
-        <f>C22-B22</f>
+      <c r="E22" s="110">
+        <f>D22-C22</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="118" t="inlineStr">
+      <c r="A23" s="108" t="inlineStr">
         <is>
           <t>참가자4</t>
         </is>
       </c>
-      <c r="B23" s="124">
+      <c r="B23" s="107">
+        <f>COUNTIF(E7:E15,"✓")</f>
+        <v/>
+      </c>
+      <c r="C23" s="110">
         <f>SUMPRODUCT((E7:E15="✓")*1,K7:K15)</f>
         <v/>
       </c>
-      <c r="C23" s="124">
+      <c r="D23" s="110">
         <f>SUMPRODUCT((E7:E15="✓")*1,L7:L15)</f>
         <v/>
       </c>
-      <c r="D23" s="124">
-        <f>C23-B23</f>
+      <c r="E23" s="110">
+        <f>D23-C23</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="118" t="inlineStr">
+      <c r="A24" s="108" t="inlineStr">
         <is>
           <t>참가자5</t>
         </is>
       </c>
-      <c r="B24" s="124">
+      <c r="B24" s="107">
+        <f>COUNTIF(F7:F15,"✓")</f>
+        <v/>
+      </c>
+      <c r="C24" s="110">
         <f>SUMPRODUCT((F7:F15="✓")*1,K7:K15)</f>
         <v/>
       </c>
-      <c r="C24" s="124">
+      <c r="D24" s="110">
         <f>SUMPRODUCT((F7:F15="✓")*1,L7:L15)</f>
         <v/>
       </c>
-      <c r="D24" s="124">
-        <f>C24-B24</f>
+      <c r="E24" s="110">
+        <f>D24-C24</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="118" t="inlineStr">
+      <c r="A25" s="108" t="inlineStr">
         <is>
           <t>참가자6</t>
         </is>
       </c>
-      <c r="B25" s="124">
+      <c r="B25" s="107">
+        <f>COUNTIF(G7:G15,"✓")</f>
+        <v/>
+      </c>
+      <c r="C25" s="110">
         <f>SUMPRODUCT((G7:G15="✓")*1,K7:K15)</f>
         <v/>
       </c>
-      <c r="C25" s="124">
+      <c r="D25" s="110">
         <f>SUMPRODUCT((G7:G15="✓")*1,L7:L15)</f>
         <v/>
       </c>
-      <c r="D25" s="124">
-        <f>C25-B25</f>
+      <c r="E25" s="110">
+        <f>D25-C25</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="118" t="inlineStr">
+      <c r="A26" s="108" t="inlineStr">
         <is>
           <t>참가자7</t>
         </is>
       </c>
-      <c r="B26" s="124">
+      <c r="B26" s="107">
+        <f>COUNTIF(H7:H15,"✓")</f>
+        <v/>
+      </c>
+      <c r="C26" s="110">
         <f>SUMPRODUCT((H7:H15="✓")*1,K7:K15)</f>
         <v/>
       </c>
-      <c r="C26" s="124">
+      <c r="D26" s="110">
         <f>SUMPRODUCT((H7:H15="✓")*1,L7:L15)</f>
         <v/>
       </c>
-      <c r="D26" s="124">
-        <f>C26-B26</f>
+      <c r="E26" s="110">
+        <f>D26-C26</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="118" t="inlineStr">
+      <c r="A27" s="108" t="inlineStr">
         <is>
           <t>참가자8</t>
         </is>
       </c>
-      <c r="B27" s="124">
+      <c r="B27" s="107">
+        <f>COUNTIF(I7:I15,"✓")</f>
+        <v/>
+      </c>
+      <c r="C27" s="110">
         <f>SUMPRODUCT((I7:I15="✓")*1,K7:K15)</f>
         <v/>
       </c>
-      <c r="C27" s="124">
+      <c r="D27" s="110">
         <f>SUMPRODUCT((I7:I15="✓")*1,L7:L15)</f>
         <v/>
       </c>
-      <c r="D27" s="124">
-        <f>C27-B27</f>
+      <c r="E27" s="110">
+        <f>D27-C27</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="130" t="inlineStr">
+      <c r="A28" s="115" t="inlineStr">
         <is>
           <t>📌 TOTAL</t>
         </is>
@@ -6955,34 +6929,90 @@
         <f>SUM(D20:D27)</f>
         <v/>
       </c>
+      <c r="E28" s="88">
+        <f>SUM(E20:E27)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="131" t="inlineStr">
+      <c r="A29" s="116" t="inlineStr">
         <is>
           <t>✓Check (0=OK):</t>
         </is>
       </c>
-      <c r="B29" s="112">
-        <f>B28-K16</f>
-        <v/>
-      </c>
-      <c r="C29" s="113" t="inlineStr"/>
-      <c r="D29" s="113">
-        <f>IF(B29=0,"✅ 정확","❌ 불일치")</f>
+      <c r="C29" s="117">
+        <f>C28-K16</f>
+        <v/>
+      </c>
+      <c r="D29" s="118">
+        <f>IF(C29=0,"✅ 정확","❌ 불일치")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
     <mergeCell ref="A18:L18"/>
   </mergeCells>
-  <conditionalFormatting sqref="B29">
-    <cfRule type="cellIs" priority="1" operator="notEqual" dxfId="0">
+  <conditionalFormatting sqref="M7">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="M8">
+    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M9">
+    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M10">
+    <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M11">
+    <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M12">
+    <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M13">
+    <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M14">
+    <cfRule type="cellIs" priority="8" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M15">
+    <cfRule type="cellIs" priority="9" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C29">
+    <cfRule type="cellIs" priority="10" operator="notEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="A7 A8 A9 A10 A11 A12 A13 A14 A15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 액티비티를 선택하세요" type="list">
+      <formula1>'Master Data'!$A$86:$A$94</formula1>
+    </dataValidation>
+    <dataValidation sqref="B7 B8 B9 B10 B11 B12 B13 B14 B15 C7 C8 C9 C10 C11 C12 C13 C14 C15 D7 D8 D9 D10 D11 D12 D13 D14 D15 E7 E8 E9 E10 E11 E12 E13 E14 E15 F7 F8 F9 F10 F11 F12 F13 F14 F15 G7 G8 G9 G10 G11 G12 G13 G14 G15 H7 H8 H9 H10 H11 H12 H13 H14 H15 I7 I8 I9 I10 I11 I12 I13 I14 I15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓,"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7005,26 +7035,26 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="101" t="inlineStr">
+      <c r="A1" s="103" t="inlineStr">
         <is>
           <t>📊 PROFIT SUMMARY 2 — Activity Sub-Category Breakdown</t>
         </is>
       </c>
-      <c r="B1" s="102" t="n"/>
-      <c r="C1" s="102" t="n"/>
-      <c r="D1" s="102" t="n"/>
-      <c r="E1" s="102" t="n"/>
-      <c r="F1" s="102" t="n"/>
+      <c r="B1" s="104" t="n"/>
+      <c r="C1" s="104" t="n"/>
+      <c r="D1" s="104" t="n"/>
+      <c r="E1" s="104" t="n"/>
+      <c r="F1" s="104" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="120" t="inlineStr">
-        <is>
-          <t>⬇️ 'Package Selector 2' 체크마크 기반 → 활동별·참가자별 자동 분석</t>
+      <c r="A2" s="105" t="inlineStr">
+        <is>
+          <t>⬇️ 'Package Selector 2' ✓체크 기반 자동 분석 | Sports/Outdoor 서브카테고리 분류</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="132" t="inlineStr">
+      <c r="A4" s="119" t="inlineStr">
         <is>
           <t>Category / Activity</t>
         </is>
@@ -7056,24 +7086,24 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="133" t="inlineStr">
+      <c r="A5" s="120" t="inlineStr">
         <is>
           <t>🎫 SPORTS &amp; EVENTS</t>
         </is>
       </c>
-      <c r="B5" s="134" t="n"/>
-      <c r="C5" s="134" t="n"/>
-      <c r="D5" s="134" t="n"/>
-      <c r="E5" s="134" t="n"/>
-      <c r="F5" s="134" t="n"/>
+      <c r="B5" s="121" t="n"/>
+      <c r="C5" s="121" t="n"/>
+      <c r="D5" s="121" t="n"/>
+      <c r="E5" s="121" t="n"/>
+      <c r="F5" s="121" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="118" t="inlineStr">
+      <c r="A6" s="108" t="inlineStr">
         <is>
           <t xml:space="preserve">  NBA/MLB Game (Ticket)</t>
         </is>
       </c>
-      <c r="B6" s="135">
+      <c r="B6" s="122">
         <f>'Package Selector 2'!J7</f>
         <v/>
       </c>
@@ -7095,12 +7125,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="118" t="inlineStr">
+      <c r="A7" s="108" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sports Bar Experience</t>
         </is>
       </c>
-      <c r="B7" s="135">
+      <c r="B7" s="122">
         <f>'Package Selector 2'!J8</f>
         <v/>
       </c>
@@ -7122,7 +7152,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="136" t="inlineStr">
+      <c r="A8" s="123" t="inlineStr">
         <is>
           <t xml:space="preserve">  SPORTS SUBTOTAL</t>
         </is>
@@ -7141,24 +7171,24 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="133" t="inlineStr">
+      <c r="A10" s="120" t="inlineStr">
         <is>
           <t>🌿 OUTDOOR &amp; NATURE</t>
         </is>
       </c>
-      <c r="B10" s="134" t="n"/>
-      <c r="C10" s="134" t="n"/>
-      <c r="D10" s="134" t="n"/>
-      <c r="E10" s="134" t="n"/>
-      <c r="F10" s="134" t="n"/>
+      <c r="B10" s="121" t="n"/>
+      <c r="C10" s="121" t="n"/>
+      <c r="D10" s="121" t="n"/>
+      <c r="E10" s="121" t="n"/>
+      <c r="F10" s="121" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="118" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Local Hiking (Griffith)</t>
-        </is>
-      </c>
-      <c r="B11" s="135">
+      <c r="A11" s="108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Local Hiking (Griffith/Runyon)</t>
+        </is>
+      </c>
+      <c r="B11" s="122">
         <f>'Package Selector 2'!J9</f>
         <v/>
       </c>
@@ -7180,12 +7210,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="118" t="inlineStr">
+      <c r="A12" s="108" t="inlineStr">
         <is>
           <t xml:space="preserve">  Beach/Surf Lesson</t>
         </is>
       </c>
-      <c r="B12" s="135">
+      <c r="B12" s="122">
         <f>'Package Selector 2'!J10</f>
         <v/>
       </c>
@@ -7207,7 +7237,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="136" t="inlineStr">
+      <c r="A13" s="123" t="inlineStr">
         <is>
           <t xml:space="preserve">  OUTDOOR SUBTOTAL</t>
         </is>
@@ -7226,19 +7256,19 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="101" t="inlineStr">
+      <c r="A15" s="103" t="inlineStr">
         <is>
           <t>🏆 ACTIVITIES GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="102" t="n"/>
-      <c r="C15" s="102" t="n"/>
-      <c r="D15" s="102" t="n"/>
-      <c r="E15" s="102" t="n"/>
-      <c r="F15" s="102" t="n"/>
+      <c r="B15" s="104" t="n"/>
+      <c r="C15" s="104" t="n"/>
+      <c r="D15" s="104" t="n"/>
+      <c r="E15" s="104" t="n"/>
+      <c r="F15" s="104" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="110" t="inlineStr">
+      <c r="A16" s="106" t="inlineStr">
         <is>
           <t>📌 TOTAL ALL ACTIVITIES</t>
         </is>
@@ -7257,19 +7287,19 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="115" t="inlineStr">
+      <c r="A18" s="124" t="inlineStr">
         <is>
           <t>🔍 CROSS-CHECK vs Package Selector</t>
         </is>
       </c>
-      <c r="B18" s="116" t="n"/>
-      <c r="C18" s="116" t="n"/>
-      <c r="D18" s="116" t="n"/>
-      <c r="E18" s="116" t="n"/>
-      <c r="F18" s="116" t="n"/>
+      <c r="B18" s="125" t="n"/>
+      <c r="C18" s="125" t="n"/>
+      <c r="D18" s="125" t="n"/>
+      <c r="E18" s="125" t="n"/>
+      <c r="F18" s="125" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="137" t="inlineStr">
+      <c r="A19" s="126" t="inlineStr">
         <is>
           <t>Package Selector Activities Cost:</t>
         </is>
@@ -7280,7 +7310,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="137" t="inlineStr">
+      <c r="A20" s="126" t="inlineStr">
         <is>
           <t>Package Selector 2 Activities Cost:</t>
         </is>
@@ -7291,16 +7321,16 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="131" t="inlineStr">
+      <c r="A21" s="116" t="inlineStr">
         <is>
           <t>Difference:</t>
         </is>
       </c>
-      <c r="D21" s="138">
+      <c r="D21" s="117">
         <f>D20-D19</f>
         <v/>
       </c>
-      <c r="E21" s="113">
+      <c r="E21" s="118">
         <f>IF(D21=0,"✅ MATCH","❌ MISMATCH — check selections")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
feat: PS2 full rebuild - all 6 categories, dropdowns w/ duplicate detection, per-person SUMPRODUCT, PF2 category+person breakdown
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -253,7 +253,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -473,11 +473,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF333333"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF333333"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -809,11 +820,44 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <font>
         <b val="1"/>
@@ -830,6 +874,14 @@
       <font>
         <color rgb="009C0006"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFC7CE"/>
@@ -6246,7 +6298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:P86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="42" min="1" max="1"/>
@@ -6258,15 +6310,17 @@
     <col width="11" customWidth="1" style="42" min="7" max="7"/>
     <col width="11" customWidth="1" style="42" min="8" max="8"/>
     <col width="11" customWidth="1" style="42" min="9" max="9"/>
-    <col width="13" customWidth="1" style="42" min="10" max="10"/>
-    <col width="13" customWidth="1" style="42" min="11" max="11"/>
-    <col width="13" customWidth="1" style="42" min="12" max="12"/>
+    <col width="10" customWidth="1" style="42" min="10" max="10"/>
+    <col width="12" customWidth="1" style="42" min="11" max="11"/>
+    <col width="12" customWidth="1" style="42" min="12" max="12"/>
+    <col hidden="1" width="13" customWidth="1" style="42" min="15" max="15"/>
+    <col hidden="1" width="13" customWidth="1" style="42" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="103" t="inlineStr">
         <is>
-          <t>🎯 ACTIVITY SELECTOR — Per Person</t>
+          <t>🎯 PACKAGE SELECTOR 2 — Per Person Custom Builder</t>
         </is>
       </c>
       <c r="B1" s="104" t="n"/>
@@ -6284,7 +6338,7 @@
     <row r="2">
       <c r="A2" s="105" t="inlineStr">
         <is>
-          <t>참가자 컬럼에 ✓ 체크 → 자동 비용계산 → Profit Summary 2 반영 | 중복선택 시 ⚠️ 표시</t>
+          <t>참가자 컬럼에 ✓ 체크 → 개인별 패키지 자동구성 → 비용계산 → Profit Summary 2 반영</t>
         </is>
       </c>
     </row>
@@ -6303,11 +6357,20 @@
           <t>persons</t>
         </is>
       </c>
+      <c r="H4" s="106" t="inlineStr">
+        <is>
+          <t>⚠️ 중복항목</t>
+        </is>
+      </c>
+      <c r="I4" s="127">
+        <f>COUNTIF(O:O,"&gt;0")&amp;"건"</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="98" t="inlineStr">
-        <is>
-          <t>Activity \ Person</t>
+      <c r="A6" s="119" t="inlineStr">
+        <is>
+          <t>Category / Item</t>
         </is>
       </c>
       <c r="B6" s="98" t="inlineStr">
@@ -6352,7 +6415,7 @@
       </c>
       <c r="J6" s="98" t="inlineStr">
         <is>
-          <t>✓ Count</t>
+          <t>Qty/p</t>
         </is>
       </c>
       <c r="K6" s="98" t="inlineStr">
@@ -6365,83 +6428,91 @@
           <t>Sell/P</t>
         </is>
       </c>
-      <c r="M6" s="98" t="inlineStr">
-        <is>
-          <t>⚠️ Dup</t>
-        </is>
-      </c>
-      <c r="N6" s="98" t="inlineStr">
-        <is>
-          <t>Available Activities</t>
-        </is>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" s="109" t="inlineStr">
-        <is>
-          <t>NBA/MLB Game (Ticket)</t>
-        </is>
-      </c>
-      <c r="B7" s="81" t="inlineStr"/>
-      <c r="C7" s="81" t="inlineStr"/>
-      <c r="D7" s="81" t="inlineStr"/>
-      <c r="E7" s="81" t="inlineStr"/>
-      <c r="F7" s="81" t="inlineStr"/>
-      <c r="G7" s="81" t="inlineStr"/>
-      <c r="H7" s="81" t="inlineStr"/>
-      <c r="I7" s="81" t="inlineStr"/>
-      <c r="J7" s="107">
-        <f>COUNTIF(B7:I7,"✓")</f>
-        <v/>
-      </c>
-      <c r="K7" s="110">
-        <f>IF(J7&gt;0,VLOOKUP(A7,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="L7" s="110">
-        <f>IF(J7&gt;0,VLOOKUP(A7,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M7" s="111">
-        <f>IF(A7="","",COUNTIF($A$7:$A$6,A7)+COUNTIF($A$8:$A$15,A7))</f>
-        <v/>
-      </c>
+      <c r="A7" s="128" t="inlineStr">
+        <is>
+          <t>⛳ GOLF (1인 1라운드)</t>
+        </is>
+      </c>
+      <c r="B7" s="77" t="n"/>
+      <c r="C7" s="77" t="n"/>
+      <c r="D7" s="77" t="n"/>
+      <c r="E7" s="77" t="n"/>
+      <c r="F7" s="77" t="n"/>
+      <c r="G7" s="77" t="n"/>
+      <c r="H7" s="77" t="n"/>
+      <c r="I7" s="77" t="n"/>
+      <c r="J7" s="77" t="n"/>
+      <c r="K7" s="77" t="n"/>
+      <c r="L7" s="77" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="108" t="inlineStr">
-        <is>
-          <t>Sports Bar Experience</t>
-        </is>
-      </c>
-      <c r="B8" s="81" t="inlineStr"/>
-      <c r="C8" s="81" t="inlineStr"/>
-      <c r="D8" s="81" t="inlineStr"/>
-      <c r="E8" s="81" t="inlineStr"/>
-      <c r="F8" s="81" t="inlineStr"/>
-      <c r="G8" s="81" t="inlineStr"/>
-      <c r="H8" s="81" t="inlineStr"/>
-      <c r="I8" s="81" t="inlineStr"/>
-      <c r="J8" s="107">
-        <f>COUNTIF(B8:I8,"✓")</f>
-        <v/>
-      </c>
-      <c r="K8" s="110">
-        <f>IF(J8&gt;0,VLOOKUP(A8,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="L8" s="110">
-        <f>IF(J8&gt;0,VLOOKUP(A8,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M8" s="111">
-        <f>IF(A8="","",COUNTIF($A$7:$A$7,A8)+COUNTIF($A$9:$A$15,A8))</f>
-        <v/>
+      <c r="A8" s="119" t="inlineStr">
+        <is>
+          <t>Item (Select ▼)</t>
+        </is>
+      </c>
+      <c r="B8" s="98" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C8" s="98" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D8" s="98" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E8" s="98" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="F8" s="98" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="G8" s="98" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="H8" s="98" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="I8" s="98" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="J8" s="98" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="K8" s="98" t="inlineStr">
+        <is>
+          <t>Cost/P</t>
+        </is>
+      </c>
+      <c r="L8" s="98" t="inlineStr">
+        <is>
+          <t>Sell/P</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="109" t="inlineStr">
         <is>
-          <t>Local Hiking (Griffith/Runyon)</t>
+          <t>Trump National LA</t>
         </is>
       </c>
       <c r="B9" s="81" t="inlineStr"/>
@@ -6452,27 +6523,29 @@
       <c r="G9" s="81" t="inlineStr"/>
       <c r="H9" s="81" t="inlineStr"/>
       <c r="I9" s="81" t="inlineStr"/>
-      <c r="J9" s="107">
-        <f>COUNTIF(B9:I9,"✓")</f>
-        <v/>
-      </c>
-      <c r="K9" s="110">
-        <f>IF(J9&gt;0,VLOOKUP(A9,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="L9" s="110">
-        <f>IF(J9&gt;0,VLOOKUP(A9,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M9" s="111">
-        <f>IF(A9="","",COUNTIF($A$7:$A$8,A9)+COUNTIF($A$10:$A$15,A9))</f>
-        <v/>
+      <c r="J9" s="83" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="84">
+        <f>IF(A9="","",VLOOKUP(A9,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L9" s="84">
+        <f>IF(A9="","",VLOOKUP(A9,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O9" s="81">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="P9" s="81" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="108" t="inlineStr">
         <is>
-          <t>Beach/Surf Lesson</t>
+          <t>Sandpiper GC</t>
         </is>
       </c>
       <c r="B10" s="81" t="inlineStr"/>
@@ -6483,27 +6556,29 @@
       <c r="G10" s="81" t="inlineStr"/>
       <c r="H10" s="81" t="inlineStr"/>
       <c r="I10" s="81" t="inlineStr"/>
-      <c r="J10" s="107">
-        <f>COUNTIF(B10:I10,"✓")</f>
-        <v/>
-      </c>
-      <c r="K10" s="110">
-        <f>IF(J10&gt;0,VLOOKUP(A10,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="L10" s="110">
-        <f>IF(J10&gt;0,VLOOKUP(A10,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M10" s="111">
-        <f>IF(A10="","",COUNTIF($A$7:$A$9,A10)+COUNTIF($A$11:$A$15,A10))</f>
-        <v/>
+      <c r="J10" s="83" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="84">
+        <f>IF(A10="","",VLOOKUP(A10,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L10" s="84">
+        <f>IF(A10="","",VLOOKUP(A10,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O10" s="81">
+        <f>IF(A10="",0,COUNTIF(A$9:A9,A10))</f>
+        <v/>
+      </c>
+      <c r="P10" s="81" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="109" t="inlineStr">
         <is>
-          <t>(New Activity 5)</t>
+          <t>Hidden Valley GC</t>
         </is>
       </c>
       <c r="B11" s="81" t="inlineStr"/>
@@ -6514,29 +6589,27 @@
       <c r="G11" s="81" t="inlineStr"/>
       <c r="H11" s="81" t="inlineStr"/>
       <c r="I11" s="81" t="inlineStr"/>
-      <c r="J11" s="107">
-        <f>COUNTIF(B11:I11,"✓")</f>
-        <v/>
-      </c>
-      <c r="K11" s="112">
-        <f>IF(J11&gt;0,VLOOKUP(A11,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="L11" s="112">
-        <f>IF(J11&gt;0,VLOOKUP(A11,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M11" s="111">
-        <f>IF(A11="","",COUNTIF($A$7:$A$10,A11)+COUNTIF($A$12:$A$15,A11))</f>
-        <v/>
+      <c r="J11" s="83" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="84">
+        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L11" s="84">
+        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O11" s="81">
+        <f>IF(A11="",0,COUNTIF(A$9:A10,A11))</f>
+        <v/>
+      </c>
+      <c r="P11" s="81" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="108" t="inlineStr">
-        <is>
-          <t>(New Activity 6)</t>
-        </is>
-      </c>
+      <c r="A12" s="129" t="inlineStr"/>
       <c r="B12" s="81" t="inlineStr"/>
       <c r="C12" s="81" t="inlineStr"/>
       <c r="D12" s="81" t="inlineStr"/>
@@ -6545,29 +6618,25 @@
       <c r="G12" s="81" t="inlineStr"/>
       <c r="H12" s="81" t="inlineStr"/>
       <c r="I12" s="81" t="inlineStr"/>
-      <c r="J12" s="107">
-        <f>COUNTIF(B12:I12,"✓")</f>
-        <v/>
-      </c>
-      <c r="K12" s="112">
-        <f>IF(J12&gt;0,VLOOKUP(A12,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="L12" s="112">
-        <f>IF(J12&gt;0,VLOOKUP(A12,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M12" s="111">
-        <f>IF(A12="","",COUNTIF($A$7:$A$11,A12)+COUNTIF($A$13:$A$15,A12))</f>
-        <v/>
+      <c r="J12" s="83" t="inlineStr"/>
+      <c r="K12" s="84">
+        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L12" s="84">
+        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O12" s="81">
+        <f>IF(A12="",0,COUNTIF(A$9:A11,A12))</f>
+        <v/>
+      </c>
+      <c r="P12" s="81" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="109" t="inlineStr">
-        <is>
-          <t>(New Activity 7)</t>
-        </is>
-      </c>
+      <c r="A13" s="129" t="inlineStr"/>
       <c r="B13" s="81" t="inlineStr"/>
       <c r="C13" s="81" t="inlineStr"/>
       <c r="D13" s="81" t="inlineStr"/>
@@ -6576,441 +6645,2187 @@
       <c r="G13" s="81" t="inlineStr"/>
       <c r="H13" s="81" t="inlineStr"/>
       <c r="I13" s="81" t="inlineStr"/>
-      <c r="J13" s="107">
-        <f>COUNTIF(B13:I13,"✓")</f>
-        <v/>
-      </c>
-      <c r="K13" s="112">
-        <f>IF(J13&gt;0,VLOOKUP(A13,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="L13" s="112">
-        <f>IF(J13&gt;0,VLOOKUP(A13,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M13" s="111">
-        <f>IF(A13="","",COUNTIF($A$7:$A$12,A13)+COUNTIF($A$14:$A$15,A13))</f>
-        <v/>
+      <c r="J13" s="83" t="inlineStr"/>
+      <c r="K13" s="84">
+        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L13" s="84">
+        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O13" s="81">
+        <f>IF(A13="",0,COUNTIF(A$9:A12,A13))</f>
+        <v/>
+      </c>
+      <c r="P13" s="81" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="108" t="inlineStr">
-        <is>
-          <t>(New Activity 8)</t>
-        </is>
-      </c>
-      <c r="B14" s="81" t="inlineStr"/>
-      <c r="C14" s="81" t="inlineStr"/>
-      <c r="D14" s="81" t="inlineStr"/>
-      <c r="E14" s="81" t="inlineStr"/>
-      <c r="F14" s="81" t="inlineStr"/>
-      <c r="G14" s="81" t="inlineStr"/>
-      <c r="H14" s="81" t="inlineStr"/>
-      <c r="I14" s="81" t="inlineStr"/>
-      <c r="J14" s="107">
-        <f>COUNTIF(B14:I14,"✓")</f>
-        <v/>
-      </c>
-      <c r="K14" s="112">
-        <f>IF(J14&gt;0,VLOOKUP(A14,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="L14" s="112">
-        <f>IF(J14&gt;0,VLOOKUP(A14,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M14" s="111">
-        <f>IF(A14="","",COUNTIF($A$7:$A$13,A14)+COUNTIF($A$15:$A$15,A14))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="109" t="inlineStr">
-        <is>
-          <t>(New Activity 9)</t>
-        </is>
-      </c>
-      <c r="B15" s="81" t="inlineStr"/>
-      <c r="C15" s="81" t="inlineStr"/>
-      <c r="D15" s="81" t="inlineStr"/>
-      <c r="E15" s="81" t="inlineStr"/>
-      <c r="F15" s="81" t="inlineStr"/>
-      <c r="G15" s="81" t="inlineStr"/>
-      <c r="H15" s="81" t="inlineStr"/>
-      <c r="I15" s="81" t="inlineStr"/>
-      <c r="J15" s="107">
-        <f>COUNTIF(B15:I15,"✓")</f>
-        <v/>
-      </c>
-      <c r="K15" s="112">
-        <f>IF(J15&gt;0,VLOOKUP(A15,'Master Data'!$A$86:$C$94,2,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="L15" s="112">
-        <f>IF(J15&gt;0,VLOOKUP(A15,'Master Data'!$A$86:$C$94,3,FALSE),0)</f>
-        <v/>
-      </c>
-      <c r="M15" s="111">
-        <f>IF(A15="","",COUNTIF($A$7:$A$14,A15)+COUNTIF($A$16:$A$15,A15))</f>
+      <c r="A14" s="123" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="B14" s="130">
+        <f>SUMPRODUCT((B9:B13="✓")*1,J9:J13,K9:K13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="130">
+        <f>SUMPRODUCT((C9:C13="✓")*1,J9:J13,K9:K13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="130">
+        <f>SUMPRODUCT((D9:D13="✓")*1,J9:J13,K9:K13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="130">
+        <f>SUMPRODUCT((E9:E13="✓")*1,J9:J13,K9:K13)</f>
+        <v/>
+      </c>
+      <c r="F14" s="130">
+        <f>SUMPRODUCT((F9:F13="✓")*1,J9:J13,K9:K13)</f>
+        <v/>
+      </c>
+      <c r="G14" s="130">
+        <f>SUMPRODUCT((G9:G13="✓")*1,J9:J13,K9:K13)</f>
+        <v/>
+      </c>
+      <c r="H14" s="130">
+        <f>SUMPRODUCT((H9:H13="✓")*1,J9:J13,K9:K13)</f>
+        <v/>
+      </c>
+      <c r="I14" s="130">
+        <f>SUMPRODUCT((I9:I13="✓")*1,J9:J13,K9:K13)</f>
+        <v/>
+      </c>
+      <c r="J14" s="114" t="inlineStr"/>
+      <c r="K14" s="88">
+        <f>SUMPRODUCT((J9:J13)*(K9:K13)*(COUNTIF(B9:I13,"✓")&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="L14" s="88">
+        <f>SUMPRODUCT((J9:J13)*(L9:L13)*(COUNTIF(B9:I13,"✓")&gt;0)*1)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="113" t="inlineStr">
-        <is>
-          <t>📌 TOTALS</t>
-        </is>
-      </c>
-      <c r="B16" s="114" t="inlineStr"/>
-      <c r="C16" s="114" t="inlineStr"/>
-      <c r="D16" s="114" t="inlineStr"/>
-      <c r="E16" s="114" t="inlineStr"/>
-      <c r="F16" s="114" t="inlineStr"/>
-      <c r="G16" s="114" t="inlineStr"/>
-      <c r="H16" s="114" t="inlineStr"/>
-      <c r="I16" s="114" t="inlineStr"/>
-      <c r="J16" s="88">
-        <f>SUM(J7:J15)</f>
-        <v/>
-      </c>
-      <c r="K16" s="88">
-        <f>SUM(K7:K15)</f>
-        <v/>
-      </c>
-      <c r="L16" s="88">
-        <f>SUM(L7:L15)</f>
-        <v/>
+      <c r="A16" s="128" t="inlineStr">
+        <is>
+          <t>🏨 HOTEL (1인 1박)</t>
+        </is>
+      </c>
+      <c r="B16" s="77" t="n"/>
+      <c r="C16" s="77" t="n"/>
+      <c r="D16" s="77" t="n"/>
+      <c r="E16" s="77" t="n"/>
+      <c r="F16" s="77" t="n"/>
+      <c r="G16" s="77" t="n"/>
+      <c r="H16" s="77" t="n"/>
+      <c r="I16" s="77" t="n"/>
+      <c r="J16" s="77" t="n"/>
+      <c r="K16" s="77" t="n"/>
+      <c r="L16" s="77" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="119" t="inlineStr">
+        <is>
+          <t>Item (Select ▼)</t>
+        </is>
+      </c>
+      <c r="B17" s="98" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C17" s="98" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D17" s="98" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E17" s="98" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="F17" s="98" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="G17" s="98" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="H17" s="98" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="I17" s="98" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="J17" s="98" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="K17" s="98" t="inlineStr">
+        <is>
+          <t>Cost/P</t>
+        </is>
+      </c>
+      <c r="L17" s="98" t="inlineStr">
+        <is>
+          <t>Sell/P</t>
+        </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="103" t="inlineStr">
-        <is>
-          <t>👤 PER-PERSON ACTIVITY COST</t>
-        </is>
-      </c>
-      <c r="B18" s="104" t="n"/>
-      <c r="C18" s="104" t="n"/>
-      <c r="D18" s="104" t="n"/>
-      <c r="E18" s="104" t="n"/>
-      <c r="F18" s="104" t="n"/>
-      <c r="G18" s="104" t="n"/>
-      <c r="H18" s="104" t="n"/>
-      <c r="I18" s="104" t="n"/>
-      <c r="J18" s="104" t="n"/>
-      <c r="K18" s="104" t="n"/>
-      <c r="L18" s="104" t="n"/>
+      <c r="A18" s="109" t="inlineStr">
+        <is>
+          <t>Beverly Wilshire (5★) / Same Tier</t>
+        </is>
+      </c>
+      <c r="B18" s="81" t="inlineStr"/>
+      <c r="C18" s="81" t="inlineStr"/>
+      <c r="D18" s="81" t="inlineStr"/>
+      <c r="E18" s="81" t="inlineStr"/>
+      <c r="F18" s="81" t="inlineStr"/>
+      <c r="G18" s="81" t="inlineStr"/>
+      <c r="H18" s="81" t="inlineStr"/>
+      <c r="I18" s="81" t="inlineStr"/>
+      <c r="J18" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="K18" s="84">
+        <f>IF(A18="","",VLOOKUP(A18,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L18" s="84">
+        <f>IF(A18="","",VLOOKUP(A18,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O18" s="81">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="P18" s="81" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="98" t="inlineStr">
+      <c r="A19" s="129" t="inlineStr"/>
+      <c r="B19" s="81" t="inlineStr"/>
+      <c r="C19" s="81" t="inlineStr"/>
+      <c r="D19" s="81" t="inlineStr"/>
+      <c r="E19" s="81" t="inlineStr"/>
+      <c r="F19" s="81" t="inlineStr"/>
+      <c r="G19" s="81" t="inlineStr"/>
+      <c r="H19" s="81" t="inlineStr"/>
+      <c r="I19" s="81" t="inlineStr"/>
+      <c r="J19" s="83" t="inlineStr"/>
+      <c r="K19" s="84">
+        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L19" s="84">
+        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O19" s="81">
+        <f>IF(A19="",0,COUNTIF(A$18:A18,A19))</f>
+        <v/>
+      </c>
+      <c r="P19" s="81" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="129" t="inlineStr"/>
+      <c r="B20" s="81" t="inlineStr"/>
+      <c r="C20" s="81" t="inlineStr"/>
+      <c r="D20" s="81" t="inlineStr"/>
+      <c r="E20" s="81" t="inlineStr"/>
+      <c r="F20" s="81" t="inlineStr"/>
+      <c r="G20" s="81" t="inlineStr"/>
+      <c r="H20" s="81" t="inlineStr"/>
+      <c r="I20" s="81" t="inlineStr"/>
+      <c r="J20" s="83" t="inlineStr"/>
+      <c r="K20" s="84">
+        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L20" s="84">
+        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O20" s="81">
+        <f>IF(A20="",0,COUNTIF(A$18:A19,A20))</f>
+        <v/>
+      </c>
+      <c r="P20" s="81" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="123" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="B21" s="130">
+        <f>SUMPRODUCT((B18:B20="✓")*1,J18:J20,K18:K20)</f>
+        <v/>
+      </c>
+      <c r="C21" s="130">
+        <f>SUMPRODUCT((C18:C20="✓")*1,J18:J20,K18:K20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="130">
+        <f>SUMPRODUCT((D18:D20="✓")*1,J18:J20,K18:K20)</f>
+        <v/>
+      </c>
+      <c r="E21" s="130">
+        <f>SUMPRODUCT((E18:E20="✓")*1,J18:J20,K18:K20)</f>
+        <v/>
+      </c>
+      <c r="F21" s="130">
+        <f>SUMPRODUCT((F18:F20="✓")*1,J18:J20,K18:K20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="130">
+        <f>SUMPRODUCT((G18:G20="✓")*1,J18:J20,K18:K20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="130">
+        <f>SUMPRODUCT((H18:H20="✓")*1,J18:J20,K18:K20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="130">
+        <f>SUMPRODUCT((I18:I20="✓")*1,J18:J20,K18:K20)</f>
+        <v/>
+      </c>
+      <c r="J21" s="114" t="inlineStr"/>
+      <c r="K21" s="88">
+        <f>SUMPRODUCT((J18:J20)*(K18:K20)*(COUNTIF(B18:I20,"✓")&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="L21" s="88">
+        <f>SUMPRODUCT((J18:J20)*(L18:L20)*(COUNTIF(B18:I20,"✓")&gt;0)*1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="128" t="inlineStr">
+        <is>
+          <t>🚐 TRANSPORT (1인 기준)</t>
+        </is>
+      </c>
+      <c r="B23" s="77" t="n"/>
+      <c r="C23" s="77" t="n"/>
+      <c r="D23" s="77" t="n"/>
+      <c r="E23" s="77" t="n"/>
+      <c r="F23" s="77" t="n"/>
+      <c r="G23" s="77" t="n"/>
+      <c r="H23" s="77" t="n"/>
+      <c r="I23" s="77" t="n"/>
+      <c r="J23" s="77" t="n"/>
+      <c r="K23" s="77" t="n"/>
+      <c r="L23" s="77" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="119" t="inlineStr">
+        <is>
+          <t>Item (Select ▼)</t>
+        </is>
+      </c>
+      <c r="B24" s="98" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C24" s="98" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D24" s="98" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E24" s="98" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="F24" s="98" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="G24" s="98" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="H24" s="98" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="I24" s="98" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="J24" s="98" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="K24" s="98" t="inlineStr">
+        <is>
+          <t>Cost/P</t>
+        </is>
+      </c>
+      <c r="L24" s="98" t="inlineStr">
+        <is>
+          <t>Sell/P</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="109" t="inlineStr">
+        <is>
+          <t>Driver/Guide + Van (일당)</t>
+        </is>
+      </c>
+      <c r="B25" s="81" t="inlineStr"/>
+      <c r="C25" s="81" t="inlineStr"/>
+      <c r="D25" s="81" t="inlineStr"/>
+      <c r="E25" s="81" t="inlineStr"/>
+      <c r="F25" s="81" t="inlineStr"/>
+      <c r="G25" s="81" t="inlineStr"/>
+      <c r="H25" s="81" t="inlineStr"/>
+      <c r="I25" s="81" t="inlineStr"/>
+      <c r="J25" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="K25" s="84">
+        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L25" s="84">
+        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O25" s="81">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="P25" s="81" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="129" t="inlineStr"/>
+      <c r="B26" s="81" t="inlineStr"/>
+      <c r="C26" s="81" t="inlineStr"/>
+      <c r="D26" s="81" t="inlineStr"/>
+      <c r="E26" s="81" t="inlineStr"/>
+      <c r="F26" s="81" t="inlineStr"/>
+      <c r="G26" s="81" t="inlineStr"/>
+      <c r="H26" s="81" t="inlineStr"/>
+      <c r="I26" s="81" t="inlineStr"/>
+      <c r="J26" s="83" t="inlineStr"/>
+      <c r="K26" s="84">
+        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L26" s="84">
+        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O26" s="81">
+        <f>IF(A26="",0,COUNTIF(A$25:A25,A26))</f>
+        <v/>
+      </c>
+      <c r="P26" s="81" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="129" t="inlineStr"/>
+      <c r="B27" s="81" t="inlineStr"/>
+      <c r="C27" s="81" t="inlineStr"/>
+      <c r="D27" s="81" t="inlineStr"/>
+      <c r="E27" s="81" t="inlineStr"/>
+      <c r="F27" s="81" t="inlineStr"/>
+      <c r="G27" s="81" t="inlineStr"/>
+      <c r="H27" s="81" t="inlineStr"/>
+      <c r="I27" s="81" t="inlineStr"/>
+      <c r="J27" s="83" t="inlineStr"/>
+      <c r="K27" s="84">
+        <f>IF(A27="","",VLOOKUP(A27,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L27" s="84">
+        <f>IF(A27="","",VLOOKUP(A27,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O27" s="81">
+        <f>IF(A27="",0,COUNTIF(A$25:A26,A27))</f>
+        <v/>
+      </c>
+      <c r="P27" s="81" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="123" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="130">
+        <f>SUMPRODUCT((B25:B27="✓")*1,J25:J27,K25:K27)</f>
+        <v/>
+      </c>
+      <c r="C28" s="130">
+        <f>SUMPRODUCT((C25:C27="✓")*1,J25:J27,K25:K27)</f>
+        <v/>
+      </c>
+      <c r="D28" s="130">
+        <f>SUMPRODUCT((D25:D27="✓")*1,J25:J27,K25:K27)</f>
+        <v/>
+      </c>
+      <c r="E28" s="130">
+        <f>SUMPRODUCT((E25:E27="✓")*1,J25:J27,K25:K27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="130">
+        <f>SUMPRODUCT((F25:F27="✓")*1,J25:J27,K25:K27)</f>
+        <v/>
+      </c>
+      <c r="G28" s="130">
+        <f>SUMPRODUCT((G25:G27="✓")*1,J25:J27,K25:K27)</f>
+        <v/>
+      </c>
+      <c r="H28" s="130">
+        <f>SUMPRODUCT((H25:H27="✓")*1,J25:J27,K25:K27)</f>
+        <v/>
+      </c>
+      <c r="I28" s="130">
+        <f>SUMPRODUCT((I25:I27="✓")*1,J25:J27,K25:K27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="114" t="inlineStr"/>
+      <c r="K28" s="88">
+        <f>SUMPRODUCT((J25:J27)*(K25:K27)*(COUNTIF(B25:I27,"✓")&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="L28" s="88">
+        <f>SUMPRODUCT((J25:J27)*(L25:L27)*(COUNTIF(B25:I27,"✓")&gt;0)*1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="128" t="inlineStr">
+        <is>
+          <t>🍽️ MEALS (1인 1끼)</t>
+        </is>
+      </c>
+      <c r="B30" s="77" t="n"/>
+      <c r="C30" s="77" t="n"/>
+      <c r="D30" s="77" t="n"/>
+      <c r="E30" s="77" t="n"/>
+      <c r="F30" s="77" t="n"/>
+      <c r="G30" s="77" t="n"/>
+      <c r="H30" s="77" t="n"/>
+      <c r="I30" s="77" t="n"/>
+      <c r="J30" s="77" t="n"/>
+      <c r="K30" s="77" t="n"/>
+      <c r="L30" s="77" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="119" t="inlineStr">
+        <is>
+          <t>Item (Select ▼)</t>
+        </is>
+      </c>
+      <c r="B31" s="98" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C31" s="98" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D31" s="98" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E31" s="98" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="F31" s="98" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="G31" s="98" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="H31" s="98" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="I31" s="98" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="J31" s="98" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="K31" s="98" t="inlineStr">
+        <is>
+          <t>Cost/P</t>
+        </is>
+      </c>
+      <c r="L31" s="98" t="inlineStr">
+        <is>
+          <t>Sell/P</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="109" t="inlineStr">
+        <is>
+          <t>Breakfast (Hotel)</t>
+        </is>
+      </c>
+      <c r="B32" s="81" t="inlineStr"/>
+      <c r="C32" s="81" t="inlineStr"/>
+      <c r="D32" s="81" t="inlineStr"/>
+      <c r="E32" s="81" t="inlineStr"/>
+      <c r="F32" s="81" t="inlineStr"/>
+      <c r="G32" s="81" t="inlineStr"/>
+      <c r="H32" s="81" t="inlineStr"/>
+      <c r="I32" s="81" t="inlineStr"/>
+      <c r="J32" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="K32" s="84">
+        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L32" s="84">
+        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O32" s="81">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="P32" s="81" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="108" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="B33" s="81" t="inlineStr"/>
+      <c r="C33" s="81" t="inlineStr"/>
+      <c r="D33" s="81" t="inlineStr"/>
+      <c r="E33" s="81" t="inlineStr"/>
+      <c r="F33" s="81" t="inlineStr"/>
+      <c r="G33" s="81" t="inlineStr"/>
+      <c r="H33" s="81" t="inlineStr"/>
+      <c r="I33" s="81" t="inlineStr"/>
+      <c r="J33" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="K33" s="84">
+        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L33" s="84">
+        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O33" s="81">
+        <f>IF(A33="",0,COUNTIF(A$32:A32,A33))</f>
+        <v/>
+      </c>
+      <c r="P33" s="81" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="109" t="inlineStr">
+        <is>
+          <t>Dinner (Regular)</t>
+        </is>
+      </c>
+      <c r="B34" s="81" t="inlineStr"/>
+      <c r="C34" s="81" t="inlineStr"/>
+      <c r="D34" s="81" t="inlineStr"/>
+      <c r="E34" s="81" t="inlineStr"/>
+      <c r="F34" s="81" t="inlineStr"/>
+      <c r="G34" s="81" t="inlineStr"/>
+      <c r="H34" s="81" t="inlineStr"/>
+      <c r="I34" s="81" t="inlineStr"/>
+      <c r="J34" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="K34" s="84">
+        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L34" s="84">
+        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O34" s="81">
+        <f>IF(A34="",0,COUNTIF(A$32:A33,A34))</f>
+        <v/>
+      </c>
+      <c r="P34" s="81" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="108" t="inlineStr">
+        <is>
+          <t>Exclusive Dinner (Michelin/Fine)</t>
+        </is>
+      </c>
+      <c r="B35" s="81" t="inlineStr"/>
+      <c r="C35" s="81" t="inlineStr"/>
+      <c r="D35" s="81" t="inlineStr"/>
+      <c r="E35" s="81" t="inlineStr"/>
+      <c r="F35" s="81" t="inlineStr"/>
+      <c r="G35" s="81" t="inlineStr"/>
+      <c r="H35" s="81" t="inlineStr"/>
+      <c r="I35" s="81" t="inlineStr"/>
+      <c r="J35" s="83" t="n">
+        <v>2</v>
+      </c>
+      <c r="K35" s="84">
+        <f>IF(A35="","",VLOOKUP(A35,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L35" s="84">
+        <f>IF(A35="","",VLOOKUP(A35,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O35" s="81">
+        <f>IF(A35="",0,COUNTIF(A$32:A34,A35))</f>
+        <v/>
+      </c>
+      <c r="P35" s="81" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="129" t="inlineStr"/>
+      <c r="B36" s="81" t="inlineStr"/>
+      <c r="C36" s="81" t="inlineStr"/>
+      <c r="D36" s="81" t="inlineStr"/>
+      <c r="E36" s="81" t="inlineStr"/>
+      <c r="F36" s="81" t="inlineStr"/>
+      <c r="G36" s="81" t="inlineStr"/>
+      <c r="H36" s="81" t="inlineStr"/>
+      <c r="I36" s="81" t="inlineStr"/>
+      <c r="J36" s="83" t="inlineStr"/>
+      <c r="K36" s="84">
+        <f>IF(A36="","",VLOOKUP(A36,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L36" s="84">
+        <f>IF(A36="","",VLOOKUP(A36,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O36" s="81">
+        <f>IF(A36="",0,COUNTIF(A$32:A35,A36))</f>
+        <v/>
+      </c>
+      <c r="P36" s="81" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="123" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="B37" s="130">
+        <f>SUMPRODUCT((B32:B36="✓")*1,J32:J36,K32:K36)</f>
+        <v/>
+      </c>
+      <c r="C37" s="130">
+        <f>SUMPRODUCT((C32:C36="✓")*1,J32:J36,K32:K36)</f>
+        <v/>
+      </c>
+      <c r="D37" s="130">
+        <f>SUMPRODUCT((D32:D36="✓")*1,J32:J36,K32:K36)</f>
+        <v/>
+      </c>
+      <c r="E37" s="130">
+        <f>SUMPRODUCT((E32:E36="✓")*1,J32:J36,K32:K36)</f>
+        <v/>
+      </c>
+      <c r="F37" s="130">
+        <f>SUMPRODUCT((F32:F36="✓")*1,J32:J36,K32:K36)</f>
+        <v/>
+      </c>
+      <c r="G37" s="130">
+        <f>SUMPRODUCT((G32:G36="✓")*1,J32:J36,K32:K36)</f>
+        <v/>
+      </c>
+      <c r="H37" s="130">
+        <f>SUMPRODUCT((H32:H36="✓")*1,J32:J36,K32:K36)</f>
+        <v/>
+      </c>
+      <c r="I37" s="130">
+        <f>SUMPRODUCT((I32:I36="✓")*1,J32:J36,K32:K36)</f>
+        <v/>
+      </c>
+      <c r="J37" s="114" t="inlineStr"/>
+      <c r="K37" s="88">
+        <f>SUMPRODUCT((J32:J36)*(K32:K36)*(COUNTIF(B32:I36,"✓")&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="L37" s="88">
+        <f>SUMPRODUCT((J32:J36)*(L32:L36)*(COUNTIF(B32:I36,"✓")&gt;0)*1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="128" t="inlineStr">
+        <is>
+          <t>📦 OTHER (1인 1일)</t>
+        </is>
+      </c>
+      <c r="B39" s="77" t="n"/>
+      <c r="C39" s="77" t="n"/>
+      <c r="D39" s="77" t="n"/>
+      <c r="E39" s="77" t="n"/>
+      <c r="F39" s="77" t="n"/>
+      <c r="G39" s="77" t="n"/>
+      <c r="H39" s="77" t="n"/>
+      <c r="I39" s="77" t="n"/>
+      <c r="J39" s="77" t="n"/>
+      <c r="K39" s="77" t="n"/>
+      <c r="L39" s="77" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="119" t="inlineStr">
+        <is>
+          <t>Item (Select ▼)</t>
+        </is>
+      </c>
+      <c r="B40" s="98" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C40" s="98" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D40" s="98" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E40" s="98" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="F40" s="98" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="G40" s="98" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="H40" s="98" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="I40" s="98" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="J40" s="98" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="K40" s="98" t="inlineStr">
+        <is>
+          <t>Cost/P</t>
+        </is>
+      </c>
+      <c r="L40" s="98" t="inlineStr">
+        <is>
+          <t>Sell/P</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="109" t="inlineStr">
+        <is>
+          <t>Insurance / Tips / Contingency</t>
+        </is>
+      </c>
+      <c r="B41" s="81" t="inlineStr"/>
+      <c r="C41" s="81" t="inlineStr"/>
+      <c r="D41" s="81" t="inlineStr"/>
+      <c r="E41" s="81" t="inlineStr"/>
+      <c r="F41" s="81" t="inlineStr"/>
+      <c r="G41" s="81" t="inlineStr"/>
+      <c r="H41" s="81" t="inlineStr"/>
+      <c r="I41" s="81" t="inlineStr"/>
+      <c r="J41" s="83" t="n">
+        <v>4</v>
+      </c>
+      <c r="K41" s="84">
+        <f>IF(A41="","",VLOOKUP(A41,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L41" s="84">
+        <f>IF(A41="","",VLOOKUP(A41,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O41" s="81">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="P41" s="81" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="129" t="inlineStr"/>
+      <c r="B42" s="81" t="inlineStr"/>
+      <c r="C42" s="81" t="inlineStr"/>
+      <c r="D42" s="81" t="inlineStr"/>
+      <c r="E42" s="81" t="inlineStr"/>
+      <c r="F42" s="81" t="inlineStr"/>
+      <c r="G42" s="81" t="inlineStr"/>
+      <c r="H42" s="81" t="inlineStr"/>
+      <c r="I42" s="81" t="inlineStr"/>
+      <c r="J42" s="83" t="inlineStr"/>
+      <c r="K42" s="84">
+        <f>IF(A42="","",VLOOKUP(A42,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L42" s="84">
+        <f>IF(A42="","",VLOOKUP(A42,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O42" s="81">
+        <f>IF(A42="",0,COUNTIF(A$41:A41,A42))</f>
+        <v/>
+      </c>
+      <c r="P42" s="81" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="129" t="inlineStr"/>
+      <c r="B43" s="81" t="inlineStr"/>
+      <c r="C43" s="81" t="inlineStr"/>
+      <c r="D43" s="81" t="inlineStr"/>
+      <c r="E43" s="81" t="inlineStr"/>
+      <c r="F43" s="81" t="inlineStr"/>
+      <c r="G43" s="81" t="inlineStr"/>
+      <c r="H43" s="81" t="inlineStr"/>
+      <c r="I43" s="81" t="inlineStr"/>
+      <c r="J43" s="83" t="inlineStr"/>
+      <c r="K43" s="84">
+        <f>IF(A43="","",VLOOKUP(A43,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L43" s="84">
+        <f>IF(A43="","",VLOOKUP(A43,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O43" s="81">
+        <f>IF(A43="",0,COUNTIF(A$41:A42,A43))</f>
+        <v/>
+      </c>
+      <c r="P43" s="81" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="123" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="B44" s="130">
+        <f>SUMPRODUCT((B41:B43="✓")*1,J41:J43,K41:K43)</f>
+        <v/>
+      </c>
+      <c r="C44" s="130">
+        <f>SUMPRODUCT((C41:C43="✓")*1,J41:J43,K41:K43)</f>
+        <v/>
+      </c>
+      <c r="D44" s="130">
+        <f>SUMPRODUCT((D41:D43="✓")*1,J41:J43,K41:K43)</f>
+        <v/>
+      </c>
+      <c r="E44" s="130">
+        <f>SUMPRODUCT((E41:E43="✓")*1,J41:J43,K41:K43)</f>
+        <v/>
+      </c>
+      <c r="F44" s="130">
+        <f>SUMPRODUCT((F41:F43="✓")*1,J41:J43,K41:K43)</f>
+        <v/>
+      </c>
+      <c r="G44" s="130">
+        <f>SUMPRODUCT((G41:G43="✓")*1,J41:J43,K41:K43)</f>
+        <v/>
+      </c>
+      <c r="H44" s="130">
+        <f>SUMPRODUCT((H41:H43="✓")*1,J41:J43,K41:K43)</f>
+        <v/>
+      </c>
+      <c r="I44" s="130">
+        <f>SUMPRODUCT((I41:I43="✓")*1,J41:J43,K41:K43)</f>
+        <v/>
+      </c>
+      <c r="J44" s="114" t="inlineStr"/>
+      <c r="K44" s="88">
+        <f>SUMPRODUCT((J41:J43)*(K41:K43)*(COUNTIF(B41:I43,"✓")&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="L44" s="88">
+        <f>SUMPRODUCT((J41:J43)*(L41:L43)*(COUNTIF(B41:I43,"✓")&gt;0)*1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="128" t="inlineStr">
+        <is>
+          <t>🎯 ACTIVITIES &amp; EXPERIENCES (1인 1회)</t>
+        </is>
+      </c>
+      <c r="B46" s="77" t="n"/>
+      <c r="C46" s="77" t="n"/>
+      <c r="D46" s="77" t="n"/>
+      <c r="E46" s="77" t="n"/>
+      <c r="F46" s="77" t="n"/>
+      <c r="G46" s="77" t="n"/>
+      <c r="H46" s="77" t="n"/>
+      <c r="I46" s="77" t="n"/>
+      <c r="J46" s="77" t="n"/>
+      <c r="K46" s="77" t="n"/>
+      <c r="L46" s="77" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="119" t="inlineStr">
+        <is>
+          <t>Item (Select ▼)</t>
+        </is>
+      </c>
+      <c r="B47" s="98" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C47" s="98" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D47" s="98" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="E47" s="98" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="F47" s="98" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="G47" s="98" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="H47" s="98" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="I47" s="98" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="J47" s="98" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="K47" s="98" t="inlineStr">
+        <is>
+          <t>Cost/P</t>
+        </is>
+      </c>
+      <c r="L47" s="98" t="inlineStr">
+        <is>
+          <t>Sell/P</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="109" t="inlineStr">
+        <is>
+          <t>NBA/MLB Game (Ticket)</t>
+        </is>
+      </c>
+      <c r="B48" s="81" t="inlineStr"/>
+      <c r="C48" s="81" t="inlineStr"/>
+      <c r="D48" s="81" t="inlineStr"/>
+      <c r="E48" s="81" t="inlineStr"/>
+      <c r="F48" s="81" t="inlineStr"/>
+      <c r="G48" s="81" t="inlineStr"/>
+      <c r="H48" s="81" t="inlineStr"/>
+      <c r="I48" s="81" t="inlineStr"/>
+      <c r="J48" s="83" t="n">
+        <v>1</v>
+      </c>
+      <c r="K48" s="84">
+        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L48" s="84">
+        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O48" s="81">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="P48" s="81" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="108" t="inlineStr">
+        <is>
+          <t>Sports Bar Experience</t>
+        </is>
+      </c>
+      <c r="B49" s="81" t="inlineStr"/>
+      <c r="C49" s="81" t="inlineStr"/>
+      <c r="D49" s="81" t="inlineStr"/>
+      <c r="E49" s="81" t="inlineStr"/>
+      <c r="F49" s="81" t="inlineStr"/>
+      <c r="G49" s="81" t="inlineStr"/>
+      <c r="H49" s="81" t="inlineStr"/>
+      <c r="I49" s="81" t="inlineStr"/>
+      <c r="J49" s="83" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" s="84">
+        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L49" s="84">
+        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O49" s="81">
+        <f>IF(A49="",0,COUNTIF(A$48:A48,A49))</f>
+        <v/>
+      </c>
+      <c r="P49" s="81" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="109" t="inlineStr">
+        <is>
+          <t>Local Hiking (Griffith/Runyon)</t>
+        </is>
+      </c>
+      <c r="B50" s="81" t="inlineStr"/>
+      <c r="C50" s="81" t="inlineStr"/>
+      <c r="D50" s="81" t="inlineStr"/>
+      <c r="E50" s="81" t="inlineStr"/>
+      <c r="F50" s="81" t="inlineStr"/>
+      <c r="G50" s="81" t="inlineStr"/>
+      <c r="H50" s="81" t="inlineStr"/>
+      <c r="I50" s="81" t="inlineStr"/>
+      <c r="J50" s="83" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" s="84">
+        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L50" s="84">
+        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O50" s="81">
+        <f>IF(A50="",0,COUNTIF(A$48:A49,A50))</f>
+        <v/>
+      </c>
+      <c r="P50" s="81" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="108" t="inlineStr">
+        <is>
+          <t>Beach/Surf Lesson</t>
+        </is>
+      </c>
+      <c r="B51" s="81" t="inlineStr"/>
+      <c r="C51" s="81" t="inlineStr"/>
+      <c r="D51" s="81" t="inlineStr"/>
+      <c r="E51" s="81" t="inlineStr"/>
+      <c r="F51" s="81" t="inlineStr"/>
+      <c r="G51" s="81" t="inlineStr"/>
+      <c r="H51" s="81" t="inlineStr"/>
+      <c r="I51" s="81" t="inlineStr"/>
+      <c r="J51" s="83" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" s="84">
+        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L51" s="84">
+        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O51" s="81">
+        <f>IF(A51="",0,COUNTIF(A$48:A50,A51))</f>
+        <v/>
+      </c>
+      <c r="P51" s="81" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="129" t="inlineStr"/>
+      <c r="B52" s="81" t="inlineStr"/>
+      <c r="C52" s="81" t="inlineStr"/>
+      <c r="D52" s="81" t="inlineStr"/>
+      <c r="E52" s="81" t="inlineStr"/>
+      <c r="F52" s="81" t="inlineStr"/>
+      <c r="G52" s="81" t="inlineStr"/>
+      <c r="H52" s="81" t="inlineStr"/>
+      <c r="I52" s="81" t="inlineStr"/>
+      <c r="J52" s="83" t="inlineStr"/>
+      <c r="K52" s="84">
+        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L52" s="84">
+        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O52" s="81">
+        <f>IF(A52="",0,COUNTIF(A$48:A51,A52))</f>
+        <v/>
+      </c>
+      <c r="P52" s="81" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="129" t="inlineStr"/>
+      <c r="B53" s="81" t="inlineStr"/>
+      <c r="C53" s="81" t="inlineStr"/>
+      <c r="D53" s="81" t="inlineStr"/>
+      <c r="E53" s="81" t="inlineStr"/>
+      <c r="F53" s="81" t="inlineStr"/>
+      <c r="G53" s="81" t="inlineStr"/>
+      <c r="H53" s="81" t="inlineStr"/>
+      <c r="I53" s="81" t="inlineStr"/>
+      <c r="J53" s="83" t="inlineStr"/>
+      <c r="K53" s="84">
+        <f>IF(A53="","",VLOOKUP(A53,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L53" s="84">
+        <f>IF(A53="","",VLOOKUP(A53,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O53" s="81">
+        <f>IF(A53="",0,COUNTIF(A$48:A52,A53))</f>
+        <v/>
+      </c>
+      <c r="P53" s="81" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="129" t="inlineStr"/>
+      <c r="B54" s="81" t="inlineStr"/>
+      <c r="C54" s="81" t="inlineStr"/>
+      <c r="D54" s="81" t="inlineStr"/>
+      <c r="E54" s="81" t="inlineStr"/>
+      <c r="F54" s="81" t="inlineStr"/>
+      <c r="G54" s="81" t="inlineStr"/>
+      <c r="H54" s="81" t="inlineStr"/>
+      <c r="I54" s="81" t="inlineStr"/>
+      <c r="J54" s="83" t="inlineStr"/>
+      <c r="K54" s="84">
+        <f>IF(A54="","",VLOOKUP(A54,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L54" s="84">
+        <f>IF(A54="","",VLOOKUP(A54,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O54" s="81">
+        <f>IF(A54="",0,COUNTIF(A$48:A53,A54))</f>
+        <v/>
+      </c>
+      <c r="P54" s="81" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="129" t="inlineStr"/>
+      <c r="B55" s="81" t="inlineStr"/>
+      <c r="C55" s="81" t="inlineStr"/>
+      <c r="D55" s="81" t="inlineStr"/>
+      <c r="E55" s="81" t="inlineStr"/>
+      <c r="F55" s="81" t="inlineStr"/>
+      <c r="G55" s="81" t="inlineStr"/>
+      <c r="H55" s="81" t="inlineStr"/>
+      <c r="I55" s="81" t="inlineStr"/>
+      <c r="J55" s="83" t="inlineStr"/>
+      <c r="K55" s="84">
+        <f>IF(A55="","",VLOOKUP(A55,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L55" s="84">
+        <f>IF(A55="","",VLOOKUP(A55,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O55" s="81">
+        <f>IF(A55="",0,COUNTIF(A$48:A54,A55))</f>
+        <v/>
+      </c>
+      <c r="P55" s="81" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="129" t="inlineStr"/>
+      <c r="B56" s="81" t="inlineStr"/>
+      <c r="C56" s="81" t="inlineStr"/>
+      <c r="D56" s="81" t="inlineStr"/>
+      <c r="E56" s="81" t="inlineStr"/>
+      <c r="F56" s="81" t="inlineStr"/>
+      <c r="G56" s="81" t="inlineStr"/>
+      <c r="H56" s="81" t="inlineStr"/>
+      <c r="I56" s="81" t="inlineStr"/>
+      <c r="J56" s="83" t="inlineStr"/>
+      <c r="K56" s="84">
+        <f>IF(A56="","",VLOOKUP(A56,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="L56" s="84">
+        <f>IF(A56="","",VLOOKUP(A56,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="O56" s="81">
+        <f>IF(A56="",0,COUNTIF(A$48:A55,A56))</f>
+        <v/>
+      </c>
+      <c r="P56" s="81" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="123" t="inlineStr">
+        <is>
+          <t>SUBTOTAL</t>
+        </is>
+      </c>
+      <c r="B57" s="130">
+        <f>SUMPRODUCT((B48:B56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="C57" s="130">
+        <f>SUMPRODUCT((C48:C56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="D57" s="130">
+        <f>SUMPRODUCT((D48:D56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="E57" s="130">
+        <f>SUMPRODUCT((E48:E56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="F57" s="130">
+        <f>SUMPRODUCT((F48:F56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="G57" s="130">
+        <f>SUMPRODUCT((G48:G56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="H57" s="130">
+        <f>SUMPRODUCT((H48:H56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="I57" s="130">
+        <f>SUMPRODUCT((I48:I56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="J57" s="114" t="inlineStr"/>
+      <c r="K57" s="88">
+        <f>SUMPRODUCT((J48:J56)*(K48:K56)*(COUNTIF(B48:I56,"✓")&gt;0)*1)</f>
+        <v/>
+      </c>
+      <c r="L57" s="88">
+        <f>SUMPRODUCT((J48:J56)*(L48:L56)*(COUNTIF(B48:I56,"✓")&gt;0)*1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="103" t="inlineStr">
+        <is>
+          <t>👤 PER PERSON TOTALS</t>
+        </is>
+      </c>
+      <c r="B60" s="104" t="n"/>
+      <c r="C60" s="104" t="n"/>
+      <c r="D60" s="104" t="n"/>
+      <c r="E60" s="104" t="n"/>
+      <c r="F60" s="104" t="n"/>
+      <c r="G60" s="104" t="n"/>
+      <c r="H60" s="104" t="n"/>
+      <c r="I60" s="104" t="n"/>
+      <c r="J60" s="104" t="n"/>
+      <c r="K60" s="104" t="n"/>
+      <c r="L60" s="104" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="98" t="inlineStr">
         <is>
           <t>Person</t>
         </is>
       </c>
-      <c r="B19" s="98" t="inlineStr">
-        <is>
-          <t># Activities</t>
-        </is>
-      </c>
-      <c r="C19" s="98" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="D19" s="98" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="E19" s="98" t="inlineStr">
+      <c r="B61" s="98" t="inlineStr">
+        <is>
+          <t>Total Cost</t>
+        </is>
+      </c>
+      <c r="C61" s="98" t="inlineStr">
+        <is>
+          <t>Total Sell</t>
+        </is>
+      </c>
+      <c r="D61" s="98" t="inlineStr">
         <is>
           <t>Margin</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="108" t="inlineStr">
+      <c r="E61" s="98" t="inlineStr">
+        <is>
+          <t>Margin%</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="108" t="inlineStr">
         <is>
           <t>참가자1</t>
         </is>
       </c>
-      <c r="B20" s="107">
-        <f>COUNTIF(B7:B15,"✓")</f>
-        <v/>
-      </c>
-      <c r="C20" s="110">
-        <f>SUMPRODUCT((B7:B15="✓")*1,K7:K15)</f>
-        <v/>
-      </c>
-      <c r="D20" s="110">
-        <f>SUMPRODUCT((B7:B15="✓")*1,L7:L15)</f>
-        <v/>
-      </c>
-      <c r="E20" s="110">
-        <f>D20-C20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="108" t="inlineStr">
+      <c r="B62" s="131">
+        <f>SUMPRODUCT((B9:B13="✓")*1,J9:J13,K9:K13)+SUMPRODUCT((B18:B20="✓")*1,J18:J20,K18:K20)+SUMPRODUCT((B25:B27="✓")*1,J25:J27,K25:K27)+SUMPRODUCT((B32:B36="✓")*1,J32:J36,K32:K36)+SUMPRODUCT((B41:B43="✓")*1,J41:J43,K41:K43)+SUMPRODUCT((B48:B56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="C62" s="131">
+        <f>SUMPRODUCT((B9:B13="✓")*1,J9:J13,L9:L13)+SUMPRODUCT((B18:B20="✓")*1,J18:J20,L18:L20)+SUMPRODUCT((B25:B27="✓")*1,J25:J27,L25:L27)+SUMPRODUCT((B32:B36="✓")*1,J32:J36,L32:L36)+SUMPRODUCT((B41:B43="✓")*1,J41:J43,L41:L43)+SUMPRODUCT((B48:B56="✓")*1,J48:J56,L48:L56)</f>
+        <v/>
+      </c>
+      <c r="D62" s="110">
+        <f>C62-B62</f>
+        <v/>
+      </c>
+      <c r="E62" s="132">
+        <f>IF(C62&gt;0,D62/C62,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="108" t="inlineStr">
         <is>
           <t>참가자2</t>
         </is>
       </c>
-      <c r="B21" s="107">
-        <f>COUNTIF(C7:C15,"✓")</f>
-        <v/>
-      </c>
-      <c r="C21" s="110">
-        <f>SUMPRODUCT((C7:C15="✓")*1,K7:K15)</f>
-        <v/>
-      </c>
-      <c r="D21" s="110">
-        <f>SUMPRODUCT((C7:C15="✓")*1,L7:L15)</f>
-        <v/>
-      </c>
-      <c r="E21" s="110">
-        <f>D21-C21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="108" t="inlineStr">
+      <c r="B63" s="131">
+        <f>SUMPRODUCT((C9:C13="✓")*1,J9:J13,K9:K13)+SUMPRODUCT((C18:C20="✓")*1,J18:J20,K18:K20)+SUMPRODUCT((C25:C27="✓")*1,J25:J27,K25:K27)+SUMPRODUCT((C32:C36="✓")*1,J32:J36,K32:K36)+SUMPRODUCT((C41:C43="✓")*1,J41:J43,K41:K43)+SUMPRODUCT((C48:C56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="C63" s="131">
+        <f>SUMPRODUCT((C9:C13="✓")*1,J9:J13,L9:L13)+SUMPRODUCT((C18:C20="✓")*1,J18:J20,L18:L20)+SUMPRODUCT((C25:C27="✓")*1,J25:J27,L25:L27)+SUMPRODUCT((C32:C36="✓")*1,J32:J36,L32:L36)+SUMPRODUCT((C41:C43="✓")*1,J41:J43,L41:L43)+SUMPRODUCT((C48:C56="✓")*1,J48:J56,L48:L56)</f>
+        <v/>
+      </c>
+      <c r="D63" s="110">
+        <f>C63-B63</f>
+        <v/>
+      </c>
+      <c r="E63" s="132">
+        <f>IF(C63&gt;0,D63/C63,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="108" t="inlineStr">
         <is>
           <t>참가자3</t>
         </is>
       </c>
-      <c r="B22" s="107">
-        <f>COUNTIF(D7:D15,"✓")</f>
-        <v/>
-      </c>
-      <c r="C22" s="110">
-        <f>SUMPRODUCT((D7:D15="✓")*1,K7:K15)</f>
-        <v/>
-      </c>
-      <c r="D22" s="110">
-        <f>SUMPRODUCT((D7:D15="✓")*1,L7:L15)</f>
-        <v/>
-      </c>
-      <c r="E22" s="110">
-        <f>D22-C22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="108" t="inlineStr">
+      <c r="B64" s="131">
+        <f>SUMPRODUCT((D9:D13="✓")*1,J9:J13,K9:K13)+SUMPRODUCT((D18:D20="✓")*1,J18:J20,K18:K20)+SUMPRODUCT((D25:D27="✓")*1,J25:J27,K25:K27)+SUMPRODUCT((D32:D36="✓")*1,J32:J36,K32:K36)+SUMPRODUCT((D41:D43="✓")*1,J41:J43,K41:K43)+SUMPRODUCT((D48:D56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="C64" s="131">
+        <f>SUMPRODUCT((D9:D13="✓")*1,J9:J13,L9:L13)+SUMPRODUCT((D18:D20="✓")*1,J18:J20,L18:L20)+SUMPRODUCT((D25:D27="✓")*1,J25:J27,L25:L27)+SUMPRODUCT((D32:D36="✓")*1,J32:J36,L32:L36)+SUMPRODUCT((D41:D43="✓")*1,J41:J43,L41:L43)+SUMPRODUCT((D48:D56="✓")*1,J48:J56,L48:L56)</f>
+        <v/>
+      </c>
+      <c r="D64" s="110">
+        <f>C64-B64</f>
+        <v/>
+      </c>
+      <c r="E64" s="132">
+        <f>IF(C64&gt;0,D64/C64,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="108" t="inlineStr">
         <is>
           <t>참가자4</t>
         </is>
       </c>
-      <c r="B23" s="107">
-        <f>COUNTIF(E7:E15,"✓")</f>
-        <v/>
-      </c>
-      <c r="C23" s="110">
-        <f>SUMPRODUCT((E7:E15="✓")*1,K7:K15)</f>
-        <v/>
-      </c>
-      <c r="D23" s="110">
-        <f>SUMPRODUCT((E7:E15="✓")*1,L7:L15)</f>
-        <v/>
-      </c>
-      <c r="E23" s="110">
-        <f>D23-C23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="108" t="inlineStr">
+      <c r="B65" s="131">
+        <f>SUMPRODUCT((E9:E13="✓")*1,J9:J13,K9:K13)+SUMPRODUCT((E18:E20="✓")*1,J18:J20,K18:K20)+SUMPRODUCT((E25:E27="✓")*1,J25:J27,K25:K27)+SUMPRODUCT((E32:E36="✓")*1,J32:J36,K32:K36)+SUMPRODUCT((E41:E43="✓")*1,J41:J43,K41:K43)+SUMPRODUCT((E48:E56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="C65" s="131">
+        <f>SUMPRODUCT((E9:E13="✓")*1,J9:J13,L9:L13)+SUMPRODUCT((E18:E20="✓")*1,J18:J20,L18:L20)+SUMPRODUCT((E25:E27="✓")*1,J25:J27,L25:L27)+SUMPRODUCT((E32:E36="✓")*1,J32:J36,L32:L36)+SUMPRODUCT((E41:E43="✓")*1,J41:J43,L41:L43)+SUMPRODUCT((E48:E56="✓")*1,J48:J56,L48:L56)</f>
+        <v/>
+      </c>
+      <c r="D65" s="110">
+        <f>C65-B65</f>
+        <v/>
+      </c>
+      <c r="E65" s="132">
+        <f>IF(C65&gt;0,D65/C65,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="108" t="inlineStr">
         <is>
           <t>참가자5</t>
         </is>
       </c>
-      <c r="B24" s="107">
-        <f>COUNTIF(F7:F15,"✓")</f>
-        <v/>
-      </c>
-      <c r="C24" s="110">
-        <f>SUMPRODUCT((F7:F15="✓")*1,K7:K15)</f>
-        <v/>
-      </c>
-      <c r="D24" s="110">
-        <f>SUMPRODUCT((F7:F15="✓")*1,L7:L15)</f>
-        <v/>
-      </c>
-      <c r="E24" s="110">
-        <f>D24-C24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="108" t="inlineStr">
+      <c r="B66" s="131">
+        <f>SUMPRODUCT((F9:F13="✓")*1,J9:J13,K9:K13)+SUMPRODUCT((F18:F20="✓")*1,J18:J20,K18:K20)+SUMPRODUCT((F25:F27="✓")*1,J25:J27,K25:K27)+SUMPRODUCT((F32:F36="✓")*1,J32:J36,K32:K36)+SUMPRODUCT((F41:F43="✓")*1,J41:J43,K41:K43)+SUMPRODUCT((F48:F56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="C66" s="131">
+        <f>SUMPRODUCT((F9:F13="✓")*1,J9:J13,L9:L13)+SUMPRODUCT((F18:F20="✓")*1,J18:J20,L18:L20)+SUMPRODUCT((F25:F27="✓")*1,J25:J27,L25:L27)+SUMPRODUCT((F32:F36="✓")*1,J32:J36,L32:L36)+SUMPRODUCT((F41:F43="✓")*1,J41:J43,L41:L43)+SUMPRODUCT((F48:F56="✓")*1,J48:J56,L48:L56)</f>
+        <v/>
+      </c>
+      <c r="D66" s="110">
+        <f>C66-B66</f>
+        <v/>
+      </c>
+      <c r="E66" s="132">
+        <f>IF(C66&gt;0,D66/C66,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="108" t="inlineStr">
         <is>
           <t>참가자6</t>
         </is>
       </c>
-      <c r="B25" s="107">
-        <f>COUNTIF(G7:G15,"✓")</f>
-        <v/>
-      </c>
-      <c r="C25" s="110">
-        <f>SUMPRODUCT((G7:G15="✓")*1,K7:K15)</f>
-        <v/>
-      </c>
-      <c r="D25" s="110">
-        <f>SUMPRODUCT((G7:G15="✓")*1,L7:L15)</f>
-        <v/>
-      </c>
-      <c r="E25" s="110">
-        <f>D25-C25</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="108" t="inlineStr">
+      <c r="B67" s="131">
+        <f>SUMPRODUCT((G9:G13="✓")*1,J9:J13,K9:K13)+SUMPRODUCT((G18:G20="✓")*1,J18:J20,K18:K20)+SUMPRODUCT((G25:G27="✓")*1,J25:J27,K25:K27)+SUMPRODUCT((G32:G36="✓")*1,J32:J36,K32:K36)+SUMPRODUCT((G41:G43="✓")*1,J41:J43,K41:K43)+SUMPRODUCT((G48:G56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="C67" s="131">
+        <f>SUMPRODUCT((G9:G13="✓")*1,J9:J13,L9:L13)+SUMPRODUCT((G18:G20="✓")*1,J18:J20,L18:L20)+SUMPRODUCT((G25:G27="✓")*1,J25:J27,L25:L27)+SUMPRODUCT((G32:G36="✓")*1,J32:J36,L32:L36)+SUMPRODUCT((G41:G43="✓")*1,J41:J43,L41:L43)+SUMPRODUCT((G48:G56="✓")*1,J48:J56,L48:L56)</f>
+        <v/>
+      </c>
+      <c r="D67" s="110">
+        <f>C67-B67</f>
+        <v/>
+      </c>
+      <c r="E67" s="132">
+        <f>IF(C67&gt;0,D67/C67,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="108" t="inlineStr">
         <is>
           <t>참가자7</t>
         </is>
       </c>
-      <c r="B26" s="107">
-        <f>COUNTIF(H7:H15,"✓")</f>
-        <v/>
-      </c>
-      <c r="C26" s="110">
-        <f>SUMPRODUCT((H7:H15="✓")*1,K7:K15)</f>
-        <v/>
-      </c>
-      <c r="D26" s="110">
-        <f>SUMPRODUCT((H7:H15="✓")*1,L7:L15)</f>
-        <v/>
-      </c>
-      <c r="E26" s="110">
-        <f>D26-C26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="108" t="inlineStr">
+      <c r="B68" s="131">
+        <f>SUMPRODUCT((H9:H13="✓")*1,J9:J13,K9:K13)+SUMPRODUCT((H18:H20="✓")*1,J18:J20,K18:K20)+SUMPRODUCT((H25:H27="✓")*1,J25:J27,K25:K27)+SUMPRODUCT((H32:H36="✓")*1,J32:J36,K32:K36)+SUMPRODUCT((H41:H43="✓")*1,J41:J43,K41:K43)+SUMPRODUCT((H48:H56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="C68" s="131">
+        <f>SUMPRODUCT((H9:H13="✓")*1,J9:J13,L9:L13)+SUMPRODUCT((H18:H20="✓")*1,J18:J20,L18:L20)+SUMPRODUCT((H25:H27="✓")*1,J25:J27,L25:L27)+SUMPRODUCT((H32:H36="✓")*1,J32:J36,L32:L36)+SUMPRODUCT((H41:H43="✓")*1,J41:J43,L41:L43)+SUMPRODUCT((H48:H56="✓")*1,J48:J56,L48:L56)</f>
+        <v/>
+      </c>
+      <c r="D68" s="110">
+        <f>C68-B68</f>
+        <v/>
+      </c>
+      <c r="E68" s="132">
+        <f>IF(C68&gt;0,D68/C68,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="108" t="inlineStr">
         <is>
           <t>참가자8</t>
         </is>
       </c>
-      <c r="B27" s="107">
-        <f>COUNTIF(I7:I15,"✓")</f>
-        <v/>
-      </c>
-      <c r="C27" s="110">
-        <f>SUMPRODUCT((I7:I15="✓")*1,K7:K15)</f>
-        <v/>
-      </c>
-      <c r="D27" s="110">
-        <f>SUMPRODUCT((I7:I15="✓")*1,L7:L15)</f>
-        <v/>
-      </c>
-      <c r="E27" s="110">
-        <f>D27-C27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="115" t="inlineStr">
+      <c r="B69" s="131">
+        <f>SUMPRODUCT((I9:I13="✓")*1,J9:J13,K9:K13)+SUMPRODUCT((I18:I20="✓")*1,J18:J20,K18:K20)+SUMPRODUCT((I25:I27="✓")*1,J25:J27,K25:K27)+SUMPRODUCT((I32:I36="✓")*1,J32:J36,K32:K36)+SUMPRODUCT((I41:I43="✓")*1,J41:J43,K41:K43)+SUMPRODUCT((I48:I56="✓")*1,J48:J56,K48:K56)</f>
+        <v/>
+      </c>
+      <c r="C69" s="131">
+        <f>SUMPRODUCT((I9:I13="✓")*1,J9:J13,L9:L13)+SUMPRODUCT((I18:I20="✓")*1,J18:J20,L18:L20)+SUMPRODUCT((I25:I27="✓")*1,J25:J27,L25:L27)+SUMPRODUCT((I32:I36="✓")*1,J32:J36,L32:L36)+SUMPRODUCT((I41:I43="✓")*1,J41:J43,L41:L43)+SUMPRODUCT((I48:I56="✓")*1,J48:J56,L48:L56)</f>
+        <v/>
+      </c>
+      <c r="D69" s="110">
+        <f>C69-B69</f>
+        <v/>
+      </c>
+      <c r="E69" s="132">
+        <f>IF(C69&gt;0,D69/C69,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="115" t="inlineStr">
         <is>
           <t>📌 TOTAL</t>
         </is>
       </c>
-      <c r="B28" s="88">
-        <f>SUM(B20:B27)</f>
-        <v/>
-      </c>
-      <c r="C28" s="88">
-        <f>SUM(C20:C27)</f>
-        <v/>
-      </c>
-      <c r="D28" s="88">
-        <f>SUM(D20:D27)</f>
-        <v/>
-      </c>
-      <c r="E28" s="88">
-        <f>SUM(E20:E27)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="116" t="inlineStr">
-        <is>
-          <t>✓Check (0=OK):</t>
-        </is>
-      </c>
-      <c r="C29" s="117">
-        <f>C28-K16</f>
-        <v/>
-      </c>
-      <c r="D29" s="118">
-        <f>IF(C29=0,"✅ 정확","❌ 불일치")</f>
-        <v/>
-      </c>
+      <c r="B70" s="88">
+        <f>SUM(B62:B69)</f>
+        <v/>
+      </c>
+      <c r="C70" s="88">
+        <f>SUM(C62:C69)</f>
+        <v/>
+      </c>
+      <c r="D70" s="88">
+        <f>SUM(D62:D69)</f>
+        <v/>
+      </c>
+      <c r="E70" s="91">
+        <f>IF(C70&gt;0,D70/C70,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="124" t="inlineStr">
+        <is>
+          <t>🔍 CROSS-CHECK vs Package Selector</t>
+        </is>
+      </c>
+      <c r="B72" s="125" t="n"/>
+      <c r="C72" s="125" t="n"/>
+      <c r="D72" s="125" t="n"/>
+      <c r="E72" s="125" t="n"/>
+      <c r="F72" s="125" t="n"/>
+      <c r="G72" s="125" t="n"/>
+      <c r="H72" s="125" t="n"/>
+      <c r="I72" s="125" t="n"/>
+      <c r="J72" s="125" t="n"/>
+      <c r="K72" s="125" t="n"/>
+      <c r="L72" s="125" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="126" t="inlineStr">
+        <is>
+          <t>Package Selector Grand Total Cost:</t>
+        </is>
+      </c>
+      <c r="B73" s="133">
+        <f>'Package Selector'!G72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="126" t="inlineStr">
+        <is>
+          <t>Package Selector 2 Grand Total Cost:</t>
+        </is>
+      </c>
+      <c r="B74" s="133">
+        <f>B70</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="116" t="inlineStr">
+        <is>
+          <t>Difference:</t>
+        </is>
+      </c>
+      <c r="B75" s="117">
+        <f>B74-B73</f>
+        <v/>
+      </c>
+      <c r="C75" s="118">
+        <f>IF(B75=0,"✅ MATCH","❌ MISMATCH")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="134" t="inlineStr">
+        <is>
+          <t>⚠️ DUPLICATE ITEMS (중복항목)</t>
+        </is>
+      </c>
+      <c r="B77" s="135" t="n"/>
+      <c r="C77" s="135" t="n"/>
+      <c r="D77" s="135" t="n"/>
+      <c r="E77" s="135" t="n"/>
+      <c r="F77" s="135" t="n"/>
+      <c r="G77" s="135" t="n"/>
+      <c r="H77" s="135" t="n"/>
+      <c r="I77" s="135" t="n"/>
+      <c r="J77" s="135" t="n"/>
+      <c r="K77" s="135" t="n"/>
+      <c r="L77" s="135" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="136" t="inlineStr">
+        <is>
+          <t>중복 발생 항목:</t>
+        </is>
+      </c>
+      <c r="B78" s="136">
+        <f>IF(COUNTIF(O:O,"&gt;0")=0,"✅ 중복 없음","❌ "&amp;COUNTIF(O:O,"&gt;0")&amp;"건 중복 — 위 O열 빨간셀 확인")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="124" t="inlineStr">
+        <is>
+          <t>💡 USAGE TIPS</t>
+        </is>
+      </c>
+      <c r="B80" s="125" t="n"/>
+      <c r="C80" s="125" t="n"/>
+      <c r="D80" s="125" t="n"/>
+      <c r="E80" s="125" t="n"/>
+      <c r="F80" s="125" t="n"/>
+      <c r="G80" s="125" t="n"/>
+      <c r="H80" s="125" t="n"/>
+      <c r="I80" s="125" t="n"/>
+      <c r="J80" s="125" t="n"/>
+      <c r="K80" s="125" t="n"/>
+      <c r="L80" s="125" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="108" t="inlineStr">
+        <is>
+          <t>① A열: 드롭다운에서 항목 선택 (Master Data 연동)</t>
+        </is>
+      </c>
+      <c r="B81" s="81" t="n"/>
+      <c r="C81" s="81" t="n"/>
+      <c r="D81" s="81" t="n"/>
+      <c r="E81" s="81" t="n"/>
+      <c r="F81" s="81" t="n"/>
+      <c r="G81" s="81" t="n"/>
+      <c r="H81" s="81" t="n"/>
+      <c r="I81" s="81" t="n"/>
+      <c r="J81" s="81" t="n"/>
+      <c r="K81" s="81" t="n"/>
+      <c r="L81" s="81" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="108" t="inlineStr">
+        <is>
+          <t>② 참가자열(B~I): ✓ 체크 = 해당 참가자에게 이 항목 포함</t>
+        </is>
+      </c>
+      <c r="B82" s="81" t="n"/>
+      <c r="C82" s="81" t="n"/>
+      <c r="D82" s="81" t="n"/>
+      <c r="E82" s="81" t="n"/>
+      <c r="F82" s="81" t="n"/>
+      <c r="G82" s="81" t="n"/>
+      <c r="H82" s="81" t="n"/>
+      <c r="I82" s="81" t="n"/>
+      <c r="J82" s="81" t="n"/>
+      <c r="K82" s="81" t="n"/>
+      <c r="L82" s="81" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="108" t="inlineStr">
+        <is>
+          <t>③ Qty/p: 1인당 수량 (골프: 라운드수, 호텔: 박수, 식사: 끼니수)</t>
+        </is>
+      </c>
+      <c r="B83" s="81" t="n"/>
+      <c r="C83" s="81" t="n"/>
+      <c r="D83" s="81" t="n"/>
+      <c r="E83" s="81" t="n"/>
+      <c r="F83" s="81" t="n"/>
+      <c r="G83" s="81" t="n"/>
+      <c r="H83" s="81" t="n"/>
+      <c r="I83" s="81" t="n"/>
+      <c r="J83" s="81" t="n"/>
+      <c r="K83" s="81" t="n"/>
+      <c r="L83" s="81" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="108" t="inlineStr">
+        <is>
+          <t>④ 중복항목: 같은 섹션 내 동일항목 중복선택 → O열 빨간불</t>
+        </is>
+      </c>
+      <c r="B84" s="81" t="n"/>
+      <c r="C84" s="81" t="n"/>
+      <c r="D84" s="81" t="n"/>
+      <c r="E84" s="81" t="n"/>
+      <c r="F84" s="81" t="n"/>
+      <c r="G84" s="81" t="n"/>
+      <c r="H84" s="81" t="n"/>
+      <c r="I84" s="81" t="n"/>
+      <c r="J84" s="81" t="n"/>
+      <c r="K84" s="81" t="n"/>
+      <c r="L84" s="81" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="108" t="inlineStr">
+        <is>
+          <t>⑤ 교차검증: Package Selector 총액과 일치여부 자동확인</t>
+        </is>
+      </c>
+      <c r="B85" s="81" t="n"/>
+      <c r="C85" s="81" t="n"/>
+      <c r="D85" s="81" t="n"/>
+      <c r="E85" s="81" t="n"/>
+      <c r="F85" s="81" t="n"/>
+      <c r="G85" s="81" t="n"/>
+      <c r="H85" s="81" t="n"/>
+      <c r="I85" s="81" t="n"/>
+      <c r="J85" s="81" t="n"/>
+      <c r="K85" s="81" t="n"/>
+      <c r="L85" s="81" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="108" t="inlineStr">
+        <is>
+          <t>⑥ 웹사이트 적용: 이 시트 구조 그대로 interactive form 구현 가능</t>
+        </is>
+      </c>
+      <c r="B86" s="81" t="n"/>
+      <c r="C86" s="81" t="n"/>
+      <c r="D86" s="81" t="n"/>
+      <c r="E86" s="81" t="n"/>
+      <c r="F86" s="81" t="n"/>
+      <c r="G86" s="81" t="n"/>
+      <c r="H86" s="81" t="n"/>
+      <c r="I86" s="81" t="n"/>
+      <c r="J86" s="81" t="n"/>
+      <c r="K86" s="81" t="n"/>
+      <c r="L86" s="81" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="18">
+    <mergeCell ref="A30:L30"/>
     <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A16:L16"/>
+    <mergeCell ref="A72:L72"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A60:L60"/>
+    <mergeCell ref="A21"/>
+    <mergeCell ref="A44"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A46:L46"/>
+    <mergeCell ref="A57"/>
+    <mergeCell ref="A77:L77"/>
+    <mergeCell ref="A80:L80"/>
+    <mergeCell ref="A28"/>
+    <mergeCell ref="A14"/>
+    <mergeCell ref="A39:L39"/>
+    <mergeCell ref="A37"/>
   </mergeCells>
-  <conditionalFormatting sqref="M7">
-    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+  <conditionalFormatting sqref="A9">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M8">
+  <conditionalFormatting sqref="O9">
     <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M9">
-    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="0">
+  <conditionalFormatting sqref="A10">
+    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M10">
+  <conditionalFormatting sqref="O10">
     <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M11">
-    <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="0">
+  <conditionalFormatting sqref="A11">
+    <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M12">
+  <conditionalFormatting sqref="O11">
     <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M13">
-    <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="0">
+  <conditionalFormatting sqref="A12">
+    <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M14">
+  <conditionalFormatting sqref="O12">
     <cfRule type="cellIs" priority="8" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M15">
-    <cfRule type="cellIs" priority="9" operator="greaterThan" dxfId="0">
+  <conditionalFormatting sqref="A13">
+    <cfRule type="cellIs" priority="9" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C29">
-    <cfRule type="cellIs" priority="10" operator="notEqual" dxfId="1">
+  <conditionalFormatting sqref="O13">
+    <cfRule type="cellIs" priority="10" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="A7 A8 A9 A10 A11 A12 A13 A14 A15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 액티비티를 선택하세요" type="list">
+  <conditionalFormatting sqref="A18">
+    <cfRule type="cellIs" priority="11" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O18">
+    <cfRule type="cellIs" priority="12" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A19">
+    <cfRule type="cellIs" priority="13" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O19">
+    <cfRule type="cellIs" priority="14" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A20">
+    <cfRule type="cellIs" priority="15" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O20">
+    <cfRule type="cellIs" priority="16" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A25">
+    <cfRule type="cellIs" priority="17" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O25">
+    <cfRule type="cellIs" priority="18" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A26">
+    <cfRule type="cellIs" priority="19" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O26">
+    <cfRule type="cellIs" priority="20" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A27">
+    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O27">
+    <cfRule type="cellIs" priority="22" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A32">
+    <cfRule type="cellIs" priority="23" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O32">
+    <cfRule type="cellIs" priority="24" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A33">
+    <cfRule type="cellIs" priority="25" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O33">
+    <cfRule type="cellIs" priority="26" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A34">
+    <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O34">
+    <cfRule type="cellIs" priority="28" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A35">
+    <cfRule type="cellIs" priority="29" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O35">
+    <cfRule type="cellIs" priority="30" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A36">
+    <cfRule type="cellIs" priority="31" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O36">
+    <cfRule type="cellIs" priority="32" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A41">
+    <cfRule type="cellIs" priority="33" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O41">
+    <cfRule type="cellIs" priority="34" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A42">
+    <cfRule type="cellIs" priority="35" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O42">
+    <cfRule type="cellIs" priority="36" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A43">
+    <cfRule type="cellIs" priority="37" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O43">
+    <cfRule type="cellIs" priority="38" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A48">
+    <cfRule type="cellIs" priority="39" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O48">
+    <cfRule type="cellIs" priority="40" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A49">
+    <cfRule type="cellIs" priority="41" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O49">
+    <cfRule type="cellIs" priority="42" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A50">
+    <cfRule type="cellIs" priority="43" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O50">
+    <cfRule type="cellIs" priority="44" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A51">
+    <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O51">
+    <cfRule type="cellIs" priority="46" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A52">
+    <cfRule type="cellIs" priority="47" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O52">
+    <cfRule type="cellIs" priority="48" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A53">
+    <cfRule type="cellIs" priority="49" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O53">
+    <cfRule type="cellIs" priority="50" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A54">
+    <cfRule type="cellIs" priority="51" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O54">
+    <cfRule type="cellIs" priority="52" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A55">
+    <cfRule type="cellIs" priority="53" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O55">
+    <cfRule type="cellIs" priority="54" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A56">
+    <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O56">
+    <cfRule type="cellIs" priority="56" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B75">
+    <cfRule type="cellIs" priority="57" operator="notEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="7">
+    <dataValidation sqref="B9 B10 B11 B12 B13 B18 B19 B20 B25 B26 B27 B32 B33 B34 B35 B36 B41 B42 B43 B48 B49 B50 B51 B52 B53 B54 B55 B56 C9 C10 C11 C12 C13 C18 C19 C20 C25 C26 C27 C32 C33 C34 C35 C36 C41 C42 C43 C48 C49 C50 C51 C52 C53 C54 C55 C56 D9 D10 D11 D12 D13 D18 D19 D20 D25 D26 D27 D32 D33 D34 D35 D36 D41 D42 D43 D48 D49 D50 D51 D52 D53 D54 D55 D56 E9 E10 E11 E12 E13 E18 E19 E20 E25 E26 E27 E32 E33 E34 E35 E36 E41 E42 E43 E48 E49 E50 E51 E52 E53 E54 E55 E56 F9 F10 F11 F12 F13 F18 F19 F20 F25 F26 F27 F32 F33 F34 F35 F36 F41 F42 F43 F48 F49 F50 F51 F52 F53 F54 F55 F56 G9 G10 G11 G12 G13 G18 G19 G20 G25 G26 G27 G32 G33 G34 G35 G36 G41 G42 G43 G48 G49 G50 G51 G52 G53 G54 G55 G56 H9 H10 H11 H12 H13 H18 H19 H20 H25 H26 H27 H32 H33 H34 H35 H36 H41 H42 H43 H48 H49 H50 H51 H52 H53 H54 H55 H56 I9 I10 I11 I12 I13 I18 I19 I20 I25 I26 I27 I32 I33 I34 I35 I36 I41 I42 I43 I48 I49 I50 I51 I52 I53 I54 I55 I56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓,"</formula1>
+    </dataValidation>
+    <dataValidation sqref="A9 A10 A11 A12 A13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$7:$A$14</formula1>
+    </dataValidation>
+    <dataValidation sqref="A18 A19 A20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$19:$A$24</formula1>
+    </dataValidation>
+    <dataValidation sqref="A25 A26 A27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$28:$A$34</formula1>
+    </dataValidation>
+    <dataValidation sqref="A32 A33 A34 A35 A36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$38:$A$46</formula1>
+    </dataValidation>
+    <dataValidation sqref="A41 A42 A43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
+      <formula1>'Master Data'!$A$50:$A$56</formula1>
+    </dataValidation>
+    <dataValidation sqref="A48 A49 A50 A51 A52 A53 A54 A55 A56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="올바른 항목을 선택하세요" type="list">
       <formula1>'Master Data'!$A$86:$A$94</formula1>
-    </dataValidation>
-    <dataValidation sqref="B7 B8 B9 B10 B11 B12 B13 B14 B15 C7 C8 C9 C10 C11 C12 C13 C14 C15 D7 D8 D9 D10 D11 D12 D13 D14 D15 E7 E8 E9 E10 E11 E12 E13 E14 E15 F7 F8 F9 F10 F11 F12 F13 F14 F15 G7 G8 G9 G10 G11 G12 G13 G14 G15 H7 H8 H9 H10 H11 H12 H13 H14 H15 I7 I8 I9 I10 I11 I12 I13 I14 I15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"✓,"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7023,7 +8838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="42" min="1" max="1"/>
@@ -7032,12 +8847,13 @@
     <col width="14" customWidth="1" style="42" min="4" max="4"/>
     <col width="14" customWidth="1" style="42" min="5" max="5"/>
     <col width="14" customWidth="1" style="42" min="6" max="6"/>
+    <col width="14" customWidth="1" style="42" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="103" t="inlineStr">
         <is>
-          <t>📊 PROFIT SUMMARY 2 — Activity Sub-Category Breakdown</t>
+          <t>📊 PROFIT SUMMARY 2 — Category + Per Person Breakdown</t>
         </is>
       </c>
       <c r="B1" s="104" t="n"/>
@@ -7045,310 +8861,607 @@
       <c r="D1" s="104" t="n"/>
       <c r="E1" s="104" t="n"/>
       <c r="F1" s="104" t="n"/>
+      <c r="G1" s="104" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="105" t="inlineStr">
         <is>
-          <t>⬇️ 'Package Selector 2' ✓체크 기반 자동 분석 | Sports/Outdoor 서브카테고리 분류</t>
+          <t>⬇️ 'Package Selector 2' ✓체크 기반 자동 분석 | 카테고리별 + 참가자별</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="119" t="inlineStr">
         <is>
-          <t>Category / Activity</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="B4" s="98" t="inlineStr">
         <is>
-          <t>Participants</t>
+          <t>Total Cost</t>
         </is>
       </c>
       <c r="C4" s="98" t="inlineStr">
         <is>
-          <t>Cost/Person</t>
+          <t>Total Sell</t>
         </is>
       </c>
       <c r="D4" s="98" t="inlineStr">
         <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="E4" s="98" t="inlineStr">
+        <is>
+          <t>Margin%</t>
+        </is>
+      </c>
+      <c r="F4" s="98" t="inlineStr">
+        <is>
+          <t>Per Person</t>
+        </is>
+      </c>
+      <c r="G4" s="98" t="inlineStr">
+        <is>
+          <t>% of Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="136" t="inlineStr">
+        <is>
+          <t>GOLF</t>
+        </is>
+      </c>
+      <c r="B5" s="84">
+        <f>'Package Selector 2'!K14</f>
+        <v/>
+      </c>
+      <c r="C5" s="84">
+        <f>'Package Selector 2'!L14</f>
+        <v/>
+      </c>
+      <c r="D5" s="84">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="137">
+        <f>IF(C5&gt;0,D5/C5,0)</f>
+        <v/>
+      </c>
+      <c r="F5" s="84">
+        <f>IF('Package Selector'!G5&gt;0,B5/'Package Selector'!G5,0)</f>
+        <v/>
+      </c>
+      <c r="G5" s="137">
+        <f>IF(B11&gt;0,B5/B11,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="136" t="inlineStr">
+        <is>
+          <t>HOTEL</t>
+        </is>
+      </c>
+      <c r="B6" s="84">
+        <f>'Package Selector 2'!K21</f>
+        <v/>
+      </c>
+      <c r="C6" s="84">
+        <f>'Package Selector 2'!L21</f>
+        <v/>
+      </c>
+      <c r="D6" s="84">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="137">
+        <f>IF(C6&gt;0,D6/C6,0)</f>
+        <v/>
+      </c>
+      <c r="F6" s="84">
+        <f>IF('Package Selector'!G5&gt;0,B6/'Package Selector'!G5,0)</f>
+        <v/>
+      </c>
+      <c r="G6" s="137">
+        <f>IF(B12&gt;0,B6/B12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="136" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="B7" s="84">
+        <f>'Package Selector 2'!K28</f>
+        <v/>
+      </c>
+      <c r="C7" s="84">
+        <f>'Package Selector 2'!L28</f>
+        <v/>
+      </c>
+      <c r="D7" s="84">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="137">
+        <f>IF(C7&gt;0,D7/C7,0)</f>
+        <v/>
+      </c>
+      <c r="F7" s="84">
+        <f>IF('Package Selector'!G5&gt;0,B7/'Package Selector'!G5,0)</f>
+        <v/>
+      </c>
+      <c r="G7" s="137">
+        <f>IF(B13&gt;0,B7/B13,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="136" t="inlineStr">
+        <is>
+          <t>MEALS</t>
+        </is>
+      </c>
+      <c r="B8" s="84">
+        <f>'Package Selector 2'!K37</f>
+        <v/>
+      </c>
+      <c r="C8" s="84">
+        <f>'Package Selector 2'!L37</f>
+        <v/>
+      </c>
+      <c r="D8" s="84">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="137">
+        <f>IF(C8&gt;0,D8/C8,0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="84">
+        <f>IF('Package Selector'!G5&gt;0,B8/'Package Selector'!G5,0)</f>
+        <v/>
+      </c>
+      <c r="G8" s="137">
+        <f>IF(B14&gt;0,B8/B14,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="136" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="B9" s="84">
+        <f>'Package Selector 2'!K44</f>
+        <v/>
+      </c>
+      <c r="C9" s="84">
+        <f>'Package Selector 2'!L44</f>
+        <v/>
+      </c>
+      <c r="D9" s="84">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="137">
+        <f>IF(C9&gt;0,D9/C9,0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="84">
+        <f>IF('Package Selector'!G5&gt;0,B9/'Package Selector'!G5,0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="137">
+        <f>IF(B15&gt;0,B9/B15,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="136" t="inlineStr">
+        <is>
+          <t>ACTIVITIES</t>
+        </is>
+      </c>
+      <c r="B10" s="84">
+        <f>'Package Selector 2'!K57</f>
+        <v/>
+      </c>
+      <c r="C10" s="84">
+        <f>'Package Selector 2'!L57</f>
+        <v/>
+      </c>
+      <c r="D10" s="84">
+        <f>C10-B10</f>
+        <v/>
+      </c>
+      <c r="E10" s="137">
+        <f>IF(C10&gt;0,D10/C10,0)</f>
+        <v/>
+      </c>
+      <c r="F10" s="84">
+        <f>IF('Package Selector'!G5&gt;0,B10/'Package Selector'!G5,0)</f>
+        <v/>
+      </c>
+      <c r="G10" s="137">
+        <f>IF(B16&gt;0,B10/B16,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="115" t="inlineStr">
+        <is>
+          <t>📌 GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="B11" s="88">
+        <f>SUM(B5:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="88">
+        <f>SUM(C5:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="88">
+        <f>SUM(D5:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="91">
+        <f>IF(C11&gt;0,D11/C11,0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="88">
+        <f>IF('Package Selector'!G5&gt;0,B11/'Package Selector'!G5,0)</f>
+        <v/>
+      </c>
+      <c r="G11" s="91">
+        <f>1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="103" t="inlineStr">
+        <is>
+          <t>👤 PER PERSON DETAIL</t>
+        </is>
+      </c>
+      <c r="B13" s="104" t="n"/>
+      <c r="C13" s="104" t="n"/>
+      <c r="D13" s="104" t="n"/>
+      <c r="E13" s="104" t="n"/>
+      <c r="F13" s="104" t="n"/>
+      <c r="G13" s="104" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="119" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="B14" s="98" t="inlineStr">
+        <is>
           <t>Total Cost</t>
         </is>
       </c>
-      <c r="E4" s="98" t="inlineStr">
+      <c r="C14" s="98" t="inlineStr">
         <is>
           <t>Total Sell</t>
         </is>
       </c>
-      <c r="F4" s="98" t="inlineStr">
-        <is>
-          <t>Total Margin</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="120" t="inlineStr">
-        <is>
-          <t>🎫 SPORTS &amp; EVENTS</t>
-        </is>
-      </c>
-      <c r="B5" s="121" t="n"/>
-      <c r="C5" s="121" t="n"/>
-      <c r="D5" s="121" t="n"/>
-      <c r="E5" s="121" t="n"/>
-      <c r="F5" s="121" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NBA/MLB Game (Ticket)</t>
-        </is>
-      </c>
-      <c r="B6" s="122">
-        <f>'Package Selector 2'!J7</f>
-        <v/>
-      </c>
-      <c r="C6" s="84">
-        <f>'Package Selector 2'!K7</f>
-        <v/>
-      </c>
-      <c r="D6" s="84">
-        <f>B6*C6</f>
-        <v/>
-      </c>
-      <c r="E6" s="84">
-        <f>B6*'Package Selector 2'!L7</f>
-        <v/>
-      </c>
-      <c r="F6" s="84">
-        <f>E6-D6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Sports Bar Experience</t>
-        </is>
-      </c>
-      <c r="B7" s="122">
-        <f>'Package Selector 2'!J8</f>
-        <v/>
-      </c>
-      <c r="C7" s="84">
-        <f>'Package Selector 2'!K8</f>
-        <v/>
-      </c>
-      <c r="D7" s="84">
-        <f>B7*C7</f>
-        <v/>
-      </c>
-      <c r="E7" s="84">
-        <f>B7*'Package Selector 2'!L8</f>
-        <v/>
-      </c>
-      <c r="F7" s="84">
-        <f>E7-D7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="123" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SPORTS SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="D8" s="88">
-        <f>SUM(D6:D7)</f>
-        <v/>
-      </c>
-      <c r="E8" s="88">
-        <f>SUM(E6:E7)</f>
-        <v/>
-      </c>
-      <c r="F8" s="88">
-        <f>SUM(F6:F7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="120" t="inlineStr">
-        <is>
-          <t>🌿 OUTDOOR &amp; NATURE</t>
-        </is>
-      </c>
-      <c r="B10" s="121" t="n"/>
-      <c r="C10" s="121" t="n"/>
-      <c r="D10" s="121" t="n"/>
-      <c r="E10" s="121" t="n"/>
-      <c r="F10" s="121" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Local Hiking (Griffith/Runyon)</t>
-        </is>
-      </c>
-      <c r="B11" s="122">
-        <f>'Package Selector 2'!J9</f>
-        <v/>
-      </c>
-      <c r="C11" s="84">
-        <f>'Package Selector 2'!K9</f>
-        <v/>
-      </c>
-      <c r="D11" s="84">
-        <f>B11*C11</f>
-        <v/>
-      </c>
-      <c r="E11" s="84">
-        <f>B11*'Package Selector 2'!L9</f>
-        <v/>
-      </c>
-      <c r="F11" s="84">
-        <f>E11-D11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Beach/Surf Lesson</t>
-        </is>
-      </c>
-      <c r="B12" s="122">
-        <f>'Package Selector 2'!J10</f>
-        <v/>
-      </c>
-      <c r="C12" s="84">
-        <f>'Package Selector 2'!K10</f>
-        <v/>
-      </c>
-      <c r="D12" s="84">
-        <f>B12*C12</f>
-        <v/>
-      </c>
-      <c r="E12" s="84">
-        <f>B12*'Package Selector 2'!L10</f>
-        <v/>
-      </c>
-      <c r="F12" s="84">
-        <f>E12-D12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="123" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  OUTDOOR SUBTOTAL</t>
-        </is>
-      </c>
-      <c r="D13" s="88">
-        <f>SUM(D11:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="88">
-        <f>SUM(E11:E12)</f>
-        <v/>
-      </c>
-      <c r="F13" s="88">
-        <f>SUM(F11:F12)</f>
-        <v/>
+      <c r="D14" s="98" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="E14" s="98" t="inlineStr">
+        <is>
+          <t>Margin%</t>
+        </is>
+      </c>
+      <c r="F14" s="98" t="inlineStr">
+        <is>
+          <t># Items</t>
+        </is>
+      </c>
+      <c r="G14" s="98" t="inlineStr">
+        <is>
+          <t>✓Check</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="103" t="inlineStr">
-        <is>
-          <t>🏆 ACTIVITIES GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="B15" s="104" t="n"/>
-      <c r="C15" s="104" t="n"/>
-      <c r="D15" s="104" t="n"/>
-      <c r="E15" s="104" t="n"/>
-      <c r="F15" s="104" t="n"/>
+      <c r="A15" s="108" t="inlineStr">
+        <is>
+          <t>참가자1</t>
+        </is>
+      </c>
+      <c r="B15" s="84">
+        <f>'Package Selector 2'!B62</f>
+        <v/>
+      </c>
+      <c r="C15" s="84">
+        <f>'Package Selector 2'!C62</f>
+        <v/>
+      </c>
+      <c r="D15" s="84">
+        <f>'Package Selector 2'!D62</f>
+        <v/>
+      </c>
+      <c r="E15" s="137">
+        <f>'Package Selector 2'!E62</f>
+        <v/>
+      </c>
+      <c r="F15" s="122">
+        <f>COUNTIF('Package Selector 2'!B9:B13,"✓")+COUNTIF('Package Selector 2'!B18:B20,"✓")+COUNTIF('Package Selector 2'!B25:B27,"✓")+COUNTIF('Package Selector 2'!B32:B36,"✓")+COUNTIF('Package Selector 2'!B41:B43,"✓")+COUNTIF('Package Selector 2'!B48:B56,"✓")</f>
+        <v/>
+      </c>
+      <c r="G15" s="84">
+        <f>'Package Selector 2'!D62</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="106" t="inlineStr">
-        <is>
-          <t>📌 TOTAL ALL ACTIVITIES</t>
-        </is>
-      </c>
-      <c r="D16" s="88">
-        <f>D8+D13</f>
-        <v/>
-      </c>
-      <c r="E16" s="88">
-        <f>E8+E13</f>
-        <v/>
-      </c>
-      <c r="F16" s="88">
-        <f>F8+F13</f>
+      <c r="A16" s="108" t="inlineStr">
+        <is>
+          <t>참가자2</t>
+        </is>
+      </c>
+      <c r="B16" s="84">
+        <f>'Package Selector 2'!B63</f>
+        <v/>
+      </c>
+      <c r="C16" s="84">
+        <f>'Package Selector 2'!C63</f>
+        <v/>
+      </c>
+      <c r="D16" s="84">
+        <f>'Package Selector 2'!D63</f>
+        <v/>
+      </c>
+      <c r="E16" s="137">
+        <f>'Package Selector 2'!E63</f>
+        <v/>
+      </c>
+      <c r="F16" s="122">
+        <f>COUNTIF('Package Selector 2'!C9:C13,"✓")+COUNTIF('Package Selector 2'!C18:C20,"✓")+COUNTIF('Package Selector 2'!C25:C27,"✓")+COUNTIF('Package Selector 2'!C32:C36,"✓")+COUNTIF('Package Selector 2'!C41:C43,"✓")+COUNTIF('Package Selector 2'!C48:C56,"✓")</f>
+        <v/>
+      </c>
+      <c r="G16" s="84">
+        <f>'Package Selector 2'!D63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="108" t="inlineStr">
+        <is>
+          <t>참가자3</t>
+        </is>
+      </c>
+      <c r="B17" s="84">
+        <f>'Package Selector 2'!B64</f>
+        <v/>
+      </c>
+      <c r="C17" s="84">
+        <f>'Package Selector 2'!C64</f>
+        <v/>
+      </c>
+      <c r="D17" s="84">
+        <f>'Package Selector 2'!D64</f>
+        <v/>
+      </c>
+      <c r="E17" s="137">
+        <f>'Package Selector 2'!E64</f>
+        <v/>
+      </c>
+      <c r="F17" s="122">
+        <f>COUNTIF('Package Selector 2'!D9:D13,"✓")+COUNTIF('Package Selector 2'!D18:D20,"✓")+COUNTIF('Package Selector 2'!D25:D27,"✓")+COUNTIF('Package Selector 2'!D32:D36,"✓")+COUNTIF('Package Selector 2'!D41:D43,"✓")+COUNTIF('Package Selector 2'!D48:D56,"✓")</f>
+        <v/>
+      </c>
+      <c r="G17" s="84">
+        <f>'Package Selector 2'!D64</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="124" t="inlineStr">
-        <is>
-          <t>🔍 CROSS-CHECK vs Package Selector</t>
-        </is>
-      </c>
-      <c r="B18" s="125" t="n"/>
-      <c r="C18" s="125" t="n"/>
-      <c r="D18" s="125" t="n"/>
-      <c r="E18" s="125" t="n"/>
-      <c r="F18" s="125" t="n"/>
+      <c r="A18" s="108" t="inlineStr">
+        <is>
+          <t>참가자4</t>
+        </is>
+      </c>
+      <c r="B18" s="84">
+        <f>'Package Selector 2'!B65</f>
+        <v/>
+      </c>
+      <c r="C18" s="84">
+        <f>'Package Selector 2'!C65</f>
+        <v/>
+      </c>
+      <c r="D18" s="84">
+        <f>'Package Selector 2'!D65</f>
+        <v/>
+      </c>
+      <c r="E18" s="137">
+        <f>'Package Selector 2'!E65</f>
+        <v/>
+      </c>
+      <c r="F18" s="122">
+        <f>COUNTIF('Package Selector 2'!E9:E13,"✓")+COUNTIF('Package Selector 2'!E18:E20,"✓")+COUNTIF('Package Selector 2'!E25:E27,"✓")+COUNTIF('Package Selector 2'!E32:E36,"✓")+COUNTIF('Package Selector 2'!E41:E43,"✓")+COUNTIF('Package Selector 2'!E48:E56,"✓")</f>
+        <v/>
+      </c>
+      <c r="G18" s="84">
+        <f>'Package Selector 2'!D65</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="126" t="inlineStr">
-        <is>
-          <t>Package Selector Activities Cost:</t>
-        </is>
+      <c r="A19" s="108" t="inlineStr">
+        <is>
+          <t>참가자5</t>
+        </is>
+      </c>
+      <c r="B19" s="84">
+        <f>'Package Selector 2'!B66</f>
+        <v/>
+      </c>
+      <c r="C19" s="84">
+        <f>'Package Selector 2'!C66</f>
+        <v/>
       </c>
       <c r="D19" s="84">
-        <f>'Package Selector'!G62</f>
+        <f>'Package Selector 2'!D66</f>
+        <v/>
+      </c>
+      <c r="E19" s="137">
+        <f>'Package Selector 2'!E66</f>
+        <v/>
+      </c>
+      <c r="F19" s="122">
+        <f>COUNTIF('Package Selector 2'!F9:F13,"✓")+COUNTIF('Package Selector 2'!F18:F20,"✓")+COUNTIF('Package Selector 2'!F25:F27,"✓")+COUNTIF('Package Selector 2'!F32:F36,"✓")+COUNTIF('Package Selector 2'!F41:F43,"✓")+COUNTIF('Package Selector 2'!F48:F56,"✓")</f>
+        <v/>
+      </c>
+      <c r="G19" s="84">
+        <f>'Package Selector 2'!D66</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="126" t="inlineStr">
-        <is>
-          <t>Package Selector 2 Activities Cost:</t>
-        </is>
+      <c r="A20" s="108" t="inlineStr">
+        <is>
+          <t>참가자6</t>
+        </is>
+      </c>
+      <c r="B20" s="84">
+        <f>'Package Selector 2'!B67</f>
+        <v/>
+      </c>
+      <c r="C20" s="84">
+        <f>'Package Selector 2'!C67</f>
+        <v/>
       </c>
       <c r="D20" s="84">
-        <f>D16</f>
+        <f>'Package Selector 2'!D67</f>
+        <v/>
+      </c>
+      <c r="E20" s="137">
+        <f>'Package Selector 2'!E67</f>
+        <v/>
+      </c>
+      <c r="F20" s="122">
+        <f>COUNTIF('Package Selector 2'!G9:G13,"✓")+COUNTIF('Package Selector 2'!G18:G20,"✓")+COUNTIF('Package Selector 2'!G25:G27,"✓")+COUNTIF('Package Selector 2'!G32:G36,"✓")+COUNTIF('Package Selector 2'!G41:G43,"✓")+COUNTIF('Package Selector 2'!G48:G56,"✓")</f>
+        <v/>
+      </c>
+      <c r="G20" s="84">
+        <f>'Package Selector 2'!D67</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="116" t="inlineStr">
-        <is>
-          <t>Difference:</t>
-        </is>
-      </c>
-      <c r="D21" s="117">
-        <f>D20-D19</f>
-        <v/>
-      </c>
-      <c r="E21" s="118">
-        <f>IF(D21=0,"✅ MATCH","❌ MISMATCH — check selections")</f>
+      <c r="A21" s="108" t="inlineStr">
+        <is>
+          <t>참가자7</t>
+        </is>
+      </c>
+      <c r="B21" s="84">
+        <f>'Package Selector 2'!B68</f>
+        <v/>
+      </c>
+      <c r="C21" s="84">
+        <f>'Package Selector 2'!C68</f>
+        <v/>
+      </c>
+      <c r="D21" s="84">
+        <f>'Package Selector 2'!D68</f>
+        <v/>
+      </c>
+      <c r="E21" s="137">
+        <f>'Package Selector 2'!E68</f>
+        <v/>
+      </c>
+      <c r="F21" s="122">
+        <f>COUNTIF('Package Selector 2'!H9:H13,"✓")+COUNTIF('Package Selector 2'!H18:H20,"✓")+COUNTIF('Package Selector 2'!H25:H27,"✓")+COUNTIF('Package Selector 2'!H32:H36,"✓")+COUNTIF('Package Selector 2'!H41:H43,"✓")+COUNTIF('Package Selector 2'!H48:H56,"✓")</f>
+        <v/>
+      </c>
+      <c r="G21" s="84">
+        <f>'Package Selector 2'!D68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="108" t="inlineStr">
+        <is>
+          <t>참가자8</t>
+        </is>
+      </c>
+      <c r="B22" s="84">
+        <f>'Package Selector 2'!B69</f>
+        <v/>
+      </c>
+      <c r="C22" s="84">
+        <f>'Package Selector 2'!C69</f>
+        <v/>
+      </c>
+      <c r="D22" s="84">
+        <f>'Package Selector 2'!D69</f>
+        <v/>
+      </c>
+      <c r="E22" s="137">
+        <f>'Package Selector 2'!E69</f>
+        <v/>
+      </c>
+      <c r="F22" s="122">
+        <f>COUNTIF('Package Selector 2'!I9:I13,"✓")+COUNTIF('Package Selector 2'!I18:I20,"✓")+COUNTIF('Package Selector 2'!I25:I27,"✓")+COUNTIF('Package Selector 2'!I32:I36,"✓")+COUNTIF('Package Selector 2'!I41:I43,"✓")+COUNTIF('Package Selector 2'!I48:I56,"✓")</f>
+        <v/>
+      </c>
+      <c r="G22" s="84">
+        <f>'Package Selector 2'!D69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="115" t="inlineStr">
+        <is>
+          <t>📌 TOTAL</t>
+        </is>
+      </c>
+      <c r="B23" s="88">
+        <f>SUM(B15:B22)</f>
+        <v/>
+      </c>
+      <c r="C23" s="88">
+        <f>SUM(C15:C22)</f>
+        <v/>
+      </c>
+      <c r="D23" s="88">
+        <f>SUM(D15:D22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="116" t="inlineStr">
+        <is>
+          <t>Cross-check (PP sum = Grand Total):</t>
+        </is>
+      </c>
+      <c r="B24" s="117">
+        <f>B23-B11</f>
+        <v/>
+      </c>
+      <c r="C24" s="118">
+        <f>IF(B24=0,"✅","❌")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A15:F15"/>
+  <mergeCells count="3">
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D21">
-    <cfRule type="cellIs" priority="1" operator="notEqual" dxfId="1">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: unified builder - freeze panes, margin% col, alphabetical sort, checkbox style, P1-4 only, D9 fix, cross-check in frozen area
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -486,7 +486,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="143">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -860,11 +860,17 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
     <dxf>
       <font>
         <b val="1"/>
@@ -907,6 +913,20 @@
         <patternFill patternType="solid">
           <fgColor rgb="FFFFC7CE"/>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00006100"/>
+        <sz val="14"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF92D050"/>
+          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1357,14 +1377,14 @@
     <row r="7">
       <c r="A7" s="70" t="inlineStr">
         <is>
-          <t>Trump National LA</t>
+          <t>Hidden Valley GC</t>
         </is>
       </c>
       <c r="B7" s="71" t="n">
-        <v>210</v>
+        <v>109</v>
       </c>
       <c r="C7" s="71" t="n">
-        <v>210</v>
+        <v>109</v>
       </c>
       <c r="D7" s="5">
         <f>IF(A7="","",C7-B7)</f>
@@ -1407,14 +1427,14 @@
     <row r="9" ht="30.75" customHeight="1" s="42">
       <c r="A9" s="70" t="inlineStr">
         <is>
-          <t>Hidden Valley GC</t>
+          <t>Trump National LA</t>
         </is>
       </c>
       <c r="B9" s="71" t="n">
-        <v>109</v>
+        <v>210</v>
       </c>
       <c r="C9" s="71" t="n">
-        <v>109</v>
+        <v>210</v>
       </c>
       <c r="D9" s="5">
         <f>IF(A9="","",C9-B9)</f>
@@ -1643,14 +1663,14 @@
     <row r="28" ht="16.5" customHeight="1" s="42">
       <c r="A28" s="70" t="inlineStr">
         <is>
-          <t>Driver/Guide + Van (일당)</t>
+          <t>Airport Roundtrip Pickup</t>
         </is>
       </c>
       <c r="B28" s="71" t="n">
-        <v>125</v>
+        <v>75</v>
       </c>
       <c r="C28" s="71" t="n">
-        <v>175</v>
+        <v>120</v>
       </c>
       <c r="D28" s="5">
         <f>IF(A28="","",C28-B28)</f>
@@ -1665,14 +1685,14 @@
     <row r="29">
       <c r="A29" s="70" t="inlineStr">
         <is>
-          <t>Airport Roundtrip Pickup</t>
+          <t>Driver/Guide + Van (일당)</t>
         </is>
       </c>
       <c r="B29" s="71" t="n">
-        <v>75</v>
+        <v>125</v>
       </c>
       <c r="C29" s="71" t="n">
-        <v>120</v>
+        <v>175</v>
       </c>
       <c r="D29" s="5">
         <f>IF(A29="","",C29-B29)</f>
@@ -1801,14 +1821,14 @@
     <row r="39">
       <c r="A39" s="70" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner (Regular)</t>
         </is>
       </c>
       <c r="B39" s="71" t="n">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="C39" s="71" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="D39" s="5">
         <f>IF(A39="","",C39-B39)</f>
@@ -1823,14 +1843,14 @@
     <row r="40">
       <c r="A40" s="70" t="inlineStr">
         <is>
-          <t>Dinner (Regular)</t>
+          <t>Exclusive Dinner (Michelin/Fine)</t>
         </is>
       </c>
       <c r="B40" s="71" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="C40" s="71" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="D40" s="5">
         <f>IF(A40="","",C40-B40)</f>
@@ -1845,14 +1865,14 @@
     <row r="41">
       <c r="A41" s="70" t="inlineStr">
         <is>
-          <t>Exclusive Dinner (Michelin/Fine)</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="B41" s="71" t="n">
-        <v>120</v>
+        <v>40</v>
       </c>
       <c r="C41" s="71" t="n">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="D41" s="5">
         <f>IF(A41="","",C41-B41)</f>
@@ -2028,6 +2048,7 @@
       </c>
       <c r="F55" s="6" t="n"/>
     </row>
+    <row r="56"/>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
         <is>
@@ -2646,7 +2667,7 @@
     <row r="86">
       <c r="A86" s="74" t="inlineStr">
         <is>
-          <t>NBA/MLB Game (Ticket)</t>
+          <t>(New Activity 5)</t>
         </is>
       </c>
       <c r="B86" s="75" t="n">
@@ -2674,7 +2695,7 @@
     <row r="87">
       <c r="A87" s="74" t="inlineStr">
         <is>
-          <t>Sports Bar Experience</t>
+          <t>(New Activity 6)</t>
         </is>
       </c>
       <c r="B87" s="75" t="n">
@@ -2702,7 +2723,7 @@
     <row r="88">
       <c r="A88" s="74" t="inlineStr">
         <is>
-          <t>Local Hiking (Griffith/Runyon)</t>
+          <t>(New Activity 7)</t>
         </is>
       </c>
       <c r="B88" s="75" t="n">
@@ -2730,7 +2751,7 @@
     <row r="89">
       <c r="A89" s="74" t="inlineStr">
         <is>
-          <t>Beach/Surf Lesson</t>
+          <t>(New Activity 8)</t>
         </is>
       </c>
       <c r="B89" s="75" t="n">
@@ -2758,7 +2779,7 @@
     <row r="90">
       <c r="A90" s="74" t="inlineStr">
         <is>
-          <t>(New Activity 5)</t>
+          <t>(New Activity 9)</t>
         </is>
       </c>
       <c r="B90" s="49" t="n"/>
@@ -2774,11 +2795,15 @@
     <row r="91">
       <c r="A91" s="74" t="inlineStr">
         <is>
-          <t>(New Activity 6)</t>
-        </is>
-      </c>
-      <c r="B91" s="49" t="n"/>
-      <c r="C91" s="49" t="n"/>
+          <t>Beach/Surf Lesson</t>
+        </is>
+      </c>
+      <c r="B91" s="49" t="n">
+        <v>60</v>
+      </c>
+      <c r="C91" s="49" t="n">
+        <v>100</v>
+      </c>
       <c r="D91" s="51">
         <f>IF(A91="","",C91-B91)</f>
         <v/>
@@ -2790,11 +2815,15 @@
     <row r="92">
       <c r="A92" s="74" t="inlineStr">
         <is>
-          <t>(New Activity 7)</t>
-        </is>
-      </c>
-      <c r="B92" s="49" t="n"/>
-      <c r="C92" s="49" t="n"/>
+          <t>Local Hiking (Griffith/Runyon)</t>
+        </is>
+      </c>
+      <c r="B92" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="C92" s="49" t="n">
+        <v>30</v>
+      </c>
       <c r="D92" s="51">
         <f>IF(A92="","",C92-B92)</f>
         <v/>
@@ -2806,11 +2835,15 @@
     <row r="93">
       <c r="A93" s="74" t="inlineStr">
         <is>
-          <t>(New Activity 8)</t>
-        </is>
-      </c>
-      <c r="B93" s="49" t="n"/>
-      <c r="C93" s="49" t="n"/>
+          <t>NBA/MLB Game (Ticket)</t>
+        </is>
+      </c>
+      <c r="B93" s="49" t="n">
+        <v>120</v>
+      </c>
+      <c r="C93" s="49" t="n">
+        <v>180</v>
+      </c>
       <c r="D93" s="51">
         <f>IF(A93="","",C93-B93)</f>
         <v/>
@@ -2822,11 +2855,15 @@
     <row r="94">
       <c r="A94" s="74" t="inlineStr">
         <is>
-          <t>(New Activity 9)</t>
-        </is>
-      </c>
-      <c r="B94" s="49" t="n"/>
-      <c r="C94" s="49" t="n"/>
+          <t>Sports Bar Experience</t>
+        </is>
+      </c>
+      <c r="B94" s="49" t="n">
+        <v>60</v>
+      </c>
+      <c r="C94" s="49" t="n">
+        <v>90</v>
+      </c>
       <c r="D94" s="51">
         <f>IF(A94="","",C94-B94)</f>
         <v/>
@@ -3283,24 +3320,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O97"/>
+  <dimension ref="A1:Q76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" style="42" min="1" max="1"/>
-    <col width="8" customWidth="1" style="42" min="2" max="2"/>
+    <col width="28" customWidth="1" style="42" min="1" max="1"/>
+    <col width="7" customWidth="1" style="42" min="2" max="2"/>
     <col width="11" customWidth="1" style="42" min="3" max="3"/>
     <col width="11" customWidth="1" style="42" min="4" max="4"/>
-    <col width="11" customWidth="1" style="42" min="5" max="5"/>
-    <col width="11" customWidth="1" style="42" min="6" max="6"/>
-    <col width="11" customWidth="1" style="42" min="7" max="7"/>
-    <col width="11" customWidth="1" style="42" min="8" max="8"/>
-    <col width="11" customWidth="1" style="42" min="9" max="9"/>
-    <col width="11" customWidth="1" style="42" min="10" max="10"/>
-    <col width="11" customWidth="1" style="42" min="11" max="11"/>
-    <col width="13" customWidth="1" style="42" min="12" max="12"/>
-    <col width="13" customWidth="1" style="42" min="13" max="13"/>
-    <col width="11" customWidth="1" style="42" min="14" max="14"/>
-    <col hidden="1" width="13" customWidth="1" style="42" min="15" max="15"/>
+    <col width="8" customWidth="1" style="42" min="5" max="5"/>
+    <col width="10" customWidth="1" style="42" min="6" max="6"/>
+    <col width="10" customWidth="1" style="42" min="7" max="7"/>
+    <col width="10" customWidth="1" style="42" min="8" max="8"/>
+    <col width="10" customWidth="1" style="42" min="9" max="9"/>
+    <col width="5" customWidth="1" style="42" min="10" max="10"/>
+    <col width="12" customWidth="1" style="42" min="11" max="11"/>
+    <col width="12" customWidth="1" style="42" min="12" max="12"/>
+    <col hidden="1" width="10" customWidth="1" style="42" min="13" max="13"/>
+    <col hidden="1" width="10" customWidth="1" style="42" min="14" max="14"/>
+    <col hidden="1" width="10" customWidth="1" style="42" min="15" max="15"/>
+    <col hidden="1" width="10" customWidth="1" style="42" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" style="42" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3320,13 +3359,11 @@
       <c r="J1" s="104" t="n"/>
       <c r="K1" s="104" t="n"/>
       <c r="L1" s="104" t="n"/>
-      <c r="M1" s="104" t="n"/>
-      <c r="N1" s="104" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="105" t="inlineStr">
         <is>
-          <t>항목 선택 → 참가자 ✓ 체크 → 자동 비용계산</t>
+          <t>항목 선택 → ✓ 체크 → 자동계산 | P1~P4 기본, +버튼으로 P5~P8 확장</t>
         </is>
       </c>
     </row>
@@ -3337,28 +3374,19 @@
         </is>
       </c>
       <c r="B4" s="129" t="inlineStr"/>
-      <c r="C4" s="86" t="n"/>
-      <c r="D4" s="87" t="n"/>
-      <c r="E4" s="106" t="inlineStr">
+      <c r="D4" s="106" t="inlineStr">
         <is>
           <t>Golfers:</t>
         </is>
       </c>
-      <c r="F4" s="138" t="n">
+      <c r="E4" s="138" t="n">
         <v>4</v>
       </c>
-      <c r="G4" s="108" t="inlineStr">
+      <c r="F4" s="108" t="inlineStr">
         <is>
           <t>persons</t>
         </is>
       </c>
-      <c r="I4" s="106" t="inlineStr">
-        <is>
-          <t>Duration:</t>
-        </is>
-      </c>
-      <c r="J4" s="139" t="inlineStr"/>
-      <c r="K4" s="87" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="103" t="inlineStr">
@@ -3377,13 +3405,11 @@
       <c r="J6" s="104" t="n"/>
       <c r="K6" s="104" t="n"/>
       <c r="L6" s="104" t="n"/>
-      <c r="M6" s="104" t="n"/>
-      <c r="N6" s="104" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="140" t="inlineStr">
         <is>
-          <t>Outbound</t>
+          <t>Outbound:</t>
         </is>
       </c>
       <c r="B7" s="126" t="inlineStr">
@@ -3398,7 +3424,7 @@
       </c>
       <c r="D7" s="126" t="inlineStr">
         <is>
-          <t>Flight:</t>
+          <t>Flight#:</t>
         </is>
       </c>
       <c r="E7" s="82" t="inlineStr">
@@ -3408,28 +3434,28 @@
       </c>
       <c r="F7" s="126" t="inlineStr">
         <is>
-          <t>Dep ICN:</t>
+          <t>Dep:</t>
         </is>
       </c>
       <c r="G7" s="122">
-        <f>IF(E7="","",VLOOKUP(E7,'Master Data'!$A$60:$D$69,3,FALSE))</f>
+        <f>IF(E7="","",VLOOKUP(E7,'Master Data'!$A$60:$D$63,3,FALSE))</f>
         <v/>
       </c>
       <c r="H7" s="126" t="inlineStr">
         <is>
-          <t>Arr LAX:</t>
+          <t>Arr:</t>
         </is>
       </c>
       <c r="I7" s="122">
-        <f>IF(E7="","",VLOOKUP(E7,'Master Data'!$A$60:$D$69,4,FALSE))</f>
-        <v/>
-      </c>
-      <c r="K7" s="126" t="inlineStr">
+        <f>IF(E7="","",VLOOKUP(E7,'Master Data'!$A$60:$D$63,4,FALSE))</f>
+        <v/>
+      </c>
+      <c r="J7" s="126" t="inlineStr">
         <is>
           <t>Seat:</t>
         </is>
       </c>
-      <c r="L7" s="82" t="inlineStr">
+      <c r="K7" s="82" t="inlineStr">
         <is>
           <t>Economy</t>
         </is>
@@ -3438,7 +3464,7 @@
     <row r="8">
       <c r="A8" s="140" t="inlineStr">
         <is>
-          <t>Return</t>
+          <t>Return:</t>
         </is>
       </c>
       <c r="B8" s="126" t="inlineStr">
@@ -3453,7 +3479,7 @@
       </c>
       <c r="D8" s="126" t="inlineStr">
         <is>
-          <t>Flight:</t>
+          <t>Flight#:</t>
         </is>
       </c>
       <c r="E8" s="82" t="inlineStr">
@@ -3463,28 +3489,28 @@
       </c>
       <c r="F8" s="126" t="inlineStr">
         <is>
-          <t>Dep LAX:</t>
+          <t>Dep:</t>
         </is>
       </c>
       <c r="G8" s="122">
-        <f>IF(E8="","",VLOOKUP(E8,'Master Data'!$A$74:$D$83,3,FALSE))</f>
+        <f>IF(E8="","",VLOOKUP(E8,'Master Data'!$A$74:$D$77,3,FALSE))</f>
         <v/>
       </c>
       <c r="H8" s="126" t="inlineStr">
         <is>
-          <t>Arr ICN:</t>
+          <t>Arr:</t>
         </is>
       </c>
       <c r="I8" s="122">
-        <f>IF(E8="","",VLOOKUP(E8,'Master Data'!$A$74:$D$83,4,FALSE))</f>
-        <v/>
-      </c>
-      <c r="K8" s="126" t="inlineStr">
+        <f>IF(E8="","",VLOOKUP(E8,'Master Data'!$A$74:$D$77,4,FALSE))</f>
+        <v/>
+      </c>
+      <c r="J8" s="126" t="inlineStr">
         <is>
           <t>Seat:</t>
         </is>
       </c>
-      <c r="L8" s="82" t="inlineStr">
+      <c r="K8" s="82" t="inlineStr">
         <is>
           <t>Economy</t>
         </is>
@@ -3493,7 +3519,7 @@
     <row r="9">
       <c r="A9" s="106" t="inlineStr">
         <is>
-          <t>Trip Duration:</t>
+          <t>Duration:</t>
         </is>
       </c>
       <c r="B9" s="122">
@@ -3506,7 +3532,7 @@
         </is>
       </c>
       <c r="D9" s="122">
-        <f>IF(C9&lt;&gt;"",C9+1,"")</f>
+        <f>IF(B9&lt;&gt;"",B9+1,"")</f>
         <v/>
       </c>
       <c r="E9" s="108" t="inlineStr">
@@ -3515,35 +3541,54 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="134" t="inlineStr">
+        <is>
+          <t>⚠️ DUPLICATE CHECK</t>
+        </is>
+      </c>
+      <c r="B11" s="136">
+        <f>IF(SUM(Q:Q)&gt;0,"❌ "&amp;SUM(Q:Q)&amp;" duplicate(s) — check hidden Q column","✅ No duplicates")</f>
+        <v/>
+      </c>
+    </row>
     <row r="12">
-      <c r="A12" s="103" t="inlineStr">
-        <is>
-          <t>📊 ITEM SELECTOR — 드롭다운 선택 → 참가자 ✓ 체크 → 자동계산</t>
-        </is>
-      </c>
-      <c r="B12" s="104" t="n"/>
-      <c r="C12" s="104" t="n"/>
-      <c r="D12" s="104" t="n"/>
-      <c r="E12" s="104" t="n"/>
-      <c r="F12" s="104" t="n"/>
-      <c r="G12" s="104" t="n"/>
-      <c r="H12" s="104" t="n"/>
-      <c r="I12" s="104" t="n"/>
-      <c r="J12" s="104" t="n"/>
-      <c r="K12" s="104" t="n"/>
-      <c r="L12" s="104" t="n"/>
-      <c r="M12" s="104" t="n"/>
-      <c r="N12" s="104" t="n"/>
+      <c r="A12" s="116" t="inlineStr">
+        <is>
+          <t>Cross-Check:</t>
+        </is>
+      </c>
+      <c r="B12" s="133">
+        <f>K68</f>
+        <v/>
+      </c>
+      <c r="C12" s="81" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="D12" s="133">
+        <f>B76</f>
+        <v/>
+      </c>
+      <c r="E12" s="117">
+        <f>B12-D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="118">
+        <f>IF(E12=0,"✅ MATCH","❌ MISMATCH")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="119" t="inlineStr">
         <is>
-          <t>Category / Item</t>
+          <t>Item (Select ▼)</t>
         </is>
       </c>
       <c r="B13" s="98" t="inlineStr">
         <is>
-          <t>Qty/p</t>
+          <t>Qty</t>
         </is>
       </c>
       <c r="C13" s="98" t="inlineStr">
@@ -3558,52 +3603,67 @@
       </c>
       <c r="E13" s="98" t="inlineStr">
         <is>
+          <t>Margin%</t>
+        </is>
+      </c>
+      <c r="F13" s="98" t="inlineStr">
+        <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="F13" s="98" t="inlineStr">
+      <c r="G13" s="98" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="G13" s="98" t="inlineStr">
+      <c r="H13" s="98" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="H13" s="98" t="inlineStr">
+      <c r="I13" s="98" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="I13" s="98" t="inlineStr">
+      <c r="J13" s="141" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K13" s="98" t="inlineStr">
+        <is>
+          <t>Tot Cost</t>
+        </is>
+      </c>
+      <c r="L13" s="98" t="inlineStr">
+        <is>
+          <t>Tot Sell</t>
+        </is>
+      </c>
+      <c r="M13" s="98" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="J13" s="98" t="inlineStr">
+      <c r="N13" s="98" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
-      <c r="K13" s="98" t="inlineStr">
+      <c r="O13" s="98" t="inlineStr">
         <is>
           <t>P7</t>
         </is>
       </c>
-      <c r="L13" s="98" t="inlineStr">
+      <c r="P13" s="98" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
       </c>
-      <c r="M13" s="98" t="inlineStr">
-        <is>
-          <t>Total Cost</t>
-        </is>
-      </c>
-      <c r="N13" s="98" t="inlineStr">
-        <is>
-          <t>Total Sell</t>
+      <c r="Q13" s="98" t="inlineStr">
+        <is>
+          <t>Dup</t>
         </is>
       </c>
     </row>
@@ -3624,17 +3684,15 @@
       <c r="J14" s="77" t="n"/>
       <c r="K14" s="77" t="n"/>
       <c r="L14" s="77" t="n"/>
-      <c r="M14" s="77" t="n"/>
-      <c r="N14" s="77" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="109" t="inlineStr">
         <is>
-          <t>Trump National LA</t>
+          <t>Hidden Valley GC</t>
         </is>
       </c>
       <c r="B15" s="83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C15" s="84">
         <f>IF(A15="","",VLOOKUP(A15,'Master Data'!$A$7:$C$14,2,FALSE))</f>
@@ -3644,23 +3702,32 @@
         <f>IF(A15="","",VLOOKUP(A15,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E15" s="81" t="inlineStr"/>
+      <c r="E15" s="137">
+        <f>IF(D15&gt;0,(D15-C15)/D15,0)</f>
+        <v/>
+      </c>
       <c r="F15" s="81" t="inlineStr"/>
       <c r="G15" s="81" t="inlineStr"/>
       <c r="H15" s="81" t="inlineStr"/>
       <c r="I15" s="81" t="inlineStr"/>
-      <c r="J15" s="81" t="inlineStr"/>
-      <c r="K15" s="81" t="inlineStr"/>
-      <c r="L15" s="81" t="inlineStr"/>
-      <c r="M15" s="84">
-        <f>IF(A15="","",COUNTIF(E15:L15,"✓")*B15*C15)</f>
-        <v/>
-      </c>
-      <c r="N15" s="84">
-        <f>IF(A15="","",COUNTIF(E15:L15,"✓")*B15*D15)</f>
-        <v/>
-      </c>
-      <c r="O15" s="81">
+      <c r="J15" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K15" s="84">
+        <f>IF(A15="","",(COUNTIF(F15,"✓")+COUNTIF(G15,"✓")+COUNTIF(H15,"✓")+COUNTIF(I15,"✓")+COUNTIF(M15,"✓")+COUNTIF(N15,"✓")+COUNTIF(O15,"✓")+COUNTIF(P15,"✓"))*B15*C15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="84">
+        <f>IF(A15="","",(COUNTIF(F15,"✓")+COUNTIF(G15,"✓")+COUNTIF(H15,"✓")+COUNTIF(I15,"✓")+COUNTIF(M15,"✓")+COUNTIF(N15,"✓")+COUNTIF(O15,"✓")+COUNTIF(P15,"✓"))*B15*D15)</f>
+        <v/>
+      </c>
+      <c r="M15" s="81" t="inlineStr"/>
+      <c r="N15" s="81" t="inlineStr"/>
+      <c r="O15" s="81" t="inlineStr"/>
+      <c r="P15" s="81" t="inlineStr"/>
+      <c r="Q15" s="81">
         <f>0</f>
         <v/>
       </c>
@@ -3682,23 +3749,32 @@
         <f>IF(A16="","",VLOOKUP(A16,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E16" s="81" t="inlineStr"/>
+      <c r="E16" s="137">
+        <f>IF(D16&gt;0,(D16-C16)/D16,0)</f>
+        <v/>
+      </c>
       <c r="F16" s="81" t="inlineStr"/>
       <c r="G16" s="81" t="inlineStr"/>
       <c r="H16" s="81" t="inlineStr"/>
       <c r="I16" s="81" t="inlineStr"/>
-      <c r="J16" s="81" t="inlineStr"/>
-      <c r="K16" s="81" t="inlineStr"/>
-      <c r="L16" s="81" t="inlineStr"/>
-      <c r="M16" s="84">
-        <f>IF(A16="","",COUNTIF(E16:L16,"✓")*B16*C16)</f>
-        <v/>
-      </c>
-      <c r="N16" s="84">
-        <f>IF(A16="","",COUNTIF(E16:L16,"✓")*B16*D16)</f>
-        <v/>
-      </c>
-      <c r="O16" s="81">
+      <c r="J16" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K16" s="84">
+        <f>IF(A16="","",(COUNTIF(F16,"✓")+COUNTIF(G16,"✓")+COUNTIF(H16,"✓")+COUNTIF(I16,"✓")+COUNTIF(M16,"✓")+COUNTIF(N16,"✓")+COUNTIF(O16,"✓")+COUNTIF(P16,"✓"))*B16*C16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="84">
+        <f>IF(A16="","",(COUNTIF(F16,"✓")+COUNTIF(G16,"✓")+COUNTIF(H16,"✓")+COUNTIF(I16,"✓")+COUNTIF(M16,"✓")+COUNTIF(N16,"✓")+COUNTIF(O16,"✓")+COUNTIF(P16,"✓"))*B16*D16)</f>
+        <v/>
+      </c>
+      <c r="M16" s="81" t="inlineStr"/>
+      <c r="N16" s="81" t="inlineStr"/>
+      <c r="O16" s="81" t="inlineStr"/>
+      <c r="P16" s="81" t="inlineStr"/>
+      <c r="Q16" s="81">
         <f>IF(A16="",0,COUNTIF(A$15:A15,A16))</f>
         <v/>
       </c>
@@ -3706,11 +3782,11 @@
     <row r="17">
       <c r="A17" s="109" t="inlineStr">
         <is>
-          <t>Hidden Valley GC</t>
+          <t>Trump National LA</t>
         </is>
       </c>
       <c r="B17" s="83" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C17" s="84">
         <f>IF(A17="","",VLOOKUP(A17,'Master Data'!$A$7:$C$14,2,FALSE))</f>
@@ -3720,23 +3796,32 @@
         <f>IF(A17="","",VLOOKUP(A17,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E17" s="81" t="inlineStr"/>
+      <c r="E17" s="137">
+        <f>IF(D17&gt;0,(D17-C17)/D17,0)</f>
+        <v/>
+      </c>
       <c r="F17" s="81" t="inlineStr"/>
       <c r="G17" s="81" t="inlineStr"/>
       <c r="H17" s="81" t="inlineStr"/>
       <c r="I17" s="81" t="inlineStr"/>
-      <c r="J17" s="81" t="inlineStr"/>
-      <c r="K17" s="81" t="inlineStr"/>
-      <c r="L17" s="81" t="inlineStr"/>
-      <c r="M17" s="84">
-        <f>IF(A17="","",COUNTIF(E17:L17,"✓")*B17*C17)</f>
-        <v/>
-      </c>
-      <c r="N17" s="84">
-        <f>IF(A17="","",COUNTIF(E17:L17,"✓")*B17*D17)</f>
-        <v/>
-      </c>
-      <c r="O17" s="81">
+      <c r="J17" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K17" s="84">
+        <f>IF(A17="","",(COUNTIF(F17,"✓")+COUNTIF(G17,"✓")+COUNTIF(H17,"✓")+COUNTIF(I17,"✓")+COUNTIF(M17,"✓")+COUNTIF(N17,"✓")+COUNTIF(O17,"✓")+COUNTIF(P17,"✓"))*B17*C17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="84">
+        <f>IF(A17="","",(COUNTIF(F17,"✓")+COUNTIF(G17,"✓")+COUNTIF(H17,"✓")+COUNTIF(I17,"✓")+COUNTIF(M17,"✓")+COUNTIF(N17,"✓")+COUNTIF(O17,"✓")+COUNTIF(P17,"✓"))*B17*D17)</f>
+        <v/>
+      </c>
+      <c r="M17" s="81" t="inlineStr"/>
+      <c r="N17" s="81" t="inlineStr"/>
+      <c r="O17" s="81" t="inlineStr"/>
+      <c r="P17" s="81" t="inlineStr"/>
+      <c r="Q17" s="81">
         <f>IF(A17="",0,COUNTIF(A$15:A16,A17))</f>
         <v/>
       </c>
@@ -3752,23 +3837,32 @@
         <f>IF(A18="","",VLOOKUP(A18,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E18" s="81" t="inlineStr"/>
+      <c r="E18" s="137">
+        <f>IF(D18&gt;0,(D18-C18)/D18,0)</f>
+        <v/>
+      </c>
       <c r="F18" s="81" t="inlineStr"/>
       <c r="G18" s="81" t="inlineStr"/>
       <c r="H18" s="81" t="inlineStr"/>
       <c r="I18" s="81" t="inlineStr"/>
-      <c r="J18" s="81" t="inlineStr"/>
-      <c r="K18" s="81" t="inlineStr"/>
-      <c r="L18" s="81" t="inlineStr"/>
-      <c r="M18" s="84">
-        <f>IF(A18="","",COUNTIF(E18:L18,"✓")*B18*C18)</f>
-        <v/>
-      </c>
-      <c r="N18" s="84">
-        <f>IF(A18="","",COUNTIF(E18:L18,"✓")*B18*D18)</f>
-        <v/>
-      </c>
-      <c r="O18" s="81">
+      <c r="J18" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K18" s="84">
+        <f>IF(A18="","",(COUNTIF(F18,"✓")+COUNTIF(G18,"✓")+COUNTIF(H18,"✓")+COUNTIF(I18,"✓")+COUNTIF(M18,"✓")+COUNTIF(N18,"✓")+COUNTIF(O18,"✓")+COUNTIF(P18,"✓"))*B18*C18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="84">
+        <f>IF(A18="","",(COUNTIF(F18,"✓")+COUNTIF(G18,"✓")+COUNTIF(H18,"✓")+COUNTIF(I18,"✓")+COUNTIF(M18,"✓")+COUNTIF(N18,"✓")+COUNTIF(O18,"✓")+COUNTIF(P18,"✓"))*B18*D18)</f>
+        <v/>
+      </c>
+      <c r="M18" s="81" t="inlineStr"/>
+      <c r="N18" s="81" t="inlineStr"/>
+      <c r="O18" s="81" t="inlineStr"/>
+      <c r="P18" s="81" t="inlineStr"/>
+      <c r="Q18" s="81">
         <f>IF(A18="",0,COUNTIF(A$15:A17,A18))</f>
         <v/>
       </c>
@@ -3784,23 +3878,32 @@
         <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E19" s="81" t="inlineStr"/>
+      <c r="E19" s="137">
+        <f>IF(D19&gt;0,(D19-C19)/D19,0)</f>
+        <v/>
+      </c>
       <c r="F19" s="81" t="inlineStr"/>
       <c r="G19" s="81" t="inlineStr"/>
       <c r="H19" s="81" t="inlineStr"/>
       <c r="I19" s="81" t="inlineStr"/>
-      <c r="J19" s="81" t="inlineStr"/>
-      <c r="K19" s="81" t="inlineStr"/>
-      <c r="L19" s="81" t="inlineStr"/>
-      <c r="M19" s="84">
-        <f>IF(A19="","",COUNTIF(E19:L19,"✓")*B19*C19)</f>
-        <v/>
-      </c>
-      <c r="N19" s="84">
-        <f>IF(A19="","",COUNTIF(E19:L19,"✓")*B19*D19)</f>
-        <v/>
-      </c>
-      <c r="O19" s="81">
+      <c r="J19" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K19" s="84">
+        <f>IF(A19="","",(COUNTIF(F19,"✓")+COUNTIF(G19,"✓")+COUNTIF(H19,"✓")+COUNTIF(I19,"✓")+COUNTIF(M19,"✓")+COUNTIF(N19,"✓")+COUNTIF(O19,"✓")+COUNTIF(P19,"✓"))*B19*C19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="84">
+        <f>IF(A19="","",(COUNTIF(F19,"✓")+COUNTIF(G19,"✓")+COUNTIF(H19,"✓")+COUNTIF(I19,"✓")+COUNTIF(M19,"✓")+COUNTIF(N19,"✓")+COUNTIF(O19,"✓")+COUNTIF(P19,"✓"))*B19*D19)</f>
+        <v/>
+      </c>
+      <c r="M19" s="81" t="inlineStr"/>
+      <c r="N19" s="81" t="inlineStr"/>
+      <c r="O19" s="81" t="inlineStr"/>
+      <c r="P19" s="81" t="inlineStr"/>
+      <c r="Q19" s="81">
         <f>IF(A19="",0,COUNTIF(A$15:A18,A19))</f>
         <v/>
       </c>
@@ -3814,10 +3917,7 @@
       <c r="B20" s="114" t="inlineStr"/>
       <c r="C20" s="114" t="inlineStr"/>
       <c r="D20" s="114" t="inlineStr"/>
-      <c r="E20" s="130">
-        <f>SUMPRODUCT((E15:E19="✓")*1,B15:B19,C15:C19)</f>
-        <v/>
-      </c>
+      <c r="E20" s="114" t="inlineStr"/>
       <c r="F20" s="130">
         <f>SUMPRODUCT((F15:F19="✓")*1,B15:B19,C15:C19)</f>
         <v/>
@@ -3834,24 +3934,29 @@
         <f>SUMPRODUCT((I15:I19="✓")*1,B15:B19,C15:C19)</f>
         <v/>
       </c>
-      <c r="J20" s="130">
-        <f>SUMPRODUCT((J15:J19="✓")*1,B15:B19,C15:C19)</f>
-        <v/>
-      </c>
-      <c r="K20" s="130">
-        <f>SUMPRODUCT((K15:K19="✓")*1,B15:B19,C15:C19)</f>
-        <v/>
-      </c>
-      <c r="L20" s="130">
-        <f>SUMPRODUCT((L15:L19="✓")*1,B15:B19,C15:C19)</f>
-        <v/>
-      </c>
-      <c r="M20" s="88">
-        <f>SUM(M15:M19)</f>
-        <v/>
-      </c>
-      <c r="N20" s="88">
-        <f>SUM(N15:N19)</f>
+      <c r="J20" s="114" t="inlineStr"/>
+      <c r="K20" s="88">
+        <f>SUM(K15:K19)</f>
+        <v/>
+      </c>
+      <c r="L20" s="88">
+        <f>SUM(L15:L19)</f>
+        <v/>
+      </c>
+      <c r="M20" s="130">
+        <f>SUMPRODUCT((M15:M19="✓")*1,B15:B19,C15:C19)</f>
+        <v/>
+      </c>
+      <c r="N20" s="130">
+        <f>SUMPRODUCT((N15:N19="✓")*1,B15:B19,C15:C19)</f>
+        <v/>
+      </c>
+      <c r="O20" s="130">
+        <f>SUMPRODUCT((O15:O19="✓")*1,B15:B19,C15:C19)</f>
+        <v/>
+      </c>
+      <c r="P20" s="130">
+        <f>SUMPRODUCT((P15:P19="✓")*1,B15:B19,C15:C19)</f>
         <v/>
       </c>
     </row>
@@ -3872,8 +3977,6 @@
       <c r="J22" s="77" t="n"/>
       <c r="K22" s="77" t="n"/>
       <c r="L22" s="77" t="n"/>
-      <c r="M22" s="77" t="n"/>
-      <c r="N22" s="77" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="109" t="inlineStr">
@@ -3892,23 +3995,32 @@
         <f>IF(A23="","",VLOOKUP(A23,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E23" s="81" t="inlineStr"/>
+      <c r="E23" s="137">
+        <f>IF(D23&gt;0,(D23-C23)/D23,0)</f>
+        <v/>
+      </c>
       <c r="F23" s="81" t="inlineStr"/>
       <c r="G23" s="81" t="inlineStr"/>
       <c r="H23" s="81" t="inlineStr"/>
       <c r="I23" s="81" t="inlineStr"/>
-      <c r="J23" s="81" t="inlineStr"/>
-      <c r="K23" s="81" t="inlineStr"/>
-      <c r="L23" s="81" t="inlineStr"/>
-      <c r="M23" s="84">
-        <f>IF(A23="","",COUNTIF(E23:L23,"✓")*B23*C23)</f>
-        <v/>
-      </c>
-      <c r="N23" s="84">
-        <f>IF(A23="","",COUNTIF(E23:L23,"✓")*B23*D23)</f>
-        <v/>
-      </c>
-      <c r="O23" s="81">
+      <c r="J23" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K23" s="84">
+        <f>IF(A23="","",(COUNTIF(F23,"✓")+COUNTIF(G23,"✓")+COUNTIF(H23,"✓")+COUNTIF(I23,"✓")+COUNTIF(M23,"✓")+COUNTIF(N23,"✓")+COUNTIF(O23,"✓")+COUNTIF(P23,"✓"))*B23*C23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="84">
+        <f>IF(A23="","",(COUNTIF(F23,"✓")+COUNTIF(G23,"✓")+COUNTIF(H23,"✓")+COUNTIF(I23,"✓")+COUNTIF(M23,"✓")+COUNTIF(N23,"✓")+COUNTIF(O23,"✓")+COUNTIF(P23,"✓"))*B23*D23)</f>
+        <v/>
+      </c>
+      <c r="M23" s="81" t="inlineStr"/>
+      <c r="N23" s="81" t="inlineStr"/>
+      <c r="O23" s="81" t="inlineStr"/>
+      <c r="P23" s="81" t="inlineStr"/>
+      <c r="Q23" s="81">
         <f>0</f>
         <v/>
       </c>
@@ -3924,23 +4036,32 @@
         <f>IF(A24="","",VLOOKUP(A24,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E24" s="81" t="inlineStr"/>
+      <c r="E24" s="137">
+        <f>IF(D24&gt;0,(D24-C24)/D24,0)</f>
+        <v/>
+      </c>
       <c r="F24" s="81" t="inlineStr"/>
       <c r="G24" s="81" t="inlineStr"/>
       <c r="H24" s="81" t="inlineStr"/>
       <c r="I24" s="81" t="inlineStr"/>
-      <c r="J24" s="81" t="inlineStr"/>
-      <c r="K24" s="81" t="inlineStr"/>
-      <c r="L24" s="81" t="inlineStr"/>
-      <c r="M24" s="84">
-        <f>IF(A24="","",COUNTIF(E24:L24,"✓")*B24*C24)</f>
-        <v/>
-      </c>
-      <c r="N24" s="84">
-        <f>IF(A24="","",COUNTIF(E24:L24,"✓")*B24*D24)</f>
-        <v/>
-      </c>
-      <c r="O24" s="81">
+      <c r="J24" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K24" s="84">
+        <f>IF(A24="","",(COUNTIF(F24,"✓")+COUNTIF(G24,"✓")+COUNTIF(H24,"✓")+COUNTIF(I24,"✓")+COUNTIF(M24,"✓")+COUNTIF(N24,"✓")+COUNTIF(O24,"✓")+COUNTIF(P24,"✓"))*B24*C24)</f>
+        <v/>
+      </c>
+      <c r="L24" s="84">
+        <f>IF(A24="","",(COUNTIF(F24,"✓")+COUNTIF(G24,"✓")+COUNTIF(H24,"✓")+COUNTIF(I24,"✓")+COUNTIF(M24,"✓")+COUNTIF(N24,"✓")+COUNTIF(O24,"✓")+COUNTIF(P24,"✓"))*B24*D24)</f>
+        <v/>
+      </c>
+      <c r="M24" s="81" t="inlineStr"/>
+      <c r="N24" s="81" t="inlineStr"/>
+      <c r="O24" s="81" t="inlineStr"/>
+      <c r="P24" s="81" t="inlineStr"/>
+      <c r="Q24" s="81">
         <f>IF(A24="",0,COUNTIF(A$23:A23,A24))</f>
         <v/>
       </c>
@@ -3956,23 +4077,32 @@
         <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E25" s="81" t="inlineStr"/>
+      <c r="E25" s="137">
+        <f>IF(D25&gt;0,(D25-C25)/D25,0)</f>
+        <v/>
+      </c>
       <c r="F25" s="81" t="inlineStr"/>
       <c r="G25" s="81" t="inlineStr"/>
       <c r="H25" s="81" t="inlineStr"/>
       <c r="I25" s="81" t="inlineStr"/>
-      <c r="J25" s="81" t="inlineStr"/>
-      <c r="K25" s="81" t="inlineStr"/>
-      <c r="L25" s="81" t="inlineStr"/>
-      <c r="M25" s="84">
-        <f>IF(A25="","",COUNTIF(E25:L25,"✓")*B25*C25)</f>
-        <v/>
-      </c>
-      <c r="N25" s="84">
-        <f>IF(A25="","",COUNTIF(E25:L25,"✓")*B25*D25)</f>
-        <v/>
-      </c>
-      <c r="O25" s="81">
+      <c r="J25" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K25" s="84">
+        <f>IF(A25="","",(COUNTIF(F25,"✓")+COUNTIF(G25,"✓")+COUNTIF(H25,"✓")+COUNTIF(I25,"✓")+COUNTIF(M25,"✓")+COUNTIF(N25,"✓")+COUNTIF(O25,"✓")+COUNTIF(P25,"✓"))*B25*C25)</f>
+        <v/>
+      </c>
+      <c r="L25" s="84">
+        <f>IF(A25="","",(COUNTIF(F25,"✓")+COUNTIF(G25,"✓")+COUNTIF(H25,"✓")+COUNTIF(I25,"✓")+COUNTIF(M25,"✓")+COUNTIF(N25,"✓")+COUNTIF(O25,"✓")+COUNTIF(P25,"✓"))*B25*D25)</f>
+        <v/>
+      </c>
+      <c r="M25" s="81" t="inlineStr"/>
+      <c r="N25" s="81" t="inlineStr"/>
+      <c r="O25" s="81" t="inlineStr"/>
+      <c r="P25" s="81" t="inlineStr"/>
+      <c r="Q25" s="81">
         <f>IF(A25="",0,COUNTIF(A$23:A24,A25))</f>
         <v/>
       </c>
@@ -3986,10 +4116,7 @@
       <c r="B26" s="114" t="inlineStr"/>
       <c r="C26" s="114" t="inlineStr"/>
       <c r="D26" s="114" t="inlineStr"/>
-      <c r="E26" s="130">
-        <f>SUMPRODUCT((E23:E25="✓")*1,B23:B25,C23:C25)</f>
-        <v/>
-      </c>
+      <c r="E26" s="114" t="inlineStr"/>
       <c r="F26" s="130">
         <f>SUMPRODUCT((F23:F25="✓")*1,B23:B25,C23:C25)</f>
         <v/>
@@ -4006,24 +4133,29 @@
         <f>SUMPRODUCT((I23:I25="✓")*1,B23:B25,C23:C25)</f>
         <v/>
       </c>
-      <c r="J26" s="130">
-        <f>SUMPRODUCT((J23:J25="✓")*1,B23:B25,C23:C25)</f>
-        <v/>
-      </c>
-      <c r="K26" s="130">
-        <f>SUMPRODUCT((K23:K25="✓")*1,B23:B25,C23:C25)</f>
-        <v/>
-      </c>
-      <c r="L26" s="130">
-        <f>SUMPRODUCT((L23:L25="✓")*1,B23:B25,C23:C25)</f>
-        <v/>
-      </c>
-      <c r="M26" s="88">
-        <f>SUM(M23:M25)</f>
-        <v/>
-      </c>
-      <c r="N26" s="88">
-        <f>SUM(N23:N25)</f>
+      <c r="J26" s="114" t="inlineStr"/>
+      <c r="K26" s="88">
+        <f>SUM(K23:K25)</f>
+        <v/>
+      </c>
+      <c r="L26" s="88">
+        <f>SUM(L23:L25)</f>
+        <v/>
+      </c>
+      <c r="M26" s="130">
+        <f>SUMPRODUCT((M23:M25="✓")*1,B23:B25,C23:C25)</f>
+        <v/>
+      </c>
+      <c r="N26" s="130">
+        <f>SUMPRODUCT((N23:N25="✓")*1,B23:B25,C23:C25)</f>
+        <v/>
+      </c>
+      <c r="O26" s="130">
+        <f>SUMPRODUCT((O23:O25="✓")*1,B23:B25,C23:C25)</f>
+        <v/>
+      </c>
+      <c r="P26" s="130">
+        <f>SUMPRODUCT((P23:P25="✓")*1,B23:B25,C23:C25)</f>
         <v/>
       </c>
     </row>
@@ -4044,8 +4176,6 @@
       <c r="J28" s="77" t="n"/>
       <c r="K28" s="77" t="n"/>
       <c r="L28" s="77" t="n"/>
-      <c r="M28" s="77" t="n"/>
-      <c r="N28" s="77" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="109" t="inlineStr">
@@ -4064,23 +4194,32 @@
         <f>IF(A29="","",VLOOKUP(A29,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E29" s="81" t="inlineStr"/>
+      <c r="E29" s="137">
+        <f>IF(D29&gt;0,(D29-C29)/D29,0)</f>
+        <v/>
+      </c>
       <c r="F29" s="81" t="inlineStr"/>
       <c r="G29" s="81" t="inlineStr"/>
       <c r="H29" s="81" t="inlineStr"/>
       <c r="I29" s="81" t="inlineStr"/>
-      <c r="J29" s="81" t="inlineStr"/>
-      <c r="K29" s="81" t="inlineStr"/>
-      <c r="L29" s="81" t="inlineStr"/>
-      <c r="M29" s="84">
-        <f>IF(A29="","",COUNTIF(E29:L29,"✓")*B29*C29)</f>
-        <v/>
-      </c>
-      <c r="N29" s="84">
-        <f>IF(A29="","",COUNTIF(E29:L29,"✓")*B29*D29)</f>
-        <v/>
-      </c>
-      <c r="O29" s="81">
+      <c r="J29" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K29" s="84">
+        <f>IF(A29="","",(COUNTIF(F29,"✓")+COUNTIF(G29,"✓")+COUNTIF(H29,"✓")+COUNTIF(I29,"✓")+COUNTIF(M29,"✓")+COUNTIF(N29,"✓")+COUNTIF(O29,"✓")+COUNTIF(P29,"✓"))*B29*C29)</f>
+        <v/>
+      </c>
+      <c r="L29" s="84">
+        <f>IF(A29="","",(COUNTIF(F29,"✓")+COUNTIF(G29,"✓")+COUNTIF(H29,"✓")+COUNTIF(I29,"✓")+COUNTIF(M29,"✓")+COUNTIF(N29,"✓")+COUNTIF(O29,"✓")+COUNTIF(P29,"✓"))*B29*D29)</f>
+        <v/>
+      </c>
+      <c r="M29" s="81" t="inlineStr"/>
+      <c r="N29" s="81" t="inlineStr"/>
+      <c r="O29" s="81" t="inlineStr"/>
+      <c r="P29" s="81" t="inlineStr"/>
+      <c r="Q29" s="81">
         <f>0</f>
         <v/>
       </c>
@@ -4096,23 +4235,32 @@
         <f>IF(A30="","",VLOOKUP(A30,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E30" s="81" t="inlineStr"/>
+      <c r="E30" s="137">
+        <f>IF(D30&gt;0,(D30-C30)/D30,0)</f>
+        <v/>
+      </c>
       <c r="F30" s="81" t="inlineStr"/>
       <c r="G30" s="81" t="inlineStr"/>
       <c r="H30" s="81" t="inlineStr"/>
       <c r="I30" s="81" t="inlineStr"/>
-      <c r="J30" s="81" t="inlineStr"/>
-      <c r="K30" s="81" t="inlineStr"/>
-      <c r="L30" s="81" t="inlineStr"/>
-      <c r="M30" s="84">
-        <f>IF(A30="","",COUNTIF(E30:L30,"✓")*B30*C30)</f>
-        <v/>
-      </c>
-      <c r="N30" s="84">
-        <f>IF(A30="","",COUNTIF(E30:L30,"✓")*B30*D30)</f>
-        <v/>
-      </c>
-      <c r="O30" s="81">
+      <c r="J30" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K30" s="84">
+        <f>IF(A30="","",(COUNTIF(F30,"✓")+COUNTIF(G30,"✓")+COUNTIF(H30,"✓")+COUNTIF(I30,"✓")+COUNTIF(M30,"✓")+COUNTIF(N30,"✓")+COUNTIF(O30,"✓")+COUNTIF(P30,"✓"))*B30*C30)</f>
+        <v/>
+      </c>
+      <c r="L30" s="84">
+        <f>IF(A30="","",(COUNTIF(F30,"✓")+COUNTIF(G30,"✓")+COUNTIF(H30,"✓")+COUNTIF(I30,"✓")+COUNTIF(M30,"✓")+COUNTIF(N30,"✓")+COUNTIF(O30,"✓")+COUNTIF(P30,"✓"))*B30*D30)</f>
+        <v/>
+      </c>
+      <c r="M30" s="81" t="inlineStr"/>
+      <c r="N30" s="81" t="inlineStr"/>
+      <c r="O30" s="81" t="inlineStr"/>
+      <c r="P30" s="81" t="inlineStr"/>
+      <c r="Q30" s="81">
         <f>IF(A30="",0,COUNTIF(A$29:A29,A30))</f>
         <v/>
       </c>
@@ -4128,23 +4276,32 @@
         <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E31" s="81" t="inlineStr"/>
+      <c r="E31" s="137">
+        <f>IF(D31&gt;0,(D31-C31)/D31,0)</f>
+        <v/>
+      </c>
       <c r="F31" s="81" t="inlineStr"/>
       <c r="G31" s="81" t="inlineStr"/>
       <c r="H31" s="81" t="inlineStr"/>
       <c r="I31" s="81" t="inlineStr"/>
-      <c r="J31" s="81" t="inlineStr"/>
-      <c r="K31" s="81" t="inlineStr"/>
-      <c r="L31" s="81" t="inlineStr"/>
-      <c r="M31" s="84">
-        <f>IF(A31="","",COUNTIF(E31:L31,"✓")*B31*C31)</f>
-        <v/>
-      </c>
-      <c r="N31" s="84">
-        <f>IF(A31="","",COUNTIF(E31:L31,"✓")*B31*D31)</f>
-        <v/>
-      </c>
-      <c r="O31" s="81">
+      <c r="J31" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K31" s="84">
+        <f>IF(A31="","",(COUNTIF(F31,"✓")+COUNTIF(G31,"✓")+COUNTIF(H31,"✓")+COUNTIF(I31,"✓")+COUNTIF(M31,"✓")+COUNTIF(N31,"✓")+COUNTIF(O31,"✓")+COUNTIF(P31,"✓"))*B31*C31)</f>
+        <v/>
+      </c>
+      <c r="L31" s="84">
+        <f>IF(A31="","",(COUNTIF(F31,"✓")+COUNTIF(G31,"✓")+COUNTIF(H31,"✓")+COUNTIF(I31,"✓")+COUNTIF(M31,"✓")+COUNTIF(N31,"✓")+COUNTIF(O31,"✓")+COUNTIF(P31,"✓"))*B31*D31)</f>
+        <v/>
+      </c>
+      <c r="M31" s="81" t="inlineStr"/>
+      <c r="N31" s="81" t="inlineStr"/>
+      <c r="O31" s="81" t="inlineStr"/>
+      <c r="P31" s="81" t="inlineStr"/>
+      <c r="Q31" s="81">
         <f>IF(A31="",0,COUNTIF(A$29:A30,A31))</f>
         <v/>
       </c>
@@ -4158,10 +4315,7 @@
       <c r="B32" s="114" t="inlineStr"/>
       <c r="C32" s="114" t="inlineStr"/>
       <c r="D32" s="114" t="inlineStr"/>
-      <c r="E32" s="130">
-        <f>SUMPRODUCT((E29:E31="✓")*1,B29:B31,C29:C31)</f>
-        <v/>
-      </c>
+      <c r="E32" s="114" t="inlineStr"/>
       <c r="F32" s="130">
         <f>SUMPRODUCT((F29:F31="✓")*1,B29:B31,C29:C31)</f>
         <v/>
@@ -4178,24 +4332,29 @@
         <f>SUMPRODUCT((I29:I31="✓")*1,B29:B31,C29:C31)</f>
         <v/>
       </c>
-      <c r="J32" s="130">
-        <f>SUMPRODUCT((J29:J31="✓")*1,B29:B31,C29:C31)</f>
-        <v/>
-      </c>
-      <c r="K32" s="130">
-        <f>SUMPRODUCT((K29:K31="✓")*1,B29:B31,C29:C31)</f>
-        <v/>
-      </c>
-      <c r="L32" s="130">
-        <f>SUMPRODUCT((L29:L31="✓")*1,B29:B31,C29:C31)</f>
-        <v/>
-      </c>
-      <c r="M32" s="88">
-        <f>SUM(M29:M31)</f>
-        <v/>
-      </c>
-      <c r="N32" s="88">
-        <f>SUM(N29:N31)</f>
+      <c r="J32" s="114" t="inlineStr"/>
+      <c r="K32" s="88">
+        <f>SUM(K29:K31)</f>
+        <v/>
+      </c>
+      <c r="L32" s="88">
+        <f>SUM(L29:L31)</f>
+        <v/>
+      </c>
+      <c r="M32" s="130">
+        <f>SUMPRODUCT((M29:M31="✓")*1,B29:B31,C29:C31)</f>
+        <v/>
+      </c>
+      <c r="N32" s="130">
+        <f>SUMPRODUCT((N29:N31="✓")*1,B29:B31,C29:C31)</f>
+        <v/>
+      </c>
+      <c r="O32" s="130">
+        <f>SUMPRODUCT((O29:O31="✓")*1,B29:B31,C29:C31)</f>
+        <v/>
+      </c>
+      <c r="P32" s="130">
+        <f>SUMPRODUCT((P29:P31="✓")*1,B29:B31,C29:C31)</f>
         <v/>
       </c>
     </row>
@@ -4216,8 +4375,6 @@
       <c r="J34" s="77" t="n"/>
       <c r="K34" s="77" t="n"/>
       <c r="L34" s="77" t="n"/>
-      <c r="M34" s="77" t="n"/>
-      <c r="N34" s="77" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="109" t="inlineStr">
@@ -4236,23 +4393,32 @@
         <f>IF(A35="","",VLOOKUP(A35,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E35" s="81" t="inlineStr"/>
+      <c r="E35" s="137">
+        <f>IF(D35&gt;0,(D35-C35)/D35,0)</f>
+        <v/>
+      </c>
       <c r="F35" s="81" t="inlineStr"/>
       <c r="G35" s="81" t="inlineStr"/>
       <c r="H35" s="81" t="inlineStr"/>
       <c r="I35" s="81" t="inlineStr"/>
-      <c r="J35" s="81" t="inlineStr"/>
-      <c r="K35" s="81" t="inlineStr"/>
-      <c r="L35" s="81" t="inlineStr"/>
-      <c r="M35" s="84">
-        <f>IF(A35="","",COUNTIF(E35:L35,"✓")*B35*C35)</f>
-        <v/>
-      </c>
-      <c r="N35" s="84">
-        <f>IF(A35="","",COUNTIF(E35:L35,"✓")*B35*D35)</f>
-        <v/>
-      </c>
-      <c r="O35" s="81">
+      <c r="J35" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K35" s="84">
+        <f>IF(A35="","",(COUNTIF(F35,"✓")+COUNTIF(G35,"✓")+COUNTIF(H35,"✓")+COUNTIF(I35,"✓")+COUNTIF(M35,"✓")+COUNTIF(N35,"✓")+COUNTIF(O35,"✓")+COUNTIF(P35,"✓"))*B35*C35)</f>
+        <v/>
+      </c>
+      <c r="L35" s="84">
+        <f>IF(A35="","",(COUNTIF(F35,"✓")+COUNTIF(G35,"✓")+COUNTIF(H35,"✓")+COUNTIF(I35,"✓")+COUNTIF(M35,"✓")+COUNTIF(N35,"✓")+COUNTIF(O35,"✓")+COUNTIF(P35,"✓"))*B35*D35)</f>
+        <v/>
+      </c>
+      <c r="M35" s="81" t="inlineStr"/>
+      <c r="N35" s="81" t="inlineStr"/>
+      <c r="O35" s="81" t="inlineStr"/>
+      <c r="P35" s="81" t="inlineStr"/>
+      <c r="Q35" s="81">
         <f>0</f>
         <v/>
       </c>
@@ -4260,7 +4426,7 @@
     <row r="36">
       <c r="A36" s="108" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Dinner (Regular)</t>
         </is>
       </c>
       <c r="B36" s="83" t="n">
@@ -4274,23 +4440,32 @@
         <f>IF(A36="","",VLOOKUP(A36,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E36" s="81" t="inlineStr"/>
+      <c r="E36" s="137">
+        <f>IF(D36&gt;0,(D36-C36)/D36,0)</f>
+        <v/>
+      </c>
       <c r="F36" s="81" t="inlineStr"/>
       <c r="G36" s="81" t="inlineStr"/>
       <c r="H36" s="81" t="inlineStr"/>
       <c r="I36" s="81" t="inlineStr"/>
-      <c r="J36" s="81" t="inlineStr"/>
-      <c r="K36" s="81" t="inlineStr"/>
-      <c r="L36" s="81" t="inlineStr"/>
-      <c r="M36" s="84">
-        <f>IF(A36="","",COUNTIF(E36:L36,"✓")*B36*C36)</f>
-        <v/>
-      </c>
-      <c r="N36" s="84">
-        <f>IF(A36="","",COUNTIF(E36:L36,"✓")*B36*D36)</f>
-        <v/>
-      </c>
-      <c r="O36" s="81">
+      <c r="J36" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K36" s="84">
+        <f>IF(A36="","",(COUNTIF(F36,"✓")+COUNTIF(G36,"✓")+COUNTIF(H36,"✓")+COUNTIF(I36,"✓")+COUNTIF(M36,"✓")+COUNTIF(N36,"✓")+COUNTIF(O36,"✓")+COUNTIF(P36,"✓"))*B36*C36)</f>
+        <v/>
+      </c>
+      <c r="L36" s="84">
+        <f>IF(A36="","",(COUNTIF(F36,"✓")+COUNTIF(G36,"✓")+COUNTIF(H36,"✓")+COUNTIF(I36,"✓")+COUNTIF(M36,"✓")+COUNTIF(N36,"✓")+COUNTIF(O36,"✓")+COUNTIF(P36,"✓"))*B36*D36)</f>
+        <v/>
+      </c>
+      <c r="M36" s="81" t="inlineStr"/>
+      <c r="N36" s="81" t="inlineStr"/>
+      <c r="O36" s="81" t="inlineStr"/>
+      <c r="P36" s="81" t="inlineStr"/>
+      <c r="Q36" s="81">
         <f>IF(A36="",0,COUNTIF(A$35:A35,A36))</f>
         <v/>
       </c>
@@ -4298,11 +4473,11 @@
     <row r="37">
       <c r="A37" s="109" t="inlineStr">
         <is>
-          <t>Dinner (Regular)</t>
+          <t>Exclusive Dinner (Michelin/Fine)</t>
         </is>
       </c>
       <c r="B37" s="83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C37" s="84">
         <f>IF(A37="","",VLOOKUP(A37,'Master Data'!$A$38:$C$46,2,FALSE))</f>
@@ -4312,23 +4487,32 @@
         <f>IF(A37="","",VLOOKUP(A37,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E37" s="81" t="inlineStr"/>
+      <c r="E37" s="137">
+        <f>IF(D37&gt;0,(D37-C37)/D37,0)</f>
+        <v/>
+      </c>
       <c r="F37" s="81" t="inlineStr"/>
       <c r="G37" s="81" t="inlineStr"/>
       <c r="H37" s="81" t="inlineStr"/>
       <c r="I37" s="81" t="inlineStr"/>
-      <c r="J37" s="81" t="inlineStr"/>
-      <c r="K37" s="81" t="inlineStr"/>
-      <c r="L37" s="81" t="inlineStr"/>
-      <c r="M37" s="84">
-        <f>IF(A37="","",COUNTIF(E37:L37,"✓")*B37*C37)</f>
-        <v/>
-      </c>
-      <c r="N37" s="84">
-        <f>IF(A37="","",COUNTIF(E37:L37,"✓")*B37*D37)</f>
-        <v/>
-      </c>
-      <c r="O37" s="81">
+      <c r="J37" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K37" s="84">
+        <f>IF(A37="","",(COUNTIF(F37,"✓")+COUNTIF(G37,"✓")+COUNTIF(H37,"✓")+COUNTIF(I37,"✓")+COUNTIF(M37,"✓")+COUNTIF(N37,"✓")+COUNTIF(O37,"✓")+COUNTIF(P37,"✓"))*B37*C37)</f>
+        <v/>
+      </c>
+      <c r="L37" s="84">
+        <f>IF(A37="","",(COUNTIF(F37,"✓")+COUNTIF(G37,"✓")+COUNTIF(H37,"✓")+COUNTIF(I37,"✓")+COUNTIF(M37,"✓")+COUNTIF(N37,"✓")+COUNTIF(O37,"✓")+COUNTIF(P37,"✓"))*B37*D37)</f>
+        <v/>
+      </c>
+      <c r="M37" s="81" t="inlineStr"/>
+      <c r="N37" s="81" t="inlineStr"/>
+      <c r="O37" s="81" t="inlineStr"/>
+      <c r="P37" s="81" t="inlineStr"/>
+      <c r="Q37" s="81">
         <f>IF(A37="",0,COUNTIF(A$35:A36,A37))</f>
         <v/>
       </c>
@@ -4336,11 +4520,11 @@
     <row r="38">
       <c r="A38" s="108" t="inlineStr">
         <is>
-          <t>Exclusive Dinner (Michelin/Fine)</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="B38" s="83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C38" s="84">
         <f>IF(A38="","",VLOOKUP(A38,'Master Data'!$A$38:$C$46,2,FALSE))</f>
@@ -4350,23 +4534,32 @@
         <f>IF(A38="","",VLOOKUP(A38,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E38" s="81" t="inlineStr"/>
+      <c r="E38" s="137">
+        <f>IF(D38&gt;0,(D38-C38)/D38,0)</f>
+        <v/>
+      </c>
       <c r="F38" s="81" t="inlineStr"/>
       <c r="G38" s="81" t="inlineStr"/>
       <c r="H38" s="81" t="inlineStr"/>
       <c r="I38" s="81" t="inlineStr"/>
-      <c r="J38" s="81" t="inlineStr"/>
-      <c r="K38" s="81" t="inlineStr"/>
-      <c r="L38" s="81" t="inlineStr"/>
-      <c r="M38" s="84">
-        <f>IF(A38="","",COUNTIF(E38:L38,"✓")*B38*C38)</f>
-        <v/>
-      </c>
-      <c r="N38" s="84">
-        <f>IF(A38="","",COUNTIF(E38:L38,"✓")*B38*D38)</f>
-        <v/>
-      </c>
-      <c r="O38" s="81">
+      <c r="J38" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K38" s="84">
+        <f>IF(A38="","",(COUNTIF(F38,"✓")+COUNTIF(G38,"✓")+COUNTIF(H38,"✓")+COUNTIF(I38,"✓")+COUNTIF(M38,"✓")+COUNTIF(N38,"✓")+COUNTIF(O38,"✓")+COUNTIF(P38,"✓"))*B38*C38)</f>
+        <v/>
+      </c>
+      <c r="L38" s="84">
+        <f>IF(A38="","",(COUNTIF(F38,"✓")+COUNTIF(G38,"✓")+COUNTIF(H38,"✓")+COUNTIF(I38,"✓")+COUNTIF(M38,"✓")+COUNTIF(N38,"✓")+COUNTIF(O38,"✓")+COUNTIF(P38,"✓"))*B38*D38)</f>
+        <v/>
+      </c>
+      <c r="M38" s="81" t="inlineStr"/>
+      <c r="N38" s="81" t="inlineStr"/>
+      <c r="O38" s="81" t="inlineStr"/>
+      <c r="P38" s="81" t="inlineStr"/>
+      <c r="Q38" s="81">
         <f>IF(A38="",0,COUNTIF(A$35:A37,A38))</f>
         <v/>
       </c>
@@ -4382,23 +4575,32 @@
         <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E39" s="81" t="inlineStr"/>
+      <c r="E39" s="137">
+        <f>IF(D39&gt;0,(D39-C39)/D39,0)</f>
+        <v/>
+      </c>
       <c r="F39" s="81" t="inlineStr"/>
       <c r="G39" s="81" t="inlineStr"/>
       <c r="H39" s="81" t="inlineStr"/>
       <c r="I39" s="81" t="inlineStr"/>
-      <c r="J39" s="81" t="inlineStr"/>
-      <c r="K39" s="81" t="inlineStr"/>
-      <c r="L39" s="81" t="inlineStr"/>
-      <c r="M39" s="84">
-        <f>IF(A39="","",COUNTIF(E39:L39,"✓")*B39*C39)</f>
-        <v/>
-      </c>
-      <c r="N39" s="84">
-        <f>IF(A39="","",COUNTIF(E39:L39,"✓")*B39*D39)</f>
-        <v/>
-      </c>
-      <c r="O39" s="81">
+      <c r="J39" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K39" s="84">
+        <f>IF(A39="","",(COUNTIF(F39,"✓")+COUNTIF(G39,"✓")+COUNTIF(H39,"✓")+COUNTIF(I39,"✓")+COUNTIF(M39,"✓")+COUNTIF(N39,"✓")+COUNTIF(O39,"✓")+COUNTIF(P39,"✓"))*B39*C39)</f>
+        <v/>
+      </c>
+      <c r="L39" s="84">
+        <f>IF(A39="","",(COUNTIF(F39,"✓")+COUNTIF(G39,"✓")+COUNTIF(H39,"✓")+COUNTIF(I39,"✓")+COUNTIF(M39,"✓")+COUNTIF(N39,"✓")+COUNTIF(O39,"✓")+COUNTIF(P39,"✓"))*B39*D39)</f>
+        <v/>
+      </c>
+      <c r="M39" s="81" t="inlineStr"/>
+      <c r="N39" s="81" t="inlineStr"/>
+      <c r="O39" s="81" t="inlineStr"/>
+      <c r="P39" s="81" t="inlineStr"/>
+      <c r="Q39" s="81">
         <f>IF(A39="",0,COUNTIF(A$35:A38,A39))</f>
         <v/>
       </c>
@@ -4412,10 +4614,7 @@
       <c r="B40" s="114" t="inlineStr"/>
       <c r="C40" s="114" t="inlineStr"/>
       <c r="D40" s="114" t="inlineStr"/>
-      <c r="E40" s="130">
-        <f>SUMPRODUCT((E35:E39="✓")*1,B35:B39,C35:C39)</f>
-        <v/>
-      </c>
+      <c r="E40" s="114" t="inlineStr"/>
       <c r="F40" s="130">
         <f>SUMPRODUCT((F35:F39="✓")*1,B35:B39,C35:C39)</f>
         <v/>
@@ -4432,24 +4631,29 @@
         <f>SUMPRODUCT((I35:I39="✓")*1,B35:B39,C35:C39)</f>
         <v/>
       </c>
-      <c r="J40" s="130">
-        <f>SUMPRODUCT((J35:J39="✓")*1,B35:B39,C35:C39)</f>
-        <v/>
-      </c>
-      <c r="K40" s="130">
-        <f>SUMPRODUCT((K35:K39="✓")*1,B35:B39,C35:C39)</f>
-        <v/>
-      </c>
-      <c r="L40" s="130">
-        <f>SUMPRODUCT((L35:L39="✓")*1,B35:B39,C35:C39)</f>
-        <v/>
-      </c>
-      <c r="M40" s="88">
-        <f>SUM(M35:M39)</f>
-        <v/>
-      </c>
-      <c r="N40" s="88">
-        <f>SUM(N35:N39)</f>
+      <c r="J40" s="114" t="inlineStr"/>
+      <c r="K40" s="88">
+        <f>SUM(K35:K39)</f>
+        <v/>
+      </c>
+      <c r="L40" s="88">
+        <f>SUM(L35:L39)</f>
+        <v/>
+      </c>
+      <c r="M40" s="130">
+        <f>SUMPRODUCT((M35:M39="✓")*1,B35:B39,C35:C39)</f>
+        <v/>
+      </c>
+      <c r="N40" s="130">
+        <f>SUMPRODUCT((N35:N39="✓")*1,B35:B39,C35:C39)</f>
+        <v/>
+      </c>
+      <c r="O40" s="130">
+        <f>SUMPRODUCT((O35:O39="✓")*1,B35:B39,C35:C39)</f>
+        <v/>
+      </c>
+      <c r="P40" s="130">
+        <f>SUMPRODUCT((P35:P39="✓")*1,B35:B39,C35:C39)</f>
         <v/>
       </c>
     </row>
@@ -4470,8 +4674,6 @@
       <c r="J42" s="77" t="n"/>
       <c r="K42" s="77" t="n"/>
       <c r="L42" s="77" t="n"/>
-      <c r="M42" s="77" t="n"/>
-      <c r="N42" s="77" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="109" t="inlineStr">
@@ -4490,23 +4692,32 @@
         <f>IF(A43="","",VLOOKUP(A43,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E43" s="81" t="inlineStr"/>
+      <c r="E43" s="137">
+        <f>IF(D43&gt;0,(D43-C43)/D43,0)</f>
+        <v/>
+      </c>
       <c r="F43" s="81" t="inlineStr"/>
       <c r="G43" s="81" t="inlineStr"/>
       <c r="H43" s="81" t="inlineStr"/>
       <c r="I43" s="81" t="inlineStr"/>
-      <c r="J43" s="81" t="inlineStr"/>
-      <c r="K43" s="81" t="inlineStr"/>
-      <c r="L43" s="81" t="inlineStr"/>
-      <c r="M43" s="84">
-        <f>IF(A43="","",COUNTIF(E43:L43,"✓")*B43*C43)</f>
-        <v/>
-      </c>
-      <c r="N43" s="84">
-        <f>IF(A43="","",COUNTIF(E43:L43,"✓")*B43*D43)</f>
-        <v/>
-      </c>
-      <c r="O43" s="81">
+      <c r="J43" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K43" s="84">
+        <f>IF(A43="","",(COUNTIF(F43,"✓")+COUNTIF(G43,"✓")+COUNTIF(H43,"✓")+COUNTIF(I43,"✓")+COUNTIF(M43,"✓")+COUNTIF(N43,"✓")+COUNTIF(O43,"✓")+COUNTIF(P43,"✓"))*B43*C43)</f>
+        <v/>
+      </c>
+      <c r="L43" s="84">
+        <f>IF(A43="","",(COUNTIF(F43,"✓")+COUNTIF(G43,"✓")+COUNTIF(H43,"✓")+COUNTIF(I43,"✓")+COUNTIF(M43,"✓")+COUNTIF(N43,"✓")+COUNTIF(O43,"✓")+COUNTIF(P43,"✓"))*B43*D43)</f>
+        <v/>
+      </c>
+      <c r="M43" s="81" t="inlineStr"/>
+      <c r="N43" s="81" t="inlineStr"/>
+      <c r="O43" s="81" t="inlineStr"/>
+      <c r="P43" s="81" t="inlineStr"/>
+      <c r="Q43" s="81">
         <f>0</f>
         <v/>
       </c>
@@ -4522,23 +4733,32 @@
         <f>IF(A44="","",VLOOKUP(A44,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E44" s="81" t="inlineStr"/>
+      <c r="E44" s="137">
+        <f>IF(D44&gt;0,(D44-C44)/D44,0)</f>
+        <v/>
+      </c>
       <c r="F44" s="81" t="inlineStr"/>
       <c r="G44" s="81" t="inlineStr"/>
       <c r="H44" s="81" t="inlineStr"/>
       <c r="I44" s="81" t="inlineStr"/>
-      <c r="J44" s="81" t="inlineStr"/>
-      <c r="K44" s="81" t="inlineStr"/>
-      <c r="L44" s="81" t="inlineStr"/>
-      <c r="M44" s="84">
-        <f>IF(A44="","",COUNTIF(E44:L44,"✓")*B44*C44)</f>
-        <v/>
-      </c>
-      <c r="N44" s="84">
-        <f>IF(A44="","",COUNTIF(E44:L44,"✓")*B44*D44)</f>
-        <v/>
-      </c>
-      <c r="O44" s="81">
+      <c r="J44" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K44" s="84">
+        <f>IF(A44="","",(COUNTIF(F44,"✓")+COUNTIF(G44,"✓")+COUNTIF(H44,"✓")+COUNTIF(I44,"✓")+COUNTIF(M44,"✓")+COUNTIF(N44,"✓")+COUNTIF(O44,"✓")+COUNTIF(P44,"✓"))*B44*C44)</f>
+        <v/>
+      </c>
+      <c r="L44" s="84">
+        <f>IF(A44="","",(COUNTIF(F44,"✓")+COUNTIF(G44,"✓")+COUNTIF(H44,"✓")+COUNTIF(I44,"✓")+COUNTIF(M44,"✓")+COUNTIF(N44,"✓")+COUNTIF(O44,"✓")+COUNTIF(P44,"✓"))*B44*D44)</f>
+        <v/>
+      </c>
+      <c r="M44" s="81" t="inlineStr"/>
+      <c r="N44" s="81" t="inlineStr"/>
+      <c r="O44" s="81" t="inlineStr"/>
+      <c r="P44" s="81" t="inlineStr"/>
+      <c r="Q44" s="81">
         <f>IF(A44="",0,COUNTIF(A$43:A43,A44))</f>
         <v/>
       </c>
@@ -4554,23 +4774,32 @@
         <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E45" s="81" t="inlineStr"/>
+      <c r="E45" s="137">
+        <f>IF(D45&gt;0,(D45-C45)/D45,0)</f>
+        <v/>
+      </c>
       <c r="F45" s="81" t="inlineStr"/>
       <c r="G45" s="81" t="inlineStr"/>
       <c r="H45" s="81" t="inlineStr"/>
       <c r="I45" s="81" t="inlineStr"/>
-      <c r="J45" s="81" t="inlineStr"/>
-      <c r="K45" s="81" t="inlineStr"/>
-      <c r="L45" s="81" t="inlineStr"/>
-      <c r="M45" s="84">
-        <f>IF(A45="","",COUNTIF(E45:L45,"✓")*B45*C45)</f>
-        <v/>
-      </c>
-      <c r="N45" s="84">
-        <f>IF(A45="","",COUNTIF(E45:L45,"✓")*B45*D45)</f>
-        <v/>
-      </c>
-      <c r="O45" s="81">
+      <c r="J45" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K45" s="84">
+        <f>IF(A45="","",(COUNTIF(F45,"✓")+COUNTIF(G45,"✓")+COUNTIF(H45,"✓")+COUNTIF(I45,"✓")+COUNTIF(M45,"✓")+COUNTIF(N45,"✓")+COUNTIF(O45,"✓")+COUNTIF(P45,"✓"))*B45*C45)</f>
+        <v/>
+      </c>
+      <c r="L45" s="84">
+        <f>IF(A45="","",(COUNTIF(F45,"✓")+COUNTIF(G45,"✓")+COUNTIF(H45,"✓")+COUNTIF(I45,"✓")+COUNTIF(M45,"✓")+COUNTIF(N45,"✓")+COUNTIF(O45,"✓")+COUNTIF(P45,"✓"))*B45*D45)</f>
+        <v/>
+      </c>
+      <c r="M45" s="81" t="inlineStr"/>
+      <c r="N45" s="81" t="inlineStr"/>
+      <c r="O45" s="81" t="inlineStr"/>
+      <c r="P45" s="81" t="inlineStr"/>
+      <c r="Q45" s="81">
         <f>IF(A45="",0,COUNTIF(A$43:A44,A45))</f>
         <v/>
       </c>
@@ -4584,10 +4813,7 @@
       <c r="B46" s="114" t="inlineStr"/>
       <c r="C46" s="114" t="inlineStr"/>
       <c r="D46" s="114" t="inlineStr"/>
-      <c r="E46" s="130">
-        <f>SUMPRODUCT((E43:E45="✓")*1,B43:B45,C43:C45)</f>
-        <v/>
-      </c>
+      <c r="E46" s="114" t="inlineStr"/>
       <c r="F46" s="130">
         <f>SUMPRODUCT((F43:F45="✓")*1,B43:B45,C43:C45)</f>
         <v/>
@@ -4604,24 +4830,29 @@
         <f>SUMPRODUCT((I43:I45="✓")*1,B43:B45,C43:C45)</f>
         <v/>
       </c>
-      <c r="J46" s="130">
-        <f>SUMPRODUCT((J43:J45="✓")*1,B43:B45,C43:C45)</f>
-        <v/>
-      </c>
-      <c r="K46" s="130">
-        <f>SUMPRODUCT((K43:K45="✓")*1,B43:B45,C43:C45)</f>
-        <v/>
-      </c>
-      <c r="L46" s="130">
-        <f>SUMPRODUCT((L43:L45="✓")*1,B43:B45,C43:C45)</f>
-        <v/>
-      </c>
-      <c r="M46" s="88">
-        <f>SUM(M43:M45)</f>
-        <v/>
-      </c>
-      <c r="N46" s="88">
-        <f>SUM(N43:N45)</f>
+      <c r="J46" s="114" t="inlineStr"/>
+      <c r="K46" s="88">
+        <f>SUM(K43:K45)</f>
+        <v/>
+      </c>
+      <c r="L46" s="88">
+        <f>SUM(L43:L45)</f>
+        <v/>
+      </c>
+      <c r="M46" s="130">
+        <f>SUMPRODUCT((M43:M45="✓")*1,B43:B45,C43:C45)</f>
+        <v/>
+      </c>
+      <c r="N46" s="130">
+        <f>SUMPRODUCT((N43:N45="✓")*1,B43:B45,C43:C45)</f>
+        <v/>
+      </c>
+      <c r="O46" s="130">
+        <f>SUMPRODUCT((O43:O45="✓")*1,B43:B45,C43:C45)</f>
+        <v/>
+      </c>
+      <c r="P46" s="130">
+        <f>SUMPRODUCT((P43:P45="✓")*1,B43:B45,C43:C45)</f>
         <v/>
       </c>
     </row>
@@ -4642,13 +4873,11 @@
       <c r="J48" s="77" t="n"/>
       <c r="K48" s="77" t="n"/>
       <c r="L48" s="77" t="n"/>
-      <c r="M48" s="77" t="n"/>
-      <c r="N48" s="77" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="109" t="inlineStr">
         <is>
-          <t>NBA/MLB Game (Ticket)</t>
+          <t>Beach/Surf Lesson</t>
         </is>
       </c>
       <c r="B49" s="83" t="n">
@@ -4662,23 +4891,32 @@
         <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E49" s="81" t="inlineStr"/>
+      <c r="E49" s="137">
+        <f>IF(D49&gt;0,(D49-C49)/D49,0)</f>
+        <v/>
+      </c>
       <c r="F49" s="81" t="inlineStr"/>
       <c r="G49" s="81" t="inlineStr"/>
       <c r="H49" s="81" t="inlineStr"/>
       <c r="I49" s="81" t="inlineStr"/>
-      <c r="J49" s="81" t="inlineStr"/>
-      <c r="K49" s="81" t="inlineStr"/>
-      <c r="L49" s="81" t="inlineStr"/>
-      <c r="M49" s="84">
-        <f>IF(A49="","",COUNTIF(E49:L49,"✓")*B49*C49)</f>
-        <v/>
-      </c>
-      <c r="N49" s="84">
-        <f>IF(A49="","",COUNTIF(E49:L49,"✓")*B49*D49)</f>
-        <v/>
-      </c>
-      <c r="O49" s="81">
+      <c r="J49" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K49" s="84">
+        <f>IF(A49="","",(COUNTIF(F49,"✓")+COUNTIF(G49,"✓")+COUNTIF(H49,"✓")+COUNTIF(I49,"✓")+COUNTIF(M49,"✓")+COUNTIF(N49,"✓")+COUNTIF(O49,"✓")+COUNTIF(P49,"✓"))*B49*C49)</f>
+        <v/>
+      </c>
+      <c r="L49" s="84">
+        <f>IF(A49="","",(COUNTIF(F49,"✓")+COUNTIF(G49,"✓")+COUNTIF(H49,"✓")+COUNTIF(I49,"✓")+COUNTIF(M49,"✓")+COUNTIF(N49,"✓")+COUNTIF(O49,"✓")+COUNTIF(P49,"✓"))*B49*D49)</f>
+        <v/>
+      </c>
+      <c r="M49" s="81" t="inlineStr"/>
+      <c r="N49" s="81" t="inlineStr"/>
+      <c r="O49" s="81" t="inlineStr"/>
+      <c r="P49" s="81" t="inlineStr"/>
+      <c r="Q49" s="81">
         <f>0</f>
         <v/>
       </c>
@@ -4686,7 +4924,7 @@
     <row r="50">
       <c r="A50" s="108" t="inlineStr">
         <is>
-          <t>Sports Bar Experience</t>
+          <t>Local Hiking (Griffith/Runyon)</t>
         </is>
       </c>
       <c r="B50" s="83" t="n">
@@ -4700,23 +4938,32 @@
         <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E50" s="81" t="inlineStr"/>
+      <c r="E50" s="137">
+        <f>IF(D50&gt;0,(D50-C50)/D50,0)</f>
+        <v/>
+      </c>
       <c r="F50" s="81" t="inlineStr"/>
       <c r="G50" s="81" t="inlineStr"/>
       <c r="H50" s="81" t="inlineStr"/>
       <c r="I50" s="81" t="inlineStr"/>
-      <c r="J50" s="81" t="inlineStr"/>
-      <c r="K50" s="81" t="inlineStr"/>
-      <c r="L50" s="81" t="inlineStr"/>
-      <c r="M50" s="84">
-        <f>IF(A50="","",COUNTIF(E50:L50,"✓")*B50*C50)</f>
-        <v/>
-      </c>
-      <c r="N50" s="84">
-        <f>IF(A50="","",COUNTIF(E50:L50,"✓")*B50*D50)</f>
-        <v/>
-      </c>
-      <c r="O50" s="81">
+      <c r="J50" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K50" s="84">
+        <f>IF(A50="","",(COUNTIF(F50,"✓")+COUNTIF(G50,"✓")+COUNTIF(H50,"✓")+COUNTIF(I50,"✓")+COUNTIF(M50,"✓")+COUNTIF(N50,"✓")+COUNTIF(O50,"✓")+COUNTIF(P50,"✓"))*B50*C50)</f>
+        <v/>
+      </c>
+      <c r="L50" s="84">
+        <f>IF(A50="","",(COUNTIF(F50,"✓")+COUNTIF(G50,"✓")+COUNTIF(H50,"✓")+COUNTIF(I50,"✓")+COUNTIF(M50,"✓")+COUNTIF(N50,"✓")+COUNTIF(O50,"✓")+COUNTIF(P50,"✓"))*B50*D50)</f>
+        <v/>
+      </c>
+      <c r="M50" s="81" t="inlineStr"/>
+      <c r="N50" s="81" t="inlineStr"/>
+      <c r="O50" s="81" t="inlineStr"/>
+      <c r="P50" s="81" t="inlineStr"/>
+      <c r="Q50" s="81">
         <f>IF(A50="",0,COUNTIF(A$49:A49,A50))</f>
         <v/>
       </c>
@@ -4724,7 +4971,7 @@
     <row r="51">
       <c r="A51" s="109" t="inlineStr">
         <is>
-          <t>Local Hiking (Griffith/Runyon)</t>
+          <t>NBA/MLB Game (Ticket)</t>
         </is>
       </c>
       <c r="B51" s="83" t="n">
@@ -4738,23 +4985,32 @@
         <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E51" s="81" t="inlineStr"/>
+      <c r="E51" s="137">
+        <f>IF(D51&gt;0,(D51-C51)/D51,0)</f>
+        <v/>
+      </c>
       <c r="F51" s="81" t="inlineStr"/>
       <c r="G51" s="81" t="inlineStr"/>
       <c r="H51" s="81" t="inlineStr"/>
       <c r="I51" s="81" t="inlineStr"/>
-      <c r="J51" s="81" t="inlineStr"/>
-      <c r="K51" s="81" t="inlineStr"/>
-      <c r="L51" s="81" t="inlineStr"/>
-      <c r="M51" s="84">
-        <f>IF(A51="","",COUNTIF(E51:L51,"✓")*B51*C51)</f>
-        <v/>
-      </c>
-      <c r="N51" s="84">
-        <f>IF(A51="","",COUNTIF(E51:L51,"✓")*B51*D51)</f>
-        <v/>
-      </c>
-      <c r="O51" s="81">
+      <c r="J51" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K51" s="84">
+        <f>IF(A51="","",(COUNTIF(F51,"✓")+COUNTIF(G51,"✓")+COUNTIF(H51,"✓")+COUNTIF(I51,"✓")+COUNTIF(M51,"✓")+COUNTIF(N51,"✓")+COUNTIF(O51,"✓")+COUNTIF(P51,"✓"))*B51*C51)</f>
+        <v/>
+      </c>
+      <c r="L51" s="84">
+        <f>IF(A51="","",(COUNTIF(F51,"✓")+COUNTIF(G51,"✓")+COUNTIF(H51,"✓")+COUNTIF(I51,"✓")+COUNTIF(M51,"✓")+COUNTIF(N51,"✓")+COUNTIF(O51,"✓")+COUNTIF(P51,"✓"))*B51*D51)</f>
+        <v/>
+      </c>
+      <c r="M51" s="81" t="inlineStr"/>
+      <c r="N51" s="81" t="inlineStr"/>
+      <c r="O51" s="81" t="inlineStr"/>
+      <c r="P51" s="81" t="inlineStr"/>
+      <c r="Q51" s="81">
         <f>IF(A51="",0,COUNTIF(A$49:A50,A51))</f>
         <v/>
       </c>
@@ -4762,7 +5018,7 @@
     <row r="52">
       <c r="A52" s="108" t="inlineStr">
         <is>
-          <t>Beach/Surf Lesson</t>
+          <t>Sports Bar Experience</t>
         </is>
       </c>
       <c r="B52" s="83" t="n">
@@ -4776,23 +5032,32 @@
         <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E52" s="81" t="inlineStr"/>
+      <c r="E52" s="137">
+        <f>IF(D52&gt;0,(D52-C52)/D52,0)</f>
+        <v/>
+      </c>
       <c r="F52" s="81" t="inlineStr"/>
       <c r="G52" s="81" t="inlineStr"/>
       <c r="H52" s="81" t="inlineStr"/>
       <c r="I52" s="81" t="inlineStr"/>
-      <c r="J52" s="81" t="inlineStr"/>
-      <c r="K52" s="81" t="inlineStr"/>
-      <c r="L52" s="81" t="inlineStr"/>
-      <c r="M52" s="84">
-        <f>IF(A52="","",COUNTIF(E52:L52,"✓")*B52*C52)</f>
-        <v/>
-      </c>
-      <c r="N52" s="84">
-        <f>IF(A52="","",COUNTIF(E52:L52,"✓")*B52*D52)</f>
-        <v/>
-      </c>
-      <c r="O52" s="81">
+      <c r="J52" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K52" s="84">
+        <f>IF(A52="","",(COUNTIF(F52,"✓")+COUNTIF(G52,"✓")+COUNTIF(H52,"✓")+COUNTIF(I52,"✓")+COUNTIF(M52,"✓")+COUNTIF(N52,"✓")+COUNTIF(O52,"✓")+COUNTIF(P52,"✓"))*B52*C52)</f>
+        <v/>
+      </c>
+      <c r="L52" s="84">
+        <f>IF(A52="","",(COUNTIF(F52,"✓")+COUNTIF(G52,"✓")+COUNTIF(H52,"✓")+COUNTIF(I52,"✓")+COUNTIF(M52,"✓")+COUNTIF(N52,"✓")+COUNTIF(O52,"✓")+COUNTIF(P52,"✓"))*B52*D52)</f>
+        <v/>
+      </c>
+      <c r="M52" s="81" t="inlineStr"/>
+      <c r="N52" s="81" t="inlineStr"/>
+      <c r="O52" s="81" t="inlineStr"/>
+      <c r="P52" s="81" t="inlineStr"/>
+      <c r="Q52" s="81">
         <f>IF(A52="",0,COUNTIF(A$49:A51,A52))</f>
         <v/>
       </c>
@@ -4808,23 +5073,32 @@
         <f>IF(A53="","",VLOOKUP(A53,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E53" s="81" t="inlineStr"/>
+      <c r="E53" s="137">
+        <f>IF(D53&gt;0,(D53-C53)/D53,0)</f>
+        <v/>
+      </c>
       <c r="F53" s="81" t="inlineStr"/>
       <c r="G53" s="81" t="inlineStr"/>
       <c r="H53" s="81" t="inlineStr"/>
       <c r="I53" s="81" t="inlineStr"/>
-      <c r="J53" s="81" t="inlineStr"/>
-      <c r="K53" s="81" t="inlineStr"/>
-      <c r="L53" s="81" t="inlineStr"/>
-      <c r="M53" s="84">
-        <f>IF(A53="","",COUNTIF(E53:L53,"✓")*B53*C53)</f>
-        <v/>
-      </c>
-      <c r="N53" s="84">
-        <f>IF(A53="","",COUNTIF(E53:L53,"✓")*B53*D53)</f>
-        <v/>
-      </c>
-      <c r="O53" s="81">
+      <c r="J53" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K53" s="84">
+        <f>IF(A53="","",(COUNTIF(F53,"✓")+COUNTIF(G53,"✓")+COUNTIF(H53,"✓")+COUNTIF(I53,"✓")+COUNTIF(M53,"✓")+COUNTIF(N53,"✓")+COUNTIF(O53,"✓")+COUNTIF(P53,"✓"))*B53*C53)</f>
+        <v/>
+      </c>
+      <c r="L53" s="84">
+        <f>IF(A53="","",(COUNTIF(F53,"✓")+COUNTIF(G53,"✓")+COUNTIF(H53,"✓")+COUNTIF(I53,"✓")+COUNTIF(M53,"✓")+COUNTIF(N53,"✓")+COUNTIF(O53,"✓")+COUNTIF(P53,"✓"))*B53*D53)</f>
+        <v/>
+      </c>
+      <c r="M53" s="81" t="inlineStr"/>
+      <c r="N53" s="81" t="inlineStr"/>
+      <c r="O53" s="81" t="inlineStr"/>
+      <c r="P53" s="81" t="inlineStr"/>
+      <c r="Q53" s="81">
         <f>IF(A53="",0,COUNTIF(A$49:A52,A53))</f>
         <v/>
       </c>
@@ -4840,23 +5114,32 @@
         <f>IF(A54="","",VLOOKUP(A54,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E54" s="81" t="inlineStr"/>
+      <c r="E54" s="137">
+        <f>IF(D54&gt;0,(D54-C54)/D54,0)</f>
+        <v/>
+      </c>
       <c r="F54" s="81" t="inlineStr"/>
       <c r="G54" s="81" t="inlineStr"/>
       <c r="H54" s="81" t="inlineStr"/>
       <c r="I54" s="81" t="inlineStr"/>
-      <c r="J54" s="81" t="inlineStr"/>
-      <c r="K54" s="81" t="inlineStr"/>
-      <c r="L54" s="81" t="inlineStr"/>
-      <c r="M54" s="84">
-        <f>IF(A54="","",COUNTIF(E54:L54,"✓")*B54*C54)</f>
-        <v/>
-      </c>
-      <c r="N54" s="84">
-        <f>IF(A54="","",COUNTIF(E54:L54,"✓")*B54*D54)</f>
-        <v/>
-      </c>
-      <c r="O54" s="81">
+      <c r="J54" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K54" s="84">
+        <f>IF(A54="","",(COUNTIF(F54,"✓")+COUNTIF(G54,"✓")+COUNTIF(H54,"✓")+COUNTIF(I54,"✓")+COUNTIF(M54,"✓")+COUNTIF(N54,"✓")+COUNTIF(O54,"✓")+COUNTIF(P54,"✓"))*B54*C54)</f>
+        <v/>
+      </c>
+      <c r="L54" s="84">
+        <f>IF(A54="","",(COUNTIF(F54,"✓")+COUNTIF(G54,"✓")+COUNTIF(H54,"✓")+COUNTIF(I54,"✓")+COUNTIF(M54,"✓")+COUNTIF(N54,"✓")+COUNTIF(O54,"✓")+COUNTIF(P54,"✓"))*B54*D54)</f>
+        <v/>
+      </c>
+      <c r="M54" s="81" t="inlineStr"/>
+      <c r="N54" s="81" t="inlineStr"/>
+      <c r="O54" s="81" t="inlineStr"/>
+      <c r="P54" s="81" t="inlineStr"/>
+      <c r="Q54" s="81">
         <f>IF(A54="",0,COUNTIF(A$49:A53,A54))</f>
         <v/>
       </c>
@@ -4872,23 +5155,32 @@
         <f>IF(A55="","",VLOOKUP(A55,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E55" s="81" t="inlineStr"/>
+      <c r="E55" s="137">
+        <f>IF(D55&gt;0,(D55-C55)/D55,0)</f>
+        <v/>
+      </c>
       <c r="F55" s="81" t="inlineStr"/>
       <c r="G55" s="81" t="inlineStr"/>
       <c r="H55" s="81" t="inlineStr"/>
       <c r="I55" s="81" t="inlineStr"/>
-      <c r="J55" s="81" t="inlineStr"/>
-      <c r="K55" s="81" t="inlineStr"/>
-      <c r="L55" s="81" t="inlineStr"/>
-      <c r="M55" s="84">
-        <f>IF(A55="","",COUNTIF(E55:L55,"✓")*B55*C55)</f>
-        <v/>
-      </c>
-      <c r="N55" s="84">
-        <f>IF(A55="","",COUNTIF(E55:L55,"✓")*B55*D55)</f>
-        <v/>
-      </c>
-      <c r="O55" s="81">
+      <c r="J55" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K55" s="84">
+        <f>IF(A55="","",(COUNTIF(F55,"✓")+COUNTIF(G55,"✓")+COUNTIF(H55,"✓")+COUNTIF(I55,"✓")+COUNTIF(M55,"✓")+COUNTIF(N55,"✓")+COUNTIF(O55,"✓")+COUNTIF(P55,"✓"))*B55*C55)</f>
+        <v/>
+      </c>
+      <c r="L55" s="84">
+        <f>IF(A55="","",(COUNTIF(F55,"✓")+COUNTIF(G55,"✓")+COUNTIF(H55,"✓")+COUNTIF(I55,"✓")+COUNTIF(M55,"✓")+COUNTIF(N55,"✓")+COUNTIF(O55,"✓")+COUNTIF(P55,"✓"))*B55*D55)</f>
+        <v/>
+      </c>
+      <c r="M55" s="81" t="inlineStr"/>
+      <c r="N55" s="81" t="inlineStr"/>
+      <c r="O55" s="81" t="inlineStr"/>
+      <c r="P55" s="81" t="inlineStr"/>
+      <c r="Q55" s="81">
         <f>IF(A55="",0,COUNTIF(A$49:A54,A55))</f>
         <v/>
       </c>
@@ -4904,23 +5196,32 @@
         <f>IF(A56="","",VLOOKUP(A56,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E56" s="81" t="inlineStr"/>
+      <c r="E56" s="137">
+        <f>IF(D56&gt;0,(D56-C56)/D56,0)</f>
+        <v/>
+      </c>
       <c r="F56" s="81" t="inlineStr"/>
       <c r="G56" s="81" t="inlineStr"/>
       <c r="H56" s="81" t="inlineStr"/>
       <c r="I56" s="81" t="inlineStr"/>
-      <c r="J56" s="81" t="inlineStr"/>
-      <c r="K56" s="81" t="inlineStr"/>
-      <c r="L56" s="81" t="inlineStr"/>
-      <c r="M56" s="84">
-        <f>IF(A56="","",COUNTIF(E56:L56,"✓")*B56*C56)</f>
-        <v/>
-      </c>
-      <c r="N56" s="84">
-        <f>IF(A56="","",COUNTIF(E56:L56,"✓")*B56*D56)</f>
-        <v/>
-      </c>
-      <c r="O56" s="81">
+      <c r="J56" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K56" s="84">
+        <f>IF(A56="","",(COUNTIF(F56,"✓")+COUNTIF(G56,"✓")+COUNTIF(H56,"✓")+COUNTIF(I56,"✓")+COUNTIF(M56,"✓")+COUNTIF(N56,"✓")+COUNTIF(O56,"✓")+COUNTIF(P56,"✓"))*B56*C56)</f>
+        <v/>
+      </c>
+      <c r="L56" s="84">
+        <f>IF(A56="","",(COUNTIF(F56,"✓")+COUNTIF(G56,"✓")+COUNTIF(H56,"✓")+COUNTIF(I56,"✓")+COUNTIF(M56,"✓")+COUNTIF(N56,"✓")+COUNTIF(O56,"✓")+COUNTIF(P56,"✓"))*B56*D56)</f>
+        <v/>
+      </c>
+      <c r="M56" s="81" t="inlineStr"/>
+      <c r="N56" s="81" t="inlineStr"/>
+      <c r="O56" s="81" t="inlineStr"/>
+      <c r="P56" s="81" t="inlineStr"/>
+      <c r="Q56" s="81">
         <f>IF(A56="",0,COUNTIF(A$49:A55,A56))</f>
         <v/>
       </c>
@@ -4936,23 +5237,32 @@
         <f>IF(A57="","",VLOOKUP(A57,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E57" s="81" t="inlineStr"/>
+      <c r="E57" s="137">
+        <f>IF(D57&gt;0,(D57-C57)/D57,0)</f>
+        <v/>
+      </c>
       <c r="F57" s="81" t="inlineStr"/>
       <c r="G57" s="81" t="inlineStr"/>
       <c r="H57" s="81" t="inlineStr"/>
       <c r="I57" s="81" t="inlineStr"/>
-      <c r="J57" s="81" t="inlineStr"/>
-      <c r="K57" s="81" t="inlineStr"/>
-      <c r="L57" s="81" t="inlineStr"/>
-      <c r="M57" s="84">
-        <f>IF(A57="","",COUNTIF(E57:L57,"✓")*B57*C57)</f>
-        <v/>
-      </c>
-      <c r="N57" s="84">
-        <f>IF(A57="","",COUNTIF(E57:L57,"✓")*B57*D57)</f>
-        <v/>
-      </c>
-      <c r="O57" s="81">
+      <c r="J57" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K57" s="84">
+        <f>IF(A57="","",(COUNTIF(F57,"✓")+COUNTIF(G57,"✓")+COUNTIF(H57,"✓")+COUNTIF(I57,"✓")+COUNTIF(M57,"✓")+COUNTIF(N57,"✓")+COUNTIF(O57,"✓")+COUNTIF(P57,"✓"))*B57*C57)</f>
+        <v/>
+      </c>
+      <c r="L57" s="84">
+        <f>IF(A57="","",(COUNTIF(F57,"✓")+COUNTIF(G57,"✓")+COUNTIF(H57,"✓")+COUNTIF(I57,"✓")+COUNTIF(M57,"✓")+COUNTIF(N57,"✓")+COUNTIF(O57,"✓")+COUNTIF(P57,"✓"))*B57*D57)</f>
+        <v/>
+      </c>
+      <c r="M57" s="81" t="inlineStr"/>
+      <c r="N57" s="81" t="inlineStr"/>
+      <c r="O57" s="81" t="inlineStr"/>
+      <c r="P57" s="81" t="inlineStr"/>
+      <c r="Q57" s="81">
         <f>IF(A57="",0,COUNTIF(A$49:A56,A57))</f>
         <v/>
       </c>
@@ -4966,10 +5276,7 @@
       <c r="B58" s="114" t="inlineStr"/>
       <c r="C58" s="114" t="inlineStr"/>
       <c r="D58" s="114" t="inlineStr"/>
-      <c r="E58" s="130">
-        <f>SUMPRODUCT((E49:E57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
+      <c r="E58" s="114" t="inlineStr"/>
       <c r="F58" s="130">
         <f>SUMPRODUCT((F49:F57="✓")*1,B49:B57,C49:C57)</f>
         <v/>
@@ -4986,24 +5293,29 @@
         <f>SUMPRODUCT((I49:I57="✓")*1,B49:B57,C49:C57)</f>
         <v/>
       </c>
-      <c r="J58" s="130">
-        <f>SUMPRODUCT((J49:J57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="K58" s="130">
-        <f>SUMPRODUCT((K49:K57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="L58" s="130">
-        <f>SUMPRODUCT((L49:L57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="M58" s="88">
-        <f>SUM(M49:M57)</f>
-        <v/>
-      </c>
-      <c r="N58" s="88">
-        <f>SUM(N49:N57)</f>
+      <c r="J58" s="114" t="inlineStr"/>
+      <c r="K58" s="88">
+        <f>SUM(K49:K57)</f>
+        <v/>
+      </c>
+      <c r="L58" s="88">
+        <f>SUM(L49:L57)</f>
+        <v/>
+      </c>
+      <c r="M58" s="130">
+        <f>SUMPRODUCT((M49:M57="✓")*1,B49:B57,C49:C57)</f>
+        <v/>
+      </c>
+      <c r="N58" s="130">
+        <f>SUMPRODUCT((N49:N57="✓")*1,B49:B57,C49:C57)</f>
+        <v/>
+      </c>
+      <c r="O58" s="130">
+        <f>SUMPRODUCT((O49:O57="✓")*1,B49:B57,C49:C57)</f>
+        <v/>
+      </c>
+      <c r="P58" s="130">
+        <f>SUMPRODUCT((P49:P57="✓")*1,B49:B57,C49:C57)</f>
         <v/>
       </c>
     </row>
@@ -5024,8 +5336,6 @@
       <c r="J61" s="104" t="n"/>
       <c r="K61" s="104" t="n"/>
       <c r="L61" s="104" t="n"/>
-      <c r="M61" s="104" t="n"/>
-      <c r="N61" s="104" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="108" t="inlineStr">
@@ -5033,12 +5343,12 @@
           <t>GOLF</t>
         </is>
       </c>
-      <c r="M62" s="84">
-        <f>M20</f>
-        <v/>
-      </c>
-      <c r="N62" s="84">
-        <f>N20</f>
+      <c r="K62" s="84">
+        <f>K20</f>
+        <v/>
+      </c>
+      <c r="L62" s="84">
+        <f>L20</f>
         <v/>
       </c>
     </row>
@@ -5048,12 +5358,12 @@
           <t>HOTEL</t>
         </is>
       </c>
-      <c r="M63" s="84">
-        <f>M26</f>
-        <v/>
-      </c>
-      <c r="N63" s="84">
-        <f>N26</f>
+      <c r="K63" s="84">
+        <f>K26</f>
+        <v/>
+      </c>
+      <c r="L63" s="84">
+        <f>L26</f>
         <v/>
       </c>
     </row>
@@ -5063,12 +5373,12 @@
           <t>TRANSPORT</t>
         </is>
       </c>
-      <c r="M64" s="84">
-        <f>M32</f>
-        <v/>
-      </c>
-      <c r="N64" s="84">
-        <f>N32</f>
+      <c r="K64" s="84">
+        <f>K32</f>
+        <v/>
+      </c>
+      <c r="L64" s="84">
+        <f>L32</f>
         <v/>
       </c>
     </row>
@@ -5078,12 +5388,12 @@
           <t>MEALS</t>
         </is>
       </c>
-      <c r="M65" s="84">
-        <f>M40</f>
-        <v/>
-      </c>
-      <c r="N65" s="84">
-        <f>N40</f>
+      <c r="K65" s="84">
+        <f>K40</f>
+        <v/>
+      </c>
+      <c r="L65" s="84">
+        <f>L40</f>
         <v/>
       </c>
     </row>
@@ -5093,12 +5403,12 @@
           <t>OTHER</t>
         </is>
       </c>
-      <c r="M66" s="84">
-        <f>M46</f>
-        <v/>
-      </c>
-      <c r="N66" s="84">
-        <f>N46</f>
+      <c r="K66" s="84">
+        <f>K46</f>
+        <v/>
+      </c>
+      <c r="L66" s="84">
+        <f>L46</f>
         <v/>
       </c>
     </row>
@@ -5108,12 +5418,12 @@
           <t>ACTIVITIES</t>
         </is>
       </c>
-      <c r="M67" s="84">
-        <f>M58</f>
-        <v/>
-      </c>
-      <c r="N67" s="84">
-        <f>N58</f>
+      <c r="K67" s="84">
+        <f>K58</f>
+        <v/>
+      </c>
+      <c r="L67" s="84">
+        <f>L58</f>
         <v/>
       </c>
     </row>
@@ -5123,21 +5433,21 @@
           <t>📌 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B68" s="116" t="inlineStr">
+      <c r="C68" s="116" t="inlineStr">
         <is>
           <t>Margin:</t>
         </is>
       </c>
-      <c r="C68" s="91">
-        <f>IF(N68&gt;0,(N68-M68)/N68,0)</f>
-        <v/>
-      </c>
-      <c r="M68" s="88">
-        <f>SUM(M62:M67)</f>
-        <v/>
-      </c>
-      <c r="N68" s="88">
-        <f>SUM(N62:N67)</f>
+      <c r="D68" s="91">
+        <f>IF(L68&gt;0,(L68-K68)/L68,0)</f>
+        <v/>
+      </c>
+      <c r="K68" s="88">
+        <f>SUM(K62:K67)</f>
+        <v/>
+      </c>
+      <c r="L68" s="88">
+        <f>SUM(L62:L67)</f>
         <v/>
       </c>
     </row>
@@ -5158,8 +5468,6 @@
       <c r="J70" s="104" t="n"/>
       <c r="K70" s="104" t="n"/>
       <c r="L70" s="104" t="n"/>
-      <c r="M70" s="104" t="n"/>
-      <c r="N70" s="104" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="98" t="inlineStr">
@@ -5187,6 +5495,11 @@
           <t>%</t>
         </is>
       </c>
+      <c r="F71" s="98" t="inlineStr">
+        <is>
+          <t>#Items</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="108" t="inlineStr">
@@ -5195,11 +5508,11 @@
         </is>
       </c>
       <c r="B72" s="131">
-        <f>SUMPRODUCT((E15:E19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((E23:E25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((E29:E31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((E35:E39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((E43:E45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((E49:E57="✓")*1,B49:B57,C49:C57)</f>
+        <f>SUMPRODUCT((F15:F19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((F23:F25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((F29:F31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((F35:F39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((F43:F45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((F49:F57="✓")*1,B49:B57,C49:C57)</f>
         <v/>
       </c>
       <c r="C72" s="131">
-        <f>SUMPRODUCT((E15:E19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((E23:E25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((E29:E31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((E35:E39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((E43:E45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((E49:E57="✓")*1,B49:B57,D49:D57)</f>
+        <f>SUMPRODUCT((F15:F19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((F23:F25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((F29:F31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((F35:F39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((F43:F45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((F49:F57="✓")*1,B49:B57,D49:D57)</f>
         <v/>
       </c>
       <c r="D72" s="110">
@@ -5210,6 +5523,10 @@
         <f>IF(C72&gt;0,D72/C72,0)</f>
         <v/>
       </c>
+      <c r="F72" s="139">
+        <f>COUNTIF(F15:F19,"✓")+COUNTIF(F23:F25,"✓")+COUNTIF(F29:F31,"✓")+COUNTIF(F35:F39,"✓")+COUNTIF(F43:F45,"✓")+COUNTIF(F49:F57,"✓")</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="108" t="inlineStr">
@@ -5218,11 +5535,11 @@
         </is>
       </c>
       <c r="B73" s="131">
-        <f>SUMPRODUCT((F15:F19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((F23:F25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((F29:F31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((F35:F39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((F43:F45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((F49:F57="✓")*1,B49:B57,C49:C57)</f>
+        <f>SUMPRODUCT((G15:G19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((G23:G25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((G29:G31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((G35:G39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((G43:G45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((G49:G57="✓")*1,B49:B57,C49:C57)</f>
         <v/>
       </c>
       <c r="C73" s="131">
-        <f>SUMPRODUCT((F15:F19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((F23:F25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((F29:F31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((F35:F39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((F43:F45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((F49:F57="✓")*1,B49:B57,D49:D57)</f>
+        <f>SUMPRODUCT((G15:G19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((G23:G25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((G29:G31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((G35:G39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((G43:G45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((G49:G57="✓")*1,B49:B57,D49:D57)</f>
         <v/>
       </c>
       <c r="D73" s="110">
@@ -5233,6 +5550,10 @@
         <f>IF(C73&gt;0,D73/C73,0)</f>
         <v/>
       </c>
+      <c r="F73" s="139">
+        <f>COUNTIF(G15:G19,"✓")+COUNTIF(G23:G25,"✓")+COUNTIF(G29:G31,"✓")+COUNTIF(G35:G39,"✓")+COUNTIF(G43:G45,"✓")+COUNTIF(G49:G57,"✓")</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="108" t="inlineStr">
@@ -5241,11 +5562,11 @@
         </is>
       </c>
       <c r="B74" s="131">
-        <f>SUMPRODUCT((G15:G19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((G23:G25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((G29:G31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((G35:G39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((G43:G45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((G49:G57="✓")*1,B49:B57,C49:C57)</f>
+        <f>SUMPRODUCT((H15:H19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((H23:H25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((H29:H31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((H35:H39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((H43:H45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((H49:H57="✓")*1,B49:B57,C49:C57)</f>
         <v/>
       </c>
       <c r="C74" s="131">
-        <f>SUMPRODUCT((G15:G19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((G23:G25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((G29:G31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((G35:G39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((G43:G45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((G49:G57="✓")*1,B49:B57,D49:D57)</f>
+        <f>SUMPRODUCT((H15:H19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((H23:H25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((H29:H31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((H35:H39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((H43:H45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((H49:H57="✓")*1,B49:B57,D49:D57)</f>
         <v/>
       </c>
       <c r="D74" s="110">
@@ -5256,6 +5577,10 @@
         <f>IF(C74&gt;0,D74/C74,0)</f>
         <v/>
       </c>
+      <c r="F74" s="139">
+        <f>COUNTIF(H15:H19,"✓")+COUNTIF(H23:H25,"✓")+COUNTIF(H29:H31,"✓")+COUNTIF(H35:H39,"✓")+COUNTIF(H43:H45,"✓")+COUNTIF(H49:H57,"✓")</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="108" t="inlineStr">
@@ -5264,11 +5589,11 @@
         </is>
       </c>
       <c r="B75" s="131">
-        <f>SUMPRODUCT((H15:H19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((H23:H25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((H29:H31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((H35:H39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((H43:H45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((H49:H57="✓")*1,B49:B57,C49:C57)</f>
+        <f>SUMPRODUCT((I15:I19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((I23:I25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((I29:I31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((I35:I39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((I43:I45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((I49:I57="✓")*1,B49:B57,C49:C57)</f>
         <v/>
       </c>
       <c r="C75" s="131">
-        <f>SUMPRODUCT((H15:H19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((H23:H25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((H29:H31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((H35:H39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((H43:H45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((H49:H57="✓")*1,B49:B57,D49:D57)</f>
+        <f>SUMPRODUCT((I15:I19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((I23:I25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((I29:I31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((I35:I39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((I43:I45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((I49:I57="✓")*1,B49:B57,D49:D57)</f>
         <v/>
       </c>
       <c r="D75" s="110">
@@ -5279,528 +5604,756 @@
         <f>IF(C75&gt;0,D75/C75,0)</f>
         <v/>
       </c>
+      <c r="F75" s="139">
+        <f>COUNTIF(I15:I19,"✓")+COUNTIF(I23:I25,"✓")+COUNTIF(I29:I31,"✓")+COUNTIF(I35:I39,"✓")+COUNTIF(I43:I45,"✓")+COUNTIF(I49:I57,"✓")</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="108" t="inlineStr">
-        <is>
-          <t>참가자5</t>
-        </is>
-      </c>
-      <c r="B76" s="131">
-        <f>SUMPRODUCT((I15:I19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((I23:I25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((I29:I31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((I35:I39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((I43:I45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((I49:I57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="C76" s="131">
-        <f>SUMPRODUCT((I15:I19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((I23:I25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((I29:I31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((I35:I39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((I43:I45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((I49:I57="✓")*1,B49:B57,D49:D57)</f>
-        <v/>
-      </c>
-      <c r="D76" s="110">
-        <f>C76-B76</f>
-        <v/>
-      </c>
-      <c r="E76" s="132">
+      <c r="A76" s="115" t="inlineStr">
+        <is>
+          <t>📌 TOTAL</t>
+        </is>
+      </c>
+      <c r="B76" s="88">
+        <f>SUM(B72:B75)</f>
+        <v/>
+      </c>
+      <c r="C76" s="88">
+        <f>SUM(C72:C75)</f>
+        <v/>
+      </c>
+      <c r="D76" s="88">
+        <f>SUM(D72:D75)</f>
+        <v/>
+      </c>
+      <c r="E76" s="91">
         <f>IF(C76&gt;0,D76/C76,0)</f>
         <v/>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="108" t="inlineStr">
-        <is>
-          <t>참가자6</t>
-        </is>
-      </c>
-      <c r="B77" s="131">
-        <f>SUMPRODUCT((J15:J19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((J23:J25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((J29:J31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((J35:J39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((J43:J45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((J49:J57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="C77" s="131">
-        <f>SUMPRODUCT((J15:J19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((J23:J25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((J29:J31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((J35:J39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((J43:J45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((J49:J57="✓")*1,B49:B57,D49:D57)</f>
-        <v/>
-      </c>
-      <c r="D77" s="110">
-        <f>C77-B77</f>
-        <v/>
-      </c>
-      <c r="E77" s="132">
-        <f>IF(C77&gt;0,D77/C77,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="108" t="inlineStr">
-        <is>
-          <t>참가자7</t>
-        </is>
-      </c>
-      <c r="B78" s="131">
-        <f>SUMPRODUCT((K15:K19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((K23:K25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((K29:K31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((K35:K39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((K43:K45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((K49:K57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="C78" s="131">
-        <f>SUMPRODUCT((K15:K19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((K23:K25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((K29:K31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((K35:K39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((K43:K45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((K49:K57="✓")*1,B49:B57,D49:D57)</f>
-        <v/>
-      </c>
-      <c r="D78" s="110">
-        <f>C78-B78</f>
-        <v/>
-      </c>
-      <c r="E78" s="132">
-        <f>IF(C78&gt;0,D78/C78,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="108" t="inlineStr">
-        <is>
-          <t>참가자8</t>
-        </is>
-      </c>
-      <c r="B79" s="131">
-        <f>SUMPRODUCT((L15:L19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((L23:L25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((L29:L31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((L35:L39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((L43:L45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((L49:L57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="C79" s="131">
-        <f>SUMPRODUCT((L15:L19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((L23:L25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((L29:L31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((L35:L39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((L43:L45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((L49:L57="✓")*1,B49:B57,D49:D57)</f>
-        <v/>
-      </c>
-      <c r="D79" s="110">
-        <f>C79-B79</f>
-        <v/>
-      </c>
-      <c r="E79" s="132">
-        <f>IF(C79&gt;0,D79/C79,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="115" t="inlineStr">
-        <is>
-          <t>📌 TOTAL</t>
-        </is>
-      </c>
-      <c r="B80" s="88">
-        <f>SUM(B72:B79)</f>
-        <v/>
-      </c>
-      <c r="C80" s="88">
-        <f>SUM(C72:C79)</f>
-        <v/>
-      </c>
-      <c r="D80" s="88">
-        <f>SUM(D72:D79)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="134" t="inlineStr">
-        <is>
-          <t>⚠️ DUPLICATE ITEMS</t>
-        </is>
-      </c>
-      <c r="B82" s="135" t="n"/>
-      <c r="C82" s="135" t="n"/>
-      <c r="D82" s="135" t="n"/>
-      <c r="E82" s="135" t="n"/>
-      <c r="F82" s="135" t="n"/>
-      <c r="G82" s="135" t="n"/>
-      <c r="H82" s="135" t="n"/>
-      <c r="I82" s="135" t="n"/>
-      <c r="J82" s="135" t="n"/>
-      <c r="K82" s="135" t="n"/>
-      <c r="L82" s="135" t="n"/>
-      <c r="M82" s="135" t="n"/>
-      <c r="N82" s="135" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="136">
-        <f>IF(SUM(O:O)&gt;0,"❌ "&amp;SUM(O:O)&amp;" duplicate(s) detected — check red cells in hidden column O","✅ No duplicates")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="124" t="inlineStr">
-        <is>
-          <t>🔍 CROSS-CHECKS</t>
-        </is>
-      </c>
-      <c r="B85" s="125" t="n"/>
-      <c r="C85" s="125" t="n"/>
-      <c r="D85" s="125" t="n"/>
-      <c r="E85" s="125" t="n"/>
-      <c r="F85" s="125" t="n"/>
-      <c r="G85" s="125" t="n"/>
-      <c r="H85" s="125" t="n"/>
-      <c r="I85" s="125" t="n"/>
-      <c r="J85" s="125" t="n"/>
-      <c r="K85" s="125" t="n"/>
-      <c r="L85" s="125" t="n"/>
-      <c r="M85" s="125" t="n"/>
-      <c r="N85" s="125" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="126" t="inlineStr">
-        <is>
-          <t>Grand Total Cost (item table):</t>
-        </is>
-      </c>
-      <c r="M86" s="84">
-        <f>M68</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="126" t="inlineStr">
-        <is>
-          <t>Per Person Sum:</t>
-        </is>
-      </c>
-      <c r="M87" s="84">
-        <f>B80</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="116" t="inlineStr">
-        <is>
-          <t>Difference:</t>
-        </is>
-      </c>
-      <c r="M88" s="117">
-        <f>M87-M86</f>
-        <v/>
-      </c>
-      <c r="N88" s="118">
-        <f>IF(M88=0,"✅ MATCH","❌ MISMATCH")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="124" t="inlineStr">
-        <is>
-          <t>💡 HOW TO USE</t>
-        </is>
-      </c>
-      <c r="B90" s="125" t="n"/>
-      <c r="C90" s="125" t="n"/>
-      <c r="D90" s="125" t="n"/>
-      <c r="E90" s="125" t="n"/>
-      <c r="F90" s="125" t="n"/>
-      <c r="G90" s="125" t="n"/>
-      <c r="H90" s="125" t="n"/>
-      <c r="I90" s="125" t="n"/>
-      <c r="J90" s="125" t="n"/>
-      <c r="K90" s="125" t="n"/>
-      <c r="L90" s="125" t="n"/>
-      <c r="M90" s="125" t="n"/>
-      <c r="N90" s="125" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="108" t="inlineStr">
-        <is>
-          <t>① A열: 드롭다운에서 항목 선택 (Master Data 연동)  |  빈칸은 신규항목 추가용</t>
-        </is>
-      </c>
-      <c r="B91" s="81" t="n"/>
-      <c r="C91" s="81" t="n"/>
-      <c r="D91" s="81" t="n"/>
-      <c r="E91" s="81" t="n"/>
-      <c r="F91" s="81" t="n"/>
-      <c r="G91" s="81" t="n"/>
-      <c r="H91" s="81" t="n"/>
-      <c r="I91" s="81" t="n"/>
-      <c r="J91" s="81" t="n"/>
-      <c r="K91" s="81" t="n"/>
-      <c r="L91" s="81" t="n"/>
-      <c r="M91" s="81" t="n"/>
-      <c r="N91" s="81" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="108" t="inlineStr">
-        <is>
-          <t>② Qty/p: 1인당 수량 (골프=라운드, 호텔=박, 식사=끼니)</t>
-        </is>
-      </c>
-      <c r="B92" s="81" t="n"/>
-      <c r="C92" s="81" t="n"/>
-      <c r="D92" s="81" t="n"/>
-      <c r="E92" s="81" t="n"/>
-      <c r="F92" s="81" t="n"/>
-      <c r="G92" s="81" t="n"/>
-      <c r="H92" s="81" t="n"/>
-      <c r="I92" s="81" t="n"/>
-      <c r="J92" s="81" t="n"/>
-      <c r="K92" s="81" t="n"/>
-      <c r="L92" s="81" t="n"/>
-      <c r="M92" s="81" t="n"/>
-      <c r="N92" s="81" t="n"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="108" t="inlineStr">
-        <is>
-          <t>③ P1~P8: ✓ 체크 = 해당 참가자에게 이 항목 포함 (드롭다운)</t>
-        </is>
-      </c>
-      <c r="B93" s="81" t="n"/>
-      <c r="C93" s="81" t="n"/>
-      <c r="D93" s="81" t="n"/>
-      <c r="E93" s="81" t="n"/>
-      <c r="F93" s="81" t="n"/>
-      <c r="G93" s="81" t="n"/>
-      <c r="H93" s="81" t="n"/>
-      <c r="I93" s="81" t="n"/>
-      <c r="J93" s="81" t="n"/>
-      <c r="K93" s="81" t="n"/>
-      <c r="L93" s="81" t="n"/>
-      <c r="M93" s="81" t="n"/>
-      <c r="N93" s="81" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="108" t="inlineStr">
-        <is>
-          <t>④ Total = (✓ 수) × Qty × Cost/P  —  자동계산</t>
-        </is>
-      </c>
-      <c r="B94" s="81" t="n"/>
-      <c r="C94" s="81" t="n"/>
-      <c r="D94" s="81" t="n"/>
-      <c r="E94" s="81" t="n"/>
-      <c r="F94" s="81" t="n"/>
-      <c r="G94" s="81" t="n"/>
-      <c r="H94" s="81" t="n"/>
-      <c r="I94" s="81" t="n"/>
-      <c r="J94" s="81" t="n"/>
-      <c r="K94" s="81" t="n"/>
-      <c r="L94" s="81" t="n"/>
-      <c r="M94" s="81" t="n"/>
-      <c r="N94" s="81" t="n"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="108" t="inlineStr">
-        <is>
-          <t>⑤ 중복: 같은 섹션 내 동일항목 중복선택 → O열 빨간불 (hidden)</t>
-        </is>
-      </c>
-      <c r="B95" s="81" t="n"/>
-      <c r="C95" s="81" t="n"/>
-      <c r="D95" s="81" t="n"/>
-      <c r="E95" s="81" t="n"/>
-      <c r="F95" s="81" t="n"/>
-      <c r="G95" s="81" t="n"/>
-      <c r="H95" s="81" t="n"/>
-      <c r="I95" s="81" t="n"/>
-      <c r="J95" s="81" t="n"/>
-      <c r="K95" s="81" t="n"/>
-      <c r="L95" s="81" t="n"/>
-      <c r="M95" s="81" t="n"/>
-      <c r="N95" s="81" t="n"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="108" t="inlineStr">
-        <is>
-          <t>⑥ Per Person = SUMPRODUCT 전체 카테고리 합산</t>
-        </is>
-      </c>
-      <c r="B96" s="81" t="n"/>
-      <c r="C96" s="81" t="n"/>
-      <c r="D96" s="81" t="n"/>
-      <c r="E96" s="81" t="n"/>
-      <c r="F96" s="81" t="n"/>
-      <c r="G96" s="81" t="n"/>
-      <c r="H96" s="81" t="n"/>
-      <c r="I96" s="81" t="n"/>
-      <c r="J96" s="81" t="n"/>
-      <c r="K96" s="81" t="n"/>
-      <c r="L96" s="81" t="n"/>
-      <c r="M96" s="81" t="n"/>
-      <c r="N96" s="81" t="n"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="108" t="inlineStr">
-        <is>
-          <t>⑦ 교차검증: Item Table 총액 = Per Person 합계 → ✅</t>
-        </is>
-      </c>
-      <c r="B97" s="81" t="n"/>
-      <c r="C97" s="81" t="n"/>
-      <c r="D97" s="81" t="n"/>
-      <c r="E97" s="81" t="n"/>
-      <c r="F97" s="81" t="n"/>
-      <c r="G97" s="81" t="n"/>
-      <c r="H97" s="81" t="n"/>
-      <c r="I97" s="81" t="n"/>
-      <c r="J97" s="81" t="n"/>
-      <c r="K97" s="81" t="n"/>
-      <c r="L97" s="81" t="n"/>
-      <c r="M97" s="81" t="n"/>
-      <c r="N97" s="81" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="17">
-    <mergeCell ref="A70:N70"/>
-    <mergeCell ref="A85:N85"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="A61:N61"/>
-    <mergeCell ref="A6:N6"/>
-    <mergeCell ref="A22:N22"/>
-    <mergeCell ref="A34:N34"/>
-    <mergeCell ref="A12:N12"/>
-    <mergeCell ref="A48:N48"/>
-    <mergeCell ref="A2:N2"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="A82:N82"/>
-    <mergeCell ref="A90:N90"/>
-    <mergeCell ref="A42:N42"/>
-    <mergeCell ref="A28:N28"/>
-    <mergeCell ref="A14:N14"/>
-    <mergeCell ref="A1:N1"/>
+  <mergeCells count="12">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A42:L42"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A28:L28"/>
+    <mergeCell ref="A34:L34"/>
+    <mergeCell ref="A14:L14"/>
+    <mergeCell ref="A61:L61"/>
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A70:L70"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="A48:L48"/>
   </mergeCells>
-  <conditionalFormatting sqref="O15">
-    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O16">
-    <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O17">
-    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O18">
-    <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O19">
+  <conditionalFormatting sqref="F15">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G15">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H15">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I15">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q15">
     <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O23">
-    <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O24">
-    <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O25">
-    <cfRule type="cellIs" priority="8" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O29">
-    <cfRule type="cellIs" priority="9" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O30">
+  <conditionalFormatting sqref="F16">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G16">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I16">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q16">
     <cfRule type="cellIs" priority="10" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O31">
-    <cfRule type="cellIs" priority="11" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O35">
-    <cfRule type="cellIs" priority="12" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O36">
-    <cfRule type="cellIs" priority="13" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O37">
-    <cfRule type="cellIs" priority="14" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O38">
+  <conditionalFormatting sqref="F17">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I17">
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q17">
     <cfRule type="cellIs" priority="15" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O39">
-    <cfRule type="cellIs" priority="16" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O43">
-    <cfRule type="cellIs" priority="17" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O44">
-    <cfRule type="cellIs" priority="18" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O45">
-    <cfRule type="cellIs" priority="19" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O49">
+  <conditionalFormatting sqref="F18">
+    <cfRule type="cellIs" priority="16" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G18">
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H18">
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I18">
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q18">
     <cfRule type="cellIs" priority="20" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O50">
-    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O51">
-    <cfRule type="cellIs" priority="22" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O52">
-    <cfRule type="cellIs" priority="23" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O53">
-    <cfRule type="cellIs" priority="24" operator="greaterThan" dxfId="3">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O54">
+  <conditionalFormatting sqref="F19">
+    <cfRule type="cellIs" priority="21" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G19">
+    <cfRule type="cellIs" priority="22" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H19">
+    <cfRule type="cellIs" priority="23" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I19">
+    <cfRule type="cellIs" priority="24" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q19">
     <cfRule type="cellIs" priority="25" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O55">
-    <cfRule type="cellIs" priority="26" operator="greaterThan" dxfId="3">
+  <conditionalFormatting sqref="F23">
+    <cfRule type="cellIs" priority="26" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G23">
+    <cfRule type="cellIs" priority="27" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H23">
+    <cfRule type="cellIs" priority="28" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I23">
+    <cfRule type="cellIs" priority="29" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q23">
+    <cfRule type="cellIs" priority="30" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O56">
-    <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="3">
+  <conditionalFormatting sqref="F24">
+    <cfRule type="cellIs" priority="31" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G24">
+    <cfRule type="cellIs" priority="32" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24">
+    <cfRule type="cellIs" priority="33" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I24">
+    <cfRule type="cellIs" priority="34" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q24">
+    <cfRule type="cellIs" priority="35" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O57">
-    <cfRule type="cellIs" priority="28" operator="greaterThan" dxfId="3">
+  <conditionalFormatting sqref="F25">
+    <cfRule type="cellIs" priority="36" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G25">
+    <cfRule type="cellIs" priority="37" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
+    <cfRule type="cellIs" priority="38" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I25">
+    <cfRule type="cellIs" priority="39" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q25">
+    <cfRule type="cellIs" priority="40" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M88">
-    <cfRule type="cellIs" priority="29" operator="notEqual" dxfId="3">
+  <conditionalFormatting sqref="F29">
+    <cfRule type="cellIs" priority="41" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G29">
+    <cfRule type="cellIs" priority="42" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H29">
+    <cfRule type="cellIs" priority="43" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I29">
+    <cfRule type="cellIs" priority="44" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q29">
+    <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F30">
+    <cfRule type="cellIs" priority="46" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30">
+    <cfRule type="cellIs" priority="47" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H30">
+    <cfRule type="cellIs" priority="48" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I30">
+    <cfRule type="cellIs" priority="49" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q30">
+    <cfRule type="cellIs" priority="50" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F31">
+    <cfRule type="cellIs" priority="51" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G31">
+    <cfRule type="cellIs" priority="52" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H31">
+    <cfRule type="cellIs" priority="53" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I31">
+    <cfRule type="cellIs" priority="54" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q31">
+    <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F35">
+    <cfRule type="cellIs" priority="56" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G35">
+    <cfRule type="cellIs" priority="57" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H35">
+    <cfRule type="cellIs" priority="58" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I35">
+    <cfRule type="cellIs" priority="59" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q35">
+    <cfRule type="cellIs" priority="60" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F36">
+    <cfRule type="cellIs" priority="61" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G36">
+    <cfRule type="cellIs" priority="62" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="cellIs" priority="63" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I36">
+    <cfRule type="cellIs" priority="64" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q36">
+    <cfRule type="cellIs" priority="65" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F37">
+    <cfRule type="cellIs" priority="66" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G37">
+    <cfRule type="cellIs" priority="67" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H37">
+    <cfRule type="cellIs" priority="68" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I37">
+    <cfRule type="cellIs" priority="69" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q37">
+    <cfRule type="cellIs" priority="70" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F38">
+    <cfRule type="cellIs" priority="71" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G38">
+    <cfRule type="cellIs" priority="72" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H38">
+    <cfRule type="cellIs" priority="73" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I38">
+    <cfRule type="cellIs" priority="74" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q38">
+    <cfRule type="cellIs" priority="75" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F39">
+    <cfRule type="cellIs" priority="76" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G39">
+    <cfRule type="cellIs" priority="77" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H39">
+    <cfRule type="cellIs" priority="78" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I39">
+    <cfRule type="cellIs" priority="79" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q39">
+    <cfRule type="cellIs" priority="80" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F43">
+    <cfRule type="cellIs" priority="81" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G43">
+    <cfRule type="cellIs" priority="82" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H43">
+    <cfRule type="cellIs" priority="83" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I43">
+    <cfRule type="cellIs" priority="84" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q43">
+    <cfRule type="cellIs" priority="85" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F44">
+    <cfRule type="cellIs" priority="86" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G44">
+    <cfRule type="cellIs" priority="87" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H44">
+    <cfRule type="cellIs" priority="88" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I44">
+    <cfRule type="cellIs" priority="89" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q44">
+    <cfRule type="cellIs" priority="90" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F45">
+    <cfRule type="cellIs" priority="91" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G45">
+    <cfRule type="cellIs" priority="92" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H45">
+    <cfRule type="cellIs" priority="93" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I45">
+    <cfRule type="cellIs" priority="94" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q45">
+    <cfRule type="cellIs" priority="95" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F49">
+    <cfRule type="cellIs" priority="96" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G49">
+    <cfRule type="cellIs" priority="97" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H49">
+    <cfRule type="cellIs" priority="98" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I49">
+    <cfRule type="cellIs" priority="99" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q49">
+    <cfRule type="cellIs" priority="100" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F50">
+    <cfRule type="cellIs" priority="101" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G50">
+    <cfRule type="cellIs" priority="102" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H50">
+    <cfRule type="cellIs" priority="103" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I50">
+    <cfRule type="cellIs" priority="104" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q50">
+    <cfRule type="cellIs" priority="105" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F51">
+    <cfRule type="cellIs" priority="106" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G51">
+    <cfRule type="cellIs" priority="107" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H51">
+    <cfRule type="cellIs" priority="108" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I51">
+    <cfRule type="cellIs" priority="109" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q51">
+    <cfRule type="cellIs" priority="110" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F52">
+    <cfRule type="cellIs" priority="111" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G52">
+    <cfRule type="cellIs" priority="112" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H52">
+    <cfRule type="cellIs" priority="113" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I52">
+    <cfRule type="cellIs" priority="114" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q52">
+    <cfRule type="cellIs" priority="115" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F53">
+    <cfRule type="cellIs" priority="116" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G53">
+    <cfRule type="cellIs" priority="117" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H53">
+    <cfRule type="cellIs" priority="118" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I53">
+    <cfRule type="cellIs" priority="119" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q53">
+    <cfRule type="cellIs" priority="120" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F54">
+    <cfRule type="cellIs" priority="121" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G54">
+    <cfRule type="cellIs" priority="122" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H54">
+    <cfRule type="cellIs" priority="123" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I54">
+    <cfRule type="cellIs" priority="124" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q54">
+    <cfRule type="cellIs" priority="125" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F55">
+    <cfRule type="cellIs" priority="126" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G55">
+    <cfRule type="cellIs" priority="127" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H55">
+    <cfRule type="cellIs" priority="128" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I55">
+    <cfRule type="cellIs" priority="129" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q55">
+    <cfRule type="cellIs" priority="130" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F56">
+    <cfRule type="cellIs" priority="131" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G56">
+    <cfRule type="cellIs" priority="132" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H56">
+    <cfRule type="cellIs" priority="133" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I56">
+    <cfRule type="cellIs" priority="134" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q56">
+    <cfRule type="cellIs" priority="135" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F57">
+    <cfRule type="cellIs" priority="136" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G57">
+    <cfRule type="cellIs" priority="137" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H57">
+    <cfRule type="cellIs" priority="138" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I57">
+    <cfRule type="cellIs" priority="139" operator="equal" dxfId="4">
+      <formula>"✓"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q57">
+    <cfRule type="cellIs" priority="140" operator="greaterThan" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E12">
+    <cfRule type="cellIs" priority="141" operator="notEqual" dxfId="3">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="11">
-    <dataValidation sqref="F4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"2,4,6,8"</formula1>
     </dataValidation>
     <dataValidation sqref="E7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -5809,10 +6362,10 @@
     <dataValidation sqref="E8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>'Master Data'!$A$74:$A$77</formula1>
     </dataValidation>
-    <dataValidation sqref="L7 L8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"First, Business, Premium Economy, Economy"</formula1>
     </dataValidation>
-    <dataValidation sqref="E15 E16 E17 E18 E19 E23 E24 E25 E29 E30 E31 E35 E36 E37 E38 E39 E43 E44 E45 E49 E50 E51 E52 E53 E54 E55 E56 E57 F15 F16 F17 F18 F19 F23 F24 F25 F29 F30 F31 F35 F36 F37 F38 F39 F43 F44 F45 F49 F50 F51 F52 F53 F54 F55 F56 F57 G15 G16 G17 G18 G19 G23 G24 G25 G29 G30 G31 G35 G36 G37 G38 G39 G43 G44 G45 G49 G50 G51 G52 G53 G54 G55 G56 G57 H15 H16 H17 H18 H19 H23 H24 H25 H29 H30 H31 H35 H36 H37 H38 H39 H43 H44 H45 H49 H50 H51 H52 H53 H54 H55 H56 H57 I15 I16 I17 I18 I19 I23 I24 I25 I29 I30 I31 I35 I36 I37 I38 I39 I43 I44 I45 I49 I50 I51 I52 I53 I54 I55 I56 I57 J15 J16 J17 J18 J19 J23 J24 J25 J29 J30 J31 J35 J36 J37 J38 J39 J43 J44 J45 J49 J50 J51 J52 J53 J54 J55 J56 J57 K15 K16 K17 K18 K19 K23 K24 K25 K29 K30 K31 K35 K36 K37 K38 K39 K43 K44 K45 K49 K50 K51 K52 K53 K54 K55 K56 K57 L15 L16 L17 L18 L19 L23 L24 L25 L29 L30 L31 L35 L36 L37 L38 L39 L43 L44 L45 L49 L50 L51 L52 L53 L54 L55 L56 L57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F15 F16 F17 F18 F19 F23 F24 F25 F29 F30 F31 F35 F36 F37 F38 F39 F43 F44 F45 F49 F50 F51 F52 F53 F54 F55 F56 F57 G15 G16 G17 G18 G19 G23 G24 G25 G29 G30 G31 G35 G36 G37 G38 G39 G43 G44 G45 G49 G50 G51 G52 G53 G54 G55 G56 G57 H15 H16 H17 H18 H19 H23 H24 H25 H29 H30 H31 H35 H36 H37 H38 H39 H43 H44 H45 H49 H50 H51 H52 H53 H54 H55 H56 H57 I15 I16 I17 I18 I19 I23 I24 I25 I29 I30 I31 I35 I36 I37 I38 I39 I43 I44 I45 I49 I50 I51 I52 I53 I54 I55 I56 I57 M15 M16 M17 M18 M19 M23 M24 M25 M29 M30 M31 M35 M36 M37 M38 M39 M43 M44 M45 M49 M50 M51 M52 M53 M54 M55 M56 M57 N15 N16 N17 N18 N19 N23 N24 N25 N29 N30 N31 N35 N36 N37 N38 N39 N43 N44 N45 N49 N50 N51 N52 N53 N54 N55 N56 N57 O15 O16 O17 O18 O19 O23 O24 O25 O29 O30 O31 O35 O36 O37 O38 O39 O43 O44 O45 O49 O50 O51 O52 O53 O54 O55 O56 O57 P15 P16 P17 P18 P19 P23 P24 P25 P29 P30 P31 P35 P36 P37 P38 P39 P43 P44 P45 P49 P50 P51 P52 P53 P54 P55 P56 P57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"✓,"</formula1>
     </dataValidation>
     <dataValidation sqref="A15 A16 A17 A18 A19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -5847,18 +6400,18 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" style="42" min="1" max="1"/>
-    <col width="14" customWidth="1" style="42" min="2" max="2"/>
-    <col width="14" customWidth="1" style="42" min="3" max="3"/>
-    <col width="14" customWidth="1" style="42" min="4" max="4"/>
-    <col width="14" customWidth="1" style="42" min="5" max="5"/>
-    <col width="14" customWidth="1" style="42" min="6" max="6"/>
+    <col width="22" customWidth="1" style="42" min="1" max="1"/>
+    <col width="13" customWidth="1" style="42" min="2" max="2"/>
+    <col width="13" customWidth="1" style="42" min="3" max="3"/>
+    <col width="13" customWidth="1" style="42" min="4" max="4"/>
+    <col width="13" customWidth="1" style="42" min="5" max="5"/>
+    <col width="13" customWidth="1" style="42" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="103" t="inlineStr">
         <is>
-          <t>📊 PROFIT SUMMARY — Auto-Generated from Package Selector</t>
+          <t>📊 PROFIT SUMMARY</t>
         </is>
       </c>
       <c r="B1" s="104" t="n"/>
@@ -5868,7 +6421,7 @@
       <c r="F1" s="104" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="119" t="inlineStr">
+      <c r="A4" s="98" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
@@ -5906,11 +6459,11 @@
         </is>
       </c>
       <c r="B5" s="84">
-        <f>'Package Selector'!M20</f>
+        <f>'Package Selector'!K20</f>
         <v/>
       </c>
       <c r="C5" s="84">
-        <f>'Package Selector'!N20</f>
+        <f>'Package Selector'!L20</f>
         <v/>
       </c>
       <c r="D5" s="84">
@@ -5922,7 +6475,7 @@
         <v/>
       </c>
       <c r="F5" s="84">
-        <f>IF(F4&gt;0,B5/F4,0)</f>
+        <f>IF(E4&gt;0,B5/E4,0)</f>
         <v/>
       </c>
     </row>
@@ -5933,11 +6486,11 @@
         </is>
       </c>
       <c r="B6" s="84">
-        <f>'Package Selector'!M26</f>
+        <f>'Package Selector'!K26</f>
         <v/>
       </c>
       <c r="C6" s="84">
-        <f>'Package Selector'!N26</f>
+        <f>'Package Selector'!L26</f>
         <v/>
       </c>
       <c r="D6" s="84">
@@ -5949,7 +6502,7 @@
         <v/>
       </c>
       <c r="F6" s="84">
-        <f>IF(F4&gt;0,B6/F4,0)</f>
+        <f>IF(E4&gt;0,B6/E4,0)</f>
         <v/>
       </c>
     </row>
@@ -5960,11 +6513,11 @@
         </is>
       </c>
       <c r="B7" s="84">
-        <f>'Package Selector'!M32</f>
+        <f>'Package Selector'!K32</f>
         <v/>
       </c>
       <c r="C7" s="84">
-        <f>'Package Selector'!N32</f>
+        <f>'Package Selector'!L32</f>
         <v/>
       </c>
       <c r="D7" s="84">
@@ -5976,7 +6529,7 @@
         <v/>
       </c>
       <c r="F7" s="84">
-        <f>IF(F4&gt;0,B7/F4,0)</f>
+        <f>IF(E4&gt;0,B7/E4,0)</f>
         <v/>
       </c>
     </row>
@@ -5987,11 +6540,11 @@
         </is>
       </c>
       <c r="B8" s="84">
-        <f>'Package Selector'!M40</f>
+        <f>'Package Selector'!K40</f>
         <v/>
       </c>
       <c r="C8" s="84">
-        <f>'Package Selector'!N40</f>
+        <f>'Package Selector'!L40</f>
         <v/>
       </c>
       <c r="D8" s="84">
@@ -6003,7 +6556,7 @@
         <v/>
       </c>
       <c r="F8" s="84">
-        <f>IF(F4&gt;0,B8/F4,0)</f>
+        <f>IF(E4&gt;0,B8/E4,0)</f>
         <v/>
       </c>
     </row>
@@ -6014,11 +6567,11 @@
         </is>
       </c>
       <c r="B9" s="84">
-        <f>'Package Selector'!M46</f>
+        <f>'Package Selector'!K46</f>
         <v/>
       </c>
       <c r="C9" s="84">
-        <f>'Package Selector'!N46</f>
+        <f>'Package Selector'!L46</f>
         <v/>
       </c>
       <c r="D9" s="84">
@@ -6030,7 +6583,7 @@
         <v/>
       </c>
       <c r="F9" s="84">
-        <f>IF(F4&gt;0,B9/F4,0)</f>
+        <f>IF(E4&gt;0,B9/E4,0)</f>
         <v/>
       </c>
     </row>
@@ -6041,11 +6594,11 @@
         </is>
       </c>
       <c r="B10" s="84">
-        <f>'Package Selector'!M58</f>
+        <f>'Package Selector'!K58</f>
         <v/>
       </c>
       <c r="C10" s="84">
-        <f>'Package Selector'!N58</f>
+        <f>'Package Selector'!L58</f>
         <v/>
       </c>
       <c r="D10" s="84">
@@ -6057,7 +6610,7 @@
         <v/>
       </c>
       <c r="F10" s="84">
-        <f>IF(F4&gt;0,B10/F4,0)</f>
+        <f>IF(E4&gt;0,B10/E4,0)</f>
         <v/>
       </c>
     </row>
@@ -6084,7 +6637,7 @@
         <v/>
       </c>
       <c r="F11" s="88">
-        <f>IF(F4&gt;0,B11/F4,0)</f>
+        <f>IF(E4&gt;0,B11/E4,0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: name-input P1-P4, black-circle toggle, linked per-person names, freeze@row15
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -127,6 +127,12 @@
       <name val="Calibri"/>
       <color rgb="00888888"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A3450"/>
+      <sz val="16"/>
     </font>
   </fonts>
   <fills count="22">
@@ -251,7 +257,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -482,11 +488,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF1A3450"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF1A3450"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF1A3450"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF1A3450"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="143">
+  <cellXfs count="144">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -866,11 +886,14 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
     <dxf>
       <font>
         <b val="1"/>
@@ -927,6 +950,19 @@
         <patternFill patternType="solid">
           <fgColor rgb="FF92D050"/>
           <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="16"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF1A3450"/>
+          <bgColor rgb="FF1A3450"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3320,7 +3356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q76"/>
+  <dimension ref="A1:R77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="42" min="1" max="1"/>
@@ -3328,24 +3364,24 @@
     <col width="11" customWidth="1" style="42" min="3" max="3"/>
     <col width="11" customWidth="1" style="42" min="4" max="4"/>
     <col width="8" customWidth="1" style="42" min="5" max="5"/>
-    <col width="10" customWidth="1" style="42" min="6" max="6"/>
-    <col width="10" customWidth="1" style="42" min="7" max="7"/>
-    <col width="10" customWidth="1" style="42" min="8" max="8"/>
-    <col width="10" customWidth="1" style="42" min="9" max="9"/>
+    <col width="8" customWidth="1" style="42" min="6" max="6"/>
+    <col width="8" customWidth="1" style="42" min="7" max="7"/>
+    <col width="8" customWidth="1" style="42" min="8" max="8"/>
+    <col width="8" customWidth="1" style="42" min="9" max="9"/>
     <col width="5" customWidth="1" style="42" min="10" max="10"/>
     <col width="12" customWidth="1" style="42" min="11" max="11"/>
     <col width="12" customWidth="1" style="42" min="12" max="12"/>
-    <col hidden="1" width="10" customWidth="1" style="42" min="13" max="13"/>
-    <col hidden="1" width="10" customWidth="1" style="42" min="14" max="14"/>
-    <col hidden="1" width="10" customWidth="1" style="42" min="15" max="15"/>
-    <col hidden="1" width="10" customWidth="1" style="42" min="16" max="16"/>
-    <col hidden="1" width="13" customWidth="1" style="42" min="17" max="17"/>
+    <col hidden="1" width="8" customWidth="1" style="42" min="13" max="13"/>
+    <col hidden="1" width="8" customWidth="1" style="42" min="14" max="14"/>
+    <col hidden="1" width="8" customWidth="1" style="42" min="15" max="15"/>
+    <col hidden="1" width="8" customWidth="1" style="42" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" style="42" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="103" t="inlineStr">
         <is>
-          <t>🎯 PACKAGE SELECTOR — All-in-One Builder</t>
+          <t>🎯 PACKAGE SELECTOR — All-in-One</t>
         </is>
       </c>
       <c r="B1" s="104" t="n"/>
@@ -3363,7 +3399,7 @@
     <row r="2">
       <c r="A2" s="105" t="inlineStr">
         <is>
-          <t>항목 선택 → ✓ 체크 → 자동계산 | P1~P4 기본, +버튼으로 P5~P8 확장</t>
+          <t>● = toggle on/off | P1~P4 names editable | freeze @ row 13</t>
         </is>
       </c>
     </row>
@@ -3382,89 +3418,81 @@
       <c r="E4" s="138" t="n">
         <v>4</v>
       </c>
-      <c r="F4" s="108" t="inlineStr">
-        <is>
-          <t>persons</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="103" t="inlineStr">
-        <is>
-          <t>✈️ FLIGHT DETAILS (현지시간 기준)</t>
-        </is>
-      </c>
-      <c r="B6" s="104" t="n"/>
-      <c r="C6" s="104" t="n"/>
-      <c r="D6" s="104" t="n"/>
-      <c r="E6" s="104" t="n"/>
-      <c r="F6" s="104" t="n"/>
-      <c r="G6" s="104" t="n"/>
-      <c r="H6" s="104" t="n"/>
-      <c r="I6" s="104" t="n"/>
-      <c r="J6" s="104" t="n"/>
-      <c r="K6" s="104" t="n"/>
-      <c r="L6" s="104" t="n"/>
+      <c r="G4" s="106" t="inlineStr">
+        <is>
+          <t>P1:</t>
+        </is>
+      </c>
+      <c r="H4" s="106" t="inlineStr">
+        <is>
+          <t>P2:</t>
+        </is>
+      </c>
+      <c r="I4" s="106" t="inlineStr">
+        <is>
+          <t>P3:</t>
+        </is>
+      </c>
+      <c r="J4" s="106" t="inlineStr">
+        <is>
+          <t>P4:</t>
+        </is>
+      </c>
+      <c r="K4" s="129" t="inlineStr">
+        <is>
+          <t>Guest4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="106" t="inlineStr">
+        <is>
+          <t>Names:</t>
+        </is>
+      </c>
+      <c r="B5" s="129" t="inlineStr">
+        <is>
+          <t>Guest1</t>
+        </is>
+      </c>
+      <c r="C5" s="129" t="inlineStr">
+        <is>
+          <t>Guest2</t>
+        </is>
+      </c>
+      <c r="D5" s="129" t="inlineStr">
+        <is>
+          <t>Guest3</t>
+        </is>
+      </c>
+      <c r="E5" s="129" t="inlineStr">
+        <is>
+          <t>Guest4</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="140" t="inlineStr">
-        <is>
-          <t>Outbound:</t>
-        </is>
-      </c>
-      <c r="B7" s="126" t="inlineStr">
-        <is>
-          <t>Date:</t>
-        </is>
-      </c>
-      <c r="C7" s="82" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="D7" s="126" t="inlineStr">
-        <is>
-          <t>Flight#:</t>
-        </is>
-      </c>
-      <c r="E7" s="82" t="inlineStr">
-        <is>
-          <t>KE011</t>
-        </is>
-      </c>
-      <c r="F7" s="126" t="inlineStr">
-        <is>
-          <t>Dep:</t>
-        </is>
-      </c>
-      <c r="G7" s="122">
-        <f>IF(E7="","",VLOOKUP(E7,'Master Data'!$A$60:$D$63,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="H7" s="126" t="inlineStr">
-        <is>
-          <t>Arr:</t>
-        </is>
-      </c>
-      <c r="I7" s="122">
-        <f>IF(E7="","",VLOOKUP(E7,'Master Data'!$A$60:$D$63,4,FALSE))</f>
-        <v/>
-      </c>
-      <c r="J7" s="126" t="inlineStr">
-        <is>
-          <t>Seat:</t>
-        </is>
-      </c>
-      <c r="K7" s="82" t="inlineStr">
-        <is>
-          <t>Economy</t>
-        </is>
-      </c>
+      <c r="A7" s="103" t="inlineStr">
+        <is>
+          <t>✈️ FLIGHT DETAILS</t>
+        </is>
+      </c>
+      <c r="B7" s="104" t="n"/>
+      <c r="C7" s="104" t="n"/>
+      <c r="D7" s="104" t="n"/>
+      <c r="E7" s="104" t="n"/>
+      <c r="F7" s="104" t="n"/>
+      <c r="G7" s="104" t="n"/>
+      <c r="H7" s="104" t="n"/>
+      <c r="I7" s="104" t="n"/>
+      <c r="J7" s="104" t="n"/>
+      <c r="K7" s="104" t="n"/>
+      <c r="L7" s="104" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="140" t="inlineStr">
         <is>
-          <t>Return:</t>
+          <t>Out:</t>
         </is>
       </c>
       <c r="B8" s="126" t="inlineStr">
@@ -3474,272 +3502,276 @@
       </c>
       <c r="C8" s="82" t="inlineStr">
         <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="D8" s="126" t="inlineStr">
+        <is>
+          <t>Flight:</t>
+        </is>
+      </c>
+      <c r="E8" s="82" t="inlineStr">
+        <is>
+          <t>KE011</t>
+        </is>
+      </c>
+      <c r="F8" s="126" t="inlineStr">
+        <is>
+          <t>Dep:</t>
+        </is>
+      </c>
+      <c r="G8" s="122">
+        <f>IF(E8="","",VLOOKUP(E8,'Master Data'!$A$60:$D$63,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="H8" s="126" t="inlineStr">
+        <is>
+          <t>Arr:</t>
+        </is>
+      </c>
+      <c r="I8" s="122">
+        <f>IF(E8="","",VLOOKUP(E8,'Master Data'!$A$60:$D$63,4,FALSE))</f>
+        <v/>
+      </c>
+      <c r="J8" s="126" t="inlineStr">
+        <is>
+          <t>Seat:</t>
+        </is>
+      </c>
+      <c r="K8" s="82" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="140" t="inlineStr">
+        <is>
+          <t>Ret:</t>
+        </is>
+      </c>
+      <c r="B9" s="126" t="inlineStr">
+        <is>
+          <t>Date:</t>
+        </is>
+      </c>
+      <c r="C9" s="82" t="inlineStr">
+        <is>
           <t>2026-05-30</t>
         </is>
       </c>
-      <c r="D8" s="126" t="inlineStr">
-        <is>
-          <t>Flight#:</t>
-        </is>
-      </c>
-      <c r="E8" s="82" t="inlineStr">
+      <c r="D9" s="126" t="inlineStr">
+        <is>
+          <t>Flight:</t>
+        </is>
+      </c>
+      <c r="E9" s="82" t="inlineStr">
         <is>
           <t>KE018</t>
         </is>
       </c>
-      <c r="F8" s="126" t="inlineStr">
+      <c r="F9" s="126" t="inlineStr">
         <is>
           <t>Dep:</t>
         </is>
       </c>
-      <c r="G8" s="122">
-        <f>IF(E8="","",VLOOKUP(E8,'Master Data'!$A$74:$D$77,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="H8" s="126" t="inlineStr">
+      <c r="G9" s="122">
+        <f>IF(E9="","",VLOOKUP(E9,'Master Data'!$A$74:$D$77,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="H9" s="126" t="inlineStr">
         <is>
           <t>Arr:</t>
         </is>
       </c>
-      <c r="I8" s="122">
-        <f>IF(E8="","",VLOOKUP(E8,'Master Data'!$A$74:$D$77,4,FALSE))</f>
-        <v/>
-      </c>
-      <c r="J8" s="126" t="inlineStr">
+      <c r="I9" s="122">
+        <f>IF(E9="","",VLOOKUP(E9,'Master Data'!$A$74:$D$77,4,FALSE))</f>
+        <v/>
+      </c>
+      <c r="J9" s="126" t="inlineStr">
         <is>
           <t>Seat:</t>
         </is>
       </c>
-      <c r="K8" s="82" t="inlineStr">
+      <c r="K9" s="82" t="inlineStr">
         <is>
           <t>Economy</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="106" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="106" t="inlineStr">
         <is>
           <t>Duration:</t>
         </is>
       </c>
-      <c r="B9" s="122">
-        <f>IF(AND(C7&lt;&gt;"",C8&lt;&gt;""),C8-C7,"")</f>
-        <v/>
-      </c>
-      <c r="C9" s="108" t="inlineStr">
+      <c r="B10" s="122">
+        <f>IF(AND(C8&lt;&gt;"",C9&lt;&gt;""),C9-C8,"")</f>
+        <v/>
+      </c>
+      <c r="C10" s="108" t="inlineStr">
         <is>
           <t>nights</t>
         </is>
       </c>
-      <c r="D9" s="122">
-        <f>IF(B9&lt;&gt;"",B9+1,"")</f>
-        <v/>
-      </c>
-      <c r="E9" s="108" t="inlineStr">
+      <c r="D10" s="122">
+        <f>IF(B10&lt;&gt;"",B10+1,"")</f>
+        <v/>
+      </c>
+      <c r="E10" s="108" t="inlineStr">
         <is>
           <t>days</t>
         </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="134" t="inlineStr">
-        <is>
-          <t>⚠️ DUPLICATE CHECK</t>
-        </is>
-      </c>
-      <c r="B11" s="136">
-        <f>IF(SUM(Q:Q)&gt;0,"❌ "&amp;SUM(Q:Q)&amp;" duplicate(s) — check hidden Q column","✅ No duplicates")</f>
-        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="116" t="inlineStr">
         <is>
-          <t>Cross-Check:</t>
-        </is>
-      </c>
-      <c r="B12" s="133">
-        <f>K68</f>
-        <v/>
-      </c>
-      <c r="C12" s="81" t="inlineStr">
+          <t>Dup Check:</t>
+        </is>
+      </c>
+      <c r="B12" s="136">
+        <f>IF(SUM(R:R)&gt;0,"❌ "&amp;SUM(R:R)&amp;" dup(s)","✅ OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="116" t="inlineStr">
+        <is>
+          <t>X-Check:</t>
+        </is>
+      </c>
+      <c r="B13" s="133">
+        <f>K69</f>
+        <v/>
+      </c>
+      <c r="C13" s="81" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="D12" s="133">
-        <f>B76</f>
-        <v/>
-      </c>
-      <c r="E12" s="117">
-        <f>B12-D12</f>
-        <v/>
-      </c>
-      <c r="F12" s="118">
-        <f>IF(E12=0,"✅ MATCH","❌ MISMATCH")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="119" t="inlineStr">
+      <c r="D13" s="133">
+        <f>B77</f>
+        <v/>
+      </c>
+      <c r="E13" s="117">
+        <f>B13-D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="136">
+        <f>IF(E13=0,"✅ MATCH","❌ MISMATCH")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="119" t="inlineStr">
         <is>
           <t>Item (Select ▼)</t>
         </is>
       </c>
-      <c r="B13" s="98" t="inlineStr">
+      <c r="B14" s="98" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="C13" s="98" t="inlineStr">
+      <c r="C14" s="98" t="inlineStr">
         <is>
           <t>Cost/P</t>
         </is>
       </c>
-      <c r="D13" s="98" t="inlineStr">
+      <c r="D14" s="98" t="inlineStr">
         <is>
           <t>Sell/P</t>
         </is>
       </c>
-      <c r="E13" s="98" t="inlineStr">
+      <c r="E14" s="98" t="inlineStr">
         <is>
           <t>Margin%</t>
         </is>
       </c>
-      <c r="F13" s="98" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="G13" s="98" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="H13" s="98" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="I13" s="98" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="J13" s="141" t="inlineStr">
+      <c r="F14" s="98">
+        <f>B5</f>
+        <v/>
+      </c>
+      <c r="G14" s="98">
+        <f>C5</f>
+        <v/>
+      </c>
+      <c r="H14" s="98">
+        <f>D5</f>
+        <v/>
+      </c>
+      <c r="I14" s="98">
+        <f>E5</f>
+        <v/>
+      </c>
+      <c r="J14" s="141" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K13" s="98" t="inlineStr">
+      <c r="K14" s="98" t="inlineStr">
         <is>
           <t>Tot Cost</t>
         </is>
       </c>
-      <c r="L13" s="98" t="inlineStr">
+      <c r="L14" s="98" t="inlineStr">
         <is>
           <t>Tot Sell</t>
         </is>
       </c>
-      <c r="M13" s="98" t="inlineStr">
+      <c r="M14" s="98" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="N13" s="98" t="inlineStr">
+      <c r="N14" s="98" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
-      <c r="O13" s="98" t="inlineStr">
+      <c r="O14" s="98" t="inlineStr">
         <is>
           <t>P7</t>
         </is>
       </c>
-      <c r="P13" s="98" t="inlineStr">
+      <c r="P14" s="98" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
       </c>
-      <c r="Q13" s="98" t="inlineStr">
+      <c r="R14" s="98" t="inlineStr">
         <is>
           <t>Dup</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="128" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="128" t="inlineStr">
         <is>
           <t>⛳ GOLF</t>
         </is>
       </c>
-      <c r="B14" s="77" t="n"/>
-      <c r="C14" s="77" t="n"/>
-      <c r="D14" s="77" t="n"/>
-      <c r="E14" s="77" t="n"/>
-      <c r="F14" s="77" t="n"/>
-      <c r="G14" s="77" t="n"/>
-      <c r="H14" s="77" t="n"/>
-      <c r="I14" s="77" t="n"/>
-      <c r="J14" s="77" t="n"/>
-      <c r="K14" s="77" t="n"/>
-      <c r="L14" s="77" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="109" t="inlineStr">
+      <c r="B15" s="77" t="n"/>
+      <c r="C15" s="77" t="n"/>
+      <c r="D15" s="77" t="n"/>
+      <c r="E15" s="77" t="n"/>
+      <c r="F15" s="77" t="n"/>
+      <c r="G15" s="77" t="n"/>
+      <c r="H15" s="77" t="n"/>
+      <c r="I15" s="77" t="n"/>
+      <c r="J15" s="77" t="n"/>
+      <c r="K15" s="77" t="n"/>
+      <c r="L15" s="77" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="109" t="inlineStr">
         <is>
           <t>Hidden Valley GC</t>
         </is>
       </c>
-      <c r="B15" s="83" t="n">
+      <c r="B16" s="83" t="n">
         <v>1</v>
-      </c>
-      <c r="C15" s="84">
-        <f>IF(A15="","",VLOOKUP(A15,'Master Data'!$A$7:$C$14,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D15" s="84">
-        <f>IF(A15="","",VLOOKUP(A15,'Master Data'!$A$7:$C$14,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E15" s="137">
-        <f>IF(D15&gt;0,(D15-C15)/D15,0)</f>
-        <v/>
-      </c>
-      <c r="F15" s="81" t="inlineStr"/>
-      <c r="G15" s="81" t="inlineStr"/>
-      <c r="H15" s="81" t="inlineStr"/>
-      <c r="I15" s="81" t="inlineStr"/>
-      <c r="J15" s="142" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="K15" s="84">
-        <f>IF(A15="","",(COUNTIF(F15,"✓")+COUNTIF(G15,"✓")+COUNTIF(H15,"✓")+COUNTIF(I15,"✓")+COUNTIF(M15,"✓")+COUNTIF(N15,"✓")+COUNTIF(O15,"✓")+COUNTIF(P15,"✓"))*B15*C15)</f>
-        <v/>
-      </c>
-      <c r="L15" s="84">
-        <f>IF(A15="","",(COUNTIF(F15,"✓")+COUNTIF(G15,"✓")+COUNTIF(H15,"✓")+COUNTIF(I15,"✓")+COUNTIF(M15,"✓")+COUNTIF(N15,"✓")+COUNTIF(O15,"✓")+COUNTIF(P15,"✓"))*B15*D15)</f>
-        <v/>
-      </c>
-      <c r="M15" s="81" t="inlineStr"/>
-      <c r="N15" s="81" t="inlineStr"/>
-      <c r="O15" s="81" t="inlineStr"/>
-      <c r="P15" s="81" t="inlineStr"/>
-      <c r="Q15" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="108" t="inlineStr">
-        <is>
-          <t>Sandpiper GC</t>
-        </is>
-      </c>
-      <c r="B16" s="83" t="n">
-        <v>2</v>
       </c>
       <c r="C16" s="84">
         <f>IF(A16="","",VLOOKUP(A16,'Master Data'!$A$7:$C$14,2,FALSE))</f>
@@ -3753,36 +3785,36 @@
         <f>IF(D16&gt;0,(D16-C16)/D16,0)</f>
         <v/>
       </c>
-      <c r="F16" s="81" t="inlineStr"/>
-      <c r="G16" s="81" t="inlineStr"/>
-      <c r="H16" s="81" t="inlineStr"/>
-      <c r="I16" s="81" t="inlineStr"/>
+      <c r="F16" s="143" t="inlineStr"/>
+      <c r="G16" s="143" t="inlineStr"/>
+      <c r="H16" s="143" t="inlineStr"/>
+      <c r="I16" s="143" t="inlineStr"/>
       <c r="J16" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K16" s="84">
-        <f>IF(A16="","",(COUNTIF(F16,"✓")+COUNTIF(G16,"✓")+COUNTIF(H16,"✓")+COUNTIF(I16,"✓")+COUNTIF(M16,"✓")+COUNTIF(N16,"✓")+COUNTIF(O16,"✓")+COUNTIF(P16,"✓"))*B16*C16)</f>
+        <f>IF(A16="","",(COUNTIF(F16,"●")+COUNTIF(G16,"●")+COUNTIF(H16,"●")+COUNTIF(I16,"●")+COUNTIF(M16,"●")+COUNTIF(N16,"●")+COUNTIF(O16,"●")+COUNTIF(P16,"●"))*B16*C16)</f>
         <v/>
       </c>
       <c r="L16" s="84">
-        <f>IF(A16="","",(COUNTIF(F16,"✓")+COUNTIF(G16,"✓")+COUNTIF(H16,"✓")+COUNTIF(I16,"✓")+COUNTIF(M16,"✓")+COUNTIF(N16,"✓")+COUNTIF(O16,"✓")+COUNTIF(P16,"✓"))*B16*D16)</f>
-        <v/>
-      </c>
-      <c r="M16" s="81" t="inlineStr"/>
-      <c r="N16" s="81" t="inlineStr"/>
-      <c r="O16" s="81" t="inlineStr"/>
-      <c r="P16" s="81" t="inlineStr"/>
-      <c r="Q16" s="81">
-        <f>IF(A16="",0,COUNTIF(A$15:A15,A16))</f>
+        <f>IF(A16="","",(COUNTIF(F16,"●")+COUNTIF(G16,"●")+COUNTIF(H16,"●")+COUNTIF(I16,"●")+COUNTIF(M16,"●")+COUNTIF(N16,"●")+COUNTIF(O16,"●")+COUNTIF(P16,"●"))*B16*D16)</f>
+        <v/>
+      </c>
+      <c r="M16" s="143" t="inlineStr"/>
+      <c r="N16" s="143" t="inlineStr"/>
+      <c r="O16" s="143" t="inlineStr"/>
+      <c r="P16" s="143" t="inlineStr"/>
+      <c r="R16" s="81">
+        <f>0</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="109" t="inlineStr">
-        <is>
-          <t>Trump National LA</t>
+      <c r="A17" s="108" t="inlineStr">
+        <is>
+          <t>Sandpiper GC</t>
         </is>
       </c>
       <c r="B17" s="83" t="n">
@@ -3800,35 +3832,41 @@
         <f>IF(D17&gt;0,(D17-C17)/D17,0)</f>
         <v/>
       </c>
-      <c r="F17" s="81" t="inlineStr"/>
-      <c r="G17" s="81" t="inlineStr"/>
-      <c r="H17" s="81" t="inlineStr"/>
-      <c r="I17" s="81" t="inlineStr"/>
+      <c r="F17" s="143" t="inlineStr"/>
+      <c r="G17" s="143" t="inlineStr"/>
+      <c r="H17" s="143" t="inlineStr"/>
+      <c r="I17" s="143" t="inlineStr"/>
       <c r="J17" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K17" s="84">
-        <f>IF(A17="","",(COUNTIF(F17,"✓")+COUNTIF(G17,"✓")+COUNTIF(H17,"✓")+COUNTIF(I17,"✓")+COUNTIF(M17,"✓")+COUNTIF(N17,"✓")+COUNTIF(O17,"✓")+COUNTIF(P17,"✓"))*B17*C17)</f>
+        <f>IF(A17="","",(COUNTIF(F17,"●")+COUNTIF(G17,"●")+COUNTIF(H17,"●")+COUNTIF(I17,"●")+COUNTIF(M17,"●")+COUNTIF(N17,"●")+COUNTIF(O17,"●")+COUNTIF(P17,"●"))*B17*C17)</f>
         <v/>
       </c>
       <c r="L17" s="84">
-        <f>IF(A17="","",(COUNTIF(F17,"✓")+COUNTIF(G17,"✓")+COUNTIF(H17,"✓")+COUNTIF(I17,"✓")+COUNTIF(M17,"✓")+COUNTIF(N17,"✓")+COUNTIF(O17,"✓")+COUNTIF(P17,"✓"))*B17*D17)</f>
-        <v/>
-      </c>
-      <c r="M17" s="81" t="inlineStr"/>
-      <c r="N17" s="81" t="inlineStr"/>
-      <c r="O17" s="81" t="inlineStr"/>
-      <c r="P17" s="81" t="inlineStr"/>
-      <c r="Q17" s="81">
-        <f>IF(A17="",0,COUNTIF(A$15:A16,A17))</f>
+        <f>IF(A17="","",(COUNTIF(F17,"●")+COUNTIF(G17,"●")+COUNTIF(H17,"●")+COUNTIF(I17,"●")+COUNTIF(M17,"●")+COUNTIF(N17,"●")+COUNTIF(O17,"●")+COUNTIF(P17,"●"))*B17*D17)</f>
+        <v/>
+      </c>
+      <c r="M17" s="143" t="inlineStr"/>
+      <c r="N17" s="143" t="inlineStr"/>
+      <c r="O17" s="143" t="inlineStr"/>
+      <c r="P17" s="143" t="inlineStr"/>
+      <c r="R17" s="81">
+        <f>IF(A17="",0,COUNTIF(A$16:A16,A17))</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="129" t="inlineStr"/>
-      <c r="B18" s="83" t="inlineStr"/>
+      <c r="A18" s="109" t="inlineStr">
+        <is>
+          <t>Trump National LA</t>
+        </is>
+      </c>
+      <c r="B18" s="83" t="n">
+        <v>2</v>
+      </c>
       <c r="C18" s="84">
         <f>IF(A18="","",VLOOKUP(A18,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
@@ -3841,29 +3879,29 @@
         <f>IF(D18&gt;0,(D18-C18)/D18,0)</f>
         <v/>
       </c>
-      <c r="F18" s="81" t="inlineStr"/>
-      <c r="G18" s="81" t="inlineStr"/>
-      <c r="H18" s="81" t="inlineStr"/>
-      <c r="I18" s="81" t="inlineStr"/>
+      <c r="F18" s="143" t="inlineStr"/>
+      <c r="G18" s="143" t="inlineStr"/>
+      <c r="H18" s="143" t="inlineStr"/>
+      <c r="I18" s="143" t="inlineStr"/>
       <c r="J18" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K18" s="84">
-        <f>IF(A18="","",(COUNTIF(F18,"✓")+COUNTIF(G18,"✓")+COUNTIF(H18,"✓")+COUNTIF(I18,"✓")+COUNTIF(M18,"✓")+COUNTIF(N18,"✓")+COUNTIF(O18,"✓")+COUNTIF(P18,"✓"))*B18*C18)</f>
+        <f>IF(A18="","",(COUNTIF(F18,"●")+COUNTIF(G18,"●")+COUNTIF(H18,"●")+COUNTIF(I18,"●")+COUNTIF(M18,"●")+COUNTIF(N18,"●")+COUNTIF(O18,"●")+COUNTIF(P18,"●"))*B18*C18)</f>
         <v/>
       </c>
       <c r="L18" s="84">
-        <f>IF(A18="","",(COUNTIF(F18,"✓")+COUNTIF(G18,"✓")+COUNTIF(H18,"✓")+COUNTIF(I18,"✓")+COUNTIF(M18,"✓")+COUNTIF(N18,"✓")+COUNTIF(O18,"✓")+COUNTIF(P18,"✓"))*B18*D18)</f>
-        <v/>
-      </c>
-      <c r="M18" s="81" t="inlineStr"/>
-      <c r="N18" s="81" t="inlineStr"/>
-      <c r="O18" s="81" t="inlineStr"/>
-      <c r="P18" s="81" t="inlineStr"/>
-      <c r="Q18" s="81">
-        <f>IF(A18="",0,COUNTIF(A$15:A17,A18))</f>
+        <f>IF(A18="","",(COUNTIF(F18,"●")+COUNTIF(G18,"●")+COUNTIF(H18,"●")+COUNTIF(I18,"●")+COUNTIF(M18,"●")+COUNTIF(N18,"●")+COUNTIF(O18,"●")+COUNTIF(P18,"●"))*B18*D18)</f>
+        <v/>
+      </c>
+      <c r="M18" s="143" t="inlineStr"/>
+      <c r="N18" s="143" t="inlineStr"/>
+      <c r="O18" s="143" t="inlineStr"/>
+      <c r="P18" s="143" t="inlineStr"/>
+      <c r="R18" s="81">
+        <f>IF(A18="",0,COUNTIF(A$16:A17,A18))</f>
         <v/>
       </c>
     </row>
@@ -3882,152 +3920,152 @@
         <f>IF(D19&gt;0,(D19-C19)/D19,0)</f>
         <v/>
       </c>
-      <c r="F19" s="81" t="inlineStr"/>
-      <c r="G19" s="81" t="inlineStr"/>
-      <c r="H19" s="81" t="inlineStr"/>
-      <c r="I19" s="81" t="inlineStr"/>
+      <c r="F19" s="143" t="inlineStr"/>
+      <c r="G19" s="143" t="inlineStr"/>
+      <c r="H19" s="143" t="inlineStr"/>
+      <c r="I19" s="143" t="inlineStr"/>
       <c r="J19" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K19" s="84">
-        <f>IF(A19="","",(COUNTIF(F19,"✓")+COUNTIF(G19,"✓")+COUNTIF(H19,"✓")+COUNTIF(I19,"✓")+COUNTIF(M19,"✓")+COUNTIF(N19,"✓")+COUNTIF(O19,"✓")+COUNTIF(P19,"✓"))*B19*C19)</f>
+        <f>IF(A19="","",(COUNTIF(F19,"●")+COUNTIF(G19,"●")+COUNTIF(H19,"●")+COUNTIF(I19,"●")+COUNTIF(M19,"●")+COUNTIF(N19,"●")+COUNTIF(O19,"●")+COUNTIF(P19,"●"))*B19*C19)</f>
         <v/>
       </c>
       <c r="L19" s="84">
-        <f>IF(A19="","",(COUNTIF(F19,"✓")+COUNTIF(G19,"✓")+COUNTIF(H19,"✓")+COUNTIF(I19,"✓")+COUNTIF(M19,"✓")+COUNTIF(N19,"✓")+COUNTIF(O19,"✓")+COUNTIF(P19,"✓"))*B19*D19)</f>
-        <v/>
-      </c>
-      <c r="M19" s="81" t="inlineStr"/>
-      <c r="N19" s="81" t="inlineStr"/>
-      <c r="O19" s="81" t="inlineStr"/>
-      <c r="P19" s="81" t="inlineStr"/>
-      <c r="Q19" s="81">
-        <f>IF(A19="",0,COUNTIF(A$15:A18,A19))</f>
+        <f>IF(A19="","",(COUNTIF(F19,"●")+COUNTIF(G19,"●")+COUNTIF(H19,"●")+COUNTIF(I19,"●")+COUNTIF(M19,"●")+COUNTIF(N19,"●")+COUNTIF(O19,"●")+COUNTIF(P19,"●"))*B19*D19)</f>
+        <v/>
+      </c>
+      <c r="M19" s="143" t="inlineStr"/>
+      <c r="N19" s="143" t="inlineStr"/>
+      <c r="O19" s="143" t="inlineStr"/>
+      <c r="P19" s="143" t="inlineStr"/>
+      <c r="R19" s="81">
+        <f>IF(A19="",0,COUNTIF(A$16:A18,A19))</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="123" t="inlineStr">
+      <c r="A20" s="129" t="inlineStr"/>
+      <c r="B20" s="83" t="inlineStr"/>
+      <c r="C20" s="84">
+        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D20" s="84">
+        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E20" s="137">
+        <f>IF(D20&gt;0,(D20-C20)/D20,0)</f>
+        <v/>
+      </c>
+      <c r="F20" s="143" t="inlineStr"/>
+      <c r="G20" s="143" t="inlineStr"/>
+      <c r="H20" s="143" t="inlineStr"/>
+      <c r="I20" s="143" t="inlineStr"/>
+      <c r="J20" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K20" s="84">
+        <f>IF(A20="","",(COUNTIF(F20,"●")+COUNTIF(G20,"●")+COUNTIF(H20,"●")+COUNTIF(I20,"●")+COUNTIF(M20,"●")+COUNTIF(N20,"●")+COUNTIF(O20,"●")+COUNTIF(P20,"●"))*B20*C20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="84">
+        <f>IF(A20="","",(COUNTIF(F20,"●")+COUNTIF(G20,"●")+COUNTIF(H20,"●")+COUNTIF(I20,"●")+COUNTIF(M20,"●")+COUNTIF(N20,"●")+COUNTIF(O20,"●")+COUNTIF(P20,"●"))*B20*D20)</f>
+        <v/>
+      </c>
+      <c r="M20" s="143" t="inlineStr"/>
+      <c r="N20" s="143" t="inlineStr"/>
+      <c r="O20" s="143" t="inlineStr"/>
+      <c r="P20" s="143" t="inlineStr"/>
+      <c r="R20" s="81">
+        <f>IF(A20="",0,COUNTIF(A$16:A19,A20))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B20" s="114" t="inlineStr"/>
-      <c r="C20" s="114" t="inlineStr"/>
-      <c r="D20" s="114" t="inlineStr"/>
-      <c r="E20" s="114" t="inlineStr"/>
-      <c r="F20" s="130">
-        <f>SUMPRODUCT((F15:F19="✓")*1,B15:B19,C15:C19)</f>
-        <v/>
-      </c>
-      <c r="G20" s="130">
-        <f>SUMPRODUCT((G15:G19="✓")*1,B15:B19,C15:C19)</f>
-        <v/>
-      </c>
-      <c r="H20" s="130">
-        <f>SUMPRODUCT((H15:H19="✓")*1,B15:B19,C15:C19)</f>
-        <v/>
-      </c>
-      <c r="I20" s="130">
-        <f>SUMPRODUCT((I15:I19="✓")*1,B15:B19,C15:C19)</f>
-        <v/>
-      </c>
-      <c r="J20" s="114" t="inlineStr"/>
-      <c r="K20" s="88">
-        <f>SUM(K15:K19)</f>
-        <v/>
-      </c>
-      <c r="L20" s="88">
-        <f>SUM(L15:L19)</f>
-        <v/>
-      </c>
-      <c r="M20" s="130">
-        <f>SUMPRODUCT((M15:M19="✓")*1,B15:B19,C15:C19)</f>
-        <v/>
-      </c>
-      <c r="N20" s="130">
-        <f>SUMPRODUCT((N15:N19="✓")*1,B15:B19,C15:C19)</f>
-        <v/>
-      </c>
-      <c r="O20" s="130">
-        <f>SUMPRODUCT((O15:O19="✓")*1,B15:B19,C15:C19)</f>
-        <v/>
-      </c>
-      <c r="P20" s="130">
-        <f>SUMPRODUCT((P15:P19="✓")*1,B15:B19,C15:C19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="128" t="inlineStr">
+      <c r="B21" s="114" t="inlineStr"/>
+      <c r="C21" s="114" t="inlineStr"/>
+      <c r="D21" s="114" t="inlineStr"/>
+      <c r="E21" s="114" t="inlineStr"/>
+      <c r="F21" s="130">
+        <f>SUMPRODUCT((F16:F20="●")*1,B16:B20,C16:C20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="130">
+        <f>SUMPRODUCT((G16:G20="●")*1,B16:B20,C16:C20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="130">
+        <f>SUMPRODUCT((H16:H20="●")*1,B16:B20,C16:C20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="130">
+        <f>SUMPRODUCT((I16:I20="●")*1,B16:B20,C16:C20)</f>
+        <v/>
+      </c>
+      <c r="J21" s="114" t="inlineStr"/>
+      <c r="K21" s="88">
+        <f>SUM(K16:K20)</f>
+        <v/>
+      </c>
+      <c r="L21" s="88">
+        <f>SUM(L16:L20)</f>
+        <v/>
+      </c>
+      <c r="M21" s="130">
+        <f>SUMPRODUCT((M16:M20="●")*1,B16:B20,C16:C20)</f>
+        <v/>
+      </c>
+      <c r="N21" s="130">
+        <f>SUMPRODUCT((N16:N20="●")*1,B16:B20,C16:C20)</f>
+        <v/>
+      </c>
+      <c r="O21" s="130">
+        <f>SUMPRODUCT((O16:O20="●")*1,B16:B20,C16:C20)</f>
+        <v/>
+      </c>
+      <c r="P21" s="130">
+        <f>SUMPRODUCT((P16:P20="●")*1,B16:B20,C16:C20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="128" t="inlineStr">
         <is>
           <t>🏨 HOTEL</t>
         </is>
       </c>
-      <c r="B22" s="77" t="n"/>
-      <c r="C22" s="77" t="n"/>
-      <c r="D22" s="77" t="n"/>
-      <c r="E22" s="77" t="n"/>
-      <c r="F22" s="77" t="n"/>
-      <c r="G22" s="77" t="n"/>
-      <c r="H22" s="77" t="n"/>
-      <c r="I22" s="77" t="n"/>
-      <c r="J22" s="77" t="n"/>
-      <c r="K22" s="77" t="n"/>
-      <c r="L22" s="77" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="109" t="inlineStr">
+      <c r="B23" s="77" t="n"/>
+      <c r="C23" s="77" t="n"/>
+      <c r="D23" s="77" t="n"/>
+      <c r="E23" s="77" t="n"/>
+      <c r="F23" s="77" t="n"/>
+      <c r="G23" s="77" t="n"/>
+      <c r="H23" s="77" t="n"/>
+      <c r="I23" s="77" t="n"/>
+      <c r="J23" s="77" t="n"/>
+      <c r="K23" s="77" t="n"/>
+      <c r="L23" s="77" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="109" t="inlineStr">
         <is>
           <t>Beverly Wilshire (5★) / Same Tier</t>
         </is>
       </c>
-      <c r="B23" s="83" t="n">
+      <c r="B24" s="83" t="n">
         <v>3</v>
       </c>
-      <c r="C23" s="84">
-        <f>IF(A23="","",VLOOKUP(A23,'Master Data'!$A$19:$C$24,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D23" s="84">
-        <f>IF(A23="","",VLOOKUP(A23,'Master Data'!$A$19:$C$24,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E23" s="137">
-        <f>IF(D23&gt;0,(D23-C23)/D23,0)</f>
-        <v/>
-      </c>
-      <c r="F23" s="81" t="inlineStr"/>
-      <c r="G23" s="81" t="inlineStr"/>
-      <c r="H23" s="81" t="inlineStr"/>
-      <c r="I23" s="81" t="inlineStr"/>
-      <c r="J23" s="142" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="K23" s="84">
-        <f>IF(A23="","",(COUNTIF(F23,"✓")+COUNTIF(G23,"✓")+COUNTIF(H23,"✓")+COUNTIF(I23,"✓")+COUNTIF(M23,"✓")+COUNTIF(N23,"✓")+COUNTIF(O23,"✓")+COUNTIF(P23,"✓"))*B23*C23)</f>
-        <v/>
-      </c>
-      <c r="L23" s="84">
-        <f>IF(A23="","",(COUNTIF(F23,"✓")+COUNTIF(G23,"✓")+COUNTIF(H23,"✓")+COUNTIF(I23,"✓")+COUNTIF(M23,"✓")+COUNTIF(N23,"✓")+COUNTIF(O23,"✓")+COUNTIF(P23,"✓"))*B23*D23)</f>
-        <v/>
-      </c>
-      <c r="M23" s="81" t="inlineStr"/>
-      <c r="N23" s="81" t="inlineStr"/>
-      <c r="O23" s="81" t="inlineStr"/>
-      <c r="P23" s="81" t="inlineStr"/>
-      <c r="Q23" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="129" t="inlineStr"/>
-      <c r="B24" s="83" t="inlineStr"/>
       <c r="C24" s="84">
         <f>IF(A24="","",VLOOKUP(A24,'Master Data'!$A$19:$C$24,2,FALSE))</f>
         <v/>
@@ -4040,29 +4078,29 @@
         <f>IF(D24&gt;0,(D24-C24)/D24,0)</f>
         <v/>
       </c>
-      <c r="F24" s="81" t="inlineStr"/>
-      <c r="G24" s="81" t="inlineStr"/>
-      <c r="H24" s="81" t="inlineStr"/>
-      <c r="I24" s="81" t="inlineStr"/>
+      <c r="F24" s="143" t="inlineStr"/>
+      <c r="G24" s="143" t="inlineStr"/>
+      <c r="H24" s="143" t="inlineStr"/>
+      <c r="I24" s="143" t="inlineStr"/>
       <c r="J24" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K24" s="84">
-        <f>IF(A24="","",(COUNTIF(F24,"✓")+COUNTIF(G24,"✓")+COUNTIF(H24,"✓")+COUNTIF(I24,"✓")+COUNTIF(M24,"✓")+COUNTIF(N24,"✓")+COUNTIF(O24,"✓")+COUNTIF(P24,"✓"))*B24*C24)</f>
+        <f>IF(A24="","",(COUNTIF(F24,"●")+COUNTIF(G24,"●")+COUNTIF(H24,"●")+COUNTIF(I24,"●")+COUNTIF(M24,"●")+COUNTIF(N24,"●")+COUNTIF(O24,"●")+COUNTIF(P24,"●"))*B24*C24)</f>
         <v/>
       </c>
       <c r="L24" s="84">
-        <f>IF(A24="","",(COUNTIF(F24,"✓")+COUNTIF(G24,"✓")+COUNTIF(H24,"✓")+COUNTIF(I24,"✓")+COUNTIF(M24,"✓")+COUNTIF(N24,"✓")+COUNTIF(O24,"✓")+COUNTIF(P24,"✓"))*B24*D24)</f>
-        <v/>
-      </c>
-      <c r="M24" s="81" t="inlineStr"/>
-      <c r="N24" s="81" t="inlineStr"/>
-      <c r="O24" s="81" t="inlineStr"/>
-      <c r="P24" s="81" t="inlineStr"/>
-      <c r="Q24" s="81">
-        <f>IF(A24="",0,COUNTIF(A$23:A23,A24))</f>
+        <f>IF(A24="","",(COUNTIF(F24,"●")+COUNTIF(G24,"●")+COUNTIF(H24,"●")+COUNTIF(I24,"●")+COUNTIF(M24,"●")+COUNTIF(N24,"●")+COUNTIF(O24,"●")+COUNTIF(P24,"●"))*B24*D24)</f>
+        <v/>
+      </c>
+      <c r="M24" s="143" t="inlineStr"/>
+      <c r="N24" s="143" t="inlineStr"/>
+      <c r="O24" s="143" t="inlineStr"/>
+      <c r="P24" s="143" t="inlineStr"/>
+      <c r="R24" s="81">
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -4081,152 +4119,152 @@
         <f>IF(D25&gt;0,(D25-C25)/D25,0)</f>
         <v/>
       </c>
-      <c r="F25" s="81" t="inlineStr"/>
-      <c r="G25" s="81" t="inlineStr"/>
-      <c r="H25" s="81" t="inlineStr"/>
-      <c r="I25" s="81" t="inlineStr"/>
+      <c r="F25" s="143" t="inlineStr"/>
+      <c r="G25" s="143" t="inlineStr"/>
+      <c r="H25" s="143" t="inlineStr"/>
+      <c r="I25" s="143" t="inlineStr"/>
       <c r="J25" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K25" s="84">
-        <f>IF(A25="","",(COUNTIF(F25,"✓")+COUNTIF(G25,"✓")+COUNTIF(H25,"✓")+COUNTIF(I25,"✓")+COUNTIF(M25,"✓")+COUNTIF(N25,"✓")+COUNTIF(O25,"✓")+COUNTIF(P25,"✓"))*B25*C25)</f>
+        <f>IF(A25="","",(COUNTIF(F25,"●")+COUNTIF(G25,"●")+COUNTIF(H25,"●")+COUNTIF(I25,"●")+COUNTIF(M25,"●")+COUNTIF(N25,"●")+COUNTIF(O25,"●")+COUNTIF(P25,"●"))*B25*C25)</f>
         <v/>
       </c>
       <c r="L25" s="84">
-        <f>IF(A25="","",(COUNTIF(F25,"✓")+COUNTIF(G25,"✓")+COUNTIF(H25,"✓")+COUNTIF(I25,"✓")+COUNTIF(M25,"✓")+COUNTIF(N25,"✓")+COUNTIF(O25,"✓")+COUNTIF(P25,"✓"))*B25*D25)</f>
-        <v/>
-      </c>
-      <c r="M25" s="81" t="inlineStr"/>
-      <c r="N25" s="81" t="inlineStr"/>
-      <c r="O25" s="81" t="inlineStr"/>
-      <c r="P25" s="81" t="inlineStr"/>
-      <c r="Q25" s="81">
-        <f>IF(A25="",0,COUNTIF(A$23:A24,A25))</f>
+        <f>IF(A25="","",(COUNTIF(F25,"●")+COUNTIF(G25,"●")+COUNTIF(H25,"●")+COUNTIF(I25,"●")+COUNTIF(M25,"●")+COUNTIF(N25,"●")+COUNTIF(O25,"●")+COUNTIF(P25,"●"))*B25*D25)</f>
+        <v/>
+      </c>
+      <c r="M25" s="143" t="inlineStr"/>
+      <c r="N25" s="143" t="inlineStr"/>
+      <c r="O25" s="143" t="inlineStr"/>
+      <c r="P25" s="143" t="inlineStr"/>
+      <c r="R25" s="81">
+        <f>IF(A25="",0,COUNTIF(A$24:A24,A25))</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="123" t="inlineStr">
+      <c r="A26" s="129" t="inlineStr"/>
+      <c r="B26" s="83" t="inlineStr"/>
+      <c r="C26" s="84">
+        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D26" s="84">
+        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E26" s="137">
+        <f>IF(D26&gt;0,(D26-C26)/D26,0)</f>
+        <v/>
+      </c>
+      <c r="F26" s="143" t="inlineStr"/>
+      <c r="G26" s="143" t="inlineStr"/>
+      <c r="H26" s="143" t="inlineStr"/>
+      <c r="I26" s="143" t="inlineStr"/>
+      <c r="J26" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K26" s="84">
+        <f>IF(A26="","",(COUNTIF(F26,"●")+COUNTIF(G26,"●")+COUNTIF(H26,"●")+COUNTIF(I26,"●")+COUNTIF(M26,"●")+COUNTIF(N26,"●")+COUNTIF(O26,"●")+COUNTIF(P26,"●"))*B26*C26)</f>
+        <v/>
+      </c>
+      <c r="L26" s="84">
+        <f>IF(A26="","",(COUNTIF(F26,"●")+COUNTIF(G26,"●")+COUNTIF(H26,"●")+COUNTIF(I26,"●")+COUNTIF(M26,"●")+COUNTIF(N26,"●")+COUNTIF(O26,"●")+COUNTIF(P26,"●"))*B26*D26)</f>
+        <v/>
+      </c>
+      <c r="M26" s="143" t="inlineStr"/>
+      <c r="N26" s="143" t="inlineStr"/>
+      <c r="O26" s="143" t="inlineStr"/>
+      <c r="P26" s="143" t="inlineStr"/>
+      <c r="R26" s="81">
+        <f>IF(A26="",0,COUNTIF(A$24:A25,A26))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B26" s="114" t="inlineStr"/>
-      <c r="C26" s="114" t="inlineStr"/>
-      <c r="D26" s="114" t="inlineStr"/>
-      <c r="E26" s="114" t="inlineStr"/>
-      <c r="F26" s="130">
-        <f>SUMPRODUCT((F23:F25="✓")*1,B23:B25,C23:C25)</f>
-        <v/>
-      </c>
-      <c r="G26" s="130">
-        <f>SUMPRODUCT((G23:G25="✓")*1,B23:B25,C23:C25)</f>
-        <v/>
-      </c>
-      <c r="H26" s="130">
-        <f>SUMPRODUCT((H23:H25="✓")*1,B23:B25,C23:C25)</f>
-        <v/>
-      </c>
-      <c r="I26" s="130">
-        <f>SUMPRODUCT((I23:I25="✓")*1,B23:B25,C23:C25)</f>
-        <v/>
-      </c>
-      <c r="J26" s="114" t="inlineStr"/>
-      <c r="K26" s="88">
-        <f>SUM(K23:K25)</f>
-        <v/>
-      </c>
-      <c r="L26" s="88">
-        <f>SUM(L23:L25)</f>
-        <v/>
-      </c>
-      <c r="M26" s="130">
-        <f>SUMPRODUCT((M23:M25="✓")*1,B23:B25,C23:C25)</f>
-        <v/>
-      </c>
-      <c r="N26" s="130">
-        <f>SUMPRODUCT((N23:N25="✓")*1,B23:B25,C23:C25)</f>
-        <v/>
-      </c>
-      <c r="O26" s="130">
-        <f>SUMPRODUCT((O23:O25="✓")*1,B23:B25,C23:C25)</f>
-        <v/>
-      </c>
-      <c r="P26" s="130">
-        <f>SUMPRODUCT((P23:P25="✓")*1,B23:B25,C23:C25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="128" t="inlineStr">
+      <c r="B27" s="114" t="inlineStr"/>
+      <c r="C27" s="114" t="inlineStr"/>
+      <c r="D27" s="114" t="inlineStr"/>
+      <c r="E27" s="114" t="inlineStr"/>
+      <c r="F27" s="130">
+        <f>SUMPRODUCT((F24:F26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="G27" s="130">
+        <f>SUMPRODUCT((G24:G26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="H27" s="130">
+        <f>SUMPRODUCT((H24:H26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="I27" s="130">
+        <f>SUMPRODUCT((I24:I26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="J27" s="114" t="inlineStr"/>
+      <c r="K27" s="88">
+        <f>SUM(K24:K26)</f>
+        <v/>
+      </c>
+      <c r="L27" s="88">
+        <f>SUM(L24:L26)</f>
+        <v/>
+      </c>
+      <c r="M27" s="130">
+        <f>SUMPRODUCT((M24:M26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="N27" s="130">
+        <f>SUMPRODUCT((N24:N26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="O27" s="130">
+        <f>SUMPRODUCT((O24:O26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="P27" s="130">
+        <f>SUMPRODUCT((P24:P26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="128" t="inlineStr">
         <is>
           <t>🚐 TRANSPORT</t>
         </is>
       </c>
-      <c r="B28" s="77" t="n"/>
-      <c r="C28" s="77" t="n"/>
-      <c r="D28" s="77" t="n"/>
-      <c r="E28" s="77" t="n"/>
-      <c r="F28" s="77" t="n"/>
-      <c r="G28" s="77" t="n"/>
-      <c r="H28" s="77" t="n"/>
-      <c r="I28" s="77" t="n"/>
-      <c r="J28" s="77" t="n"/>
-      <c r="K28" s="77" t="n"/>
-      <c r="L28" s="77" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="109" t="inlineStr">
+      <c r="B29" s="77" t="n"/>
+      <c r="C29" s="77" t="n"/>
+      <c r="D29" s="77" t="n"/>
+      <c r="E29" s="77" t="n"/>
+      <c r="F29" s="77" t="n"/>
+      <c r="G29" s="77" t="n"/>
+      <c r="H29" s="77" t="n"/>
+      <c r="I29" s="77" t="n"/>
+      <c r="J29" s="77" t="n"/>
+      <c r="K29" s="77" t="n"/>
+      <c r="L29" s="77" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="109" t="inlineStr">
         <is>
           <t>Driver/Guide + Van (일당)</t>
         </is>
       </c>
-      <c r="B29" s="83" t="n">
+      <c r="B30" s="83" t="n">
         <v>3</v>
       </c>
-      <c r="C29" s="84">
-        <f>IF(A29="","",VLOOKUP(A29,'Master Data'!$A$28:$C$34,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D29" s="84">
-        <f>IF(A29="","",VLOOKUP(A29,'Master Data'!$A$28:$C$34,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E29" s="137">
-        <f>IF(D29&gt;0,(D29-C29)/D29,0)</f>
-        <v/>
-      </c>
-      <c r="F29" s="81" t="inlineStr"/>
-      <c r="G29" s="81" t="inlineStr"/>
-      <c r="H29" s="81" t="inlineStr"/>
-      <c r="I29" s="81" t="inlineStr"/>
-      <c r="J29" s="142" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="K29" s="84">
-        <f>IF(A29="","",(COUNTIF(F29,"✓")+COUNTIF(G29,"✓")+COUNTIF(H29,"✓")+COUNTIF(I29,"✓")+COUNTIF(M29,"✓")+COUNTIF(N29,"✓")+COUNTIF(O29,"✓")+COUNTIF(P29,"✓"))*B29*C29)</f>
-        <v/>
-      </c>
-      <c r="L29" s="84">
-        <f>IF(A29="","",(COUNTIF(F29,"✓")+COUNTIF(G29,"✓")+COUNTIF(H29,"✓")+COUNTIF(I29,"✓")+COUNTIF(M29,"✓")+COUNTIF(N29,"✓")+COUNTIF(O29,"✓")+COUNTIF(P29,"✓"))*B29*D29)</f>
-        <v/>
-      </c>
-      <c r="M29" s="81" t="inlineStr"/>
-      <c r="N29" s="81" t="inlineStr"/>
-      <c r="O29" s="81" t="inlineStr"/>
-      <c r="P29" s="81" t="inlineStr"/>
-      <c r="Q29" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="129" t="inlineStr"/>
-      <c r="B30" s="83" t="inlineStr"/>
       <c r="C30" s="84">
         <f>IF(A30="","",VLOOKUP(A30,'Master Data'!$A$28:$C$34,2,FALSE))</f>
         <v/>
@@ -4239,29 +4277,29 @@
         <f>IF(D30&gt;0,(D30-C30)/D30,0)</f>
         <v/>
       </c>
-      <c r="F30" s="81" t="inlineStr"/>
-      <c r="G30" s="81" t="inlineStr"/>
-      <c r="H30" s="81" t="inlineStr"/>
-      <c r="I30" s="81" t="inlineStr"/>
+      <c r="F30" s="143" t="inlineStr"/>
+      <c r="G30" s="143" t="inlineStr"/>
+      <c r="H30" s="143" t="inlineStr"/>
+      <c r="I30" s="143" t="inlineStr"/>
       <c r="J30" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K30" s="84">
-        <f>IF(A30="","",(COUNTIF(F30,"✓")+COUNTIF(G30,"✓")+COUNTIF(H30,"✓")+COUNTIF(I30,"✓")+COUNTIF(M30,"✓")+COUNTIF(N30,"✓")+COUNTIF(O30,"✓")+COUNTIF(P30,"✓"))*B30*C30)</f>
+        <f>IF(A30="","",(COUNTIF(F30,"●")+COUNTIF(G30,"●")+COUNTIF(H30,"●")+COUNTIF(I30,"●")+COUNTIF(M30,"●")+COUNTIF(N30,"●")+COUNTIF(O30,"●")+COUNTIF(P30,"●"))*B30*C30)</f>
         <v/>
       </c>
       <c r="L30" s="84">
-        <f>IF(A30="","",(COUNTIF(F30,"✓")+COUNTIF(G30,"✓")+COUNTIF(H30,"✓")+COUNTIF(I30,"✓")+COUNTIF(M30,"✓")+COUNTIF(N30,"✓")+COUNTIF(O30,"✓")+COUNTIF(P30,"✓"))*B30*D30)</f>
-        <v/>
-      </c>
-      <c r="M30" s="81" t="inlineStr"/>
-      <c r="N30" s="81" t="inlineStr"/>
-      <c r="O30" s="81" t="inlineStr"/>
-      <c r="P30" s="81" t="inlineStr"/>
-      <c r="Q30" s="81">
-        <f>IF(A30="",0,COUNTIF(A$29:A29,A30))</f>
+        <f>IF(A30="","",(COUNTIF(F30,"●")+COUNTIF(G30,"●")+COUNTIF(H30,"●")+COUNTIF(I30,"●")+COUNTIF(M30,"●")+COUNTIF(N30,"●")+COUNTIF(O30,"●")+COUNTIF(P30,"●"))*B30*D30)</f>
+        <v/>
+      </c>
+      <c r="M30" s="143" t="inlineStr"/>
+      <c r="N30" s="143" t="inlineStr"/>
+      <c r="O30" s="143" t="inlineStr"/>
+      <c r="P30" s="143" t="inlineStr"/>
+      <c r="R30" s="81">
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -4280,153 +4318,147 @@
         <f>IF(D31&gt;0,(D31-C31)/D31,0)</f>
         <v/>
       </c>
-      <c r="F31" s="81" t="inlineStr"/>
-      <c r="G31" s="81" t="inlineStr"/>
-      <c r="H31" s="81" t="inlineStr"/>
-      <c r="I31" s="81" t="inlineStr"/>
+      <c r="F31" s="143" t="inlineStr"/>
+      <c r="G31" s="143" t="inlineStr"/>
+      <c r="H31" s="143" t="inlineStr"/>
+      <c r="I31" s="143" t="inlineStr"/>
       <c r="J31" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K31" s="84">
-        <f>IF(A31="","",(COUNTIF(F31,"✓")+COUNTIF(G31,"✓")+COUNTIF(H31,"✓")+COUNTIF(I31,"✓")+COUNTIF(M31,"✓")+COUNTIF(N31,"✓")+COUNTIF(O31,"✓")+COUNTIF(P31,"✓"))*B31*C31)</f>
+        <f>IF(A31="","",(COUNTIF(F31,"●")+COUNTIF(G31,"●")+COUNTIF(H31,"●")+COUNTIF(I31,"●")+COUNTIF(M31,"●")+COUNTIF(N31,"●")+COUNTIF(O31,"●")+COUNTIF(P31,"●"))*B31*C31)</f>
         <v/>
       </c>
       <c r="L31" s="84">
-        <f>IF(A31="","",(COUNTIF(F31,"✓")+COUNTIF(G31,"✓")+COUNTIF(H31,"✓")+COUNTIF(I31,"✓")+COUNTIF(M31,"✓")+COUNTIF(N31,"✓")+COUNTIF(O31,"✓")+COUNTIF(P31,"✓"))*B31*D31)</f>
-        <v/>
-      </c>
-      <c r="M31" s="81" t="inlineStr"/>
-      <c r="N31" s="81" t="inlineStr"/>
-      <c r="O31" s="81" t="inlineStr"/>
-      <c r="P31" s="81" t="inlineStr"/>
-      <c r="Q31" s="81">
-        <f>IF(A31="",0,COUNTIF(A$29:A30,A31))</f>
+        <f>IF(A31="","",(COUNTIF(F31,"●")+COUNTIF(G31,"●")+COUNTIF(H31,"●")+COUNTIF(I31,"●")+COUNTIF(M31,"●")+COUNTIF(N31,"●")+COUNTIF(O31,"●")+COUNTIF(P31,"●"))*B31*D31)</f>
+        <v/>
+      </c>
+      <c r="M31" s="143" t="inlineStr"/>
+      <c r="N31" s="143" t="inlineStr"/>
+      <c r="O31" s="143" t="inlineStr"/>
+      <c r="P31" s="143" t="inlineStr"/>
+      <c r="R31" s="81">
+        <f>IF(A31="",0,COUNTIF(A$30:A30,A31))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="123" t="inlineStr">
+      <c r="A32" s="129" t="inlineStr"/>
+      <c r="B32" s="83" t="inlineStr"/>
+      <c r="C32" s="84">
+        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D32" s="84">
+        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E32" s="137">
+        <f>IF(D32&gt;0,(D32-C32)/D32,0)</f>
+        <v/>
+      </c>
+      <c r="F32" s="143" t="inlineStr"/>
+      <c r="G32" s="143" t="inlineStr"/>
+      <c r="H32" s="143" t="inlineStr"/>
+      <c r="I32" s="143" t="inlineStr"/>
+      <c r="J32" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K32" s="84">
+        <f>IF(A32="","",(COUNTIF(F32,"●")+COUNTIF(G32,"●")+COUNTIF(H32,"●")+COUNTIF(I32,"●")+COUNTIF(M32,"●")+COUNTIF(N32,"●")+COUNTIF(O32,"●")+COUNTIF(P32,"●"))*B32*C32)</f>
+        <v/>
+      </c>
+      <c r="L32" s="84">
+        <f>IF(A32="","",(COUNTIF(F32,"●")+COUNTIF(G32,"●")+COUNTIF(H32,"●")+COUNTIF(I32,"●")+COUNTIF(M32,"●")+COUNTIF(N32,"●")+COUNTIF(O32,"●")+COUNTIF(P32,"●"))*B32*D32)</f>
+        <v/>
+      </c>
+      <c r="M32" s="143" t="inlineStr"/>
+      <c r="N32" s="143" t="inlineStr"/>
+      <c r="O32" s="143" t="inlineStr"/>
+      <c r="P32" s="143" t="inlineStr"/>
+      <c r="R32" s="81">
+        <f>IF(A32="",0,COUNTIF(A$30:A31,A32))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B32" s="114" t="inlineStr"/>
-      <c r="C32" s="114" t="inlineStr"/>
-      <c r="D32" s="114" t="inlineStr"/>
-      <c r="E32" s="114" t="inlineStr"/>
-      <c r="F32" s="130">
-        <f>SUMPRODUCT((F29:F31="✓")*1,B29:B31,C29:C31)</f>
-        <v/>
-      </c>
-      <c r="G32" s="130">
-        <f>SUMPRODUCT((G29:G31="✓")*1,B29:B31,C29:C31)</f>
-        <v/>
-      </c>
-      <c r="H32" s="130">
-        <f>SUMPRODUCT((H29:H31="✓")*1,B29:B31,C29:C31)</f>
-        <v/>
-      </c>
-      <c r="I32" s="130">
-        <f>SUMPRODUCT((I29:I31="✓")*1,B29:B31,C29:C31)</f>
-        <v/>
-      </c>
-      <c r="J32" s="114" t="inlineStr"/>
-      <c r="K32" s="88">
-        <f>SUM(K29:K31)</f>
-        <v/>
-      </c>
-      <c r="L32" s="88">
-        <f>SUM(L29:L31)</f>
-        <v/>
-      </c>
-      <c r="M32" s="130">
-        <f>SUMPRODUCT((M29:M31="✓")*1,B29:B31,C29:C31)</f>
-        <v/>
-      </c>
-      <c r="N32" s="130">
-        <f>SUMPRODUCT((N29:N31="✓")*1,B29:B31,C29:C31)</f>
-        <v/>
-      </c>
-      <c r="O32" s="130">
-        <f>SUMPRODUCT((O29:O31="✓")*1,B29:B31,C29:C31)</f>
-        <v/>
-      </c>
-      <c r="P32" s="130">
-        <f>SUMPRODUCT((P29:P31="✓")*1,B29:B31,C29:C31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="128" t="inlineStr">
+      <c r="B33" s="114" t="inlineStr"/>
+      <c r="C33" s="114" t="inlineStr"/>
+      <c r="D33" s="114" t="inlineStr"/>
+      <c r="E33" s="114" t="inlineStr"/>
+      <c r="F33" s="130">
+        <f>SUMPRODUCT((F30:F32="●")*1,B30:B32,C30:C32)</f>
+        <v/>
+      </c>
+      <c r="G33" s="130">
+        <f>SUMPRODUCT((G30:G32="●")*1,B30:B32,C30:C32)</f>
+        <v/>
+      </c>
+      <c r="H33" s="130">
+        <f>SUMPRODUCT((H30:H32="●")*1,B30:B32,C30:C32)</f>
+        <v/>
+      </c>
+      <c r="I33" s="130">
+        <f>SUMPRODUCT((I30:I32="●")*1,B30:B32,C30:C32)</f>
+        <v/>
+      </c>
+      <c r="J33" s="114" t="inlineStr"/>
+      <c r="K33" s="88">
+        <f>SUM(K30:K32)</f>
+        <v/>
+      </c>
+      <c r="L33" s="88">
+        <f>SUM(L30:L32)</f>
+        <v/>
+      </c>
+      <c r="M33" s="130">
+        <f>SUMPRODUCT((M30:M32="●")*1,B30:B32,C30:C32)</f>
+        <v/>
+      </c>
+      <c r="N33" s="130">
+        <f>SUMPRODUCT((N30:N32="●")*1,B30:B32,C30:C32)</f>
+        <v/>
+      </c>
+      <c r="O33" s="130">
+        <f>SUMPRODUCT((O30:O32="●")*1,B30:B32,C30:C32)</f>
+        <v/>
+      </c>
+      <c r="P33" s="130">
+        <f>SUMPRODUCT((P30:P32="●")*1,B30:B32,C30:C32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="128" t="inlineStr">
         <is>
           <t>🍽️ MEALS</t>
         </is>
       </c>
-      <c r="B34" s="77" t="n"/>
-      <c r="C34" s="77" t="n"/>
-      <c r="D34" s="77" t="n"/>
-      <c r="E34" s="77" t="n"/>
-      <c r="F34" s="77" t="n"/>
-      <c r="G34" s="77" t="n"/>
-      <c r="H34" s="77" t="n"/>
-      <c r="I34" s="77" t="n"/>
-      <c r="J34" s="77" t="n"/>
-      <c r="K34" s="77" t="n"/>
-      <c r="L34" s="77" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="109" t="inlineStr">
+      <c r="B35" s="77" t="n"/>
+      <c r="C35" s="77" t="n"/>
+      <c r="D35" s="77" t="n"/>
+      <c r="E35" s="77" t="n"/>
+      <c r="F35" s="77" t="n"/>
+      <c r="G35" s="77" t="n"/>
+      <c r="H35" s="77" t="n"/>
+      <c r="I35" s="77" t="n"/>
+      <c r="J35" s="77" t="n"/>
+      <c r="K35" s="77" t="n"/>
+      <c r="L35" s="77" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="109" t="inlineStr">
         <is>
           <t>Breakfast (Hotel)</t>
-        </is>
-      </c>
-      <c r="B35" s="83" t="n">
-        <v>3</v>
-      </c>
-      <c r="C35" s="84">
-        <f>IF(A35="","",VLOOKUP(A35,'Master Data'!$A$38:$C$46,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D35" s="84">
-        <f>IF(A35="","",VLOOKUP(A35,'Master Data'!$A$38:$C$46,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E35" s="137">
-        <f>IF(D35&gt;0,(D35-C35)/D35,0)</f>
-        <v/>
-      </c>
-      <c r="F35" s="81" t="inlineStr"/>
-      <c r="G35" s="81" t="inlineStr"/>
-      <c r="H35" s="81" t="inlineStr"/>
-      <c r="I35" s="81" t="inlineStr"/>
-      <c r="J35" s="142" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="K35" s="84">
-        <f>IF(A35="","",(COUNTIF(F35,"✓")+COUNTIF(G35,"✓")+COUNTIF(H35,"✓")+COUNTIF(I35,"✓")+COUNTIF(M35,"✓")+COUNTIF(N35,"✓")+COUNTIF(O35,"✓")+COUNTIF(P35,"✓"))*B35*C35)</f>
-        <v/>
-      </c>
-      <c r="L35" s="84">
-        <f>IF(A35="","",(COUNTIF(F35,"✓")+COUNTIF(G35,"✓")+COUNTIF(H35,"✓")+COUNTIF(I35,"✓")+COUNTIF(M35,"✓")+COUNTIF(N35,"✓")+COUNTIF(O35,"✓")+COUNTIF(P35,"✓"))*B35*D35)</f>
-        <v/>
-      </c>
-      <c r="M35" s="81" t="inlineStr"/>
-      <c r="N35" s="81" t="inlineStr"/>
-      <c r="O35" s="81" t="inlineStr"/>
-      <c r="P35" s="81" t="inlineStr"/>
-      <c r="Q35" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="108" t="inlineStr">
-        <is>
-          <t>Dinner (Regular)</t>
         </is>
       </c>
       <c r="B36" s="83" t="n">
@@ -4444,40 +4476,40 @@
         <f>IF(D36&gt;0,(D36-C36)/D36,0)</f>
         <v/>
       </c>
-      <c r="F36" s="81" t="inlineStr"/>
-      <c r="G36" s="81" t="inlineStr"/>
-      <c r="H36" s="81" t="inlineStr"/>
-      <c r="I36" s="81" t="inlineStr"/>
+      <c r="F36" s="143" t="inlineStr"/>
+      <c r="G36" s="143" t="inlineStr"/>
+      <c r="H36" s="143" t="inlineStr"/>
+      <c r="I36" s="143" t="inlineStr"/>
       <c r="J36" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K36" s="84">
-        <f>IF(A36="","",(COUNTIF(F36,"✓")+COUNTIF(G36,"✓")+COUNTIF(H36,"✓")+COUNTIF(I36,"✓")+COUNTIF(M36,"✓")+COUNTIF(N36,"✓")+COUNTIF(O36,"✓")+COUNTIF(P36,"✓"))*B36*C36)</f>
+        <f>IF(A36="","",(COUNTIF(F36,"●")+COUNTIF(G36,"●")+COUNTIF(H36,"●")+COUNTIF(I36,"●")+COUNTIF(M36,"●")+COUNTIF(N36,"●")+COUNTIF(O36,"●")+COUNTIF(P36,"●"))*B36*C36)</f>
         <v/>
       </c>
       <c r="L36" s="84">
-        <f>IF(A36="","",(COUNTIF(F36,"✓")+COUNTIF(G36,"✓")+COUNTIF(H36,"✓")+COUNTIF(I36,"✓")+COUNTIF(M36,"✓")+COUNTIF(N36,"✓")+COUNTIF(O36,"✓")+COUNTIF(P36,"✓"))*B36*D36)</f>
-        <v/>
-      </c>
-      <c r="M36" s="81" t="inlineStr"/>
-      <c r="N36" s="81" t="inlineStr"/>
-      <c r="O36" s="81" t="inlineStr"/>
-      <c r="P36" s="81" t="inlineStr"/>
-      <c r="Q36" s="81">
-        <f>IF(A36="",0,COUNTIF(A$35:A35,A36))</f>
+        <f>IF(A36="","",(COUNTIF(F36,"●")+COUNTIF(G36,"●")+COUNTIF(H36,"●")+COUNTIF(I36,"●")+COUNTIF(M36,"●")+COUNTIF(N36,"●")+COUNTIF(O36,"●")+COUNTIF(P36,"●"))*B36*D36)</f>
+        <v/>
+      </c>
+      <c r="M36" s="143" t="inlineStr"/>
+      <c r="N36" s="143" t="inlineStr"/>
+      <c r="O36" s="143" t="inlineStr"/>
+      <c r="P36" s="143" t="inlineStr"/>
+      <c r="R36" s="81">
+        <f>0</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="109" t="inlineStr">
-        <is>
-          <t>Exclusive Dinner (Michelin/Fine)</t>
+      <c r="A37" s="108" t="inlineStr">
+        <is>
+          <t>Dinner (Regular)</t>
         </is>
       </c>
       <c r="B37" s="83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C37" s="84">
         <f>IF(A37="","",VLOOKUP(A37,'Master Data'!$A$38:$C$46,2,FALSE))</f>
@@ -4491,40 +4523,40 @@
         <f>IF(D37&gt;0,(D37-C37)/D37,0)</f>
         <v/>
       </c>
-      <c r="F37" s="81" t="inlineStr"/>
-      <c r="G37" s="81" t="inlineStr"/>
-      <c r="H37" s="81" t="inlineStr"/>
-      <c r="I37" s="81" t="inlineStr"/>
+      <c r="F37" s="143" t="inlineStr"/>
+      <c r="G37" s="143" t="inlineStr"/>
+      <c r="H37" s="143" t="inlineStr"/>
+      <c r="I37" s="143" t="inlineStr"/>
       <c r="J37" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K37" s="84">
-        <f>IF(A37="","",(COUNTIF(F37,"✓")+COUNTIF(G37,"✓")+COUNTIF(H37,"✓")+COUNTIF(I37,"✓")+COUNTIF(M37,"✓")+COUNTIF(N37,"✓")+COUNTIF(O37,"✓")+COUNTIF(P37,"✓"))*B37*C37)</f>
+        <f>IF(A37="","",(COUNTIF(F37,"●")+COUNTIF(G37,"●")+COUNTIF(H37,"●")+COUNTIF(I37,"●")+COUNTIF(M37,"●")+COUNTIF(N37,"●")+COUNTIF(O37,"●")+COUNTIF(P37,"●"))*B37*C37)</f>
         <v/>
       </c>
       <c r="L37" s="84">
-        <f>IF(A37="","",(COUNTIF(F37,"✓")+COUNTIF(G37,"✓")+COUNTIF(H37,"✓")+COUNTIF(I37,"✓")+COUNTIF(M37,"✓")+COUNTIF(N37,"✓")+COUNTIF(O37,"✓")+COUNTIF(P37,"✓"))*B37*D37)</f>
-        <v/>
-      </c>
-      <c r="M37" s="81" t="inlineStr"/>
-      <c r="N37" s="81" t="inlineStr"/>
-      <c r="O37" s="81" t="inlineStr"/>
-      <c r="P37" s="81" t="inlineStr"/>
-      <c r="Q37" s="81">
-        <f>IF(A37="",0,COUNTIF(A$35:A36,A37))</f>
+        <f>IF(A37="","",(COUNTIF(F37,"●")+COUNTIF(G37,"●")+COUNTIF(H37,"●")+COUNTIF(I37,"●")+COUNTIF(M37,"●")+COUNTIF(N37,"●")+COUNTIF(O37,"●")+COUNTIF(P37,"●"))*B37*D37)</f>
+        <v/>
+      </c>
+      <c r="M37" s="143" t="inlineStr"/>
+      <c r="N37" s="143" t="inlineStr"/>
+      <c r="O37" s="143" t="inlineStr"/>
+      <c r="P37" s="143" t="inlineStr"/>
+      <c r="R37" s="81">
+        <f>IF(A37="",0,COUNTIF(A$36:A36,A37))</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="108" t="inlineStr">
-        <is>
-          <t>Lunch</t>
+      <c r="A38" s="109" t="inlineStr">
+        <is>
+          <t>Exclusive Dinner (Michelin/Fine)</t>
         </is>
       </c>
       <c r="B38" s="83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C38" s="84">
         <f>IF(A38="","",VLOOKUP(A38,'Master Data'!$A$38:$C$46,2,FALSE))</f>
@@ -4538,35 +4570,41 @@
         <f>IF(D38&gt;0,(D38-C38)/D38,0)</f>
         <v/>
       </c>
-      <c r="F38" s="81" t="inlineStr"/>
-      <c r="G38" s="81" t="inlineStr"/>
-      <c r="H38" s="81" t="inlineStr"/>
-      <c r="I38" s="81" t="inlineStr"/>
+      <c r="F38" s="143" t="inlineStr"/>
+      <c r="G38" s="143" t="inlineStr"/>
+      <c r="H38" s="143" t="inlineStr"/>
+      <c r="I38" s="143" t="inlineStr"/>
       <c r="J38" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K38" s="84">
-        <f>IF(A38="","",(COUNTIF(F38,"✓")+COUNTIF(G38,"✓")+COUNTIF(H38,"✓")+COUNTIF(I38,"✓")+COUNTIF(M38,"✓")+COUNTIF(N38,"✓")+COUNTIF(O38,"✓")+COUNTIF(P38,"✓"))*B38*C38)</f>
+        <f>IF(A38="","",(COUNTIF(F38,"●")+COUNTIF(G38,"●")+COUNTIF(H38,"●")+COUNTIF(I38,"●")+COUNTIF(M38,"●")+COUNTIF(N38,"●")+COUNTIF(O38,"●")+COUNTIF(P38,"●"))*B38*C38)</f>
         <v/>
       </c>
       <c r="L38" s="84">
-        <f>IF(A38="","",(COUNTIF(F38,"✓")+COUNTIF(G38,"✓")+COUNTIF(H38,"✓")+COUNTIF(I38,"✓")+COUNTIF(M38,"✓")+COUNTIF(N38,"✓")+COUNTIF(O38,"✓")+COUNTIF(P38,"✓"))*B38*D38)</f>
-        <v/>
-      </c>
-      <c r="M38" s="81" t="inlineStr"/>
-      <c r="N38" s="81" t="inlineStr"/>
-      <c r="O38" s="81" t="inlineStr"/>
-      <c r="P38" s="81" t="inlineStr"/>
-      <c r="Q38" s="81">
-        <f>IF(A38="",0,COUNTIF(A$35:A37,A38))</f>
+        <f>IF(A38="","",(COUNTIF(F38,"●")+COUNTIF(G38,"●")+COUNTIF(H38,"●")+COUNTIF(I38,"●")+COUNTIF(M38,"●")+COUNTIF(N38,"●")+COUNTIF(O38,"●")+COUNTIF(P38,"●"))*B38*D38)</f>
+        <v/>
+      </c>
+      <c r="M38" s="143" t="inlineStr"/>
+      <c r="N38" s="143" t="inlineStr"/>
+      <c r="O38" s="143" t="inlineStr"/>
+      <c r="P38" s="143" t="inlineStr"/>
+      <c r="R38" s="81">
+        <f>IF(A38="",0,COUNTIF(A$36:A37,A38))</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="129" t="inlineStr"/>
-      <c r="B39" s="83" t="inlineStr"/>
+      <c r="A39" s="108" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="B39" s="83" t="n">
+        <v>3</v>
+      </c>
       <c r="C39" s="84">
         <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
@@ -4579,152 +4617,152 @@
         <f>IF(D39&gt;0,(D39-C39)/D39,0)</f>
         <v/>
       </c>
-      <c r="F39" s="81" t="inlineStr"/>
-      <c r="G39" s="81" t="inlineStr"/>
-      <c r="H39" s="81" t="inlineStr"/>
-      <c r="I39" s="81" t="inlineStr"/>
+      <c r="F39" s="143" t="inlineStr"/>
+      <c r="G39" s="143" t="inlineStr"/>
+      <c r="H39" s="143" t="inlineStr"/>
+      <c r="I39" s="143" t="inlineStr"/>
       <c r="J39" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K39" s="84">
-        <f>IF(A39="","",(COUNTIF(F39,"✓")+COUNTIF(G39,"✓")+COUNTIF(H39,"✓")+COUNTIF(I39,"✓")+COUNTIF(M39,"✓")+COUNTIF(N39,"✓")+COUNTIF(O39,"✓")+COUNTIF(P39,"✓"))*B39*C39)</f>
+        <f>IF(A39="","",(COUNTIF(F39,"●")+COUNTIF(G39,"●")+COUNTIF(H39,"●")+COUNTIF(I39,"●")+COUNTIF(M39,"●")+COUNTIF(N39,"●")+COUNTIF(O39,"●")+COUNTIF(P39,"●"))*B39*C39)</f>
         <v/>
       </c>
       <c r="L39" s="84">
-        <f>IF(A39="","",(COUNTIF(F39,"✓")+COUNTIF(G39,"✓")+COUNTIF(H39,"✓")+COUNTIF(I39,"✓")+COUNTIF(M39,"✓")+COUNTIF(N39,"✓")+COUNTIF(O39,"✓")+COUNTIF(P39,"✓"))*B39*D39)</f>
-        <v/>
-      </c>
-      <c r="M39" s="81" t="inlineStr"/>
-      <c r="N39" s="81" t="inlineStr"/>
-      <c r="O39" s="81" t="inlineStr"/>
-      <c r="P39" s="81" t="inlineStr"/>
-      <c r="Q39" s="81">
-        <f>IF(A39="",0,COUNTIF(A$35:A38,A39))</f>
+        <f>IF(A39="","",(COUNTIF(F39,"●")+COUNTIF(G39,"●")+COUNTIF(H39,"●")+COUNTIF(I39,"●")+COUNTIF(M39,"●")+COUNTIF(N39,"●")+COUNTIF(O39,"●")+COUNTIF(P39,"●"))*B39*D39)</f>
+        <v/>
+      </c>
+      <c r="M39" s="143" t="inlineStr"/>
+      <c r="N39" s="143" t="inlineStr"/>
+      <c r="O39" s="143" t="inlineStr"/>
+      <c r="P39" s="143" t="inlineStr"/>
+      <c r="R39" s="81">
+        <f>IF(A39="",0,COUNTIF(A$36:A38,A39))</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="123" t="inlineStr">
+      <c r="A40" s="129" t="inlineStr"/>
+      <c r="B40" s="83" t="inlineStr"/>
+      <c r="C40" s="84">
+        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D40" s="84">
+        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E40" s="137">
+        <f>IF(D40&gt;0,(D40-C40)/D40,0)</f>
+        <v/>
+      </c>
+      <c r="F40" s="143" t="inlineStr"/>
+      <c r="G40" s="143" t="inlineStr"/>
+      <c r="H40" s="143" t="inlineStr"/>
+      <c r="I40" s="143" t="inlineStr"/>
+      <c r="J40" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K40" s="84">
+        <f>IF(A40="","",(COUNTIF(F40,"●")+COUNTIF(G40,"●")+COUNTIF(H40,"●")+COUNTIF(I40,"●")+COUNTIF(M40,"●")+COUNTIF(N40,"●")+COUNTIF(O40,"●")+COUNTIF(P40,"●"))*B40*C40)</f>
+        <v/>
+      </c>
+      <c r="L40" s="84">
+        <f>IF(A40="","",(COUNTIF(F40,"●")+COUNTIF(G40,"●")+COUNTIF(H40,"●")+COUNTIF(I40,"●")+COUNTIF(M40,"●")+COUNTIF(N40,"●")+COUNTIF(O40,"●")+COUNTIF(P40,"●"))*B40*D40)</f>
+        <v/>
+      </c>
+      <c r="M40" s="143" t="inlineStr"/>
+      <c r="N40" s="143" t="inlineStr"/>
+      <c r="O40" s="143" t="inlineStr"/>
+      <c r="P40" s="143" t="inlineStr"/>
+      <c r="R40" s="81">
+        <f>IF(A40="",0,COUNTIF(A$36:A39,A40))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B40" s="114" t="inlineStr"/>
-      <c r="C40" s="114" t="inlineStr"/>
-      <c r="D40" s="114" t="inlineStr"/>
-      <c r="E40" s="114" t="inlineStr"/>
-      <c r="F40" s="130">
-        <f>SUMPRODUCT((F35:F39="✓")*1,B35:B39,C35:C39)</f>
-        <v/>
-      </c>
-      <c r="G40" s="130">
-        <f>SUMPRODUCT((G35:G39="✓")*1,B35:B39,C35:C39)</f>
-        <v/>
-      </c>
-      <c r="H40" s="130">
-        <f>SUMPRODUCT((H35:H39="✓")*1,B35:B39,C35:C39)</f>
-        <v/>
-      </c>
-      <c r="I40" s="130">
-        <f>SUMPRODUCT((I35:I39="✓")*1,B35:B39,C35:C39)</f>
-        <v/>
-      </c>
-      <c r="J40" s="114" t="inlineStr"/>
-      <c r="K40" s="88">
-        <f>SUM(K35:K39)</f>
-        <v/>
-      </c>
-      <c r="L40" s="88">
-        <f>SUM(L35:L39)</f>
-        <v/>
-      </c>
-      <c r="M40" s="130">
-        <f>SUMPRODUCT((M35:M39="✓")*1,B35:B39,C35:C39)</f>
-        <v/>
-      </c>
-      <c r="N40" s="130">
-        <f>SUMPRODUCT((N35:N39="✓")*1,B35:B39,C35:C39)</f>
-        <v/>
-      </c>
-      <c r="O40" s="130">
-        <f>SUMPRODUCT((O35:O39="✓")*1,B35:B39,C35:C39)</f>
-        <v/>
-      </c>
-      <c r="P40" s="130">
-        <f>SUMPRODUCT((P35:P39="✓")*1,B35:B39,C35:C39)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="128" t="inlineStr">
+      <c r="B41" s="114" t="inlineStr"/>
+      <c r="C41" s="114" t="inlineStr"/>
+      <c r="D41" s="114" t="inlineStr"/>
+      <c r="E41" s="114" t="inlineStr"/>
+      <c r="F41" s="130">
+        <f>SUMPRODUCT((F36:F40="●")*1,B36:B40,C36:C40)</f>
+        <v/>
+      </c>
+      <c r="G41" s="130">
+        <f>SUMPRODUCT((G36:G40="●")*1,B36:B40,C36:C40)</f>
+        <v/>
+      </c>
+      <c r="H41" s="130">
+        <f>SUMPRODUCT((H36:H40="●")*1,B36:B40,C36:C40)</f>
+        <v/>
+      </c>
+      <c r="I41" s="130">
+        <f>SUMPRODUCT((I36:I40="●")*1,B36:B40,C36:C40)</f>
+        <v/>
+      </c>
+      <c r="J41" s="114" t="inlineStr"/>
+      <c r="K41" s="88">
+        <f>SUM(K36:K40)</f>
+        <v/>
+      </c>
+      <c r="L41" s="88">
+        <f>SUM(L36:L40)</f>
+        <v/>
+      </c>
+      <c r="M41" s="130">
+        <f>SUMPRODUCT((M36:M40="●")*1,B36:B40,C36:C40)</f>
+        <v/>
+      </c>
+      <c r="N41" s="130">
+        <f>SUMPRODUCT((N36:N40="●")*1,B36:B40,C36:C40)</f>
+        <v/>
+      </c>
+      <c r="O41" s="130">
+        <f>SUMPRODUCT((O36:O40="●")*1,B36:B40,C36:C40)</f>
+        <v/>
+      </c>
+      <c r="P41" s="130">
+        <f>SUMPRODUCT((P36:P40="●")*1,B36:B40,C36:C40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="128" t="inlineStr">
         <is>
           <t>📦 OTHER</t>
         </is>
       </c>
-      <c r="B42" s="77" t="n"/>
-      <c r="C42" s="77" t="n"/>
-      <c r="D42" s="77" t="n"/>
-      <c r="E42" s="77" t="n"/>
-      <c r="F42" s="77" t="n"/>
-      <c r="G42" s="77" t="n"/>
-      <c r="H42" s="77" t="n"/>
-      <c r="I42" s="77" t="n"/>
-      <c r="J42" s="77" t="n"/>
-      <c r="K42" s="77" t="n"/>
-      <c r="L42" s="77" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="109" t="inlineStr">
+      <c r="B43" s="77" t="n"/>
+      <c r="C43" s="77" t="n"/>
+      <c r="D43" s="77" t="n"/>
+      <c r="E43" s="77" t="n"/>
+      <c r="F43" s="77" t="n"/>
+      <c r="G43" s="77" t="n"/>
+      <c r="H43" s="77" t="n"/>
+      <c r="I43" s="77" t="n"/>
+      <c r="J43" s="77" t="n"/>
+      <c r="K43" s="77" t="n"/>
+      <c r="L43" s="77" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="109" t="inlineStr">
         <is>
           <t>Insurance / Tips / Contingency</t>
         </is>
       </c>
-      <c r="B43" s="83" t="n">
+      <c r="B44" s="83" t="n">
         <v>4</v>
       </c>
-      <c r="C43" s="84">
-        <f>IF(A43="","",VLOOKUP(A43,'Master Data'!$A$50:$C$56,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D43" s="84">
-        <f>IF(A43="","",VLOOKUP(A43,'Master Data'!$A$50:$C$56,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E43" s="137">
-        <f>IF(D43&gt;0,(D43-C43)/D43,0)</f>
-        <v/>
-      </c>
-      <c r="F43" s="81" t="inlineStr"/>
-      <c r="G43" s="81" t="inlineStr"/>
-      <c r="H43" s="81" t="inlineStr"/>
-      <c r="I43" s="81" t="inlineStr"/>
-      <c r="J43" s="142" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="K43" s="84">
-        <f>IF(A43="","",(COUNTIF(F43,"✓")+COUNTIF(G43,"✓")+COUNTIF(H43,"✓")+COUNTIF(I43,"✓")+COUNTIF(M43,"✓")+COUNTIF(N43,"✓")+COUNTIF(O43,"✓")+COUNTIF(P43,"✓"))*B43*C43)</f>
-        <v/>
-      </c>
-      <c r="L43" s="84">
-        <f>IF(A43="","",(COUNTIF(F43,"✓")+COUNTIF(G43,"✓")+COUNTIF(H43,"✓")+COUNTIF(I43,"✓")+COUNTIF(M43,"✓")+COUNTIF(N43,"✓")+COUNTIF(O43,"✓")+COUNTIF(P43,"✓"))*B43*D43)</f>
-        <v/>
-      </c>
-      <c r="M43" s="81" t="inlineStr"/>
-      <c r="N43" s="81" t="inlineStr"/>
-      <c r="O43" s="81" t="inlineStr"/>
-      <c r="P43" s="81" t="inlineStr"/>
-      <c r="Q43" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="129" t="inlineStr"/>
-      <c r="B44" s="83" t="inlineStr"/>
       <c r="C44" s="84">
         <f>IF(A44="","",VLOOKUP(A44,'Master Data'!$A$50:$C$56,2,FALSE))</f>
         <v/>
@@ -4737,29 +4775,29 @@
         <f>IF(D44&gt;0,(D44-C44)/D44,0)</f>
         <v/>
       </c>
-      <c r="F44" s="81" t="inlineStr"/>
-      <c r="G44" s="81" t="inlineStr"/>
-      <c r="H44" s="81" t="inlineStr"/>
-      <c r="I44" s="81" t="inlineStr"/>
+      <c r="F44" s="143" t="inlineStr"/>
+      <c r="G44" s="143" t="inlineStr"/>
+      <c r="H44" s="143" t="inlineStr"/>
+      <c r="I44" s="143" t="inlineStr"/>
       <c r="J44" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K44" s="84">
-        <f>IF(A44="","",(COUNTIF(F44,"✓")+COUNTIF(G44,"✓")+COUNTIF(H44,"✓")+COUNTIF(I44,"✓")+COUNTIF(M44,"✓")+COUNTIF(N44,"✓")+COUNTIF(O44,"✓")+COUNTIF(P44,"✓"))*B44*C44)</f>
+        <f>IF(A44="","",(COUNTIF(F44,"●")+COUNTIF(G44,"●")+COUNTIF(H44,"●")+COUNTIF(I44,"●")+COUNTIF(M44,"●")+COUNTIF(N44,"●")+COUNTIF(O44,"●")+COUNTIF(P44,"●"))*B44*C44)</f>
         <v/>
       </c>
       <c r="L44" s="84">
-        <f>IF(A44="","",(COUNTIF(F44,"✓")+COUNTIF(G44,"✓")+COUNTIF(H44,"✓")+COUNTIF(I44,"✓")+COUNTIF(M44,"✓")+COUNTIF(N44,"✓")+COUNTIF(O44,"✓")+COUNTIF(P44,"✓"))*B44*D44)</f>
-        <v/>
-      </c>
-      <c r="M44" s="81" t="inlineStr"/>
-      <c r="N44" s="81" t="inlineStr"/>
-      <c r="O44" s="81" t="inlineStr"/>
-      <c r="P44" s="81" t="inlineStr"/>
-      <c r="Q44" s="81">
-        <f>IF(A44="",0,COUNTIF(A$43:A43,A44))</f>
+        <f>IF(A44="","",(COUNTIF(F44,"●")+COUNTIF(G44,"●")+COUNTIF(H44,"●")+COUNTIF(I44,"●")+COUNTIF(M44,"●")+COUNTIF(N44,"●")+COUNTIF(O44,"●")+COUNTIF(P44,"●"))*B44*D44)</f>
+        <v/>
+      </c>
+      <c r="M44" s="143" t="inlineStr"/>
+      <c r="N44" s="143" t="inlineStr"/>
+      <c r="O44" s="143" t="inlineStr"/>
+      <c r="P44" s="143" t="inlineStr"/>
+      <c r="R44" s="81">
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -4778,153 +4816,147 @@
         <f>IF(D45&gt;0,(D45-C45)/D45,0)</f>
         <v/>
       </c>
-      <c r="F45" s="81" t="inlineStr"/>
-      <c r="G45" s="81" t="inlineStr"/>
-      <c r="H45" s="81" t="inlineStr"/>
-      <c r="I45" s="81" t="inlineStr"/>
+      <c r="F45" s="143" t="inlineStr"/>
+      <c r="G45" s="143" t="inlineStr"/>
+      <c r="H45" s="143" t="inlineStr"/>
+      <c r="I45" s="143" t="inlineStr"/>
       <c r="J45" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K45" s="84">
-        <f>IF(A45="","",(COUNTIF(F45,"✓")+COUNTIF(G45,"✓")+COUNTIF(H45,"✓")+COUNTIF(I45,"✓")+COUNTIF(M45,"✓")+COUNTIF(N45,"✓")+COUNTIF(O45,"✓")+COUNTIF(P45,"✓"))*B45*C45)</f>
+        <f>IF(A45="","",(COUNTIF(F45,"●")+COUNTIF(G45,"●")+COUNTIF(H45,"●")+COUNTIF(I45,"●")+COUNTIF(M45,"●")+COUNTIF(N45,"●")+COUNTIF(O45,"●")+COUNTIF(P45,"●"))*B45*C45)</f>
         <v/>
       </c>
       <c r="L45" s="84">
-        <f>IF(A45="","",(COUNTIF(F45,"✓")+COUNTIF(G45,"✓")+COUNTIF(H45,"✓")+COUNTIF(I45,"✓")+COUNTIF(M45,"✓")+COUNTIF(N45,"✓")+COUNTIF(O45,"✓")+COUNTIF(P45,"✓"))*B45*D45)</f>
-        <v/>
-      </c>
-      <c r="M45" s="81" t="inlineStr"/>
-      <c r="N45" s="81" t="inlineStr"/>
-      <c r="O45" s="81" t="inlineStr"/>
-      <c r="P45" s="81" t="inlineStr"/>
-      <c r="Q45" s="81">
-        <f>IF(A45="",0,COUNTIF(A$43:A44,A45))</f>
+        <f>IF(A45="","",(COUNTIF(F45,"●")+COUNTIF(G45,"●")+COUNTIF(H45,"●")+COUNTIF(I45,"●")+COUNTIF(M45,"●")+COUNTIF(N45,"●")+COUNTIF(O45,"●")+COUNTIF(P45,"●"))*B45*D45)</f>
+        <v/>
+      </c>
+      <c r="M45" s="143" t="inlineStr"/>
+      <c r="N45" s="143" t="inlineStr"/>
+      <c r="O45" s="143" t="inlineStr"/>
+      <c r="P45" s="143" t="inlineStr"/>
+      <c r="R45" s="81">
+        <f>IF(A45="",0,COUNTIF(A$44:A44,A45))</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="123" t="inlineStr">
+      <c r="A46" s="129" t="inlineStr"/>
+      <c r="B46" s="83" t="inlineStr"/>
+      <c r="C46" s="84">
+        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D46" s="84">
+        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E46" s="137">
+        <f>IF(D46&gt;0,(D46-C46)/D46,0)</f>
+        <v/>
+      </c>
+      <c r="F46" s="143" t="inlineStr"/>
+      <c r="G46" s="143" t="inlineStr"/>
+      <c r="H46" s="143" t="inlineStr"/>
+      <c r="I46" s="143" t="inlineStr"/>
+      <c r="J46" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K46" s="84">
+        <f>IF(A46="","",(COUNTIF(F46,"●")+COUNTIF(G46,"●")+COUNTIF(H46,"●")+COUNTIF(I46,"●")+COUNTIF(M46,"●")+COUNTIF(N46,"●")+COUNTIF(O46,"●")+COUNTIF(P46,"●"))*B46*C46)</f>
+        <v/>
+      </c>
+      <c r="L46" s="84">
+        <f>IF(A46="","",(COUNTIF(F46,"●")+COUNTIF(G46,"●")+COUNTIF(H46,"●")+COUNTIF(I46,"●")+COUNTIF(M46,"●")+COUNTIF(N46,"●")+COUNTIF(O46,"●")+COUNTIF(P46,"●"))*B46*D46)</f>
+        <v/>
+      </c>
+      <c r="M46" s="143" t="inlineStr"/>
+      <c r="N46" s="143" t="inlineStr"/>
+      <c r="O46" s="143" t="inlineStr"/>
+      <c r="P46" s="143" t="inlineStr"/>
+      <c r="R46" s="81">
+        <f>IF(A46="",0,COUNTIF(A$44:A45,A46))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B46" s="114" t="inlineStr"/>
-      <c r="C46" s="114" t="inlineStr"/>
-      <c r="D46" s="114" t="inlineStr"/>
-      <c r="E46" s="114" t="inlineStr"/>
-      <c r="F46" s="130">
-        <f>SUMPRODUCT((F43:F45="✓")*1,B43:B45,C43:C45)</f>
-        <v/>
-      </c>
-      <c r="G46" s="130">
-        <f>SUMPRODUCT((G43:G45="✓")*1,B43:B45,C43:C45)</f>
-        <v/>
-      </c>
-      <c r="H46" s="130">
-        <f>SUMPRODUCT((H43:H45="✓")*1,B43:B45,C43:C45)</f>
-        <v/>
-      </c>
-      <c r="I46" s="130">
-        <f>SUMPRODUCT((I43:I45="✓")*1,B43:B45,C43:C45)</f>
-        <v/>
-      </c>
-      <c r="J46" s="114" t="inlineStr"/>
-      <c r="K46" s="88">
-        <f>SUM(K43:K45)</f>
-        <v/>
-      </c>
-      <c r="L46" s="88">
-        <f>SUM(L43:L45)</f>
-        <v/>
-      </c>
-      <c r="M46" s="130">
-        <f>SUMPRODUCT((M43:M45="✓")*1,B43:B45,C43:C45)</f>
-        <v/>
-      </c>
-      <c r="N46" s="130">
-        <f>SUMPRODUCT((N43:N45="✓")*1,B43:B45,C43:C45)</f>
-        <v/>
-      </c>
-      <c r="O46" s="130">
-        <f>SUMPRODUCT((O43:O45="✓")*1,B43:B45,C43:C45)</f>
-        <v/>
-      </c>
-      <c r="P46" s="130">
-        <f>SUMPRODUCT((P43:P45="✓")*1,B43:B45,C43:C45)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="128" t="inlineStr">
+      <c r="B47" s="114" t="inlineStr"/>
+      <c r="C47" s="114" t="inlineStr"/>
+      <c r="D47" s="114" t="inlineStr"/>
+      <c r="E47" s="114" t="inlineStr"/>
+      <c r="F47" s="130">
+        <f>SUMPRODUCT((F44:F46="●")*1,B44:B46,C44:C46)</f>
+        <v/>
+      </c>
+      <c r="G47" s="130">
+        <f>SUMPRODUCT((G44:G46="●")*1,B44:B46,C44:C46)</f>
+        <v/>
+      </c>
+      <c r="H47" s="130">
+        <f>SUMPRODUCT((H44:H46="●")*1,B44:B46,C44:C46)</f>
+        <v/>
+      </c>
+      <c r="I47" s="130">
+        <f>SUMPRODUCT((I44:I46="●")*1,B44:B46,C44:C46)</f>
+        <v/>
+      </c>
+      <c r="J47" s="114" t="inlineStr"/>
+      <c r="K47" s="88">
+        <f>SUM(K44:K46)</f>
+        <v/>
+      </c>
+      <c r="L47" s="88">
+        <f>SUM(L44:L46)</f>
+        <v/>
+      </c>
+      <c r="M47" s="130">
+        <f>SUMPRODUCT((M44:M46="●")*1,B44:B46,C44:C46)</f>
+        <v/>
+      </c>
+      <c r="N47" s="130">
+        <f>SUMPRODUCT((N44:N46="●")*1,B44:B46,C44:C46)</f>
+        <v/>
+      </c>
+      <c r="O47" s="130">
+        <f>SUMPRODUCT((O44:O46="●")*1,B44:B46,C44:C46)</f>
+        <v/>
+      </c>
+      <c r="P47" s="130">
+        <f>SUMPRODUCT((P44:P46="●")*1,B44:B46,C44:C46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="128" t="inlineStr">
         <is>
           <t>🎯 ACTIVITIES</t>
         </is>
       </c>
-      <c r="B48" s="77" t="n"/>
-      <c r="C48" s="77" t="n"/>
-      <c r="D48" s="77" t="n"/>
-      <c r="E48" s="77" t="n"/>
-      <c r="F48" s="77" t="n"/>
-      <c r="G48" s="77" t="n"/>
-      <c r="H48" s="77" t="n"/>
-      <c r="I48" s="77" t="n"/>
-      <c r="J48" s="77" t="n"/>
-      <c r="K48" s="77" t="n"/>
-      <c r="L48" s="77" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="109" t="inlineStr">
+      <c r="B49" s="77" t="n"/>
+      <c r="C49" s="77" t="n"/>
+      <c r="D49" s="77" t="n"/>
+      <c r="E49" s="77" t="n"/>
+      <c r="F49" s="77" t="n"/>
+      <c r="G49" s="77" t="n"/>
+      <c r="H49" s="77" t="n"/>
+      <c r="I49" s="77" t="n"/>
+      <c r="J49" s="77" t="n"/>
+      <c r="K49" s="77" t="n"/>
+      <c r="L49" s="77" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="109" t="inlineStr">
         <is>
           <t>Beach/Surf Lesson</t>
-        </is>
-      </c>
-      <c r="B49" s="83" t="n">
-        <v>1</v>
-      </c>
-      <c r="C49" s="84">
-        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D49" s="84">
-        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E49" s="137">
-        <f>IF(D49&gt;0,(D49-C49)/D49,0)</f>
-        <v/>
-      </c>
-      <c r="F49" s="81" t="inlineStr"/>
-      <c r="G49" s="81" t="inlineStr"/>
-      <c r="H49" s="81" t="inlineStr"/>
-      <c r="I49" s="81" t="inlineStr"/>
-      <c r="J49" s="142" t="inlineStr">
-        <is>
-          <t>+</t>
-        </is>
-      </c>
-      <c r="K49" s="84">
-        <f>IF(A49="","",(COUNTIF(F49,"✓")+COUNTIF(G49,"✓")+COUNTIF(H49,"✓")+COUNTIF(I49,"✓")+COUNTIF(M49,"✓")+COUNTIF(N49,"✓")+COUNTIF(O49,"✓")+COUNTIF(P49,"✓"))*B49*C49)</f>
-        <v/>
-      </c>
-      <c r="L49" s="84">
-        <f>IF(A49="","",(COUNTIF(F49,"✓")+COUNTIF(G49,"✓")+COUNTIF(H49,"✓")+COUNTIF(I49,"✓")+COUNTIF(M49,"✓")+COUNTIF(N49,"✓")+COUNTIF(O49,"✓")+COUNTIF(P49,"✓"))*B49*D49)</f>
-        <v/>
-      </c>
-      <c r="M49" s="81" t="inlineStr"/>
-      <c r="N49" s="81" t="inlineStr"/>
-      <c r="O49" s="81" t="inlineStr"/>
-      <c r="P49" s="81" t="inlineStr"/>
-      <c r="Q49" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="108" t="inlineStr">
-        <is>
-          <t>Local Hiking (Griffith/Runyon)</t>
         </is>
       </c>
       <c r="B50" s="83" t="n">
@@ -4942,36 +4974,36 @@
         <f>IF(D50&gt;0,(D50-C50)/D50,0)</f>
         <v/>
       </c>
-      <c r="F50" s="81" t="inlineStr"/>
-      <c r="G50" s="81" t="inlineStr"/>
-      <c r="H50" s="81" t="inlineStr"/>
-      <c r="I50" s="81" t="inlineStr"/>
+      <c r="F50" s="143" t="inlineStr"/>
+      <c r="G50" s="143" t="inlineStr"/>
+      <c r="H50" s="143" t="inlineStr"/>
+      <c r="I50" s="143" t="inlineStr"/>
       <c r="J50" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K50" s="84">
-        <f>IF(A50="","",(COUNTIF(F50,"✓")+COUNTIF(G50,"✓")+COUNTIF(H50,"✓")+COUNTIF(I50,"✓")+COUNTIF(M50,"✓")+COUNTIF(N50,"✓")+COUNTIF(O50,"✓")+COUNTIF(P50,"✓"))*B50*C50)</f>
+        <f>IF(A50="","",(COUNTIF(F50,"●")+COUNTIF(G50,"●")+COUNTIF(H50,"●")+COUNTIF(I50,"●")+COUNTIF(M50,"●")+COUNTIF(N50,"●")+COUNTIF(O50,"●")+COUNTIF(P50,"●"))*B50*C50)</f>
         <v/>
       </c>
       <c r="L50" s="84">
-        <f>IF(A50="","",(COUNTIF(F50,"✓")+COUNTIF(G50,"✓")+COUNTIF(H50,"✓")+COUNTIF(I50,"✓")+COUNTIF(M50,"✓")+COUNTIF(N50,"✓")+COUNTIF(O50,"✓")+COUNTIF(P50,"✓"))*B50*D50)</f>
-        <v/>
-      </c>
-      <c r="M50" s="81" t="inlineStr"/>
-      <c r="N50" s="81" t="inlineStr"/>
-      <c r="O50" s="81" t="inlineStr"/>
-      <c r="P50" s="81" t="inlineStr"/>
-      <c r="Q50" s="81">
-        <f>IF(A50="",0,COUNTIF(A$49:A49,A50))</f>
+        <f>IF(A50="","",(COUNTIF(F50,"●")+COUNTIF(G50,"●")+COUNTIF(H50,"●")+COUNTIF(I50,"●")+COUNTIF(M50,"●")+COUNTIF(N50,"●")+COUNTIF(O50,"●")+COUNTIF(P50,"●"))*B50*D50)</f>
+        <v/>
+      </c>
+      <c r="M50" s="143" t="inlineStr"/>
+      <c r="N50" s="143" t="inlineStr"/>
+      <c r="O50" s="143" t="inlineStr"/>
+      <c r="P50" s="143" t="inlineStr"/>
+      <c r="R50" s="81">
+        <f>0</f>
         <v/>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="109" t="inlineStr">
-        <is>
-          <t>NBA/MLB Game (Ticket)</t>
+      <c r="A51" s="108" t="inlineStr">
+        <is>
+          <t>Local Hiking (Griffith/Runyon)</t>
         </is>
       </c>
       <c r="B51" s="83" t="n">
@@ -4989,36 +5021,36 @@
         <f>IF(D51&gt;0,(D51-C51)/D51,0)</f>
         <v/>
       </c>
-      <c r="F51" s="81" t="inlineStr"/>
-      <c r="G51" s="81" t="inlineStr"/>
-      <c r="H51" s="81" t="inlineStr"/>
-      <c r="I51" s="81" t="inlineStr"/>
+      <c r="F51" s="143" t="inlineStr"/>
+      <c r="G51" s="143" t="inlineStr"/>
+      <c r="H51" s="143" t="inlineStr"/>
+      <c r="I51" s="143" t="inlineStr"/>
       <c r="J51" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K51" s="84">
-        <f>IF(A51="","",(COUNTIF(F51,"✓")+COUNTIF(G51,"✓")+COUNTIF(H51,"✓")+COUNTIF(I51,"✓")+COUNTIF(M51,"✓")+COUNTIF(N51,"✓")+COUNTIF(O51,"✓")+COUNTIF(P51,"✓"))*B51*C51)</f>
+        <f>IF(A51="","",(COUNTIF(F51,"●")+COUNTIF(G51,"●")+COUNTIF(H51,"●")+COUNTIF(I51,"●")+COUNTIF(M51,"●")+COUNTIF(N51,"●")+COUNTIF(O51,"●")+COUNTIF(P51,"●"))*B51*C51)</f>
         <v/>
       </c>
       <c r="L51" s="84">
-        <f>IF(A51="","",(COUNTIF(F51,"✓")+COUNTIF(G51,"✓")+COUNTIF(H51,"✓")+COUNTIF(I51,"✓")+COUNTIF(M51,"✓")+COUNTIF(N51,"✓")+COUNTIF(O51,"✓")+COUNTIF(P51,"✓"))*B51*D51)</f>
-        <v/>
-      </c>
-      <c r="M51" s="81" t="inlineStr"/>
-      <c r="N51" s="81" t="inlineStr"/>
-      <c r="O51" s="81" t="inlineStr"/>
-      <c r="P51" s="81" t="inlineStr"/>
-      <c r="Q51" s="81">
-        <f>IF(A51="",0,COUNTIF(A$49:A50,A51))</f>
+        <f>IF(A51="","",(COUNTIF(F51,"●")+COUNTIF(G51,"●")+COUNTIF(H51,"●")+COUNTIF(I51,"●")+COUNTIF(M51,"●")+COUNTIF(N51,"●")+COUNTIF(O51,"●")+COUNTIF(P51,"●"))*B51*D51)</f>
+        <v/>
+      </c>
+      <c r="M51" s="143" t="inlineStr"/>
+      <c r="N51" s="143" t="inlineStr"/>
+      <c r="O51" s="143" t="inlineStr"/>
+      <c r="P51" s="143" t="inlineStr"/>
+      <c r="R51" s="81">
+        <f>IF(A51="",0,COUNTIF(A$50:A50,A51))</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="108" t="inlineStr">
-        <is>
-          <t>Sports Bar Experience</t>
+      <c r="A52" s="109" t="inlineStr">
+        <is>
+          <t>NBA/MLB Game (Ticket)</t>
         </is>
       </c>
       <c r="B52" s="83" t="n">
@@ -5036,35 +5068,41 @@
         <f>IF(D52&gt;0,(D52-C52)/D52,0)</f>
         <v/>
       </c>
-      <c r="F52" s="81" t="inlineStr"/>
-      <c r="G52" s="81" t="inlineStr"/>
-      <c r="H52" s="81" t="inlineStr"/>
-      <c r="I52" s="81" t="inlineStr"/>
+      <c r="F52" s="143" t="inlineStr"/>
+      <c r="G52" s="143" t="inlineStr"/>
+      <c r="H52" s="143" t="inlineStr"/>
+      <c r="I52" s="143" t="inlineStr"/>
       <c r="J52" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K52" s="84">
-        <f>IF(A52="","",(COUNTIF(F52,"✓")+COUNTIF(G52,"✓")+COUNTIF(H52,"✓")+COUNTIF(I52,"✓")+COUNTIF(M52,"✓")+COUNTIF(N52,"✓")+COUNTIF(O52,"✓")+COUNTIF(P52,"✓"))*B52*C52)</f>
+        <f>IF(A52="","",(COUNTIF(F52,"●")+COUNTIF(G52,"●")+COUNTIF(H52,"●")+COUNTIF(I52,"●")+COUNTIF(M52,"●")+COUNTIF(N52,"●")+COUNTIF(O52,"●")+COUNTIF(P52,"●"))*B52*C52)</f>
         <v/>
       </c>
       <c r="L52" s="84">
-        <f>IF(A52="","",(COUNTIF(F52,"✓")+COUNTIF(G52,"✓")+COUNTIF(H52,"✓")+COUNTIF(I52,"✓")+COUNTIF(M52,"✓")+COUNTIF(N52,"✓")+COUNTIF(O52,"✓")+COUNTIF(P52,"✓"))*B52*D52)</f>
-        <v/>
-      </c>
-      <c r="M52" s="81" t="inlineStr"/>
-      <c r="N52" s="81" t="inlineStr"/>
-      <c r="O52" s="81" t="inlineStr"/>
-      <c r="P52" s="81" t="inlineStr"/>
-      <c r="Q52" s="81">
-        <f>IF(A52="",0,COUNTIF(A$49:A51,A52))</f>
+        <f>IF(A52="","",(COUNTIF(F52,"●")+COUNTIF(G52,"●")+COUNTIF(H52,"●")+COUNTIF(I52,"●")+COUNTIF(M52,"●")+COUNTIF(N52,"●")+COUNTIF(O52,"●")+COUNTIF(P52,"●"))*B52*D52)</f>
+        <v/>
+      </c>
+      <c r="M52" s="143" t="inlineStr"/>
+      <c r="N52" s="143" t="inlineStr"/>
+      <c r="O52" s="143" t="inlineStr"/>
+      <c r="P52" s="143" t="inlineStr"/>
+      <c r="R52" s="81">
+        <f>IF(A52="",0,COUNTIF(A$50:A51,A52))</f>
         <v/>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="129" t="inlineStr"/>
-      <c r="B53" s="83" t="inlineStr"/>
+      <c r="A53" s="108" t="inlineStr">
+        <is>
+          <t>Sports Bar Experience</t>
+        </is>
+      </c>
+      <c r="B53" s="83" t="n">
+        <v>1</v>
+      </c>
       <c r="C53" s="84">
         <f>IF(A53="","",VLOOKUP(A53,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
@@ -5077,29 +5115,29 @@
         <f>IF(D53&gt;0,(D53-C53)/D53,0)</f>
         <v/>
       </c>
-      <c r="F53" s="81" t="inlineStr"/>
-      <c r="G53" s="81" t="inlineStr"/>
-      <c r="H53" s="81" t="inlineStr"/>
-      <c r="I53" s="81" t="inlineStr"/>
+      <c r="F53" s="143" t="inlineStr"/>
+      <c r="G53" s="143" t="inlineStr"/>
+      <c r="H53" s="143" t="inlineStr"/>
+      <c r="I53" s="143" t="inlineStr"/>
       <c r="J53" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K53" s="84">
-        <f>IF(A53="","",(COUNTIF(F53,"✓")+COUNTIF(G53,"✓")+COUNTIF(H53,"✓")+COUNTIF(I53,"✓")+COUNTIF(M53,"✓")+COUNTIF(N53,"✓")+COUNTIF(O53,"✓")+COUNTIF(P53,"✓"))*B53*C53)</f>
+        <f>IF(A53="","",(COUNTIF(F53,"●")+COUNTIF(G53,"●")+COUNTIF(H53,"●")+COUNTIF(I53,"●")+COUNTIF(M53,"●")+COUNTIF(N53,"●")+COUNTIF(O53,"●")+COUNTIF(P53,"●"))*B53*C53)</f>
         <v/>
       </c>
       <c r="L53" s="84">
-        <f>IF(A53="","",(COUNTIF(F53,"✓")+COUNTIF(G53,"✓")+COUNTIF(H53,"✓")+COUNTIF(I53,"✓")+COUNTIF(M53,"✓")+COUNTIF(N53,"✓")+COUNTIF(O53,"✓")+COUNTIF(P53,"✓"))*B53*D53)</f>
-        <v/>
-      </c>
-      <c r="M53" s="81" t="inlineStr"/>
-      <c r="N53" s="81" t="inlineStr"/>
-      <c r="O53" s="81" t="inlineStr"/>
-      <c r="P53" s="81" t="inlineStr"/>
-      <c r="Q53" s="81">
-        <f>IF(A53="",0,COUNTIF(A$49:A52,A53))</f>
+        <f>IF(A53="","",(COUNTIF(F53,"●")+COUNTIF(G53,"●")+COUNTIF(H53,"●")+COUNTIF(I53,"●")+COUNTIF(M53,"●")+COUNTIF(N53,"●")+COUNTIF(O53,"●")+COUNTIF(P53,"●"))*B53*D53)</f>
+        <v/>
+      </c>
+      <c r="M53" s="143" t="inlineStr"/>
+      <c r="N53" s="143" t="inlineStr"/>
+      <c r="O53" s="143" t="inlineStr"/>
+      <c r="P53" s="143" t="inlineStr"/>
+      <c r="R53" s="81">
+        <f>IF(A53="",0,COUNTIF(A$50:A52,A53))</f>
         <v/>
       </c>
     </row>
@@ -5118,29 +5156,29 @@
         <f>IF(D54&gt;0,(D54-C54)/D54,0)</f>
         <v/>
       </c>
-      <c r="F54" s="81" t="inlineStr"/>
-      <c r="G54" s="81" t="inlineStr"/>
-      <c r="H54" s="81" t="inlineStr"/>
-      <c r="I54" s="81" t="inlineStr"/>
+      <c r="F54" s="143" t="inlineStr"/>
+      <c r="G54" s="143" t="inlineStr"/>
+      <c r="H54" s="143" t="inlineStr"/>
+      <c r="I54" s="143" t="inlineStr"/>
       <c r="J54" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K54" s="84">
-        <f>IF(A54="","",(COUNTIF(F54,"✓")+COUNTIF(G54,"✓")+COUNTIF(H54,"✓")+COUNTIF(I54,"✓")+COUNTIF(M54,"✓")+COUNTIF(N54,"✓")+COUNTIF(O54,"✓")+COUNTIF(P54,"✓"))*B54*C54)</f>
+        <f>IF(A54="","",(COUNTIF(F54,"●")+COUNTIF(G54,"●")+COUNTIF(H54,"●")+COUNTIF(I54,"●")+COUNTIF(M54,"●")+COUNTIF(N54,"●")+COUNTIF(O54,"●")+COUNTIF(P54,"●"))*B54*C54)</f>
         <v/>
       </c>
       <c r="L54" s="84">
-        <f>IF(A54="","",(COUNTIF(F54,"✓")+COUNTIF(G54,"✓")+COUNTIF(H54,"✓")+COUNTIF(I54,"✓")+COUNTIF(M54,"✓")+COUNTIF(N54,"✓")+COUNTIF(O54,"✓")+COUNTIF(P54,"✓"))*B54*D54)</f>
-        <v/>
-      </c>
-      <c r="M54" s="81" t="inlineStr"/>
-      <c r="N54" s="81" t="inlineStr"/>
-      <c r="O54" s="81" t="inlineStr"/>
-      <c r="P54" s="81" t="inlineStr"/>
-      <c r="Q54" s="81">
-        <f>IF(A54="",0,COUNTIF(A$49:A53,A54))</f>
+        <f>IF(A54="","",(COUNTIF(F54,"●")+COUNTIF(G54,"●")+COUNTIF(H54,"●")+COUNTIF(I54,"●")+COUNTIF(M54,"●")+COUNTIF(N54,"●")+COUNTIF(O54,"●")+COUNTIF(P54,"●"))*B54*D54)</f>
+        <v/>
+      </c>
+      <c r="M54" s="143" t="inlineStr"/>
+      <c r="N54" s="143" t="inlineStr"/>
+      <c r="O54" s="143" t="inlineStr"/>
+      <c r="P54" s="143" t="inlineStr"/>
+      <c r="R54" s="81">
+        <f>IF(A54="",0,COUNTIF(A$50:A53,A54))</f>
         <v/>
       </c>
     </row>
@@ -5159,29 +5197,29 @@
         <f>IF(D55&gt;0,(D55-C55)/D55,0)</f>
         <v/>
       </c>
-      <c r="F55" s="81" t="inlineStr"/>
-      <c r="G55" s="81" t="inlineStr"/>
-      <c r="H55" s="81" t="inlineStr"/>
-      <c r="I55" s="81" t="inlineStr"/>
+      <c r="F55" s="143" t="inlineStr"/>
+      <c r="G55" s="143" t="inlineStr"/>
+      <c r="H55" s="143" t="inlineStr"/>
+      <c r="I55" s="143" t="inlineStr"/>
       <c r="J55" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K55" s="84">
-        <f>IF(A55="","",(COUNTIF(F55,"✓")+COUNTIF(G55,"✓")+COUNTIF(H55,"✓")+COUNTIF(I55,"✓")+COUNTIF(M55,"✓")+COUNTIF(N55,"✓")+COUNTIF(O55,"✓")+COUNTIF(P55,"✓"))*B55*C55)</f>
+        <f>IF(A55="","",(COUNTIF(F55,"●")+COUNTIF(G55,"●")+COUNTIF(H55,"●")+COUNTIF(I55,"●")+COUNTIF(M55,"●")+COUNTIF(N55,"●")+COUNTIF(O55,"●")+COUNTIF(P55,"●"))*B55*C55)</f>
         <v/>
       </c>
       <c r="L55" s="84">
-        <f>IF(A55="","",(COUNTIF(F55,"✓")+COUNTIF(G55,"✓")+COUNTIF(H55,"✓")+COUNTIF(I55,"✓")+COUNTIF(M55,"✓")+COUNTIF(N55,"✓")+COUNTIF(O55,"✓")+COUNTIF(P55,"✓"))*B55*D55)</f>
-        <v/>
-      </c>
-      <c r="M55" s="81" t="inlineStr"/>
-      <c r="N55" s="81" t="inlineStr"/>
-      <c r="O55" s="81" t="inlineStr"/>
-      <c r="P55" s="81" t="inlineStr"/>
-      <c r="Q55" s="81">
-        <f>IF(A55="",0,COUNTIF(A$49:A54,A55))</f>
+        <f>IF(A55="","",(COUNTIF(F55,"●")+COUNTIF(G55,"●")+COUNTIF(H55,"●")+COUNTIF(I55,"●")+COUNTIF(M55,"●")+COUNTIF(N55,"●")+COUNTIF(O55,"●")+COUNTIF(P55,"●"))*B55*D55)</f>
+        <v/>
+      </c>
+      <c r="M55" s="143" t="inlineStr"/>
+      <c r="N55" s="143" t="inlineStr"/>
+      <c r="O55" s="143" t="inlineStr"/>
+      <c r="P55" s="143" t="inlineStr"/>
+      <c r="R55" s="81">
+        <f>IF(A55="",0,COUNTIF(A$50:A54,A55))</f>
         <v/>
       </c>
     </row>
@@ -5200,29 +5238,29 @@
         <f>IF(D56&gt;0,(D56-C56)/D56,0)</f>
         <v/>
       </c>
-      <c r="F56" s="81" t="inlineStr"/>
-      <c r="G56" s="81" t="inlineStr"/>
-      <c r="H56" s="81" t="inlineStr"/>
-      <c r="I56" s="81" t="inlineStr"/>
+      <c r="F56" s="143" t="inlineStr"/>
+      <c r="G56" s="143" t="inlineStr"/>
+      <c r="H56" s="143" t="inlineStr"/>
+      <c r="I56" s="143" t="inlineStr"/>
       <c r="J56" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K56" s="84">
-        <f>IF(A56="","",(COUNTIF(F56,"✓")+COUNTIF(G56,"✓")+COUNTIF(H56,"✓")+COUNTIF(I56,"✓")+COUNTIF(M56,"✓")+COUNTIF(N56,"✓")+COUNTIF(O56,"✓")+COUNTIF(P56,"✓"))*B56*C56)</f>
+        <f>IF(A56="","",(COUNTIF(F56,"●")+COUNTIF(G56,"●")+COUNTIF(H56,"●")+COUNTIF(I56,"●")+COUNTIF(M56,"●")+COUNTIF(N56,"●")+COUNTIF(O56,"●")+COUNTIF(P56,"●"))*B56*C56)</f>
         <v/>
       </c>
       <c r="L56" s="84">
-        <f>IF(A56="","",(COUNTIF(F56,"✓")+COUNTIF(G56,"✓")+COUNTIF(H56,"✓")+COUNTIF(I56,"✓")+COUNTIF(M56,"✓")+COUNTIF(N56,"✓")+COUNTIF(O56,"✓")+COUNTIF(P56,"✓"))*B56*D56)</f>
-        <v/>
-      </c>
-      <c r="M56" s="81" t="inlineStr"/>
-      <c r="N56" s="81" t="inlineStr"/>
-      <c r="O56" s="81" t="inlineStr"/>
-      <c r="P56" s="81" t="inlineStr"/>
-      <c r="Q56" s="81">
-        <f>IF(A56="",0,COUNTIF(A$49:A55,A56))</f>
+        <f>IF(A56="","",(COUNTIF(F56,"●")+COUNTIF(G56,"●")+COUNTIF(H56,"●")+COUNTIF(I56,"●")+COUNTIF(M56,"●")+COUNTIF(N56,"●")+COUNTIF(O56,"●")+COUNTIF(P56,"●"))*B56*D56)</f>
+        <v/>
+      </c>
+      <c r="M56" s="143" t="inlineStr"/>
+      <c r="N56" s="143" t="inlineStr"/>
+      <c r="O56" s="143" t="inlineStr"/>
+      <c r="P56" s="143" t="inlineStr"/>
+      <c r="R56" s="81">
+        <f>IF(A56="",0,COUNTIF(A$50:A55,A56))</f>
         <v/>
       </c>
     </row>
@@ -5241,305 +5279,318 @@
         <f>IF(D57&gt;0,(D57-C57)/D57,0)</f>
         <v/>
       </c>
-      <c r="F57" s="81" t="inlineStr"/>
-      <c r="G57" s="81" t="inlineStr"/>
-      <c r="H57" s="81" t="inlineStr"/>
-      <c r="I57" s="81" t="inlineStr"/>
+      <c r="F57" s="143" t="inlineStr"/>
+      <c r="G57" s="143" t="inlineStr"/>
+      <c r="H57" s="143" t="inlineStr"/>
+      <c r="I57" s="143" t="inlineStr"/>
       <c r="J57" s="142" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
       <c r="K57" s="84">
-        <f>IF(A57="","",(COUNTIF(F57,"✓")+COUNTIF(G57,"✓")+COUNTIF(H57,"✓")+COUNTIF(I57,"✓")+COUNTIF(M57,"✓")+COUNTIF(N57,"✓")+COUNTIF(O57,"✓")+COUNTIF(P57,"✓"))*B57*C57)</f>
+        <f>IF(A57="","",(COUNTIF(F57,"●")+COUNTIF(G57,"●")+COUNTIF(H57,"●")+COUNTIF(I57,"●")+COUNTIF(M57,"●")+COUNTIF(N57,"●")+COUNTIF(O57,"●")+COUNTIF(P57,"●"))*B57*C57)</f>
         <v/>
       </c>
       <c r="L57" s="84">
-        <f>IF(A57="","",(COUNTIF(F57,"✓")+COUNTIF(G57,"✓")+COUNTIF(H57,"✓")+COUNTIF(I57,"✓")+COUNTIF(M57,"✓")+COUNTIF(N57,"✓")+COUNTIF(O57,"✓")+COUNTIF(P57,"✓"))*B57*D57)</f>
-        <v/>
-      </c>
-      <c r="M57" s="81" t="inlineStr"/>
-      <c r="N57" s="81" t="inlineStr"/>
-      <c r="O57" s="81" t="inlineStr"/>
-      <c r="P57" s="81" t="inlineStr"/>
-      <c r="Q57" s="81">
-        <f>IF(A57="",0,COUNTIF(A$49:A56,A57))</f>
+        <f>IF(A57="","",(COUNTIF(F57,"●")+COUNTIF(G57,"●")+COUNTIF(H57,"●")+COUNTIF(I57,"●")+COUNTIF(M57,"●")+COUNTIF(N57,"●")+COUNTIF(O57,"●")+COUNTIF(P57,"●"))*B57*D57)</f>
+        <v/>
+      </c>
+      <c r="M57" s="143" t="inlineStr"/>
+      <c r="N57" s="143" t="inlineStr"/>
+      <c r="O57" s="143" t="inlineStr"/>
+      <c r="P57" s="143" t="inlineStr"/>
+      <c r="R57" s="81">
+        <f>IF(A57="",0,COUNTIF(A$50:A56,A57))</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="123" t="inlineStr">
+      <c r="A58" s="129" t="inlineStr"/>
+      <c r="B58" s="83" t="inlineStr"/>
+      <c r="C58" s="84">
+        <f>IF(A58="","",VLOOKUP(A58,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D58" s="84">
+        <f>IF(A58="","",VLOOKUP(A58,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E58" s="137">
+        <f>IF(D58&gt;0,(D58-C58)/D58,0)</f>
+        <v/>
+      </c>
+      <c r="F58" s="143" t="inlineStr"/>
+      <c r="G58" s="143" t="inlineStr"/>
+      <c r="H58" s="143" t="inlineStr"/>
+      <c r="I58" s="143" t="inlineStr"/>
+      <c r="J58" s="142" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="K58" s="84">
+        <f>IF(A58="","",(COUNTIF(F58,"●")+COUNTIF(G58,"●")+COUNTIF(H58,"●")+COUNTIF(I58,"●")+COUNTIF(M58,"●")+COUNTIF(N58,"●")+COUNTIF(O58,"●")+COUNTIF(P58,"●"))*B58*C58)</f>
+        <v/>
+      </c>
+      <c r="L58" s="84">
+        <f>IF(A58="","",(COUNTIF(F58,"●")+COUNTIF(G58,"●")+COUNTIF(H58,"●")+COUNTIF(I58,"●")+COUNTIF(M58,"●")+COUNTIF(N58,"●")+COUNTIF(O58,"●")+COUNTIF(P58,"●"))*B58*D58)</f>
+        <v/>
+      </c>
+      <c r="M58" s="143" t="inlineStr"/>
+      <c r="N58" s="143" t="inlineStr"/>
+      <c r="O58" s="143" t="inlineStr"/>
+      <c r="P58" s="143" t="inlineStr"/>
+      <c r="R58" s="81">
+        <f>IF(A58="",0,COUNTIF(A$50:A57,A58))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B58" s="114" t="inlineStr"/>
-      <c r="C58" s="114" t="inlineStr"/>
-      <c r="D58" s="114" t="inlineStr"/>
-      <c r="E58" s="114" t="inlineStr"/>
-      <c r="F58" s="130">
-        <f>SUMPRODUCT((F49:F57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="G58" s="130">
-        <f>SUMPRODUCT((G49:G57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="H58" s="130">
-        <f>SUMPRODUCT((H49:H57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="I58" s="130">
-        <f>SUMPRODUCT((I49:I57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="J58" s="114" t="inlineStr"/>
-      <c r="K58" s="88">
-        <f>SUM(K49:K57)</f>
-        <v/>
-      </c>
-      <c r="L58" s="88">
-        <f>SUM(L49:L57)</f>
-        <v/>
-      </c>
-      <c r="M58" s="130">
-        <f>SUMPRODUCT((M49:M57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="N58" s="130">
-        <f>SUMPRODUCT((N49:N57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="O58" s="130">
-        <f>SUMPRODUCT((O49:O57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="P58" s="130">
-        <f>SUMPRODUCT((P49:P57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="103" t="inlineStr">
+      <c r="B59" s="114" t="inlineStr"/>
+      <c r="C59" s="114" t="inlineStr"/>
+      <c r="D59" s="114" t="inlineStr"/>
+      <c r="E59" s="114" t="inlineStr"/>
+      <c r="F59" s="130">
+        <f>SUMPRODUCT((F50:F58="●")*1,B50:B58,C50:C58)</f>
+        <v/>
+      </c>
+      <c r="G59" s="130">
+        <f>SUMPRODUCT((G50:G58="●")*1,B50:B58,C50:C58)</f>
+        <v/>
+      </c>
+      <c r="H59" s="130">
+        <f>SUMPRODUCT((H50:H58="●")*1,B50:B58,C50:C58)</f>
+        <v/>
+      </c>
+      <c r="I59" s="130">
+        <f>SUMPRODUCT((I50:I58="●")*1,B50:B58,C50:C58)</f>
+        <v/>
+      </c>
+      <c r="J59" s="114" t="inlineStr"/>
+      <c r="K59" s="88">
+        <f>SUM(K50:K58)</f>
+        <v/>
+      </c>
+      <c r="L59" s="88">
+        <f>SUM(L50:L58)</f>
+        <v/>
+      </c>
+      <c r="M59" s="130">
+        <f>SUMPRODUCT((M50:M58="●")*1,B50:B58,C50:C58)</f>
+        <v/>
+      </c>
+      <c r="N59" s="130">
+        <f>SUMPRODUCT((N50:N58="●")*1,B50:B58,C50:C58)</f>
+        <v/>
+      </c>
+      <c r="O59" s="130">
+        <f>SUMPRODUCT((O50:O58="●")*1,B50:B58,C50:C58)</f>
+        <v/>
+      </c>
+      <c r="P59" s="130">
+        <f>SUMPRODUCT((P50:P58="●")*1,B50:B58,C50:C58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="103" t="inlineStr">
         <is>
           <t>🏆 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B61" s="104" t="n"/>
-      <c r="C61" s="104" t="n"/>
-      <c r="D61" s="104" t="n"/>
-      <c r="E61" s="104" t="n"/>
-      <c r="F61" s="104" t="n"/>
-      <c r="G61" s="104" t="n"/>
-      <c r="H61" s="104" t="n"/>
-      <c r="I61" s="104" t="n"/>
-      <c r="J61" s="104" t="n"/>
-      <c r="K61" s="104" t="n"/>
-      <c r="L61" s="104" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="108" t="inlineStr">
-        <is>
-          <t>GOLF</t>
-        </is>
-      </c>
-      <c r="K62" s="84">
-        <f>K20</f>
-        <v/>
-      </c>
-      <c r="L62" s="84">
-        <f>L20</f>
-        <v/>
-      </c>
+      <c r="B62" s="104" t="n"/>
+      <c r="C62" s="104" t="n"/>
+      <c r="D62" s="104" t="n"/>
+      <c r="E62" s="104" t="n"/>
+      <c r="F62" s="104" t="n"/>
+      <c r="G62" s="104" t="n"/>
+      <c r="H62" s="104" t="n"/>
+      <c r="I62" s="104" t="n"/>
+      <c r="J62" s="104" t="n"/>
+      <c r="K62" s="104" t="n"/>
+      <c r="L62" s="104" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="108" t="inlineStr">
         <is>
-          <t>HOTEL</t>
+          <t>GOLF</t>
         </is>
       </c>
       <c r="K63" s="84">
-        <f>K26</f>
+        <f>K21</f>
         <v/>
       </c>
       <c r="L63" s="84">
-        <f>L26</f>
+        <f>L21</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="108" t="inlineStr">
         <is>
-          <t>TRANSPORT</t>
+          <t>HOTEL</t>
         </is>
       </c>
       <c r="K64" s="84">
-        <f>K32</f>
+        <f>K27</f>
         <v/>
       </c>
       <c r="L64" s="84">
-        <f>L32</f>
+        <f>L27</f>
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="108" t="inlineStr">
         <is>
-          <t>MEALS</t>
+          <t>TRANSPORT</t>
         </is>
       </c>
       <c r="K65" s="84">
-        <f>K40</f>
+        <f>K33</f>
         <v/>
       </c>
       <c r="L65" s="84">
-        <f>L40</f>
+        <f>L33</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="108" t="inlineStr">
         <is>
-          <t>OTHER</t>
+          <t xml:space="preserve"> MEALS</t>
         </is>
       </c>
       <c r="K66" s="84">
-        <f>K46</f>
+        <f>K41</f>
         <v/>
       </c>
       <c r="L66" s="84">
-        <f>L46</f>
+        <f>L41</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="108" t="inlineStr">
         <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="K67" s="84">
+        <f>K47</f>
+        <v/>
+      </c>
+      <c r="L67" s="84">
+        <f>L47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="108" t="inlineStr">
+        <is>
           <t>ACTIVITIES</t>
         </is>
       </c>
-      <c r="K67" s="84">
-        <f>K58</f>
-        <v/>
-      </c>
-      <c r="L67" s="84">
-        <f>L58</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="115" t="inlineStr">
+      <c r="K68" s="84">
+        <f>K59</f>
+        <v/>
+      </c>
+      <c r="L68" s="84">
+        <f>L59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="115" t="inlineStr">
         <is>
           <t>📌 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C68" s="116" t="inlineStr">
+      <c r="C69" s="116" t="inlineStr">
         <is>
           <t>Margin:</t>
         </is>
       </c>
-      <c r="D68" s="91">
-        <f>IF(L68&gt;0,(L68-K68)/L68,0)</f>
-        <v/>
-      </c>
-      <c r="K68" s="88">
-        <f>SUM(K62:K67)</f>
-        <v/>
-      </c>
-      <c r="L68" s="88">
-        <f>SUM(L62:L67)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="103" t="inlineStr">
+      <c r="D69" s="91">
+        <f>IF(L69&gt;0,(L69-K69)/L69,0)</f>
+        <v/>
+      </c>
+      <c r="K69" s="88">
+        <f>SUM(K63:K68)</f>
+        <v/>
+      </c>
+      <c r="L69" s="88">
+        <f>SUM(L63:L68)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="103" t="inlineStr">
         <is>
           <t>👤 PER PERSON SUMMARY</t>
         </is>
       </c>
-      <c r="B70" s="104" t="n"/>
-      <c r="C70" s="104" t="n"/>
-      <c r="D70" s="104" t="n"/>
-      <c r="E70" s="104" t="n"/>
-      <c r="F70" s="104" t="n"/>
-      <c r="G70" s="104" t="n"/>
-      <c r="H70" s="104" t="n"/>
-      <c r="I70" s="104" t="n"/>
-      <c r="J70" s="104" t="n"/>
-      <c r="K70" s="104" t="n"/>
-      <c r="L70" s="104" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="98" t="inlineStr">
+      <c r="B71" s="104" t="n"/>
+      <c r="C71" s="104" t="n"/>
+      <c r="D71" s="104" t="n"/>
+      <c r="E71" s="104" t="n"/>
+      <c r="F71" s="104" t="n"/>
+      <c r="G71" s="104" t="n"/>
+      <c r="H71" s="104" t="n"/>
+      <c r="I71" s="104" t="n"/>
+      <c r="J71" s="104" t="n"/>
+      <c r="K71" s="104" t="n"/>
+      <c r="L71" s="104" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="98" t="inlineStr">
         <is>
           <t>Person</t>
         </is>
       </c>
-      <c r="B71" s="98" t="inlineStr">
+      <c r="B72" s="98" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="C71" s="98" t="inlineStr">
+      <c r="C72" s="98" t="inlineStr">
         <is>
           <t>Sell</t>
         </is>
       </c>
-      <c r="D71" s="98" t="inlineStr">
+      <c r="D72" s="98" t="inlineStr">
         <is>
           <t>Margin</t>
         </is>
       </c>
-      <c r="E71" s="98" t="inlineStr">
+      <c r="E72" s="98" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F71" s="98" t="inlineStr">
-        <is>
-          <t>#Items</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="108" t="inlineStr">
-        <is>
-          <t>참가자1</t>
-        </is>
-      </c>
-      <c r="B72" s="131">
-        <f>SUMPRODUCT((F15:F19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((F23:F25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((F29:F31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((F35:F39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((F43:F45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((F49:F57="✓")*1,B49:B57,C49:C57)</f>
-        <v/>
-      </c>
-      <c r="C72" s="131">
-        <f>SUMPRODUCT((F15:F19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((F23:F25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((F29:F31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((F35:F39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((F43:F45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((F49:F57="✓")*1,B49:B57,D49:D57)</f>
-        <v/>
-      </c>
-      <c r="D72" s="110">
-        <f>C72-B72</f>
-        <v/>
-      </c>
-      <c r="E72" s="132">
-        <f>IF(C72&gt;0,D72/C72,0)</f>
-        <v/>
-      </c>
-      <c r="F72" s="139">
-        <f>COUNTIF(F15:F19,"✓")+COUNTIF(F23:F25,"✓")+COUNTIF(F29:F31,"✓")+COUNTIF(F35:F39,"✓")+COUNTIF(F43:F45,"✓")+COUNTIF(F49:F57,"✓")</f>
-        <v/>
+      <c r="F72" s="98" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="108" t="inlineStr">
-        <is>
-          <t>참가자2</t>
-        </is>
+      <c r="A73" s="108">
+        <f>B5</f>
+        <v/>
       </c>
       <c r="B73" s="131">
-        <f>SUMPRODUCT((G15:G19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((G23:G25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((G29:G31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((G35:G39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((G43:G45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((G49:G57="✓")*1,B49:B57,C49:C57)</f>
+        <f>SUMPRODUCT((F16:F20="●")*1,B16:B20,C16:C20)+SUMPRODUCT((F24:F26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((F30:F32="●")*1,B30:B32,C30:C32)+SUMPRODUCT((F36:F40="●")*1,B36:B40,C36:C40)+SUMPRODUCT((F44:F46="●")*1,B44:B46,C44:C46)+SUMPRODUCT((F50:F58="●")*1,B50:B58,C50:C58)</f>
         <v/>
       </c>
       <c r="C73" s="131">
-        <f>SUMPRODUCT((G15:G19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((G23:G25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((G29:G31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((G35:G39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((G43:G45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((G49:G57="✓")*1,B49:B57,D49:D57)</f>
+        <f>SUMPRODUCT((F16:F20="●")*1,B16:B20,D16:D20)+SUMPRODUCT((F24:F26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((F30:F32="●")*1,B30:B32,D30:D32)+SUMPRODUCT((F36:F40="●")*1,B36:B40,D36:D40)+SUMPRODUCT((F44:F46="●")*1,B44:B46,D44:D46)+SUMPRODUCT((F50:F58="●")*1,B50:B58,D50:D58)</f>
         <v/>
       </c>
       <c r="D73" s="110">
@@ -5551,22 +5602,21 @@
         <v/>
       </c>
       <c r="F73" s="139">
-        <f>COUNTIF(G15:G19,"✓")+COUNTIF(G23:G25,"✓")+COUNTIF(G29:G31,"✓")+COUNTIF(G35:G39,"✓")+COUNTIF(G43:G45,"✓")+COUNTIF(G49:G57,"✓")</f>
+        <f>COUNTIF(F16:F20,"●")+COUNTIF(F24:F26,"●")+COUNTIF(F30:F32,"●")+COUNTIF(F36:F40,"●")+COUNTIF(F44:F46,"●")+COUNTIF(F50:F58,"●")</f>
         <v/>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="108" t="inlineStr">
-        <is>
-          <t>참가자3</t>
-        </is>
+      <c r="A74" s="108">
+        <f>C5</f>
+        <v/>
       </c>
       <c r="B74" s="131">
-        <f>SUMPRODUCT((H15:H19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((H23:H25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((H29:H31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((H35:H39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((H43:H45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((H49:H57="✓")*1,B49:B57,C49:C57)</f>
+        <f>SUMPRODUCT((G16:G20="●")*1,B16:B20,C16:C20)+SUMPRODUCT((G24:G26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((G30:G32="●")*1,B30:B32,C30:C32)+SUMPRODUCT((G36:G40="●")*1,B36:B40,C36:C40)+SUMPRODUCT((G44:G46="●")*1,B44:B46,C44:C46)+SUMPRODUCT((G50:G58="●")*1,B50:B58,C50:C58)</f>
         <v/>
       </c>
       <c r="C74" s="131">
-        <f>SUMPRODUCT((H15:H19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((H23:H25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((H29:H31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((H35:H39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((H43:H45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((H49:H57="✓")*1,B49:B57,D49:D57)</f>
+        <f>SUMPRODUCT((G16:G20="●")*1,B16:B20,D16:D20)+SUMPRODUCT((G24:G26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((G30:G32="●")*1,B30:B32,D30:D32)+SUMPRODUCT((G36:G40="●")*1,B36:B40,D36:D40)+SUMPRODUCT((G44:G46="●")*1,B44:B46,D44:D46)+SUMPRODUCT((G50:G58="●")*1,B50:B58,D50:D58)</f>
         <v/>
       </c>
       <c r="D74" s="110">
@@ -5578,22 +5628,21 @@
         <v/>
       </c>
       <c r="F74" s="139">
-        <f>COUNTIF(H15:H19,"✓")+COUNTIF(H23:H25,"✓")+COUNTIF(H29:H31,"✓")+COUNTIF(H35:H39,"✓")+COUNTIF(H43:H45,"✓")+COUNTIF(H49:H57,"✓")</f>
+        <f>COUNTIF(G16:G20,"●")+COUNTIF(G24:G26,"●")+COUNTIF(G30:G32,"●")+COUNTIF(G36:G40,"●")+COUNTIF(G44:G46,"●")+COUNTIF(G50:G58,"●")</f>
         <v/>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="108" t="inlineStr">
-        <is>
-          <t>참가자4</t>
-        </is>
+      <c r="A75" s="108">
+        <f>D5</f>
+        <v/>
       </c>
       <c r="B75" s="131">
-        <f>SUMPRODUCT((I15:I19="✓")*1,B15:B19,C15:C19)+SUMPRODUCT((I23:I25="✓")*1,B23:B25,C23:C25)+SUMPRODUCT((I29:I31="✓")*1,B29:B31,C29:C31)+SUMPRODUCT((I35:I39="✓")*1,B35:B39,C35:C39)+SUMPRODUCT((I43:I45="✓")*1,B43:B45,C43:C45)+SUMPRODUCT((I49:I57="✓")*1,B49:B57,C49:C57)</f>
+        <f>SUMPRODUCT((H16:H20="●")*1,B16:B20,C16:C20)+SUMPRODUCT((H24:H26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((H30:H32="●")*1,B30:B32,C30:C32)+SUMPRODUCT((H36:H40="●")*1,B36:B40,C36:C40)+SUMPRODUCT((H44:H46="●")*1,B44:B46,C44:C46)+SUMPRODUCT((H50:H58="●")*1,B50:B58,C50:C58)</f>
         <v/>
       </c>
       <c r="C75" s="131">
-        <f>SUMPRODUCT((I15:I19="✓")*1,B15:B19,D15:D19)+SUMPRODUCT((I23:I25="✓")*1,B23:B25,D23:D25)+SUMPRODUCT((I29:I31="✓")*1,B29:B31,D29:D31)+SUMPRODUCT((I35:I39="✓")*1,B35:B39,D35:D39)+SUMPRODUCT((I43:I45="✓")*1,B43:B45,D43:D45)+SUMPRODUCT((I49:I57="✓")*1,B49:B57,D49:D57)</f>
+        <f>SUMPRODUCT((H16:H20="●")*1,B16:B20,D16:D20)+SUMPRODUCT((H24:H26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((H30:H32="●")*1,B30:B32,D30:D32)+SUMPRODUCT((H36:H40="●")*1,B36:B40,D36:D40)+SUMPRODUCT((H44:H46="●")*1,B44:B46,D44:D46)+SUMPRODUCT((H50:H58="●")*1,B50:B58,D50:D58)</f>
         <v/>
       </c>
       <c r="D75" s="110">
@@ -5605,749 +5654,771 @@
         <v/>
       </c>
       <c r="F75" s="139">
-        <f>COUNTIF(I15:I19,"✓")+COUNTIF(I23:I25,"✓")+COUNTIF(I29:I31,"✓")+COUNTIF(I35:I39,"✓")+COUNTIF(I43:I45,"✓")+COUNTIF(I49:I57,"✓")</f>
+        <f>COUNTIF(H16:H20,"●")+COUNTIF(H24:H26,"●")+COUNTIF(H30:H32,"●")+COUNTIF(H36:H40,"●")+COUNTIF(H44:H46,"●")+COUNTIF(H50:H58,"●")</f>
         <v/>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="115" t="inlineStr">
+      <c r="A76" s="108">
+        <f>E5</f>
+        <v/>
+      </c>
+      <c r="B76" s="131">
+        <f>SUMPRODUCT((I16:I20="●")*1,B16:B20,C16:C20)+SUMPRODUCT((I24:I26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((I30:I32="●")*1,B30:B32,C30:C32)+SUMPRODUCT((I36:I40="●")*1,B36:B40,C36:C40)+SUMPRODUCT((I44:I46="●")*1,B44:B46,C44:C46)+SUMPRODUCT((I50:I58="●")*1,B50:B58,C50:C58)</f>
+        <v/>
+      </c>
+      <c r="C76" s="131">
+        <f>SUMPRODUCT((I16:I20="●")*1,B16:B20,D16:D20)+SUMPRODUCT((I24:I26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((I30:I32="●")*1,B30:B32,D30:D32)+SUMPRODUCT((I36:I40="●")*1,B36:B40,D36:D40)+SUMPRODUCT((I44:I46="●")*1,B44:B46,D44:D46)+SUMPRODUCT((I50:I58="●")*1,B50:B58,D50:D58)</f>
+        <v/>
+      </c>
+      <c r="D76" s="110">
+        <f>C76-B76</f>
+        <v/>
+      </c>
+      <c r="E76" s="132">
+        <f>IF(C76&gt;0,D76/C76,0)</f>
+        <v/>
+      </c>
+      <c r="F76" s="139">
+        <f>COUNTIF(I16:I20,"●")+COUNTIF(I24:I26,"●")+COUNTIF(I30:I32,"●")+COUNTIF(I36:I40,"●")+COUNTIF(I44:I46,"●")+COUNTIF(I50:I58,"●")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="115" t="inlineStr">
         <is>
           <t>📌 TOTAL</t>
         </is>
       </c>
-      <c r="B76" s="88">
-        <f>SUM(B72:B75)</f>
-        <v/>
-      </c>
-      <c r="C76" s="88">
-        <f>SUM(C72:C75)</f>
-        <v/>
-      </c>
-      <c r="D76" s="88">
-        <f>SUM(D72:D75)</f>
-        <v/>
-      </c>
-      <c r="E76" s="91">
-        <f>IF(C76&gt;0,D76/C76,0)</f>
+      <c r="B77" s="88">
+        <f>SUM(B73:B76)</f>
+        <v/>
+      </c>
+      <c r="C77" s="88">
+        <f>SUM(C73:C76)</f>
+        <v/>
+      </c>
+      <c r="D77" s="88">
+        <f>SUM(D73:D76)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
     <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A42:L42"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A7:L7"/>
+    <mergeCell ref="A29:L29"/>
+    <mergeCell ref="A43:L43"/>
+    <mergeCell ref="A71:L71"/>
+    <mergeCell ref="A49:L49"/>
     <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A28:L28"/>
-    <mergeCell ref="A34:L34"/>
-    <mergeCell ref="A14:L14"/>
-    <mergeCell ref="A61:L61"/>
-    <mergeCell ref="A6:L6"/>
-    <mergeCell ref="A22:L22"/>
-    <mergeCell ref="A70:L70"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="A35:L35"/>
     <mergeCell ref="B4:C4"/>
-    <mergeCell ref="A48:L48"/>
+    <mergeCell ref="A62:L62"/>
   </mergeCells>
-  <conditionalFormatting sqref="F15">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G15">
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H15">
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I15">
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q15">
+  <conditionalFormatting sqref="F16">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G16">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H16">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I16">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R16">
     <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F16">
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G16">
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H16">
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I16">
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q16">
+  <conditionalFormatting sqref="F17">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H17">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I17">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R17">
     <cfRule type="cellIs" priority="10" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F17">
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G17">
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H17">
-    <cfRule type="cellIs" priority="13" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I17">
-    <cfRule type="cellIs" priority="14" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q17">
+  <conditionalFormatting sqref="F18">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G18">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H18">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I18">
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R18">
     <cfRule type="cellIs" priority="15" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F18">
-    <cfRule type="cellIs" priority="16" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G18">
-    <cfRule type="cellIs" priority="17" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H18">
-    <cfRule type="cellIs" priority="18" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I18">
-    <cfRule type="cellIs" priority="19" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q18">
+  <conditionalFormatting sqref="F19">
+    <cfRule type="cellIs" priority="16" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G19">
+    <cfRule type="cellIs" priority="17" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H19">
+    <cfRule type="cellIs" priority="18" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I19">
+    <cfRule type="cellIs" priority="19" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R19">
     <cfRule type="cellIs" priority="20" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F19">
-    <cfRule type="cellIs" priority="21" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G19">
-    <cfRule type="cellIs" priority="22" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H19">
-    <cfRule type="cellIs" priority="23" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I19">
-    <cfRule type="cellIs" priority="24" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q19">
+  <conditionalFormatting sqref="F20">
+    <cfRule type="cellIs" priority="21" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G20">
+    <cfRule type="cellIs" priority="22" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H20">
+    <cfRule type="cellIs" priority="23" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I20">
+    <cfRule type="cellIs" priority="24" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R20">
     <cfRule type="cellIs" priority="25" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F23">
-    <cfRule type="cellIs" priority="26" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G23">
-    <cfRule type="cellIs" priority="27" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H23">
-    <cfRule type="cellIs" priority="28" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I23">
-    <cfRule type="cellIs" priority="29" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q23">
+  <conditionalFormatting sqref="F24">
+    <cfRule type="cellIs" priority="26" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G24">
+    <cfRule type="cellIs" priority="27" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H24">
+    <cfRule type="cellIs" priority="28" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I24">
+    <cfRule type="cellIs" priority="29" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R24">
     <cfRule type="cellIs" priority="30" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F24">
-    <cfRule type="cellIs" priority="31" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G24">
-    <cfRule type="cellIs" priority="32" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H24">
-    <cfRule type="cellIs" priority="33" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I24">
-    <cfRule type="cellIs" priority="34" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q24">
+  <conditionalFormatting sqref="F25">
+    <cfRule type="cellIs" priority="31" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G25">
+    <cfRule type="cellIs" priority="32" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H25">
+    <cfRule type="cellIs" priority="33" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I25">
+    <cfRule type="cellIs" priority="34" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R25">
     <cfRule type="cellIs" priority="35" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F25">
-    <cfRule type="cellIs" priority="36" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G25">
-    <cfRule type="cellIs" priority="37" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H25">
-    <cfRule type="cellIs" priority="38" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I25">
-    <cfRule type="cellIs" priority="39" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q25">
+  <conditionalFormatting sqref="F26">
+    <cfRule type="cellIs" priority="36" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G26">
+    <cfRule type="cellIs" priority="37" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H26">
+    <cfRule type="cellIs" priority="38" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I26">
+    <cfRule type="cellIs" priority="39" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R26">
     <cfRule type="cellIs" priority="40" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F29">
-    <cfRule type="cellIs" priority="41" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G29">
-    <cfRule type="cellIs" priority="42" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H29">
-    <cfRule type="cellIs" priority="43" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I29">
-    <cfRule type="cellIs" priority="44" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q29">
+  <conditionalFormatting sqref="F30">
+    <cfRule type="cellIs" priority="41" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G30">
+    <cfRule type="cellIs" priority="42" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H30">
+    <cfRule type="cellIs" priority="43" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I30">
+    <cfRule type="cellIs" priority="44" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R30">
     <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F30">
-    <cfRule type="cellIs" priority="46" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G30">
-    <cfRule type="cellIs" priority="47" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H30">
-    <cfRule type="cellIs" priority="48" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I30">
-    <cfRule type="cellIs" priority="49" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q30">
+  <conditionalFormatting sqref="F31">
+    <cfRule type="cellIs" priority="46" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G31">
+    <cfRule type="cellIs" priority="47" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H31">
+    <cfRule type="cellIs" priority="48" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I31">
+    <cfRule type="cellIs" priority="49" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R31">
     <cfRule type="cellIs" priority="50" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F31">
-    <cfRule type="cellIs" priority="51" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G31">
-    <cfRule type="cellIs" priority="52" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H31">
-    <cfRule type="cellIs" priority="53" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I31">
-    <cfRule type="cellIs" priority="54" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q31">
+  <conditionalFormatting sqref="F32">
+    <cfRule type="cellIs" priority="51" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G32">
+    <cfRule type="cellIs" priority="52" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H32">
+    <cfRule type="cellIs" priority="53" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I32">
+    <cfRule type="cellIs" priority="54" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R32">
     <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F35">
-    <cfRule type="cellIs" priority="56" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G35">
-    <cfRule type="cellIs" priority="57" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H35">
-    <cfRule type="cellIs" priority="58" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I35">
-    <cfRule type="cellIs" priority="59" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q35">
+  <conditionalFormatting sqref="F36">
+    <cfRule type="cellIs" priority="56" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G36">
+    <cfRule type="cellIs" priority="57" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="cellIs" priority="58" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I36">
+    <cfRule type="cellIs" priority="59" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R36">
     <cfRule type="cellIs" priority="60" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F36">
-    <cfRule type="cellIs" priority="61" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G36">
-    <cfRule type="cellIs" priority="62" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H36">
-    <cfRule type="cellIs" priority="63" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I36">
-    <cfRule type="cellIs" priority="64" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q36">
+  <conditionalFormatting sqref="F37">
+    <cfRule type="cellIs" priority="61" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G37">
+    <cfRule type="cellIs" priority="62" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H37">
+    <cfRule type="cellIs" priority="63" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I37">
+    <cfRule type="cellIs" priority="64" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R37">
     <cfRule type="cellIs" priority="65" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F37">
-    <cfRule type="cellIs" priority="66" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G37">
-    <cfRule type="cellIs" priority="67" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H37">
-    <cfRule type="cellIs" priority="68" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I37">
-    <cfRule type="cellIs" priority="69" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q37">
+  <conditionalFormatting sqref="F38">
+    <cfRule type="cellIs" priority="66" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G38">
+    <cfRule type="cellIs" priority="67" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H38">
+    <cfRule type="cellIs" priority="68" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I38">
+    <cfRule type="cellIs" priority="69" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R38">
     <cfRule type="cellIs" priority="70" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F38">
-    <cfRule type="cellIs" priority="71" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G38">
-    <cfRule type="cellIs" priority="72" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H38">
-    <cfRule type="cellIs" priority="73" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I38">
-    <cfRule type="cellIs" priority="74" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q38">
+  <conditionalFormatting sqref="F39">
+    <cfRule type="cellIs" priority="71" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G39">
+    <cfRule type="cellIs" priority="72" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H39">
+    <cfRule type="cellIs" priority="73" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I39">
+    <cfRule type="cellIs" priority="74" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R39">
     <cfRule type="cellIs" priority="75" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F39">
-    <cfRule type="cellIs" priority="76" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G39">
-    <cfRule type="cellIs" priority="77" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H39">
-    <cfRule type="cellIs" priority="78" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I39">
-    <cfRule type="cellIs" priority="79" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q39">
+  <conditionalFormatting sqref="F40">
+    <cfRule type="cellIs" priority="76" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G40">
+    <cfRule type="cellIs" priority="77" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H40">
+    <cfRule type="cellIs" priority="78" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I40">
+    <cfRule type="cellIs" priority="79" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R40">
     <cfRule type="cellIs" priority="80" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F43">
-    <cfRule type="cellIs" priority="81" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G43">
-    <cfRule type="cellIs" priority="82" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H43">
-    <cfRule type="cellIs" priority="83" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I43">
-    <cfRule type="cellIs" priority="84" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q43">
+  <conditionalFormatting sqref="F44">
+    <cfRule type="cellIs" priority="81" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G44">
+    <cfRule type="cellIs" priority="82" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H44">
+    <cfRule type="cellIs" priority="83" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I44">
+    <cfRule type="cellIs" priority="84" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R44">
     <cfRule type="cellIs" priority="85" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F44">
-    <cfRule type="cellIs" priority="86" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G44">
-    <cfRule type="cellIs" priority="87" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H44">
-    <cfRule type="cellIs" priority="88" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I44">
-    <cfRule type="cellIs" priority="89" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q44">
+  <conditionalFormatting sqref="F45">
+    <cfRule type="cellIs" priority="86" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G45">
+    <cfRule type="cellIs" priority="87" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H45">
+    <cfRule type="cellIs" priority="88" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I45">
+    <cfRule type="cellIs" priority="89" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R45">
     <cfRule type="cellIs" priority="90" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F45">
-    <cfRule type="cellIs" priority="91" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G45">
-    <cfRule type="cellIs" priority="92" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H45">
-    <cfRule type="cellIs" priority="93" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I45">
-    <cfRule type="cellIs" priority="94" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q45">
+  <conditionalFormatting sqref="F46">
+    <cfRule type="cellIs" priority="91" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G46">
+    <cfRule type="cellIs" priority="92" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H46">
+    <cfRule type="cellIs" priority="93" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I46">
+    <cfRule type="cellIs" priority="94" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R46">
     <cfRule type="cellIs" priority="95" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F49">
-    <cfRule type="cellIs" priority="96" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G49">
-    <cfRule type="cellIs" priority="97" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H49">
-    <cfRule type="cellIs" priority="98" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I49">
-    <cfRule type="cellIs" priority="99" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q49">
+  <conditionalFormatting sqref="F50">
+    <cfRule type="cellIs" priority="96" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G50">
+    <cfRule type="cellIs" priority="97" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H50">
+    <cfRule type="cellIs" priority="98" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I50">
+    <cfRule type="cellIs" priority="99" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R50">
     <cfRule type="cellIs" priority="100" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F50">
-    <cfRule type="cellIs" priority="101" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G50">
-    <cfRule type="cellIs" priority="102" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H50">
-    <cfRule type="cellIs" priority="103" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I50">
-    <cfRule type="cellIs" priority="104" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q50">
+  <conditionalFormatting sqref="F51">
+    <cfRule type="cellIs" priority="101" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G51">
+    <cfRule type="cellIs" priority="102" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H51">
+    <cfRule type="cellIs" priority="103" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I51">
+    <cfRule type="cellIs" priority="104" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R51">
     <cfRule type="cellIs" priority="105" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F51">
-    <cfRule type="cellIs" priority="106" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G51">
-    <cfRule type="cellIs" priority="107" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H51">
-    <cfRule type="cellIs" priority="108" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I51">
-    <cfRule type="cellIs" priority="109" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q51">
+  <conditionalFormatting sqref="F52">
+    <cfRule type="cellIs" priority="106" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G52">
+    <cfRule type="cellIs" priority="107" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H52">
+    <cfRule type="cellIs" priority="108" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I52">
+    <cfRule type="cellIs" priority="109" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R52">
     <cfRule type="cellIs" priority="110" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F52">
-    <cfRule type="cellIs" priority="111" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G52">
-    <cfRule type="cellIs" priority="112" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H52">
-    <cfRule type="cellIs" priority="113" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I52">
-    <cfRule type="cellIs" priority="114" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q52">
+  <conditionalFormatting sqref="F53">
+    <cfRule type="cellIs" priority="111" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G53">
+    <cfRule type="cellIs" priority="112" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H53">
+    <cfRule type="cellIs" priority="113" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I53">
+    <cfRule type="cellIs" priority="114" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R53">
     <cfRule type="cellIs" priority="115" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F53">
-    <cfRule type="cellIs" priority="116" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G53">
-    <cfRule type="cellIs" priority="117" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H53">
-    <cfRule type="cellIs" priority="118" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I53">
-    <cfRule type="cellIs" priority="119" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q53">
+  <conditionalFormatting sqref="F54">
+    <cfRule type="cellIs" priority="116" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G54">
+    <cfRule type="cellIs" priority="117" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H54">
+    <cfRule type="cellIs" priority="118" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I54">
+    <cfRule type="cellIs" priority="119" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R54">
     <cfRule type="cellIs" priority="120" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F54">
-    <cfRule type="cellIs" priority="121" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G54">
-    <cfRule type="cellIs" priority="122" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H54">
-    <cfRule type="cellIs" priority="123" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I54">
-    <cfRule type="cellIs" priority="124" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q54">
+  <conditionalFormatting sqref="F55">
+    <cfRule type="cellIs" priority="121" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G55">
+    <cfRule type="cellIs" priority="122" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H55">
+    <cfRule type="cellIs" priority="123" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I55">
+    <cfRule type="cellIs" priority="124" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R55">
     <cfRule type="cellIs" priority="125" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F55">
-    <cfRule type="cellIs" priority="126" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G55">
-    <cfRule type="cellIs" priority="127" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H55">
-    <cfRule type="cellIs" priority="128" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I55">
-    <cfRule type="cellIs" priority="129" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q55">
+  <conditionalFormatting sqref="F56">
+    <cfRule type="cellIs" priority="126" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G56">
+    <cfRule type="cellIs" priority="127" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H56">
+    <cfRule type="cellIs" priority="128" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I56">
+    <cfRule type="cellIs" priority="129" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R56">
     <cfRule type="cellIs" priority="130" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F56">
-    <cfRule type="cellIs" priority="131" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G56">
-    <cfRule type="cellIs" priority="132" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H56">
-    <cfRule type="cellIs" priority="133" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I56">
-    <cfRule type="cellIs" priority="134" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q56">
+  <conditionalFormatting sqref="F57">
+    <cfRule type="cellIs" priority="131" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G57">
+    <cfRule type="cellIs" priority="132" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H57">
+    <cfRule type="cellIs" priority="133" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I57">
+    <cfRule type="cellIs" priority="134" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R57">
     <cfRule type="cellIs" priority="135" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F57">
-    <cfRule type="cellIs" priority="136" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G57">
-    <cfRule type="cellIs" priority="137" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H57">
-    <cfRule type="cellIs" priority="138" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I57">
-    <cfRule type="cellIs" priority="139" operator="equal" dxfId="4">
-      <formula>"✓"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q57">
+  <conditionalFormatting sqref="F58">
+    <cfRule type="cellIs" priority="136" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G58">
+    <cfRule type="cellIs" priority="137" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H58">
+    <cfRule type="cellIs" priority="138" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I58">
+    <cfRule type="cellIs" priority="139" operator="equal" dxfId="5">
+      <formula>"●"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R58">
     <cfRule type="cellIs" priority="140" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E12">
+  <conditionalFormatting sqref="E13">
     <cfRule type="cellIs" priority="141" operator="notEqual" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6356,34 +6427,34 @@
     <dataValidation sqref="E4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"2,4,6,8"</formula1>
     </dataValidation>
-    <dataValidation sqref="E7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>'Master Data'!$A$60:$A$63</formula1>
     </dataValidation>
-    <dataValidation sqref="E8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>'Master Data'!$A$74:$A$77</formula1>
     </dataValidation>
-    <dataValidation sqref="K7 K8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K8 K9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"First, Business, Premium Economy, Economy"</formula1>
     </dataValidation>
-    <dataValidation sqref="F15 F16 F17 F18 F19 F23 F24 F25 F29 F30 F31 F35 F36 F37 F38 F39 F43 F44 F45 F49 F50 F51 F52 F53 F54 F55 F56 F57 G15 G16 G17 G18 G19 G23 G24 G25 G29 G30 G31 G35 G36 G37 G38 G39 G43 G44 G45 G49 G50 G51 G52 G53 G54 G55 G56 G57 H15 H16 H17 H18 H19 H23 H24 H25 H29 H30 H31 H35 H36 H37 H38 H39 H43 H44 H45 H49 H50 H51 H52 H53 H54 H55 H56 H57 I15 I16 I17 I18 I19 I23 I24 I25 I29 I30 I31 I35 I36 I37 I38 I39 I43 I44 I45 I49 I50 I51 I52 I53 I54 I55 I56 I57 M15 M16 M17 M18 M19 M23 M24 M25 M29 M30 M31 M35 M36 M37 M38 M39 M43 M44 M45 M49 M50 M51 M52 M53 M54 M55 M56 M57 N15 N16 N17 N18 N19 N23 N24 N25 N29 N30 N31 N35 N36 N37 N38 N39 N43 N44 N45 N49 N50 N51 N52 N53 N54 N55 N56 N57 O15 O16 O17 O18 O19 O23 O24 O25 O29 O30 O31 O35 O36 O37 O38 O39 O43 O44 O45 O49 O50 O51 O52 O53 O54 O55 O56 O57 P15 P16 P17 P18 P19 P23 P24 P25 P29 P30 P31 P35 P36 P37 P38 P39 P43 P44 P45 P49 P50 P51 P52 P53 P54 P55 P56 P57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"✓,"</formula1>
+    <dataValidation sqref="F16 F17 F18 F19 F20 F24 F25 F26 F30 F31 F32 F36 F37 F38 F39 F40 F44 F45 F46 F50 F51 F52 F53 F54 F55 F56 F57 F58 G16 G17 G18 G19 G20 G24 G25 G26 G30 G31 G32 G36 G37 G38 G39 G40 G44 G45 G46 G50 G51 G52 G53 G54 G55 G56 G57 G58 H16 H17 H18 H19 H20 H24 H25 H26 H30 H31 H32 H36 H37 H38 H39 H40 H44 H45 H46 H50 H51 H52 H53 H54 H55 H56 H57 H58 I16 I17 I18 I19 I20 I24 I25 I26 I30 I31 I32 I36 I37 I38 I39 I40 I44 I45 I46 I50 I51 I52 I53 I54 I55 I56 I57 I58 M16 M17 M18 M19 M20 M24 M25 M26 M30 M31 M32 M36 M37 M38 M39 M40 M44 M45 M46 M50 M51 M52 M53 M54 M55 M56 M57 M58 N16 N17 N18 N19 N20 N24 N25 N26 N30 N31 N32 N36 N37 N38 N39 N40 N44 N45 N46 N50 N51 N52 N53 N54 N55 N56 N57 N58 O16 O17 O18 O19 O20 O24 O25 O26 O30 O31 O32 O36 O37 O38 O39 O40 O44 O45 O46 O50 O51 O52 O53 O54 O55 O56 O57 O58 P16 P17 P18 P19 P20 P24 P25 P26 P30 P31 P32 P36 P37 P38 P39 P40 P44 P45 P46 P50 P51 P52 P53 P54 P55 P56 P57 P58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"●",</formula1>
     </dataValidation>
-    <dataValidation sqref="A15 A16 A17 A18 A19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A16 A17 A18 A19 A20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Master Data'!$A$7:$A$14</formula1>
     </dataValidation>
-    <dataValidation sqref="A23 A24 A25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A24 A25 A26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Master Data'!$A$19:$A$24</formula1>
     </dataValidation>
-    <dataValidation sqref="A29 A30 A31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A30 A31 A32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Master Data'!$A$28:$A$34</formula1>
     </dataValidation>
-    <dataValidation sqref="A35 A36 A37 A38 A39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A36 A37 A38 A39 A40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Master Data'!$A$38:$A$46</formula1>
     </dataValidation>
-    <dataValidation sqref="A43 A44 A45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A44 A45 A46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Master Data'!$A$50:$A$56</formula1>
     </dataValidation>
-    <dataValidation sqref="A49 A50 A51 A52 A53 A54 A55 A56 A57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A50 A51 A52 A53 A54 A55 A56 A57 A58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Master Data'!$A$86:$A$94</formula1>
     </dataValidation>
   </dataValidations>
@@ -6459,11 +6530,11 @@
         </is>
       </c>
       <c r="B5" s="84">
-        <f>'Package Selector'!K20</f>
+        <f>'Package Selector'!K21</f>
         <v/>
       </c>
       <c r="C5" s="84">
-        <f>'Package Selector'!L20</f>
+        <f>'Package Selector'!L21</f>
         <v/>
       </c>
       <c r="D5" s="84">
@@ -6486,11 +6557,11 @@
         </is>
       </c>
       <c r="B6" s="84">
-        <f>'Package Selector'!K26</f>
+        <f>'Package Selector'!K27</f>
         <v/>
       </c>
       <c r="C6" s="84">
-        <f>'Package Selector'!L26</f>
+        <f>'Package Selector'!L27</f>
         <v/>
       </c>
       <c r="D6" s="84">
@@ -6513,11 +6584,11 @@
         </is>
       </c>
       <c r="B7" s="84">
-        <f>'Package Selector'!K32</f>
+        <f>'Package Selector'!K33</f>
         <v/>
       </c>
       <c r="C7" s="84">
-        <f>'Package Selector'!L32</f>
+        <f>'Package Selector'!L33</f>
         <v/>
       </c>
       <c r="D7" s="84">
@@ -6536,15 +6607,15 @@
     <row r="8">
       <c r="A8" s="136" t="inlineStr">
         <is>
-          <t>MEALS</t>
+          <t xml:space="preserve"> MEALS</t>
         </is>
       </c>
       <c r="B8" s="84">
-        <f>'Package Selector'!K40</f>
+        <f>'Package Selector'!K41</f>
         <v/>
       </c>
       <c r="C8" s="84">
-        <f>'Package Selector'!L40</f>
+        <f>'Package Selector'!L41</f>
         <v/>
       </c>
       <c r="D8" s="84">
@@ -6567,11 +6638,11 @@
         </is>
       </c>
       <c r="B9" s="84">
-        <f>'Package Selector'!K46</f>
+        <f>'Package Selector'!K47</f>
         <v/>
       </c>
       <c r="C9" s="84">
-        <f>'Package Selector'!L46</f>
+        <f>'Package Selector'!L47</f>
         <v/>
       </c>
       <c r="D9" s="84">
@@ -6594,11 +6665,11 @@
         </is>
       </c>
       <c r="B10" s="84">
-        <f>'Package Selector'!K58</f>
+        <f>'Package Selector'!K59</f>
         <v/>
       </c>
       <c r="C10" s="84">
-        <f>'Package Selector'!L58</f>
+        <f>'Package Selector'!L59</f>
         <v/>
       </c>
       <c r="D10" s="84">

</xml_diff>

<commit_message>
fix: clean frozen section (out/return separate rows), Master Data values restored, ● toggle allow_blank
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -1452,11 +1452,11 @@
         <v/>
       </c>
       <c r="E7" s="4" t="n">
-        <v>111</v>
+        <v>45</v>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Member guest | Cart incl. | Replay ~50%</t>
+          <t>teeitup.com | 9Stamps=1free | Replay twilight</t>
         </is>
       </c>
     </row>
@@ -1502,11 +1502,11 @@
         <v/>
       </c>
       <c r="E9" s="4" t="n">
-        <v>45</v>
+        <v>111</v>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>teeitup.com | 9Stamps=1free | Replay twilight</t>
+          <t>Member guest | Cart incl. | Replay ~50%</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,6 @@
       </c>
       <c r="F55" s="6" t="n"/>
     </row>
-    <row r="56"/>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
         <is>
@@ -2728,14 +2727,14 @@
     <row r="86">
       <c r="A86" s="74" t="inlineStr">
         <is>
-          <t>(New Activity 5)</t>
+          <t>Beach/Surf Lesson</t>
         </is>
       </c>
       <c r="B86" s="75" t="n">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="C86" s="75" t="n">
-        <v>180</v>
+        <v>100</v>
       </c>
       <c r="D86" s="51">
         <f>IF(A86="","",C86-B86)</f>
@@ -2749,21 +2748,21 @@
       </c>
       <c r="G86" s="49" t="inlineStr">
         <is>
-          <t>Seasonal; group rates available</t>
+          <t>2hr session; equipment incl.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="74" t="inlineStr">
         <is>
-          <t>(New Activity 6)</t>
+          <t>Local Hiking (Griffith/Runyon)</t>
         </is>
       </c>
       <c r="B87" s="75" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="C87" s="75" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="D87" s="51">
         <f>IF(A87="","",C87-B87)</f>
@@ -2777,21 +2776,21 @@
       </c>
       <c r="G87" s="49" t="inlineStr">
         <is>
-          <t>Premium sports bar with food/drinks</t>
+          <t>Guided tour included</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="74" t="inlineStr">
         <is>
-          <t>(New Activity 7)</t>
+          <t>NBA/MLB Game (Ticket)</t>
         </is>
       </c>
       <c r="B88" s="75" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="C88" s="75" t="n">
-        <v>30</v>
+        <v>180</v>
       </c>
       <c r="D88" s="51">
         <f>IF(A88="","",C88-B88)</f>
@@ -2805,21 +2804,21 @@
       </c>
       <c r="G88" s="49" t="inlineStr">
         <is>
-          <t>Guided tour included</t>
+          <t>Seasonal; group rates available</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="74" t="inlineStr">
         <is>
-          <t>(New Activity 8)</t>
+          <t>Sports Bar Experience</t>
         </is>
       </c>
       <c r="B89" s="75" t="n">
         <v>60</v>
       </c>
       <c r="C89" s="75" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="D89" s="51">
         <f>IF(A89="","",C89-B89)</f>
@@ -2833,7 +2832,7 @@
       </c>
       <c r="G89" s="49" t="inlineStr">
         <is>
-          <t>2hr session; equipment incl.</t>
+          <t>Premium sports bar with food/drinks</t>
         </is>
       </c>
     </row>
@@ -3381,7 +3380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P68"/>
+  <dimension ref="A1:P71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="42" min="1" max="1"/>
@@ -3426,7 +3425,6 @@
         </is>
       </c>
       <c r="B2" s="129" t="inlineStr"/>
-      <c r="C2" s="87" t="n"/>
       <c r="D2" s="106" t="inlineStr">
         <is>
           <t>Golfers:</t>
@@ -3455,330 +3453,261 @@
           <t>Guest4</t>
         </is>
       </c>
-      <c r="J2" s="129" t="inlineStr">
-        <is>
-          <t>Guest4</t>
-        </is>
-      </c>
     </row>
     <row r="3">
-      <c r="A3" s="140" t="inlineStr">
-        <is>
-          <t>✈️ Out:</t>
-        </is>
-      </c>
-      <c r="B3" s="82" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="C3" s="82" t="inlineStr">
-        <is>
-          <t>KE011</t>
-        </is>
-      </c>
-      <c r="D3" s="122">
-        <f>IF(C3="","",VLOOKUP(C3,'Master Data'!$A$60:$D$63,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E3" s="122">
-        <f>IF(C3="","",VLOOKUP(C3,'Master Data'!$A$60:$D$63,4,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F3" s="82" t="inlineStr">
-        <is>
-          <t>Economy</t>
-        </is>
-      </c>
-      <c r="G3" s="140" t="inlineStr">
-        <is>
-          <t>Ret:</t>
-        </is>
-      </c>
-      <c r="H3" s="82" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="I3" s="82" t="inlineStr">
-        <is>
-          <t>KE018</t>
-        </is>
-      </c>
-      <c r="J3" s="122">
-        <f>IF(I3="","",VLOOKUP(I3,'Master Data'!$A$74:$D$77,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="K3" s="122">
-        <f>IF(I3="","",VLOOKUP(I3,'Master Data'!$A$74:$D$77,4,FALSE))</f>
-        <v/>
-      </c>
+      <c r="A3" s="128" t="inlineStr">
+        <is>
+          <t>✈️ OUTBOUND</t>
+        </is>
+      </c>
+      <c r="B3" s="77" t="n"/>
+      <c r="C3" s="77" t="n"/>
+      <c r="D3" s="77" t="n"/>
+      <c r="E3" s="77" t="n"/>
+      <c r="F3" s="77" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="77" t="n"/>
+      <c r="I3" s="77" t="n"/>
+      <c r="J3" s="77" t="n"/>
+      <c r="K3" s="77" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="106" t="inlineStr">
         <is>
-          <t>Nights:</t>
-        </is>
-      </c>
-      <c r="B4" s="122">
-        <f>IF(AND(B3&lt;&gt;"",H3&lt;&gt;""),H3-B3,"")</f>
-        <v/>
-      </c>
-      <c r="C4" s="144">
-        <f>IF(B4&lt;&gt;"",B4+1,"")&amp;" days"</f>
-        <v/>
-      </c>
-      <c r="E4" s="106" t="inlineStr">
-        <is>
-          <t>Dup:</t>
-        </is>
-      </c>
-      <c r="F4" s="136">
-        <f>IF(SUM(R:R)&gt;0,"❌"&amp;SUM(R:R)&amp;"dup","✅")</f>
-        <v/>
-      </c>
-      <c r="H4" s="106" t="inlineStr">
-        <is>
-          <t>X-Ck:</t>
-        </is>
-      </c>
-      <c r="I4" s="133">
-        <f>J60</f>
-        <v/>
-      </c>
-      <c r="J4" s="133">
-        <f>B68</f>
-        <v/>
-      </c>
-      <c r="K4" s="136">
-        <f>IF(I4-J4=0,"✅MATCH","❌")</f>
-        <v/>
+          <t>Date:</t>
+        </is>
+      </c>
+      <c r="B4" s="82" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C4" s="106" t="inlineStr">
+        <is>
+          <t>Flight:</t>
+        </is>
+      </c>
+      <c r="D4" s="82" t="inlineStr">
+        <is>
+          <t>KE011</t>
+        </is>
+      </c>
+      <c r="E4" s="144">
+        <f>IF(D4="","",VLOOKUP(D4,'Master Data'!$A$60:$D$63,3,FALSE))&amp;" → "&amp;IF(D4="","",VLOOKUP(D4,'Master Data'!$A$60:$D$63,4,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F4" s="86" t="n"/>
+      <c r="G4" s="86" t="n"/>
+      <c r="H4" s="87" t="n"/>
+      <c r="I4" s="106" t="inlineStr">
+        <is>
+          <t>Seat:</t>
+        </is>
+      </c>
+      <c r="J4" s="82" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="119" t="inlineStr">
+      <c r="A5" s="128" t="inlineStr">
+        <is>
+          <t>✈️ RETURN</t>
+        </is>
+      </c>
+      <c r="B5" s="77" t="n"/>
+      <c r="C5" s="77" t="n"/>
+      <c r="D5" s="77" t="n"/>
+      <c r="E5" s="77" t="n"/>
+      <c r="F5" s="77" t="n"/>
+      <c r="G5" s="77" t="n"/>
+      <c r="H5" s="77" t="n"/>
+      <c r="I5" s="77" t="n"/>
+      <c r="J5" s="77" t="n"/>
+      <c r="K5" s="77" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="106" t="inlineStr">
+        <is>
+          <t>Date:</t>
+        </is>
+      </c>
+      <c r="B6" s="82" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="C6" s="106" t="inlineStr">
+        <is>
+          <t>Flight:</t>
+        </is>
+      </c>
+      <c r="D6" s="82" t="inlineStr">
+        <is>
+          <t>KE018</t>
+        </is>
+      </c>
+      <c r="E6" s="144">
+        <f>IF(D6="","",VLOOKUP(D6,'Master Data'!$A$74:$D$77,3,FALSE))&amp;" → "&amp;IF(D6="","",VLOOKUP(D6,'Master Data'!$A$74:$D$77,4,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F6" s="86" t="n"/>
+      <c r="G6" s="86" t="n"/>
+      <c r="H6" s="87" t="n"/>
+      <c r="I6" s="106" t="inlineStr">
+        <is>
+          <t>Duration:</t>
+        </is>
+      </c>
+      <c r="J6" s="144">
+        <f>IF(AND(B4&lt;&gt;"",B6&lt;&gt;""),B6-B4,"")&amp;"N "&amp;IF(B10&lt;&gt;"",B10+1,"")&amp;"D"</f>
+        <v/>
+      </c>
+      <c r="K6" s="87" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="106" t="inlineStr">
+        <is>
+          <t>Status:</t>
+        </is>
+      </c>
+      <c r="B7" s="136">
+        <f>IF(SUM(R:R)&gt;0,"❌"&amp;SUM(R:R)&amp;" dup","✅")</f>
+        <v/>
+      </c>
+      <c r="D7" s="106" t="inlineStr">
+        <is>
+          <t>X-Check:</t>
+        </is>
+      </c>
+      <c r="E7" s="133">
+        <f>J63</f>
+        <v/>
+      </c>
+      <c r="F7" s="81" t="inlineStr">
+        <is>
+          <t>vs</t>
+        </is>
+      </c>
+      <c r="G7" s="133">
+        <f>B71</f>
+        <v/>
+      </c>
+      <c r="H7" s="81" t="inlineStr">
+        <is>
+          <t>=</t>
+        </is>
+      </c>
+      <c r="I7" s="136">
+        <f>IF(E7-G7=0,"✅MATCH","❌")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="119" t="inlineStr">
         <is>
           <t>Item ▼</t>
         </is>
       </c>
-      <c r="B5" s="98" t="inlineStr">
+      <c r="B8" s="98" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="C5" s="98" t="inlineStr">
+      <c r="C8" s="98" t="inlineStr">
         <is>
           <t>Cost/P</t>
         </is>
       </c>
-      <c r="D5" s="98" t="inlineStr">
+      <c r="D8" s="98" t="inlineStr">
         <is>
           <t>Sell/P</t>
         </is>
       </c>
-      <c r="E5" s="98" t="inlineStr">
+      <c r="E8" s="98" t="inlineStr">
         <is>
           <t>M%</t>
         </is>
       </c>
-      <c r="F5" s="98">
+      <c r="F8" s="98">
         <f>F2</f>
         <v/>
       </c>
-      <c r="G5" s="98">
+      <c r="G8" s="98">
         <f>G2</f>
         <v/>
       </c>
-      <c r="H5" s="98">
+      <c r="H8" s="98">
         <f>H2</f>
         <v/>
       </c>
-      <c r="I5" s="98">
+      <c r="I8" s="98">
         <f>I2</f>
         <v/>
       </c>
-      <c r="J5" s="98" t="inlineStr">
+      <c r="J8" s="98" t="inlineStr">
         <is>
           <t>TotCost</t>
         </is>
       </c>
-      <c r="K5" s="98" t="inlineStr">
+      <c r="K8" s="98" t="inlineStr">
         <is>
           <t>TotSell</t>
         </is>
       </c>
-      <c r="L5" s="98" t="inlineStr">
+      <c r="L8" s="98" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="M5" s="98" t="inlineStr">
+      <c r="M8" s="98" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
-      <c r="N5" s="98" t="inlineStr">
+      <c r="N8" s="98" t="inlineStr">
         <is>
           <t>P7</t>
         </is>
       </c>
-      <c r="O5" s="98" t="inlineStr">
+      <c r="O8" s="98" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
       </c>
-      <c r="P5" s="98" t="inlineStr">
+      <c r="P8" s="98" t="inlineStr">
         <is>
           <t>Dup</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="128" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="128" t="inlineStr">
         <is>
           <t>⛳ GOLF</t>
         </is>
       </c>
-      <c r="B6" s="77" t="n"/>
-      <c r="C6" s="77" t="n"/>
-      <c r="D6" s="77" t="n"/>
-      <c r="E6" s="77" t="n"/>
-      <c r="F6" s="77" t="n"/>
-      <c r="G6" s="77" t="n"/>
-      <c r="H6" s="77" t="n"/>
-      <c r="I6" s="77" t="n"/>
-      <c r="J6" s="77" t="n"/>
-      <c r="K6" s="77" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="109" t="inlineStr">
+      <c r="B9" s="77" t="n"/>
+      <c r="C9" s="77" t="n"/>
+      <c r="D9" s="77" t="n"/>
+      <c r="E9" s="77" t="n"/>
+      <c r="F9" s="77" t="n"/>
+      <c r="G9" s="77" t="n"/>
+      <c r="H9" s="77" t="n"/>
+      <c r="I9" s="77" t="n"/>
+      <c r="J9" s="77" t="n"/>
+      <c r="K9" s="77" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="109" t="inlineStr">
         <is>
           <t>Hidden Valley GC</t>
         </is>
       </c>
-      <c r="B7" s="83" t="n">
+      <c r="B10" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="84">
-        <f>IF(A7="","",VLOOKUP(A7,'Master Data'!$A$7:$C$14,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D7" s="84">
-        <f>IF(A7="","",VLOOKUP(A7,'Master Data'!$A$7:$C$14,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E7" s="137">
-        <f>IF(D7&gt;0,(D7-C7)/D7,0)</f>
-        <v/>
-      </c>
-      <c r="F7" s="145" t="inlineStr"/>
-      <c r="G7" s="145" t="inlineStr"/>
-      <c r="H7" s="145" t="inlineStr"/>
-      <c r="I7" s="145" t="inlineStr"/>
-      <c r="J7" s="84">
-        <f>IF(A7="","",(COUNTIF(F7,"●")+COUNTIF(G7,"●")+COUNTIF(H7,"●")+COUNTIF(I7,"●")+COUNTIF(L7,"●")+COUNTIF(M7,"●")+COUNTIF(N7,"●")+COUNTIF(O7,"●"))*B7*C7)</f>
-        <v/>
-      </c>
-      <c r="K7" s="84">
-        <f>IF(A7="","",(COUNTIF(F7,"●")+COUNTIF(G7,"●")+COUNTIF(H7,"●")+COUNTIF(I7,"●")+COUNTIF(L7,"●")+COUNTIF(M7,"●")+COUNTIF(N7,"●")+COUNTIF(O7,"●"))*B7*D7)</f>
-        <v/>
-      </c>
-      <c r="L7" s="145" t="inlineStr"/>
-      <c r="M7" s="145" t="inlineStr"/>
-      <c r="N7" s="145" t="inlineStr"/>
-      <c r="O7" s="145" t="inlineStr"/>
-      <c r="P7" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="108" t="inlineStr">
-        <is>
-          <t>Sandpiper GC</t>
-        </is>
-      </c>
-      <c r="B8" s="83" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" s="84">
-        <f>IF(A8="","",VLOOKUP(A8,'Master Data'!$A$7:$C$14,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D8" s="84">
-        <f>IF(A8="","",VLOOKUP(A8,'Master Data'!$A$7:$C$14,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E8" s="137">
-        <f>IF(D8&gt;0,(D8-C8)/D8,0)</f>
-        <v/>
-      </c>
-      <c r="F8" s="145" t="inlineStr"/>
-      <c r="G8" s="145" t="inlineStr"/>
-      <c r="H8" s="145" t="inlineStr"/>
-      <c r="I8" s="145" t="inlineStr"/>
-      <c r="J8" s="84">
-        <f>IF(A8="","",(COUNTIF(F8,"●")+COUNTIF(G8,"●")+COUNTIF(H8,"●")+COUNTIF(I8,"●")+COUNTIF(L8,"●")+COUNTIF(M8,"●")+COUNTIF(N8,"●")+COUNTIF(O8,"●"))*B8*C8)</f>
-        <v/>
-      </c>
-      <c r="K8" s="84">
-        <f>IF(A8="","",(COUNTIF(F8,"●")+COUNTIF(G8,"●")+COUNTIF(H8,"●")+COUNTIF(I8,"●")+COUNTIF(L8,"●")+COUNTIF(M8,"●")+COUNTIF(N8,"●")+COUNTIF(O8,"●"))*B8*D8)</f>
-        <v/>
-      </c>
-      <c r="L8" s="145" t="inlineStr"/>
-      <c r="M8" s="145" t="inlineStr"/>
-      <c r="N8" s="145" t="inlineStr"/>
-      <c r="O8" s="145" t="inlineStr"/>
-      <c r="P8" s="81">
-        <f>IF(A8="",0,COUNTIF(A$7:A7,A8))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="109" t="inlineStr">
-        <is>
-          <t>Trump National LA</t>
-        </is>
-      </c>
-      <c r="B9" s="83" t="n">
-        <v>2</v>
-      </c>
-      <c r="C9" s="84">
-        <f>IF(A9="","",VLOOKUP(A9,'Master Data'!$A$7:$C$14,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D9" s="84">
-        <f>IF(A9="","",VLOOKUP(A9,'Master Data'!$A$7:$C$14,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E9" s="137">
-        <f>IF(D9&gt;0,(D9-C9)/D9,0)</f>
-        <v/>
-      </c>
-      <c r="F9" s="145" t="inlineStr"/>
-      <c r="G9" s="145" t="inlineStr"/>
-      <c r="H9" s="145" t="inlineStr"/>
-      <c r="I9" s="145" t="inlineStr"/>
-      <c r="J9" s="84">
-        <f>IF(A9="","",(COUNTIF(F9,"●")+COUNTIF(G9,"●")+COUNTIF(H9,"●")+COUNTIF(I9,"●")+COUNTIF(L9,"●")+COUNTIF(M9,"●")+COUNTIF(N9,"●")+COUNTIF(O9,"●"))*B9*C9)</f>
-        <v/>
-      </c>
-      <c r="K9" s="84">
-        <f>IF(A9="","",(COUNTIF(F9,"●")+COUNTIF(G9,"●")+COUNTIF(H9,"●")+COUNTIF(I9,"●")+COUNTIF(L9,"●")+COUNTIF(M9,"●")+COUNTIF(N9,"●")+COUNTIF(O9,"●"))*B9*D9)</f>
-        <v/>
-      </c>
-      <c r="L9" s="145" t="inlineStr"/>
-      <c r="M9" s="145" t="inlineStr"/>
-      <c r="N9" s="145" t="inlineStr"/>
-      <c r="O9" s="145" t="inlineStr"/>
-      <c r="P9" s="81">
-        <f>IF(A9="",0,COUNTIF(A$7:A8,A9))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="129" t="inlineStr"/>
-      <c r="B10" s="83" t="inlineStr"/>
       <c r="C10" s="84">
         <f>IF(A10="","",VLOOKUP(A10,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
@@ -3808,13 +3737,19 @@
       <c r="N10" s="145" t="inlineStr"/>
       <c r="O10" s="145" t="inlineStr"/>
       <c r="P10" s="81">
-        <f>IF(A10="",0,COUNTIF(A$7:A9,A10))</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="129" t="inlineStr"/>
-      <c r="B11" s="83" t="inlineStr"/>
+      <c r="A11" s="108" t="inlineStr">
+        <is>
+          <t>Sandpiper GC</t>
+        </is>
+      </c>
+      <c r="B11" s="83" t="n">
+        <v>2</v>
+      </c>
       <c r="C11" s="84">
         <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
@@ -3844,572 +3779,560 @@
       <c r="N11" s="145" t="inlineStr"/>
       <c r="O11" s="145" t="inlineStr"/>
       <c r="P11" s="81">
-        <f>IF(A11="",0,COUNTIF(A$7:A10,A11))</f>
+        <f>IF(A11="",0,COUNTIF(A$10:A10,A11))</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="123" t="inlineStr">
+      <c r="A12" s="109" t="inlineStr">
+        <is>
+          <t>Trump National LA</t>
+        </is>
+      </c>
+      <c r="B12" s="83" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="84">
+        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D12" s="84">
+        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E12" s="137">
+        <f>IF(D12&gt;0,(D12-C12)/D12,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="145" t="inlineStr"/>
+      <c r="G12" s="145" t="inlineStr"/>
+      <c r="H12" s="145" t="inlineStr"/>
+      <c r="I12" s="145" t="inlineStr"/>
+      <c r="J12" s="84">
+        <f>IF(A12="","",(COUNTIF(F12,"●")+COUNTIF(G12,"●")+COUNTIF(H12,"●")+COUNTIF(I12,"●")+COUNTIF(L12,"●")+COUNTIF(M12,"●")+COUNTIF(N12,"●")+COUNTIF(O12,"●"))*B12*C12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="84">
+        <f>IF(A12="","",(COUNTIF(F12,"●")+COUNTIF(G12,"●")+COUNTIF(H12,"●")+COUNTIF(I12,"●")+COUNTIF(L12,"●")+COUNTIF(M12,"●")+COUNTIF(N12,"●")+COUNTIF(O12,"●"))*B12*D12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="145" t="inlineStr"/>
+      <c r="M12" s="145" t="inlineStr"/>
+      <c r="N12" s="145" t="inlineStr"/>
+      <c r="O12" s="145" t="inlineStr"/>
+      <c r="P12" s="81">
+        <f>IF(A12="",0,COUNTIF(A$10:A11,A12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="129" t="inlineStr"/>
+      <c r="B13" s="83" t="inlineStr"/>
+      <c r="C13" s="84">
+        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D13" s="84">
+        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E13" s="137">
+        <f>IF(D13&gt;0,(D13-C13)/D13,0)</f>
+        <v/>
+      </c>
+      <c r="F13" s="145" t="inlineStr"/>
+      <c r="G13" s="145" t="inlineStr"/>
+      <c r="H13" s="145" t="inlineStr"/>
+      <c r="I13" s="145" t="inlineStr"/>
+      <c r="J13" s="84">
+        <f>IF(A13="","",(COUNTIF(F13,"●")+COUNTIF(G13,"●")+COUNTIF(H13,"●")+COUNTIF(I13,"●")+COUNTIF(L13,"●")+COUNTIF(M13,"●")+COUNTIF(N13,"●")+COUNTIF(O13,"●"))*B13*C13)</f>
+        <v/>
+      </c>
+      <c r="K13" s="84">
+        <f>IF(A13="","",(COUNTIF(F13,"●")+COUNTIF(G13,"●")+COUNTIF(H13,"●")+COUNTIF(I13,"●")+COUNTIF(L13,"●")+COUNTIF(M13,"●")+COUNTIF(N13,"●")+COUNTIF(O13,"●"))*B13*D13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="145" t="inlineStr"/>
+      <c r="M13" s="145" t="inlineStr"/>
+      <c r="N13" s="145" t="inlineStr"/>
+      <c r="O13" s="145" t="inlineStr"/>
+      <c r="P13" s="81">
+        <f>IF(A13="",0,COUNTIF(A$10:A12,A13))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="129" t="inlineStr"/>
+      <c r="B14" s="83" t="inlineStr"/>
+      <c r="C14" s="84">
+        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D14" s="84">
+        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E14" s="137">
+        <f>IF(D14&gt;0,(D14-C14)/D14,0)</f>
+        <v/>
+      </c>
+      <c r="F14" s="145" t="inlineStr"/>
+      <c r="G14" s="145" t="inlineStr"/>
+      <c r="H14" s="145" t="inlineStr"/>
+      <c r="I14" s="145" t="inlineStr"/>
+      <c r="J14" s="84">
+        <f>IF(A14="","",(COUNTIF(F14,"●")+COUNTIF(G14,"●")+COUNTIF(H14,"●")+COUNTIF(I14,"●")+COUNTIF(L14,"●")+COUNTIF(M14,"●")+COUNTIF(N14,"●")+COUNTIF(O14,"●"))*B14*C14)</f>
+        <v/>
+      </c>
+      <c r="K14" s="84">
+        <f>IF(A14="","",(COUNTIF(F14,"●")+COUNTIF(G14,"●")+COUNTIF(H14,"●")+COUNTIF(I14,"●")+COUNTIF(L14,"●")+COUNTIF(M14,"●")+COUNTIF(N14,"●")+COUNTIF(O14,"●"))*B14*D14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="145" t="inlineStr"/>
+      <c r="M14" s="145" t="inlineStr"/>
+      <c r="N14" s="145" t="inlineStr"/>
+      <c r="O14" s="145" t="inlineStr"/>
+      <c r="P14" s="81">
+        <f>IF(A14="",0,COUNTIF(A$10:A13,A14))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B12" s="114" t="inlineStr"/>
-      <c r="C12" s="114" t="inlineStr"/>
-      <c r="D12" s="114" t="inlineStr"/>
-      <c r="E12" s="114" t="inlineStr"/>
-      <c r="F12" s="130">
-        <f>SUMPRODUCT((F7:F11="●")*1,B7:B11,C7:C11)</f>
-        <v/>
-      </c>
-      <c r="G12" s="130">
-        <f>SUMPRODUCT((G7:G11="●")*1,B7:B11,C7:C11)</f>
-        <v/>
-      </c>
-      <c r="H12" s="130">
-        <f>SUMPRODUCT((H7:H11="●")*1,B7:B11,C7:C11)</f>
-        <v/>
-      </c>
-      <c r="I12" s="130">
-        <f>SUMPRODUCT((I7:I11="●")*1,B7:B11,C7:C11)</f>
-        <v/>
-      </c>
-      <c r="J12" s="88">
-        <f>SUM(J7:J11)</f>
-        <v/>
-      </c>
-      <c r="K12" s="88">
-        <f>SUM(K7:K11)</f>
-        <v/>
-      </c>
-      <c r="L12" s="130">
-        <f>SUMPRODUCT((L7:L11="●")*1,B7:B11,C7:C11)</f>
-        <v/>
-      </c>
-      <c r="M12" s="130">
-        <f>SUMPRODUCT((M7:M11="●")*1,B7:B11,C7:C11)</f>
-        <v/>
-      </c>
-      <c r="N12" s="130">
-        <f>SUMPRODUCT((N7:N11="●")*1,B7:B11,C7:C11)</f>
-        <v/>
-      </c>
-      <c r="O12" s="130">
-        <f>SUMPRODUCT((O7:O11="●")*1,B7:B11,C7:C11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="128" t="inlineStr">
+      <c r="B15" s="114" t="inlineStr"/>
+      <c r="C15" s="114" t="inlineStr"/>
+      <c r="D15" s="114" t="inlineStr"/>
+      <c r="E15" s="114" t="inlineStr"/>
+      <c r="F15" s="130">
+        <f>SUMPRODUCT((F10:F14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="130">
+        <f>SUMPRODUCT((G10:G14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="130">
+        <f>SUMPRODUCT((H10:H14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="I15" s="130">
+        <f>SUMPRODUCT((I10:I14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="J15" s="88">
+        <f>SUM(J10:J14)</f>
+        <v/>
+      </c>
+      <c r="K15" s="88">
+        <f>SUM(K10:K14)</f>
+        <v/>
+      </c>
+      <c r="L15" s="130">
+        <f>SUMPRODUCT((L10:L14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="M15" s="130">
+        <f>SUMPRODUCT((M10:M14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="N15" s="130">
+        <f>SUMPRODUCT((N10:N14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="O15" s="130">
+        <f>SUMPRODUCT((O10:O14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="128" t="inlineStr">
         <is>
           <t>🏨 HOTEL</t>
         </is>
       </c>
-      <c r="B14" s="77" t="n"/>
-      <c r="C14" s="77" t="n"/>
-      <c r="D14" s="77" t="n"/>
-      <c r="E14" s="77" t="n"/>
-      <c r="F14" s="77" t="n"/>
-      <c r="G14" s="77" t="n"/>
-      <c r="H14" s="77" t="n"/>
-      <c r="I14" s="77" t="n"/>
-      <c r="J14" s="77" t="n"/>
-      <c r="K14" s="77" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="109" t="inlineStr">
+      <c r="B17" s="77" t="n"/>
+      <c r="C17" s="77" t="n"/>
+      <c r="D17" s="77" t="n"/>
+      <c r="E17" s="77" t="n"/>
+      <c r="F17" s="77" t="n"/>
+      <c r="G17" s="77" t="n"/>
+      <c r="H17" s="77" t="n"/>
+      <c r="I17" s="77" t="n"/>
+      <c r="J17" s="77" t="n"/>
+      <c r="K17" s="77" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="109" t="inlineStr">
         <is>
           <t>Beverly Wilshire (5★) / Same Tier</t>
         </is>
       </c>
-      <c r="B15" s="83" t="n">
+      <c r="B18" s="83" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="84">
-        <f>IF(A15="","",VLOOKUP(A15,'Master Data'!$A$19:$C$24,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D15" s="84">
-        <f>IF(A15="","",VLOOKUP(A15,'Master Data'!$A$19:$C$24,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E15" s="137">
-        <f>IF(D15&gt;0,(D15-C15)/D15,0)</f>
-        <v/>
-      </c>
-      <c r="F15" s="145" t="inlineStr"/>
-      <c r="G15" s="145" t="inlineStr"/>
-      <c r="H15" s="145" t="inlineStr"/>
-      <c r="I15" s="145" t="inlineStr"/>
-      <c r="J15" s="84">
-        <f>IF(A15="","",(COUNTIF(F15,"●")+COUNTIF(G15,"●")+COUNTIF(H15,"●")+COUNTIF(I15,"●")+COUNTIF(L15,"●")+COUNTIF(M15,"●")+COUNTIF(N15,"●")+COUNTIF(O15,"●"))*B15*C15)</f>
-        <v/>
-      </c>
-      <c r="K15" s="84">
-        <f>IF(A15="","",(COUNTIF(F15,"●")+COUNTIF(G15,"●")+COUNTIF(H15,"●")+COUNTIF(I15,"●")+COUNTIF(L15,"●")+COUNTIF(M15,"●")+COUNTIF(N15,"●")+COUNTIF(O15,"●"))*B15*D15)</f>
-        <v/>
-      </c>
-      <c r="L15" s="145" t="inlineStr"/>
-      <c r="M15" s="145" t="inlineStr"/>
-      <c r="N15" s="145" t="inlineStr"/>
-      <c r="O15" s="145" t="inlineStr"/>
-      <c r="P15" s="81">
+      <c r="C18" s="84">
+        <f>IF(A18="","",VLOOKUP(A18,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D18" s="84">
+        <f>IF(A18="","",VLOOKUP(A18,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E18" s="137">
+        <f>IF(D18&gt;0,(D18-C18)/D18,0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="145" t="inlineStr"/>
+      <c r="G18" s="145" t="inlineStr"/>
+      <c r="H18" s="145" t="inlineStr"/>
+      <c r="I18" s="145" t="inlineStr"/>
+      <c r="J18" s="84">
+        <f>IF(A18="","",(COUNTIF(F18,"●")+COUNTIF(G18,"●")+COUNTIF(H18,"●")+COUNTIF(I18,"●")+COUNTIF(L18,"●")+COUNTIF(M18,"●")+COUNTIF(N18,"●")+COUNTIF(O18,"●"))*B18*C18)</f>
+        <v/>
+      </c>
+      <c r="K18" s="84">
+        <f>IF(A18="","",(COUNTIF(F18,"●")+COUNTIF(G18,"●")+COUNTIF(H18,"●")+COUNTIF(I18,"●")+COUNTIF(L18,"●")+COUNTIF(M18,"●")+COUNTIF(N18,"●")+COUNTIF(O18,"●"))*B18*D18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="145" t="inlineStr"/>
+      <c r="M18" s="145" t="inlineStr"/>
+      <c r="N18" s="145" t="inlineStr"/>
+      <c r="O18" s="145" t="inlineStr"/>
+      <c r="P18" s="81">
         <f>0</f>
         <v/>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="129" t="inlineStr"/>
-      <c r="B16" s="83" t="inlineStr"/>
-      <c r="C16" s="84">
-        <f>IF(A16="","",VLOOKUP(A16,'Master Data'!$A$19:$C$24,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D16" s="84">
-        <f>IF(A16="","",VLOOKUP(A16,'Master Data'!$A$19:$C$24,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E16" s="137">
-        <f>IF(D16&gt;0,(D16-C16)/D16,0)</f>
-        <v/>
-      </c>
-      <c r="F16" s="145" t="inlineStr"/>
-      <c r="G16" s="145" t="inlineStr"/>
-      <c r="H16" s="145" t="inlineStr"/>
-      <c r="I16" s="145" t="inlineStr"/>
-      <c r="J16" s="84">
-        <f>IF(A16="","",(COUNTIF(F16,"●")+COUNTIF(G16,"●")+COUNTIF(H16,"●")+COUNTIF(I16,"●")+COUNTIF(L16,"●")+COUNTIF(M16,"●")+COUNTIF(N16,"●")+COUNTIF(O16,"●"))*B16*C16)</f>
-        <v/>
-      </c>
-      <c r="K16" s="84">
-        <f>IF(A16="","",(COUNTIF(F16,"●")+COUNTIF(G16,"●")+COUNTIF(H16,"●")+COUNTIF(I16,"●")+COUNTIF(L16,"●")+COUNTIF(M16,"●")+COUNTIF(N16,"●")+COUNTIF(O16,"●"))*B16*D16)</f>
-        <v/>
-      </c>
-      <c r="L16" s="145" t="inlineStr"/>
-      <c r="M16" s="145" t="inlineStr"/>
-      <c r="N16" s="145" t="inlineStr"/>
-      <c r="O16" s="145" t="inlineStr"/>
-      <c r="P16" s="81">
-        <f>IF(A16="",0,COUNTIF(A$15:A15,A16))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="129" t="inlineStr"/>
-      <c r="B17" s="83" t="inlineStr"/>
-      <c r="C17" s="84">
-        <f>IF(A17="","",VLOOKUP(A17,'Master Data'!$A$19:$C$24,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D17" s="84">
-        <f>IF(A17="","",VLOOKUP(A17,'Master Data'!$A$19:$C$24,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E17" s="137">
-        <f>IF(D17&gt;0,(D17-C17)/D17,0)</f>
-        <v/>
-      </c>
-      <c r="F17" s="145" t="inlineStr"/>
-      <c r="G17" s="145" t="inlineStr"/>
-      <c r="H17" s="145" t="inlineStr"/>
-      <c r="I17" s="145" t="inlineStr"/>
-      <c r="J17" s="84">
-        <f>IF(A17="","",(COUNTIF(F17,"●")+COUNTIF(G17,"●")+COUNTIF(H17,"●")+COUNTIF(I17,"●")+COUNTIF(L17,"●")+COUNTIF(M17,"●")+COUNTIF(N17,"●")+COUNTIF(O17,"●"))*B17*C17)</f>
-        <v/>
-      </c>
-      <c r="K17" s="84">
-        <f>IF(A17="","",(COUNTIF(F17,"●")+COUNTIF(G17,"●")+COUNTIF(H17,"●")+COUNTIF(I17,"●")+COUNTIF(L17,"●")+COUNTIF(M17,"●")+COUNTIF(N17,"●")+COUNTIF(O17,"●"))*B17*D17)</f>
-        <v/>
-      </c>
-      <c r="L17" s="145" t="inlineStr"/>
-      <c r="M17" s="145" t="inlineStr"/>
-      <c r="N17" s="145" t="inlineStr"/>
-      <c r="O17" s="145" t="inlineStr"/>
-      <c r="P17" s="81">
-        <f>IF(A17="",0,COUNTIF(A$15:A16,A17))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="123" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="129" t="inlineStr"/>
+      <c r="B19" s="83" t="inlineStr"/>
+      <c r="C19" s="84">
+        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D19" s="84">
+        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E19" s="137">
+        <f>IF(D19&gt;0,(D19-C19)/D19,0)</f>
+        <v/>
+      </c>
+      <c r="F19" s="145" t="inlineStr"/>
+      <c r="G19" s="145" t="inlineStr"/>
+      <c r="H19" s="145" t="inlineStr"/>
+      <c r="I19" s="145" t="inlineStr"/>
+      <c r="J19" s="84">
+        <f>IF(A19="","",(COUNTIF(F19,"●")+COUNTIF(G19,"●")+COUNTIF(H19,"●")+COUNTIF(I19,"●")+COUNTIF(L19,"●")+COUNTIF(M19,"●")+COUNTIF(N19,"●")+COUNTIF(O19,"●"))*B19*C19)</f>
+        <v/>
+      </c>
+      <c r="K19" s="84">
+        <f>IF(A19="","",(COUNTIF(F19,"●")+COUNTIF(G19,"●")+COUNTIF(H19,"●")+COUNTIF(I19,"●")+COUNTIF(L19,"●")+COUNTIF(M19,"●")+COUNTIF(N19,"●")+COUNTIF(O19,"●"))*B19*D19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="145" t="inlineStr"/>
+      <c r="M19" s="145" t="inlineStr"/>
+      <c r="N19" s="145" t="inlineStr"/>
+      <c r="O19" s="145" t="inlineStr"/>
+      <c r="P19" s="81">
+        <f>IF(A19="",0,COUNTIF(A$18:A18,A19))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="129" t="inlineStr"/>
+      <c r="B20" s="83" t="inlineStr"/>
+      <c r="C20" s="84">
+        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D20" s="84">
+        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E20" s="137">
+        <f>IF(D20&gt;0,(D20-C20)/D20,0)</f>
+        <v/>
+      </c>
+      <c r="F20" s="145" t="inlineStr"/>
+      <c r="G20" s="145" t="inlineStr"/>
+      <c r="H20" s="145" t="inlineStr"/>
+      <c r="I20" s="145" t="inlineStr"/>
+      <c r="J20" s="84">
+        <f>IF(A20="","",(COUNTIF(F20,"●")+COUNTIF(G20,"●")+COUNTIF(H20,"●")+COUNTIF(I20,"●")+COUNTIF(L20,"●")+COUNTIF(M20,"●")+COUNTIF(N20,"●")+COUNTIF(O20,"●"))*B20*C20)</f>
+        <v/>
+      </c>
+      <c r="K20" s="84">
+        <f>IF(A20="","",(COUNTIF(F20,"●")+COUNTIF(G20,"●")+COUNTIF(H20,"●")+COUNTIF(I20,"●")+COUNTIF(L20,"●")+COUNTIF(M20,"●")+COUNTIF(N20,"●")+COUNTIF(O20,"●"))*B20*D20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="145" t="inlineStr"/>
+      <c r="M20" s="145" t="inlineStr"/>
+      <c r="N20" s="145" t="inlineStr"/>
+      <c r="O20" s="145" t="inlineStr"/>
+      <c r="P20" s="81">
+        <f>IF(A20="",0,COUNTIF(A$18:A19,A20))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B18" s="114" t="inlineStr"/>
-      <c r="C18" s="114" t="inlineStr"/>
-      <c r="D18" s="114" t="inlineStr"/>
-      <c r="E18" s="114" t="inlineStr"/>
-      <c r="F18" s="130">
-        <f>SUMPRODUCT((F15:F17="●")*1,B15:B17,C15:C17)</f>
-        <v/>
-      </c>
-      <c r="G18" s="130">
-        <f>SUMPRODUCT((G15:G17="●")*1,B15:B17,C15:C17)</f>
-        <v/>
-      </c>
-      <c r="H18" s="130">
-        <f>SUMPRODUCT((H15:H17="●")*1,B15:B17,C15:C17)</f>
-        <v/>
-      </c>
-      <c r="I18" s="130">
-        <f>SUMPRODUCT((I15:I17="●")*1,B15:B17,C15:C17)</f>
-        <v/>
-      </c>
-      <c r="J18" s="88">
-        <f>SUM(J15:J17)</f>
-        <v/>
-      </c>
-      <c r="K18" s="88">
-        <f>SUM(K15:K17)</f>
-        <v/>
-      </c>
-      <c r="L18" s="130">
-        <f>SUMPRODUCT((L15:L17="●")*1,B15:B17,C15:C17)</f>
-        <v/>
-      </c>
-      <c r="M18" s="130">
-        <f>SUMPRODUCT((M15:M17="●")*1,B15:B17,C15:C17)</f>
-        <v/>
-      </c>
-      <c r="N18" s="130">
-        <f>SUMPRODUCT((N15:N17="●")*1,B15:B17,C15:C17)</f>
-        <v/>
-      </c>
-      <c r="O18" s="130">
-        <f>SUMPRODUCT((O15:O17="●")*1,B15:B17,C15:C17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="128" t="inlineStr">
+      <c r="B21" s="114" t="inlineStr"/>
+      <c r="C21" s="114" t="inlineStr"/>
+      <c r="D21" s="114" t="inlineStr"/>
+      <c r="E21" s="114" t="inlineStr"/>
+      <c r="F21" s="130">
+        <f>SUMPRODUCT((F18:F20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="G21" s="130">
+        <f>SUMPRODUCT((G18:G20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="H21" s="130">
+        <f>SUMPRODUCT((H18:H20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="I21" s="130">
+        <f>SUMPRODUCT((I18:I20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="J21" s="88">
+        <f>SUM(J18:J20)</f>
+        <v/>
+      </c>
+      <c r="K21" s="88">
+        <f>SUM(K18:K20)</f>
+        <v/>
+      </c>
+      <c r="L21" s="130">
+        <f>SUMPRODUCT((L18:L20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="M21" s="130">
+        <f>SUMPRODUCT((M18:M20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="N21" s="130">
+        <f>SUMPRODUCT((N18:N20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="O21" s="130">
+        <f>SUMPRODUCT((O18:O20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="128" t="inlineStr">
         <is>
           <t>🚐 TRANSPORT</t>
         </is>
       </c>
-      <c r="B20" s="77" t="n"/>
-      <c r="C20" s="77" t="n"/>
-      <c r="D20" s="77" t="n"/>
-      <c r="E20" s="77" t="n"/>
-      <c r="F20" s="77" t="n"/>
-      <c r="G20" s="77" t="n"/>
-      <c r="H20" s="77" t="n"/>
-      <c r="I20" s="77" t="n"/>
-      <c r="J20" s="77" t="n"/>
-      <c r="K20" s="77" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="109" t="inlineStr">
+      <c r="B23" s="77" t="n"/>
+      <c r="C23" s="77" t="n"/>
+      <c r="D23" s="77" t="n"/>
+      <c r="E23" s="77" t="n"/>
+      <c r="F23" s="77" t="n"/>
+      <c r="G23" s="77" t="n"/>
+      <c r="H23" s="77" t="n"/>
+      <c r="I23" s="77" t="n"/>
+      <c r="J23" s="77" t="n"/>
+      <c r="K23" s="77" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="109" t="inlineStr">
         <is>
           <t>Driver/Guide + Van (일당)</t>
         </is>
       </c>
-      <c r="B21" s="83" t="n">
+      <c r="B24" s="83" t="n">
         <v>3</v>
       </c>
-      <c r="C21" s="84">
-        <f>IF(A21="","",VLOOKUP(A21,'Master Data'!$A$28:$C$34,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D21" s="84">
-        <f>IF(A21="","",VLOOKUP(A21,'Master Data'!$A$28:$C$34,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E21" s="137">
-        <f>IF(D21&gt;0,(D21-C21)/D21,0)</f>
-        <v/>
-      </c>
-      <c r="F21" s="145" t="inlineStr"/>
-      <c r="G21" s="145" t="inlineStr"/>
-      <c r="H21" s="145" t="inlineStr"/>
-      <c r="I21" s="145" t="inlineStr"/>
-      <c r="J21" s="84">
-        <f>IF(A21="","",(COUNTIF(F21,"●")+COUNTIF(G21,"●")+COUNTIF(H21,"●")+COUNTIF(I21,"●")+COUNTIF(L21,"●")+COUNTIF(M21,"●")+COUNTIF(N21,"●")+COUNTIF(O21,"●"))*B21*C21)</f>
-        <v/>
-      </c>
-      <c r="K21" s="84">
-        <f>IF(A21="","",(COUNTIF(F21,"●")+COUNTIF(G21,"●")+COUNTIF(H21,"●")+COUNTIF(I21,"●")+COUNTIF(L21,"●")+COUNTIF(M21,"●")+COUNTIF(N21,"●")+COUNTIF(O21,"●"))*B21*D21)</f>
-        <v/>
-      </c>
-      <c r="L21" s="145" t="inlineStr"/>
-      <c r="M21" s="145" t="inlineStr"/>
-      <c r="N21" s="145" t="inlineStr"/>
-      <c r="O21" s="145" t="inlineStr"/>
-      <c r="P21" s="81">
+      <c r="C24" s="84">
+        <f>IF(A24="","",VLOOKUP(A24,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D24" s="84">
+        <f>IF(A24="","",VLOOKUP(A24,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E24" s="137">
+        <f>IF(D24&gt;0,(D24-C24)/D24,0)</f>
+        <v/>
+      </c>
+      <c r="F24" s="145" t="inlineStr"/>
+      <c r="G24" s="145" t="inlineStr"/>
+      <c r="H24" s="145" t="inlineStr"/>
+      <c r="I24" s="145" t="inlineStr"/>
+      <c r="J24" s="84">
+        <f>IF(A24="","",(COUNTIF(F24,"●")+COUNTIF(G24,"●")+COUNTIF(H24,"●")+COUNTIF(I24,"●")+COUNTIF(L24,"●")+COUNTIF(M24,"●")+COUNTIF(N24,"●")+COUNTIF(O24,"●"))*B24*C24)</f>
+        <v/>
+      </c>
+      <c r="K24" s="84">
+        <f>IF(A24="","",(COUNTIF(F24,"●")+COUNTIF(G24,"●")+COUNTIF(H24,"●")+COUNTIF(I24,"●")+COUNTIF(L24,"●")+COUNTIF(M24,"●")+COUNTIF(N24,"●")+COUNTIF(O24,"●"))*B24*D24)</f>
+        <v/>
+      </c>
+      <c r="L24" s="145" t="inlineStr"/>
+      <c r="M24" s="145" t="inlineStr"/>
+      <c r="N24" s="145" t="inlineStr"/>
+      <c r="O24" s="145" t="inlineStr"/>
+      <c r="P24" s="81">
         <f>0</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="129" t="inlineStr"/>
-      <c r="B22" s="83" t="inlineStr"/>
-      <c r="C22" s="84">
-        <f>IF(A22="","",VLOOKUP(A22,'Master Data'!$A$28:$C$34,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D22" s="84">
-        <f>IF(A22="","",VLOOKUP(A22,'Master Data'!$A$28:$C$34,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E22" s="137">
-        <f>IF(D22&gt;0,(D22-C22)/D22,0)</f>
-        <v/>
-      </c>
-      <c r="F22" s="145" t="inlineStr"/>
-      <c r="G22" s="145" t="inlineStr"/>
-      <c r="H22" s="145" t="inlineStr"/>
-      <c r="I22" s="145" t="inlineStr"/>
-      <c r="J22" s="84">
-        <f>IF(A22="","",(COUNTIF(F22,"●")+COUNTIF(G22,"●")+COUNTIF(H22,"●")+COUNTIF(I22,"●")+COUNTIF(L22,"●")+COUNTIF(M22,"●")+COUNTIF(N22,"●")+COUNTIF(O22,"●"))*B22*C22)</f>
-        <v/>
-      </c>
-      <c r="K22" s="84">
-        <f>IF(A22="","",(COUNTIF(F22,"●")+COUNTIF(G22,"●")+COUNTIF(H22,"●")+COUNTIF(I22,"●")+COUNTIF(L22,"●")+COUNTIF(M22,"●")+COUNTIF(N22,"●")+COUNTIF(O22,"●"))*B22*D22)</f>
-        <v/>
-      </c>
-      <c r="L22" s="145" t="inlineStr"/>
-      <c r="M22" s="145" t="inlineStr"/>
-      <c r="N22" s="145" t="inlineStr"/>
-      <c r="O22" s="145" t="inlineStr"/>
-      <c r="P22" s="81">
-        <f>IF(A22="",0,COUNTIF(A$21:A21,A22))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="129" t="inlineStr"/>
-      <c r="B23" s="83" t="inlineStr"/>
-      <c r="C23" s="84">
-        <f>IF(A23="","",VLOOKUP(A23,'Master Data'!$A$28:$C$34,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D23" s="84">
-        <f>IF(A23="","",VLOOKUP(A23,'Master Data'!$A$28:$C$34,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E23" s="137">
-        <f>IF(D23&gt;0,(D23-C23)/D23,0)</f>
-        <v/>
-      </c>
-      <c r="F23" s="145" t="inlineStr"/>
-      <c r="G23" s="145" t="inlineStr"/>
-      <c r="H23" s="145" t="inlineStr"/>
-      <c r="I23" s="145" t="inlineStr"/>
-      <c r="J23" s="84">
-        <f>IF(A23="","",(COUNTIF(F23,"●")+COUNTIF(G23,"●")+COUNTIF(H23,"●")+COUNTIF(I23,"●")+COUNTIF(L23,"●")+COUNTIF(M23,"●")+COUNTIF(N23,"●")+COUNTIF(O23,"●"))*B23*C23)</f>
-        <v/>
-      </c>
-      <c r="K23" s="84">
-        <f>IF(A23="","",(COUNTIF(F23,"●")+COUNTIF(G23,"●")+COUNTIF(H23,"●")+COUNTIF(I23,"●")+COUNTIF(L23,"●")+COUNTIF(M23,"●")+COUNTIF(N23,"●")+COUNTIF(O23,"●"))*B23*D23)</f>
-        <v/>
-      </c>
-      <c r="L23" s="145" t="inlineStr"/>
-      <c r="M23" s="145" t="inlineStr"/>
-      <c r="N23" s="145" t="inlineStr"/>
-      <c r="O23" s="145" t="inlineStr"/>
-      <c r="P23" s="81">
-        <f>IF(A23="",0,COUNTIF(A$21:A22,A23))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="123" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="129" t="inlineStr"/>
+      <c r="B25" s="83" t="inlineStr"/>
+      <c r="C25" s="84">
+        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D25" s="84">
+        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E25" s="137">
+        <f>IF(D25&gt;0,(D25-C25)/D25,0)</f>
+        <v/>
+      </c>
+      <c r="F25" s="145" t="inlineStr"/>
+      <c r="G25" s="145" t="inlineStr"/>
+      <c r="H25" s="145" t="inlineStr"/>
+      <c r="I25" s="145" t="inlineStr"/>
+      <c r="J25" s="84">
+        <f>IF(A25="","",(COUNTIF(F25,"●")+COUNTIF(G25,"●")+COUNTIF(H25,"●")+COUNTIF(I25,"●")+COUNTIF(L25,"●")+COUNTIF(M25,"●")+COUNTIF(N25,"●")+COUNTIF(O25,"●"))*B25*C25)</f>
+        <v/>
+      </c>
+      <c r="K25" s="84">
+        <f>IF(A25="","",(COUNTIF(F25,"●")+COUNTIF(G25,"●")+COUNTIF(H25,"●")+COUNTIF(I25,"●")+COUNTIF(L25,"●")+COUNTIF(M25,"●")+COUNTIF(N25,"●")+COUNTIF(O25,"●"))*B25*D25)</f>
+        <v/>
+      </c>
+      <c r="L25" s="145" t="inlineStr"/>
+      <c r="M25" s="145" t="inlineStr"/>
+      <c r="N25" s="145" t="inlineStr"/>
+      <c r="O25" s="145" t="inlineStr"/>
+      <c r="P25" s="81">
+        <f>IF(A25="",0,COUNTIF(A$24:A24,A25))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="129" t="inlineStr"/>
+      <c r="B26" s="83" t="inlineStr"/>
+      <c r="C26" s="84">
+        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D26" s="84">
+        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E26" s="137">
+        <f>IF(D26&gt;0,(D26-C26)/D26,0)</f>
+        <v/>
+      </c>
+      <c r="F26" s="145" t="inlineStr"/>
+      <c r="G26" s="145" t="inlineStr"/>
+      <c r="H26" s="145" t="inlineStr"/>
+      <c r="I26" s="145" t="inlineStr"/>
+      <c r="J26" s="84">
+        <f>IF(A26="","",(COUNTIF(F26,"●")+COUNTIF(G26,"●")+COUNTIF(H26,"●")+COUNTIF(I26,"●")+COUNTIF(L26,"●")+COUNTIF(M26,"●")+COUNTIF(N26,"●")+COUNTIF(O26,"●"))*B26*C26)</f>
+        <v/>
+      </c>
+      <c r="K26" s="84">
+        <f>IF(A26="","",(COUNTIF(F26,"●")+COUNTIF(G26,"●")+COUNTIF(H26,"●")+COUNTIF(I26,"●")+COUNTIF(L26,"●")+COUNTIF(M26,"●")+COUNTIF(N26,"●")+COUNTIF(O26,"●"))*B26*D26)</f>
+        <v/>
+      </c>
+      <c r="L26" s="145" t="inlineStr"/>
+      <c r="M26" s="145" t="inlineStr"/>
+      <c r="N26" s="145" t="inlineStr"/>
+      <c r="O26" s="145" t="inlineStr"/>
+      <c r="P26" s="81">
+        <f>IF(A26="",0,COUNTIF(A$24:A25,A26))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B24" s="114" t="inlineStr"/>
-      <c r="C24" s="114" t="inlineStr"/>
-      <c r="D24" s="114" t="inlineStr"/>
-      <c r="E24" s="114" t="inlineStr"/>
-      <c r="F24" s="130">
-        <f>SUMPRODUCT((F21:F23="●")*1,B21:B23,C21:C23)</f>
-        <v/>
-      </c>
-      <c r="G24" s="130">
-        <f>SUMPRODUCT((G21:G23="●")*1,B21:B23,C21:C23)</f>
-        <v/>
-      </c>
-      <c r="H24" s="130">
-        <f>SUMPRODUCT((H21:H23="●")*1,B21:B23,C21:C23)</f>
-        <v/>
-      </c>
-      <c r="I24" s="130">
-        <f>SUMPRODUCT((I21:I23="●")*1,B21:B23,C21:C23)</f>
-        <v/>
-      </c>
-      <c r="J24" s="88">
-        <f>SUM(J21:J23)</f>
-        <v/>
-      </c>
-      <c r="K24" s="88">
-        <f>SUM(K21:K23)</f>
-        <v/>
-      </c>
-      <c r="L24" s="130">
-        <f>SUMPRODUCT((L21:L23="●")*1,B21:B23,C21:C23)</f>
-        <v/>
-      </c>
-      <c r="M24" s="130">
-        <f>SUMPRODUCT((M21:M23="●")*1,B21:B23,C21:C23)</f>
-        <v/>
-      </c>
-      <c r="N24" s="130">
-        <f>SUMPRODUCT((N21:N23="●")*1,B21:B23,C21:C23)</f>
-        <v/>
-      </c>
-      <c r="O24" s="130">
-        <f>SUMPRODUCT((O21:O23="●")*1,B21:B23,C21:C23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="128" t="inlineStr">
+      <c r="B27" s="114" t="inlineStr"/>
+      <c r="C27" s="114" t="inlineStr"/>
+      <c r="D27" s="114" t="inlineStr"/>
+      <c r="E27" s="114" t="inlineStr"/>
+      <c r="F27" s="130">
+        <f>SUMPRODUCT((F24:F26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="G27" s="130">
+        <f>SUMPRODUCT((G24:G26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="H27" s="130">
+        <f>SUMPRODUCT((H24:H26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="I27" s="130">
+        <f>SUMPRODUCT((I24:I26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="J27" s="88">
+        <f>SUM(J24:J26)</f>
+        <v/>
+      </c>
+      <c r="K27" s="88">
+        <f>SUM(K24:K26)</f>
+        <v/>
+      </c>
+      <c r="L27" s="130">
+        <f>SUMPRODUCT((L24:L26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="M27" s="130">
+        <f>SUMPRODUCT((M24:M26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="N27" s="130">
+        <f>SUMPRODUCT((N24:N26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="O27" s="130">
+        <f>SUMPRODUCT((O24:O26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="128" t="inlineStr">
         <is>
           <t>🍽️ MEALS</t>
         </is>
       </c>
-      <c r="B26" s="77" t="n"/>
-      <c r="C26" s="77" t="n"/>
-      <c r="D26" s="77" t="n"/>
-      <c r="E26" s="77" t="n"/>
-      <c r="F26" s="77" t="n"/>
-      <c r="G26" s="77" t="n"/>
-      <c r="H26" s="77" t="n"/>
-      <c r="I26" s="77" t="n"/>
-      <c r="J26" s="77" t="n"/>
-      <c r="K26" s="77" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="109" t="inlineStr">
+      <c r="B29" s="77" t="n"/>
+      <c r="C29" s="77" t="n"/>
+      <c r="D29" s="77" t="n"/>
+      <c r="E29" s="77" t="n"/>
+      <c r="F29" s="77" t="n"/>
+      <c r="G29" s="77" t="n"/>
+      <c r="H29" s="77" t="n"/>
+      <c r="I29" s="77" t="n"/>
+      <c r="J29" s="77" t="n"/>
+      <c r="K29" s="77" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="109" t="inlineStr">
         <is>
           <t>Breakfast (Hotel)</t>
-        </is>
-      </c>
-      <c r="B27" s="83" t="n">
-        <v>3</v>
-      </c>
-      <c r="C27" s="84">
-        <f>IF(A27="","",VLOOKUP(A27,'Master Data'!$A$38:$C$46,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D27" s="84">
-        <f>IF(A27="","",VLOOKUP(A27,'Master Data'!$A$38:$C$46,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E27" s="137">
-        <f>IF(D27&gt;0,(D27-C27)/D27,0)</f>
-        <v/>
-      </c>
-      <c r="F27" s="145" t="inlineStr"/>
-      <c r="G27" s="145" t="inlineStr"/>
-      <c r="H27" s="145" t="inlineStr"/>
-      <c r="I27" s="145" t="inlineStr"/>
-      <c r="J27" s="84">
-        <f>IF(A27="","",(COUNTIF(F27,"●")+COUNTIF(G27,"●")+COUNTIF(H27,"●")+COUNTIF(I27,"●")+COUNTIF(L27,"●")+COUNTIF(M27,"●")+COUNTIF(N27,"●")+COUNTIF(O27,"●"))*B27*C27)</f>
-        <v/>
-      </c>
-      <c r="K27" s="84">
-        <f>IF(A27="","",(COUNTIF(F27,"●")+COUNTIF(G27,"●")+COUNTIF(H27,"●")+COUNTIF(I27,"●")+COUNTIF(L27,"●")+COUNTIF(M27,"●")+COUNTIF(N27,"●")+COUNTIF(O27,"●"))*B27*D27)</f>
-        <v/>
-      </c>
-      <c r="L27" s="145" t="inlineStr"/>
-      <c r="M27" s="145" t="inlineStr"/>
-      <c r="N27" s="145" t="inlineStr"/>
-      <c r="O27" s="145" t="inlineStr"/>
-      <c r="P27" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="108" t="inlineStr">
-        <is>
-          <t>Dinner (Regular)</t>
-        </is>
-      </c>
-      <c r="B28" s="83" t="n">
-        <v>3</v>
-      </c>
-      <c r="C28" s="84">
-        <f>IF(A28="","",VLOOKUP(A28,'Master Data'!$A$38:$C$46,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D28" s="84">
-        <f>IF(A28="","",VLOOKUP(A28,'Master Data'!$A$38:$C$46,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E28" s="137">
-        <f>IF(D28&gt;0,(D28-C28)/D28,0)</f>
-        <v/>
-      </c>
-      <c r="F28" s="145" t="inlineStr"/>
-      <c r="G28" s="145" t="inlineStr"/>
-      <c r="H28" s="145" t="inlineStr"/>
-      <c r="I28" s="145" t="inlineStr"/>
-      <c r="J28" s="84">
-        <f>IF(A28="","",(COUNTIF(F28,"●")+COUNTIF(G28,"●")+COUNTIF(H28,"●")+COUNTIF(I28,"●")+COUNTIF(L28,"●")+COUNTIF(M28,"●")+COUNTIF(N28,"●")+COUNTIF(O28,"●"))*B28*C28)</f>
-        <v/>
-      </c>
-      <c r="K28" s="84">
-        <f>IF(A28="","",(COUNTIF(F28,"●")+COUNTIF(G28,"●")+COUNTIF(H28,"●")+COUNTIF(I28,"●")+COUNTIF(L28,"●")+COUNTIF(M28,"●")+COUNTIF(N28,"●")+COUNTIF(O28,"●"))*B28*D28)</f>
-        <v/>
-      </c>
-      <c r="L28" s="145" t="inlineStr"/>
-      <c r="M28" s="145" t="inlineStr"/>
-      <c r="N28" s="145" t="inlineStr"/>
-      <c r="O28" s="145" t="inlineStr"/>
-      <c r="P28" s="81">
-        <f>IF(A28="",0,COUNTIF(A$27:A27,A28))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="109" t="inlineStr">
-        <is>
-          <t>Exclusive Dinner (Michelin/Fine)</t>
-        </is>
-      </c>
-      <c r="B29" s="83" t="n">
-        <v>2</v>
-      </c>
-      <c r="C29" s="84">
-        <f>IF(A29="","",VLOOKUP(A29,'Master Data'!$A$38:$C$46,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D29" s="84">
-        <f>IF(A29="","",VLOOKUP(A29,'Master Data'!$A$38:$C$46,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E29" s="137">
-        <f>IF(D29&gt;0,(D29-C29)/D29,0)</f>
-        <v/>
-      </c>
-      <c r="F29" s="145" t="inlineStr"/>
-      <c r="G29" s="145" t="inlineStr"/>
-      <c r="H29" s="145" t="inlineStr"/>
-      <c r="I29" s="145" t="inlineStr"/>
-      <c r="J29" s="84">
-        <f>IF(A29="","",(COUNTIF(F29,"●")+COUNTIF(G29,"●")+COUNTIF(H29,"●")+COUNTIF(I29,"●")+COUNTIF(L29,"●")+COUNTIF(M29,"●")+COUNTIF(N29,"●")+COUNTIF(O29,"●"))*B29*C29)</f>
-        <v/>
-      </c>
-      <c r="K29" s="84">
-        <f>IF(A29="","",(COUNTIF(F29,"●")+COUNTIF(G29,"●")+COUNTIF(H29,"●")+COUNTIF(I29,"●")+COUNTIF(L29,"●")+COUNTIF(M29,"●")+COUNTIF(N29,"●")+COUNTIF(O29,"●"))*B29*D29)</f>
-        <v/>
-      </c>
-      <c r="L29" s="145" t="inlineStr"/>
-      <c r="M29" s="145" t="inlineStr"/>
-      <c r="N29" s="145" t="inlineStr"/>
-      <c r="O29" s="145" t="inlineStr"/>
-      <c r="P29" s="81">
-        <f>IF(A29="",0,COUNTIF(A$27:A28,A29))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="108" t="inlineStr">
-        <is>
-          <t>Lunch</t>
         </is>
       </c>
       <c r="B30" s="83" t="n">
@@ -4444,13 +4367,19 @@
       <c r="N30" s="145" t="inlineStr"/>
       <c r="O30" s="145" t="inlineStr"/>
       <c r="P30" s="81">
-        <f>IF(A30="",0,COUNTIF(A$27:A29,A30))</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="129" t="inlineStr"/>
-      <c r="B31" s="83" t="inlineStr"/>
+      <c r="A31" s="108" t="inlineStr">
+        <is>
+          <t>Dinner (Regular)</t>
+        </is>
+      </c>
+      <c r="B31" s="83" t="n">
+        <v>3</v>
+      </c>
       <c r="C31" s="84">
         <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
@@ -4480,390 +4409,384 @@
       <c r="N31" s="145" t="inlineStr"/>
       <c r="O31" s="145" t="inlineStr"/>
       <c r="P31" s="81">
-        <f>IF(A31="",0,COUNTIF(A$27:A30,A31))</f>
+        <f>IF(A31="",0,COUNTIF(A$30:A30,A31))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="123" t="inlineStr">
+      <c r="A32" s="109" t="inlineStr">
+        <is>
+          <t>Exclusive Dinner (Michelin/Fine)</t>
+        </is>
+      </c>
+      <c r="B32" s="83" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" s="84">
+        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D32" s="84">
+        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E32" s="137">
+        <f>IF(D32&gt;0,(D32-C32)/D32,0)</f>
+        <v/>
+      </c>
+      <c r="F32" s="145" t="inlineStr"/>
+      <c r="G32" s="145" t="inlineStr"/>
+      <c r="H32" s="145" t="inlineStr"/>
+      <c r="I32" s="145" t="inlineStr"/>
+      <c r="J32" s="84">
+        <f>IF(A32="","",(COUNTIF(F32,"●")+COUNTIF(G32,"●")+COUNTIF(H32,"●")+COUNTIF(I32,"●")+COUNTIF(L32,"●")+COUNTIF(M32,"●")+COUNTIF(N32,"●")+COUNTIF(O32,"●"))*B32*C32)</f>
+        <v/>
+      </c>
+      <c r="K32" s="84">
+        <f>IF(A32="","",(COUNTIF(F32,"●")+COUNTIF(G32,"●")+COUNTIF(H32,"●")+COUNTIF(I32,"●")+COUNTIF(L32,"●")+COUNTIF(M32,"●")+COUNTIF(N32,"●")+COUNTIF(O32,"●"))*B32*D32)</f>
+        <v/>
+      </c>
+      <c r="L32" s="145" t="inlineStr"/>
+      <c r="M32" s="145" t="inlineStr"/>
+      <c r="N32" s="145" t="inlineStr"/>
+      <c r="O32" s="145" t="inlineStr"/>
+      <c r="P32" s="81">
+        <f>IF(A32="",0,COUNTIF(A$30:A31,A32))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="108" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="B33" s="83" t="n">
+        <v>3</v>
+      </c>
+      <c r="C33" s="84">
+        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D33" s="84">
+        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E33" s="137">
+        <f>IF(D33&gt;0,(D33-C33)/D33,0)</f>
+        <v/>
+      </c>
+      <c r="F33" s="145" t="inlineStr"/>
+      <c r="G33" s="145" t="inlineStr"/>
+      <c r="H33" s="145" t="inlineStr"/>
+      <c r="I33" s="145" t="inlineStr"/>
+      <c r="J33" s="84">
+        <f>IF(A33="","",(COUNTIF(F33,"●")+COUNTIF(G33,"●")+COUNTIF(H33,"●")+COUNTIF(I33,"●")+COUNTIF(L33,"●")+COUNTIF(M33,"●")+COUNTIF(N33,"●")+COUNTIF(O33,"●"))*B33*C33)</f>
+        <v/>
+      </c>
+      <c r="K33" s="84">
+        <f>IF(A33="","",(COUNTIF(F33,"●")+COUNTIF(G33,"●")+COUNTIF(H33,"●")+COUNTIF(I33,"●")+COUNTIF(L33,"●")+COUNTIF(M33,"●")+COUNTIF(N33,"●")+COUNTIF(O33,"●"))*B33*D33)</f>
+        <v/>
+      </c>
+      <c r="L33" s="145" t="inlineStr"/>
+      <c r="M33" s="145" t="inlineStr"/>
+      <c r="N33" s="145" t="inlineStr"/>
+      <c r="O33" s="145" t="inlineStr"/>
+      <c r="P33" s="81">
+        <f>IF(A33="",0,COUNTIF(A$30:A32,A33))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="129" t="inlineStr"/>
+      <c r="B34" s="83" t="inlineStr"/>
+      <c r="C34" s="84">
+        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D34" s="84">
+        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E34" s="137">
+        <f>IF(D34&gt;0,(D34-C34)/D34,0)</f>
+        <v/>
+      </c>
+      <c r="F34" s="145" t="inlineStr"/>
+      <c r="G34" s="145" t="inlineStr"/>
+      <c r="H34" s="145" t="inlineStr"/>
+      <c r="I34" s="145" t="inlineStr"/>
+      <c r="J34" s="84">
+        <f>IF(A34="","",(COUNTIF(F34,"●")+COUNTIF(G34,"●")+COUNTIF(H34,"●")+COUNTIF(I34,"●")+COUNTIF(L34,"●")+COUNTIF(M34,"●")+COUNTIF(N34,"●")+COUNTIF(O34,"●"))*B34*C34)</f>
+        <v/>
+      </c>
+      <c r="K34" s="84">
+        <f>IF(A34="","",(COUNTIF(F34,"●")+COUNTIF(G34,"●")+COUNTIF(H34,"●")+COUNTIF(I34,"●")+COUNTIF(L34,"●")+COUNTIF(M34,"●")+COUNTIF(N34,"●")+COUNTIF(O34,"●"))*B34*D34)</f>
+        <v/>
+      </c>
+      <c r="L34" s="145" t="inlineStr"/>
+      <c r="M34" s="145" t="inlineStr"/>
+      <c r="N34" s="145" t="inlineStr"/>
+      <c r="O34" s="145" t="inlineStr"/>
+      <c r="P34" s="81">
+        <f>IF(A34="",0,COUNTIF(A$30:A33,A34))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B32" s="114" t="inlineStr"/>
-      <c r="C32" s="114" t="inlineStr"/>
-      <c r="D32" s="114" t="inlineStr"/>
-      <c r="E32" s="114" t="inlineStr"/>
-      <c r="F32" s="130">
-        <f>SUMPRODUCT((F27:F31="●")*1,B27:B31,C27:C31)</f>
-        <v/>
-      </c>
-      <c r="G32" s="130">
-        <f>SUMPRODUCT((G27:G31="●")*1,B27:B31,C27:C31)</f>
-        <v/>
-      </c>
-      <c r="H32" s="130">
-        <f>SUMPRODUCT((H27:H31="●")*1,B27:B31,C27:C31)</f>
-        <v/>
-      </c>
-      <c r="I32" s="130">
-        <f>SUMPRODUCT((I27:I31="●")*1,B27:B31,C27:C31)</f>
-        <v/>
-      </c>
-      <c r="J32" s="88">
-        <f>SUM(J27:J31)</f>
-        <v/>
-      </c>
-      <c r="K32" s="88">
-        <f>SUM(K27:K31)</f>
-        <v/>
-      </c>
-      <c r="L32" s="130">
-        <f>SUMPRODUCT((L27:L31="●")*1,B27:B31,C27:C31)</f>
-        <v/>
-      </c>
-      <c r="M32" s="130">
-        <f>SUMPRODUCT((M27:M31="●")*1,B27:B31,C27:C31)</f>
-        <v/>
-      </c>
-      <c r="N32" s="130">
-        <f>SUMPRODUCT((N27:N31="●")*1,B27:B31,C27:C31)</f>
-        <v/>
-      </c>
-      <c r="O32" s="130">
-        <f>SUMPRODUCT((O27:O31="●")*1,B27:B31,C27:C31)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="128" t="inlineStr">
+      <c r="B35" s="114" t="inlineStr"/>
+      <c r="C35" s="114" t="inlineStr"/>
+      <c r="D35" s="114" t="inlineStr"/>
+      <c r="E35" s="114" t="inlineStr"/>
+      <c r="F35" s="130">
+        <f>SUMPRODUCT((F30:F34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="G35" s="130">
+        <f>SUMPRODUCT((G30:G34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="H35" s="130">
+        <f>SUMPRODUCT((H30:H34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="I35" s="130">
+        <f>SUMPRODUCT((I30:I34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="J35" s="88">
+        <f>SUM(J30:J34)</f>
+        <v/>
+      </c>
+      <c r="K35" s="88">
+        <f>SUM(K30:K34)</f>
+        <v/>
+      </c>
+      <c r="L35" s="130">
+        <f>SUMPRODUCT((L30:L34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="M35" s="130">
+        <f>SUMPRODUCT((M30:M34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="N35" s="130">
+        <f>SUMPRODUCT((N30:N34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="O35" s="130">
+        <f>SUMPRODUCT((O30:O34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="128" t="inlineStr">
         <is>
           <t>📦 OTHER</t>
         </is>
       </c>
-      <c r="B34" s="77" t="n"/>
-      <c r="C34" s="77" t="n"/>
-      <c r="D34" s="77" t="n"/>
-      <c r="E34" s="77" t="n"/>
-      <c r="F34" s="77" t="n"/>
-      <c r="G34" s="77" t="n"/>
-      <c r="H34" s="77" t="n"/>
-      <c r="I34" s="77" t="n"/>
-      <c r="J34" s="77" t="n"/>
-      <c r="K34" s="77" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="109" t="inlineStr">
+      <c r="B37" s="77" t="n"/>
+      <c r="C37" s="77" t="n"/>
+      <c r="D37" s="77" t="n"/>
+      <c r="E37" s="77" t="n"/>
+      <c r="F37" s="77" t="n"/>
+      <c r="G37" s="77" t="n"/>
+      <c r="H37" s="77" t="n"/>
+      <c r="I37" s="77" t="n"/>
+      <c r="J37" s="77" t="n"/>
+      <c r="K37" s="77" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="109" t="inlineStr">
         <is>
           <t>Insurance / Tips / Contingency</t>
         </is>
       </c>
-      <c r="B35" s="83" t="n">
+      <c r="B38" s="83" t="n">
         <v>4</v>
       </c>
-      <c r="C35" s="84">
-        <f>IF(A35="","",VLOOKUP(A35,'Master Data'!$A$50:$C$56,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D35" s="84">
-        <f>IF(A35="","",VLOOKUP(A35,'Master Data'!$A$50:$C$56,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E35" s="137">
-        <f>IF(D35&gt;0,(D35-C35)/D35,0)</f>
-        <v/>
-      </c>
-      <c r="F35" s="145" t="inlineStr"/>
-      <c r="G35" s="145" t="inlineStr"/>
-      <c r="H35" s="145" t="inlineStr"/>
-      <c r="I35" s="145" t="inlineStr"/>
-      <c r="J35" s="84">
-        <f>IF(A35="","",(COUNTIF(F35,"●")+COUNTIF(G35,"●")+COUNTIF(H35,"●")+COUNTIF(I35,"●")+COUNTIF(L35,"●")+COUNTIF(M35,"●")+COUNTIF(N35,"●")+COUNTIF(O35,"●"))*B35*C35)</f>
-        <v/>
-      </c>
-      <c r="K35" s="84">
-        <f>IF(A35="","",(COUNTIF(F35,"●")+COUNTIF(G35,"●")+COUNTIF(H35,"●")+COUNTIF(I35,"●")+COUNTIF(L35,"●")+COUNTIF(M35,"●")+COUNTIF(N35,"●")+COUNTIF(O35,"●"))*B35*D35)</f>
-        <v/>
-      </c>
-      <c r="L35" s="145" t="inlineStr"/>
-      <c r="M35" s="145" t="inlineStr"/>
-      <c r="N35" s="145" t="inlineStr"/>
-      <c r="O35" s="145" t="inlineStr"/>
-      <c r="P35" s="81">
+      <c r="C38" s="84">
+        <f>IF(A38="","",VLOOKUP(A38,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D38" s="84">
+        <f>IF(A38="","",VLOOKUP(A38,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E38" s="137">
+        <f>IF(D38&gt;0,(D38-C38)/D38,0)</f>
+        <v/>
+      </c>
+      <c r="F38" s="145" t="inlineStr"/>
+      <c r="G38" s="145" t="inlineStr"/>
+      <c r="H38" s="145" t="inlineStr"/>
+      <c r="I38" s="145" t="inlineStr"/>
+      <c r="J38" s="84">
+        <f>IF(A38="","",(COUNTIF(F38,"●")+COUNTIF(G38,"●")+COUNTIF(H38,"●")+COUNTIF(I38,"●")+COUNTIF(L38,"●")+COUNTIF(M38,"●")+COUNTIF(N38,"●")+COUNTIF(O38,"●"))*B38*C38)</f>
+        <v/>
+      </c>
+      <c r="K38" s="84">
+        <f>IF(A38="","",(COUNTIF(F38,"●")+COUNTIF(G38,"●")+COUNTIF(H38,"●")+COUNTIF(I38,"●")+COUNTIF(L38,"●")+COUNTIF(M38,"●")+COUNTIF(N38,"●")+COUNTIF(O38,"●"))*B38*D38)</f>
+        <v/>
+      </c>
+      <c r="L38" s="145" t="inlineStr"/>
+      <c r="M38" s="145" t="inlineStr"/>
+      <c r="N38" s="145" t="inlineStr"/>
+      <c r="O38" s="145" t="inlineStr"/>
+      <c r="P38" s="81">
         <f>0</f>
         <v/>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="129" t="inlineStr"/>
-      <c r="B36" s="83" t="inlineStr"/>
-      <c r="C36" s="84">
-        <f>IF(A36="","",VLOOKUP(A36,'Master Data'!$A$50:$C$56,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D36" s="84">
-        <f>IF(A36="","",VLOOKUP(A36,'Master Data'!$A$50:$C$56,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E36" s="137">
-        <f>IF(D36&gt;0,(D36-C36)/D36,0)</f>
-        <v/>
-      </c>
-      <c r="F36" s="145" t="inlineStr"/>
-      <c r="G36" s="145" t="inlineStr"/>
-      <c r="H36" s="145" t="inlineStr"/>
-      <c r="I36" s="145" t="inlineStr"/>
-      <c r="J36" s="84">
-        <f>IF(A36="","",(COUNTIF(F36,"●")+COUNTIF(G36,"●")+COUNTIF(H36,"●")+COUNTIF(I36,"●")+COUNTIF(L36,"●")+COUNTIF(M36,"●")+COUNTIF(N36,"●")+COUNTIF(O36,"●"))*B36*C36)</f>
-        <v/>
-      </c>
-      <c r="K36" s="84">
-        <f>IF(A36="","",(COUNTIF(F36,"●")+COUNTIF(G36,"●")+COUNTIF(H36,"●")+COUNTIF(I36,"●")+COUNTIF(L36,"●")+COUNTIF(M36,"●")+COUNTIF(N36,"●")+COUNTIF(O36,"●"))*B36*D36)</f>
-        <v/>
-      </c>
-      <c r="L36" s="145" t="inlineStr"/>
-      <c r="M36" s="145" t="inlineStr"/>
-      <c r="N36" s="145" t="inlineStr"/>
-      <c r="O36" s="145" t="inlineStr"/>
-      <c r="P36" s="81">
-        <f>IF(A36="",0,COUNTIF(A$35:A35,A36))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="129" t="inlineStr"/>
-      <c r="B37" s="83" t="inlineStr"/>
-      <c r="C37" s="84">
-        <f>IF(A37="","",VLOOKUP(A37,'Master Data'!$A$50:$C$56,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D37" s="84">
-        <f>IF(A37="","",VLOOKUP(A37,'Master Data'!$A$50:$C$56,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E37" s="137">
-        <f>IF(D37&gt;0,(D37-C37)/D37,0)</f>
-        <v/>
-      </c>
-      <c r="F37" s="145" t="inlineStr"/>
-      <c r="G37" s="145" t="inlineStr"/>
-      <c r="H37" s="145" t="inlineStr"/>
-      <c r="I37" s="145" t="inlineStr"/>
-      <c r="J37" s="84">
-        <f>IF(A37="","",(COUNTIF(F37,"●")+COUNTIF(G37,"●")+COUNTIF(H37,"●")+COUNTIF(I37,"●")+COUNTIF(L37,"●")+COUNTIF(M37,"●")+COUNTIF(N37,"●")+COUNTIF(O37,"●"))*B37*C37)</f>
-        <v/>
-      </c>
-      <c r="K37" s="84">
-        <f>IF(A37="","",(COUNTIF(F37,"●")+COUNTIF(G37,"●")+COUNTIF(H37,"●")+COUNTIF(I37,"●")+COUNTIF(L37,"●")+COUNTIF(M37,"●")+COUNTIF(N37,"●")+COUNTIF(O37,"●"))*B37*D37)</f>
-        <v/>
-      </c>
-      <c r="L37" s="145" t="inlineStr"/>
-      <c r="M37" s="145" t="inlineStr"/>
-      <c r="N37" s="145" t="inlineStr"/>
-      <c r="O37" s="145" t="inlineStr"/>
-      <c r="P37" s="81">
-        <f>IF(A37="",0,COUNTIF(A$35:A36,A37))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="123" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="129" t="inlineStr"/>
+      <c r="B39" s="83" t="inlineStr"/>
+      <c r="C39" s="84">
+        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D39" s="84">
+        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E39" s="137">
+        <f>IF(D39&gt;0,(D39-C39)/D39,0)</f>
+        <v/>
+      </c>
+      <c r="F39" s="145" t="inlineStr"/>
+      <c r="G39" s="145" t="inlineStr"/>
+      <c r="H39" s="145" t="inlineStr"/>
+      <c r="I39" s="145" t="inlineStr"/>
+      <c r="J39" s="84">
+        <f>IF(A39="","",(COUNTIF(F39,"●")+COUNTIF(G39,"●")+COUNTIF(H39,"●")+COUNTIF(I39,"●")+COUNTIF(L39,"●")+COUNTIF(M39,"●")+COUNTIF(N39,"●")+COUNTIF(O39,"●"))*B39*C39)</f>
+        <v/>
+      </c>
+      <c r="K39" s="84">
+        <f>IF(A39="","",(COUNTIF(F39,"●")+COUNTIF(G39,"●")+COUNTIF(H39,"●")+COUNTIF(I39,"●")+COUNTIF(L39,"●")+COUNTIF(M39,"●")+COUNTIF(N39,"●")+COUNTIF(O39,"●"))*B39*D39)</f>
+        <v/>
+      </c>
+      <c r="L39" s="145" t="inlineStr"/>
+      <c r="M39" s="145" t="inlineStr"/>
+      <c r="N39" s="145" t="inlineStr"/>
+      <c r="O39" s="145" t="inlineStr"/>
+      <c r="P39" s="81">
+        <f>IF(A39="",0,COUNTIF(A$38:A38,A39))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="129" t="inlineStr"/>
+      <c r="B40" s="83" t="inlineStr"/>
+      <c r="C40" s="84">
+        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D40" s="84">
+        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E40" s="137">
+        <f>IF(D40&gt;0,(D40-C40)/D40,0)</f>
+        <v/>
+      </c>
+      <c r="F40" s="145" t="inlineStr"/>
+      <c r="G40" s="145" t="inlineStr"/>
+      <c r="H40" s="145" t="inlineStr"/>
+      <c r="I40" s="145" t="inlineStr"/>
+      <c r="J40" s="84">
+        <f>IF(A40="","",(COUNTIF(F40,"●")+COUNTIF(G40,"●")+COUNTIF(H40,"●")+COUNTIF(I40,"●")+COUNTIF(L40,"●")+COUNTIF(M40,"●")+COUNTIF(N40,"●")+COUNTIF(O40,"●"))*B40*C40)</f>
+        <v/>
+      </c>
+      <c r="K40" s="84">
+        <f>IF(A40="","",(COUNTIF(F40,"●")+COUNTIF(G40,"●")+COUNTIF(H40,"●")+COUNTIF(I40,"●")+COUNTIF(L40,"●")+COUNTIF(M40,"●")+COUNTIF(N40,"●")+COUNTIF(O40,"●"))*B40*D40)</f>
+        <v/>
+      </c>
+      <c r="L40" s="145" t="inlineStr"/>
+      <c r="M40" s="145" t="inlineStr"/>
+      <c r="N40" s="145" t="inlineStr"/>
+      <c r="O40" s="145" t="inlineStr"/>
+      <c r="P40" s="81">
+        <f>IF(A40="",0,COUNTIF(A$38:A39,A40))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B38" s="114" t="inlineStr"/>
-      <c r="C38" s="114" t="inlineStr"/>
-      <c r="D38" s="114" t="inlineStr"/>
-      <c r="E38" s="114" t="inlineStr"/>
-      <c r="F38" s="130">
-        <f>SUMPRODUCT((F35:F37="●")*1,B35:B37,C35:C37)</f>
-        <v/>
-      </c>
-      <c r="G38" s="130">
-        <f>SUMPRODUCT((G35:G37="●")*1,B35:B37,C35:C37)</f>
-        <v/>
-      </c>
-      <c r="H38" s="130">
-        <f>SUMPRODUCT((H35:H37="●")*1,B35:B37,C35:C37)</f>
-        <v/>
-      </c>
-      <c r="I38" s="130">
-        <f>SUMPRODUCT((I35:I37="●")*1,B35:B37,C35:C37)</f>
-        <v/>
-      </c>
-      <c r="J38" s="88">
-        <f>SUM(J35:J37)</f>
-        <v/>
-      </c>
-      <c r="K38" s="88">
-        <f>SUM(K35:K37)</f>
-        <v/>
-      </c>
-      <c r="L38" s="130">
-        <f>SUMPRODUCT((L35:L37="●")*1,B35:B37,C35:C37)</f>
-        <v/>
-      </c>
-      <c r="M38" s="130">
-        <f>SUMPRODUCT((M35:M37="●")*1,B35:B37,C35:C37)</f>
-        <v/>
-      </c>
-      <c r="N38" s="130">
-        <f>SUMPRODUCT((N35:N37="●")*1,B35:B37,C35:C37)</f>
-        <v/>
-      </c>
-      <c r="O38" s="130">
-        <f>SUMPRODUCT((O35:O37="●")*1,B35:B37,C35:C37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="128" t="inlineStr">
+      <c r="B41" s="114" t="inlineStr"/>
+      <c r="C41" s="114" t="inlineStr"/>
+      <c r="D41" s="114" t="inlineStr"/>
+      <c r="E41" s="114" t="inlineStr"/>
+      <c r="F41" s="130">
+        <f>SUMPRODUCT((F38:F40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="G41" s="130">
+        <f>SUMPRODUCT((G38:G40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="H41" s="130">
+        <f>SUMPRODUCT((H38:H40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="I41" s="130">
+        <f>SUMPRODUCT((I38:I40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="J41" s="88">
+        <f>SUM(J38:J40)</f>
+        <v/>
+      </c>
+      <c r="K41" s="88">
+        <f>SUM(K38:K40)</f>
+        <v/>
+      </c>
+      <c r="L41" s="130">
+        <f>SUMPRODUCT((L38:L40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="M41" s="130">
+        <f>SUMPRODUCT((M38:M40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="N41" s="130">
+        <f>SUMPRODUCT((N38:N40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="O41" s="130">
+        <f>SUMPRODUCT((O38:O40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="128" t="inlineStr">
         <is>
           <t>🎯 ACTIVITIES</t>
         </is>
       </c>
-      <c r="B40" s="77" t="n"/>
-      <c r="C40" s="77" t="n"/>
-      <c r="D40" s="77" t="n"/>
-      <c r="E40" s="77" t="n"/>
-      <c r="F40" s="77" t="n"/>
-      <c r="G40" s="77" t="n"/>
-      <c r="H40" s="77" t="n"/>
-      <c r="I40" s="77" t="n"/>
-      <c r="J40" s="77" t="n"/>
-      <c r="K40" s="77" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="109" t="inlineStr">
+      <c r="B43" s="77" t="n"/>
+      <c r="C43" s="77" t="n"/>
+      <c r="D43" s="77" t="n"/>
+      <c r="E43" s="77" t="n"/>
+      <c r="F43" s="77" t="n"/>
+      <c r="G43" s="77" t="n"/>
+      <c r="H43" s="77" t="n"/>
+      <c r="I43" s="77" t="n"/>
+      <c r="J43" s="77" t="n"/>
+      <c r="K43" s="77" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="109" t="inlineStr">
         <is>
           <t>Beach/Surf Lesson</t>
-        </is>
-      </c>
-      <c r="B41" s="83" t="n">
-        <v>1</v>
-      </c>
-      <c r="C41" s="84">
-        <f>IF(A41="","",VLOOKUP(A41,'Master Data'!$A$86:$C$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D41" s="84">
-        <f>IF(A41="","",VLOOKUP(A41,'Master Data'!$A$86:$C$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E41" s="137">
-        <f>IF(D41&gt;0,(D41-C41)/D41,0)</f>
-        <v/>
-      </c>
-      <c r="F41" s="145" t="inlineStr"/>
-      <c r="G41" s="145" t="inlineStr"/>
-      <c r="H41" s="145" t="inlineStr"/>
-      <c r="I41" s="145" t="inlineStr"/>
-      <c r="J41" s="84">
-        <f>IF(A41="","",(COUNTIF(F41,"●")+COUNTIF(G41,"●")+COUNTIF(H41,"●")+COUNTIF(I41,"●")+COUNTIF(L41,"●")+COUNTIF(M41,"●")+COUNTIF(N41,"●")+COUNTIF(O41,"●"))*B41*C41)</f>
-        <v/>
-      </c>
-      <c r="K41" s="84">
-        <f>IF(A41="","",(COUNTIF(F41,"●")+COUNTIF(G41,"●")+COUNTIF(H41,"●")+COUNTIF(I41,"●")+COUNTIF(L41,"●")+COUNTIF(M41,"●")+COUNTIF(N41,"●")+COUNTIF(O41,"●"))*B41*D41)</f>
-        <v/>
-      </c>
-      <c r="L41" s="145" t="inlineStr"/>
-      <c r="M41" s="145" t="inlineStr"/>
-      <c r="N41" s="145" t="inlineStr"/>
-      <c r="O41" s="145" t="inlineStr"/>
-      <c r="P41" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="108" t="inlineStr">
-        <is>
-          <t>Local Hiking (Griffith/Runyon)</t>
-        </is>
-      </c>
-      <c r="B42" s="83" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" s="84">
-        <f>IF(A42="","",VLOOKUP(A42,'Master Data'!$A$86:$C$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D42" s="84">
-        <f>IF(A42="","",VLOOKUP(A42,'Master Data'!$A$86:$C$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E42" s="137">
-        <f>IF(D42&gt;0,(D42-C42)/D42,0)</f>
-        <v/>
-      </c>
-      <c r="F42" s="145" t="inlineStr"/>
-      <c r="G42" s="145" t="inlineStr"/>
-      <c r="H42" s="145" t="inlineStr"/>
-      <c r="I42" s="145" t="inlineStr"/>
-      <c r="J42" s="84">
-        <f>IF(A42="","",(COUNTIF(F42,"●")+COUNTIF(G42,"●")+COUNTIF(H42,"●")+COUNTIF(I42,"●")+COUNTIF(L42,"●")+COUNTIF(M42,"●")+COUNTIF(N42,"●")+COUNTIF(O42,"●"))*B42*C42)</f>
-        <v/>
-      </c>
-      <c r="K42" s="84">
-        <f>IF(A42="","",(COUNTIF(F42,"●")+COUNTIF(G42,"●")+COUNTIF(H42,"●")+COUNTIF(I42,"●")+COUNTIF(L42,"●")+COUNTIF(M42,"●")+COUNTIF(N42,"●")+COUNTIF(O42,"●"))*B42*D42)</f>
-        <v/>
-      </c>
-      <c r="L42" s="145" t="inlineStr"/>
-      <c r="M42" s="145" t="inlineStr"/>
-      <c r="N42" s="145" t="inlineStr"/>
-      <c r="O42" s="145" t="inlineStr"/>
-      <c r="P42" s="81">
-        <f>IF(A42="",0,COUNTIF(A$41:A41,A42))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="109" t="inlineStr">
-        <is>
-          <t>NBA/MLB Game (Ticket)</t>
-        </is>
-      </c>
-      <c r="B43" s="83" t="n">
-        <v>1</v>
-      </c>
-      <c r="C43" s="84">
-        <f>IF(A43="","",VLOOKUP(A43,'Master Data'!$A$86:$C$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D43" s="84">
-        <f>IF(A43="","",VLOOKUP(A43,'Master Data'!$A$86:$C$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E43" s="137">
-        <f>IF(D43&gt;0,(D43-C43)/D43,0)</f>
-        <v/>
-      </c>
-      <c r="F43" s="145" t="inlineStr"/>
-      <c r="G43" s="145" t="inlineStr"/>
-      <c r="H43" s="145" t="inlineStr"/>
-      <c r="I43" s="145" t="inlineStr"/>
-      <c r="J43" s="84">
-        <f>IF(A43="","",(COUNTIF(F43,"●")+COUNTIF(G43,"●")+COUNTIF(H43,"●")+COUNTIF(I43,"●")+COUNTIF(L43,"●")+COUNTIF(M43,"●")+COUNTIF(N43,"●")+COUNTIF(O43,"●"))*B43*C43)</f>
-        <v/>
-      </c>
-      <c r="K43" s="84">
-        <f>IF(A43="","",(COUNTIF(F43,"●")+COUNTIF(G43,"●")+COUNTIF(H43,"●")+COUNTIF(I43,"●")+COUNTIF(L43,"●")+COUNTIF(M43,"●")+COUNTIF(N43,"●")+COUNTIF(O43,"●"))*B43*D43)</f>
-        <v/>
-      </c>
-      <c r="L43" s="145" t="inlineStr"/>
-      <c r="M43" s="145" t="inlineStr"/>
-      <c r="N43" s="145" t="inlineStr"/>
-      <c r="O43" s="145" t="inlineStr"/>
-      <c r="P43" s="81">
-        <f>IF(A43="",0,COUNTIF(A$41:A42,A43))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="108" t="inlineStr">
-        <is>
-          <t>Sports Bar Experience</t>
         </is>
       </c>
       <c r="B44" s="83" t="n">
@@ -4898,13 +4821,19 @@
       <c r="N44" s="145" t="inlineStr"/>
       <c r="O44" s="145" t="inlineStr"/>
       <c r="P44" s="81">
-        <f>IF(A44="",0,COUNTIF(A$41:A43,A44))</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="129" t="inlineStr"/>
-      <c r="B45" s="83" t="inlineStr"/>
+      <c r="A45" s="108" t="inlineStr">
+        <is>
+          <t>Local Hiking (Griffith/Runyon)</t>
+        </is>
+      </c>
+      <c r="B45" s="83" t="n">
+        <v>1</v>
+      </c>
       <c r="C45" s="84">
         <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
@@ -4934,13 +4863,19 @@
       <c r="N45" s="145" t="inlineStr"/>
       <c r="O45" s="145" t="inlineStr"/>
       <c r="P45" s="81">
-        <f>IF(A45="",0,COUNTIF(A$41:A44,A45))</f>
+        <f>IF(A45="",0,COUNTIF(A$44:A44,A45))</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="129" t="inlineStr"/>
-      <c r="B46" s="83" t="inlineStr"/>
+      <c r="A46" s="109" t="inlineStr">
+        <is>
+          <t>NBA/MLB Game (Ticket)</t>
+        </is>
+      </c>
+      <c r="B46" s="83" t="n">
+        <v>1</v>
+      </c>
       <c r="C46" s="84">
         <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
@@ -4970,13 +4905,19 @@
       <c r="N46" s="145" t="inlineStr"/>
       <c r="O46" s="145" t="inlineStr"/>
       <c r="P46" s="81">
-        <f>IF(A46="",0,COUNTIF(A$41:A45,A46))</f>
+        <f>IF(A46="",0,COUNTIF(A$44:A45,A46))</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="129" t="inlineStr"/>
-      <c r="B47" s="83" t="inlineStr"/>
+      <c r="A47" s="108" t="inlineStr">
+        <is>
+          <t>Sports Bar Experience</t>
+        </is>
+      </c>
+      <c r="B47" s="83" t="n">
+        <v>1</v>
+      </c>
       <c r="C47" s="84">
         <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
@@ -5006,7 +4947,7 @@
       <c r="N47" s="145" t="inlineStr"/>
       <c r="O47" s="145" t="inlineStr"/>
       <c r="P47" s="81">
-        <f>IF(A47="",0,COUNTIF(A$41:A46,A47))</f>
+        <f>IF(A47="",0,COUNTIF(A$44:A46,A47))</f>
         <v/>
       </c>
     </row>
@@ -5042,7 +4983,7 @@
       <c r="N48" s="145" t="inlineStr"/>
       <c r="O48" s="145" t="inlineStr"/>
       <c r="P48" s="81">
-        <f>IF(A48="",0,COUNTIF(A$41:A47,A48))</f>
+        <f>IF(A48="",0,COUNTIF(A$44:A47,A48))</f>
         <v/>
       </c>
     </row>
@@ -5078,330 +5019,360 @@
       <c r="N49" s="145" t="inlineStr"/>
       <c r="O49" s="145" t="inlineStr"/>
       <c r="P49" s="81">
-        <f>IF(A49="",0,COUNTIF(A$41:A48,A49))</f>
+        <f>IF(A49="",0,COUNTIF(A$44:A48,A49))</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="123" t="inlineStr">
+      <c r="A50" s="129" t="inlineStr"/>
+      <c r="B50" s="83" t="inlineStr"/>
+      <c r="C50" s="84">
+        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D50" s="84">
+        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E50" s="137">
+        <f>IF(D50&gt;0,(D50-C50)/D50,0)</f>
+        <v/>
+      </c>
+      <c r="F50" s="145" t="inlineStr"/>
+      <c r="G50" s="145" t="inlineStr"/>
+      <c r="H50" s="145" t="inlineStr"/>
+      <c r="I50" s="145" t="inlineStr"/>
+      <c r="J50" s="84">
+        <f>IF(A50="","",(COUNTIF(F50,"●")+COUNTIF(G50,"●")+COUNTIF(H50,"●")+COUNTIF(I50,"●")+COUNTIF(L50,"●")+COUNTIF(M50,"●")+COUNTIF(N50,"●")+COUNTIF(O50,"●"))*B50*C50)</f>
+        <v/>
+      </c>
+      <c r="K50" s="84">
+        <f>IF(A50="","",(COUNTIF(F50,"●")+COUNTIF(G50,"●")+COUNTIF(H50,"●")+COUNTIF(I50,"●")+COUNTIF(L50,"●")+COUNTIF(M50,"●")+COUNTIF(N50,"●")+COUNTIF(O50,"●"))*B50*D50)</f>
+        <v/>
+      </c>
+      <c r="L50" s="145" t="inlineStr"/>
+      <c r="M50" s="145" t="inlineStr"/>
+      <c r="N50" s="145" t="inlineStr"/>
+      <c r="O50" s="145" t="inlineStr"/>
+      <c r="P50" s="81">
+        <f>IF(A50="",0,COUNTIF(A$44:A49,A50))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="129" t="inlineStr"/>
+      <c r="B51" s="83" t="inlineStr"/>
+      <c r="C51" s="84">
+        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D51" s="84">
+        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E51" s="137">
+        <f>IF(D51&gt;0,(D51-C51)/D51,0)</f>
+        <v/>
+      </c>
+      <c r="F51" s="145" t="inlineStr"/>
+      <c r="G51" s="145" t="inlineStr"/>
+      <c r="H51" s="145" t="inlineStr"/>
+      <c r="I51" s="145" t="inlineStr"/>
+      <c r="J51" s="84">
+        <f>IF(A51="","",(COUNTIF(F51,"●")+COUNTIF(G51,"●")+COUNTIF(H51,"●")+COUNTIF(I51,"●")+COUNTIF(L51,"●")+COUNTIF(M51,"●")+COUNTIF(N51,"●")+COUNTIF(O51,"●"))*B51*C51)</f>
+        <v/>
+      </c>
+      <c r="K51" s="84">
+        <f>IF(A51="","",(COUNTIF(F51,"●")+COUNTIF(G51,"●")+COUNTIF(H51,"●")+COUNTIF(I51,"●")+COUNTIF(L51,"●")+COUNTIF(M51,"●")+COUNTIF(N51,"●")+COUNTIF(O51,"●"))*B51*D51)</f>
+        <v/>
+      </c>
+      <c r="L51" s="145" t="inlineStr"/>
+      <c r="M51" s="145" t="inlineStr"/>
+      <c r="N51" s="145" t="inlineStr"/>
+      <c r="O51" s="145" t="inlineStr"/>
+      <c r="P51" s="81">
+        <f>IF(A51="",0,COUNTIF(A$44:A50,A51))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="129" t="inlineStr"/>
+      <c r="B52" s="83" t="inlineStr"/>
+      <c r="C52" s="84">
+        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D52" s="84">
+        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E52" s="137">
+        <f>IF(D52&gt;0,(D52-C52)/D52,0)</f>
+        <v/>
+      </c>
+      <c r="F52" s="145" t="inlineStr"/>
+      <c r="G52" s="145" t="inlineStr"/>
+      <c r="H52" s="145" t="inlineStr"/>
+      <c r="I52" s="145" t="inlineStr"/>
+      <c r="J52" s="84">
+        <f>IF(A52="","",(COUNTIF(F52,"●")+COUNTIF(G52,"●")+COUNTIF(H52,"●")+COUNTIF(I52,"●")+COUNTIF(L52,"●")+COUNTIF(M52,"●")+COUNTIF(N52,"●")+COUNTIF(O52,"●"))*B52*C52)</f>
+        <v/>
+      </c>
+      <c r="K52" s="84">
+        <f>IF(A52="","",(COUNTIF(F52,"●")+COUNTIF(G52,"●")+COUNTIF(H52,"●")+COUNTIF(I52,"●")+COUNTIF(L52,"●")+COUNTIF(M52,"●")+COUNTIF(N52,"●")+COUNTIF(O52,"●"))*B52*D52)</f>
+        <v/>
+      </c>
+      <c r="L52" s="145" t="inlineStr"/>
+      <c r="M52" s="145" t="inlineStr"/>
+      <c r="N52" s="145" t="inlineStr"/>
+      <c r="O52" s="145" t="inlineStr"/>
+      <c r="P52" s="81">
+        <f>IF(A52="",0,COUNTIF(A$44:A51,A52))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B50" s="114" t="inlineStr"/>
-      <c r="C50" s="114" t="inlineStr"/>
-      <c r="D50" s="114" t="inlineStr"/>
-      <c r="E50" s="114" t="inlineStr"/>
-      <c r="F50" s="130">
-        <f>SUMPRODUCT((F41:F49="●")*1,B41:B49,C41:C49)</f>
-        <v/>
-      </c>
-      <c r="G50" s="130">
-        <f>SUMPRODUCT((G41:G49="●")*1,B41:B49,C41:C49)</f>
-        <v/>
-      </c>
-      <c r="H50" s="130">
-        <f>SUMPRODUCT((H41:H49="●")*1,B41:B49,C41:C49)</f>
-        <v/>
-      </c>
-      <c r="I50" s="130">
-        <f>SUMPRODUCT((I41:I49="●")*1,B41:B49,C41:C49)</f>
-        <v/>
-      </c>
-      <c r="J50" s="88">
-        <f>SUM(J41:J49)</f>
-        <v/>
-      </c>
-      <c r="K50" s="88">
-        <f>SUM(K41:K49)</f>
-        <v/>
-      </c>
-      <c r="L50" s="130">
-        <f>SUMPRODUCT((L41:L49="●")*1,B41:B49,C41:C49)</f>
-        <v/>
-      </c>
-      <c r="M50" s="130">
-        <f>SUMPRODUCT((M41:M49="●")*1,B41:B49,C41:C49)</f>
-        <v/>
-      </c>
-      <c r="N50" s="130">
-        <f>SUMPRODUCT((N41:N49="●")*1,B41:B49,C41:C49)</f>
-        <v/>
-      </c>
-      <c r="O50" s="130">
-        <f>SUMPRODUCT((O41:O49="●")*1,B41:B49,C41:C49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="103" t="inlineStr">
+      <c r="B53" s="114" t="inlineStr"/>
+      <c r="C53" s="114" t="inlineStr"/>
+      <c r="D53" s="114" t="inlineStr"/>
+      <c r="E53" s="114" t="inlineStr"/>
+      <c r="F53" s="130">
+        <f>SUMPRODUCT((F44:F52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="G53" s="130">
+        <f>SUMPRODUCT((G44:G52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="H53" s="130">
+        <f>SUMPRODUCT((H44:H52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="I53" s="130">
+        <f>SUMPRODUCT((I44:I52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="J53" s="88">
+        <f>SUM(J44:J52)</f>
+        <v/>
+      </c>
+      <c r="K53" s="88">
+        <f>SUM(K44:K52)</f>
+        <v/>
+      </c>
+      <c r="L53" s="130">
+        <f>SUMPRODUCT((L44:L52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="M53" s="130">
+        <f>SUMPRODUCT((M44:M52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="N53" s="130">
+        <f>SUMPRODUCT((N44:N52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="O53" s="130">
+        <f>SUMPRODUCT((O44:O52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="103" t="inlineStr">
         <is>
           <t>🏆 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B53" s="104" t="n"/>
-      <c r="C53" s="104" t="n"/>
-      <c r="D53" s="104" t="n"/>
-      <c r="E53" s="104" t="n"/>
-      <c r="F53" s="104" t="n"/>
-      <c r="G53" s="104" t="n"/>
-      <c r="H53" s="104" t="n"/>
-      <c r="I53" s="104" t="n"/>
-      <c r="J53" s="104" t="n"/>
-      <c r="K53" s="104" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="108" t="inlineStr">
-        <is>
-          <t>GOLF</t>
-        </is>
-      </c>
-      <c r="J54" s="84">
-        <f>J12</f>
-        <v/>
-      </c>
-      <c r="K54" s="84">
-        <f>K12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="108" t="inlineStr">
-        <is>
-          <t>HOTEL</t>
-        </is>
-      </c>
-      <c r="J55" s="84">
-        <f>J18</f>
-        <v/>
-      </c>
-      <c r="K55" s="84">
-        <f>K18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="108" t="inlineStr">
-        <is>
-          <t>TRANSPORT</t>
-        </is>
-      </c>
-      <c r="J56" s="84">
-        <f>J24</f>
-        <v/>
-      </c>
-      <c r="K56" s="84">
-        <f>K24</f>
-        <v/>
-      </c>
+      <c r="B56" s="104" t="n"/>
+      <c r="C56" s="104" t="n"/>
+      <c r="D56" s="104" t="n"/>
+      <c r="E56" s="104" t="n"/>
+      <c r="F56" s="104" t="n"/>
+      <c r="G56" s="104" t="n"/>
+      <c r="H56" s="104" t="n"/>
+      <c r="I56" s="104" t="n"/>
+      <c r="J56" s="104" t="n"/>
+      <c r="K56" s="104" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="108" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MEALS</t>
+          <t>GOLF</t>
         </is>
       </c>
       <c r="J57" s="84">
-        <f>J32</f>
+        <f>J15</f>
         <v/>
       </c>
       <c r="K57" s="84">
-        <f>K32</f>
+        <f>K15</f>
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="108" t="inlineStr">
         <is>
-          <t>OTHER</t>
+          <t>HOTEL</t>
         </is>
       </c>
       <c r="J58" s="84">
-        <f>J38</f>
+        <f>J21</f>
         <v/>
       </c>
       <c r="K58" s="84">
-        <f>K38</f>
+        <f>K21</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="108" t="inlineStr">
         <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="J59" s="84">
+        <f>J27</f>
+        <v/>
+      </c>
+      <c r="K59" s="84">
+        <f>K27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="108" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MEALS</t>
+        </is>
+      </c>
+      <c r="J60" s="84">
+        <f>J35</f>
+        <v/>
+      </c>
+      <c r="K60" s="84">
+        <f>K35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="108" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="J61" s="84">
+        <f>J41</f>
+        <v/>
+      </c>
+      <c r="K61" s="84">
+        <f>K41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="108" t="inlineStr">
+        <is>
           <t>ACTIVITIES</t>
         </is>
       </c>
-      <c r="J59" s="84">
-        <f>J50</f>
-        <v/>
-      </c>
-      <c r="K59" s="84">
-        <f>K50</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="115" t="inlineStr">
+      <c r="J62" s="84">
+        <f>J53</f>
+        <v/>
+      </c>
+      <c r="K62" s="84">
+        <f>K53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="115" t="inlineStr">
         <is>
           <t>📌 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C60" s="106" t="inlineStr">
+      <c r="C63" s="106" t="inlineStr">
         <is>
           <t>Margin:</t>
         </is>
       </c>
-      <c r="D60" s="91">
-        <f>IF(K60&gt;0,(K60-J60)/K60,0)</f>
-        <v/>
-      </c>
-      <c r="J60" s="88">
-        <f>SUM(J54:J59)</f>
-        <v/>
-      </c>
-      <c r="K60" s="88">
-        <f>SUM(K54:K59)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="103" t="inlineStr">
+      <c r="D63" s="91">
+        <f>IF(K63&gt;0,(K63-J63)/K63,0)</f>
+        <v/>
+      </c>
+      <c r="J63" s="88">
+        <f>SUM(J57:J62)</f>
+        <v/>
+      </c>
+      <c r="K63" s="88">
+        <f>SUM(K57:K62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="103" t="inlineStr">
         <is>
           <t>👤 PER PERSON</t>
         </is>
       </c>
-      <c r="B62" s="104" t="n"/>
-      <c r="C62" s="104" t="n"/>
-      <c r="D62" s="104" t="n"/>
-      <c r="E62" s="104" t="n"/>
-      <c r="F62" s="104" t="n"/>
-      <c r="G62" s="104" t="n"/>
-      <c r="H62" s="104" t="n"/>
-      <c r="I62" s="104" t="n"/>
-      <c r="J62" s="104" t="n"/>
-      <c r="K62" s="104" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="98" t="inlineStr">
+      <c r="B65" s="104" t="n"/>
+      <c r="C65" s="104" t="n"/>
+      <c r="D65" s="104" t="n"/>
+      <c r="E65" s="104" t="n"/>
+      <c r="F65" s="104" t="n"/>
+      <c r="G65" s="104" t="n"/>
+      <c r="H65" s="104" t="n"/>
+      <c r="I65" s="104" t="n"/>
+      <c r="J65" s="104" t="n"/>
+      <c r="K65" s="104" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="98" t="inlineStr">
         <is>
           <t>Person</t>
         </is>
       </c>
-      <c r="B63" s="98" t="inlineStr">
+      <c r="B66" s="98" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="C63" s="98" t="inlineStr">
+      <c r="C66" s="98" t="inlineStr">
         <is>
           <t>Sell</t>
         </is>
       </c>
-      <c r="D63" s="98" t="inlineStr">
+      <c r="D66" s="98" t="inlineStr">
         <is>
           <t>Margin</t>
         </is>
       </c>
-      <c r="E63" s="98" t="inlineStr">
+      <c r="E66" s="98" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F63" s="98" t="inlineStr">
+      <c r="F66" s="98" t="inlineStr">
         <is>
           <t>#</t>
         </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="108">
-        <f>F2</f>
-        <v/>
-      </c>
-      <c r="B64" s="131">
-        <f>SUMPRODUCT((F7:F11="●")*1,B7:B11,C7:C11)+SUMPRODUCT((F15:F17="●")*1,B15:B17,C15:C17)+SUMPRODUCT((F21:F23="●")*1,B21:B23,C21:C23)+SUMPRODUCT((F27:F31="●")*1,B27:B31,C27:C31)+SUMPRODUCT((F35:F37="●")*1,B35:B37,C35:C37)+SUMPRODUCT((F41:F49="●")*1,B41:B49,C41:C49)</f>
-        <v/>
-      </c>
-      <c r="C64" s="131">
-        <f>SUMPRODUCT((F7:F11="●")*1,B7:B11,D7:D11)+SUMPRODUCT((F15:F17="●")*1,B15:B17,D15:D17)+SUMPRODUCT((F21:F23="●")*1,B21:B23,D21:D23)+SUMPRODUCT((F27:F31="●")*1,B27:B31,D27:D31)+SUMPRODUCT((F35:F37="●")*1,B35:B37,D35:D37)+SUMPRODUCT((F41:F49="●")*1,B41:B49,D41:D49)</f>
-        <v/>
-      </c>
-      <c r="D64" s="110">
-        <f>C64-B64</f>
-        <v/>
-      </c>
-      <c r="E64" s="132">
-        <f>IF(C64&gt;0,D64/C64,0)</f>
-        <v/>
-      </c>
-      <c r="F64" s="139">
-        <f>COUNTIF(F7:F11,"●")+COUNTIF(F15:F17,"●")+COUNTIF(F21:F23,"●")+COUNTIF(F27:F31,"●")+COUNTIF(F35:F37,"●")+COUNTIF(F41:F49,"●")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="108">
-        <f>G2</f>
-        <v/>
-      </c>
-      <c r="B65" s="131">
-        <f>SUMPRODUCT((G7:G11="●")*1,B7:B11,C7:C11)+SUMPRODUCT((G15:G17="●")*1,B15:B17,C15:C17)+SUMPRODUCT((G21:G23="●")*1,B21:B23,C21:C23)+SUMPRODUCT((G27:G31="●")*1,B27:B31,C27:C31)+SUMPRODUCT((G35:G37="●")*1,B35:B37,C35:C37)+SUMPRODUCT((G41:G49="●")*1,B41:B49,C41:C49)</f>
-        <v/>
-      </c>
-      <c r="C65" s="131">
-        <f>SUMPRODUCT((G7:G11="●")*1,B7:B11,D7:D11)+SUMPRODUCT((G15:G17="●")*1,B15:B17,D15:D17)+SUMPRODUCT((G21:G23="●")*1,B21:B23,D21:D23)+SUMPRODUCT((G27:G31="●")*1,B27:B31,D27:D31)+SUMPRODUCT((G35:G37="●")*1,B35:B37,D35:D37)+SUMPRODUCT((G41:G49="●")*1,B41:B49,D41:D49)</f>
-        <v/>
-      </c>
-      <c r="D65" s="110">
-        <f>C65-B65</f>
-        <v/>
-      </c>
-      <c r="E65" s="132">
-        <f>IF(C65&gt;0,D65/C65,0)</f>
-        <v/>
-      </c>
-      <c r="F65" s="139">
-        <f>COUNTIF(G7:G11,"●")+COUNTIF(G15:G17,"●")+COUNTIF(G21:G23,"●")+COUNTIF(G27:G31,"●")+COUNTIF(G35:G37,"●")+COUNTIF(G41:G49,"●")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="108">
-        <f>H2</f>
-        <v/>
-      </c>
-      <c r="B66" s="131">
-        <f>SUMPRODUCT((H7:H11="●")*1,B7:B11,C7:C11)+SUMPRODUCT((H15:H17="●")*1,B15:B17,C15:C17)+SUMPRODUCT((H21:H23="●")*1,B21:B23,C21:C23)+SUMPRODUCT((H27:H31="●")*1,B27:B31,C27:C31)+SUMPRODUCT((H35:H37="●")*1,B35:B37,C35:C37)+SUMPRODUCT((H41:H49="●")*1,B41:B49,C41:C49)</f>
-        <v/>
-      </c>
-      <c r="C66" s="131">
-        <f>SUMPRODUCT((H7:H11="●")*1,B7:B11,D7:D11)+SUMPRODUCT((H15:H17="●")*1,B15:B17,D15:D17)+SUMPRODUCT((H21:H23="●")*1,B21:B23,D21:D23)+SUMPRODUCT((H27:H31="●")*1,B27:B31,D27:D31)+SUMPRODUCT((H35:H37="●")*1,B35:B37,D35:D37)+SUMPRODUCT((H41:H49="●")*1,B41:B49,D41:D49)</f>
-        <v/>
-      </c>
-      <c r="D66" s="110">
-        <f>C66-B66</f>
-        <v/>
-      </c>
-      <c r="E66" s="132">
-        <f>IF(C66&gt;0,D66/C66,0)</f>
-        <v/>
-      </c>
-      <c r="F66" s="139">
-        <f>COUNTIF(H7:H11,"●")+COUNTIF(H15:H17,"●")+COUNTIF(H21:H23,"●")+COUNTIF(H27:H31,"●")+COUNTIF(H35:H37,"●")+COUNTIF(H41:H49,"●")</f>
-        <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="108">
-        <f>I2</f>
+        <f>F2</f>
         <v/>
       </c>
       <c r="B67" s="131">
-        <f>SUMPRODUCT((I7:I11="●")*1,B7:B11,C7:C11)+SUMPRODUCT((I15:I17="●")*1,B15:B17,C15:C17)+SUMPRODUCT((I21:I23="●")*1,B21:B23,C21:C23)+SUMPRODUCT((I27:I31="●")*1,B27:B31,C27:C31)+SUMPRODUCT((I35:I37="●")*1,B35:B37,C35:C37)+SUMPRODUCT((I41:I49="●")*1,B41:B49,C41:C49)</f>
+        <f>SUMPRODUCT((F10:F14="●")*1,B10:B14,C10:C14)+SUMPRODUCT((F18:F20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((F24:F26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((F30:F34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((F38:F40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((F44:F52="●")*1,B44:B52,C44:C52)</f>
         <v/>
       </c>
       <c r="C67" s="131">
-        <f>SUMPRODUCT((I7:I11="●")*1,B7:B11,D7:D11)+SUMPRODUCT((I15:I17="●")*1,B15:B17,D15:D17)+SUMPRODUCT((I21:I23="●")*1,B21:B23,D21:D23)+SUMPRODUCT((I27:I31="●")*1,B27:B31,D27:D31)+SUMPRODUCT((I35:I37="●")*1,B35:B37,D35:D37)+SUMPRODUCT((I41:I49="●")*1,B41:B49,D41:D49)</f>
+        <f>SUMPRODUCT((F10:F14="●")*1,B10:B14,D10:D14)+SUMPRODUCT((F18:F20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((F24:F26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((F30:F34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((F38:F40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((F44:F52="●")*1,B44:B52,D44:D52)</f>
         <v/>
       </c>
       <c r="D67" s="110">
@@ -5413,743 +5384,826 @@
         <v/>
       </c>
       <c r="F67" s="139">
-        <f>COUNTIF(I7:I11,"●")+COUNTIF(I15:I17,"●")+COUNTIF(I21:I23,"●")+COUNTIF(I27:I31,"●")+COUNTIF(I35:I37,"●")+COUNTIF(I41:I49,"●")</f>
+        <f>COUNTIF(F10:F14,"●")+COUNTIF(F18:F20,"●")+COUNTIF(F24:F26,"●")+COUNTIF(F30:F34,"●")+COUNTIF(F38:F40,"●")+COUNTIF(F44:F52,"●")</f>
         <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="115" t="inlineStr">
+      <c r="A68" s="108">
+        <f>G2</f>
+        <v/>
+      </c>
+      <c r="B68" s="131">
+        <f>SUMPRODUCT((G10:G14="●")*1,B10:B14,C10:C14)+SUMPRODUCT((G18:G20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((G24:G26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((G30:G34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((G38:G40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((G44:G52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="C68" s="131">
+        <f>SUMPRODUCT((G10:G14="●")*1,B10:B14,D10:D14)+SUMPRODUCT((G18:G20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((G24:G26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((G30:G34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((G38:G40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((G44:G52="●")*1,B44:B52,D44:D52)</f>
+        <v/>
+      </c>
+      <c r="D68" s="110">
+        <f>C68-B68</f>
+        <v/>
+      </c>
+      <c r="E68" s="132">
+        <f>IF(C68&gt;0,D68/C68,0)</f>
+        <v/>
+      </c>
+      <c r="F68" s="139">
+        <f>COUNTIF(G10:G14,"●")+COUNTIF(G18:G20,"●")+COUNTIF(G24:G26,"●")+COUNTIF(G30:G34,"●")+COUNTIF(G38:G40,"●")+COUNTIF(G44:G52,"●")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="108">
+        <f>H2</f>
+        <v/>
+      </c>
+      <c r="B69" s="131">
+        <f>SUMPRODUCT((H10:H14="●")*1,B10:B14,C10:C14)+SUMPRODUCT((H18:H20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((H24:H26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((H30:H34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((H38:H40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((H44:H52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="C69" s="131">
+        <f>SUMPRODUCT((H10:H14="●")*1,B10:B14,D10:D14)+SUMPRODUCT((H18:H20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((H24:H26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((H30:H34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((H38:H40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((H44:H52="●")*1,B44:B52,D44:D52)</f>
+        <v/>
+      </c>
+      <c r="D69" s="110">
+        <f>C69-B69</f>
+        <v/>
+      </c>
+      <c r="E69" s="132">
+        <f>IF(C69&gt;0,D69/C69,0)</f>
+        <v/>
+      </c>
+      <c r="F69" s="139">
+        <f>COUNTIF(H10:H14,"●")+COUNTIF(H18:H20,"●")+COUNTIF(H24:H26,"●")+COUNTIF(H30:H34,"●")+COUNTIF(H38:H40,"●")+COUNTIF(H44:H52,"●")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="108">
+        <f>I2</f>
+        <v/>
+      </c>
+      <c r="B70" s="131">
+        <f>SUMPRODUCT((I10:I14="●")*1,B10:B14,C10:C14)+SUMPRODUCT((I18:I20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((I24:I26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((I30:I34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((I38:I40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((I44:I52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="C70" s="131">
+        <f>SUMPRODUCT((I10:I14="●")*1,B10:B14,D10:D14)+SUMPRODUCT((I18:I20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((I24:I26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((I30:I34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((I38:I40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((I44:I52="●")*1,B44:B52,D44:D52)</f>
+        <v/>
+      </c>
+      <c r="D70" s="110">
+        <f>C70-B70</f>
+        <v/>
+      </c>
+      <c r="E70" s="132">
+        <f>IF(C70&gt;0,D70/C70,0)</f>
+        <v/>
+      </c>
+      <c r="F70" s="139">
+        <f>COUNTIF(I10:I14,"●")+COUNTIF(I18:I20,"●")+COUNTIF(I24:I26,"●")+COUNTIF(I30:I34,"●")+COUNTIF(I38:I40,"●")+COUNTIF(I44:I52,"●")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="115" t="inlineStr">
         <is>
           <t>📌 TOTAL</t>
         </is>
       </c>
-      <c r="B68" s="88">
-        <f>SUM(B64:B67)</f>
-        <v/>
-      </c>
-      <c r="C68" s="88">
-        <f>SUM(C64:C67)</f>
-        <v/>
-      </c>
-      <c r="D68" s="88">
-        <f>SUM(D64:D67)</f>
+      <c r="B71" s="88">
+        <f>SUM(B67:B70)</f>
+        <v/>
+      </c>
+      <c r="C71" s="88">
+        <f>SUM(C67:C70)</f>
+        <v/>
+      </c>
+      <c r="D71" s="88">
+        <f>SUM(D67:D70)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A6:K6"/>
-    <mergeCell ref="A53:K53"/>
-    <mergeCell ref="A34:K34"/>
+  <mergeCells count="15">
+    <mergeCell ref="A56:K56"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="A62:K62"/>
-    <mergeCell ref="A20:K20"/>
-    <mergeCell ref="A26:K26"/>
-    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A37:K37"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A23:K23"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A29:K29"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="A43:K43"/>
+    <mergeCell ref="E6:H6"/>
+    <mergeCell ref="A65:K65"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A40:K40"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A9:K9"/>
   </mergeCells>
-  <conditionalFormatting sqref="F7">
+  <conditionalFormatting sqref="F10">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G7">
+  <conditionalFormatting sqref="G10">
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7">
+  <conditionalFormatting sqref="H10">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I7">
+  <conditionalFormatting sqref="I10">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P7">
+  <conditionalFormatting sqref="P10">
     <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F8">
+  <conditionalFormatting sqref="F11">
     <cfRule type="cellIs" priority="6" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G8">
+  <conditionalFormatting sqref="G11">
     <cfRule type="cellIs" priority="7" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H8">
+  <conditionalFormatting sqref="H11">
     <cfRule type="cellIs" priority="8" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I8">
+  <conditionalFormatting sqref="I11">
     <cfRule type="cellIs" priority="9" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P8">
+  <conditionalFormatting sqref="P11">
     <cfRule type="cellIs" priority="10" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F9">
+  <conditionalFormatting sqref="F12">
     <cfRule type="cellIs" priority="11" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G9">
+  <conditionalFormatting sqref="G12">
     <cfRule type="cellIs" priority="12" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9">
+  <conditionalFormatting sqref="H12">
     <cfRule type="cellIs" priority="13" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I9">
+  <conditionalFormatting sqref="I12">
     <cfRule type="cellIs" priority="14" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P9">
+  <conditionalFormatting sqref="P12">
     <cfRule type="cellIs" priority="15" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F10">
+  <conditionalFormatting sqref="F13">
     <cfRule type="cellIs" priority="16" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G10">
+  <conditionalFormatting sqref="G13">
     <cfRule type="cellIs" priority="17" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H10">
+  <conditionalFormatting sqref="H13">
     <cfRule type="cellIs" priority="18" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I10">
+  <conditionalFormatting sqref="I13">
     <cfRule type="cellIs" priority="19" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P10">
+  <conditionalFormatting sqref="P13">
     <cfRule type="cellIs" priority="20" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F11">
+  <conditionalFormatting sqref="F14">
     <cfRule type="cellIs" priority="21" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11">
+  <conditionalFormatting sqref="G14">
     <cfRule type="cellIs" priority="22" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H11">
+  <conditionalFormatting sqref="H14">
     <cfRule type="cellIs" priority="23" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I11">
+  <conditionalFormatting sqref="I14">
     <cfRule type="cellIs" priority="24" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P11">
+  <conditionalFormatting sqref="P14">
     <cfRule type="cellIs" priority="25" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F15">
+  <conditionalFormatting sqref="F18">
     <cfRule type="cellIs" priority="26" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G15">
+  <conditionalFormatting sqref="G18">
     <cfRule type="cellIs" priority="27" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H15">
+  <conditionalFormatting sqref="H18">
     <cfRule type="cellIs" priority="28" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I15">
+  <conditionalFormatting sqref="I18">
     <cfRule type="cellIs" priority="29" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P15">
+  <conditionalFormatting sqref="P18">
     <cfRule type="cellIs" priority="30" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F16">
+  <conditionalFormatting sqref="F19">
     <cfRule type="cellIs" priority="31" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16">
+  <conditionalFormatting sqref="G19">
     <cfRule type="cellIs" priority="32" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H16">
+  <conditionalFormatting sqref="H19">
     <cfRule type="cellIs" priority="33" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I16">
+  <conditionalFormatting sqref="I19">
     <cfRule type="cellIs" priority="34" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P16">
+  <conditionalFormatting sqref="P19">
     <cfRule type="cellIs" priority="35" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F17">
+  <conditionalFormatting sqref="F20">
     <cfRule type="cellIs" priority="36" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G17">
+  <conditionalFormatting sqref="G20">
     <cfRule type="cellIs" priority="37" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H17">
+  <conditionalFormatting sqref="H20">
     <cfRule type="cellIs" priority="38" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I17">
+  <conditionalFormatting sqref="I20">
     <cfRule type="cellIs" priority="39" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P17">
+  <conditionalFormatting sqref="P20">
     <cfRule type="cellIs" priority="40" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F21">
+  <conditionalFormatting sqref="F24">
     <cfRule type="cellIs" priority="41" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G21">
+  <conditionalFormatting sqref="G24">
     <cfRule type="cellIs" priority="42" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H21">
+  <conditionalFormatting sqref="H24">
     <cfRule type="cellIs" priority="43" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I21">
+  <conditionalFormatting sqref="I24">
     <cfRule type="cellIs" priority="44" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P21">
+  <conditionalFormatting sqref="P24">
     <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F22">
+  <conditionalFormatting sqref="F25">
     <cfRule type="cellIs" priority="46" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G22">
+  <conditionalFormatting sqref="G25">
     <cfRule type="cellIs" priority="47" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H22">
+  <conditionalFormatting sqref="H25">
     <cfRule type="cellIs" priority="48" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I22">
+  <conditionalFormatting sqref="I25">
     <cfRule type="cellIs" priority="49" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P22">
+  <conditionalFormatting sqref="P25">
     <cfRule type="cellIs" priority="50" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F23">
+  <conditionalFormatting sqref="F26">
     <cfRule type="cellIs" priority="51" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G23">
+  <conditionalFormatting sqref="G26">
     <cfRule type="cellIs" priority="52" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H23">
+  <conditionalFormatting sqref="H26">
     <cfRule type="cellIs" priority="53" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I23">
+  <conditionalFormatting sqref="I26">
     <cfRule type="cellIs" priority="54" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P23">
+  <conditionalFormatting sqref="P26">
     <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F27">
+  <conditionalFormatting sqref="F30">
     <cfRule type="cellIs" priority="56" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G27">
+  <conditionalFormatting sqref="G30">
     <cfRule type="cellIs" priority="57" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H27">
+  <conditionalFormatting sqref="H30">
     <cfRule type="cellIs" priority="58" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I27">
+  <conditionalFormatting sqref="I30">
     <cfRule type="cellIs" priority="59" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P27">
+  <conditionalFormatting sqref="P30">
     <cfRule type="cellIs" priority="60" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F28">
+  <conditionalFormatting sqref="F31">
     <cfRule type="cellIs" priority="61" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G28">
+  <conditionalFormatting sqref="G31">
     <cfRule type="cellIs" priority="62" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H28">
+  <conditionalFormatting sqref="H31">
     <cfRule type="cellIs" priority="63" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I28">
+  <conditionalFormatting sqref="I31">
     <cfRule type="cellIs" priority="64" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P28">
+  <conditionalFormatting sqref="P31">
     <cfRule type="cellIs" priority="65" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F29">
+  <conditionalFormatting sqref="F32">
     <cfRule type="cellIs" priority="66" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G29">
+  <conditionalFormatting sqref="G32">
     <cfRule type="cellIs" priority="67" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H29">
+  <conditionalFormatting sqref="H32">
     <cfRule type="cellIs" priority="68" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I29">
+  <conditionalFormatting sqref="I32">
     <cfRule type="cellIs" priority="69" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P29">
+  <conditionalFormatting sqref="P32">
     <cfRule type="cellIs" priority="70" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F30">
+  <conditionalFormatting sqref="F33">
     <cfRule type="cellIs" priority="71" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G30">
+  <conditionalFormatting sqref="G33">
     <cfRule type="cellIs" priority="72" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H30">
+  <conditionalFormatting sqref="H33">
     <cfRule type="cellIs" priority="73" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I30">
+  <conditionalFormatting sqref="I33">
     <cfRule type="cellIs" priority="74" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P30">
+  <conditionalFormatting sqref="P33">
     <cfRule type="cellIs" priority="75" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F31">
+  <conditionalFormatting sqref="F34">
     <cfRule type="cellIs" priority="76" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G31">
+  <conditionalFormatting sqref="G34">
     <cfRule type="cellIs" priority="77" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H31">
+  <conditionalFormatting sqref="H34">
     <cfRule type="cellIs" priority="78" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I31">
+  <conditionalFormatting sqref="I34">
     <cfRule type="cellIs" priority="79" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P31">
+  <conditionalFormatting sqref="P34">
     <cfRule type="cellIs" priority="80" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F35">
+  <conditionalFormatting sqref="F38">
     <cfRule type="cellIs" priority="81" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G35">
+  <conditionalFormatting sqref="G38">
     <cfRule type="cellIs" priority="82" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H35">
+  <conditionalFormatting sqref="H38">
     <cfRule type="cellIs" priority="83" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I35">
+  <conditionalFormatting sqref="I38">
     <cfRule type="cellIs" priority="84" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P35">
+  <conditionalFormatting sqref="P38">
     <cfRule type="cellIs" priority="85" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F36">
+  <conditionalFormatting sqref="F39">
     <cfRule type="cellIs" priority="86" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G36">
+  <conditionalFormatting sqref="G39">
     <cfRule type="cellIs" priority="87" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H36">
+  <conditionalFormatting sqref="H39">
     <cfRule type="cellIs" priority="88" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I36">
+  <conditionalFormatting sqref="I39">
     <cfRule type="cellIs" priority="89" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P36">
+  <conditionalFormatting sqref="P39">
     <cfRule type="cellIs" priority="90" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F37">
+  <conditionalFormatting sqref="F40">
     <cfRule type="cellIs" priority="91" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G37">
+  <conditionalFormatting sqref="G40">
     <cfRule type="cellIs" priority="92" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H37">
+  <conditionalFormatting sqref="H40">
     <cfRule type="cellIs" priority="93" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I37">
+  <conditionalFormatting sqref="I40">
     <cfRule type="cellIs" priority="94" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P37">
+  <conditionalFormatting sqref="P40">
     <cfRule type="cellIs" priority="95" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F41">
+  <conditionalFormatting sqref="F44">
     <cfRule type="cellIs" priority="96" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G41">
+  <conditionalFormatting sqref="G44">
     <cfRule type="cellIs" priority="97" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H41">
+  <conditionalFormatting sqref="H44">
     <cfRule type="cellIs" priority="98" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I41">
+  <conditionalFormatting sqref="I44">
     <cfRule type="cellIs" priority="99" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P41">
+  <conditionalFormatting sqref="P44">
     <cfRule type="cellIs" priority="100" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F42">
+  <conditionalFormatting sqref="F45">
     <cfRule type="cellIs" priority="101" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G42">
+  <conditionalFormatting sqref="G45">
     <cfRule type="cellIs" priority="102" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H42">
+  <conditionalFormatting sqref="H45">
     <cfRule type="cellIs" priority="103" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I42">
+  <conditionalFormatting sqref="I45">
     <cfRule type="cellIs" priority="104" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P42">
+  <conditionalFormatting sqref="P45">
     <cfRule type="cellIs" priority="105" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F43">
+  <conditionalFormatting sqref="F46">
     <cfRule type="cellIs" priority="106" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G43">
+  <conditionalFormatting sqref="G46">
     <cfRule type="cellIs" priority="107" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H43">
+  <conditionalFormatting sqref="H46">
     <cfRule type="cellIs" priority="108" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I43">
+  <conditionalFormatting sqref="I46">
     <cfRule type="cellIs" priority="109" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P43">
+  <conditionalFormatting sqref="P46">
     <cfRule type="cellIs" priority="110" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F44">
+  <conditionalFormatting sqref="F47">
     <cfRule type="cellIs" priority="111" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G44">
+  <conditionalFormatting sqref="G47">
     <cfRule type="cellIs" priority="112" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H44">
+  <conditionalFormatting sqref="H47">
     <cfRule type="cellIs" priority="113" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I44">
+  <conditionalFormatting sqref="I47">
     <cfRule type="cellIs" priority="114" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P44">
+  <conditionalFormatting sqref="P47">
     <cfRule type="cellIs" priority="115" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F45">
+  <conditionalFormatting sqref="F48">
     <cfRule type="cellIs" priority="116" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G45">
+  <conditionalFormatting sqref="G48">
     <cfRule type="cellIs" priority="117" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H45">
+  <conditionalFormatting sqref="H48">
     <cfRule type="cellIs" priority="118" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I45">
+  <conditionalFormatting sqref="I48">
     <cfRule type="cellIs" priority="119" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P45">
+  <conditionalFormatting sqref="P48">
     <cfRule type="cellIs" priority="120" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F46">
+  <conditionalFormatting sqref="F49">
     <cfRule type="cellIs" priority="121" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G46">
+  <conditionalFormatting sqref="G49">
     <cfRule type="cellIs" priority="122" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H46">
+  <conditionalFormatting sqref="H49">
     <cfRule type="cellIs" priority="123" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I46">
+  <conditionalFormatting sqref="I49">
     <cfRule type="cellIs" priority="124" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P46">
+  <conditionalFormatting sqref="P49">
     <cfRule type="cellIs" priority="125" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F47">
+  <conditionalFormatting sqref="F50">
     <cfRule type="cellIs" priority="126" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G47">
+  <conditionalFormatting sqref="G50">
     <cfRule type="cellIs" priority="127" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H47">
+  <conditionalFormatting sqref="H50">
     <cfRule type="cellIs" priority="128" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I47">
+  <conditionalFormatting sqref="I50">
     <cfRule type="cellIs" priority="129" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P47">
+  <conditionalFormatting sqref="P50">
     <cfRule type="cellIs" priority="130" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F48">
+  <conditionalFormatting sqref="F51">
     <cfRule type="cellIs" priority="131" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G48">
+  <conditionalFormatting sqref="G51">
     <cfRule type="cellIs" priority="132" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H48">
+  <conditionalFormatting sqref="H51">
     <cfRule type="cellIs" priority="133" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I48">
+  <conditionalFormatting sqref="I51">
     <cfRule type="cellIs" priority="134" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P48">
+  <conditionalFormatting sqref="P51">
     <cfRule type="cellIs" priority="135" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F49">
+  <conditionalFormatting sqref="F52">
     <cfRule type="cellIs" priority="136" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G49">
+  <conditionalFormatting sqref="G52">
     <cfRule type="cellIs" priority="137" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H49">
+  <conditionalFormatting sqref="H52">
     <cfRule type="cellIs" priority="138" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I49">
+  <conditionalFormatting sqref="I52">
     <cfRule type="cellIs" priority="139" operator="equal" dxfId="6">
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P49">
+  <conditionalFormatting sqref="P52">
     <cfRule type="cellIs" priority="140" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K4">
+  <conditionalFormatting sqref="I7">
     <cfRule type="cellIs" priority="141" operator="equal" dxfId="3">
       <formula>"❌"</formula>
     </cfRule>
@@ -6158,34 +6212,34 @@
     <dataValidation sqref="E2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"2,4,6,8"</formula1>
     </dataValidation>
-    <dataValidation sqref="C3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>'Master Data'!$A$60:$A$63</formula1>
     </dataValidation>
-    <dataValidation sqref="I3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="J4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"First,Business,Premium Economy,Economy"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>'Master Data'!$A$74:$A$77</formula1>
     </dataValidation>
-    <dataValidation sqref="F3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"First,Business,Premium Economy,Economy"</formula1>
+    <dataValidation sqref="F10 F11 F12 F13 F14 F18 F19 F20 F24 F25 F26 F30 F31 F32 F33 F34 F38 F39 F40 F44 F45 F46 F47 F48 F49 F50 F51 F52 G10 G11 G12 G13 G14 G18 G19 G20 G24 G25 G26 G30 G31 G32 G33 G34 G38 G39 G40 G44 G45 G46 G47 G48 G49 G50 G51 G52 H10 H11 H12 H13 H14 H18 H19 H20 H24 H25 H26 H30 H31 H32 H33 H34 H38 H39 H40 H44 H45 H46 H47 H48 H49 H50 H51 H52 I10 I11 I12 I13 I14 I18 I19 I20 I24 I25 I26 I30 I31 I32 I33 I34 I38 I39 I40 I44 I45 I46 I47 I48 I49 I50 I51 I52 L10 L11 L12 L13 L14 L18 L19 L20 L24 L25 L26 L30 L31 L32 L33 L34 L38 L39 L40 L44 L45 L46 L47 L48 L49 L50 L51 L52 M10 M11 M12 M13 M14 M18 M19 M20 M24 M25 M26 M30 M31 M32 M33 M34 M38 M39 M40 M44 M45 M46 M47 M48 M49 M50 M51 M52 N10 N11 N12 N13 N14 N18 N19 N20 N24 N25 N26 N30 N31 N32 N33 N34 N38 N39 N40 N44 N45 N46 N47 N48 N49 N50 N51 N52 O10 O11 O12 O13 O14 O18 O19 O20 O24 O25 O26 O30 O31 O32 O33 O34 O38 O39 O40 O44 O45 O46 O47 O48 O49 O50 O51 O52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Toggle" error="● = ON, blank = OFF" type="list">
+      <formula1>"●"</formula1>
     </dataValidation>
-    <dataValidation sqref="F7 F8 F9 F10 F11 F15 F16 F17 F21 F22 F23 F27 F28 F29 F30 F31 F35 F36 F37 F41 F42 F43 F44 F45 F46 F47 F48 F49 G7 G8 G9 G10 G11 G15 G16 G17 G21 G22 G23 G27 G28 G29 G30 G31 G35 G36 G37 G41 G42 G43 G44 G45 G46 G47 G48 G49 H7 H8 H9 H10 H11 H15 H16 H17 H21 H22 H23 H27 H28 H29 H30 H31 H35 H36 H37 H41 H42 H43 H44 H45 H46 H47 H48 H49 I7 I8 I9 I10 I11 I15 I16 I17 I21 I22 I23 I27 I28 I29 I30 I31 I35 I36 I37 I41 I42 I43 I44 I45 I46 I47 I48 I49 L7 L8 L9 L10 L11 L15 L16 L17 L21 L22 L23 L27 L28 L29 L30 L31 L35 L36 L37 L41 L42 L43 L44 L45 L46 L47 L48 L49 M7 M8 M9 M10 M11 M15 M16 M17 M21 M22 M23 M27 M28 M29 M30 M31 M35 M36 M37 M41 M42 M43 M44 M45 M46 M47 M48 M49 N7 N8 N9 N10 N11 N15 N16 N17 N21 N22 N23 N27 N28 N29 N30 N31 N35 N36 N37 N41 N42 N43 N44 N45 N46 N47 N48 N49 O7 O8 O9 O10 O11 O15 O16 O17 O21 O22 O23 O27 O28 O29 O30 O31 O35 O36 O37 O41 O42 O43 O44 O45 O46 O47 O48 O49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"●",</formula1>
-    </dataValidation>
-    <dataValidation sqref="A7 A8 A9 A10 A11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A10 A11 A12 A13 A14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Master Data'!$A$7:$A$14</formula1>
     </dataValidation>
-    <dataValidation sqref="A15 A16 A17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A18 A19 A20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Master Data'!$A$19:$A$24</formula1>
     </dataValidation>
-    <dataValidation sqref="A21 A22 A23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A24 A25 A26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Master Data'!$A$28:$A$34</formula1>
     </dataValidation>
-    <dataValidation sqref="A27 A28 A29 A30 A31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A30 A31 A32 A33 A34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Master Data'!$A$38:$A$46</formula1>
     </dataValidation>
-    <dataValidation sqref="A35 A36 A37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A38 A39 A40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Master Data'!$A$50:$A$56</formula1>
     </dataValidation>
-    <dataValidation sqref="A41 A42 A43 A44 A45 A46 A47 A48 A49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A44 A45 A46 A47 A48 A49 A50 A51 A52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>'Master Data'!$A$86:$A$94</formula1>
     </dataValidation>
   </dataValidations>
@@ -6261,11 +6315,11 @@
         </is>
       </c>
       <c r="B5" s="84">
-        <f>'Package Selector'!J12</f>
+        <f>'Package Selector'!J15</f>
         <v/>
       </c>
       <c r="C5" s="84">
-        <f>'Package Selector'!K12</f>
+        <f>'Package Selector'!K15</f>
         <v/>
       </c>
       <c r="D5" s="84">
@@ -6288,11 +6342,11 @@
         </is>
       </c>
       <c r="B6" s="84">
-        <f>'Package Selector'!J18</f>
+        <f>'Package Selector'!J21</f>
         <v/>
       </c>
       <c r="C6" s="84">
-        <f>'Package Selector'!K18</f>
+        <f>'Package Selector'!K21</f>
         <v/>
       </c>
       <c r="D6" s="84">
@@ -6315,11 +6369,11 @@
         </is>
       </c>
       <c r="B7" s="84">
-        <f>'Package Selector'!J24</f>
+        <f>'Package Selector'!J27</f>
         <v/>
       </c>
       <c r="C7" s="84">
-        <f>'Package Selector'!K24</f>
+        <f>'Package Selector'!K27</f>
         <v/>
       </c>
       <c r="D7" s="84">
@@ -6342,11 +6396,11 @@
         </is>
       </c>
       <c r="B8" s="84">
-        <f>'Package Selector'!J32</f>
+        <f>'Package Selector'!J35</f>
         <v/>
       </c>
       <c r="C8" s="84">
-        <f>'Package Selector'!K32</f>
+        <f>'Package Selector'!K35</f>
         <v/>
       </c>
       <c r="D8" s="84">
@@ -6369,11 +6423,11 @@
         </is>
       </c>
       <c r="B9" s="84">
-        <f>'Package Selector'!J38</f>
+        <f>'Package Selector'!J41</f>
         <v/>
       </c>
       <c r="C9" s="84">
-        <f>'Package Selector'!K38</f>
+        <f>'Package Selector'!K41</f>
         <v/>
       </c>
       <c r="D9" s="84">
@@ -6396,11 +6450,11 @@
         </is>
       </c>
       <c r="B10" s="84">
-        <f>'Package Selector'!J50</f>
+        <f>'Package Selector'!J53</f>
         <v/>
       </c>
       <c r="C10" s="84">
-        <f>'Package Selector'!K50</f>
+        <f>'Package Selector'!K53</f>
         <v/>
       </c>
       <c r="D10" s="84">

</xml_diff>

<commit_message>
feat: Duration fix, Master Data margin$, Package Types restructured, Guest Package tab
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -9,7 +9,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Types" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Selector" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profit Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Summary" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guest Package" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -512,7 +513,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="146">
+  <cellXfs count="157">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -899,6 +900,37 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="17" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1418,7 +1450,7 @@
           <t>Sell ($)</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="146" t="inlineStr">
         <is>
           <t>Margin ($)</t>
         </is>
@@ -1594,9 +1626,9 @@
           <t>Sell/night</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Margin</t>
+      <c r="D18" s="146" t="inlineStr">
+        <is>
+          <t>Margin ($)</t>
         </is>
       </c>
       <c r="E18" s="2" t="n"/>
@@ -1708,9 +1740,9 @@
           <t>Sell/p</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Margin</t>
+      <c r="D27" s="146" t="inlineStr">
+        <is>
+          <t>Margin ($)</t>
         </is>
       </c>
       <c r="E27" s="2" t="n"/>
@@ -1844,9 +1876,9 @@
           <t>Sell</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>Margin</t>
+      <c r="D37" s="146" t="inlineStr">
+        <is>
+          <t>Margin ($)</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
@@ -2024,9 +2056,9 @@
           <t>Sell</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Margin</t>
+      <c r="D49" s="146" t="inlineStr">
+        <is>
+          <t>Margin ($)</t>
         </is>
       </c>
       <c r="E49" s="2" t="n"/>
@@ -2109,6 +2141,7 @@
       </c>
       <c r="F55" s="6" t="n"/>
     </row>
+    <row r="56"/>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
         <is>
@@ -2708,7 +2741,7 @@
           <t>Sell ($)</t>
         </is>
       </c>
-      <c r="D85" s="46" t="inlineStr">
+      <c r="D85" s="146" t="inlineStr">
         <is>
           <t>Margin ($)</t>
         </is>
@@ -2736,7 +2769,7 @@
       <c r="C86" s="75" t="n">
         <v>100</v>
       </c>
-      <c r="D86" s="51">
+      <c r="D86" s="147">
         <f>IF(A86="","",C86-B86)</f>
         <v/>
       </c>
@@ -2764,7 +2797,7 @@
       <c r="C87" s="75" t="n">
         <v>30</v>
       </c>
-      <c r="D87" s="51">
+      <c r="D87" s="147">
         <f>IF(A87="","",C87-B87)</f>
         <v/>
       </c>
@@ -2792,7 +2825,7 @@
       <c r="C88" s="75" t="n">
         <v>180</v>
       </c>
-      <c r="D88" s="51">
+      <c r="D88" s="147">
         <f>IF(A88="","",C88-B88)</f>
         <v/>
       </c>
@@ -2820,7 +2853,7 @@
       <c r="C89" s="75" t="n">
         <v>90</v>
       </c>
-      <c r="D89" s="51">
+      <c r="D89" s="147">
         <f>IF(A89="","",C89-B89)</f>
         <v/>
       </c>
@@ -2844,7 +2877,7 @@
       </c>
       <c r="B90" s="49" t="n"/>
       <c r="C90" s="49" t="n"/>
-      <c r="D90" s="51">
+      <c r="D90" s="147">
         <f>IF(A90="","",C90-B90)</f>
         <v/>
       </c>
@@ -2864,7 +2897,7 @@
       <c r="C91" s="49" t="n">
         <v>100</v>
       </c>
-      <c r="D91" s="51">
+      <c r="D91" s="147">
         <f>IF(A91="","",C91-B91)</f>
         <v/>
       </c>
@@ -2884,7 +2917,7 @@
       <c r="C92" s="49" t="n">
         <v>30</v>
       </c>
-      <c r="D92" s="51">
+      <c r="D92" s="147">
         <f>IF(A92="","",C92-B92)</f>
         <v/>
       </c>
@@ -2904,7 +2937,7 @@
       <c r="C93" s="49" t="n">
         <v>180</v>
       </c>
-      <c r="D93" s="51">
+      <c r="D93" s="147">
         <f>IF(A93="","",C93-B93)</f>
         <v/>
       </c>
@@ -2924,7 +2957,7 @@
       <c r="C94" s="49" t="n">
         <v>90</v>
       </c>
-      <c r="D94" s="51">
+      <c r="D94" s="147">
         <f>IF(A94="","",C94-B94)</f>
         <v/>
       </c>
@@ -2955,7 +2988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" style="42" min="1" max="1"/>
@@ -2987,6 +3020,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="16.5" customHeight="1" s="42">
       <c r="A4" s="76" t="inlineStr">
         <is>
@@ -2995,63 +3029,76 @@
       </c>
       <c r="B4" s="76" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>일정</t>
         </is>
       </c>
       <c r="C4" s="76" t="inlineStr">
         <is>
-          <t>일정</t>
+          <t>패키지명</t>
         </is>
       </c>
       <c r="D4" s="76" t="inlineStr">
         <is>
-          <t>패키지명</t>
+          <t>박</t>
         </is>
       </c>
       <c r="E4" s="76" t="inlineStr">
         <is>
-          <t>박</t>
+          <t>일</t>
         </is>
       </c>
       <c r="F4" s="76" t="inlineStr">
         <is>
-          <t>일</t>
+          <t>Rds</t>
         </is>
       </c>
       <c r="G4" s="76" t="inlineStr">
         <is>
-          <t>Rds</t>
-        </is>
-      </c>
-      <c r="H4" s="76" t="inlineStr">
-        <is>
-          <t>코스구성</t>
-        </is>
-      </c>
-      <c r="I4" s="77" t="inlineStr">
+          <t>패키지 구성</t>
+        </is>
+      </c>
+      <c r="H4" s="77" t="inlineStr">
         <is>
           <t>⛳ 골프</t>
         </is>
       </c>
-      <c r="J4" s="92" t="n"/>
-      <c r="K4" s="93" t="inlineStr">
+      <c r="I4" s="77" t="n"/>
+      <c r="J4" s="77" t="inlineStr">
         <is>
           <t>🔄 리플레이</t>
         </is>
       </c>
-      <c r="L4" s="92" t="n"/>
-      <c r="M4" s="77" t="inlineStr">
+      <c r="K4" s="77" t="n"/>
+      <c r="L4" s="77" t="inlineStr">
         <is>
           <t>🏨 호텔</t>
         </is>
       </c>
-      <c r="N4" s="92" t="n"/>
-      <c r="O4" s="76" t="inlineStr">
+      <c r="M4" s="77" t="n"/>
+      <c r="N4" s="77" t="inlineStr">
+        <is>
+          <t>🚐 교통</t>
+        </is>
+      </c>
+      <c r="O4" s="77" t="n"/>
+      <c r="P4" s="77" t="inlineStr">
+        <is>
+          <t>🍽️ 식사</t>
+        </is>
+      </c>
+      <c r="Q4" s="77" t="n"/>
+      <c r="R4" s="77" t="inlineStr">
+        <is>
+          <t>📦 기타</t>
+        </is>
+      </c>
+      <c r="S4" s="77" t="n"/>
+      <c r="T4" s="76" t="inlineStr">
         <is>
           <t>마진</t>
         </is>
       </c>
-      <c r="P4" s="76" t="inlineStr">
+      <c r="U4" s="76" t="inlineStr">
         <is>
           <t>마진율</t>
         </is>
@@ -3065,105 +3112,141 @@
       <c r="E5" s="78" t="n"/>
       <c r="F5" s="78" t="n"/>
       <c r="G5" s="78" t="n"/>
-      <c r="H5" s="78" t="n"/>
-      <c r="I5" s="78" t="inlineStr">
+      <c r="H5" s="148" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="J5" s="78" t="inlineStr">
+      <c r="I5" s="148" t="inlineStr">
         <is>
           <t>Sell</t>
         </is>
       </c>
-      <c r="K5" s="96" t="inlineStr">
+      <c r="J5" s="148" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="L5" s="96" t="inlineStr">
+      <c r="K5" s="148" t="inlineStr">
         <is>
           <t>Sell</t>
         </is>
       </c>
-      <c r="M5" s="78" t="inlineStr">
+      <c r="L5" s="148" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="N5" s="78" t="inlineStr">
+      <c r="M5" s="148" t="inlineStr">
         <is>
           <t>Sell</t>
         </is>
       </c>
-      <c r="O5" s="76" t="inlineStr">
-        <is>
-          <t>마진</t>
-        </is>
-      </c>
-      <c r="P5" s="76" t="inlineStr">
-        <is>
-          <t>마진율</t>
-        </is>
-      </c>
+      <c r="N5" s="148" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="O5" s="148" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="P5" s="148" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="Q5" s="148" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="R5" s="148" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="S5" s="148" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="T5" s="148" t="inlineStr"/>
+      <c r="U5" s="148" t="inlineStr"/>
     </row>
     <row r="6" ht="51" customHeight="1" s="42">
       <c r="A6" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>S1</t>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>3N4D</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>3N4D</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
           <t>트럼프 + 샌드파이퍼 오션뷰</t>
         </is>
       </c>
+      <c r="D6" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="E6" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="G6" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Trump×1 + Sand×1</t>
         </is>
       </c>
+      <c r="H6" s="149" t="inlineStr">
+        <is>
+          <t>G2·H3·T3·M3B3L3D2Ex·I4</t>
+        </is>
+      </c>
       <c r="I6" s="5" t="n">
-        <v>340</v>
-      </c>
-      <c r="J6" s="5" t="n">
         <v>745</v>
       </c>
+      <c r="J6" s="79" t="n">
+        <v>0</v>
+      </c>
       <c r="K6" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="79" t="n">
         <v>120</v>
       </c>
+      <c r="L6" s="5" t="n">
+        <v>825</v>
+      </c>
       <c r="M6" s="5" t="n">
-        <v>825</v>
-      </c>
-      <c r="N6" s="5" t="n">
         <v>1125</v>
       </c>
-      <c r="O6" s="79">
-        <f>(J6+L6+N6)-(I6+K6+M6)</f>
-        <v/>
-      </c>
-      <c r="P6" s="80">
-        <f>IF(J6+L6+N6&gt;0,(J6+L6+N6-I6-K6-M6)/(J6+L6+N6),0)</f>
+      <c r="N6" s="79" t="n">
+        <v>375</v>
+      </c>
+      <c r="O6" s="79" t="n">
+        <v>525</v>
+      </c>
+      <c r="P6" s="79" t="n">
+        <v>810</v>
+      </c>
+      <c r="Q6" s="79" t="n">
+        <v>1215</v>
+      </c>
+      <c r="R6" s="79" t="n">
+        <v>200</v>
+      </c>
+      <c r="S6" s="79" t="n">
+        <v>300</v>
+      </c>
+      <c r="T6" s="79">
+        <f>(J6+L6+N6+P6+R6+T6)-(I6+K6+M6+O6+Q6+S6)</f>
+        <v/>
+      </c>
+      <c r="U6" s="80">
+        <f>IF(J6+L6+N6+P6+R6+T6&gt;0,((J6+L6+N6+P6+R6+T6)-(I6+K6+M6+O6+Q6+S6))/(J6+L6+N6+P6+R6+T6),0)</f>
         <v/>
       </c>
     </row>
@@ -3171,59 +3254,74 @@
       <c r="A7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>S2</t>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>3N4D</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>3N4D</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
           <t>트럼프 + 히든밸리 밸리뷰</t>
         </is>
       </c>
+      <c r="D7" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="E7" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="G7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Trump×1 + HV×1</t>
         </is>
       </c>
+      <c r="H7" s="149" t="inlineStr">
+        <is>
+          <t>G2·H3·T3·M3B3L3D2Ex·I4</t>
+        </is>
+      </c>
       <c r="I7" s="5" t="n">
-        <v>319</v>
-      </c>
-      <c r="J7" s="5" t="n">
         <v>609</v>
+      </c>
+      <c r="J7" s="79" t="n">
+        <v>45</v>
       </c>
       <c r="K7" s="79" t="n">
         <v>45</v>
       </c>
-      <c r="L7" s="79" t="n">
-        <v>45</v>
+      <c r="L7" s="5" t="n">
+        <v>825</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>825</v>
-      </c>
-      <c r="N7" s="5" t="n">
         <v>1125</v>
       </c>
-      <c r="O7" s="79">
-        <f>(J7+L7+N7)-(I7+K7+M7)</f>
-        <v/>
-      </c>
-      <c r="P7" s="80">
-        <f>IF(J7+L7+N7&gt;0,(J7+L7+N7-I7-K7-M7)/(J7+L7+N7),0)</f>
+      <c r="N7" s="79" t="n">
+        <v>375</v>
+      </c>
+      <c r="O7" s="79" t="n">
+        <v>525</v>
+      </c>
+      <c r="P7" s="79" t="n">
+        <v>810</v>
+      </c>
+      <c r="Q7" s="79" t="n">
+        <v>1215</v>
+      </c>
+      <c r="R7" s="79" t="n">
+        <v>200</v>
+      </c>
+      <c r="S7" s="79" t="n">
+        <v>300</v>
+      </c>
+      <c r="T7" s="79">
+        <f>(J7+L7+N7+P7+R7+T7)-(I7+K7+M7+O7+Q7+S7)</f>
+        <v/>
+      </c>
+      <c r="U7" s="80">
+        <f>IF(J7+L7+N7+P7+R7+T7&gt;0,((J7+L7+N7+P7+R7+T7)-(I7+K7+M7+O7+Q7+S7))/(J7+L7+N7+P7+R7+T7),0)</f>
         <v/>
       </c>
     </row>
@@ -3231,59 +3329,74 @@
       <c r="A8" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>S3</t>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>3N4D</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>3N4D</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
           <t>샌드파이퍼 + 히든밸리</t>
         </is>
       </c>
+      <c r="D8" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="E8" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="G8" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Sand×1 + HV×1</t>
         </is>
       </c>
+      <c r="H8" s="149" t="inlineStr">
+        <is>
+          <t>G2·H3·T3·M3B3L3D2Ex·I4</t>
+        </is>
+      </c>
       <c r="I8" s="5" t="n">
-        <v>239</v>
-      </c>
-      <c r="J8" s="5" t="n">
         <v>354</v>
+      </c>
+      <c r="J8" s="79" t="n">
+        <v>45</v>
       </c>
       <c r="K8" s="79" t="n">
         <v>45</v>
       </c>
-      <c r="L8" s="79" t="n">
-        <v>45</v>
+      <c r="L8" s="5" t="n">
+        <v>825</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>825</v>
-      </c>
-      <c r="N8" s="5" t="n">
         <v>1125</v>
       </c>
-      <c r="O8" s="79">
-        <f>(J8+L8+N8)-(I8+K8+M8)</f>
-        <v/>
-      </c>
-      <c r="P8" s="80">
-        <f>IF(J8+L8+N8&gt;0,(J8+L8+N8-I8-K8-M8)/(J8+L8+N8),0)</f>
+      <c r="N8" s="79" t="n">
+        <v>375</v>
+      </c>
+      <c r="O8" s="79" t="n">
+        <v>525</v>
+      </c>
+      <c r="P8" s="79" t="n">
+        <v>810</v>
+      </c>
+      <c r="Q8" s="79" t="n">
+        <v>1215</v>
+      </c>
+      <c r="R8" s="79" t="n">
+        <v>200</v>
+      </c>
+      <c r="S8" s="79" t="n">
+        <v>300</v>
+      </c>
+      <c r="T8" s="79">
+        <f>(J8+L8+N8+P8+R8+T8)-(I8+K8+M8+O8+Q8+S8)</f>
+        <v/>
+      </c>
+      <c r="U8" s="80">
+        <f>IF(J8+L8+N8+P8+R8+T8&gt;0,((J8+L8+N8+P8+R8+T8)-(I8+K8+M8+O8+Q8+S8))/(J8+L8+N8+P8+R8+T8),0)</f>
         <v/>
       </c>
     </row>
@@ -3297,78 +3410,98 @@
       <c r="G9" s="10" t="n"/>
       <c r="H9" s="10" t="n"/>
       <c r="I9" s="10" t="n"/>
-      <c r="J9" s="10" t="n"/>
+      <c r="L9" s="10" t="n"/>
       <c r="M9" s="10" t="n"/>
-      <c r="N9" s="10" t="n"/>
-      <c r="O9" s="10" t="n"/>
-      <c r="P9" s="10" t="n"/>
+      <c r="T9" s="10" t="n"/>
+      <c r="U9" s="10" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>M1</t>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>5N7D</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>5N7D</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
           <t>트럼프+샌드+히든 3色 시그니처</t>
         </is>
       </c>
+      <c r="D10" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="E10" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="G10" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Trump×1+Sand×1+HV×1</t>
         </is>
       </c>
+      <c r="H10" s="149" t="inlineStr">
+        <is>
+          <t>G3·H5·T5·M5B5L5D2Ex·I5</t>
+        </is>
+      </c>
       <c r="I10" s="5" t="n">
-        <v>449</v>
-      </c>
-      <c r="J10" s="5" t="n">
         <v>854</v>
       </c>
+      <c r="J10" s="79" t="n">
+        <v>45</v>
+      </c>
       <c r="K10" s="79" t="n">
-        <v>45</v>
-      </c>
-      <c r="L10" s="79" t="n">
         <v>165</v>
       </c>
+      <c r="L10" s="5" t="n">
+        <v>1375</v>
+      </c>
       <c r="M10" s="5" t="n">
-        <v>1375</v>
-      </c>
-      <c r="N10" s="5" t="n">
         <v>1875</v>
       </c>
-      <c r="O10" s="79">
-        <f>(J10+L10+N10)-(I10+K10+M10)</f>
-        <v/>
-      </c>
-      <c r="P10" s="80">
-        <f>IF(J10+L10+N10&gt;0,(J10+L10+N10-I10-K10-M10)/(J10+L10+N10),0)</f>
+      <c r="N10" s="79" t="n">
+        <v>625</v>
+      </c>
+      <c r="O10" s="79" t="n">
+        <v>875</v>
+      </c>
+      <c r="P10" s="79" t="n">
+        <v>1350</v>
+      </c>
+      <c r="Q10" s="79" t="n">
+        <v>2025</v>
+      </c>
+      <c r="R10" s="79" t="n">
+        <v>250</v>
+      </c>
+      <c r="S10" s="79" t="n">
+        <v>375</v>
+      </c>
+      <c r="T10" s="79">
+        <f>(J10+L10+N10+P10+R10+T10)-(I10+K10+M10+O10+Q10+S10)</f>
+        <v/>
+      </c>
+      <c r="U10" s="80">
+        <f>IF(J10+L10+N10+P10+R10+T10&gt;0,((J10+L10+N10+P10+R10+T10)-(I10+K10+M10+O10+Q10+S10))/(J10+L10+N10+P10+R10+T10),0)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="10">
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="L4:M4"/>
+    <mergeCell ref="H4:I4"/>
     <mergeCell ref="K4:L4"/>
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A1:U1"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="R4:S4"/>
+    <mergeCell ref="N4:O4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3407,16 +3540,16 @@
           <t>🎯 PACKAGE SELECTOR</t>
         </is>
       </c>
-      <c r="B1" s="104" t="n"/>
-      <c r="C1" s="104" t="n"/>
-      <c r="D1" s="104" t="n"/>
-      <c r="E1" s="104" t="n"/>
-      <c r="F1" s="104" t="n"/>
-      <c r="G1" s="104" t="n"/>
-      <c r="H1" s="104" t="n"/>
-      <c r="I1" s="104" t="n"/>
-      <c r="J1" s="104" t="n"/>
-      <c r="K1" s="104" t="n"/>
+      <c r="B1" s="150" t="n"/>
+      <c r="C1" s="150" t="n"/>
+      <c r="D1" s="150" t="n"/>
+      <c r="E1" s="150" t="n"/>
+      <c r="F1" s="150" t="n"/>
+      <c r="G1" s="150" t="n"/>
+      <c r="H1" s="150" t="n"/>
+      <c r="I1" s="150" t="n"/>
+      <c r="J1" s="150" t="n"/>
+      <c r="K1" s="92" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="106" t="inlineStr">
@@ -3425,6 +3558,7 @@
         </is>
       </c>
       <c r="B2" s="129" t="inlineStr"/>
+      <c r="C2" s="87" t="n"/>
       <c r="D2" s="106" t="inlineStr">
         <is>
           <t>Golfers:</t>
@@ -3460,16 +3594,16 @@
           <t>✈️ OUTBOUND</t>
         </is>
       </c>
-      <c r="B3" s="77" t="n"/>
-      <c r="C3" s="77" t="n"/>
-      <c r="D3" s="77" t="n"/>
-      <c r="E3" s="77" t="n"/>
-      <c r="F3" s="77" t="n"/>
-      <c r="G3" s="77" t="n"/>
-      <c r="H3" s="77" t="n"/>
-      <c r="I3" s="77" t="n"/>
-      <c r="J3" s="77" t="n"/>
-      <c r="K3" s="77" t="n"/>
+      <c r="B3" s="150" t="n"/>
+      <c r="C3" s="150" t="n"/>
+      <c r="D3" s="150" t="n"/>
+      <c r="E3" s="150" t="n"/>
+      <c r="F3" s="150" t="n"/>
+      <c r="G3" s="150" t="n"/>
+      <c r="H3" s="150" t="n"/>
+      <c r="I3" s="150" t="n"/>
+      <c r="J3" s="150" t="n"/>
+      <c r="K3" s="92" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="106" t="inlineStr">
@@ -3516,16 +3650,16 @@
           <t>✈️ RETURN</t>
         </is>
       </c>
-      <c r="B5" s="77" t="n"/>
-      <c r="C5" s="77" t="n"/>
-      <c r="D5" s="77" t="n"/>
-      <c r="E5" s="77" t="n"/>
-      <c r="F5" s="77" t="n"/>
-      <c r="G5" s="77" t="n"/>
-      <c r="H5" s="77" t="n"/>
-      <c r="I5" s="77" t="n"/>
-      <c r="J5" s="77" t="n"/>
-      <c r="K5" s="77" t="n"/>
+      <c r="B5" s="150" t="n"/>
+      <c r="C5" s="150" t="n"/>
+      <c r="D5" s="150" t="n"/>
+      <c r="E5" s="150" t="n"/>
+      <c r="F5" s="150" t="n"/>
+      <c r="G5" s="150" t="n"/>
+      <c r="H5" s="150" t="n"/>
+      <c r="I5" s="150" t="n"/>
+      <c r="J5" s="150" t="n"/>
+      <c r="K5" s="92" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="106" t="inlineStr">
@@ -3561,7 +3695,7 @@
         </is>
       </c>
       <c r="J6" s="144">
-        <f>IF(AND(B4&lt;&gt;"",B6&lt;&gt;""),B6-B4,"")&amp;"N "&amp;IF(B10&lt;&gt;"",B10+1,"")&amp;"D"</f>
+        <f>IF(AND(B4&lt;&gt;"",B6&lt;&gt;""),B6-B4,"")&amp;"N "&amp;IF(AND(B4&lt;&gt;"",B6&lt;&gt;""),B6-B4+1,"")&amp;"D"</f>
         <v/>
       </c>
       <c r="K6" s="87" t="n"/>
@@ -3688,16 +3822,16 @@
           <t>⛳ GOLF</t>
         </is>
       </c>
-      <c r="B9" s="77" t="n"/>
-      <c r="C9" s="77" t="n"/>
-      <c r="D9" s="77" t="n"/>
-      <c r="E9" s="77" t="n"/>
-      <c r="F9" s="77" t="n"/>
-      <c r="G9" s="77" t="n"/>
-      <c r="H9" s="77" t="n"/>
-      <c r="I9" s="77" t="n"/>
-      <c r="J9" s="77" t="n"/>
-      <c r="K9" s="77" t="n"/>
+      <c r="B9" s="150" t="n"/>
+      <c r="C9" s="150" t="n"/>
+      <c r="D9" s="150" t="n"/>
+      <c r="E9" s="150" t="n"/>
+      <c r="F9" s="150" t="n"/>
+      <c r="G9" s="150" t="n"/>
+      <c r="H9" s="150" t="n"/>
+      <c r="I9" s="150" t="n"/>
+      <c r="J9" s="150" t="n"/>
+      <c r="K9" s="92" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="109" t="inlineStr">
@@ -3954,16 +4088,16 @@
           <t>🏨 HOTEL</t>
         </is>
       </c>
-      <c r="B17" s="77" t="n"/>
-      <c r="C17" s="77" t="n"/>
-      <c r="D17" s="77" t="n"/>
-      <c r="E17" s="77" t="n"/>
-      <c r="F17" s="77" t="n"/>
-      <c r="G17" s="77" t="n"/>
-      <c r="H17" s="77" t="n"/>
-      <c r="I17" s="77" t="n"/>
-      <c r="J17" s="77" t="n"/>
-      <c r="K17" s="77" t="n"/>
+      <c r="B17" s="150" t="n"/>
+      <c r="C17" s="150" t="n"/>
+      <c r="D17" s="150" t="n"/>
+      <c r="E17" s="150" t="n"/>
+      <c r="F17" s="150" t="n"/>
+      <c r="G17" s="150" t="n"/>
+      <c r="H17" s="150" t="n"/>
+      <c r="I17" s="150" t="n"/>
+      <c r="J17" s="150" t="n"/>
+      <c r="K17" s="92" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="109" t="inlineStr">
@@ -4136,16 +4270,16 @@
           <t>🚐 TRANSPORT</t>
         </is>
       </c>
-      <c r="B23" s="77" t="n"/>
-      <c r="C23" s="77" t="n"/>
-      <c r="D23" s="77" t="n"/>
-      <c r="E23" s="77" t="n"/>
-      <c r="F23" s="77" t="n"/>
-      <c r="G23" s="77" t="n"/>
-      <c r="H23" s="77" t="n"/>
-      <c r="I23" s="77" t="n"/>
-      <c r="J23" s="77" t="n"/>
-      <c r="K23" s="77" t="n"/>
+      <c r="B23" s="150" t="n"/>
+      <c r="C23" s="150" t="n"/>
+      <c r="D23" s="150" t="n"/>
+      <c r="E23" s="150" t="n"/>
+      <c r="F23" s="150" t="n"/>
+      <c r="G23" s="150" t="n"/>
+      <c r="H23" s="150" t="n"/>
+      <c r="I23" s="150" t="n"/>
+      <c r="J23" s="150" t="n"/>
+      <c r="K23" s="92" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="109" t="inlineStr">
@@ -4318,16 +4452,16 @@
           <t>🍽️ MEALS</t>
         </is>
       </c>
-      <c r="B29" s="77" t="n"/>
-      <c r="C29" s="77" t="n"/>
-      <c r="D29" s="77" t="n"/>
-      <c r="E29" s="77" t="n"/>
-      <c r="F29" s="77" t="n"/>
-      <c r="G29" s="77" t="n"/>
-      <c r="H29" s="77" t="n"/>
-      <c r="I29" s="77" t="n"/>
-      <c r="J29" s="77" t="n"/>
-      <c r="K29" s="77" t="n"/>
+      <c r="B29" s="150" t="n"/>
+      <c r="C29" s="150" t="n"/>
+      <c r="D29" s="150" t="n"/>
+      <c r="E29" s="150" t="n"/>
+      <c r="F29" s="150" t="n"/>
+      <c r="G29" s="150" t="n"/>
+      <c r="H29" s="150" t="n"/>
+      <c r="I29" s="150" t="n"/>
+      <c r="J29" s="150" t="n"/>
+      <c r="K29" s="92" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="109" t="inlineStr">
@@ -4590,16 +4724,16 @@
           <t>📦 OTHER</t>
         </is>
       </c>
-      <c r="B37" s="77" t="n"/>
-      <c r="C37" s="77" t="n"/>
-      <c r="D37" s="77" t="n"/>
-      <c r="E37" s="77" t="n"/>
-      <c r="F37" s="77" t="n"/>
-      <c r="G37" s="77" t="n"/>
-      <c r="H37" s="77" t="n"/>
-      <c r="I37" s="77" t="n"/>
-      <c r="J37" s="77" t="n"/>
-      <c r="K37" s="77" t="n"/>
+      <c r="B37" s="150" t="n"/>
+      <c r="C37" s="150" t="n"/>
+      <c r="D37" s="150" t="n"/>
+      <c r="E37" s="150" t="n"/>
+      <c r="F37" s="150" t="n"/>
+      <c r="G37" s="150" t="n"/>
+      <c r="H37" s="150" t="n"/>
+      <c r="I37" s="150" t="n"/>
+      <c r="J37" s="150" t="n"/>
+      <c r="K37" s="92" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="109" t="inlineStr">
@@ -4772,16 +4906,16 @@
           <t>🎯 ACTIVITIES</t>
         </is>
       </c>
-      <c r="B43" s="77" t="n"/>
-      <c r="C43" s="77" t="n"/>
-      <c r="D43" s="77" t="n"/>
-      <c r="E43" s="77" t="n"/>
-      <c r="F43" s="77" t="n"/>
-      <c r="G43" s="77" t="n"/>
-      <c r="H43" s="77" t="n"/>
-      <c r="I43" s="77" t="n"/>
-      <c r="J43" s="77" t="n"/>
-      <c r="K43" s="77" t="n"/>
+      <c r="B43" s="150" t="n"/>
+      <c r="C43" s="150" t="n"/>
+      <c r="D43" s="150" t="n"/>
+      <c r="E43" s="150" t="n"/>
+      <c r="F43" s="150" t="n"/>
+      <c r="G43" s="150" t="n"/>
+      <c r="H43" s="150" t="n"/>
+      <c r="I43" s="150" t="n"/>
+      <c r="J43" s="150" t="n"/>
+      <c r="K43" s="92" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="109" t="inlineStr">
@@ -5188,16 +5322,16 @@
           <t>🏆 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B56" s="104" t="n"/>
-      <c r="C56" s="104" t="n"/>
-      <c r="D56" s="104" t="n"/>
-      <c r="E56" s="104" t="n"/>
-      <c r="F56" s="104" t="n"/>
-      <c r="G56" s="104" t="n"/>
-      <c r="H56" s="104" t="n"/>
-      <c r="I56" s="104" t="n"/>
-      <c r="J56" s="104" t="n"/>
-      <c r="K56" s="104" t="n"/>
+      <c r="B56" s="150" t="n"/>
+      <c r="C56" s="150" t="n"/>
+      <c r="D56" s="150" t="n"/>
+      <c r="E56" s="150" t="n"/>
+      <c r="F56" s="150" t="n"/>
+      <c r="G56" s="150" t="n"/>
+      <c r="H56" s="150" t="n"/>
+      <c r="I56" s="150" t="n"/>
+      <c r="J56" s="150" t="n"/>
+      <c r="K56" s="92" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="108" t="inlineStr">
@@ -5319,16 +5453,16 @@
           <t>👤 PER PERSON</t>
         </is>
       </c>
-      <c r="B65" s="104" t="n"/>
-      <c r="C65" s="104" t="n"/>
-      <c r="D65" s="104" t="n"/>
-      <c r="E65" s="104" t="n"/>
-      <c r="F65" s="104" t="n"/>
-      <c r="G65" s="104" t="n"/>
-      <c r="H65" s="104" t="n"/>
-      <c r="I65" s="104" t="n"/>
-      <c r="J65" s="104" t="n"/>
-      <c r="K65" s="104" t="n"/>
+      <c r="B65" s="150" t="n"/>
+      <c r="C65" s="150" t="n"/>
+      <c r="D65" s="150" t="n"/>
+      <c r="E65" s="150" t="n"/>
+      <c r="F65" s="150" t="n"/>
+      <c r="G65" s="150" t="n"/>
+      <c r="H65" s="150" t="n"/>
+      <c r="I65" s="150" t="n"/>
+      <c r="J65" s="150" t="n"/>
+      <c r="K65" s="92" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="98" t="inlineStr">
@@ -5489,7 +5623,6 @@
   <mergeCells count="15">
     <mergeCell ref="A56:K56"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="A37:K37"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A23:K23"/>
     <mergeCell ref="J6:K6"/>
@@ -5498,9 +5631,10 @@
     <mergeCell ref="A43:K43"/>
     <mergeCell ref="E6:H6"/>
     <mergeCell ref="A65:K65"/>
+    <mergeCell ref="A17:K17"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A37:K37"/>
     <mergeCell ref="A9:K9"/>
   </mergeCells>
   <conditionalFormatting sqref="F10">
@@ -6267,14 +6401,14 @@
     <row r="1">
       <c r="A1" s="103" t="inlineStr">
         <is>
-          <t>📊 PROFIT SUMMARY</t>
-        </is>
-      </c>
-      <c r="B1" s="104" t="n"/>
-      <c r="C1" s="104" t="n"/>
-      <c r="D1" s="104" t="n"/>
-      <c r="E1" s="104" t="n"/>
-      <c r="F1" s="104" t="n"/>
+          <t>📊 PACKAGE SUMMARY — Current Selection</t>
+        </is>
+      </c>
+      <c r="B1" s="150" t="n"/>
+      <c r="C1" s="150" t="n"/>
+      <c r="D1" s="150" t="n"/>
+      <c r="E1" s="150" t="n"/>
+      <c r="F1" s="92" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="98" t="inlineStr">
@@ -6503,4 +6637,231 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" style="42" min="1" max="1"/>
+    <col width="18" customWidth="1" style="42" min="2" max="2"/>
+    <col width="18" customWidth="1" style="42" min="3" max="3"/>
+    <col width="18" customWidth="1" style="42" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="103" t="inlineStr">
+        <is>
+          <t>🎫 GUEST PACKAGE — Client Summary</t>
+        </is>
+      </c>
+      <c r="B1" s="104" t="n"/>
+      <c r="C1" s="104" t="n"/>
+      <c r="D1" s="104" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="106" t="inlineStr">
+        <is>
+          <t>Package:</t>
+        </is>
+      </c>
+      <c r="B3" s="151">
+        <f>'Package Selector'!B2</f>
+        <v/>
+      </c>
+      <c r="C3" s="86" t="n"/>
+      <c r="D3" s="87" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="106" t="inlineStr">
+        <is>
+          <t>Guests:</t>
+        </is>
+      </c>
+      <c r="B4" s="152">
+        <f>'Package Selector'!E2</f>
+        <v/>
+      </c>
+      <c r="C4" s="108" t="inlineStr">
+        <is>
+          <t>persons</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="106" t="inlineStr">
+        <is>
+          <t>Duration:</t>
+        </is>
+      </c>
+      <c r="B5" s="151">
+        <f>'Package Selector'!J6</f>
+        <v/>
+      </c>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="87" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="124" t="inlineStr">
+        <is>
+          <t>📋 PACKAGE INCLUDES</t>
+        </is>
+      </c>
+      <c r="B7" s="125" t="n"/>
+      <c r="C7" s="125" t="n"/>
+      <c r="D7" s="125" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="140" t="inlineStr">
+        <is>
+          <t>⛳ Golf</t>
+        </is>
+      </c>
+      <c r="B8" s="108">
+        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F9:I14,"●")&gt;0),A9:A14,""))</f>
+        <v/>
+      </c>
+      <c r="C8" s="86" t="n"/>
+      <c r="D8" s="87" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="140" t="inlineStr">
+        <is>
+          <t>🏨 Hotel</t>
+        </is>
+      </c>
+      <c r="B9" s="108">
+        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F17:I21,"●")&gt;0),A17:A21,""))</f>
+        <v/>
+      </c>
+      <c r="C9" s="86" t="n"/>
+      <c r="D9" s="87" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="140" t="inlineStr">
+        <is>
+          <t>🚐 Transport</t>
+        </is>
+      </c>
+      <c r="B10" s="108">
+        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F23:I27,"●")&gt;0),A23:A27,""))</f>
+        <v/>
+      </c>
+      <c r="C10" s="86" t="n"/>
+      <c r="D10" s="87" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="140" t="inlineStr">
+        <is>
+          <t>🍽️ Meals</t>
+        </is>
+      </c>
+      <c r="B11" s="108">
+        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F29:I35,"●")&gt;0),A29:A35,""))</f>
+        <v/>
+      </c>
+      <c r="C11" s="86" t="n"/>
+      <c r="D11" s="87" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="140" t="inlineStr">
+        <is>
+          <t>📦 Other</t>
+        </is>
+      </c>
+      <c r="B12" s="108">
+        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F37:I41,"●")&gt;0),A37:A41,""))</f>
+        <v/>
+      </c>
+      <c r="C12" s="86" t="n"/>
+      <c r="D12" s="87" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="140" t="inlineStr">
+        <is>
+          <t>🎯 Activities</t>
+        </is>
+      </c>
+      <c r="B13" s="108">
+        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F43:I53,"●")&gt;0),A43:A53,""))</f>
+        <v/>
+      </c>
+      <c r="C13" s="86" t="n"/>
+      <c r="D13" s="87" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="104" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="124" t="inlineStr">
+        <is>
+          <t>💰 ALL-INCLUSIVE PRICE</t>
+        </is>
+      </c>
+      <c r="B16" s="125" t="n"/>
+      <c r="C16" s="125" t="n"/>
+      <c r="D16" s="125" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="106" t="inlineStr">
+        <is>
+          <t>Total Package Price:</t>
+        </is>
+      </c>
+      <c r="B17" s="153">
+        <f>'Package Selector'!K63</f>
+        <v/>
+      </c>
+      <c r="C17" s="86" t="n"/>
+      <c r="D17" s="87" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="106" t="inlineStr">
+        <is>
+          <t>Per Person:</t>
+        </is>
+      </c>
+      <c r="B18" s="154">
+        <f>IF(B4&gt;0,B11/B4,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="106" t="inlineStr">
+        <is>
+          <t>Margin:</t>
+        </is>
+      </c>
+      <c r="B19" s="155">
+        <f>B11-B14</f>
+        <v/>
+      </c>
+      <c r="C19" s="156">
+        <f>IF(B11&gt;0,B13/B11,0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="B12:D12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: per-group charging, meals reorder, Margin%, remove#, charge type logic
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -1452,20 +1452,25 @@
       </c>
       <c r="D6" s="146" t="inlineStr">
         <is>
-          <t>Margin ($)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Replay Rate ($)</t>
+          <t>Margin $</t>
+        </is>
+      </c>
+      <c r="E6" s="146" t="inlineStr">
+        <is>
+          <t>Margin %</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Margin %</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
+      <c r="H6" s="146" t="inlineStr">
+        <is>
+          <t>Charge</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="70" t="inlineStr">
@@ -1483,12 +1488,21 @@
         <f>IF(A7="","",C7-B7)</f>
         <v/>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="137">
+        <f>IF(A7="","",IF(C7&gt;0,(C7-B7)/C7,0))</f>
+        <v/>
+      </c>
+      <c r="F7" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>teeitup.com | 9Stamps=1free | Replay twilight</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Per Person</t>
         </is>
       </c>
     </row>
@@ -1508,12 +1522,21 @@
         <f>IF(A8="","",C8-B8)</f>
         <v/>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="137">
+        <f>IF(A8="","",IF(C8&gt;0,(C8-B8)/C8,0))</f>
+        <v/>
+      </c>
+      <c r="F8" s="6" t="n">
         <v>120</v>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>UnderPar deal | Replay FREE | Non-Resident</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Per Person</t>
         </is>
       </c>
     </row>
@@ -1533,12 +1556,21 @@
         <f>IF(A9="","",C9-B9)</f>
         <v/>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="137">
+        <f>IF(A9="","",IF(C9&gt;0,(C9-B9)/C9,0))</f>
+        <v/>
+      </c>
+      <c r="F9" s="6" t="n">
         <v>111</v>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Member guest | Cart incl. | Replay ~50%</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Per Person</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1582,10 @@
         <f>IF(A10="","",C10-B10)</f>
         <v/>
       </c>
-      <c r="E10" s="4" t="n"/>
+      <c r="E10" s="137">
+        <f>IF(A10="","",IF(C10&gt;0,(C10-B10)/C10,0))</f>
+        <v/>
+      </c>
       <c r="F10" s="6" t="n"/>
     </row>
     <row r="11">
@@ -1561,7 +1596,10 @@
         <f>IF(A11="","",C11-B11)</f>
         <v/>
       </c>
-      <c r="E11" s="4" t="n"/>
+      <c r="E11" s="137">
+        <f>IF(A11="","",IF(C11&gt;0,(C11-B11)/C11,0))</f>
+        <v/>
+      </c>
       <c r="F11" s="6" t="n"/>
     </row>
     <row r="12">
@@ -1572,7 +1610,10 @@
         <f>IF(A12="","",C12-B12)</f>
         <v/>
       </c>
-      <c r="E12" s="4" t="n"/>
+      <c r="E12" s="137">
+        <f>IF(A12="","",IF(C12&gt;0,(C12-B12)/C12,0))</f>
+        <v/>
+      </c>
       <c r="F12" s="6" t="n"/>
     </row>
     <row r="13">
@@ -1583,7 +1624,10 @@
         <f>IF(A13="","",C13-B13)</f>
         <v/>
       </c>
-      <c r="E13" s="4" t="n"/>
+      <c r="E13" s="137">
+        <f>IF(A13="","",IF(C13&gt;0,(C13-B13)/C13,0))</f>
+        <v/>
+      </c>
       <c r="F13" s="6" t="n"/>
     </row>
     <row r="14">
@@ -1594,7 +1638,10 @@
         <f>IF(A14="","",C14-B14)</f>
         <v/>
       </c>
-      <c r="E14" s="4" t="n"/>
+      <c r="E14" s="137">
+        <f>IF(A14="","",IF(C14&gt;0,(C14-B14)/C14,0))</f>
+        <v/>
+      </c>
       <c r="F14" s="6" t="n"/>
     </row>
     <row r="17">
@@ -1628,13 +1675,17 @@
       </c>
       <c r="D18" s="146" t="inlineStr">
         <is>
-          <t>Margin ($)</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n"/>
+          <t>Margin $</t>
+        </is>
+      </c>
+      <c r="E18" s="146" t="inlineStr">
+        <is>
+          <t>Margin %</t>
+        </is>
+      </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Margin %</t>
         </is>
       </c>
       <c r="G18" s="2" t="n"/>
@@ -1655,7 +1706,12 @@
         <f>IF(A19="","",C19-B19)</f>
         <v/>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="E19" s="137">
+        <f>IF(A19="","",IF(C19&gt;0,(C19-B19)/C19,0))</f>
+        <v/>
+      </c>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" t="inlineStr">
         <is>
           <t>$550/room ÷ 2 persons</t>
         </is>
@@ -1669,6 +1725,10 @@
         <f>IF(A20="","",C20-B20)</f>
         <v/>
       </c>
+      <c r="E20" s="137">
+        <f>IF(A20="","",IF(C20&gt;0,(C20-B20)/C20,0))</f>
+        <v/>
+      </c>
       <c r="F20" s="6" t="n"/>
     </row>
     <row r="21">
@@ -1679,6 +1739,10 @@
         <f>IF(A21="","",C21-B21)</f>
         <v/>
       </c>
+      <c r="E21" s="137">
+        <f>IF(A21="","",IF(C21&gt;0,(C21-B21)/C21,0))</f>
+        <v/>
+      </c>
       <c r="F21" s="6" t="n"/>
     </row>
     <row r="22">
@@ -1689,6 +1753,10 @@
         <f>IF(A22="","",C22-B22)</f>
         <v/>
       </c>
+      <c r="E22" s="137">
+        <f>IF(A22="","",IF(C22&gt;0,(C22-B22)/C22,0))</f>
+        <v/>
+      </c>
       <c r="F22" s="6" t="n"/>
     </row>
     <row r="23">
@@ -1699,6 +1767,10 @@
         <f>IF(A23="","",C23-B23)</f>
         <v/>
       </c>
+      <c r="E23" s="137">
+        <f>IF(A23="","",IF(C23&gt;0,(C23-B23)/C23,0))</f>
+        <v/>
+      </c>
       <c r="F23" s="6" t="n"/>
     </row>
     <row r="24">
@@ -1709,7 +1781,17 @@
         <f>IF(A24="","",C24-B24)</f>
         <v/>
       </c>
+      <c r="E24" s="137">
+        <f>IF(A24="","",IF(C24&gt;0,(C24-B24)/C24,0))</f>
+        <v/>
+      </c>
       <c r="F24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="E25" s="137">
+        <f>IF(A25="","",IF(C25&gt;0,(C25-B25)/C25,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="31" t="inlineStr">
@@ -1742,16 +1824,25 @@
       </c>
       <c r="D27" s="146" t="inlineStr">
         <is>
-          <t>Margin ($)</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n"/>
+          <t>Margin $</t>
+        </is>
+      </c>
+      <c r="E27" s="146" t="inlineStr">
+        <is>
+          <t>Margin %</t>
+        </is>
+      </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Margin %</t>
         </is>
       </c>
       <c r="G27" s="2" t="n"/>
+      <c r="H27" s="146" t="inlineStr">
+        <is>
+          <t>Charge</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="16.5" customHeight="1" s="42">
       <c r="A28" s="70" t="inlineStr">
@@ -1769,9 +1860,19 @@
         <f>IF(A28="","",C28-B28)</f>
         <v/>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="E28" s="137">
+        <f>IF(A28="","",IF(C28&gt;0,(C28-B28)/C28,0))</f>
+        <v/>
+      </c>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" t="inlineStr">
         <is>
           <t>$500/day ÷ 4p | Driver=Guide</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Per Group</t>
         </is>
       </c>
     </row>
@@ -1791,9 +1892,19 @@
         <f>IF(A29="","",C29-B29)</f>
         <v/>
       </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="E29" s="137">
+        <f>IF(A29="","",IF(C29&gt;0,(C29-B29)/C29,0))</f>
+        <v/>
+      </c>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" t="inlineStr">
         <is>
           <t>LAX ↔ Hotel, per person</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Per Person</t>
         </is>
       </c>
     </row>
@@ -1805,6 +1916,10 @@
         <f>IF(A30="","",C30-B30)</f>
         <v/>
       </c>
+      <c r="E30" s="137">
+        <f>IF(A30="","",IF(C30&gt;0,(C30-B30)/C30,0))</f>
+        <v/>
+      </c>
       <c r="F30" s="6" t="n"/>
     </row>
     <row r="31">
@@ -1815,6 +1930,10 @@
         <f>IF(A31="","",C31-B31)</f>
         <v/>
       </c>
+      <c r="E31" s="137">
+        <f>IF(A31="","",IF(C31&gt;0,(C31-B31)/C31,0))</f>
+        <v/>
+      </c>
       <c r="F31" s="6" t="n"/>
     </row>
     <row r="32">
@@ -1825,6 +1944,10 @@
         <f>IF(A32="","",C32-B32)</f>
         <v/>
       </c>
+      <c r="E32" s="137">
+        <f>IF(A32="","",IF(C32&gt;0,(C32-B32)/C32,0))</f>
+        <v/>
+      </c>
       <c r="F32" s="6" t="n"/>
     </row>
     <row r="33">
@@ -1835,6 +1958,10 @@
         <f>IF(A33="","",C33-B33)</f>
         <v/>
       </c>
+      <c r="E33" s="137">
+        <f>IF(A33="","",IF(C33&gt;0,(C33-B33)/C33,0))</f>
+        <v/>
+      </c>
       <c r="F33" s="6" t="n"/>
     </row>
     <row r="34">
@@ -1845,7 +1972,17 @@
         <f>IF(A34="","",C34-B34)</f>
         <v/>
       </c>
+      <c r="E34" s="137">
+        <f>IF(A34="","",IF(C34&gt;0,(C34-B34)/C34,0))</f>
+        <v/>
+      </c>
       <c r="F34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="E35" s="137">
+        <f>IF(A35="","",IF(C35&gt;0,(C35-B35)/C35,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="31" t="inlineStr">
@@ -1878,13 +2015,17 @@
       </c>
       <c r="D37" s="146" t="inlineStr">
         <is>
-          <t>Margin ($)</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="n"/>
+          <t>Margin $</t>
+        </is>
+      </c>
+      <c r="E37" s="146" t="inlineStr">
+        <is>
+          <t>Margin %</t>
+        </is>
+      </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Margin %</t>
         </is>
       </c>
       <c r="G37" s="2" t="n"/>
@@ -1905,7 +2046,12 @@
         <f>IF(A38="","",C38-B38)</f>
         <v/>
       </c>
-      <c r="F38" s="6" t="inlineStr">
+      <c r="E38" s="137">
+        <f>IF(A38="","",IF(C38&gt;0,(C38-B38)/C38,0))</f>
+        <v/>
+      </c>
+      <c r="F38" s="6" t="n"/>
+      <c r="G38" t="inlineStr">
         <is>
           <t>Daily included</t>
         </is>
@@ -1927,7 +2073,12 @@
         <f>IF(A39="","",C39-B39)</f>
         <v/>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="E39" s="137">
+        <f>IF(A39="","",IF(C39&gt;0,(C39-B39)/C39,0))</f>
+        <v/>
+      </c>
+      <c r="F39" s="6" t="n"/>
+      <c r="G39" t="inlineStr">
         <is>
           <t>Daily included</t>
         </is>
@@ -1949,7 +2100,12 @@
         <f>IF(A40="","",C40-B40)</f>
         <v/>
       </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="E40" s="137">
+        <f>IF(A40="","",IF(C40&gt;0,(C40-B40)/C40,0))</f>
+        <v/>
+      </c>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" t="inlineStr">
         <is>
           <t>Regular dinner</t>
         </is>
@@ -1971,7 +2127,12 @@
         <f>IF(A41="","",C41-B41)</f>
         <v/>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="E41" s="137">
+        <f>IF(A41="","",IF(C41&gt;0,(C41-B41)/C41,0))</f>
+        <v/>
+      </c>
+      <c r="F41" s="6" t="n"/>
+      <c r="G41" t="inlineStr">
         <is>
           <t>2x per trip</t>
         </is>
@@ -1985,6 +2146,10 @@
         <f>IF(A42="","",C42-B42)</f>
         <v/>
       </c>
+      <c r="E42" s="137">
+        <f>IF(A42="","",IF(C42&gt;0,(C42-B42)/C42,0))</f>
+        <v/>
+      </c>
       <c r="F42" s="6" t="n"/>
     </row>
     <row r="43">
@@ -1995,6 +2160,10 @@
         <f>IF(A43="","",C43-B43)</f>
         <v/>
       </c>
+      <c r="E43" s="137">
+        <f>IF(A43="","",IF(C43&gt;0,(C43-B43)/C43,0))</f>
+        <v/>
+      </c>
       <c r="F43" s="6" t="n"/>
     </row>
     <row r="44">
@@ -2005,6 +2174,10 @@
         <f>IF(A44="","",C44-B44)</f>
         <v/>
       </c>
+      <c r="E44" s="137">
+        <f>IF(A44="","",IF(C44&gt;0,(C44-B44)/C44,0))</f>
+        <v/>
+      </c>
       <c r="F44" s="6" t="n"/>
     </row>
     <row r="45">
@@ -2015,6 +2188,10 @@
         <f>IF(A45="","",C45-B45)</f>
         <v/>
       </c>
+      <c r="E45" s="137">
+        <f>IF(A45="","",IF(C45&gt;0,(C45-B45)/C45,0))</f>
+        <v/>
+      </c>
       <c r="F45" s="6" t="n"/>
     </row>
     <row r="46">
@@ -2058,13 +2235,17 @@
       </c>
       <c r="D49" s="146" t="inlineStr">
         <is>
-          <t>Margin ($)</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="n"/>
+          <t>Margin $</t>
+        </is>
+      </c>
+      <c r="E49" s="146" t="inlineStr">
+        <is>
+          <t>Margin %</t>
+        </is>
+      </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Margin %</t>
         </is>
       </c>
       <c r="G49" s="2" t="n"/>
@@ -2085,7 +2266,12 @@
         <f>IF(A50="","",C50-B50)</f>
         <v/>
       </c>
-      <c r="F50" s="6" t="inlineStr">
+      <c r="E50" s="137">
+        <f>IF(A50="","",IF(C50&gt;0,(C50-B50)/C50,0))</f>
+        <v/>
+      </c>
+      <c r="F50" s="6" t="n"/>
+      <c r="G50" t="inlineStr">
         <is>
           <t>Per person per day</t>
         </is>
@@ -2099,6 +2285,10 @@
         <f>IF(A51="","",C51-B51)</f>
         <v/>
       </c>
+      <c r="E51" s="137">
+        <f>IF(A51="","",IF(C51&gt;0,(C51-B51)/C51,0))</f>
+        <v/>
+      </c>
       <c r="F51" s="6" t="n"/>
     </row>
     <row r="52">
@@ -2109,6 +2299,10 @@
         <f>IF(A52="","",C52-B52)</f>
         <v/>
       </c>
+      <c r="E52" s="137">
+        <f>IF(A52="","",IF(C52&gt;0,(C52-B52)/C52,0))</f>
+        <v/>
+      </c>
       <c r="F52" s="6" t="n"/>
     </row>
     <row r="53">
@@ -2119,6 +2313,10 @@
         <f>IF(A53="","",C53-B53)</f>
         <v/>
       </c>
+      <c r="E53" s="137">
+        <f>IF(A53="","",IF(C53&gt;0,(C53-B53)/C53,0))</f>
+        <v/>
+      </c>
       <c r="F53" s="6" t="n"/>
     </row>
     <row r="54">
@@ -2129,6 +2327,10 @@
         <f>IF(A54="","",C54-B54)</f>
         <v/>
       </c>
+      <c r="E54" s="137">
+        <f>IF(A54="","",IF(C54&gt;0,(C54-B54)/C54,0))</f>
+        <v/>
+      </c>
       <c r="F54" s="6" t="n"/>
     </row>
     <row r="55">
@@ -2139,9 +2341,24 @@
         <f>IF(A55="","",C55-B55)</f>
         <v/>
       </c>
+      <c r="E55" s="137">
+        <f>IF(A55="","",IF(C55&gt;0,(C55-B55)/C55,0))</f>
+        <v/>
+      </c>
       <c r="F55" s="6" t="n"/>
     </row>
-    <row r="56"/>
+    <row r="56">
+      <c r="E56" s="137">
+        <f>IF(A56="","",IF(C56&gt;0,(C56-B56)/C56,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="E57" s="137">
+        <f>IF(A57="","",IF(C57&gt;0,(C57-B57)/C57,0))</f>
+        <v/>
+      </c>
+    </row>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
         <is>
@@ -2743,12 +2960,17 @@
       </c>
       <c r="D85" s="146" t="inlineStr">
         <is>
-          <t>Margin ($)</t>
+          <t>Margin $</t>
+        </is>
+      </c>
+      <c r="E85" s="146" t="inlineStr">
+        <is>
+          <t>Margin %</t>
         </is>
       </c>
       <c r="F85" s="46" t="inlineStr">
         <is>
-          <t>Per Group?</t>
+          <t>Margin %</t>
         </is>
       </c>
       <c r="G85" s="46" t="inlineStr">
@@ -2773,15 +2995,14 @@
         <f>IF(A86="","",C86-B86)</f>
         <v/>
       </c>
-      <c r="E86" s="49" t="n"/>
-      <c r="F86" s="49" t="inlineStr">
+      <c r="E86" s="137">
+        <f>IF(A86="","",IF(C86&gt;0,(C86-B86)/C86,0))</f>
+        <v/>
+      </c>
+      <c r="F86" s="49" t="n"/>
+      <c r="G86" s="49" t="inlineStr">
         <is>
           <t>1p</t>
-        </is>
-      </c>
-      <c r="G86" s="49" t="inlineStr">
-        <is>
-          <t>2hr session; equipment incl.</t>
         </is>
       </c>
     </row>
@@ -2801,15 +3022,14 @@
         <f>IF(A87="","",C87-B87)</f>
         <v/>
       </c>
-      <c r="E87" s="49" t="n"/>
-      <c r="F87" s="49" t="inlineStr">
+      <c r="E87" s="137">
+        <f>IF(A87="","",IF(C87&gt;0,(C87-B87)/C87,0))</f>
+        <v/>
+      </c>
+      <c r="F87" s="49" t="n"/>
+      <c r="G87" s="49" t="inlineStr">
         <is>
           <t>1p</t>
-        </is>
-      </c>
-      <c r="G87" s="49" t="inlineStr">
-        <is>
-          <t>Guided tour included</t>
         </is>
       </c>
     </row>
@@ -2829,15 +3049,14 @@
         <f>IF(A88="","",C88-B88)</f>
         <v/>
       </c>
-      <c r="E88" s="49" t="n"/>
-      <c r="F88" s="49" t="inlineStr">
+      <c r="E88" s="137">
+        <f>IF(A88="","",IF(C88&gt;0,(C88-B88)/C88,0))</f>
+        <v/>
+      </c>
+      <c r="F88" s="49" t="n"/>
+      <c r="G88" s="49" t="inlineStr">
         <is>
           <t>1p</t>
-        </is>
-      </c>
-      <c r="G88" s="49" t="inlineStr">
-        <is>
-          <t>Seasonal; group rates available</t>
         </is>
       </c>
     </row>
@@ -2857,15 +3076,14 @@
         <f>IF(A89="","",C89-B89)</f>
         <v/>
       </c>
-      <c r="E89" s="49" t="n"/>
-      <c r="F89" s="49" t="inlineStr">
+      <c r="E89" s="137">
+        <f>IF(A89="","",IF(C89&gt;0,(C89-B89)/C89,0))</f>
+        <v/>
+      </c>
+      <c r="F89" s="49" t="n"/>
+      <c r="G89" s="49" t="inlineStr">
         <is>
           <t>1p</t>
-        </is>
-      </c>
-      <c r="G89" s="49" t="inlineStr">
-        <is>
-          <t>Premium sports bar with food/drinks</t>
         </is>
       </c>
     </row>
@@ -2881,7 +3099,10 @@
         <f>IF(A90="","",C90-B90)</f>
         <v/>
       </c>
-      <c r="E90" s="49" t="n"/>
+      <c r="E90" s="137">
+        <f>IF(A90="","",IF(C90&gt;0,(C90-B90)/C90,0))</f>
+        <v/>
+      </c>
       <c r="F90" s="49" t="n"/>
       <c r="G90" s="49" t="n"/>
     </row>
@@ -2901,7 +3122,10 @@
         <f>IF(A91="","",C91-B91)</f>
         <v/>
       </c>
-      <c r="E91" s="49" t="n"/>
+      <c r="E91" s="137">
+        <f>IF(A91="","",IF(C91&gt;0,(C91-B91)/C91,0))</f>
+        <v/>
+      </c>
       <c r="F91" s="49" t="n"/>
       <c r="G91" s="49" t="n"/>
     </row>
@@ -2921,7 +3145,10 @@
         <f>IF(A92="","",C92-B92)</f>
         <v/>
       </c>
-      <c r="E92" s="49" t="n"/>
+      <c r="E92" s="137">
+        <f>IF(A92="","",IF(C92&gt;0,(C92-B92)/C92,0))</f>
+        <v/>
+      </c>
       <c r="F92" s="49" t="n"/>
       <c r="G92" s="49" t="n"/>
     </row>
@@ -2941,7 +3168,10 @@
         <f>IF(A93="","",C93-B93)</f>
         <v/>
       </c>
-      <c r="E93" s="49" t="n"/>
+      <c r="E93" s="137">
+        <f>IF(A93="","",IF(C93&gt;0,(C93-B93)/C93,0))</f>
+        <v/>
+      </c>
       <c r="F93" s="49" t="n"/>
       <c r="G93" s="49" t="n"/>
     </row>
@@ -3020,7 +3250,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="16.5" customHeight="1" s="42">
       <c r="A4" s="76" t="inlineStr">
         <is>
@@ -3062,37 +3291,25 @@
           <t>⛳ 골프</t>
         </is>
       </c>
-      <c r="I4" s="77" t="n"/>
-      <c r="J4" s="77" t="inlineStr">
-        <is>
-          <t>🔄 리플레이</t>
-        </is>
-      </c>
-      <c r="K4" s="77" t="n"/>
-      <c r="L4" s="77" t="inlineStr">
-        <is>
-          <t>🏨 호텔</t>
-        </is>
-      </c>
-      <c r="M4" s="77" t="n"/>
-      <c r="N4" s="77" t="inlineStr">
-        <is>
-          <t>🚐 교통</t>
-        </is>
-      </c>
-      <c r="O4" s="77" t="n"/>
+      <c r="I4" s="92" t="n"/>
+      <c r="J4" s="92" t="n"/>
+      <c r="K4" s="92" t="n"/>
+      <c r="L4" s="92" t="n"/>
+      <c r="M4" s="92" t="n"/>
+      <c r="N4" s="92" t="n"/>
+      <c r="O4" s="92" t="n"/>
       <c r="P4" s="77" t="inlineStr">
         <is>
           <t>🍽️ 식사</t>
         </is>
       </c>
-      <c r="Q4" s="77" t="n"/>
+      <c r="Q4" s="92" t="n"/>
       <c r="R4" s="77" t="inlineStr">
         <is>
           <t>📦 기타</t>
         </is>
       </c>
-      <c r="S4" s="77" t="n"/>
+      <c r="S4" s="92" t="n"/>
       <c r="T4" s="76" t="inlineStr">
         <is>
           <t>마진</t>
@@ -3513,7 +3730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P71"/>
+  <dimension ref="A1:R89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="42" min="1" max="1"/>
@@ -3531,7 +3748,8 @@
     <col hidden="1" width="8" customWidth="1" style="42" min="13" max="13"/>
     <col hidden="1" width="8" customWidth="1" style="42" min="14" max="14"/>
     <col hidden="1" width="8" customWidth="1" style="42" min="15" max="15"/>
-    <col hidden="1" width="13" customWidth="1" style="42" min="16" max="16"/>
+    <col hidden="1" width="13" customWidth="1" style="42" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" style="42" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3540,16 +3758,16 @@
           <t>🎯 PACKAGE SELECTOR</t>
         </is>
       </c>
-      <c r="B1" s="150" t="n"/>
-      <c r="C1" s="150" t="n"/>
-      <c r="D1" s="150" t="n"/>
-      <c r="E1" s="150" t="n"/>
-      <c r="F1" s="150" t="n"/>
-      <c r="G1" s="150" t="n"/>
-      <c r="H1" s="150" t="n"/>
-      <c r="I1" s="150" t="n"/>
-      <c r="J1" s="150" t="n"/>
-      <c r="K1" s="92" t="n"/>
+      <c r="B1" s="104" t="n"/>
+      <c r="C1" s="104" t="n"/>
+      <c r="D1" s="104" t="n"/>
+      <c r="E1" s="104" t="n"/>
+      <c r="F1" s="104" t="n"/>
+      <c r="G1" s="104" t="n"/>
+      <c r="H1" s="104" t="n"/>
+      <c r="I1" s="104" t="n"/>
+      <c r="J1" s="104" t="n"/>
+      <c r="K1" s="104" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="106" t="inlineStr">
@@ -3558,7 +3776,6 @@
         </is>
       </c>
       <c r="B2" s="129" t="inlineStr"/>
-      <c r="C2" s="87" t="n"/>
       <c r="D2" s="106" t="inlineStr">
         <is>
           <t>Golfers:</t>
@@ -3594,16 +3811,16 @@
           <t>✈️ OUTBOUND</t>
         </is>
       </c>
-      <c r="B3" s="150" t="n"/>
-      <c r="C3" s="150" t="n"/>
-      <c r="D3" s="150" t="n"/>
-      <c r="E3" s="150" t="n"/>
-      <c r="F3" s="150" t="n"/>
-      <c r="G3" s="150" t="n"/>
-      <c r="H3" s="150" t="n"/>
-      <c r="I3" s="150" t="n"/>
-      <c r="J3" s="150" t="n"/>
-      <c r="K3" s="92" t="n"/>
+      <c r="B3" s="77" t="n"/>
+      <c r="C3" s="77" t="n"/>
+      <c r="D3" s="77" t="n"/>
+      <c r="E3" s="77" t="n"/>
+      <c r="F3" s="77" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="77" t="n"/>
+      <c r="I3" s="77" t="n"/>
+      <c r="J3" s="77" t="n"/>
+      <c r="K3" s="77" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="106" t="inlineStr">
@@ -3650,16 +3867,16 @@
           <t>✈️ RETURN</t>
         </is>
       </c>
-      <c r="B5" s="150" t="n"/>
-      <c r="C5" s="150" t="n"/>
-      <c r="D5" s="150" t="n"/>
-      <c r="E5" s="150" t="n"/>
-      <c r="F5" s="150" t="n"/>
-      <c r="G5" s="150" t="n"/>
-      <c r="H5" s="150" t="n"/>
-      <c r="I5" s="150" t="n"/>
-      <c r="J5" s="150" t="n"/>
-      <c r="K5" s="92" t="n"/>
+      <c r="B5" s="77" t="n"/>
+      <c r="C5" s="77" t="n"/>
+      <c r="D5" s="77" t="n"/>
+      <c r="E5" s="77" t="n"/>
+      <c r="F5" s="77" t="n"/>
+      <c r="G5" s="77" t="n"/>
+      <c r="H5" s="77" t="n"/>
+      <c r="I5" s="77" t="n"/>
+      <c r="J5" s="77" t="n"/>
+      <c r="K5" s="77" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="106" t="inlineStr">
@@ -3707,7 +3924,7 @@
         </is>
       </c>
       <c r="B7" s="136">
-        <f>IF(SUM(R:R)&gt;0,"❌"&amp;SUM(R:R)&amp;" dup","✅")</f>
+        <f>IF(SUM(Q:Q)&gt;0,"❌"&amp;SUM(Q:Q)&amp;"dup","✅")</f>
         <v/>
       </c>
       <c r="D7" s="106" t="inlineStr">
@@ -3716,7 +3933,7 @@
         </is>
       </c>
       <c r="E7" s="133">
-        <f>J63</f>
+        <f>J72</f>
         <v/>
       </c>
       <c r="F7" s="81" t="inlineStr">
@@ -3725,7 +3942,7 @@
         </is>
       </c>
       <c r="G7" s="133">
-        <f>B71</f>
+        <f>B89</f>
         <v/>
       </c>
       <c r="H7" s="81" t="inlineStr">
@@ -3782,12 +3999,12 @@
       </c>
       <c r="J8" s="98" t="inlineStr">
         <is>
-          <t>TotCost</t>
+          <t>Cost</t>
         </is>
       </c>
       <c r="K8" s="98" t="inlineStr">
         <is>
-          <t>TotSell</t>
+          <t>Sell</t>
         </is>
       </c>
       <c r="L8" s="98" t="inlineStr">
@@ -3810,9 +4027,9 @@
           <t>P8</t>
         </is>
       </c>
-      <c r="P8" s="98" t="inlineStr">
-        <is>
-          <t>Dup</t>
+      <c r="Q8" s="98" t="inlineStr">
+        <is>
+          <t>Type</t>
         </is>
       </c>
     </row>
@@ -3822,16 +4039,16 @@
           <t>⛳ GOLF</t>
         </is>
       </c>
-      <c r="B9" s="150" t="n"/>
-      <c r="C9" s="150" t="n"/>
-      <c r="D9" s="150" t="n"/>
-      <c r="E9" s="150" t="n"/>
-      <c r="F9" s="150" t="n"/>
-      <c r="G9" s="150" t="n"/>
-      <c r="H9" s="150" t="n"/>
-      <c r="I9" s="150" t="n"/>
-      <c r="J9" s="150" t="n"/>
-      <c r="K9" s="92" t="n"/>
+      <c r="B9" s="77" t="n"/>
+      <c r="C9" s="77" t="n"/>
+      <c r="D9" s="77" t="n"/>
+      <c r="E9" s="77" t="n"/>
+      <c r="F9" s="77" t="n"/>
+      <c r="G9" s="77" t="n"/>
+      <c r="H9" s="77" t="n"/>
+      <c r="I9" s="77" t="n"/>
+      <c r="J9" s="77" t="n"/>
+      <c r="K9" s="77" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="109" t="inlineStr">
@@ -3870,9 +4087,14 @@
       <c r="M10" s="145" t="inlineStr"/>
       <c r="N10" s="145" t="inlineStr"/>
       <c r="O10" s="145" t="inlineStr"/>
-      <c r="P10" s="81">
+      <c r="Q10" s="81">
         <f>0</f>
         <v/>
+      </c>
+      <c r="R10" s="81" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -3912,9 +4134,14 @@
       <c r="M11" s="145" t="inlineStr"/>
       <c r="N11" s="145" t="inlineStr"/>
       <c r="O11" s="145" t="inlineStr"/>
-      <c r="P11" s="81">
+      <c r="Q11" s="81">
         <f>IF(A11="",0,COUNTIF(A$10:A10,A11))</f>
         <v/>
+      </c>
+      <c r="R11" s="81" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -3954,9 +4181,14 @@
       <c r="M12" s="145" t="inlineStr"/>
       <c r="N12" s="145" t="inlineStr"/>
       <c r="O12" s="145" t="inlineStr"/>
-      <c r="P12" s="81">
+      <c r="Q12" s="81">
         <f>IF(A12="",0,COUNTIF(A$10:A11,A12))</f>
         <v/>
+      </c>
+      <c r="R12" s="81" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -3990,10 +4222,11 @@
       <c r="M13" s="145" t="inlineStr"/>
       <c r="N13" s="145" t="inlineStr"/>
       <c r="O13" s="145" t="inlineStr"/>
-      <c r="P13" s="81">
+      <c r="Q13" s="81">
         <f>IF(A13="",0,COUNTIF(A$10:A12,A13))</f>
         <v/>
       </c>
+      <c r="R13" s="81" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="129" t="inlineStr"/>
@@ -4026,10 +4259,11 @@
       <c r="M14" s="145" t="inlineStr"/>
       <c r="N14" s="145" t="inlineStr"/>
       <c r="O14" s="145" t="inlineStr"/>
-      <c r="P14" s="81">
+      <c r="Q14" s="81">
         <f>IF(A14="",0,COUNTIF(A$10:A13,A14))</f>
         <v/>
       </c>
+      <c r="R14" s="81" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="123" t="inlineStr">
@@ -4042,19 +4276,19 @@
       <c r="D15" s="114" t="inlineStr"/>
       <c r="E15" s="114" t="inlineStr"/>
       <c r="F15" s="130">
-        <f>SUMPRODUCT((F10:F14="●")*1,B10:B14,C10:C14)</f>
+        <f>IF(F10="●",B10*C10,0)+IF(F11="●",B11*C11,0)+IF(F12="●",B12*C12,0)+IF(F13="●",B13*C13,0)+IF(F14="●",B14*C14,0)</f>
         <v/>
       </c>
       <c r="G15" s="130">
-        <f>SUMPRODUCT((G10:G14="●")*1,B10:B14,C10:C14)</f>
+        <f>IF(G10="●",B10*C10,0)+IF(G11="●",B11*C11,0)+IF(G12="●",B12*C12,0)+IF(G13="●",B13*C13,0)+IF(G14="●",B14*C14,0)</f>
         <v/>
       </c>
       <c r="H15" s="130">
-        <f>SUMPRODUCT((H10:H14="●")*1,B10:B14,C10:C14)</f>
+        <f>IF(H10="●",B10*C10,0)+IF(H11="●",B11*C11,0)+IF(H12="●",B12*C12,0)+IF(H13="●",B13*C13,0)+IF(H14="●",B14*C14,0)</f>
         <v/>
       </c>
       <c r="I15" s="130">
-        <f>SUMPRODUCT((I10:I14="●")*1,B10:B14,C10:C14)</f>
+        <f>IF(I10="●",B10*C10,0)+IF(I11="●",B11*C11,0)+IF(I12="●",B12*C12,0)+IF(I13="●",B13*C13,0)+IF(I14="●",B14*C14,0)</f>
         <v/>
       </c>
       <c r="J15" s="88">
@@ -4066,19 +4300,19 @@
         <v/>
       </c>
       <c r="L15" s="130">
-        <f>SUMPRODUCT((L10:L14="●")*1,B10:B14,C10:C14)</f>
+        <f>IF(L10="●",B10*C10,0)+IF(L11="●",B11*C11,0)+IF(L12="●",B12*C12,0)+IF(L13="●",B13*C13,0)+IF(L14="●",B14*C14,0)</f>
         <v/>
       </c>
       <c r="M15" s="130">
-        <f>SUMPRODUCT((M10:M14="●")*1,B10:B14,C10:C14)</f>
+        <f>IF(M10="●",B10*C10,0)+IF(M11="●",B11*C11,0)+IF(M12="●",B12*C12,0)+IF(M13="●",B13*C13,0)+IF(M14="●",B14*C14,0)</f>
         <v/>
       </c>
       <c r="N15" s="130">
-        <f>SUMPRODUCT((N10:N14="●")*1,B10:B14,C10:C14)</f>
+        <f>IF(N10="●",B10*C10,0)+IF(N11="●",B11*C11,0)+IF(N12="●",B12*C12,0)+IF(N13="●",B13*C13,0)+IF(N14="●",B14*C14,0)</f>
         <v/>
       </c>
       <c r="O15" s="130">
-        <f>SUMPRODUCT((O10:O14="●")*1,B10:B14,C10:C14)</f>
+        <f>IF(O10="●",B10*C10,0)+IF(O11="●",B11*C11,0)+IF(O12="●",B12*C12,0)+IF(O13="●",B13*C13,0)+IF(O14="●",B14*C14,0)</f>
         <v/>
       </c>
     </row>
@@ -4088,16 +4322,16 @@
           <t>🏨 HOTEL</t>
         </is>
       </c>
-      <c r="B17" s="150" t="n"/>
-      <c r="C17" s="150" t="n"/>
-      <c r="D17" s="150" t="n"/>
-      <c r="E17" s="150" t="n"/>
-      <c r="F17" s="150" t="n"/>
-      <c r="G17" s="150" t="n"/>
-      <c r="H17" s="150" t="n"/>
-      <c r="I17" s="150" t="n"/>
-      <c r="J17" s="150" t="n"/>
-      <c r="K17" s="92" t="n"/>
+      <c r="B17" s="77" t="n"/>
+      <c r="C17" s="77" t="n"/>
+      <c r="D17" s="77" t="n"/>
+      <c r="E17" s="77" t="n"/>
+      <c r="F17" s="77" t="n"/>
+      <c r="G17" s="77" t="n"/>
+      <c r="H17" s="77" t="n"/>
+      <c r="I17" s="77" t="n"/>
+      <c r="J17" s="77" t="n"/>
+      <c r="K17" s="77" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="109" t="inlineStr">
@@ -4136,9 +4370,14 @@
       <c r="M18" s="145" t="inlineStr"/>
       <c r="N18" s="145" t="inlineStr"/>
       <c r="O18" s="145" t="inlineStr"/>
-      <c r="P18" s="81">
+      <c r="Q18" s="81">
         <f>0</f>
         <v/>
+      </c>
+      <c r="R18" s="81" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -4172,10 +4411,11 @@
       <c r="M19" s="145" t="inlineStr"/>
       <c r="N19" s="145" t="inlineStr"/>
       <c r="O19" s="145" t="inlineStr"/>
-      <c r="P19" s="81">
+      <c r="Q19" s="81">
         <f>IF(A19="",0,COUNTIF(A$18:A18,A19))</f>
         <v/>
       </c>
+      <c r="R19" s="81" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="129" t="inlineStr"/>
@@ -4208,10 +4448,11 @@
       <c r="M20" s="145" t="inlineStr"/>
       <c r="N20" s="145" t="inlineStr"/>
       <c r="O20" s="145" t="inlineStr"/>
-      <c r="P20" s="81">
+      <c r="Q20" s="81">
         <f>IF(A20="",0,COUNTIF(A$18:A19,A20))</f>
         <v/>
       </c>
+      <c r="R20" s="81" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="123" t="inlineStr">
@@ -4224,19 +4465,19 @@
       <c r="D21" s="114" t="inlineStr"/>
       <c r="E21" s="114" t="inlineStr"/>
       <c r="F21" s="130">
-        <f>SUMPRODUCT((F18:F20="●")*1,B18:B20,C18:C20)</f>
+        <f>IF(F18="●",B18*C18,0)+IF(F19="●",B19*C19,0)+IF(F20="●",B20*C20,0)</f>
         <v/>
       </c>
       <c r="G21" s="130">
-        <f>SUMPRODUCT((G18:G20="●")*1,B18:B20,C18:C20)</f>
+        <f>IF(G18="●",B18*C18,0)+IF(G19="●",B19*C19,0)+IF(G20="●",B20*C20,0)</f>
         <v/>
       </c>
       <c r="H21" s="130">
-        <f>SUMPRODUCT((H18:H20="●")*1,B18:B20,C18:C20)</f>
+        <f>IF(H18="●",B18*C18,0)+IF(H19="●",B19*C19,0)+IF(H20="●",B20*C20,0)</f>
         <v/>
       </c>
       <c r="I21" s="130">
-        <f>SUMPRODUCT((I18:I20="●")*1,B18:B20,C18:C20)</f>
+        <f>IF(I18="●",B18*C18,0)+IF(I19="●",B19*C19,0)+IF(I20="●",B20*C20,0)</f>
         <v/>
       </c>
       <c r="J21" s="88">
@@ -4248,19 +4489,19 @@
         <v/>
       </c>
       <c r="L21" s="130">
-        <f>SUMPRODUCT((L18:L20="●")*1,B18:B20,C18:C20)</f>
+        <f>IF(L18="●",B18*C18,0)+IF(L19="●",B19*C19,0)+IF(L20="●",B20*C20,0)</f>
         <v/>
       </c>
       <c r="M21" s="130">
-        <f>SUMPRODUCT((M18:M20="●")*1,B18:B20,C18:C20)</f>
+        <f>IF(M18="●",B18*C18,0)+IF(M19="●",B19*C19,0)+IF(M20="●",B20*C20,0)</f>
         <v/>
       </c>
       <c r="N21" s="130">
-        <f>SUMPRODUCT((N18:N20="●")*1,B18:B20,C18:C20)</f>
+        <f>IF(N18="●",B18*C18,0)+IF(N19="●",B19*C19,0)+IF(N20="●",B20*C20,0)</f>
         <v/>
       </c>
       <c r="O21" s="130">
-        <f>SUMPRODUCT((O18:O20="●")*1,B18:B20,C18:C20)</f>
+        <f>IF(O18="●",B18*C18,0)+IF(O19="●",B19*C19,0)+IF(O20="●",B20*C20,0)</f>
         <v/>
       </c>
     </row>
@@ -4270,16 +4511,16 @@
           <t>🚐 TRANSPORT</t>
         </is>
       </c>
-      <c r="B23" s="150" t="n"/>
-      <c r="C23" s="150" t="n"/>
-      <c r="D23" s="150" t="n"/>
-      <c r="E23" s="150" t="n"/>
-      <c r="F23" s="150" t="n"/>
-      <c r="G23" s="150" t="n"/>
-      <c r="H23" s="150" t="n"/>
-      <c r="I23" s="150" t="n"/>
-      <c r="J23" s="150" t="n"/>
-      <c r="K23" s="92" t="n"/>
+      <c r="B23" s="77" t="n"/>
+      <c r="C23" s="77" t="n"/>
+      <c r="D23" s="77" t="n"/>
+      <c r="E23" s="77" t="n"/>
+      <c r="F23" s="77" t="n"/>
+      <c r="G23" s="77" t="n"/>
+      <c r="H23" s="77" t="n"/>
+      <c r="I23" s="77" t="n"/>
+      <c r="J23" s="77" t="n"/>
+      <c r="K23" s="77" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="109" t="inlineStr">
@@ -4307,20 +4548,25 @@
       <c r="H24" s="145" t="inlineStr"/>
       <c r="I24" s="145" t="inlineStr"/>
       <c r="J24" s="84">
-        <f>IF(A24="","",(COUNTIF(F24,"●")+COUNTIF(G24,"●")+COUNTIF(H24,"●")+COUNTIF(I24,"●")+COUNTIF(L24,"●")+COUNTIF(M24,"●")+COUNTIF(N24,"●")+COUNTIF(O24,"●"))*B24*C24)</f>
+        <f>IF(A24="","",IF(OR((F24="●")+(G24="●")+(H24="●")+(I24="●")+(L24="●")+(M24="●")+(N24="●")+(O24="●")),B24*C24,0))</f>
         <v/>
       </c>
       <c r="K24" s="84">
-        <f>IF(A24="","",(COUNTIF(F24,"●")+COUNTIF(G24,"●")+COUNTIF(H24,"●")+COUNTIF(I24,"●")+COUNTIF(L24,"●")+COUNTIF(M24,"●")+COUNTIF(N24,"●")+COUNTIF(O24,"●"))*B24*D24)</f>
+        <f>IF(A24="","",IF(OR((F24="●")+(G24="●")+(H24="●")+(I24="●")+(L24="●")+(M24="●")+(N24="●")+(O24="●")),B24*D24,0))</f>
         <v/>
       </c>
       <c r="L24" s="145" t="inlineStr"/>
       <c r="M24" s="145" t="inlineStr"/>
       <c r="N24" s="145" t="inlineStr"/>
       <c r="O24" s="145" t="inlineStr"/>
-      <c r="P24" s="81">
+      <c r="Q24" s="81">
         <f>0</f>
         <v/>
+      </c>
+      <c r="R24" s="81" t="inlineStr">
+        <is>
+          <t>pg</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -4354,10 +4600,11 @@
       <c r="M25" s="145" t="inlineStr"/>
       <c r="N25" s="145" t="inlineStr"/>
       <c r="O25" s="145" t="inlineStr"/>
-      <c r="P25" s="81">
+      <c r="Q25" s="81">
         <f>IF(A25="",0,COUNTIF(A$24:A24,A25))</f>
         <v/>
       </c>
+      <c r="R25" s="81" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="129" t="inlineStr"/>
@@ -4390,10 +4637,11 @@
       <c r="M26" s="145" t="inlineStr"/>
       <c r="N26" s="145" t="inlineStr"/>
       <c r="O26" s="145" t="inlineStr"/>
-      <c r="P26" s="81">
+      <c r="Q26" s="81">
         <f>IF(A26="",0,COUNTIF(A$24:A25,A26))</f>
         <v/>
       </c>
+      <c r="R26" s="81" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="123" t="inlineStr">
@@ -4406,19 +4654,19 @@
       <c r="D27" s="114" t="inlineStr"/>
       <c r="E27" s="114" t="inlineStr"/>
       <c r="F27" s="130">
-        <f>SUMPRODUCT((F24:F26="●")*1,B24:B26,C24:C26)</f>
+        <f>IF(OR(F24="●"),B24*C24,0)+IF(F25="●",B25*C25,0)+IF(F26="●",B26*C26,0)</f>
         <v/>
       </c>
       <c r="G27" s="130">
-        <f>SUMPRODUCT((G24:G26="●")*1,B24:B26,C24:C26)</f>
+        <f>IF(OR(G24="●"),B24*C24,0)+IF(G25="●",B25*C25,0)+IF(G26="●",B26*C26,0)</f>
         <v/>
       </c>
       <c r="H27" s="130">
-        <f>SUMPRODUCT((H24:H26="●")*1,B24:B26,C24:C26)</f>
+        <f>IF(OR(H24="●"),B24*C24,0)+IF(H25="●",B25*C25,0)+IF(H26="●",B26*C26,0)</f>
         <v/>
       </c>
       <c r="I27" s="130">
-        <f>SUMPRODUCT((I24:I26="●")*1,B24:B26,C24:C26)</f>
+        <f>IF(OR(I24="●"),B24*C24,0)+IF(I25="●",B25*C25,0)+IF(I26="●",B26*C26,0)</f>
         <v/>
       </c>
       <c r="J27" s="88">
@@ -4430,19 +4678,19 @@
         <v/>
       </c>
       <c r="L27" s="130">
-        <f>SUMPRODUCT((L24:L26="●")*1,B24:B26,C24:C26)</f>
+        <f>IF(OR(L24="●"),B24*C24,0)+IF(L25="●",B25*C25,0)+IF(L26="●",B26*C26,0)</f>
         <v/>
       </c>
       <c r="M27" s="130">
-        <f>SUMPRODUCT((M24:M26="●")*1,B24:B26,C24:C26)</f>
+        <f>IF(OR(M24="●"),B24*C24,0)+IF(M25="●",B25*C25,0)+IF(M26="●",B26*C26,0)</f>
         <v/>
       </c>
       <c r="N27" s="130">
-        <f>SUMPRODUCT((N24:N26="●")*1,B24:B26,C24:C26)</f>
+        <f>IF(OR(N24="●"),B24*C24,0)+IF(N25="●",B25*C25,0)+IF(N26="●",B26*C26,0)</f>
         <v/>
       </c>
       <c r="O27" s="130">
-        <f>SUMPRODUCT((O24:O26="●")*1,B24:B26,C24:C26)</f>
+        <f>IF(OR(O24="●"),B24*C24,0)+IF(O25="●",B25*C25,0)+IF(O26="●",B26*C26,0)</f>
         <v/>
       </c>
     </row>
@@ -4452,16 +4700,16 @@
           <t>🍽️ MEALS</t>
         </is>
       </c>
-      <c r="B29" s="150" t="n"/>
-      <c r="C29" s="150" t="n"/>
-      <c r="D29" s="150" t="n"/>
-      <c r="E29" s="150" t="n"/>
-      <c r="F29" s="150" t="n"/>
-      <c r="G29" s="150" t="n"/>
-      <c r="H29" s="150" t="n"/>
-      <c r="I29" s="150" t="n"/>
-      <c r="J29" s="150" t="n"/>
-      <c r="K29" s="92" t="n"/>
+      <c r="B29" s="77" t="n"/>
+      <c r="C29" s="77" t="n"/>
+      <c r="D29" s="77" t="n"/>
+      <c r="E29" s="77" t="n"/>
+      <c r="F29" s="77" t="n"/>
+      <c r="G29" s="77" t="n"/>
+      <c r="H29" s="77" t="n"/>
+      <c r="I29" s="77" t="n"/>
+      <c r="J29" s="77" t="n"/>
+      <c r="K29" s="77" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="109" t="inlineStr">
@@ -4500,9 +4748,14 @@
       <c r="M30" s="145" t="inlineStr"/>
       <c r="N30" s="145" t="inlineStr"/>
       <c r="O30" s="145" t="inlineStr"/>
-      <c r="P30" s="81">
+      <c r="Q30" s="81">
         <f>0</f>
         <v/>
+      </c>
+      <c r="R30" s="81" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -4542,9 +4795,14 @@
       <c r="M31" s="145" t="inlineStr"/>
       <c r="N31" s="145" t="inlineStr"/>
       <c r="O31" s="145" t="inlineStr"/>
-      <c r="P31" s="81">
+      <c r="Q31" s="81">
         <f>IF(A31="",0,COUNTIF(A$30:A30,A31))</f>
         <v/>
+      </c>
+      <c r="R31" s="81" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -4584,9 +4842,14 @@
       <c r="M32" s="145" t="inlineStr"/>
       <c r="N32" s="145" t="inlineStr"/>
       <c r="O32" s="145" t="inlineStr"/>
-      <c r="P32" s="81">
+      <c r="Q32" s="81">
         <f>IF(A32="",0,COUNTIF(A$30:A31,A32))</f>
         <v/>
+      </c>
+      <c r="R32" s="81" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -4626,9 +4889,14 @@
       <c r="M33" s="145" t="inlineStr"/>
       <c r="N33" s="145" t="inlineStr"/>
       <c r="O33" s="145" t="inlineStr"/>
-      <c r="P33" s="81">
+      <c r="Q33" s="81">
         <f>IF(A33="",0,COUNTIF(A$30:A32,A33))</f>
         <v/>
+      </c>
+      <c r="R33" s="81" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -4662,10 +4930,11 @@
       <c r="M34" s="145" t="inlineStr"/>
       <c r="N34" s="145" t="inlineStr"/>
       <c r="O34" s="145" t="inlineStr"/>
-      <c r="P34" s="81">
+      <c r="Q34" s="81">
         <f>IF(A34="",0,COUNTIF(A$30:A33,A34))</f>
         <v/>
       </c>
+      <c r="R34" s="81" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="123" t="inlineStr">
@@ -4678,19 +4947,19 @@
       <c r="D35" s="114" t="inlineStr"/>
       <c r="E35" s="114" t="inlineStr"/>
       <c r="F35" s="130">
-        <f>SUMPRODUCT((F30:F34="●")*1,B30:B34,C30:C34)</f>
+        <f>IF(F30="●",B30*C30,0)+IF(F31="●",B31*C31,0)+IF(F32="●",B32*C32,0)+IF(F33="●",B33*C33,0)+IF(F34="●",B34*C34,0)</f>
         <v/>
       </c>
       <c r="G35" s="130">
-        <f>SUMPRODUCT((G30:G34="●")*1,B30:B34,C30:C34)</f>
+        <f>IF(G30="●",B30*C30,0)+IF(G31="●",B31*C31,0)+IF(G32="●",B32*C32,0)+IF(G33="●",B33*C33,0)+IF(G34="●",B34*C34,0)</f>
         <v/>
       </c>
       <c r="H35" s="130">
-        <f>SUMPRODUCT((H30:H34="●")*1,B30:B34,C30:C34)</f>
+        <f>IF(H30="●",B30*C30,0)+IF(H31="●",B31*C31,0)+IF(H32="●",B32*C32,0)+IF(H33="●",B33*C33,0)+IF(H34="●",B34*C34,0)</f>
         <v/>
       </c>
       <c r="I35" s="130">
-        <f>SUMPRODUCT((I30:I34="●")*1,B30:B34,C30:C34)</f>
+        <f>IF(I30="●",B30*C30,0)+IF(I31="●",B31*C31,0)+IF(I32="●",B32*C32,0)+IF(I33="●",B33*C33,0)+IF(I34="●",B34*C34,0)</f>
         <v/>
       </c>
       <c r="J35" s="88">
@@ -4702,19 +4971,19 @@
         <v/>
       </c>
       <c r="L35" s="130">
-        <f>SUMPRODUCT((L30:L34="●")*1,B30:B34,C30:C34)</f>
+        <f>IF(L30="●",B30*C30,0)+IF(L31="●",B31*C31,0)+IF(L32="●",B32*C32,0)+IF(L33="●",B33*C33,0)+IF(L34="●",B34*C34,0)</f>
         <v/>
       </c>
       <c r="M35" s="130">
-        <f>SUMPRODUCT((M30:M34="●")*1,B30:B34,C30:C34)</f>
+        <f>IF(M30="●",B30*C30,0)+IF(M31="●",B31*C31,0)+IF(M32="●",B32*C32,0)+IF(M33="●",B33*C33,0)+IF(M34="●",B34*C34,0)</f>
         <v/>
       </c>
       <c r="N35" s="130">
-        <f>SUMPRODUCT((N30:N34="●")*1,B30:B34,C30:C34)</f>
+        <f>IF(N30="●",B30*C30,0)+IF(N31="●",B31*C31,0)+IF(N32="●",B32*C32,0)+IF(N33="●",B33*C33,0)+IF(N34="●",B34*C34,0)</f>
         <v/>
       </c>
       <c r="O35" s="130">
-        <f>SUMPRODUCT((O30:O34="●")*1,B30:B34,C30:C34)</f>
+        <f>IF(O30="●",B30*C30,0)+IF(O31="●",B31*C31,0)+IF(O32="●",B32*C32,0)+IF(O33="●",B33*C33,0)+IF(O34="●",B34*C34,0)</f>
         <v/>
       </c>
     </row>
@@ -4724,16 +4993,16 @@
           <t>📦 OTHER</t>
         </is>
       </c>
-      <c r="B37" s="150" t="n"/>
-      <c r="C37" s="150" t="n"/>
-      <c r="D37" s="150" t="n"/>
-      <c r="E37" s="150" t="n"/>
-      <c r="F37" s="150" t="n"/>
-      <c r="G37" s="150" t="n"/>
-      <c r="H37" s="150" t="n"/>
-      <c r="I37" s="150" t="n"/>
-      <c r="J37" s="150" t="n"/>
-      <c r="K37" s="92" t="n"/>
+      <c r="B37" s="77" t="n"/>
+      <c r="C37" s="77" t="n"/>
+      <c r="D37" s="77" t="n"/>
+      <c r="E37" s="77" t="n"/>
+      <c r="F37" s="77" t="n"/>
+      <c r="G37" s="77" t="n"/>
+      <c r="H37" s="77" t="n"/>
+      <c r="I37" s="77" t="n"/>
+      <c r="J37" s="77" t="n"/>
+      <c r="K37" s="77" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="109" t="inlineStr">
@@ -4761,20 +5030,25 @@
       <c r="H38" s="145" t="inlineStr"/>
       <c r="I38" s="145" t="inlineStr"/>
       <c r="J38" s="84">
-        <f>IF(A38="","",(COUNTIF(F38,"●")+COUNTIF(G38,"●")+COUNTIF(H38,"●")+COUNTIF(I38,"●")+COUNTIF(L38,"●")+COUNTIF(M38,"●")+COUNTIF(N38,"●")+COUNTIF(O38,"●"))*B38*C38)</f>
+        <f>IF(A38="","",IF(OR((F38="●")+(G38="●")+(H38="●")+(I38="●")+(L38="●")+(M38="●")+(N38="●")+(O38="●")),B38*C38,0))</f>
         <v/>
       </c>
       <c r="K38" s="84">
-        <f>IF(A38="","",(COUNTIF(F38,"●")+COUNTIF(G38,"●")+COUNTIF(H38,"●")+COUNTIF(I38,"●")+COUNTIF(L38,"●")+COUNTIF(M38,"●")+COUNTIF(N38,"●")+COUNTIF(O38,"●"))*B38*D38)</f>
+        <f>IF(A38="","",IF(OR((F38="●")+(G38="●")+(H38="●")+(I38="●")+(L38="●")+(M38="●")+(N38="●")+(O38="●")),B38*D38,0))</f>
         <v/>
       </c>
       <c r="L38" s="145" t="inlineStr"/>
       <c r="M38" s="145" t="inlineStr"/>
       <c r="N38" s="145" t="inlineStr"/>
       <c r="O38" s="145" t="inlineStr"/>
-      <c r="P38" s="81">
+      <c r="Q38" s="81">
         <f>0</f>
         <v/>
+      </c>
+      <c r="R38" s="81" t="inlineStr">
+        <is>
+          <t>pg</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -4808,10 +5082,11 @@
       <c r="M39" s="145" t="inlineStr"/>
       <c r="N39" s="145" t="inlineStr"/>
       <c r="O39" s="145" t="inlineStr"/>
-      <c r="P39" s="81">
+      <c r="Q39" s="81">
         <f>IF(A39="",0,COUNTIF(A$38:A38,A39))</f>
         <v/>
       </c>
+      <c r="R39" s="81" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="129" t="inlineStr"/>
@@ -4844,10 +5119,11 @@
       <c r="M40" s="145" t="inlineStr"/>
       <c r="N40" s="145" t="inlineStr"/>
       <c r="O40" s="145" t="inlineStr"/>
-      <c r="P40" s="81">
+      <c r="Q40" s="81">
         <f>IF(A40="",0,COUNTIF(A$38:A39,A40))</f>
         <v/>
       </c>
+      <c r="R40" s="81" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="123" t="inlineStr">
@@ -4860,19 +5136,19 @@
       <c r="D41" s="114" t="inlineStr"/>
       <c r="E41" s="114" t="inlineStr"/>
       <c r="F41" s="130">
-        <f>SUMPRODUCT((F38:F40="●")*1,B38:B40,C38:C40)</f>
+        <f>IF(OR(F38="●"),B38*C38,0)+IF(F39="●",B39*C39,0)+IF(F40="●",B40*C40,0)</f>
         <v/>
       </c>
       <c r="G41" s="130">
-        <f>SUMPRODUCT((G38:G40="●")*1,B38:B40,C38:C40)</f>
+        <f>IF(OR(G38="●"),B38*C38,0)+IF(G39="●",B39*C39,0)+IF(G40="●",B40*C40,0)</f>
         <v/>
       </c>
       <c r="H41" s="130">
-        <f>SUMPRODUCT((H38:H40="●")*1,B38:B40,C38:C40)</f>
+        <f>IF(OR(H38="●"),B38*C38,0)+IF(H39="●",B39*C39,0)+IF(H40="●",B40*C40,0)</f>
         <v/>
       </c>
       <c r="I41" s="130">
-        <f>SUMPRODUCT((I38:I40="●")*1,B38:B40,C38:C40)</f>
+        <f>IF(OR(I38="●"),B38*C38,0)+IF(I39="●",B39*C39,0)+IF(I40="●",B40*C40,0)</f>
         <v/>
       </c>
       <c r="J41" s="88">
@@ -4884,19 +5160,19 @@
         <v/>
       </c>
       <c r="L41" s="130">
-        <f>SUMPRODUCT((L38:L40="●")*1,B38:B40,C38:C40)</f>
+        <f>IF(OR(L38="●"),B38*C38,0)+IF(L39="●",B39*C39,0)+IF(L40="●",B40*C40,0)</f>
         <v/>
       </c>
       <c r="M41" s="130">
-        <f>SUMPRODUCT((M38:M40="●")*1,B38:B40,C38:C40)</f>
+        <f>IF(OR(M38="●"),B38*C38,0)+IF(M39="●",B39*C39,0)+IF(M40="●",B40*C40,0)</f>
         <v/>
       </c>
       <c r="N41" s="130">
-        <f>SUMPRODUCT((N38:N40="●")*1,B38:B40,C38:C40)</f>
+        <f>IF(OR(N38="●"),B38*C38,0)+IF(N39="●",B39*C39,0)+IF(N40="●",B40*C40,0)</f>
         <v/>
       </c>
       <c r="O41" s="130">
-        <f>SUMPRODUCT((O38:O40="●")*1,B38:B40,C38:C40)</f>
+        <f>IF(OR(O38="●"),B38*C38,0)+IF(O39="●",B39*C39,0)+IF(O40="●",B40*C40,0)</f>
         <v/>
       </c>
     </row>
@@ -4906,16 +5182,16 @@
           <t>🎯 ACTIVITIES</t>
         </is>
       </c>
-      <c r="B43" s="150" t="n"/>
-      <c r="C43" s="150" t="n"/>
-      <c r="D43" s="150" t="n"/>
-      <c r="E43" s="150" t="n"/>
-      <c r="F43" s="150" t="n"/>
-      <c r="G43" s="150" t="n"/>
-      <c r="H43" s="150" t="n"/>
-      <c r="I43" s="150" t="n"/>
-      <c r="J43" s="150" t="n"/>
-      <c r="K43" s="92" t="n"/>
+      <c r="B43" s="77" t="n"/>
+      <c r="C43" s="77" t="n"/>
+      <c r="D43" s="77" t="n"/>
+      <c r="E43" s="77" t="n"/>
+      <c r="F43" s="77" t="n"/>
+      <c r="G43" s="77" t="n"/>
+      <c r="H43" s="77" t="n"/>
+      <c r="I43" s="77" t="n"/>
+      <c r="J43" s="77" t="n"/>
+      <c r="K43" s="77" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="109" t="inlineStr">
@@ -4954,9 +5230,14 @@
       <c r="M44" s="145" t="inlineStr"/>
       <c r="N44" s="145" t="inlineStr"/>
       <c r="O44" s="145" t="inlineStr"/>
-      <c r="P44" s="81">
+      <c r="Q44" s="81">
         <f>0</f>
         <v/>
+      </c>
+      <c r="R44" s="81" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -4996,9 +5277,14 @@
       <c r="M45" s="145" t="inlineStr"/>
       <c r="N45" s="145" t="inlineStr"/>
       <c r="O45" s="145" t="inlineStr"/>
-      <c r="P45" s="81">
+      <c r="Q45" s="81">
         <f>IF(A45="",0,COUNTIF(A$44:A44,A45))</f>
         <v/>
+      </c>
+      <c r="R45" s="81" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -5038,9 +5324,14 @@
       <c r="M46" s="145" t="inlineStr"/>
       <c r="N46" s="145" t="inlineStr"/>
       <c r="O46" s="145" t="inlineStr"/>
-      <c r="P46" s="81">
+      <c r="Q46" s="81">
         <f>IF(A46="",0,COUNTIF(A$44:A45,A46))</f>
         <v/>
+      </c>
+      <c r="R46" s="81" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -5080,9 +5371,14 @@
       <c r="M47" s="145" t="inlineStr"/>
       <c r="N47" s="145" t="inlineStr"/>
       <c r="O47" s="145" t="inlineStr"/>
-      <c r="P47" s="81">
+      <c r="Q47" s="81">
         <f>IF(A47="",0,COUNTIF(A$44:A46,A47))</f>
         <v/>
+      </c>
+      <c r="R47" s="81" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -5116,10 +5412,11 @@
       <c r="M48" s="145" t="inlineStr"/>
       <c r="N48" s="145" t="inlineStr"/>
       <c r="O48" s="145" t="inlineStr"/>
-      <c r="P48" s="81">
+      <c r="Q48" s="81">
         <f>IF(A48="",0,COUNTIF(A$44:A47,A48))</f>
         <v/>
       </c>
+      <c r="R48" s="81" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="129" t="inlineStr"/>
@@ -5152,10 +5449,11 @@
       <c r="M49" s="145" t="inlineStr"/>
       <c r="N49" s="145" t="inlineStr"/>
       <c r="O49" s="145" t="inlineStr"/>
-      <c r="P49" s="81">
+      <c r="Q49" s="81">
         <f>IF(A49="",0,COUNTIF(A$44:A48,A49))</f>
         <v/>
       </c>
+      <c r="R49" s="81" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="129" t="inlineStr"/>
@@ -5188,10 +5486,11 @@
       <c r="M50" s="145" t="inlineStr"/>
       <c r="N50" s="145" t="inlineStr"/>
       <c r="O50" s="145" t="inlineStr"/>
-      <c r="P50" s="81">
+      <c r="Q50" s="81">
         <f>IF(A50="",0,COUNTIF(A$44:A49,A50))</f>
         <v/>
       </c>
+      <c r="R50" s="81" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="129" t="inlineStr"/>
@@ -5224,10 +5523,11 @@
       <c r="M51" s="145" t="inlineStr"/>
       <c r="N51" s="145" t="inlineStr"/>
       <c r="O51" s="145" t="inlineStr"/>
-      <c r="P51" s="81">
+      <c r="Q51" s="81">
         <f>IF(A51="",0,COUNTIF(A$44:A50,A51))</f>
         <v/>
       </c>
+      <c r="R51" s="81" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="129" t="inlineStr"/>
@@ -5260,10 +5560,11 @@
       <c r="M52" s="145" t="inlineStr"/>
       <c r="N52" s="145" t="inlineStr"/>
       <c r="O52" s="145" t="inlineStr"/>
-      <c r="P52" s="81">
+      <c r="Q52" s="81">
         <f>IF(A52="",0,COUNTIF(A$44:A51,A52))</f>
         <v/>
       </c>
+      <c r="R52" s="81" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="123" t="inlineStr">
@@ -5276,19 +5577,19 @@
       <c r="D53" s="114" t="inlineStr"/>
       <c r="E53" s="114" t="inlineStr"/>
       <c r="F53" s="130">
-        <f>SUMPRODUCT((F44:F52="●")*1,B44:B52,C44:C52)</f>
+        <f>IF(F44="●",B44*C44,0)+IF(F45="●",B45*C45,0)+IF(F46="●",B46*C46,0)+IF(F47="●",B47*C47,0)+IF(F48="●",B48*C48,0)+IF(F49="●",B49*C49,0)+IF(F50="●",B50*C50,0)+IF(F51="●",B51*C51,0)+IF(F52="●",B52*C52,0)</f>
         <v/>
       </c>
       <c r="G53" s="130">
-        <f>SUMPRODUCT((G44:G52="●")*1,B44:B52,C44:C52)</f>
+        <f>IF(G44="●",B44*C44,0)+IF(G45="●",B45*C45,0)+IF(G46="●",B46*C46,0)+IF(G47="●",B47*C47,0)+IF(G48="●",B48*C48,0)+IF(G49="●",B49*C49,0)+IF(G50="●",B50*C50,0)+IF(G51="●",B51*C51,0)+IF(G52="●",B52*C52,0)</f>
         <v/>
       </c>
       <c r="H53" s="130">
-        <f>SUMPRODUCT((H44:H52="●")*1,B44:B52,C44:C52)</f>
+        <f>IF(H44="●",B44*C44,0)+IF(H45="●",B45*C45,0)+IF(H46="●",B46*C46,0)+IF(H47="●",B47*C47,0)+IF(H48="●",B48*C48,0)+IF(H49="●",B49*C49,0)+IF(H50="●",B50*C50,0)+IF(H51="●",B51*C51,0)+IF(H52="●",B52*C52,0)</f>
         <v/>
       </c>
       <c r="I53" s="130">
-        <f>SUMPRODUCT((I44:I52="●")*1,B44:B52,C44:C52)</f>
+        <f>IF(I44="●",B44*C44,0)+IF(I45="●",B45*C45,0)+IF(I46="●",B46*C46,0)+IF(I47="●",B47*C47,0)+IF(I48="●",B48*C48,0)+IF(I49="●",B49*C49,0)+IF(I50="●",B50*C50,0)+IF(I51="●",B51*C51,0)+IF(I52="●",B52*C52,0)</f>
         <v/>
       </c>
       <c r="J53" s="88">
@@ -5300,19 +5601,19 @@
         <v/>
       </c>
       <c r="L53" s="130">
-        <f>SUMPRODUCT((L44:L52="●")*1,B44:B52,C44:C52)</f>
+        <f>IF(L44="●",B44*C44,0)+IF(L45="●",B45*C45,0)+IF(L46="●",B46*C46,0)+IF(L47="●",B47*C47,0)+IF(L48="●",B48*C48,0)+IF(L49="●",B49*C49,0)+IF(L50="●",B50*C50,0)+IF(L51="●",B51*C51,0)+IF(L52="●",B52*C52,0)</f>
         <v/>
       </c>
       <c r="M53" s="130">
-        <f>SUMPRODUCT((M44:M52="●")*1,B44:B52,C44:C52)</f>
+        <f>IF(M44="●",B44*C44,0)+IF(M45="●",B45*C45,0)+IF(M46="●",B46*C46,0)+IF(M47="●",B47*C47,0)+IF(M48="●",B48*C48,0)+IF(M49="●",B49*C49,0)+IF(M50="●",B50*C50,0)+IF(M51="●",B51*C51,0)+IF(M52="●",B52*C52,0)</f>
         <v/>
       </c>
       <c r="N53" s="130">
-        <f>SUMPRODUCT((N44:N52="●")*1,B44:B52,C44:C52)</f>
+        <f>IF(N44="●",B44*C44,0)+IF(N45="●",B45*C45,0)+IF(N46="●",B46*C46,0)+IF(N47="●",B47*C47,0)+IF(N48="●",B48*C48,0)+IF(N49="●",B49*C49,0)+IF(N50="●",B50*C50,0)+IF(N51="●",B51*C51,0)+IF(N52="●",B52*C52,0)</f>
         <v/>
       </c>
       <c r="O53" s="130">
-        <f>SUMPRODUCT((O44:O52="●")*1,B44:B52,C44:C52)</f>
+        <f>IF(O44="●",B44*C44,0)+IF(O45="●",B45*C45,0)+IF(O46="●",B46*C46,0)+IF(O47="●",B47*C47,0)+IF(O48="●",B48*C48,0)+IF(O49="●",B49*C49,0)+IF(O50="●",B50*C50,0)+IF(O51="●",B51*C51,0)+IF(O52="●",B52*C52,0)</f>
         <v/>
       </c>
     </row>
@@ -5322,307 +5623,324 @@
           <t>🏆 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B56" s="150" t="n"/>
-      <c r="C56" s="150" t="n"/>
-      <c r="D56" s="150" t="n"/>
-      <c r="E56" s="150" t="n"/>
-      <c r="F56" s="150" t="n"/>
-      <c r="G56" s="150" t="n"/>
-      <c r="H56" s="150" t="n"/>
-      <c r="I56" s="150" t="n"/>
-      <c r="J56" s="150" t="n"/>
-      <c r="K56" s="92" t="n"/>
+      <c r="B56" s="104" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="108" t="inlineStr">
+      <c r="C57" s="104" t="n"/>
+    </row>
+    <row r="58">
+      <c r="D58" s="104" t="n"/>
+    </row>
+    <row r="59">
+      <c r="E59" s="104" t="n"/>
+    </row>
+    <row r="60">
+      <c r="F60" s="104" t="n"/>
+    </row>
+    <row r="61">
+      <c r="G61" s="104" t="n"/>
+    </row>
+    <row r="62">
+      <c r="H62" s="104" t="n"/>
+    </row>
+    <row r="63">
+      <c r="I63" s="104" t="n"/>
+    </row>
+    <row r="64">
+      <c r="J64" s="104" t="n"/>
+    </row>
+    <row r="65">
+      <c r="K65" s="104" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="108" t="inlineStr">
         <is>
           <t>GOLF</t>
         </is>
       </c>
-      <c r="J57" s="84">
+      <c r="J66" s="84">
         <f>J15</f>
         <v/>
       </c>
-      <c r="K57" s="84">
+      <c r="K66" s="84">
         <f>K15</f>
         <v/>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="108" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="108" t="inlineStr">
         <is>
           <t>HOTEL</t>
         </is>
       </c>
-      <c r="J58" s="84">
+      <c r="J67" s="84">
         <f>J21</f>
         <v/>
       </c>
-      <c r="K58" s="84">
+      <c r="K67" s="84">
         <f>K21</f>
         <v/>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="108" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="108" t="inlineStr">
         <is>
           <t>TRANSPORT</t>
         </is>
       </c>
-      <c r="J59" s="84">
+      <c r="J68" s="84">
         <f>J27</f>
         <v/>
       </c>
-      <c r="K59" s="84">
+      <c r="K68" s="84">
         <f>K27</f>
         <v/>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="108" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="108" t="inlineStr">
         <is>
           <t xml:space="preserve"> MEALS</t>
         </is>
       </c>
-      <c r="J60" s="84">
+      <c r="J69" s="84">
         <f>J35</f>
         <v/>
       </c>
-      <c r="K60" s="84">
+      <c r="K69" s="84">
         <f>K35</f>
         <v/>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="108" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="108" t="inlineStr">
         <is>
           <t>OTHER</t>
         </is>
       </c>
-      <c r="J61" s="84">
+      <c r="J70" s="84">
         <f>J41</f>
         <v/>
       </c>
-      <c r="K61" s="84">
+      <c r="K70" s="84">
         <f>K41</f>
         <v/>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="108" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="108" t="inlineStr">
         <is>
           <t>ACTIVITIES</t>
         </is>
       </c>
-      <c r="J62" s="84">
+      <c r="J71" s="84">
         <f>J53</f>
         <v/>
       </c>
-      <c r="K62" s="84">
+      <c r="K71" s="84">
         <f>K53</f>
         <v/>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="115" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="115" t="inlineStr">
         <is>
           <t>📌 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="C63" s="106" t="inlineStr">
+      <c r="C72" s="106" t="inlineStr">
         <is>
           <t>Margin:</t>
         </is>
       </c>
-      <c r="D63" s="91">
-        <f>IF(K63&gt;0,(K63-J63)/K63,0)</f>
-        <v/>
-      </c>
-      <c r="J63" s="88">
-        <f>SUM(J57:J62)</f>
-        <v/>
-      </c>
-      <c r="K63" s="88">
-        <f>SUM(K57:K62)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="103" t="inlineStr">
+      <c r="D72" s="91">
+        <f>IF(K72&gt;0,(K72-J72)/K72,0)</f>
+        <v/>
+      </c>
+      <c r="J72" s="88">
+        <f>SUM(J66:J71)</f>
+        <v/>
+      </c>
+      <c r="K72" s="88">
+        <f>SUM(K66:K71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="103" t="inlineStr">
         <is>
           <t>👤 PER PERSON</t>
         </is>
       </c>
-      <c r="B65" s="150" t="n"/>
-      <c r="C65" s="150" t="n"/>
-      <c r="D65" s="150" t="n"/>
-      <c r="E65" s="150" t="n"/>
-      <c r="F65" s="150" t="n"/>
-      <c r="G65" s="150" t="n"/>
-      <c r="H65" s="150" t="n"/>
-      <c r="I65" s="150" t="n"/>
-      <c r="J65" s="150" t="n"/>
-      <c r="K65" s="92" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="98" t="inlineStr">
+      <c r="B74" s="104" t="n"/>
+    </row>
+    <row r="75">
+      <c r="C75" s="104" t="n"/>
+    </row>
+    <row r="76">
+      <c r="D76" s="104" t="n"/>
+    </row>
+    <row r="77">
+      <c r="E77" s="104" t="n"/>
+    </row>
+    <row r="78">
+      <c r="F78" s="104" t="n"/>
+    </row>
+    <row r="79">
+      <c r="G79" s="104" t="n"/>
+    </row>
+    <row r="80">
+      <c r="H80" s="104" t="n"/>
+    </row>
+    <row r="81">
+      <c r="I81" s="104" t="n"/>
+    </row>
+    <row r="82">
+      <c r="J82" s="104" t="n"/>
+    </row>
+    <row r="83">
+      <c r="K83" s="104" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="98" t="inlineStr">
         <is>
           <t>Person</t>
         </is>
       </c>
-      <c r="B66" s="98" t="inlineStr">
+      <c r="B84" s="98" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="C66" s="98" t="inlineStr">
+      <c r="C84" s="98" t="inlineStr">
         <is>
           <t>Sell</t>
         </is>
       </c>
-      <c r="D66" s="98" t="inlineStr">
+      <c r="D84" s="98" t="inlineStr">
         <is>
           <t>Margin</t>
         </is>
       </c>
-      <c r="E66" s="98" t="inlineStr">
+      <c r="E84" s="98" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F66" s="98" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="108">
+    </row>
+    <row r="85">
+      <c r="A85" s="108">
         <f>F2</f>
         <v/>
       </c>
-      <c r="B67" s="131">
-        <f>SUMPRODUCT((F10:F14="●")*1,B10:B14,C10:C14)+SUMPRODUCT((F18:F20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((F24:F26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((F30:F34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((F38:F40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((F44:F52="●")*1,B44:B52,C44:C52)</f>
-        <v/>
-      </c>
-      <c r="C67" s="131">
-        <f>SUMPRODUCT((F10:F14="●")*1,B10:B14,D10:D14)+SUMPRODUCT((F18:F20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((F24:F26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((F30:F34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((F38:F40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((F44:F52="●")*1,B44:B52,D44:D52)</f>
-        <v/>
-      </c>
-      <c r="D67" s="110">
-        <f>C67-B67</f>
-        <v/>
-      </c>
-      <c r="E67" s="132">
-        <f>IF(C67&gt;0,D67/C67,0)</f>
-        <v/>
-      </c>
-      <c r="F67" s="139">
-        <f>COUNTIF(F10:F14,"●")+COUNTIF(F18:F20,"●")+COUNTIF(F24:F26,"●")+COUNTIF(F30:F34,"●")+COUNTIF(F38:F40,"●")+COUNTIF(F44:F52,"●")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="108">
+      <c r="B85" s="131">
+        <f>IF(F10="●",B10*C10,0)+IF(F11="●",B11*C11,0)+IF(F12="●",B12*C12,0)+IF(F13="●",B13*C13,0)+IF(F14="●",B14*C14,0)+IF(F18="●",B18*C18,0)+IF(F19="●",B19*C19,0)+IF(F20="●",B20*C20,0)+IF(F24="●",B24*C24,0)+IF(F25="●",B25*C25,0)+IF(F26="●",B26*C26,0)+IF(F30="●",B30*C30,0)+IF(F31="●",B31*C31,0)+IF(F32="●",B32*C32,0)+IF(F33="●",B33*C33,0)+IF(F34="●",B34*C34,0)+IF(F38="●",B38*C38,0)+IF(F39="●",B39*C39,0)+IF(F40="●",B40*C40,0)+IF(F44="●",B44*C44,0)+IF(F45="●",B45*C45,0)+IF(F46="●",B46*C46,0)+IF(F47="●",B47*C47,0)+IF(F48="●",B48*C48,0)+IF(F49="●",B49*C49,0)+IF(F50="●",B50*C50,0)+IF(F51="●",B51*C51,0)+IF(F52="●",B52*C52,0)</f>
+        <v/>
+      </c>
+      <c r="C85" s="131">
+        <f>IF(F10="●",B10*D10,0)+IF(F11="●",B11*D11,0)+IF(F12="●",B12*D12,0)+IF(F13="●",B13*D13,0)+IF(F14="●",B14*D14,0)+IF(F18="●",B18*D18,0)+IF(F19="●",B19*D19,0)+IF(F20="●",B20*D20,0)+IF(F24="●",B24*D24,0)+IF(F25="●",B25*D25,0)+IF(F26="●",B26*D26,0)+IF(F30="●",B30*D30,0)+IF(F31="●",B31*D31,0)+IF(F32="●",B32*D32,0)+IF(F33="●",B33*D33,0)+IF(F34="●",B34*D34,0)+IF(F38="●",B38*D38,0)+IF(F39="●",B39*D39,0)+IF(F40="●",B40*D40,0)+IF(F44="●",B44*D44,0)+IF(F45="●",B45*D45,0)+IF(F46="●",B46*D46,0)+IF(F47="●",B47*D47,0)+IF(F48="●",B48*D48,0)+IF(F49="●",B49*D49,0)+IF(F50="●",B50*D50,0)+IF(F51="●",B51*D51,0)+IF(F52="●",B52*D52,0)</f>
+        <v/>
+      </c>
+      <c r="D85" s="110">
+        <f>C85-B85</f>
+        <v/>
+      </c>
+      <c r="E85" s="132">
+        <f>IF(C85&gt;0,D85/C85,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="108">
         <f>G2</f>
         <v/>
       </c>
-      <c r="B68" s="131">
-        <f>SUMPRODUCT((G10:G14="●")*1,B10:B14,C10:C14)+SUMPRODUCT((G18:G20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((G24:G26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((G30:G34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((G38:G40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((G44:G52="●")*1,B44:B52,C44:C52)</f>
-        <v/>
-      </c>
-      <c r="C68" s="131">
-        <f>SUMPRODUCT((G10:G14="●")*1,B10:B14,D10:D14)+SUMPRODUCT((G18:G20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((G24:G26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((G30:G34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((G38:G40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((G44:G52="●")*1,B44:B52,D44:D52)</f>
-        <v/>
-      </c>
-      <c r="D68" s="110">
-        <f>C68-B68</f>
-        <v/>
-      </c>
-      <c r="E68" s="132">
-        <f>IF(C68&gt;0,D68/C68,0)</f>
-        <v/>
-      </c>
-      <c r="F68" s="139">
-        <f>COUNTIF(G10:G14,"●")+COUNTIF(G18:G20,"●")+COUNTIF(G24:G26,"●")+COUNTIF(G30:G34,"●")+COUNTIF(G38:G40,"●")+COUNTIF(G44:G52,"●")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="108">
+      <c r="B86" s="131">
+        <f>IF(G10="●",B10*C10,0)+IF(G11="●",B11*C11,0)+IF(G12="●",B12*C12,0)+IF(G13="●",B13*C13,0)+IF(G14="●",B14*C14,0)+IF(G18="●",B18*C18,0)+IF(G19="●",B19*C19,0)+IF(G20="●",B20*C20,0)+IF(G24="●",B24*C24,0)+IF(G25="●",B25*C25,0)+IF(G26="●",B26*C26,0)+IF(G30="●",B30*C30,0)+IF(G31="●",B31*C31,0)+IF(G32="●",B32*C32,0)+IF(G33="●",B33*C33,0)+IF(G34="●",B34*C34,0)+IF(G38="●",B38*C38,0)+IF(G39="●",B39*C39,0)+IF(G40="●",B40*C40,0)+IF(G44="●",B44*C44,0)+IF(G45="●",B45*C45,0)+IF(G46="●",B46*C46,0)+IF(G47="●",B47*C47,0)+IF(G48="●",B48*C48,0)+IF(G49="●",B49*C49,0)+IF(G50="●",B50*C50,0)+IF(G51="●",B51*C51,0)+IF(G52="●",B52*C52,0)</f>
+        <v/>
+      </c>
+      <c r="C86" s="131">
+        <f>IF(G10="●",B10*D10,0)+IF(G11="●",B11*D11,0)+IF(G12="●",B12*D12,0)+IF(G13="●",B13*D13,0)+IF(G14="●",B14*D14,0)+IF(G18="●",B18*D18,0)+IF(G19="●",B19*D19,0)+IF(G20="●",B20*D20,0)+IF(G24="●",B24*D24,0)+IF(G25="●",B25*D25,0)+IF(G26="●",B26*D26,0)+IF(G30="●",B30*D30,0)+IF(G31="●",B31*D31,0)+IF(G32="●",B32*D32,0)+IF(G33="●",B33*D33,0)+IF(G34="●",B34*D34,0)+IF(G38="●",B38*D38,0)+IF(G39="●",B39*D39,0)+IF(G40="●",B40*D40,0)+IF(G44="●",B44*D44,0)+IF(G45="●",B45*D45,0)+IF(G46="●",B46*D46,0)+IF(G47="●",B47*D47,0)+IF(G48="●",B48*D48,0)+IF(G49="●",B49*D49,0)+IF(G50="●",B50*D50,0)+IF(G51="●",B51*D51,0)+IF(G52="●",B52*D52,0)</f>
+        <v/>
+      </c>
+      <c r="D86" s="110">
+        <f>C86-B86</f>
+        <v/>
+      </c>
+      <c r="E86" s="132">
+        <f>IF(C86&gt;0,D86/C86,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="108">
         <f>H2</f>
         <v/>
       </c>
-      <c r="B69" s="131">
-        <f>SUMPRODUCT((H10:H14="●")*1,B10:B14,C10:C14)+SUMPRODUCT((H18:H20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((H24:H26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((H30:H34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((H38:H40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((H44:H52="●")*1,B44:B52,C44:C52)</f>
-        <v/>
-      </c>
-      <c r="C69" s="131">
-        <f>SUMPRODUCT((H10:H14="●")*1,B10:B14,D10:D14)+SUMPRODUCT((H18:H20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((H24:H26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((H30:H34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((H38:H40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((H44:H52="●")*1,B44:B52,D44:D52)</f>
-        <v/>
-      </c>
-      <c r="D69" s="110">
-        <f>C69-B69</f>
-        <v/>
-      </c>
-      <c r="E69" s="132">
-        <f>IF(C69&gt;0,D69/C69,0)</f>
-        <v/>
-      </c>
-      <c r="F69" s="139">
-        <f>COUNTIF(H10:H14,"●")+COUNTIF(H18:H20,"●")+COUNTIF(H24:H26,"●")+COUNTIF(H30:H34,"●")+COUNTIF(H38:H40,"●")+COUNTIF(H44:H52,"●")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="108">
+      <c r="B87" s="131">
+        <f>IF(H10="●",B10*C10,0)+IF(H11="●",B11*C11,0)+IF(H12="●",B12*C12,0)+IF(H13="●",B13*C13,0)+IF(H14="●",B14*C14,0)+IF(H18="●",B18*C18,0)+IF(H19="●",B19*C19,0)+IF(H20="●",B20*C20,0)+IF(H24="●",B24*C24,0)+IF(H25="●",B25*C25,0)+IF(H26="●",B26*C26,0)+IF(H30="●",B30*C30,0)+IF(H31="●",B31*C31,0)+IF(H32="●",B32*C32,0)+IF(H33="●",B33*C33,0)+IF(H34="●",B34*C34,0)+IF(H38="●",B38*C38,0)+IF(H39="●",B39*C39,0)+IF(H40="●",B40*C40,0)+IF(H44="●",B44*C44,0)+IF(H45="●",B45*C45,0)+IF(H46="●",B46*C46,0)+IF(H47="●",B47*C47,0)+IF(H48="●",B48*C48,0)+IF(H49="●",B49*C49,0)+IF(H50="●",B50*C50,0)+IF(H51="●",B51*C51,0)+IF(H52="●",B52*C52,0)</f>
+        <v/>
+      </c>
+      <c r="C87" s="131">
+        <f>IF(H10="●",B10*D10,0)+IF(H11="●",B11*D11,0)+IF(H12="●",B12*D12,0)+IF(H13="●",B13*D13,0)+IF(H14="●",B14*D14,0)+IF(H18="●",B18*D18,0)+IF(H19="●",B19*D19,0)+IF(H20="●",B20*D20,0)+IF(H24="●",B24*D24,0)+IF(H25="●",B25*D25,0)+IF(H26="●",B26*D26,0)+IF(H30="●",B30*D30,0)+IF(H31="●",B31*D31,0)+IF(H32="●",B32*D32,0)+IF(H33="●",B33*D33,0)+IF(H34="●",B34*D34,0)+IF(H38="●",B38*D38,0)+IF(H39="●",B39*D39,0)+IF(H40="●",B40*D40,0)+IF(H44="●",B44*D44,0)+IF(H45="●",B45*D45,0)+IF(H46="●",B46*D46,0)+IF(H47="●",B47*D47,0)+IF(H48="●",B48*D48,0)+IF(H49="●",B49*D49,0)+IF(H50="●",B50*D50,0)+IF(H51="●",B51*D51,0)+IF(H52="●",B52*D52,0)</f>
+        <v/>
+      </c>
+      <c r="D87" s="110">
+        <f>C87-B87</f>
+        <v/>
+      </c>
+      <c r="E87" s="132">
+        <f>IF(C87&gt;0,D87/C87,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="108">
         <f>I2</f>
         <v/>
       </c>
-      <c r="B70" s="131">
-        <f>SUMPRODUCT((I10:I14="●")*1,B10:B14,C10:C14)+SUMPRODUCT((I18:I20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((I24:I26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((I30:I34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((I38:I40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((I44:I52="●")*1,B44:B52,C44:C52)</f>
-        <v/>
-      </c>
-      <c r="C70" s="131">
-        <f>SUMPRODUCT((I10:I14="●")*1,B10:B14,D10:D14)+SUMPRODUCT((I18:I20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((I24:I26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((I30:I34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((I38:I40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((I44:I52="●")*1,B44:B52,D44:D52)</f>
-        <v/>
-      </c>
-      <c r="D70" s="110">
-        <f>C70-B70</f>
-        <v/>
-      </c>
-      <c r="E70" s="132">
-        <f>IF(C70&gt;0,D70/C70,0)</f>
-        <v/>
-      </c>
-      <c r="F70" s="139">
-        <f>COUNTIF(I10:I14,"●")+COUNTIF(I18:I20,"●")+COUNTIF(I24:I26,"●")+COUNTIF(I30:I34,"●")+COUNTIF(I38:I40,"●")+COUNTIF(I44:I52,"●")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="115" t="inlineStr">
+      <c r="B88" s="131">
+        <f>IF(I10="●",B10*C10,0)+IF(I11="●",B11*C11,0)+IF(I12="●",B12*C12,0)+IF(I13="●",B13*C13,0)+IF(I14="●",B14*C14,0)+IF(I18="●",B18*C18,0)+IF(I19="●",B19*C19,0)+IF(I20="●",B20*C20,0)+IF(I24="●",B24*C24,0)+IF(I25="●",B25*C25,0)+IF(I26="●",B26*C26,0)+IF(I30="●",B30*C30,0)+IF(I31="●",B31*C31,0)+IF(I32="●",B32*C32,0)+IF(I33="●",B33*C33,0)+IF(I34="●",B34*C34,0)+IF(I38="●",B38*C38,0)+IF(I39="●",B39*C39,0)+IF(I40="●",B40*C40,0)+IF(I44="●",B44*C44,0)+IF(I45="●",B45*C45,0)+IF(I46="●",B46*C46,0)+IF(I47="●",B47*C47,0)+IF(I48="●",B48*C48,0)+IF(I49="●",B49*C49,0)+IF(I50="●",B50*C50,0)+IF(I51="●",B51*C51,0)+IF(I52="●",B52*C52,0)</f>
+        <v/>
+      </c>
+      <c r="C88" s="131">
+        <f>IF(I10="●",B10*D10,0)+IF(I11="●",B11*D11,0)+IF(I12="●",B12*D12,0)+IF(I13="●",B13*D13,0)+IF(I14="●",B14*D14,0)+IF(I18="●",B18*D18,0)+IF(I19="●",B19*D19,0)+IF(I20="●",B20*D20,0)+IF(I24="●",B24*D24,0)+IF(I25="●",B25*D25,0)+IF(I26="●",B26*D26,0)+IF(I30="●",B30*D30,0)+IF(I31="●",B31*D31,0)+IF(I32="●",B32*D32,0)+IF(I33="●",B33*D33,0)+IF(I34="●",B34*D34,0)+IF(I38="●",B38*D38,0)+IF(I39="●",B39*D39,0)+IF(I40="●",B40*D40,0)+IF(I44="●",B44*D44,0)+IF(I45="●",B45*D45,0)+IF(I46="●",B46*D46,0)+IF(I47="●",B47*D47,0)+IF(I48="●",B48*D48,0)+IF(I49="●",B49*D49,0)+IF(I50="●",B50*D50,0)+IF(I51="●",B51*D51,0)+IF(I52="●",B52*D52,0)</f>
+        <v/>
+      </c>
+      <c r="D88" s="110">
+        <f>C88-B88</f>
+        <v/>
+      </c>
+      <c r="E88" s="132">
+        <f>IF(C88&gt;0,D88/C88,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="115" t="inlineStr">
         <is>
           <t>📌 TOTAL</t>
         </is>
       </c>
-      <c r="B71" s="88">
-        <f>SUM(B67:B70)</f>
-        <v/>
-      </c>
-      <c r="C71" s="88">
-        <f>SUM(C67:C70)</f>
-        <v/>
-      </c>
-      <c r="D71" s="88">
-        <f>SUM(D67:D70)</f>
+      <c r="B89" s="88">
+        <f>SUM(B85:B88)</f>
+        <v/>
+      </c>
+      <c r="C89" s="88">
+        <f>SUM(C85:C88)</f>
+        <v/>
+      </c>
+      <c r="D89" s="88">
+        <f>SUM(D85:D88)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A74:K74"/>
     <mergeCell ref="A56:K56"/>
     <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A37:K37"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A23:K23"/>
     <mergeCell ref="J6:K6"/>
@@ -5630,11 +5948,9 @@
     <mergeCell ref="E4:H4"/>
     <mergeCell ref="A43:K43"/>
     <mergeCell ref="E6:H6"/>
-    <mergeCell ref="A65:K65"/>
-    <mergeCell ref="A17:K17"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A37:K37"/>
+    <mergeCell ref="A17:K17"/>
     <mergeCell ref="A9:K9"/>
   </mergeCells>
   <conditionalFormatting sqref="F10">
@@ -5657,7 +5973,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P10">
+  <conditionalFormatting sqref="Q10">
     <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5682,7 +5998,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P11">
+  <conditionalFormatting sqref="Q11">
     <cfRule type="cellIs" priority="10" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5707,7 +6023,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P12">
+  <conditionalFormatting sqref="Q12">
     <cfRule type="cellIs" priority="15" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5732,7 +6048,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P13">
+  <conditionalFormatting sqref="Q13">
     <cfRule type="cellIs" priority="20" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5757,7 +6073,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P14">
+  <conditionalFormatting sqref="Q14">
     <cfRule type="cellIs" priority="25" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5782,7 +6098,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P18">
+  <conditionalFormatting sqref="Q18">
     <cfRule type="cellIs" priority="30" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5807,7 +6123,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P19">
+  <conditionalFormatting sqref="Q19">
     <cfRule type="cellIs" priority="35" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5832,7 +6148,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P20">
+  <conditionalFormatting sqref="Q20">
     <cfRule type="cellIs" priority="40" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5857,7 +6173,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P24">
+  <conditionalFormatting sqref="Q24">
     <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5882,7 +6198,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P25">
+  <conditionalFormatting sqref="Q25">
     <cfRule type="cellIs" priority="50" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5907,7 +6223,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P26">
+  <conditionalFormatting sqref="Q26">
     <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5932,7 +6248,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P30">
+  <conditionalFormatting sqref="Q30">
     <cfRule type="cellIs" priority="60" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5957,7 +6273,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P31">
+  <conditionalFormatting sqref="Q31">
     <cfRule type="cellIs" priority="65" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5982,7 +6298,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P32">
+  <conditionalFormatting sqref="Q32">
     <cfRule type="cellIs" priority="70" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6007,7 +6323,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P33">
+  <conditionalFormatting sqref="Q33">
     <cfRule type="cellIs" priority="75" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6032,7 +6348,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P34">
+  <conditionalFormatting sqref="Q34">
     <cfRule type="cellIs" priority="80" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6057,7 +6373,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P38">
+  <conditionalFormatting sqref="Q38">
     <cfRule type="cellIs" priority="85" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6082,7 +6398,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P39">
+  <conditionalFormatting sqref="Q39">
     <cfRule type="cellIs" priority="90" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6107,7 +6423,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P40">
+  <conditionalFormatting sqref="Q40">
     <cfRule type="cellIs" priority="95" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6132,7 +6448,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P44">
+  <conditionalFormatting sqref="Q44">
     <cfRule type="cellIs" priority="100" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6157,7 +6473,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P45">
+  <conditionalFormatting sqref="Q45">
     <cfRule type="cellIs" priority="105" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6182,7 +6498,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P46">
+  <conditionalFormatting sqref="Q46">
     <cfRule type="cellIs" priority="110" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6207,7 +6523,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P47">
+  <conditionalFormatting sqref="Q47">
     <cfRule type="cellIs" priority="115" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6232,7 +6548,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P48">
+  <conditionalFormatting sqref="Q48">
     <cfRule type="cellIs" priority="120" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6257,7 +6573,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P49">
+  <conditionalFormatting sqref="Q49">
     <cfRule type="cellIs" priority="125" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6282,7 +6598,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P50">
+  <conditionalFormatting sqref="Q50">
     <cfRule type="cellIs" priority="130" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6307,7 +6623,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P51">
+  <conditionalFormatting sqref="Q51">
     <cfRule type="cellIs" priority="135" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6332,7 +6648,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P52">
+  <conditionalFormatting sqref="Q52">
     <cfRule type="cellIs" priority="140" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6355,7 +6671,7 @@
     <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>'Master Data'!$A$74:$A$77</formula1>
     </dataValidation>
-    <dataValidation sqref="F10 F11 F12 F13 F14 F18 F19 F20 F24 F25 F26 F30 F31 F32 F33 F34 F38 F39 F40 F44 F45 F46 F47 F48 F49 F50 F51 F52 G10 G11 G12 G13 G14 G18 G19 G20 G24 G25 G26 G30 G31 G32 G33 G34 G38 G39 G40 G44 G45 G46 G47 G48 G49 G50 G51 G52 H10 H11 H12 H13 H14 H18 H19 H20 H24 H25 H26 H30 H31 H32 H33 H34 H38 H39 H40 H44 H45 H46 H47 H48 H49 H50 H51 H52 I10 I11 I12 I13 I14 I18 I19 I20 I24 I25 I26 I30 I31 I32 I33 I34 I38 I39 I40 I44 I45 I46 I47 I48 I49 I50 I51 I52 L10 L11 L12 L13 L14 L18 L19 L20 L24 L25 L26 L30 L31 L32 L33 L34 L38 L39 L40 L44 L45 L46 L47 L48 L49 L50 L51 L52 M10 M11 M12 M13 M14 M18 M19 M20 M24 M25 M26 M30 M31 M32 M33 M34 M38 M39 M40 M44 M45 M46 M47 M48 M49 M50 M51 M52 N10 N11 N12 N13 N14 N18 N19 N20 N24 N25 N26 N30 N31 N32 N33 N34 N38 N39 N40 N44 N45 N46 N47 N48 N49 N50 N51 N52 O10 O11 O12 O13 O14 O18 O19 O20 O24 O25 O26 O30 O31 O32 O33 O34 O38 O39 O40 O44 O45 O46 O47 O48 O49 O50 O51 O52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Toggle" error="● = ON, blank = OFF" type="list">
+    <dataValidation sqref="F10 F11 F12 F13 F14 F18 F19 F20 F24 F25 F26 F30 F31 F32 F33 F34 F38 F39 F40 F44 F45 F46 F47 F48 F49 F50 F51 F52 G10 G11 G12 G13 G14 G18 G19 G20 G24 G25 G26 G30 G31 G32 G33 G34 G38 G39 G40 G44 G45 G46 G47 G48 G49 G50 G51 G52 H10 H11 H12 H13 H14 H18 H19 H20 H24 H25 H26 H30 H31 H32 H33 H34 H38 H39 H40 H44 H45 H46 H47 H48 H49 H50 H51 H52 I10 I11 I12 I13 I14 I18 I19 I20 I24 I25 I26 I30 I31 I32 I33 I34 I38 I39 I40 I44 I45 I46 I47 I48 I49 I50 I51 I52 L10 L11 L12 L13 L14 L18 L19 L20 L24 L25 L26 L30 L31 L32 L33 L34 L38 L39 L40 L44 L45 L46 L47 L48 L49 L50 L51 L52 M10 M11 M12 M13 M14 M18 M19 M20 M24 M25 M26 M30 M31 M32 M33 M34 M38 M39 M40 M44 M45 M46 M47 M48 M49 M50 M51 M52 N10 N11 N12 N13 N14 N18 N19 N20 N24 N25 N26 N30 N31 N32 N33 N34 N38 N39 N40 N44 N45 N46 N47 N48 N49 N50 N51 N52 O10 O11 O12 O13 O14 O18 O19 O20 O24 O25 O26 O30 O31 O32 O33 O34 O38 O39 O40 O44 O45 O46 O47 O48 O49 O50 O51 O52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="● = ON, blank = OFF" type="list">
       <formula1>"●"</formula1>
     </dataValidation>
     <dataValidation sqref="A10 A11 A12 A13 A14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -6401,14 +6717,14 @@
     <row r="1">
       <c r="A1" s="103" t="inlineStr">
         <is>
-          <t>📊 PACKAGE SUMMARY — Current Selection</t>
-        </is>
-      </c>
-      <c r="B1" s="150" t="n"/>
-      <c r="C1" s="150" t="n"/>
-      <c r="D1" s="150" t="n"/>
-      <c r="E1" s="150" t="n"/>
-      <c r="F1" s="92" t="n"/>
+          <t>📊 PACKAGE SUMMARY</t>
+        </is>
+      </c>
+      <c r="B1" s="104" t="n"/>
+      <c r="C1" s="104" t="n"/>
+      <c r="D1" s="104" t="n"/>
+      <c r="E1" s="104" t="n"/>
+      <c r="F1" s="104" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="98" t="inlineStr">
@@ -6620,14 +6936,6 @@
       </c>
       <c r="D11" s="88">
         <f>SUM(D5:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="91">
-        <f>IF(C11&gt;0,D11/C11,0)</f>
-        <v/>
-      </c>
-      <c r="F11" s="88">
-        <f>IF(E2&gt;0,B11/E2,0)</f>
         <v/>
       </c>
     </row>
@@ -6645,7 +6953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="42" min="1" max="1"/>
@@ -6657,7 +6965,7 @@
     <row r="1">
       <c r="A1" s="103" t="inlineStr">
         <is>
-          <t>🎫 GUEST PACKAGE — Client Summary</t>
+          <t>🎫 GUEST PACKAGE</t>
         </is>
       </c>
       <c r="B1" s="104" t="n"/>
@@ -6687,11 +6995,6 @@
         <f>'Package Selector'!E2</f>
         <v/>
       </c>
-      <c r="C4" s="108" t="inlineStr">
-        <is>
-          <t>persons</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="106" t="inlineStr">
@@ -6707,23 +7010,26 @@
       <c r="D5" s="87" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="124" t="inlineStr">
-        <is>
-          <t>📋 PACKAGE INCLUDES</t>
-        </is>
-      </c>
-      <c r="B7" s="125" t="n"/>
-      <c r="C7" s="125" t="n"/>
-      <c r="D7" s="125" t="n"/>
+      <c r="A7" s="140" t="inlineStr">
+        <is>
+          <t>⛳ Golf</t>
+        </is>
+      </c>
+      <c r="B7" s="108">
+        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F9:I14,"●")+COUNTIF(L9:O14,"●"))&gt;0,A9:A14,""))</f>
+        <v/>
+      </c>
+      <c r="C7" s="86" t="n"/>
+      <c r="D7" s="87" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="140" t="inlineStr">
         <is>
-          <t>⛳ Golf</t>
+          <t>🏨 Hotel</t>
         </is>
       </c>
       <c r="B8" s="108">
-        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F9:I14,"●")&gt;0),A9:A14,""))</f>
+        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F17:I21,"●")+COUNTIF(L17:O21,"●"))&gt;0,A17:A21,""))</f>
         <v/>
       </c>
       <c r="C8" s="86" t="n"/>
@@ -6732,11 +7038,11 @@
     <row r="9">
       <c r="A9" s="140" t="inlineStr">
         <is>
-          <t>🏨 Hotel</t>
+          <t>🚐 Transport</t>
         </is>
       </c>
       <c r="B9" s="108">
-        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F17:I21,"●")&gt;0),A17:A21,""))</f>
+        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F23:I27,"●")+COUNTIF(L23:O27,"●"))&gt;0,A23:A27,""))</f>
         <v/>
       </c>
       <c r="C9" s="86" t="n"/>
@@ -6745,11 +7051,11 @@
     <row r="10">
       <c r="A10" s="140" t="inlineStr">
         <is>
-          <t>🚐 Transport</t>
+          <t>🍽️ Meals</t>
         </is>
       </c>
       <c r="B10" s="108">
-        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F23:I27,"●")&gt;0),A23:A27,""))</f>
+        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F29:I35,"●")+COUNTIF(L29:O35,"●"))&gt;0,A29:A35,""))</f>
         <v/>
       </c>
       <c r="C10" s="86" t="n"/>
@@ -6758,11 +7064,11 @@
     <row r="11">
       <c r="A11" s="140" t="inlineStr">
         <is>
-          <t>🍽️ Meals</t>
+          <t>📦 Other</t>
         </is>
       </c>
       <c r="B11" s="108">
-        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F29:I35,"●")&gt;0),A29:A35,""))</f>
+        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F37:I41,"●")+COUNTIF(L37:O41,"●"))&gt;0,A37:A41,""))</f>
         <v/>
       </c>
       <c r="C11" s="86" t="n"/>
@@ -6771,96 +7077,49 @@
     <row r="12">
       <c r="A12" s="140" t="inlineStr">
         <is>
-          <t>📦 Other</t>
+          <t>🎯 Activities</t>
         </is>
       </c>
       <c r="B12" s="108">
-        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F37:I41,"●")&gt;0),A37:A41,""))</f>
+        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F43:I53,"●")+COUNTIF(L43:O53,"●"))&gt;0,A43:A53,""))</f>
         <v/>
       </c>
       <c r="C12" s="86" t="n"/>
       <c r="D12" s="87" t="n"/>
     </row>
-    <row r="13">
-      <c r="A13" s="140" t="inlineStr">
-        <is>
-          <t>🎯 Activities</t>
-        </is>
-      </c>
-      <c r="B13" s="108">
-        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F43:I53,"●")&gt;0),A43:A53,""))</f>
-        <v/>
-      </c>
-      <c r="C13" s="86" t="n"/>
-      <c r="D13" s="87" t="n"/>
+    <row r="14">
+      <c r="A14" s="124" t="inlineStr">
+        <is>
+          <t>💰 ALL-INCLUSIVE PRICE</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="104" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="124" t="inlineStr">
-        <is>
-          <t>💰 ALL-INCLUSIVE PRICE</t>
-        </is>
-      </c>
-      <c r="B16" s="125" t="n"/>
-      <c r="C16" s="125" t="n"/>
-      <c r="D16" s="125" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="106" t="inlineStr">
-        <is>
-          <t>Total Package Price:</t>
-        </is>
-      </c>
-      <c r="B17" s="153">
-        <f>'Package Selector'!K63</f>
-        <v/>
-      </c>
-      <c r="C17" s="86" t="n"/>
-      <c r="D17" s="87" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="106" t="inlineStr">
-        <is>
-          <t>Per Person:</t>
-        </is>
-      </c>
-      <c r="B18" s="154">
-        <f>IF(B4&gt;0,B11/B4,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="106" t="inlineStr">
-        <is>
-          <t>Margin:</t>
-        </is>
-      </c>
-      <c r="B19" s="155">
-        <f>B11-B14</f>
-        <v/>
-      </c>
-      <c r="C19" s="156">
-        <f>IF(B11&gt;0,B13/B11,0)</f>
-        <v/>
-      </c>
+      <c r="A15" s="106" t="inlineStr">
+        <is>
+          <t>Total:</t>
+        </is>
+      </c>
+      <c r="B15" s="153">
+        <f>'Package Selector'!K72</f>
+        <v/>
+      </c>
+      <c r="C15" s="86" t="n"/>
+      <c r="D15" s="87" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="11">
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B15:D15"/>
     <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B17:D17"/>
     <mergeCell ref="B9:D9"/>
-    <mergeCell ref="A7:D7"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A16:D16"/>
     <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: meals alphabetical order, remove 9 empty rows before Per Person
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -3730,7 +3730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R89"/>
+  <dimension ref="A1:R80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="42" min="1" max="1"/>
@@ -3758,16 +3758,16 @@
           <t>🎯 PACKAGE SELECTOR</t>
         </is>
       </c>
-      <c r="B1" s="104" t="n"/>
-      <c r="C1" s="104" t="n"/>
-      <c r="D1" s="104" t="n"/>
-      <c r="E1" s="104" t="n"/>
-      <c r="F1" s="104" t="n"/>
-      <c r="G1" s="104" t="n"/>
-      <c r="H1" s="104" t="n"/>
-      <c r="I1" s="104" t="n"/>
-      <c r="J1" s="104" t="n"/>
-      <c r="K1" s="104" t="n"/>
+      <c r="B1" s="150" t="n"/>
+      <c r="C1" s="150" t="n"/>
+      <c r="D1" s="150" t="n"/>
+      <c r="E1" s="150" t="n"/>
+      <c r="F1" s="150" t="n"/>
+      <c r="G1" s="150" t="n"/>
+      <c r="H1" s="150" t="n"/>
+      <c r="I1" s="150" t="n"/>
+      <c r="J1" s="150" t="n"/>
+      <c r="K1" s="92" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="106" t="inlineStr">
@@ -3776,6 +3776,7 @@
         </is>
       </c>
       <c r="B2" s="129" t="inlineStr"/>
+      <c r="C2" s="87" t="n"/>
       <c r="D2" s="106" t="inlineStr">
         <is>
           <t>Golfers:</t>
@@ -3811,16 +3812,16 @@
           <t>✈️ OUTBOUND</t>
         </is>
       </c>
-      <c r="B3" s="77" t="n"/>
-      <c r="C3" s="77" t="n"/>
-      <c r="D3" s="77" t="n"/>
-      <c r="E3" s="77" t="n"/>
-      <c r="F3" s="77" t="n"/>
-      <c r="G3" s="77" t="n"/>
-      <c r="H3" s="77" t="n"/>
-      <c r="I3" s="77" t="n"/>
-      <c r="J3" s="77" t="n"/>
-      <c r="K3" s="77" t="n"/>
+      <c r="B3" s="150" t="n"/>
+      <c r="C3" s="150" t="n"/>
+      <c r="D3" s="150" t="n"/>
+      <c r="E3" s="150" t="n"/>
+      <c r="F3" s="150" t="n"/>
+      <c r="G3" s="150" t="n"/>
+      <c r="H3" s="150" t="n"/>
+      <c r="I3" s="150" t="n"/>
+      <c r="J3" s="150" t="n"/>
+      <c r="K3" s="92" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="106" t="inlineStr">
@@ -3867,16 +3868,16 @@
           <t>✈️ RETURN</t>
         </is>
       </c>
-      <c r="B5" s="77" t="n"/>
-      <c r="C5" s="77" t="n"/>
-      <c r="D5" s="77" t="n"/>
-      <c r="E5" s="77" t="n"/>
-      <c r="F5" s="77" t="n"/>
-      <c r="G5" s="77" t="n"/>
-      <c r="H5" s="77" t="n"/>
-      <c r="I5" s="77" t="n"/>
-      <c r="J5" s="77" t="n"/>
-      <c r="K5" s="77" t="n"/>
+      <c r="B5" s="150" t="n"/>
+      <c r="C5" s="150" t="n"/>
+      <c r="D5" s="150" t="n"/>
+      <c r="E5" s="150" t="n"/>
+      <c r="F5" s="150" t="n"/>
+      <c r="G5" s="150" t="n"/>
+      <c r="H5" s="150" t="n"/>
+      <c r="I5" s="150" t="n"/>
+      <c r="J5" s="150" t="n"/>
+      <c r="K5" s="92" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="106" t="inlineStr">
@@ -4039,16 +4040,16 @@
           <t>⛳ GOLF</t>
         </is>
       </c>
-      <c r="B9" s="77" t="n"/>
-      <c r="C9" s="77" t="n"/>
-      <c r="D9" s="77" t="n"/>
-      <c r="E9" s="77" t="n"/>
-      <c r="F9" s="77" t="n"/>
-      <c r="G9" s="77" t="n"/>
-      <c r="H9" s="77" t="n"/>
-      <c r="I9" s="77" t="n"/>
-      <c r="J9" s="77" t="n"/>
-      <c r="K9" s="77" t="n"/>
+      <c r="B9" s="150" t="n"/>
+      <c r="C9" s="150" t="n"/>
+      <c r="D9" s="150" t="n"/>
+      <c r="E9" s="150" t="n"/>
+      <c r="F9" s="150" t="n"/>
+      <c r="G9" s="150" t="n"/>
+      <c r="H9" s="150" t="n"/>
+      <c r="I9" s="150" t="n"/>
+      <c r="J9" s="150" t="n"/>
+      <c r="K9" s="92" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="109" t="inlineStr">
@@ -4322,16 +4323,16 @@
           <t>🏨 HOTEL</t>
         </is>
       </c>
-      <c r="B17" s="77" t="n"/>
-      <c r="C17" s="77" t="n"/>
-      <c r="D17" s="77" t="n"/>
-      <c r="E17" s="77" t="n"/>
-      <c r="F17" s="77" t="n"/>
-      <c r="G17" s="77" t="n"/>
-      <c r="H17" s="77" t="n"/>
-      <c r="I17" s="77" t="n"/>
-      <c r="J17" s="77" t="n"/>
-      <c r="K17" s="77" t="n"/>
+      <c r="B17" s="150" t="n"/>
+      <c r="C17" s="150" t="n"/>
+      <c r="D17" s="150" t="n"/>
+      <c r="E17" s="150" t="n"/>
+      <c r="F17" s="150" t="n"/>
+      <c r="G17" s="150" t="n"/>
+      <c r="H17" s="150" t="n"/>
+      <c r="I17" s="150" t="n"/>
+      <c r="J17" s="150" t="n"/>
+      <c r="K17" s="92" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="109" t="inlineStr">
@@ -4511,16 +4512,16 @@
           <t>🚐 TRANSPORT</t>
         </is>
       </c>
-      <c r="B23" s="77" t="n"/>
-      <c r="C23" s="77" t="n"/>
-      <c r="D23" s="77" t="n"/>
-      <c r="E23" s="77" t="n"/>
-      <c r="F23" s="77" t="n"/>
-      <c r="G23" s="77" t="n"/>
-      <c r="H23" s="77" t="n"/>
-      <c r="I23" s="77" t="n"/>
-      <c r="J23" s="77" t="n"/>
-      <c r="K23" s="77" t="n"/>
+      <c r="B23" s="150" t="n"/>
+      <c r="C23" s="150" t="n"/>
+      <c r="D23" s="150" t="n"/>
+      <c r="E23" s="150" t="n"/>
+      <c r="F23" s="150" t="n"/>
+      <c r="G23" s="150" t="n"/>
+      <c r="H23" s="150" t="n"/>
+      <c r="I23" s="150" t="n"/>
+      <c r="J23" s="150" t="n"/>
+      <c r="K23" s="92" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="109" t="inlineStr">
@@ -4700,16 +4701,16 @@
           <t>🍽️ MEALS</t>
         </is>
       </c>
-      <c r="B29" s="77" t="n"/>
-      <c r="C29" s="77" t="n"/>
-      <c r="D29" s="77" t="n"/>
-      <c r="E29" s="77" t="n"/>
-      <c r="F29" s="77" t="n"/>
-      <c r="G29" s="77" t="n"/>
-      <c r="H29" s="77" t="n"/>
-      <c r="I29" s="77" t="n"/>
-      <c r="J29" s="77" t="n"/>
-      <c r="K29" s="77" t="n"/>
+      <c r="B29" s="150" t="n"/>
+      <c r="C29" s="150" t="n"/>
+      <c r="D29" s="150" t="n"/>
+      <c r="E29" s="150" t="n"/>
+      <c r="F29" s="150" t="n"/>
+      <c r="G29" s="150" t="n"/>
+      <c r="H29" s="150" t="n"/>
+      <c r="I29" s="150" t="n"/>
+      <c r="J29" s="150" t="n"/>
+      <c r="K29" s="92" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="109" t="inlineStr">
@@ -4761,7 +4762,7 @@
     <row r="31">
       <c r="A31" s="108" t="inlineStr">
         <is>
-          <t>Dinner (Regular)</t>
+          <t>Lunch</t>
         </is>
       </c>
       <c r="B31" s="83" t="n">
@@ -4808,11 +4809,11 @@
     <row r="32">
       <c r="A32" s="109" t="inlineStr">
         <is>
-          <t>Exclusive Dinner (Michelin/Fine)</t>
+          <t>Dinner (Regular)</t>
         </is>
       </c>
       <c r="B32" s="83" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C32" s="84">
         <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,2,FALSE))</f>
@@ -4855,11 +4856,11 @@
     <row r="33">
       <c r="A33" s="108" t="inlineStr">
         <is>
-          <t>Lunch</t>
+          <t>Exclusive Dinner (Michelin/Fine)</t>
         </is>
       </c>
       <c r="B33" s="83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C33" s="84">
         <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,2,FALSE))</f>
@@ -4993,16 +4994,16 @@
           <t>📦 OTHER</t>
         </is>
       </c>
-      <c r="B37" s="77" t="n"/>
-      <c r="C37" s="77" t="n"/>
-      <c r="D37" s="77" t="n"/>
-      <c r="E37" s="77" t="n"/>
-      <c r="F37" s="77" t="n"/>
-      <c r="G37" s="77" t="n"/>
-      <c r="H37" s="77" t="n"/>
-      <c r="I37" s="77" t="n"/>
-      <c r="J37" s="77" t="n"/>
-      <c r="K37" s="77" t="n"/>
+      <c r="B37" s="150" t="n"/>
+      <c r="C37" s="150" t="n"/>
+      <c r="D37" s="150" t="n"/>
+      <c r="E37" s="150" t="n"/>
+      <c r="F37" s="150" t="n"/>
+      <c r="G37" s="150" t="n"/>
+      <c r="H37" s="150" t="n"/>
+      <c r="I37" s="150" t="n"/>
+      <c r="J37" s="150" t="n"/>
+      <c r="K37" s="92" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="109" t="inlineStr">
@@ -5182,16 +5183,16 @@
           <t>🎯 ACTIVITIES</t>
         </is>
       </c>
-      <c r="B43" s="77" t="n"/>
-      <c r="C43" s="77" t="n"/>
-      <c r="D43" s="77" t="n"/>
-      <c r="E43" s="77" t="n"/>
-      <c r="F43" s="77" t="n"/>
-      <c r="G43" s="77" t="n"/>
-      <c r="H43" s="77" t="n"/>
-      <c r="I43" s="77" t="n"/>
-      <c r="J43" s="77" t="n"/>
-      <c r="K43" s="77" t="n"/>
+      <c r="B43" s="150" t="n"/>
+      <c r="C43" s="150" t="n"/>
+      <c r="D43" s="150" t="n"/>
+      <c r="E43" s="150" t="n"/>
+      <c r="F43" s="150" t="n"/>
+      <c r="G43" s="150" t="n"/>
+      <c r="H43" s="150" t="n"/>
+      <c r="I43" s="150" t="n"/>
+      <c r="J43" s="150" t="n"/>
+      <c r="K43" s="92" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="109" t="inlineStr">
@@ -5623,7 +5624,16 @@
           <t>🏆 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B56" s="104" t="n"/>
+      <c r="B56" s="150" t="n"/>
+      <c r="C56" s="150" t="n"/>
+      <c r="D56" s="150" t="n"/>
+      <c r="E56" s="150" t="n"/>
+      <c r="F56" s="150" t="n"/>
+      <c r="G56" s="150" t="n"/>
+      <c r="H56" s="150" t="n"/>
+      <c r="I56" s="150" t="n"/>
+      <c r="J56" s="150" t="n"/>
+      <c r="K56" s="92" t="n"/>
     </row>
     <row r="57">
       <c r="C57" s="104" t="n"/>
@@ -5772,165 +5782,147 @@
           <t>👤 PER PERSON</t>
         </is>
       </c>
-      <c r="B74" s="104" t="n"/>
+      <c r="B74" s="150" t="n"/>
+      <c r="C74" s="150" t="n"/>
+      <c r="D74" s="150" t="n"/>
+      <c r="E74" s="150" t="n"/>
+      <c r="F74" s="150" t="n"/>
+      <c r="G74" s="150" t="n"/>
+      <c r="H74" s="150" t="n"/>
+      <c r="I74" s="150" t="n"/>
+      <c r="J74" s="150" t="n"/>
+      <c r="K74" s="92" t="n"/>
     </row>
     <row r="75">
-      <c r="C75" s="104" t="n"/>
+      <c r="A75" s="98" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="B75" s="98" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C75" s="98" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="D75" s="98" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="E75" s="98" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="D76" s="104" t="n"/>
+      <c r="A76" s="108">
+        <f>F2</f>
+        <v/>
+      </c>
+      <c r="B76" s="131">
+        <f>IF(F10="●",B10*C10,0)+IF(F11="●",B11*C11,0)+IF(F12="●",B12*C12,0)+IF(F13="●",B13*C13,0)+IF(F14="●",B14*C14,0)+IF(F18="●",B18*C18,0)+IF(F19="●",B19*C19,0)+IF(F20="●",B20*C20,0)+IF(F24="●",B24*C24,0)+IF(F25="●",B25*C25,0)+IF(F26="●",B26*C26,0)+IF(F30="●",B30*C30,0)+IF(F31="●",B31*C31,0)+IF(F32="●",B32*C32,0)+IF(F33="●",B33*C33,0)+IF(F34="●",B34*C34,0)+IF(F38="●",B38*C38,0)+IF(F39="●",B39*C39,0)+IF(F40="●",B40*C40,0)+IF(F44="●",B44*C44,0)+IF(F45="●",B45*C45,0)+IF(F46="●",B46*C46,0)+IF(F47="●",B47*C47,0)+IF(F48="●",B48*C48,0)+IF(F49="●",B49*C49,0)+IF(F50="●",B50*C50,0)+IF(F51="●",B51*C51,0)+IF(F52="●",B52*C52,0)</f>
+        <v/>
+      </c>
+      <c r="C76" s="131">
+        <f>IF(F10="●",B10*D10,0)+IF(F11="●",B11*D11,0)+IF(F12="●",B12*D12,0)+IF(F13="●",B13*D13,0)+IF(F14="●",B14*D14,0)+IF(F18="●",B18*D18,0)+IF(F19="●",B19*D19,0)+IF(F20="●",B20*D20,0)+IF(F24="●",B24*D24,0)+IF(F25="●",B25*D25,0)+IF(F26="●",B26*D26,0)+IF(F30="●",B30*D30,0)+IF(F31="●",B31*D31,0)+IF(F32="●",B32*D32,0)+IF(F33="●",B33*D33,0)+IF(F34="●",B34*D34,0)+IF(F38="●",B38*D38,0)+IF(F39="●",B39*D39,0)+IF(F40="●",B40*D40,0)+IF(F44="●",B44*D44,0)+IF(F45="●",B45*D45,0)+IF(F46="●",B46*D46,0)+IF(F47="●",B47*D47,0)+IF(F48="●",B48*D48,0)+IF(F49="●",B49*D49,0)+IF(F50="●",B50*D50,0)+IF(F51="●",B51*D51,0)+IF(F52="●",B52*D52,0)</f>
+        <v/>
+      </c>
+      <c r="D76" s="110">
+        <f>C85-B85</f>
+        <v/>
+      </c>
+      <c r="E76" s="132">
+        <f>IF(C85&gt;0,D85/C85,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
-      <c r="E77" s="104" t="n"/>
+      <c r="A77" s="108">
+        <f>G2</f>
+        <v/>
+      </c>
+      <c r="B77" s="131">
+        <f>IF(G10="●",B10*C10,0)+IF(G11="●",B11*C11,0)+IF(G12="●",B12*C12,0)+IF(G13="●",B13*C13,0)+IF(G14="●",B14*C14,0)+IF(G18="●",B18*C18,0)+IF(G19="●",B19*C19,0)+IF(G20="●",B20*C20,0)+IF(G24="●",B24*C24,0)+IF(G25="●",B25*C25,0)+IF(G26="●",B26*C26,0)+IF(G30="●",B30*C30,0)+IF(G31="●",B31*C31,0)+IF(G32="●",B32*C32,0)+IF(G33="●",B33*C33,0)+IF(G34="●",B34*C34,0)+IF(G38="●",B38*C38,0)+IF(G39="●",B39*C39,0)+IF(G40="●",B40*C40,0)+IF(G44="●",B44*C44,0)+IF(G45="●",B45*C45,0)+IF(G46="●",B46*C46,0)+IF(G47="●",B47*C47,0)+IF(G48="●",B48*C48,0)+IF(G49="●",B49*C49,0)+IF(G50="●",B50*C50,0)+IF(G51="●",B51*C51,0)+IF(G52="●",B52*C52,0)</f>
+        <v/>
+      </c>
+      <c r="C77" s="131">
+        <f>IF(G10="●",B10*D10,0)+IF(G11="●",B11*D11,0)+IF(G12="●",B12*D12,0)+IF(G13="●",B13*D13,0)+IF(G14="●",B14*D14,0)+IF(G18="●",B18*D18,0)+IF(G19="●",B19*D19,0)+IF(G20="●",B20*D20,0)+IF(G24="●",B24*D24,0)+IF(G25="●",B25*D25,0)+IF(G26="●",B26*D26,0)+IF(G30="●",B30*D30,0)+IF(G31="●",B31*D31,0)+IF(G32="●",B32*D32,0)+IF(G33="●",B33*D33,0)+IF(G34="●",B34*D34,0)+IF(G38="●",B38*D38,0)+IF(G39="●",B39*D39,0)+IF(G40="●",B40*D40,0)+IF(G44="●",B44*D44,0)+IF(G45="●",B45*D45,0)+IF(G46="●",B46*D46,0)+IF(G47="●",B47*D47,0)+IF(G48="●",B48*D48,0)+IF(G49="●",B49*D49,0)+IF(G50="●",B50*D50,0)+IF(G51="●",B51*D51,0)+IF(G52="●",B52*D52,0)</f>
+        <v/>
+      </c>
+      <c r="D77" s="110">
+        <f>C86-B86</f>
+        <v/>
+      </c>
+      <c r="E77" s="132">
+        <f>IF(C86&gt;0,D86/C86,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
-      <c r="F78" s="104" t="n"/>
+      <c r="A78" s="108">
+        <f>H2</f>
+        <v/>
+      </c>
+      <c r="B78" s="131">
+        <f>IF(H10="●",B10*C10,0)+IF(H11="●",B11*C11,0)+IF(H12="●",B12*C12,0)+IF(H13="●",B13*C13,0)+IF(H14="●",B14*C14,0)+IF(H18="●",B18*C18,0)+IF(H19="●",B19*C19,0)+IF(H20="●",B20*C20,0)+IF(H24="●",B24*C24,0)+IF(H25="●",B25*C25,0)+IF(H26="●",B26*C26,0)+IF(H30="●",B30*C30,0)+IF(H31="●",B31*C31,0)+IF(H32="●",B32*C32,0)+IF(H33="●",B33*C33,0)+IF(H34="●",B34*C34,0)+IF(H38="●",B38*C38,0)+IF(H39="●",B39*C39,0)+IF(H40="●",B40*C40,0)+IF(H44="●",B44*C44,0)+IF(H45="●",B45*C45,0)+IF(H46="●",B46*C46,0)+IF(H47="●",B47*C47,0)+IF(H48="●",B48*C48,0)+IF(H49="●",B49*C49,0)+IF(H50="●",B50*C50,0)+IF(H51="●",B51*C51,0)+IF(H52="●",B52*C52,0)</f>
+        <v/>
+      </c>
+      <c r="C78" s="131">
+        <f>IF(H10="●",B10*D10,0)+IF(H11="●",B11*D11,0)+IF(H12="●",B12*D12,0)+IF(H13="●",B13*D13,0)+IF(H14="●",B14*D14,0)+IF(H18="●",B18*D18,0)+IF(H19="●",B19*D19,0)+IF(H20="●",B20*D20,0)+IF(H24="●",B24*D24,0)+IF(H25="●",B25*D25,0)+IF(H26="●",B26*D26,0)+IF(H30="●",B30*D30,0)+IF(H31="●",B31*D31,0)+IF(H32="●",B32*D32,0)+IF(H33="●",B33*D33,0)+IF(H34="●",B34*D34,0)+IF(H38="●",B38*D38,0)+IF(H39="●",B39*D39,0)+IF(H40="●",B40*D40,0)+IF(H44="●",B44*D44,0)+IF(H45="●",B45*D45,0)+IF(H46="●",B46*D46,0)+IF(H47="●",B47*D47,0)+IF(H48="●",B48*D48,0)+IF(H49="●",B49*D49,0)+IF(H50="●",B50*D50,0)+IF(H51="●",B51*D51,0)+IF(H52="●",B52*D52,0)</f>
+        <v/>
+      </c>
+      <c r="D78" s="110">
+        <f>C87-B87</f>
+        <v/>
+      </c>
+      <c r="E78" s="132">
+        <f>IF(C87&gt;0,D87/C87,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
-      <c r="G79" s="104" t="n"/>
+      <c r="A79" s="108">
+        <f>I2</f>
+        <v/>
+      </c>
+      <c r="B79" s="131">
+        <f>IF(I10="●",B10*C10,0)+IF(I11="●",B11*C11,0)+IF(I12="●",B12*C12,0)+IF(I13="●",B13*C13,0)+IF(I14="●",B14*C14,0)+IF(I18="●",B18*C18,0)+IF(I19="●",B19*C19,0)+IF(I20="●",B20*C20,0)+IF(I24="●",B24*C24,0)+IF(I25="●",B25*C25,0)+IF(I26="●",B26*C26,0)+IF(I30="●",B30*C30,0)+IF(I31="●",B31*C31,0)+IF(I32="●",B32*C32,0)+IF(I33="●",B33*C33,0)+IF(I34="●",B34*C34,0)+IF(I38="●",B38*C38,0)+IF(I39="●",B39*C39,0)+IF(I40="●",B40*C40,0)+IF(I44="●",B44*C44,0)+IF(I45="●",B45*C45,0)+IF(I46="●",B46*C46,0)+IF(I47="●",B47*C47,0)+IF(I48="●",B48*C48,0)+IF(I49="●",B49*C49,0)+IF(I50="●",B50*C50,0)+IF(I51="●",B51*C51,0)+IF(I52="●",B52*C52,0)</f>
+        <v/>
+      </c>
+      <c r="C79" s="131">
+        <f>IF(I10="●",B10*D10,0)+IF(I11="●",B11*D11,0)+IF(I12="●",B12*D12,0)+IF(I13="●",B13*D13,0)+IF(I14="●",B14*D14,0)+IF(I18="●",B18*D18,0)+IF(I19="●",B19*D19,0)+IF(I20="●",B20*D20,0)+IF(I24="●",B24*D24,0)+IF(I25="●",B25*D25,0)+IF(I26="●",B26*D26,0)+IF(I30="●",B30*D30,0)+IF(I31="●",B31*D31,0)+IF(I32="●",B32*D32,0)+IF(I33="●",B33*D33,0)+IF(I34="●",B34*D34,0)+IF(I38="●",B38*D38,0)+IF(I39="●",B39*D39,0)+IF(I40="●",B40*D40,0)+IF(I44="●",B44*D44,0)+IF(I45="●",B45*D45,0)+IF(I46="●",B46*D46,0)+IF(I47="●",B47*D47,0)+IF(I48="●",B48*D48,0)+IF(I49="●",B49*D49,0)+IF(I50="●",B50*D50,0)+IF(I51="●",B51*D51,0)+IF(I52="●",B52*D52,0)</f>
+        <v/>
+      </c>
+      <c r="D79" s="110">
+        <f>C88-B88</f>
+        <v/>
+      </c>
+      <c r="E79" s="132">
+        <f>IF(C88&gt;0,D88/C88,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
-      <c r="H80" s="104" t="n"/>
-    </row>
-    <row r="81">
-      <c r="I81" s="104" t="n"/>
-    </row>
-    <row r="82">
-      <c r="J82" s="104" t="n"/>
-    </row>
-    <row r="83">
-      <c r="K83" s="104" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="98" t="inlineStr">
-        <is>
-          <t>Person</t>
-        </is>
-      </c>
-      <c r="B84" s="98" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="C84" s="98" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="D84" s="98" t="inlineStr">
-        <is>
-          <t>Margin</t>
-        </is>
-      </c>
-      <c r="E84" s="98" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="108">
-        <f>F2</f>
-        <v/>
-      </c>
-      <c r="B85" s="131">
-        <f>IF(F10="●",B10*C10,0)+IF(F11="●",B11*C11,0)+IF(F12="●",B12*C12,0)+IF(F13="●",B13*C13,0)+IF(F14="●",B14*C14,0)+IF(F18="●",B18*C18,0)+IF(F19="●",B19*C19,0)+IF(F20="●",B20*C20,0)+IF(F24="●",B24*C24,0)+IF(F25="●",B25*C25,0)+IF(F26="●",B26*C26,0)+IF(F30="●",B30*C30,0)+IF(F31="●",B31*C31,0)+IF(F32="●",B32*C32,0)+IF(F33="●",B33*C33,0)+IF(F34="●",B34*C34,0)+IF(F38="●",B38*C38,0)+IF(F39="●",B39*C39,0)+IF(F40="●",B40*C40,0)+IF(F44="●",B44*C44,0)+IF(F45="●",B45*C45,0)+IF(F46="●",B46*C46,0)+IF(F47="●",B47*C47,0)+IF(F48="●",B48*C48,0)+IF(F49="●",B49*C49,0)+IF(F50="●",B50*C50,0)+IF(F51="●",B51*C51,0)+IF(F52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="C85" s="131">
-        <f>IF(F10="●",B10*D10,0)+IF(F11="●",B11*D11,0)+IF(F12="●",B12*D12,0)+IF(F13="●",B13*D13,0)+IF(F14="●",B14*D14,0)+IF(F18="●",B18*D18,0)+IF(F19="●",B19*D19,0)+IF(F20="●",B20*D20,0)+IF(F24="●",B24*D24,0)+IF(F25="●",B25*D25,0)+IF(F26="●",B26*D26,0)+IF(F30="●",B30*D30,0)+IF(F31="●",B31*D31,0)+IF(F32="●",B32*D32,0)+IF(F33="●",B33*D33,0)+IF(F34="●",B34*D34,0)+IF(F38="●",B38*D38,0)+IF(F39="●",B39*D39,0)+IF(F40="●",B40*D40,0)+IF(F44="●",B44*D44,0)+IF(F45="●",B45*D45,0)+IF(F46="●",B46*D46,0)+IF(F47="●",B47*D47,0)+IF(F48="●",B48*D48,0)+IF(F49="●",B49*D49,0)+IF(F50="●",B50*D50,0)+IF(F51="●",B51*D51,0)+IF(F52="●",B52*D52,0)</f>
-        <v/>
-      </c>
-      <c r="D85" s="110">
-        <f>C85-B85</f>
-        <v/>
-      </c>
-      <c r="E85" s="132">
-        <f>IF(C85&gt;0,D85/C85,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="108">
-        <f>G2</f>
-        <v/>
-      </c>
-      <c r="B86" s="131">
-        <f>IF(G10="●",B10*C10,0)+IF(G11="●",B11*C11,0)+IF(G12="●",B12*C12,0)+IF(G13="●",B13*C13,0)+IF(G14="●",B14*C14,0)+IF(G18="●",B18*C18,0)+IF(G19="●",B19*C19,0)+IF(G20="●",B20*C20,0)+IF(G24="●",B24*C24,0)+IF(G25="●",B25*C25,0)+IF(G26="●",B26*C26,0)+IF(G30="●",B30*C30,0)+IF(G31="●",B31*C31,0)+IF(G32="●",B32*C32,0)+IF(G33="●",B33*C33,0)+IF(G34="●",B34*C34,0)+IF(G38="●",B38*C38,0)+IF(G39="●",B39*C39,0)+IF(G40="●",B40*C40,0)+IF(G44="●",B44*C44,0)+IF(G45="●",B45*C45,0)+IF(G46="●",B46*C46,0)+IF(G47="●",B47*C47,0)+IF(G48="●",B48*C48,0)+IF(G49="●",B49*C49,0)+IF(G50="●",B50*C50,0)+IF(G51="●",B51*C51,0)+IF(G52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="C86" s="131">
-        <f>IF(G10="●",B10*D10,0)+IF(G11="●",B11*D11,0)+IF(G12="●",B12*D12,0)+IF(G13="●",B13*D13,0)+IF(G14="●",B14*D14,0)+IF(G18="●",B18*D18,0)+IF(G19="●",B19*D19,0)+IF(G20="●",B20*D20,0)+IF(G24="●",B24*D24,0)+IF(G25="●",B25*D25,0)+IF(G26="●",B26*D26,0)+IF(G30="●",B30*D30,0)+IF(G31="●",B31*D31,0)+IF(G32="●",B32*D32,0)+IF(G33="●",B33*D33,0)+IF(G34="●",B34*D34,0)+IF(G38="●",B38*D38,0)+IF(G39="●",B39*D39,0)+IF(G40="●",B40*D40,0)+IF(G44="●",B44*D44,0)+IF(G45="●",B45*D45,0)+IF(G46="●",B46*D46,0)+IF(G47="●",B47*D47,0)+IF(G48="●",B48*D48,0)+IF(G49="●",B49*D49,0)+IF(G50="●",B50*D50,0)+IF(G51="●",B51*D51,0)+IF(G52="●",B52*D52,0)</f>
-        <v/>
-      </c>
-      <c r="D86" s="110">
-        <f>C86-B86</f>
-        <v/>
-      </c>
-      <c r="E86" s="132">
-        <f>IF(C86&gt;0,D86/C86,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="108">
-        <f>H2</f>
-        <v/>
-      </c>
-      <c r="B87" s="131">
-        <f>IF(H10="●",B10*C10,0)+IF(H11="●",B11*C11,0)+IF(H12="●",B12*C12,0)+IF(H13="●",B13*C13,0)+IF(H14="●",B14*C14,0)+IF(H18="●",B18*C18,0)+IF(H19="●",B19*C19,0)+IF(H20="●",B20*C20,0)+IF(H24="●",B24*C24,0)+IF(H25="●",B25*C25,0)+IF(H26="●",B26*C26,0)+IF(H30="●",B30*C30,0)+IF(H31="●",B31*C31,0)+IF(H32="●",B32*C32,0)+IF(H33="●",B33*C33,0)+IF(H34="●",B34*C34,0)+IF(H38="●",B38*C38,0)+IF(H39="●",B39*C39,0)+IF(H40="●",B40*C40,0)+IF(H44="●",B44*C44,0)+IF(H45="●",B45*C45,0)+IF(H46="●",B46*C46,0)+IF(H47="●",B47*C47,0)+IF(H48="●",B48*C48,0)+IF(H49="●",B49*C49,0)+IF(H50="●",B50*C50,0)+IF(H51="●",B51*C51,0)+IF(H52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="C87" s="131">
-        <f>IF(H10="●",B10*D10,0)+IF(H11="●",B11*D11,0)+IF(H12="●",B12*D12,0)+IF(H13="●",B13*D13,0)+IF(H14="●",B14*D14,0)+IF(H18="●",B18*D18,0)+IF(H19="●",B19*D19,0)+IF(H20="●",B20*D20,0)+IF(H24="●",B24*D24,0)+IF(H25="●",B25*D25,0)+IF(H26="●",B26*D26,0)+IF(H30="●",B30*D30,0)+IF(H31="●",B31*D31,0)+IF(H32="●",B32*D32,0)+IF(H33="●",B33*D33,0)+IF(H34="●",B34*D34,0)+IF(H38="●",B38*D38,0)+IF(H39="●",B39*D39,0)+IF(H40="●",B40*D40,0)+IF(H44="●",B44*D44,0)+IF(H45="●",B45*D45,0)+IF(H46="●",B46*D46,0)+IF(H47="●",B47*D47,0)+IF(H48="●",B48*D48,0)+IF(H49="●",B49*D49,0)+IF(H50="●",B50*D50,0)+IF(H51="●",B51*D51,0)+IF(H52="●",B52*D52,0)</f>
-        <v/>
-      </c>
-      <c r="D87" s="110">
-        <f>C87-B87</f>
-        <v/>
-      </c>
-      <c r="E87" s="132">
-        <f>IF(C87&gt;0,D87/C87,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="108">
-        <f>I2</f>
-        <v/>
-      </c>
-      <c r="B88" s="131">
-        <f>IF(I10="●",B10*C10,0)+IF(I11="●",B11*C11,0)+IF(I12="●",B12*C12,0)+IF(I13="●",B13*C13,0)+IF(I14="●",B14*C14,0)+IF(I18="●",B18*C18,0)+IF(I19="●",B19*C19,0)+IF(I20="●",B20*C20,0)+IF(I24="●",B24*C24,0)+IF(I25="●",B25*C25,0)+IF(I26="●",B26*C26,0)+IF(I30="●",B30*C30,0)+IF(I31="●",B31*C31,0)+IF(I32="●",B32*C32,0)+IF(I33="●",B33*C33,0)+IF(I34="●",B34*C34,0)+IF(I38="●",B38*C38,0)+IF(I39="●",B39*C39,0)+IF(I40="●",B40*C40,0)+IF(I44="●",B44*C44,0)+IF(I45="●",B45*C45,0)+IF(I46="●",B46*C46,0)+IF(I47="●",B47*C47,0)+IF(I48="●",B48*C48,0)+IF(I49="●",B49*C49,0)+IF(I50="●",B50*C50,0)+IF(I51="●",B51*C51,0)+IF(I52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="C88" s="131">
-        <f>IF(I10="●",B10*D10,0)+IF(I11="●",B11*D11,0)+IF(I12="●",B12*D12,0)+IF(I13="●",B13*D13,0)+IF(I14="●",B14*D14,0)+IF(I18="●",B18*D18,0)+IF(I19="●",B19*D19,0)+IF(I20="●",B20*D20,0)+IF(I24="●",B24*D24,0)+IF(I25="●",B25*D25,0)+IF(I26="●",B26*D26,0)+IF(I30="●",B30*D30,0)+IF(I31="●",B31*D31,0)+IF(I32="●",B32*D32,0)+IF(I33="●",B33*D33,0)+IF(I34="●",B34*D34,0)+IF(I38="●",B38*D38,0)+IF(I39="●",B39*D39,0)+IF(I40="●",B40*D40,0)+IF(I44="●",B44*D44,0)+IF(I45="●",B45*D45,0)+IF(I46="●",B46*D46,0)+IF(I47="●",B47*D47,0)+IF(I48="●",B48*D48,0)+IF(I49="●",B49*D49,0)+IF(I50="●",B50*D50,0)+IF(I51="●",B51*D51,0)+IF(I52="●",B52*D52,0)</f>
-        <v/>
-      </c>
-      <c r="D88" s="110">
-        <f>C88-B88</f>
-        <v/>
-      </c>
-      <c r="E88" s="132">
-        <f>IF(C88&gt;0,D88/C88,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="115" t="inlineStr">
+      <c r="A80" s="115" t="inlineStr">
         <is>
           <t>📌 TOTAL</t>
         </is>
       </c>
-      <c r="B89" s="88">
+      <c r="B80" s="88">
         <f>SUM(B85:B88)</f>
         <v/>
       </c>
-      <c r="C89" s="88">
+      <c r="C80" s="88">
         <f>SUM(C85:C88)</f>
         <v/>
       </c>
-      <c r="D89" s="88">
+      <c r="D80" s="88">
         <f>SUM(D85:D88)</f>
         <v/>
       </c>
@@ -5942,15 +5934,15 @@
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="A37:K37"/>
     <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A23:K23"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="A29:K29"/>
     <mergeCell ref="E4:H4"/>
     <mergeCell ref="A43:K43"/>
     <mergeCell ref="E6:H6"/>
+    <mergeCell ref="A17:K17"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A23:K23"/>
     <mergeCell ref="A9:K9"/>
   </mergeCells>
   <conditionalFormatting sqref="F10">
@@ -6720,11 +6712,11 @@
           <t>📊 PACKAGE SUMMARY</t>
         </is>
       </c>
-      <c r="B1" s="104" t="n"/>
-      <c r="C1" s="104" t="n"/>
-      <c r="D1" s="104" t="n"/>
-      <c r="E1" s="104" t="n"/>
-      <c r="F1" s="104" t="n"/>
+      <c r="B1" s="150" t="n"/>
+      <c r="C1" s="150" t="n"/>
+      <c r="D1" s="150" t="n"/>
+      <c r="E1" s="150" t="n"/>
+      <c r="F1" s="92" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="98" t="inlineStr">
@@ -6968,9 +6960,9 @@
           <t>🎫 GUEST PACKAGE</t>
         </is>
       </c>
-      <c r="B1" s="104" t="n"/>
-      <c r="C1" s="104" t="n"/>
-      <c r="D1" s="104" t="n"/>
+      <c r="B1" s="150" t="n"/>
+      <c r="C1" s="150" t="n"/>
+      <c r="D1" s="92" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="106" t="inlineStr">
@@ -7093,6 +7085,9 @@
           <t>💰 ALL-INCLUSIVE PRICE</t>
         </is>
       </c>
+      <c r="B14" s="150" t="n"/>
+      <c r="C14" s="150" t="n"/>
+      <c r="D14" s="92" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="106" t="inlineStr">

</xml_diff>

<commit_message>
fix: legend(PP/PG/P2), Excel Online compat(TEXTJOIN/col refs), per-group formulas, user data preserved
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
     <numFmt numFmtId="166" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -140,6 +140,18 @@
       <b val="1"/>
       <color rgb="001A3450"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A3450"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001A3450"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="22">
@@ -513,7 +525,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="160">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -931,6 +943,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1452,25 +1471,20 @@
       </c>
       <c r="D6" s="146" t="inlineStr">
         <is>
-          <t>Margin $</t>
-        </is>
-      </c>
-      <c r="E6" s="146" t="inlineStr">
-        <is>
-          <t>Margin %</t>
+          <t>Margin ($)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Replay Rate ($)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Margin %</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
-      <c r="H6" s="146" t="inlineStr">
-        <is>
-          <t>Charge</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="70" t="inlineStr">
@@ -1488,21 +1502,12 @@
         <f>IF(A7="","",C7-B7)</f>
         <v/>
       </c>
-      <c r="E7" s="137">
-        <f>IF(A7="","",IF(C7&gt;0,(C7-B7)/C7,0))</f>
-        <v/>
-      </c>
-      <c r="F7" s="6" t="n">
+      <c r="E7" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>teeitup.com | 9Stamps=1free | Replay twilight</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Per Person</t>
         </is>
       </c>
     </row>
@@ -1522,21 +1527,12 @@
         <f>IF(A8="","",C8-B8)</f>
         <v/>
       </c>
-      <c r="E8" s="137">
-        <f>IF(A8="","",IF(C8&gt;0,(C8-B8)/C8,0))</f>
-        <v/>
-      </c>
-      <c r="F8" s="6" t="n">
+      <c r="E8" s="4" t="n">
         <v>120</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>UnderPar deal | Replay FREE | Non-Resident</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Per Person</t>
         </is>
       </c>
     </row>
@@ -1556,21 +1552,12 @@
         <f>IF(A9="","",C9-B9)</f>
         <v/>
       </c>
-      <c r="E9" s="137">
-        <f>IF(A9="","",IF(C9&gt;0,(C9-B9)/C9,0))</f>
-        <v/>
-      </c>
-      <c r="F9" s="6" t="n">
+      <c r="E9" s="4" t="n">
         <v>111</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Member guest | Cart incl. | Replay ~50%</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Per Person</t>
         </is>
       </c>
     </row>
@@ -1582,10 +1569,7 @@
         <f>IF(A10="","",C10-B10)</f>
         <v/>
       </c>
-      <c r="E10" s="137">
-        <f>IF(A10="","",IF(C10&gt;0,(C10-B10)/C10,0))</f>
-        <v/>
-      </c>
+      <c r="E10" s="4" t="n"/>
       <c r="F10" s="6" t="n"/>
     </row>
     <row r="11">
@@ -1596,10 +1580,7 @@
         <f>IF(A11="","",C11-B11)</f>
         <v/>
       </c>
-      <c r="E11" s="137">
-        <f>IF(A11="","",IF(C11&gt;0,(C11-B11)/C11,0))</f>
-        <v/>
-      </c>
+      <c r="E11" s="4" t="n"/>
       <c r="F11" s="6" t="n"/>
     </row>
     <row r="12">
@@ -1610,10 +1591,7 @@
         <f>IF(A12="","",C12-B12)</f>
         <v/>
       </c>
-      <c r="E12" s="137">
-        <f>IF(A12="","",IF(C12&gt;0,(C12-B12)/C12,0))</f>
-        <v/>
-      </c>
+      <c r="E12" s="4" t="n"/>
       <c r="F12" s="6" t="n"/>
     </row>
     <row r="13">
@@ -1624,10 +1602,7 @@
         <f>IF(A13="","",C13-B13)</f>
         <v/>
       </c>
-      <c r="E13" s="137">
-        <f>IF(A13="","",IF(C13&gt;0,(C13-B13)/C13,0))</f>
-        <v/>
-      </c>
+      <c r="E13" s="4" t="n"/>
       <c r="F13" s="6" t="n"/>
     </row>
     <row r="14">
@@ -1638,10 +1613,7 @@
         <f>IF(A14="","",C14-B14)</f>
         <v/>
       </c>
-      <c r="E14" s="137">
-        <f>IF(A14="","",IF(C14&gt;0,(C14-B14)/C14,0))</f>
-        <v/>
-      </c>
+      <c r="E14" s="4" t="n"/>
       <c r="F14" s="6" t="n"/>
     </row>
     <row r="17">
@@ -1675,17 +1647,13 @@
       </c>
       <c r="D18" s="146" t="inlineStr">
         <is>
-          <t>Margin $</t>
-        </is>
-      </c>
-      <c r="E18" s="146" t="inlineStr">
-        <is>
-          <t>Margin %</t>
-        </is>
-      </c>
+          <t>Margin ($)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Margin %</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="G18" s="2" t="n"/>
@@ -1706,12 +1674,7 @@
         <f>IF(A19="","",C19-B19)</f>
         <v/>
       </c>
-      <c r="E19" s="137">
-        <f>IF(A19="","",IF(C19&gt;0,(C19-B19)/C19,0))</f>
-        <v/>
-      </c>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>$550/room ÷ 2 persons</t>
         </is>
@@ -1725,10 +1688,6 @@
         <f>IF(A20="","",C20-B20)</f>
         <v/>
       </c>
-      <c r="E20" s="137">
-        <f>IF(A20="","",IF(C20&gt;0,(C20-B20)/C20,0))</f>
-        <v/>
-      </c>
       <c r="F20" s="6" t="n"/>
     </row>
     <row r="21">
@@ -1739,10 +1698,6 @@
         <f>IF(A21="","",C21-B21)</f>
         <v/>
       </c>
-      <c r="E21" s="137">
-        <f>IF(A21="","",IF(C21&gt;0,(C21-B21)/C21,0))</f>
-        <v/>
-      </c>
       <c r="F21" s="6" t="n"/>
     </row>
     <row r="22">
@@ -1753,10 +1708,6 @@
         <f>IF(A22="","",C22-B22)</f>
         <v/>
       </c>
-      <c r="E22" s="137">
-        <f>IF(A22="","",IF(C22&gt;0,(C22-B22)/C22,0))</f>
-        <v/>
-      </c>
       <c r="F22" s="6" t="n"/>
     </row>
     <row r="23">
@@ -1767,10 +1718,6 @@
         <f>IF(A23="","",C23-B23)</f>
         <v/>
       </c>
-      <c r="E23" s="137">
-        <f>IF(A23="","",IF(C23&gt;0,(C23-B23)/C23,0))</f>
-        <v/>
-      </c>
       <c r="F23" s="6" t="n"/>
     </row>
     <row r="24">
@@ -1781,17 +1728,7 @@
         <f>IF(A24="","",C24-B24)</f>
         <v/>
       </c>
-      <c r="E24" s="137">
-        <f>IF(A24="","",IF(C24&gt;0,(C24-B24)/C24,0))</f>
-        <v/>
-      </c>
       <c r="F24" s="6" t="n"/>
-    </row>
-    <row r="25">
-      <c r="E25" s="137">
-        <f>IF(A25="","",IF(C25&gt;0,(C25-B25)/C25,0))</f>
-        <v/>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="31" t="inlineStr">
@@ -1824,25 +1761,16 @@
       </c>
       <c r="D27" s="146" t="inlineStr">
         <is>
-          <t>Margin $</t>
-        </is>
-      </c>
-      <c r="E27" s="146" t="inlineStr">
-        <is>
-          <t>Margin %</t>
-        </is>
-      </c>
+          <t>Margin ($)</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n"/>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Margin %</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="G27" s="2" t="n"/>
-      <c r="H27" s="146" t="inlineStr">
-        <is>
-          <t>Charge</t>
-        </is>
-      </c>
     </row>
     <row r="28" ht="16.5" customHeight="1" s="42">
       <c r="A28" s="70" t="inlineStr">
@@ -1860,19 +1788,9 @@
         <f>IF(A28="","",C28-B28)</f>
         <v/>
       </c>
-      <c r="E28" s="137">
-        <f>IF(A28="","",IF(C28&gt;0,(C28-B28)/C28,0))</f>
-        <v/>
-      </c>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>$500/day ÷ 4p | Driver=Guide</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Per Group</t>
         </is>
       </c>
     </row>
@@ -1892,19 +1810,9 @@
         <f>IF(A29="","",C29-B29)</f>
         <v/>
       </c>
-      <c r="E29" s="137">
-        <f>IF(A29="","",IF(C29&gt;0,(C29-B29)/C29,0))</f>
-        <v/>
-      </c>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>LAX ↔ Hotel, per person</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Per Person</t>
         </is>
       </c>
     </row>
@@ -1916,10 +1824,6 @@
         <f>IF(A30="","",C30-B30)</f>
         <v/>
       </c>
-      <c r="E30" s="137">
-        <f>IF(A30="","",IF(C30&gt;0,(C30-B30)/C30,0))</f>
-        <v/>
-      </c>
       <c r="F30" s="6" t="n"/>
     </row>
     <row r="31">
@@ -1930,10 +1834,6 @@
         <f>IF(A31="","",C31-B31)</f>
         <v/>
       </c>
-      <c r="E31" s="137">
-        <f>IF(A31="","",IF(C31&gt;0,(C31-B31)/C31,0))</f>
-        <v/>
-      </c>
       <c r="F31" s="6" t="n"/>
     </row>
     <row r="32">
@@ -1944,10 +1844,6 @@
         <f>IF(A32="","",C32-B32)</f>
         <v/>
       </c>
-      <c r="E32" s="137">
-        <f>IF(A32="","",IF(C32&gt;0,(C32-B32)/C32,0))</f>
-        <v/>
-      </c>
       <c r="F32" s="6" t="n"/>
     </row>
     <row r="33">
@@ -1958,10 +1854,6 @@
         <f>IF(A33="","",C33-B33)</f>
         <v/>
       </c>
-      <c r="E33" s="137">
-        <f>IF(A33="","",IF(C33&gt;0,(C33-B33)/C33,0))</f>
-        <v/>
-      </c>
       <c r="F33" s="6" t="n"/>
     </row>
     <row r="34">
@@ -1972,17 +1864,7 @@
         <f>IF(A34="","",C34-B34)</f>
         <v/>
       </c>
-      <c r="E34" s="137">
-        <f>IF(A34="","",IF(C34&gt;0,(C34-B34)/C34,0))</f>
-        <v/>
-      </c>
       <c r="F34" s="6" t="n"/>
-    </row>
-    <row r="35">
-      <c r="E35" s="137">
-        <f>IF(A35="","",IF(C35&gt;0,(C35-B35)/C35,0))</f>
-        <v/>
-      </c>
     </row>
     <row r="36">
       <c r="A36" s="31" t="inlineStr">
@@ -2015,17 +1897,13 @@
       </c>
       <c r="D37" s="146" t="inlineStr">
         <is>
-          <t>Margin $</t>
-        </is>
-      </c>
-      <c r="E37" s="146" t="inlineStr">
-        <is>
-          <t>Margin %</t>
-        </is>
-      </c>
+          <t>Margin ($)</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Margin %</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="G37" s="2" t="n"/>
@@ -2046,12 +1924,7 @@
         <f>IF(A38="","",C38-B38)</f>
         <v/>
       </c>
-      <c r="E38" s="137">
-        <f>IF(A38="","",IF(C38&gt;0,(C38-B38)/C38,0))</f>
-        <v/>
-      </c>
-      <c r="F38" s="6" t="n"/>
-      <c r="G38" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>Daily included</t>
         </is>
@@ -2073,12 +1946,7 @@
         <f>IF(A39="","",C39-B39)</f>
         <v/>
       </c>
-      <c r="E39" s="137">
-        <f>IF(A39="","",IF(C39&gt;0,(C39-B39)/C39,0))</f>
-        <v/>
-      </c>
-      <c r="F39" s="6" t="n"/>
-      <c r="G39" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>Daily included</t>
         </is>
@@ -2100,12 +1968,7 @@
         <f>IF(A40="","",C40-B40)</f>
         <v/>
       </c>
-      <c r="E40" s="137">
-        <f>IF(A40="","",IF(C40&gt;0,(C40-B40)/C40,0))</f>
-        <v/>
-      </c>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>Regular dinner</t>
         </is>
@@ -2127,12 +1990,7 @@
         <f>IF(A41="","",C41-B41)</f>
         <v/>
       </c>
-      <c r="E41" s="137">
-        <f>IF(A41="","",IF(C41&gt;0,(C41-B41)/C41,0))</f>
-        <v/>
-      </c>
-      <c r="F41" s="6" t="n"/>
-      <c r="G41" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>2x per trip</t>
         </is>
@@ -2146,10 +2004,6 @@
         <f>IF(A42="","",C42-B42)</f>
         <v/>
       </c>
-      <c r="E42" s="137">
-        <f>IF(A42="","",IF(C42&gt;0,(C42-B42)/C42,0))</f>
-        <v/>
-      </c>
       <c r="F42" s="6" t="n"/>
     </row>
     <row r="43">
@@ -2160,10 +2014,6 @@
         <f>IF(A43="","",C43-B43)</f>
         <v/>
       </c>
-      <c r="E43" s="137">
-        <f>IF(A43="","",IF(C43&gt;0,(C43-B43)/C43,0))</f>
-        <v/>
-      </c>
       <c r="F43" s="6" t="n"/>
     </row>
     <row r="44">
@@ -2174,10 +2024,6 @@
         <f>IF(A44="","",C44-B44)</f>
         <v/>
       </c>
-      <c r="E44" s="137">
-        <f>IF(A44="","",IF(C44&gt;0,(C44-B44)/C44,0))</f>
-        <v/>
-      </c>
       <c r="F44" s="6" t="n"/>
     </row>
     <row r="45">
@@ -2188,10 +2034,6 @@
         <f>IF(A45="","",C45-B45)</f>
         <v/>
       </c>
-      <c r="E45" s="137">
-        <f>IF(A45="","",IF(C45&gt;0,(C45-B45)/C45,0))</f>
-        <v/>
-      </c>
       <c r="F45" s="6" t="n"/>
     </row>
     <row r="46">
@@ -2235,17 +2077,13 @@
       </c>
       <c r="D49" s="146" t="inlineStr">
         <is>
-          <t>Margin $</t>
-        </is>
-      </c>
-      <c r="E49" s="146" t="inlineStr">
-        <is>
-          <t>Margin %</t>
-        </is>
-      </c>
+          <t>Margin ($)</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="n"/>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Margin %</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="G49" s="2" t="n"/>
@@ -2266,12 +2104,7 @@
         <f>IF(A50="","",C50-B50)</f>
         <v/>
       </c>
-      <c r="E50" s="137">
-        <f>IF(A50="","",IF(C50&gt;0,(C50-B50)/C50,0))</f>
-        <v/>
-      </c>
-      <c r="F50" s="6" t="n"/>
-      <c r="G50" t="inlineStr">
+      <c r="F50" s="6" t="inlineStr">
         <is>
           <t>Per person per day</t>
         </is>
@@ -2285,10 +2118,6 @@
         <f>IF(A51="","",C51-B51)</f>
         <v/>
       </c>
-      <c r="E51" s="137">
-        <f>IF(A51="","",IF(C51&gt;0,(C51-B51)/C51,0))</f>
-        <v/>
-      </c>
       <c r="F51" s="6" t="n"/>
     </row>
     <row r="52">
@@ -2299,10 +2128,6 @@
         <f>IF(A52="","",C52-B52)</f>
         <v/>
       </c>
-      <c r="E52" s="137">
-        <f>IF(A52="","",IF(C52&gt;0,(C52-B52)/C52,0))</f>
-        <v/>
-      </c>
       <c r="F52" s="6" t="n"/>
     </row>
     <row r="53">
@@ -2313,10 +2138,6 @@
         <f>IF(A53="","",C53-B53)</f>
         <v/>
       </c>
-      <c r="E53" s="137">
-        <f>IF(A53="","",IF(C53&gt;0,(C53-B53)/C53,0))</f>
-        <v/>
-      </c>
       <c r="F53" s="6" t="n"/>
     </row>
     <row r="54">
@@ -2327,10 +2148,6 @@
         <f>IF(A54="","",C54-B54)</f>
         <v/>
       </c>
-      <c r="E54" s="137">
-        <f>IF(A54="","",IF(C54&gt;0,(C54-B54)/C54,0))</f>
-        <v/>
-      </c>
       <c r="F54" s="6" t="n"/>
     </row>
     <row r="55">
@@ -2341,23 +2158,7 @@
         <f>IF(A55="","",C55-B55)</f>
         <v/>
       </c>
-      <c r="E55" s="137">
-        <f>IF(A55="","",IF(C55&gt;0,(C55-B55)/C55,0))</f>
-        <v/>
-      </c>
       <c r="F55" s="6" t="n"/>
-    </row>
-    <row r="56">
-      <c r="E56" s="137">
-        <f>IF(A56="","",IF(C56&gt;0,(C56-B56)/C56,0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="E57" s="137">
-        <f>IF(A57="","",IF(C57&gt;0,(C57-B57)/C57,0))</f>
-        <v/>
-      </c>
     </row>
     <row r="58">
       <c r="A58" s="31" t="inlineStr">
@@ -2960,17 +2761,12 @@
       </c>
       <c r="D85" s="146" t="inlineStr">
         <is>
-          <t>Margin $</t>
-        </is>
-      </c>
-      <c r="E85" s="146" t="inlineStr">
-        <is>
-          <t>Margin %</t>
+          <t>Margin ($)</t>
         </is>
       </c>
       <c r="F85" s="46" t="inlineStr">
         <is>
-          <t>Margin %</t>
+          <t>Per Group?</t>
         </is>
       </c>
       <c r="G85" s="46" t="inlineStr">
@@ -2995,14 +2791,15 @@
         <f>IF(A86="","",C86-B86)</f>
         <v/>
       </c>
-      <c r="E86" s="137">
-        <f>IF(A86="","",IF(C86&gt;0,(C86-B86)/C86,0))</f>
-        <v/>
-      </c>
-      <c r="F86" s="49" t="n"/>
+      <c r="E86" s="49" t="n"/>
+      <c r="F86" s="49" t="inlineStr">
+        <is>
+          <t>1p</t>
+        </is>
+      </c>
       <c r="G86" s="49" t="inlineStr">
         <is>
-          <t>1p</t>
+          <t>2hr session; equipment incl.</t>
         </is>
       </c>
     </row>
@@ -3022,14 +2819,15 @@
         <f>IF(A87="","",C87-B87)</f>
         <v/>
       </c>
-      <c r="E87" s="137">
-        <f>IF(A87="","",IF(C87&gt;0,(C87-B87)/C87,0))</f>
-        <v/>
-      </c>
-      <c r="F87" s="49" t="n"/>
+      <c r="E87" s="49" t="n"/>
+      <c r="F87" s="49" t="inlineStr">
+        <is>
+          <t>1p</t>
+        </is>
+      </c>
       <c r="G87" s="49" t="inlineStr">
         <is>
-          <t>1p</t>
+          <t>Guided tour included</t>
         </is>
       </c>
     </row>
@@ -3049,14 +2847,15 @@
         <f>IF(A88="","",C88-B88)</f>
         <v/>
       </c>
-      <c r="E88" s="137">
-        <f>IF(A88="","",IF(C88&gt;0,(C88-B88)/C88,0))</f>
-        <v/>
-      </c>
-      <c r="F88" s="49" t="n"/>
+      <c r="E88" s="49" t="n"/>
+      <c r="F88" s="49" t="inlineStr">
+        <is>
+          <t>1p</t>
+        </is>
+      </c>
       <c r="G88" s="49" t="inlineStr">
         <is>
-          <t>1p</t>
+          <t>Seasonal; group rates available</t>
         </is>
       </c>
     </row>
@@ -3076,14 +2875,15 @@
         <f>IF(A89="","",C89-B89)</f>
         <v/>
       </c>
-      <c r="E89" s="137">
-        <f>IF(A89="","",IF(C89&gt;0,(C89-B89)/C89,0))</f>
-        <v/>
-      </c>
-      <c r="F89" s="49" t="n"/>
+      <c r="E89" s="49" t="n"/>
+      <c r="F89" s="49" t="inlineStr">
+        <is>
+          <t>1p</t>
+        </is>
+      </c>
       <c r="G89" s="49" t="inlineStr">
         <is>
-          <t>1p</t>
+          <t>Premium sports bar with food/drinks</t>
         </is>
       </c>
     </row>
@@ -3099,10 +2899,7 @@
         <f>IF(A90="","",C90-B90)</f>
         <v/>
       </c>
-      <c r="E90" s="137">
-        <f>IF(A90="","",IF(C90&gt;0,(C90-B90)/C90,0))</f>
-        <v/>
-      </c>
+      <c r="E90" s="49" t="n"/>
       <c r="F90" s="49" t="n"/>
       <c r="G90" s="49" t="n"/>
     </row>
@@ -3122,10 +2919,7 @@
         <f>IF(A91="","",C91-B91)</f>
         <v/>
       </c>
-      <c r="E91" s="137">
-        <f>IF(A91="","",IF(C91&gt;0,(C91-B91)/C91,0))</f>
-        <v/>
-      </c>
+      <c r="E91" s="49" t="n"/>
       <c r="F91" s="49" t="n"/>
       <c r="G91" s="49" t="n"/>
     </row>
@@ -3145,10 +2939,7 @@
         <f>IF(A92="","",C92-B92)</f>
         <v/>
       </c>
-      <c r="E92" s="137">
-        <f>IF(A92="","",IF(C92&gt;0,(C92-B92)/C92,0))</f>
-        <v/>
-      </c>
+      <c r="E92" s="49" t="n"/>
       <c r="F92" s="49" t="n"/>
       <c r="G92" s="49" t="n"/>
     </row>
@@ -3168,10 +2959,7 @@
         <f>IF(A93="","",C93-B93)</f>
         <v/>
       </c>
-      <c r="E93" s="137">
-        <f>IF(A93="","",IF(C93&gt;0,(C93-B93)/C93,0))</f>
-        <v/>
-      </c>
+      <c r="E93" s="49" t="n"/>
       <c r="F93" s="49" t="n"/>
       <c r="G93" s="49" t="n"/>
     </row>
@@ -3730,7 +3518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R80"/>
+  <dimension ref="A1:R72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="42" min="1" max="1"/>
@@ -3748,8 +3536,7 @@
     <col hidden="1" width="8" customWidth="1" style="42" min="13" max="13"/>
     <col hidden="1" width="8" customWidth="1" style="42" min="14" max="14"/>
     <col hidden="1" width="8" customWidth="1" style="42" min="15" max="15"/>
-    <col hidden="1" width="13" customWidth="1" style="42" min="17" max="17"/>
-    <col hidden="1" width="13" customWidth="1" style="42" min="18" max="18"/>
+    <col hidden="1" width="13" customWidth="1" style="42" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3807,316 +3594,291 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="128" t="inlineStr">
+      <c r="A3" s="157" t="inlineStr">
+        <is>
+          <t>💰 CHARGE LEGEND:  PP=Per Person  |  PG=Per Group(1회청구)  |  P2=2인1실  |  P4=4인1조</t>
+        </is>
+      </c>
+      <c r="B3" s="158" t="n"/>
+      <c r="C3" s="158" t="n"/>
+      <c r="D3" s="158" t="n"/>
+      <c r="E3" s="158" t="n"/>
+      <c r="F3" s="158" t="n"/>
+      <c r="G3" s="158" t="n"/>
+      <c r="H3" s="158" t="n"/>
+      <c r="I3" s="158" t="n"/>
+      <c r="J3" s="158" t="n"/>
+      <c r="K3" s="158" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="128" t="inlineStr">
         <is>
           <t>✈️ OUTBOUND</t>
         </is>
       </c>
-      <c r="B3" s="150" t="n"/>
-      <c r="C3" s="150" t="n"/>
-      <c r="D3" s="150" t="n"/>
-      <c r="E3" s="150" t="n"/>
-      <c r="F3" s="150" t="n"/>
-      <c r="G3" s="150" t="n"/>
-      <c r="H3" s="150" t="n"/>
-      <c r="I3" s="150" t="n"/>
-      <c r="J3" s="150" t="n"/>
-      <c r="K3" s="92" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="106" t="inlineStr">
+      <c r="B4" s="150" t="n"/>
+      <c r="C4" s="150" t="n"/>
+      <c r="D4" s="150" t="n"/>
+      <c r="E4" s="150" t="n"/>
+      <c r="F4" s="150" t="n"/>
+      <c r="G4" s="150" t="n"/>
+      <c r="H4" s="150" t="n"/>
+      <c r="I4" s="150" t="n"/>
+      <c r="J4" s="150" t="n"/>
+      <c r="K4" s="92" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="106" t="inlineStr">
         <is>
           <t>Date:</t>
         </is>
       </c>
-      <c r="B4" s="82" t="inlineStr">
+      <c r="B5" s="82" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
       </c>
-      <c r="C4" s="106" t="inlineStr">
+      <c r="C5" s="106" t="inlineStr">
         <is>
           <t>Flight:</t>
         </is>
       </c>
-      <c r="D4" s="82" t="inlineStr">
+      <c r="D5" s="82" t="inlineStr">
         <is>
           <t>KE011</t>
         </is>
       </c>
-      <c r="E4" s="144">
+      <c r="E5" s="144">
         <f>IF(D4="","",VLOOKUP(D4,'Master Data'!$A$60:$D$63,3,FALSE))&amp;" → "&amp;IF(D4="","",VLOOKUP(D4,'Master Data'!$A$60:$D$63,4,FALSE))</f>
         <v/>
       </c>
-      <c r="F4" s="86" t="n"/>
-      <c r="G4" s="86" t="n"/>
-      <c r="H4" s="87" t="n"/>
-      <c r="I4" s="106" t="inlineStr">
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
+      <c r="H5" s="87" t="n"/>
+      <c r="I5" s="106" t="inlineStr">
         <is>
           <t>Seat:</t>
         </is>
       </c>
-      <c r="J4" s="82" t="inlineStr">
+      <c r="J5" s="82" t="inlineStr">
         <is>
           <t>Economy</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="128" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="128" t="inlineStr">
         <is>
           <t>✈️ RETURN</t>
         </is>
       </c>
-      <c r="B5" s="150" t="n"/>
-      <c r="C5" s="150" t="n"/>
-      <c r="D5" s="150" t="n"/>
-      <c r="E5" s="150" t="n"/>
-      <c r="F5" s="150" t="n"/>
-      <c r="G5" s="150" t="n"/>
-      <c r="H5" s="150" t="n"/>
-      <c r="I5" s="150" t="n"/>
-      <c r="J5" s="150" t="n"/>
-      <c r="K5" s="92" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="106" t="inlineStr">
-        <is>
-          <t>Date:</t>
-        </is>
-      </c>
-      <c r="B6" s="82" t="inlineStr">
-        <is>
-          <t>2026-05-30</t>
-        </is>
-      </c>
-      <c r="C6" s="106" t="inlineStr">
-        <is>
-          <t>Flight:</t>
-        </is>
-      </c>
-      <c r="D6" s="82" t="inlineStr">
-        <is>
-          <t>KE018</t>
-        </is>
-      </c>
-      <c r="E6" s="144">
-        <f>IF(D6="","",VLOOKUP(D6,'Master Data'!$A$74:$D$77,3,FALSE))&amp;" → "&amp;IF(D6="","",VLOOKUP(D6,'Master Data'!$A$74:$D$77,4,FALSE))</f>
-        <v/>
-      </c>
-      <c r="F6" s="86" t="n"/>
-      <c r="G6" s="86" t="n"/>
-      <c r="H6" s="87" t="n"/>
-      <c r="I6" s="106" t="inlineStr">
-        <is>
-          <t>Duration:</t>
-        </is>
-      </c>
-      <c r="J6" s="144">
-        <f>IF(AND(B4&lt;&gt;"",B6&lt;&gt;""),B6-B4,"")&amp;"N "&amp;IF(AND(B4&lt;&gt;"",B6&lt;&gt;""),B6-B4+1,"")&amp;"D"</f>
-        <v/>
-      </c>
-      <c r="K6" s="87" t="n"/>
+      <c r="B6" s="150" t="n"/>
+      <c r="C6" s="150" t="n"/>
+      <c r="D6" s="150" t="n"/>
+      <c r="E6" s="150" t="n"/>
+      <c r="F6" s="150" t="n"/>
+      <c r="G6" s="150" t="n"/>
+      <c r="H6" s="150" t="n"/>
+      <c r="I6" s="150" t="n"/>
+      <c r="J6" s="150" t="n"/>
+      <c r="K6" s="92" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="106" t="inlineStr">
         <is>
+          <t>Date:</t>
+        </is>
+      </c>
+      <c r="B7" s="82" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="C7" s="106" t="inlineStr">
+        <is>
+          <t>Flight:</t>
+        </is>
+      </c>
+      <c r="D7" s="82" t="inlineStr">
+        <is>
+          <t>KE018</t>
+        </is>
+      </c>
+      <c r="E7" s="144">
+        <f>IF(D6="","",VLOOKUP(D6,'Master Data'!$A$74:$D$77,3,FALSE))&amp;" → "&amp;IF(D6="","",VLOOKUP(D6,'Master Data'!$A$74:$D$77,4,FALSE))</f>
+        <v/>
+      </c>
+      <c r="F7" s="86" t="n"/>
+      <c r="G7" s="86" t="n"/>
+      <c r="H7" s="87" t="n"/>
+      <c r="I7" s="106" t="inlineStr">
+        <is>
+          <t>Duration:</t>
+        </is>
+      </c>
+      <c r="J7" s="144">
+        <f>IF(AND(B4&lt;&gt;"",B6&lt;&gt;""),B6-B4,"")&amp;"N "&amp;IF(AND(B4&lt;&gt;"",B6&lt;&gt;""),B6-B4+1,"")&amp;"D"</f>
+        <v/>
+      </c>
+      <c r="K7" s="87" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="106" t="inlineStr">
+        <is>
           <t>Status:</t>
         </is>
       </c>
-      <c r="B7" s="136">
-        <f>IF(SUM(Q:Q)&gt;0,"❌"&amp;SUM(Q:Q)&amp;"dup","✅")</f>
-        <v/>
-      </c>
-      <c r="D7" s="106" t="inlineStr">
+      <c r="B8" s="136">
+        <f>IF(SUM(R10:R72)&gt;0,"❌"&amp;SUM(R10:R72)&amp;" dup","✅")</f>
+        <v/>
+      </c>
+      <c r="D8" s="106" t="inlineStr">
         <is>
           <t>X-Check:</t>
         </is>
       </c>
-      <c r="E7" s="133">
-        <f>J72</f>
-        <v/>
-      </c>
-      <c r="F7" s="81" t="inlineStr">
+      <c r="E8" s="133">
+        <f>J64</f>
+        <v/>
+      </c>
+      <c r="F8" s="81" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="G7" s="133">
-        <f>B89</f>
-        <v/>
-      </c>
-      <c r="H7" s="81" t="inlineStr">
+      <c r="G8" s="133">
+        <f>B72</f>
+        <v/>
+      </c>
+      <c r="H8" s="81" t="inlineStr">
         <is>
           <t>=</t>
         </is>
       </c>
-      <c r="I7" s="136">
-        <f>IF(E7-G7=0,"✅MATCH","❌")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="119" t="inlineStr">
+      <c r="I8" s="136">
+        <f>IF(E8-G8=0,"✅MATCH","❌")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="119" t="inlineStr">
         <is>
           <t>Item ▼</t>
         </is>
       </c>
-      <c r="B8" s="98" t="inlineStr">
+      <c r="B9" s="98" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="C8" s="98" t="inlineStr">
+      <c r="C9" s="98" t="inlineStr">
         <is>
           <t>Cost/P</t>
         </is>
       </c>
-      <c r="D8" s="98" t="inlineStr">
+      <c r="D9" s="98" t="inlineStr">
         <is>
           <t>Sell/P</t>
         </is>
       </c>
-      <c r="E8" s="98" t="inlineStr">
+      <c r="E9" s="98" t="inlineStr">
         <is>
           <t>M%</t>
         </is>
       </c>
-      <c r="F8" s="98">
+      <c r="F9" s="98">
         <f>F2</f>
         <v/>
       </c>
-      <c r="G8" s="98">
+      <c r="G9" s="98">
         <f>G2</f>
         <v/>
       </c>
-      <c r="H8" s="98">
+      <c r="H9" s="98">
         <f>H2</f>
         <v/>
       </c>
-      <c r="I8" s="98">
+      <c r="I9" s="98">
         <f>I2</f>
         <v/>
       </c>
-      <c r="J8" s="98" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="K8" s="98" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="L8" s="98" t="inlineStr">
+      <c r="J9" s="98" t="inlineStr">
+        <is>
+          <t>TotCost</t>
+        </is>
+      </c>
+      <c r="K9" s="98" t="inlineStr">
+        <is>
+          <t>TotSell</t>
+        </is>
+      </c>
+      <c r="L9" s="98" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="M8" s="98" t="inlineStr">
+      <c r="M9" s="98" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
-      <c r="N8" s="98" t="inlineStr">
+      <c r="N9" s="98" t="inlineStr">
         <is>
           <t>P7</t>
         </is>
       </c>
-      <c r="O8" s="98" t="inlineStr">
+      <c r="O9" s="98" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
       </c>
-      <c r="Q8" s="98" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="128" t="inlineStr">
+      <c r="P9" s="98" t="inlineStr">
+        <is>
+          <t>Dup</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="128" t="inlineStr">
         <is>
           <t>⛳ GOLF</t>
         </is>
       </c>
-      <c r="B9" s="150" t="n"/>
-      <c r="C9" s="150" t="n"/>
-      <c r="D9" s="150" t="n"/>
-      <c r="E9" s="150" t="n"/>
-      <c r="F9" s="150" t="n"/>
-      <c r="G9" s="150" t="n"/>
-      <c r="H9" s="150" t="n"/>
-      <c r="I9" s="150" t="n"/>
-      <c r="J9" s="150" t="n"/>
-      <c r="K9" s="92" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="109" t="inlineStr">
+      <c r="B10" s="150" t="n"/>
+      <c r="C10" s="150" t="n"/>
+      <c r="D10" s="150" t="n"/>
+      <c r="E10" s="150" t="n"/>
+      <c r="F10" s="150" t="n"/>
+      <c r="G10" s="150" t="n"/>
+      <c r="H10" s="150" t="n"/>
+      <c r="I10" s="150" t="n"/>
+      <c r="J10" s="150" t="n"/>
+      <c r="K10" s="92" t="n"/>
+      <c r="L10" s="159" t="inlineStr">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="109" t="inlineStr">
         <is>
           <t>Hidden Valley GC</t>
         </is>
       </c>
-      <c r="B10" s="83" t="n">
+      <c r="B11" s="83" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="84">
+      <c r="C11" s="84">
         <f>IF(A10="","",VLOOKUP(A10,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D10" s="84">
+      <c r="D11" s="84">
         <f>IF(A10="","",VLOOKUP(A10,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E10" s="137">
+      <c r="E11" s="137">
         <f>IF(D10&gt;0,(D10-C10)/D10,0)</f>
-        <v/>
-      </c>
-      <c r="F10" s="145" t="inlineStr"/>
-      <c r="G10" s="145" t="inlineStr"/>
-      <c r="H10" s="145" t="inlineStr"/>
-      <c r="I10" s="145" t="inlineStr"/>
-      <c r="J10" s="84">
-        <f>IF(A10="","",(COUNTIF(F10,"●")+COUNTIF(G10,"●")+COUNTIF(H10,"●")+COUNTIF(I10,"●")+COUNTIF(L10,"●")+COUNTIF(M10,"●")+COUNTIF(N10,"●")+COUNTIF(O10,"●"))*B10*C10)</f>
-        <v/>
-      </c>
-      <c r="K10" s="84">
-        <f>IF(A10="","",(COUNTIF(F10,"●")+COUNTIF(G10,"●")+COUNTIF(H10,"●")+COUNTIF(I10,"●")+COUNTIF(L10,"●")+COUNTIF(M10,"●")+COUNTIF(N10,"●")+COUNTIF(O10,"●"))*B10*D10)</f>
-        <v/>
-      </c>
-      <c r="L10" s="145" t="inlineStr"/>
-      <c r="M10" s="145" t="inlineStr"/>
-      <c r="N10" s="145" t="inlineStr"/>
-      <c r="O10" s="145" t="inlineStr"/>
-      <c r="Q10" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="R10" s="81" t="inlineStr">
-        <is>
-          <t>pp</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="108" t="inlineStr">
-        <is>
-          <t>Sandpiper GC</t>
-        </is>
-      </c>
-      <c r="B11" s="83" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" s="84">
-        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D11" s="84">
-        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E11" s="137">
-        <f>IF(D11&gt;0,(D11-C11)/D11,0)</f>
         <v/>
       </c>
       <c r="F11" s="145" t="inlineStr"/>
@@ -4124,46 +3886,41 @@
       <c r="H11" s="145" t="inlineStr"/>
       <c r="I11" s="145" t="inlineStr"/>
       <c r="J11" s="84">
-        <f>IF(A11="","",(COUNTIF(F11,"●")+COUNTIF(G11,"●")+COUNTIF(H11,"●")+COUNTIF(I11,"●")+COUNTIF(L11,"●")+COUNTIF(M11,"●")+COUNTIF(N11,"●")+COUNTIF(O11,"●"))*B11*C11)</f>
+        <f>IF(A10="","",(COUNTIF(F10,"●")+COUNTIF(G10,"●")+COUNTIF(H10,"●")+COUNTIF(I10,"●")+COUNTIF(L10,"●")+COUNTIF(M10,"●")+COUNTIF(N10,"●")+COUNTIF(O10,"●"))*B10*C10)</f>
         <v/>
       </c>
       <c r="K11" s="84">
-        <f>IF(A11="","",(COUNTIF(F11,"●")+COUNTIF(G11,"●")+COUNTIF(H11,"●")+COUNTIF(I11,"●")+COUNTIF(L11,"●")+COUNTIF(M11,"●")+COUNTIF(N11,"●")+COUNTIF(O11,"●"))*B11*D11)</f>
+        <f>IF(A10="","",(COUNTIF(F10,"●")+COUNTIF(G10,"●")+COUNTIF(H10,"●")+COUNTIF(I10,"●")+COUNTIF(L10,"●")+COUNTIF(M10,"●")+COUNTIF(N10,"●")+COUNTIF(O10,"●"))*B10*D10)</f>
         <v/>
       </c>
       <c r="L11" s="145" t="inlineStr"/>
       <c r="M11" s="145" t="inlineStr"/>
       <c r="N11" s="145" t="inlineStr"/>
       <c r="O11" s="145" t="inlineStr"/>
-      <c r="Q11" s="81">
-        <f>IF(A11="",0,COUNTIF(A$10:A10,A11))</f>
-        <v/>
-      </c>
-      <c r="R11" s="81" t="inlineStr">
-        <is>
-          <t>pp</t>
-        </is>
+      <c r="P11" s="81">
+        <f>0</f>
+        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="109" t="inlineStr">
-        <is>
-          <t>Trump National LA</t>
+      <c r="A12" s="108" t="inlineStr">
+        <is>
+          <t>Sandpiper GC</t>
         </is>
       </c>
       <c r="B12" s="83" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="84">
-        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D12" s="84">
-        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E12" s="137">
-        <f>IF(D12&gt;0,(D12-C12)/D12,0)</f>
+        <f>IF(D11&gt;0,(D11-C11)/D11,0)</f>
         <v/>
       </c>
       <c r="F12" s="145" t="inlineStr"/>
@@ -4171,40 +3928,41 @@
       <c r="H12" s="145" t="inlineStr"/>
       <c r="I12" s="145" t="inlineStr"/>
       <c r="J12" s="84">
-        <f>IF(A12="","",(COUNTIF(F12,"●")+COUNTIF(G12,"●")+COUNTIF(H12,"●")+COUNTIF(I12,"●")+COUNTIF(L12,"●")+COUNTIF(M12,"●")+COUNTIF(N12,"●")+COUNTIF(O12,"●"))*B12*C12)</f>
+        <f>IF(A11="","",(COUNTIF(F11,"●")+COUNTIF(G11,"●")+COUNTIF(H11,"●")+COUNTIF(I11,"●")+COUNTIF(L11,"●")+COUNTIF(M11,"●")+COUNTIF(N11,"●")+COUNTIF(O11,"●"))*B11*C11)</f>
         <v/>
       </c>
       <c r="K12" s="84">
-        <f>IF(A12="","",(COUNTIF(F12,"●")+COUNTIF(G12,"●")+COUNTIF(H12,"●")+COUNTIF(I12,"●")+COUNTIF(L12,"●")+COUNTIF(M12,"●")+COUNTIF(N12,"●")+COUNTIF(O12,"●"))*B12*D12)</f>
+        <f>IF(A11="","",(COUNTIF(F11,"●")+COUNTIF(G11,"●")+COUNTIF(H11,"●")+COUNTIF(I11,"●")+COUNTIF(L11,"●")+COUNTIF(M11,"●")+COUNTIF(N11,"●")+COUNTIF(O11,"●"))*B11*D11)</f>
         <v/>
       </c>
       <c r="L12" s="145" t="inlineStr"/>
       <c r="M12" s="145" t="inlineStr"/>
       <c r="N12" s="145" t="inlineStr"/>
       <c r="O12" s="145" t="inlineStr"/>
-      <c r="Q12" s="81">
-        <f>IF(A12="",0,COUNTIF(A$10:A11,A12))</f>
-        <v/>
-      </c>
-      <c r="R12" s="81" t="inlineStr">
-        <is>
-          <t>pp</t>
-        </is>
+      <c r="P12" s="81">
+        <f>IF(A11="",0,COUNTIF(A$10:A10,A11))</f>
+        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="129" t="inlineStr"/>
-      <c r="B13" s="83" t="inlineStr"/>
+      <c r="A13" s="109" t="inlineStr">
+        <is>
+          <t>Trump National LA</t>
+        </is>
+      </c>
+      <c r="B13" s="83" t="n">
+        <v>2</v>
+      </c>
       <c r="C13" s="84">
-        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D13" s="84">
-        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E13" s="137">
-        <f>IF(D13&gt;0,(D13-C13)/D13,0)</f>
+        <f>IF(D12&gt;0,(D12-C12)/D12,0)</f>
         <v/>
       </c>
       <c r="F13" s="145" t="inlineStr"/>
@@ -4212,36 +3970,35 @@
       <c r="H13" s="145" t="inlineStr"/>
       <c r="I13" s="145" t="inlineStr"/>
       <c r="J13" s="84">
-        <f>IF(A13="","",(COUNTIF(F13,"●")+COUNTIF(G13,"●")+COUNTIF(H13,"●")+COUNTIF(I13,"●")+COUNTIF(L13,"●")+COUNTIF(M13,"●")+COUNTIF(N13,"●")+COUNTIF(O13,"●"))*B13*C13)</f>
+        <f>IF(A12="","",(COUNTIF(F12,"●")+COUNTIF(G12,"●")+COUNTIF(H12,"●")+COUNTIF(I12,"●")+COUNTIF(L12,"●")+COUNTIF(M12,"●")+COUNTIF(N12,"●")+COUNTIF(O12,"●"))*B12*C12)</f>
         <v/>
       </c>
       <c r="K13" s="84">
-        <f>IF(A13="","",(COUNTIF(F13,"●")+COUNTIF(G13,"●")+COUNTIF(H13,"●")+COUNTIF(I13,"●")+COUNTIF(L13,"●")+COUNTIF(M13,"●")+COUNTIF(N13,"●")+COUNTIF(O13,"●"))*B13*D13)</f>
+        <f>IF(A12="","",(COUNTIF(F12,"●")+COUNTIF(G12,"●")+COUNTIF(H12,"●")+COUNTIF(I12,"●")+COUNTIF(L12,"●")+COUNTIF(M12,"●")+COUNTIF(N12,"●")+COUNTIF(O12,"●"))*B12*D12)</f>
         <v/>
       </c>
       <c r="L13" s="145" t="inlineStr"/>
       <c r="M13" s="145" t="inlineStr"/>
       <c r="N13" s="145" t="inlineStr"/>
       <c r="O13" s="145" t="inlineStr"/>
-      <c r="Q13" s="81">
-        <f>IF(A13="",0,COUNTIF(A$10:A12,A13))</f>
-        <v/>
-      </c>
-      <c r="R13" s="81" t="inlineStr"/>
+      <c r="P13" s="81">
+        <f>IF(A12="",0,COUNTIF(A$10:A11,A12))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="129" t="inlineStr"/>
       <c r="B14" s="83" t="inlineStr"/>
       <c r="C14" s="84">
-        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D14" s="84">
-        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E14" s="137">
-        <f>IF(D14&gt;0,(D14-C14)/D14,0)</f>
+        <f>IF(D13&gt;0,(D13-C13)/D13,0)</f>
         <v/>
       </c>
       <c r="F14" s="145" t="inlineStr"/>
@@ -4249,151 +4006,151 @@
       <c r="H14" s="145" t="inlineStr"/>
       <c r="I14" s="145" t="inlineStr"/>
       <c r="J14" s="84">
-        <f>IF(A14="","",(COUNTIF(F14,"●")+COUNTIF(G14,"●")+COUNTIF(H14,"●")+COUNTIF(I14,"●")+COUNTIF(L14,"●")+COUNTIF(M14,"●")+COUNTIF(N14,"●")+COUNTIF(O14,"●"))*B14*C14)</f>
+        <f>IF(A13="","",(COUNTIF(F13,"●")+COUNTIF(G13,"●")+COUNTIF(H13,"●")+COUNTIF(I13,"●")+COUNTIF(L13,"●")+COUNTIF(M13,"●")+COUNTIF(N13,"●")+COUNTIF(O13,"●"))*B13*C13)</f>
         <v/>
       </c>
       <c r="K14" s="84">
-        <f>IF(A14="","",(COUNTIF(F14,"●")+COUNTIF(G14,"●")+COUNTIF(H14,"●")+COUNTIF(I14,"●")+COUNTIF(L14,"●")+COUNTIF(M14,"●")+COUNTIF(N14,"●")+COUNTIF(O14,"●"))*B14*D14)</f>
+        <f>IF(A13="","",(COUNTIF(F13,"●")+COUNTIF(G13,"●")+COUNTIF(H13,"●")+COUNTIF(I13,"●")+COUNTIF(L13,"●")+COUNTIF(M13,"●")+COUNTIF(N13,"●")+COUNTIF(O13,"●"))*B13*D13)</f>
         <v/>
       </c>
       <c r="L14" s="145" t="inlineStr"/>
       <c r="M14" s="145" t="inlineStr"/>
       <c r="N14" s="145" t="inlineStr"/>
       <c r="O14" s="145" t="inlineStr"/>
-      <c r="Q14" s="81">
+      <c r="P14" s="81">
+        <f>IF(A13="",0,COUNTIF(A$10:A12,A13))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="129" t="inlineStr"/>
+      <c r="B15" s="83" t="inlineStr"/>
+      <c r="C15" s="84">
+        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D15" s="84">
+        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E15" s="137">
+        <f>IF(D14&gt;0,(D14-C14)/D14,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="145" t="inlineStr"/>
+      <c r="G15" s="145" t="inlineStr"/>
+      <c r="H15" s="145" t="inlineStr"/>
+      <c r="I15" s="145" t="inlineStr"/>
+      <c r="J15" s="84">
+        <f>IF(A14="","",(COUNTIF(F14,"●")+COUNTIF(G14,"●")+COUNTIF(H14,"●")+COUNTIF(I14,"●")+COUNTIF(L14,"●")+COUNTIF(M14,"●")+COUNTIF(N14,"●")+COUNTIF(O14,"●"))*B14*C14)</f>
+        <v/>
+      </c>
+      <c r="K15" s="84">
+        <f>IF(A14="","",(COUNTIF(F14,"●")+COUNTIF(G14,"●")+COUNTIF(H14,"●")+COUNTIF(I14,"●")+COUNTIF(L14,"●")+COUNTIF(M14,"●")+COUNTIF(N14,"●")+COUNTIF(O14,"●"))*B14*D14)</f>
+        <v/>
+      </c>
+      <c r="L15" s="145" t="inlineStr"/>
+      <c r="M15" s="145" t="inlineStr"/>
+      <c r="N15" s="145" t="inlineStr"/>
+      <c r="O15" s="145" t="inlineStr"/>
+      <c r="P15" s="81">
         <f>IF(A14="",0,COUNTIF(A$10:A13,A14))</f>
         <v/>
       </c>
-      <c r="R14" s="81" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="123" t="inlineStr">
+    </row>
+    <row r="16">
+      <c r="A16" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B15" s="114" t="inlineStr"/>
-      <c r="C15" s="114" t="inlineStr"/>
-      <c r="D15" s="114" t="inlineStr"/>
-      <c r="E15" s="114" t="inlineStr"/>
-      <c r="F15" s="130">
-        <f>IF(F10="●",B10*C10,0)+IF(F11="●",B11*C11,0)+IF(F12="●",B12*C12,0)+IF(F13="●",B13*C13,0)+IF(F14="●",B14*C14,0)</f>
-        <v/>
-      </c>
-      <c r="G15" s="130">
-        <f>IF(G10="●",B10*C10,0)+IF(G11="●",B11*C11,0)+IF(G12="●",B12*C12,0)+IF(G13="●",B13*C13,0)+IF(G14="●",B14*C14,0)</f>
-        <v/>
-      </c>
-      <c r="H15" s="130">
-        <f>IF(H10="●",B10*C10,0)+IF(H11="●",B11*C11,0)+IF(H12="●",B12*C12,0)+IF(H13="●",B13*C13,0)+IF(H14="●",B14*C14,0)</f>
-        <v/>
-      </c>
-      <c r="I15" s="130">
-        <f>IF(I10="●",B10*C10,0)+IF(I11="●",B11*C11,0)+IF(I12="●",B12*C12,0)+IF(I13="●",B13*C13,0)+IF(I14="●",B14*C14,0)</f>
-        <v/>
-      </c>
-      <c r="J15" s="88">
+      <c r="B16" s="114" t="inlineStr"/>
+      <c r="C16" s="114" t="inlineStr"/>
+      <c r="D16" s="114" t="inlineStr"/>
+      <c r="E16" s="114" t="inlineStr"/>
+      <c r="F16" s="130">
+        <f>SUMPRODUCT((F10:F14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="G16" s="130">
+        <f>SUMPRODUCT((G10:G14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="H16" s="130">
+        <f>SUMPRODUCT((H10:H14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="I16" s="130">
+        <f>SUMPRODUCT((I10:I14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="J16" s="88">
         <f>SUM(J10:J14)</f>
         <v/>
       </c>
-      <c r="K15" s="88">
+      <c r="K16" s="88">
         <f>SUM(K10:K14)</f>
         <v/>
       </c>
-      <c r="L15" s="130">
-        <f>IF(L10="●",B10*C10,0)+IF(L11="●",B11*C11,0)+IF(L12="●",B12*C12,0)+IF(L13="●",B13*C13,0)+IF(L14="●",B14*C14,0)</f>
-        <v/>
-      </c>
-      <c r="M15" s="130">
-        <f>IF(M10="●",B10*C10,0)+IF(M11="●",B11*C11,0)+IF(M12="●",B12*C12,0)+IF(M13="●",B13*C13,0)+IF(M14="●",B14*C14,0)</f>
-        <v/>
-      </c>
-      <c r="N15" s="130">
-        <f>IF(N10="●",B10*C10,0)+IF(N11="●",B11*C11,0)+IF(N12="●",B12*C12,0)+IF(N13="●",B13*C13,0)+IF(N14="●",B14*C14,0)</f>
-        <v/>
-      </c>
-      <c r="O15" s="130">
-        <f>IF(O10="●",B10*C10,0)+IF(O11="●",B11*C11,0)+IF(O12="●",B12*C12,0)+IF(O13="●",B13*C13,0)+IF(O14="●",B14*C14,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="128" t="inlineStr">
+      <c r="L16" s="130">
+        <f>SUMPRODUCT((L10:L14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="M16" s="130">
+        <f>SUMPRODUCT((M10:M14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="N16" s="130">
+        <f>SUMPRODUCT((N10:N14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+      <c r="O16" s="130">
+        <f>SUMPRODUCT((O10:O14="●")*1,B10:B14,C10:C14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="128" t="inlineStr">
         <is>
           <t>🏨 HOTEL</t>
         </is>
       </c>
-      <c r="B17" s="150" t="n"/>
-      <c r="C17" s="150" t="n"/>
-      <c r="D17" s="150" t="n"/>
-      <c r="E17" s="150" t="n"/>
-      <c r="F17" s="150" t="n"/>
-      <c r="G17" s="150" t="n"/>
-      <c r="H17" s="150" t="n"/>
-      <c r="I17" s="150" t="n"/>
-      <c r="J17" s="150" t="n"/>
-      <c r="K17" s="92" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="109" t="inlineStr">
+      <c r="B18" s="150" t="n"/>
+      <c r="C18" s="150" t="n"/>
+      <c r="D18" s="150" t="n"/>
+      <c r="E18" s="150" t="n"/>
+      <c r="F18" s="150" t="n"/>
+      <c r="G18" s="150" t="n"/>
+      <c r="H18" s="150" t="n"/>
+      <c r="I18" s="150" t="n"/>
+      <c r="J18" s="150" t="n"/>
+      <c r="K18" s="92" t="n"/>
+      <c r="L18" s="159" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="109" t="inlineStr">
         <is>
           <t>Beverly Wilshire (5★) / Same Tier</t>
         </is>
       </c>
-      <c r="B18" s="83" t="n">
+      <c r="B19" s="83" t="n">
         <v>3</v>
       </c>
-      <c r="C18" s="84">
+      <c r="C19" s="84">
         <f>IF(A18="","",VLOOKUP(A18,'Master Data'!$A$19:$C$24,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D18" s="84">
+      <c r="D19" s="84">
         <f>IF(A18="","",VLOOKUP(A18,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E18" s="137">
+      <c r="E19" s="137">
         <f>IF(D18&gt;0,(D18-C18)/D18,0)</f>
-        <v/>
-      </c>
-      <c r="F18" s="145" t="inlineStr"/>
-      <c r="G18" s="145" t="inlineStr"/>
-      <c r="H18" s="145" t="inlineStr"/>
-      <c r="I18" s="145" t="inlineStr"/>
-      <c r="J18" s="84">
-        <f>IF(A18="","",(COUNTIF(F18,"●")+COUNTIF(G18,"●")+COUNTIF(H18,"●")+COUNTIF(I18,"●")+COUNTIF(L18,"●")+COUNTIF(M18,"●")+COUNTIF(N18,"●")+COUNTIF(O18,"●"))*B18*C18)</f>
-        <v/>
-      </c>
-      <c r="K18" s="84">
-        <f>IF(A18="","",(COUNTIF(F18,"●")+COUNTIF(G18,"●")+COUNTIF(H18,"●")+COUNTIF(I18,"●")+COUNTIF(L18,"●")+COUNTIF(M18,"●")+COUNTIF(N18,"●")+COUNTIF(O18,"●"))*B18*D18)</f>
-        <v/>
-      </c>
-      <c r="L18" s="145" t="inlineStr"/>
-      <c r="M18" s="145" t="inlineStr"/>
-      <c r="N18" s="145" t="inlineStr"/>
-      <c r="O18" s="145" t="inlineStr"/>
-      <c r="Q18" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="R18" s="81" t="inlineStr">
-        <is>
-          <t>pp</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="129" t="inlineStr"/>
-      <c r="B19" s="83" t="inlineStr"/>
-      <c r="C19" s="84">
-        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D19" s="84">
-        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E19" s="137">
-        <f>IF(D19&gt;0,(D19-C19)/D19,0)</f>
         <v/>
       </c>
       <c r="F19" s="145" t="inlineStr"/>
@@ -4401,36 +4158,35 @@
       <c r="H19" s="145" t="inlineStr"/>
       <c r="I19" s="145" t="inlineStr"/>
       <c r="J19" s="84">
-        <f>IF(A19="","",(COUNTIF(F19,"●")+COUNTIF(G19,"●")+COUNTIF(H19,"●")+COUNTIF(I19,"●")+COUNTIF(L19,"●")+COUNTIF(M19,"●")+COUNTIF(N19,"●")+COUNTIF(O19,"●"))*B19*C19)</f>
+        <f>IF(A18="","",(COUNTIF(F18,"●")+COUNTIF(G18,"●")+COUNTIF(H18,"●")+COUNTIF(I18,"●")+COUNTIF(L18,"●")+COUNTIF(M18,"●")+COUNTIF(N18,"●")+COUNTIF(O18,"●"))*B18*C18)</f>
         <v/>
       </c>
       <c r="K19" s="84">
-        <f>IF(A19="","",(COUNTIF(F19,"●")+COUNTIF(G19,"●")+COUNTIF(H19,"●")+COUNTIF(I19,"●")+COUNTIF(L19,"●")+COUNTIF(M19,"●")+COUNTIF(N19,"●")+COUNTIF(O19,"●"))*B19*D19)</f>
+        <f>IF(A18="","",(COUNTIF(F18,"●")+COUNTIF(G18,"●")+COUNTIF(H18,"●")+COUNTIF(I18,"●")+COUNTIF(L18,"●")+COUNTIF(M18,"●")+COUNTIF(N18,"●")+COUNTIF(O18,"●"))*B18*D18)</f>
         <v/>
       </c>
       <c r="L19" s="145" t="inlineStr"/>
       <c r="M19" s="145" t="inlineStr"/>
       <c r="N19" s="145" t="inlineStr"/>
       <c r="O19" s="145" t="inlineStr"/>
-      <c r="Q19" s="81">
-        <f>IF(A19="",0,COUNTIF(A$18:A18,A19))</f>
-        <v/>
-      </c>
-      <c r="R19" s="81" t="inlineStr"/>
+      <c r="P19" s="81">
+        <f>0</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="129" t="inlineStr"/>
       <c r="B20" s="83" t="inlineStr"/>
       <c r="C20" s="84">
-        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,2,FALSE))</f>
         <v/>
       </c>
       <c r="D20" s="84">
-        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
       <c r="E20" s="137">
-        <f>IF(D20&gt;0,(D20-C20)/D20,0)</f>
+        <f>IF(D19&gt;0,(D19-C19)/D19,0)</f>
         <v/>
       </c>
       <c r="F20" s="145" t="inlineStr"/>
@@ -4438,151 +4194,151 @@
       <c r="H20" s="145" t="inlineStr"/>
       <c r="I20" s="145" t="inlineStr"/>
       <c r="J20" s="84">
-        <f>IF(A20="","",(COUNTIF(F20,"●")+COUNTIF(G20,"●")+COUNTIF(H20,"●")+COUNTIF(I20,"●")+COUNTIF(L20,"●")+COUNTIF(M20,"●")+COUNTIF(N20,"●")+COUNTIF(O20,"●"))*B20*C20)</f>
+        <f>IF(A19="","",(COUNTIF(F19,"●")+COUNTIF(G19,"●")+COUNTIF(H19,"●")+COUNTIF(I19,"●")+COUNTIF(L19,"●")+COUNTIF(M19,"●")+COUNTIF(N19,"●")+COUNTIF(O19,"●"))*B19*C19)</f>
         <v/>
       </c>
       <c r="K20" s="84">
-        <f>IF(A20="","",(COUNTIF(F20,"●")+COUNTIF(G20,"●")+COUNTIF(H20,"●")+COUNTIF(I20,"●")+COUNTIF(L20,"●")+COUNTIF(M20,"●")+COUNTIF(N20,"●")+COUNTIF(O20,"●"))*B20*D20)</f>
+        <f>IF(A19="","",(COUNTIF(F19,"●")+COUNTIF(G19,"●")+COUNTIF(H19,"●")+COUNTIF(I19,"●")+COUNTIF(L19,"●")+COUNTIF(M19,"●")+COUNTIF(N19,"●")+COUNTIF(O19,"●"))*B19*D19)</f>
         <v/>
       </c>
       <c r="L20" s="145" t="inlineStr"/>
       <c r="M20" s="145" t="inlineStr"/>
       <c r="N20" s="145" t="inlineStr"/>
       <c r="O20" s="145" t="inlineStr"/>
-      <c r="Q20" s="81">
+      <c r="P20" s="81">
+        <f>IF(A19="",0,COUNTIF(A$18:A18,A19))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="129" t="inlineStr"/>
+      <c r="B21" s="83" t="inlineStr"/>
+      <c r="C21" s="84">
+        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D21" s="84">
+        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E21" s="137">
+        <f>IF(D20&gt;0,(D20-C20)/D20,0)</f>
+        <v/>
+      </c>
+      <c r="F21" s="145" t="inlineStr"/>
+      <c r="G21" s="145" t="inlineStr"/>
+      <c r="H21" s="145" t="inlineStr"/>
+      <c r="I21" s="145" t="inlineStr"/>
+      <c r="J21" s="84">
+        <f>IF(A20="","",(COUNTIF(F20,"●")+COUNTIF(G20,"●")+COUNTIF(H20,"●")+COUNTIF(I20,"●")+COUNTIF(L20,"●")+COUNTIF(M20,"●")+COUNTIF(N20,"●")+COUNTIF(O20,"●"))*B20*C20)</f>
+        <v/>
+      </c>
+      <c r="K21" s="84">
+        <f>IF(A20="","",(COUNTIF(F20,"●")+COUNTIF(G20,"●")+COUNTIF(H20,"●")+COUNTIF(I20,"●")+COUNTIF(L20,"●")+COUNTIF(M20,"●")+COUNTIF(N20,"●")+COUNTIF(O20,"●"))*B20*D20)</f>
+        <v/>
+      </c>
+      <c r="L21" s="145" t="inlineStr"/>
+      <c r="M21" s="145" t="inlineStr"/>
+      <c r="N21" s="145" t="inlineStr"/>
+      <c r="O21" s="145" t="inlineStr"/>
+      <c r="P21" s="81">
         <f>IF(A20="",0,COUNTIF(A$18:A19,A20))</f>
         <v/>
       </c>
-      <c r="R20" s="81" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="123" t="inlineStr">
+    </row>
+    <row r="22">
+      <c r="A22" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B21" s="114" t="inlineStr"/>
-      <c r="C21" s="114" t="inlineStr"/>
-      <c r="D21" s="114" t="inlineStr"/>
-      <c r="E21" s="114" t="inlineStr"/>
-      <c r="F21" s="130">
-        <f>IF(F18="●",B18*C18,0)+IF(F19="●",B19*C19,0)+IF(F20="●",B20*C20,0)</f>
-        <v/>
-      </c>
-      <c r="G21" s="130">
-        <f>IF(G18="●",B18*C18,0)+IF(G19="●",B19*C19,0)+IF(G20="●",B20*C20,0)</f>
-        <v/>
-      </c>
-      <c r="H21" s="130">
-        <f>IF(H18="●",B18*C18,0)+IF(H19="●",B19*C19,0)+IF(H20="●",B20*C20,0)</f>
-        <v/>
-      </c>
-      <c r="I21" s="130">
-        <f>IF(I18="●",B18*C18,0)+IF(I19="●",B19*C19,0)+IF(I20="●",B20*C20,0)</f>
-        <v/>
-      </c>
-      <c r="J21" s="88">
+      <c r="B22" s="114" t="inlineStr"/>
+      <c r="C22" s="114" t="inlineStr"/>
+      <c r="D22" s="114" t="inlineStr"/>
+      <c r="E22" s="114" t="inlineStr"/>
+      <c r="F22" s="130">
+        <f>SUMPRODUCT((F18:F20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="G22" s="130">
+        <f>SUMPRODUCT((G18:G20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="H22" s="130">
+        <f>SUMPRODUCT((H18:H20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="I22" s="130">
+        <f>SUMPRODUCT((I18:I20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="J22" s="88">
         <f>SUM(J18:J20)</f>
         <v/>
       </c>
-      <c r="K21" s="88">
+      <c r="K22" s="88">
         <f>SUM(K18:K20)</f>
         <v/>
       </c>
-      <c r="L21" s="130">
-        <f>IF(L18="●",B18*C18,0)+IF(L19="●",B19*C19,0)+IF(L20="●",B20*C20,0)</f>
-        <v/>
-      </c>
-      <c r="M21" s="130">
-        <f>IF(M18="●",B18*C18,0)+IF(M19="●",B19*C19,0)+IF(M20="●",B20*C20,0)</f>
-        <v/>
-      </c>
-      <c r="N21" s="130">
-        <f>IF(N18="●",B18*C18,0)+IF(N19="●",B19*C19,0)+IF(N20="●",B20*C20,0)</f>
-        <v/>
-      </c>
-      <c r="O21" s="130">
-        <f>IF(O18="●",B18*C18,0)+IF(O19="●",B19*C19,0)+IF(O20="●",B20*C20,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="128" t="inlineStr">
+      <c r="L22" s="130">
+        <f>SUMPRODUCT((L18:L20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="M22" s="130">
+        <f>SUMPRODUCT((M18:M20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="N22" s="130">
+        <f>SUMPRODUCT((N18:N20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+      <c r="O22" s="130">
+        <f>SUMPRODUCT((O18:O20="●")*1,B18:B20,C18:C20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="128" t="inlineStr">
         <is>
           <t>🚐 TRANSPORT</t>
         </is>
       </c>
-      <c r="B23" s="150" t="n"/>
-      <c r="C23" s="150" t="n"/>
-      <c r="D23" s="150" t="n"/>
-      <c r="E23" s="150" t="n"/>
-      <c r="F23" s="150" t="n"/>
-      <c r="G23" s="150" t="n"/>
-      <c r="H23" s="150" t="n"/>
-      <c r="I23" s="150" t="n"/>
-      <c r="J23" s="150" t="n"/>
-      <c r="K23" s="92" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="109" t="inlineStr">
+      <c r="B24" s="150" t="n"/>
+      <c r="C24" s="150" t="n"/>
+      <c r="D24" s="150" t="n"/>
+      <c r="E24" s="150" t="n"/>
+      <c r="F24" s="150" t="n"/>
+      <c r="G24" s="150" t="n"/>
+      <c r="H24" s="150" t="n"/>
+      <c r="I24" s="150" t="n"/>
+      <c r="J24" s="150" t="n"/>
+      <c r="K24" s="92" t="n"/>
+      <c r="L24" s="159" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="109" t="inlineStr">
         <is>
           <t>Driver/Guide + Van (일당)</t>
         </is>
       </c>
-      <c r="B24" s="83" t="n">
+      <c r="B25" s="83" t="n">
         <v>3</v>
       </c>
-      <c r="C24" s="84">
+      <c r="C25" s="84">
         <f>IF(A24="","",VLOOKUP(A24,'Master Data'!$A$28:$C$34,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D24" s="84">
+      <c r="D25" s="84">
         <f>IF(A24="","",VLOOKUP(A24,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E24" s="137">
+      <c r="E25" s="137">
         <f>IF(D24&gt;0,(D24-C24)/D24,0)</f>
-        <v/>
-      </c>
-      <c r="F24" s="145" t="inlineStr"/>
-      <c r="G24" s="145" t="inlineStr"/>
-      <c r="H24" s="145" t="inlineStr"/>
-      <c r="I24" s="145" t="inlineStr"/>
-      <c r="J24" s="84">
-        <f>IF(A24="","",IF(OR((F24="●")+(G24="●")+(H24="●")+(I24="●")+(L24="●")+(M24="●")+(N24="●")+(O24="●")),B24*C24,0))</f>
-        <v/>
-      </c>
-      <c r="K24" s="84">
-        <f>IF(A24="","",IF(OR((F24="●")+(G24="●")+(H24="●")+(I24="●")+(L24="●")+(M24="●")+(N24="●")+(O24="●")),B24*D24,0))</f>
-        <v/>
-      </c>
-      <c r="L24" s="145" t="inlineStr"/>
-      <c r="M24" s="145" t="inlineStr"/>
-      <c r="N24" s="145" t="inlineStr"/>
-      <c r="O24" s="145" t="inlineStr"/>
-      <c r="Q24" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="R24" s="81" t="inlineStr">
-        <is>
-          <t>pg</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="129" t="inlineStr"/>
-      <c r="B25" s="83" t="inlineStr"/>
-      <c r="C25" s="84">
-        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D25" s="84">
-        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E25" s="137">
-        <f>IF(D25&gt;0,(D25-C25)/D25,0)</f>
         <v/>
       </c>
       <c r="F25" s="145" t="inlineStr"/>
@@ -4590,36 +4346,35 @@
       <c r="H25" s="145" t="inlineStr"/>
       <c r="I25" s="145" t="inlineStr"/>
       <c r="J25" s="84">
-        <f>IF(A25="","",(COUNTIF(F25,"●")+COUNTIF(G25,"●")+COUNTIF(H25,"●")+COUNTIF(I25,"●")+COUNTIF(L25,"●")+COUNTIF(M25,"●")+COUNTIF(N25,"●")+COUNTIF(O25,"●"))*B25*C25)</f>
+        <f>IF(A25="","",IF(OR((F25="●")+(G25="●")+(H25="●")+(I25="●")+(L25="●")+(M25="●")+(N25="●")+(O25="●")),B25*C25,0))</f>
         <v/>
       </c>
       <c r="K25" s="84">
-        <f>IF(A25="","",(COUNTIF(F25,"●")+COUNTIF(G25,"●")+COUNTIF(H25,"●")+COUNTIF(I25,"●")+COUNTIF(L25,"●")+COUNTIF(M25,"●")+COUNTIF(N25,"●")+COUNTIF(O25,"●"))*B25*D25)</f>
+        <f>IF(A25="","",IF(OR((F25="●")+(G25="●")+(H25="●")+(I25="●")+(L25="●")+(M25="●")+(N25="●")+(O25="●")),B25*D25,0))</f>
         <v/>
       </c>
       <c r="L25" s="145" t="inlineStr"/>
       <c r="M25" s="145" t="inlineStr"/>
       <c r="N25" s="145" t="inlineStr"/>
       <c r="O25" s="145" t="inlineStr"/>
-      <c r="Q25" s="81">
-        <f>IF(A25="",0,COUNTIF(A$24:A24,A25))</f>
-        <v/>
-      </c>
-      <c r="R25" s="81" t="inlineStr"/>
+      <c r="P25" s="81">
+        <f>0</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="129" t="inlineStr"/>
       <c r="B26" s="83" t="inlineStr"/>
       <c r="C26" s="84">
-        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,2,FALSE))</f>
         <v/>
       </c>
       <c r="D26" s="84">
-        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
       <c r="E26" s="137">
-        <f>IF(D26&gt;0,(D26-C26)/D26,0)</f>
+        <f>IF(D25&gt;0,(D25-C25)/D25,0)</f>
         <v/>
       </c>
       <c r="F26" s="145" t="inlineStr"/>
@@ -4627,157 +4382,151 @@
       <c r="H26" s="145" t="inlineStr"/>
       <c r="I26" s="145" t="inlineStr"/>
       <c r="J26" s="84">
-        <f>IF(A26="","",(COUNTIF(F26,"●")+COUNTIF(G26,"●")+COUNTIF(H26,"●")+COUNTIF(I26,"●")+COUNTIF(L26,"●")+COUNTIF(M26,"●")+COUNTIF(N26,"●")+COUNTIF(O26,"●"))*B26*C26)</f>
+        <f>IF(A25="","",(COUNTIF(F25,"●")+COUNTIF(G25,"●")+COUNTIF(H25,"●")+COUNTIF(I25,"●")+COUNTIF(L25,"●")+COUNTIF(M25,"●")+COUNTIF(N25,"●")+COUNTIF(O25,"●"))*B25*C25)</f>
         <v/>
       </c>
       <c r="K26" s="84">
-        <f>IF(A26="","",(COUNTIF(F26,"●")+COUNTIF(G26,"●")+COUNTIF(H26,"●")+COUNTIF(I26,"●")+COUNTIF(L26,"●")+COUNTIF(M26,"●")+COUNTIF(N26,"●")+COUNTIF(O26,"●"))*B26*D26)</f>
+        <f>IF(A25="","",(COUNTIF(F25,"●")+COUNTIF(G25,"●")+COUNTIF(H25,"●")+COUNTIF(I25,"●")+COUNTIF(L25,"●")+COUNTIF(M25,"●")+COUNTIF(N25,"●")+COUNTIF(O25,"●"))*B25*D25)</f>
         <v/>
       </c>
       <c r="L26" s="145" t="inlineStr"/>
       <c r="M26" s="145" t="inlineStr"/>
       <c r="N26" s="145" t="inlineStr"/>
       <c r="O26" s="145" t="inlineStr"/>
-      <c r="Q26" s="81">
+      <c r="P26" s="81">
+        <f>IF(A25="",0,COUNTIF(A$24:A24,A25))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="129" t="inlineStr"/>
+      <c r="B27" s="83" t="inlineStr"/>
+      <c r="C27" s="84">
+        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D27" s="84">
+        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E27" s="137">
+        <f>IF(D26&gt;0,(D26-C26)/D26,0)</f>
+        <v/>
+      </c>
+      <c r="F27" s="145" t="inlineStr"/>
+      <c r="G27" s="145" t="inlineStr"/>
+      <c r="H27" s="145" t="inlineStr"/>
+      <c r="I27" s="145" t="inlineStr"/>
+      <c r="J27" s="84">
+        <f>IF(A26="","",(COUNTIF(F26,"●")+COUNTIF(G26,"●")+COUNTIF(H26,"●")+COUNTIF(I26,"●")+COUNTIF(L26,"●")+COUNTIF(M26,"●")+COUNTIF(N26,"●")+COUNTIF(O26,"●"))*B26*C26)</f>
+        <v/>
+      </c>
+      <c r="K27" s="84">
+        <f>IF(A26="","",(COUNTIF(F26,"●")+COUNTIF(G26,"●")+COUNTIF(H26,"●")+COUNTIF(I26,"●")+COUNTIF(L26,"●")+COUNTIF(M26,"●")+COUNTIF(N26,"●")+COUNTIF(O26,"●"))*B26*D26)</f>
+        <v/>
+      </c>
+      <c r="L27" s="145" t="inlineStr"/>
+      <c r="M27" s="145" t="inlineStr"/>
+      <c r="N27" s="145" t="inlineStr"/>
+      <c r="O27" s="145" t="inlineStr"/>
+      <c r="P27" s="81">
         <f>IF(A26="",0,COUNTIF(A$24:A25,A26))</f>
         <v/>
       </c>
-      <c r="R26" s="81" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="123" t="inlineStr">
+    </row>
+    <row r="28">
+      <c r="A28" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B27" s="114" t="inlineStr"/>
-      <c r="C27" s="114" t="inlineStr"/>
-      <c r="D27" s="114" t="inlineStr"/>
-      <c r="E27" s="114" t="inlineStr"/>
-      <c r="F27" s="130">
-        <f>IF(OR(F24="●"),B24*C24,0)+IF(F25="●",B25*C25,0)+IF(F26="●",B26*C26,0)</f>
-        <v/>
-      </c>
-      <c r="G27" s="130">
-        <f>IF(OR(G24="●"),B24*C24,0)+IF(G25="●",B25*C25,0)+IF(G26="●",B26*C26,0)</f>
-        <v/>
-      </c>
-      <c r="H27" s="130">
-        <f>IF(OR(H24="●"),B24*C24,0)+IF(H25="●",B25*C25,0)+IF(H26="●",B26*C26,0)</f>
-        <v/>
-      </c>
-      <c r="I27" s="130">
-        <f>IF(OR(I24="●"),B24*C24,0)+IF(I25="●",B25*C25,0)+IF(I26="●",B26*C26,0)</f>
-        <v/>
-      </c>
-      <c r="J27" s="88">
+      <c r="B28" s="114" t="inlineStr"/>
+      <c r="C28" s="114" t="inlineStr"/>
+      <c r="D28" s="114" t="inlineStr"/>
+      <c r="E28" s="114" t="inlineStr"/>
+      <c r="F28" s="130">
+        <f>SUMPRODUCT((F24:F26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="G28" s="130">
+        <f>SUMPRODUCT((G24:G26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="H28" s="130">
+        <f>SUMPRODUCT((H24:H26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="I28" s="130">
+        <f>SUMPRODUCT((I24:I26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="J28" s="88">
         <f>SUM(J24:J26)</f>
         <v/>
       </c>
-      <c r="K27" s="88">
+      <c r="K28" s="88">
         <f>SUM(K24:K26)</f>
         <v/>
       </c>
-      <c r="L27" s="130">
-        <f>IF(OR(L24="●"),B24*C24,0)+IF(L25="●",B25*C25,0)+IF(L26="●",B26*C26,0)</f>
-        <v/>
-      </c>
-      <c r="M27" s="130">
-        <f>IF(OR(M24="●"),B24*C24,0)+IF(M25="●",B25*C25,0)+IF(M26="●",B26*C26,0)</f>
-        <v/>
-      </c>
-      <c r="N27" s="130">
-        <f>IF(OR(N24="●"),B24*C24,0)+IF(N25="●",B25*C25,0)+IF(N26="●",B26*C26,0)</f>
-        <v/>
-      </c>
-      <c r="O27" s="130">
-        <f>IF(OR(O24="●"),B24*C24,0)+IF(O25="●",B25*C25,0)+IF(O26="●",B26*C26,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="128" t="inlineStr">
+      <c r="L28" s="130">
+        <f>SUMPRODUCT((L24:L26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="M28" s="130">
+        <f>SUMPRODUCT((M24:M26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="N28" s="130">
+        <f>SUMPRODUCT((N24:N26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+      <c r="O28" s="130">
+        <f>SUMPRODUCT((O24:O26="●")*1,B24:B26,C24:C26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="128" t="inlineStr">
         <is>
           <t>🍽️ MEALS</t>
         </is>
       </c>
-      <c r="B29" s="150" t="n"/>
-      <c r="C29" s="150" t="n"/>
-      <c r="D29" s="150" t="n"/>
-      <c r="E29" s="150" t="n"/>
-      <c r="F29" s="150" t="n"/>
-      <c r="G29" s="150" t="n"/>
-      <c r="H29" s="150" t="n"/>
-      <c r="I29" s="150" t="n"/>
-      <c r="J29" s="150" t="n"/>
-      <c r="K29" s="92" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="109" t="inlineStr">
+      <c r="B30" s="150" t="n"/>
+      <c r="C30" s="150" t="n"/>
+      <c r="D30" s="150" t="n"/>
+      <c r="E30" s="150" t="n"/>
+      <c r="F30" s="150" t="n"/>
+      <c r="G30" s="150" t="n"/>
+      <c r="H30" s="150" t="n"/>
+      <c r="I30" s="150" t="n"/>
+      <c r="J30" s="150" t="n"/>
+      <c r="K30" s="92" t="n"/>
+      <c r="L30" s="159" t="inlineStr">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="109" t="inlineStr">
         <is>
           <t>Breakfast (Hotel)</t>
-        </is>
-      </c>
-      <c r="B30" s="83" t="n">
-        <v>3</v>
-      </c>
-      <c r="C30" s="84">
-        <f>IF(A30="","",VLOOKUP(A30,'Master Data'!$A$38:$C$46,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D30" s="84">
-        <f>IF(A30="","",VLOOKUP(A30,'Master Data'!$A$38:$C$46,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E30" s="137">
-        <f>IF(D30&gt;0,(D30-C30)/D30,0)</f>
-        <v/>
-      </c>
-      <c r="F30" s="145" t="inlineStr"/>
-      <c r="G30" s="145" t="inlineStr"/>
-      <c r="H30" s="145" t="inlineStr"/>
-      <c r="I30" s="145" t="inlineStr"/>
-      <c r="J30" s="84">
-        <f>IF(A30="","",(COUNTIF(F30,"●")+COUNTIF(G30,"●")+COUNTIF(H30,"●")+COUNTIF(I30,"●")+COUNTIF(L30,"●")+COUNTIF(M30,"●")+COUNTIF(N30,"●")+COUNTIF(O30,"●"))*B30*C30)</f>
-        <v/>
-      </c>
-      <c r="K30" s="84">
-        <f>IF(A30="","",(COUNTIF(F30,"●")+COUNTIF(G30,"●")+COUNTIF(H30,"●")+COUNTIF(I30,"●")+COUNTIF(L30,"●")+COUNTIF(M30,"●")+COUNTIF(N30,"●")+COUNTIF(O30,"●"))*B30*D30)</f>
-        <v/>
-      </c>
-      <c r="L30" s="145" t="inlineStr"/>
-      <c r="M30" s="145" t="inlineStr"/>
-      <c r="N30" s="145" t="inlineStr"/>
-      <c r="O30" s="145" t="inlineStr"/>
-      <c r="Q30" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="R30" s="81" t="inlineStr">
-        <is>
-          <t>pp</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="108" t="inlineStr">
-        <is>
-          <t>Lunch</t>
         </is>
       </c>
       <c r="B31" s="83" t="n">
         <v>3</v>
       </c>
       <c r="C31" s="84">
-        <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A30="","",VLOOKUP(A30,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D31" s="84">
-        <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A30="","",VLOOKUP(A30,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E31" s="137">
-        <f>IF(D31&gt;0,(D31-C31)/D31,0)</f>
+        <f>IF(D30&gt;0,(D30-C30)/D30,0)</f>
         <v/>
       </c>
       <c r="F31" s="145" t="inlineStr"/>
@@ -4785,29 +4534,24 @@
       <c r="H31" s="145" t="inlineStr"/>
       <c r="I31" s="145" t="inlineStr"/>
       <c r="J31" s="84">
-        <f>IF(A31="","",(COUNTIF(F31,"●")+COUNTIF(G31,"●")+COUNTIF(H31,"●")+COUNTIF(I31,"●")+COUNTIF(L31,"●")+COUNTIF(M31,"●")+COUNTIF(N31,"●")+COUNTIF(O31,"●"))*B31*C31)</f>
+        <f>IF(A30="","",(COUNTIF(F30,"●")+COUNTIF(G30,"●")+COUNTIF(H30,"●")+COUNTIF(I30,"●")+COUNTIF(L30,"●")+COUNTIF(M30,"●")+COUNTIF(N30,"●")+COUNTIF(O30,"●"))*B30*C30)</f>
         <v/>
       </c>
       <c r="K31" s="84">
-        <f>IF(A31="","",(COUNTIF(F31,"●")+COUNTIF(G31,"●")+COUNTIF(H31,"●")+COUNTIF(I31,"●")+COUNTIF(L31,"●")+COUNTIF(M31,"●")+COUNTIF(N31,"●")+COUNTIF(O31,"●"))*B31*D31)</f>
+        <f>IF(A30="","",(COUNTIF(F30,"●")+COUNTIF(G30,"●")+COUNTIF(H30,"●")+COUNTIF(I30,"●")+COUNTIF(L30,"●")+COUNTIF(M30,"●")+COUNTIF(N30,"●")+COUNTIF(O30,"●"))*B30*D30)</f>
         <v/>
       </c>
       <c r="L31" s="145" t="inlineStr"/>
       <c r="M31" s="145" t="inlineStr"/>
       <c r="N31" s="145" t="inlineStr"/>
       <c r="O31" s="145" t="inlineStr"/>
-      <c r="Q31" s="81">
-        <f>IF(A31="",0,COUNTIF(A$30:A30,A31))</f>
-        <v/>
-      </c>
-      <c r="R31" s="81" t="inlineStr">
-        <is>
-          <t>pp</t>
-        </is>
+      <c r="P31" s="81">
+        <f>0</f>
+        <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="109" t="inlineStr">
+      <c r="A32" s="108" t="inlineStr">
         <is>
           <t>Dinner (Regular)</t>
         </is>
@@ -4816,15 +4560,15 @@
         <v>3</v>
       </c>
       <c r="C32" s="84">
-        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D32" s="84">
-        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E32" s="137">
-        <f>IF(D32&gt;0,(D32-C32)/D32,0)</f>
+        <f>IF(D31&gt;0,(D31-C31)/D31,0)</f>
         <v/>
       </c>
       <c r="F32" s="145" t="inlineStr"/>
@@ -4832,29 +4576,24 @@
       <c r="H32" s="145" t="inlineStr"/>
       <c r="I32" s="145" t="inlineStr"/>
       <c r="J32" s="84">
-        <f>IF(A32="","",(COUNTIF(F32,"●")+COUNTIF(G32,"●")+COUNTIF(H32,"●")+COUNTIF(I32,"●")+COUNTIF(L32,"●")+COUNTIF(M32,"●")+COUNTIF(N32,"●")+COUNTIF(O32,"●"))*B32*C32)</f>
+        <f>IF(A31="","",(COUNTIF(F31,"●")+COUNTIF(G31,"●")+COUNTIF(H31,"●")+COUNTIF(I31,"●")+COUNTIF(L31,"●")+COUNTIF(M31,"●")+COUNTIF(N31,"●")+COUNTIF(O31,"●"))*B31*C31)</f>
         <v/>
       </c>
       <c r="K32" s="84">
-        <f>IF(A32="","",(COUNTIF(F32,"●")+COUNTIF(G32,"●")+COUNTIF(H32,"●")+COUNTIF(I32,"●")+COUNTIF(L32,"●")+COUNTIF(M32,"●")+COUNTIF(N32,"●")+COUNTIF(O32,"●"))*B32*D32)</f>
+        <f>IF(A31="","",(COUNTIF(F31,"●")+COUNTIF(G31,"●")+COUNTIF(H31,"●")+COUNTIF(I31,"●")+COUNTIF(L31,"●")+COUNTIF(M31,"●")+COUNTIF(N31,"●")+COUNTIF(O31,"●"))*B31*D31)</f>
         <v/>
       </c>
       <c r="L32" s="145" t="inlineStr"/>
       <c r="M32" s="145" t="inlineStr"/>
       <c r="N32" s="145" t="inlineStr"/>
       <c r="O32" s="145" t="inlineStr"/>
-      <c r="Q32" s="81">
-        <f>IF(A32="",0,COUNTIF(A$30:A31,A32))</f>
-        <v/>
-      </c>
-      <c r="R32" s="81" t="inlineStr">
-        <is>
-          <t>pp</t>
-        </is>
+      <c r="P32" s="81">
+        <f>IF(A31="",0,COUNTIF(A$30:A30,A31))</f>
+        <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="108" t="inlineStr">
+      <c r="A33" s="109" t="inlineStr">
         <is>
           <t>Exclusive Dinner (Michelin/Fine)</t>
         </is>
@@ -4863,15 +4602,15 @@
         <v>2</v>
       </c>
       <c r="C33" s="84">
-        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D33" s="84">
-        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E33" s="137">
-        <f>IF(D33&gt;0,(D33-C33)/D33,0)</f>
+        <f>IF(D32&gt;0,(D32-C32)/D32,0)</f>
         <v/>
       </c>
       <c r="F33" s="145" t="inlineStr"/>
@@ -4879,40 +4618,41 @@
       <c r="H33" s="145" t="inlineStr"/>
       <c r="I33" s="145" t="inlineStr"/>
       <c r="J33" s="84">
-        <f>IF(A33="","",(COUNTIF(F33,"●")+COUNTIF(G33,"●")+COUNTIF(H33,"●")+COUNTIF(I33,"●")+COUNTIF(L33,"●")+COUNTIF(M33,"●")+COUNTIF(N33,"●")+COUNTIF(O33,"●"))*B33*C33)</f>
+        <f>IF(A32="","",(COUNTIF(F32,"●")+COUNTIF(G32,"●")+COUNTIF(H32,"●")+COUNTIF(I32,"●")+COUNTIF(L32,"●")+COUNTIF(M32,"●")+COUNTIF(N32,"●")+COUNTIF(O32,"●"))*B32*C32)</f>
         <v/>
       </c>
       <c r="K33" s="84">
-        <f>IF(A33="","",(COUNTIF(F33,"●")+COUNTIF(G33,"●")+COUNTIF(H33,"●")+COUNTIF(I33,"●")+COUNTIF(L33,"●")+COUNTIF(M33,"●")+COUNTIF(N33,"●")+COUNTIF(O33,"●"))*B33*D33)</f>
+        <f>IF(A32="","",(COUNTIF(F32,"●")+COUNTIF(G32,"●")+COUNTIF(H32,"●")+COUNTIF(I32,"●")+COUNTIF(L32,"●")+COUNTIF(M32,"●")+COUNTIF(N32,"●")+COUNTIF(O32,"●"))*B32*D32)</f>
         <v/>
       </c>
       <c r="L33" s="145" t="inlineStr"/>
       <c r="M33" s="145" t="inlineStr"/>
       <c r="N33" s="145" t="inlineStr"/>
       <c r="O33" s="145" t="inlineStr"/>
-      <c r="Q33" s="81">
-        <f>IF(A33="",0,COUNTIF(A$30:A32,A33))</f>
-        <v/>
-      </c>
-      <c r="R33" s="81" t="inlineStr">
-        <is>
-          <t>pp</t>
-        </is>
+      <c r="P33" s="81">
+        <f>IF(A32="",0,COUNTIF(A$30:A31,A32))</f>
+        <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="129" t="inlineStr"/>
-      <c r="B34" s="83" t="inlineStr"/>
+      <c r="A34" s="108" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="B34" s="83" t="n">
+        <v>3</v>
+      </c>
       <c r="C34" s="84">
-        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D34" s="84">
-        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E34" s="137">
-        <f>IF(D34&gt;0,(D34-C34)/D34,0)</f>
+        <f>IF(D33&gt;0,(D33-C33)/D33,0)</f>
         <v/>
       </c>
       <c r="F34" s="145" t="inlineStr"/>
@@ -4920,151 +4660,151 @@
       <c r="H34" s="145" t="inlineStr"/>
       <c r="I34" s="145" t="inlineStr"/>
       <c r="J34" s="84">
-        <f>IF(A34="","",(COUNTIF(F34,"●")+COUNTIF(G34,"●")+COUNTIF(H34,"●")+COUNTIF(I34,"●")+COUNTIF(L34,"●")+COUNTIF(M34,"●")+COUNTIF(N34,"●")+COUNTIF(O34,"●"))*B34*C34)</f>
+        <f>IF(A33="","",(COUNTIF(F33,"●")+COUNTIF(G33,"●")+COUNTIF(H33,"●")+COUNTIF(I33,"●")+COUNTIF(L33,"●")+COUNTIF(M33,"●")+COUNTIF(N33,"●")+COUNTIF(O33,"●"))*B33*C33)</f>
         <v/>
       </c>
       <c r="K34" s="84">
-        <f>IF(A34="","",(COUNTIF(F34,"●")+COUNTIF(G34,"●")+COUNTIF(H34,"●")+COUNTIF(I34,"●")+COUNTIF(L34,"●")+COUNTIF(M34,"●")+COUNTIF(N34,"●")+COUNTIF(O34,"●"))*B34*D34)</f>
+        <f>IF(A33="","",(COUNTIF(F33,"●")+COUNTIF(G33,"●")+COUNTIF(H33,"●")+COUNTIF(I33,"●")+COUNTIF(L33,"●")+COUNTIF(M33,"●")+COUNTIF(N33,"●")+COUNTIF(O33,"●"))*B33*D33)</f>
         <v/>
       </c>
       <c r="L34" s="145" t="inlineStr"/>
       <c r="M34" s="145" t="inlineStr"/>
       <c r="N34" s="145" t="inlineStr"/>
       <c r="O34" s="145" t="inlineStr"/>
-      <c r="Q34" s="81">
+      <c r="P34" s="81">
+        <f>IF(A33="",0,COUNTIF(A$30:A32,A33))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="129" t="inlineStr"/>
+      <c r="B35" s="83" t="inlineStr"/>
+      <c r="C35" s="84">
+        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D35" s="84">
+        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E35" s="137">
+        <f>IF(D34&gt;0,(D34-C34)/D34,0)</f>
+        <v/>
+      </c>
+      <c r="F35" s="145" t="inlineStr"/>
+      <c r="G35" s="145" t="inlineStr"/>
+      <c r="H35" s="145" t="inlineStr"/>
+      <c r="I35" s="145" t="inlineStr"/>
+      <c r="J35" s="84">
+        <f>IF(A34="","",(COUNTIF(F34,"●")+COUNTIF(G34,"●")+COUNTIF(H34,"●")+COUNTIF(I34,"●")+COUNTIF(L34,"●")+COUNTIF(M34,"●")+COUNTIF(N34,"●")+COUNTIF(O34,"●"))*B34*C34)</f>
+        <v/>
+      </c>
+      <c r="K35" s="84">
+        <f>IF(A34="","",(COUNTIF(F34,"●")+COUNTIF(G34,"●")+COUNTIF(H34,"●")+COUNTIF(I34,"●")+COUNTIF(L34,"●")+COUNTIF(M34,"●")+COUNTIF(N34,"●")+COUNTIF(O34,"●"))*B34*D34)</f>
+        <v/>
+      </c>
+      <c r="L35" s="145" t="inlineStr"/>
+      <c r="M35" s="145" t="inlineStr"/>
+      <c r="N35" s="145" t="inlineStr"/>
+      <c r="O35" s="145" t="inlineStr"/>
+      <c r="P35" s="81">
         <f>IF(A34="",0,COUNTIF(A$30:A33,A34))</f>
         <v/>
       </c>
-      <c r="R34" s="81" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="123" t="inlineStr">
+    </row>
+    <row r="36">
+      <c r="A36" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B35" s="114" t="inlineStr"/>
-      <c r="C35" s="114" t="inlineStr"/>
-      <c r="D35" s="114" t="inlineStr"/>
-      <c r="E35" s="114" t="inlineStr"/>
-      <c r="F35" s="130">
-        <f>IF(F30="●",B30*C30,0)+IF(F31="●",B31*C31,0)+IF(F32="●",B32*C32,0)+IF(F33="●",B33*C33,0)+IF(F34="●",B34*C34,0)</f>
-        <v/>
-      </c>
-      <c r="G35" s="130">
-        <f>IF(G30="●",B30*C30,0)+IF(G31="●",B31*C31,0)+IF(G32="●",B32*C32,0)+IF(G33="●",B33*C33,0)+IF(G34="●",B34*C34,0)</f>
-        <v/>
-      </c>
-      <c r="H35" s="130">
-        <f>IF(H30="●",B30*C30,0)+IF(H31="●",B31*C31,0)+IF(H32="●",B32*C32,0)+IF(H33="●",B33*C33,0)+IF(H34="●",B34*C34,0)</f>
-        <v/>
-      </c>
-      <c r="I35" s="130">
-        <f>IF(I30="●",B30*C30,0)+IF(I31="●",B31*C31,0)+IF(I32="●",B32*C32,0)+IF(I33="●",B33*C33,0)+IF(I34="●",B34*C34,0)</f>
-        <v/>
-      </c>
-      <c r="J35" s="88">
+      <c r="B36" s="114" t="inlineStr"/>
+      <c r="C36" s="114" t="inlineStr"/>
+      <c r="D36" s="114" t="inlineStr"/>
+      <c r="E36" s="114" t="inlineStr"/>
+      <c r="F36" s="130">
+        <f>SUMPRODUCT((F30:F34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="G36" s="130">
+        <f>SUMPRODUCT((G30:G34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="H36" s="130">
+        <f>SUMPRODUCT((H30:H34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="I36" s="130">
+        <f>SUMPRODUCT((I30:I34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="J36" s="88">
         <f>SUM(J30:J34)</f>
         <v/>
       </c>
-      <c r="K35" s="88">
+      <c r="K36" s="88">
         <f>SUM(K30:K34)</f>
         <v/>
       </c>
-      <c r="L35" s="130">
-        <f>IF(L30="●",B30*C30,0)+IF(L31="●",B31*C31,0)+IF(L32="●",B32*C32,0)+IF(L33="●",B33*C33,0)+IF(L34="●",B34*C34,0)</f>
-        <v/>
-      </c>
-      <c r="M35" s="130">
-        <f>IF(M30="●",B30*C30,0)+IF(M31="●",B31*C31,0)+IF(M32="●",B32*C32,0)+IF(M33="●",B33*C33,0)+IF(M34="●",B34*C34,0)</f>
-        <v/>
-      </c>
-      <c r="N35" s="130">
-        <f>IF(N30="●",B30*C30,0)+IF(N31="●",B31*C31,0)+IF(N32="●",B32*C32,0)+IF(N33="●",B33*C33,0)+IF(N34="●",B34*C34,0)</f>
-        <v/>
-      </c>
-      <c r="O35" s="130">
-        <f>IF(O30="●",B30*C30,0)+IF(O31="●",B31*C31,0)+IF(O32="●",B32*C32,0)+IF(O33="●",B33*C33,0)+IF(O34="●",B34*C34,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="128" t="inlineStr">
+      <c r="L36" s="130">
+        <f>SUMPRODUCT((L30:L34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="M36" s="130">
+        <f>SUMPRODUCT((M30:M34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="N36" s="130">
+        <f>SUMPRODUCT((N30:N34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+      <c r="O36" s="130">
+        <f>SUMPRODUCT((O30:O34="●")*1,B30:B34,C30:C34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="128" t="inlineStr">
         <is>
           <t>📦 OTHER</t>
         </is>
       </c>
-      <c r="B37" s="150" t="n"/>
-      <c r="C37" s="150" t="n"/>
-      <c r="D37" s="150" t="n"/>
-      <c r="E37" s="150" t="n"/>
-      <c r="F37" s="150" t="n"/>
-      <c r="G37" s="150" t="n"/>
-      <c r="H37" s="150" t="n"/>
-      <c r="I37" s="150" t="n"/>
-      <c r="J37" s="150" t="n"/>
-      <c r="K37" s="92" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="109" t="inlineStr">
+      <c r="B38" s="150" t="n"/>
+      <c r="C38" s="150" t="n"/>
+      <c r="D38" s="150" t="n"/>
+      <c r="E38" s="150" t="n"/>
+      <c r="F38" s="150" t="n"/>
+      <c r="G38" s="150" t="n"/>
+      <c r="H38" s="150" t="n"/>
+      <c r="I38" s="150" t="n"/>
+      <c r="J38" s="150" t="n"/>
+      <c r="K38" s="92" t="n"/>
+      <c r="L38" s="159" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="109" t="inlineStr">
         <is>
           <t>Insurance / Tips / Contingency</t>
         </is>
       </c>
-      <c r="B38" s="83" t="n">
+      <c r="B39" s="83" t="n">
         <v>4</v>
       </c>
-      <c r="C38" s="84">
+      <c r="C39" s="84">
         <f>IF(A38="","",VLOOKUP(A38,'Master Data'!$A$50:$C$56,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D38" s="84">
+      <c r="D39" s="84">
         <f>IF(A38="","",VLOOKUP(A38,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E38" s="137">
+      <c r="E39" s="137">
         <f>IF(D38&gt;0,(D38-C38)/D38,0)</f>
-        <v/>
-      </c>
-      <c r="F38" s="145" t="inlineStr"/>
-      <c r="G38" s="145" t="inlineStr"/>
-      <c r="H38" s="145" t="inlineStr"/>
-      <c r="I38" s="145" t="inlineStr"/>
-      <c r="J38" s="84">
-        <f>IF(A38="","",IF(OR((F38="●")+(G38="●")+(H38="●")+(I38="●")+(L38="●")+(M38="●")+(N38="●")+(O38="●")),B38*C38,0))</f>
-        <v/>
-      </c>
-      <c r="K38" s="84">
-        <f>IF(A38="","",IF(OR((F38="●")+(G38="●")+(H38="●")+(I38="●")+(L38="●")+(M38="●")+(N38="●")+(O38="●")),B38*D38,0))</f>
-        <v/>
-      </c>
-      <c r="L38" s="145" t="inlineStr"/>
-      <c r="M38" s="145" t="inlineStr"/>
-      <c r="N38" s="145" t="inlineStr"/>
-      <c r="O38" s="145" t="inlineStr"/>
-      <c r="Q38" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="R38" s="81" t="inlineStr">
-        <is>
-          <t>pg</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="129" t="inlineStr"/>
-      <c r="B39" s="83" t="inlineStr"/>
-      <c r="C39" s="84">
-        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D39" s="84">
-        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E39" s="137">
-        <f>IF(D39&gt;0,(D39-C39)/D39,0)</f>
         <v/>
       </c>
       <c r="F39" s="145" t="inlineStr"/>
@@ -5072,36 +4812,35 @@
       <c r="H39" s="145" t="inlineStr"/>
       <c r="I39" s="145" t="inlineStr"/>
       <c r="J39" s="84">
-        <f>IF(A39="","",(COUNTIF(F39,"●")+COUNTIF(G39,"●")+COUNTIF(H39,"●")+COUNTIF(I39,"●")+COUNTIF(L39,"●")+COUNTIF(M39,"●")+COUNTIF(N39,"●")+COUNTIF(O39,"●"))*B39*C39)</f>
+        <f>IF(A39="","",IF(OR((F39="●")+(G39="●")+(H39="●")+(I39="●")+(L39="●")+(M39="●")+(N39="●")+(O39="●")),B39*C39,0))</f>
         <v/>
       </c>
       <c r="K39" s="84">
-        <f>IF(A39="","",(COUNTIF(F39,"●")+COUNTIF(G39,"●")+COUNTIF(H39,"●")+COUNTIF(I39,"●")+COUNTIF(L39,"●")+COUNTIF(M39,"●")+COUNTIF(N39,"●")+COUNTIF(O39,"●"))*B39*D39)</f>
+        <f>IF(A39="","",IF(OR((F39="●")+(G39="●")+(H39="●")+(I39="●")+(L39="●")+(M39="●")+(N39="●")+(O39="●")),B39*D39,0))</f>
         <v/>
       </c>
       <c r="L39" s="145" t="inlineStr"/>
       <c r="M39" s="145" t="inlineStr"/>
       <c r="N39" s="145" t="inlineStr"/>
       <c r="O39" s="145" t="inlineStr"/>
-      <c r="Q39" s="81">
-        <f>IF(A39="",0,COUNTIF(A$38:A38,A39))</f>
-        <v/>
-      </c>
-      <c r="R39" s="81" t="inlineStr"/>
+      <c r="P39" s="81">
+        <f>0</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="129" t="inlineStr"/>
       <c r="B40" s="83" t="inlineStr"/>
       <c r="C40" s="84">
-        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,2,FALSE))</f>
         <v/>
       </c>
       <c r="D40" s="84">
-        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
       <c r="E40" s="137">
-        <f>IF(D40&gt;0,(D40-C40)/D40,0)</f>
+        <f>IF(D39&gt;0,(D39-C39)/D39,0)</f>
         <v/>
       </c>
       <c r="F40" s="145" t="inlineStr"/>
@@ -5109,157 +4848,151 @@
       <c r="H40" s="145" t="inlineStr"/>
       <c r="I40" s="145" t="inlineStr"/>
       <c r="J40" s="84">
-        <f>IF(A40="","",(COUNTIF(F40,"●")+COUNTIF(G40,"●")+COUNTIF(H40,"●")+COUNTIF(I40,"●")+COUNTIF(L40,"●")+COUNTIF(M40,"●")+COUNTIF(N40,"●")+COUNTIF(O40,"●"))*B40*C40)</f>
+        <f>IF(A39="","",(COUNTIF(F39,"●")+COUNTIF(G39,"●")+COUNTIF(H39,"●")+COUNTIF(I39,"●")+COUNTIF(L39,"●")+COUNTIF(M39,"●")+COUNTIF(N39,"●")+COUNTIF(O39,"●"))*B39*C39)</f>
         <v/>
       </c>
       <c r="K40" s="84">
-        <f>IF(A40="","",(COUNTIF(F40,"●")+COUNTIF(G40,"●")+COUNTIF(H40,"●")+COUNTIF(I40,"●")+COUNTIF(L40,"●")+COUNTIF(M40,"●")+COUNTIF(N40,"●")+COUNTIF(O40,"●"))*B40*D40)</f>
+        <f>IF(A39="","",(COUNTIF(F39,"●")+COUNTIF(G39,"●")+COUNTIF(H39,"●")+COUNTIF(I39,"●")+COUNTIF(L39,"●")+COUNTIF(M39,"●")+COUNTIF(N39,"●")+COUNTIF(O39,"●"))*B39*D39)</f>
         <v/>
       </c>
       <c r="L40" s="145" t="inlineStr"/>
       <c r="M40" s="145" t="inlineStr"/>
       <c r="N40" s="145" t="inlineStr"/>
       <c r="O40" s="145" t="inlineStr"/>
-      <c r="Q40" s="81">
+      <c r="P40" s="81">
+        <f>IF(A39="",0,COUNTIF(A$38:A38,A39))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="129" t="inlineStr"/>
+      <c r="B41" s="83" t="inlineStr"/>
+      <c r="C41" s="84">
+        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D41" s="84">
+        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E41" s="137">
+        <f>IF(D40&gt;0,(D40-C40)/D40,0)</f>
+        <v/>
+      </c>
+      <c r="F41" s="145" t="inlineStr"/>
+      <c r="G41" s="145" t="inlineStr"/>
+      <c r="H41" s="145" t="inlineStr"/>
+      <c r="I41" s="145" t="inlineStr"/>
+      <c r="J41" s="84">
+        <f>IF(A40="","",(COUNTIF(F40,"●")+COUNTIF(G40,"●")+COUNTIF(H40,"●")+COUNTIF(I40,"●")+COUNTIF(L40,"●")+COUNTIF(M40,"●")+COUNTIF(N40,"●")+COUNTIF(O40,"●"))*B40*C40)</f>
+        <v/>
+      </c>
+      <c r="K41" s="84">
+        <f>IF(A40="","",(COUNTIF(F40,"●")+COUNTIF(G40,"●")+COUNTIF(H40,"●")+COUNTIF(I40,"●")+COUNTIF(L40,"●")+COUNTIF(M40,"●")+COUNTIF(N40,"●")+COUNTIF(O40,"●"))*B40*D40)</f>
+        <v/>
+      </c>
+      <c r="L41" s="145" t="inlineStr"/>
+      <c r="M41" s="145" t="inlineStr"/>
+      <c r="N41" s="145" t="inlineStr"/>
+      <c r="O41" s="145" t="inlineStr"/>
+      <c r="P41" s="81">
         <f>IF(A40="",0,COUNTIF(A$38:A39,A40))</f>
         <v/>
       </c>
-      <c r="R40" s="81" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="123" t="inlineStr">
+    </row>
+    <row r="42">
+      <c r="A42" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B41" s="114" t="inlineStr"/>
-      <c r="C41" s="114" t="inlineStr"/>
-      <c r="D41" s="114" t="inlineStr"/>
-      <c r="E41" s="114" t="inlineStr"/>
-      <c r="F41" s="130">
-        <f>IF(OR(F38="●"),B38*C38,0)+IF(F39="●",B39*C39,0)+IF(F40="●",B40*C40,0)</f>
-        <v/>
-      </c>
-      <c r="G41" s="130">
-        <f>IF(OR(G38="●"),B38*C38,0)+IF(G39="●",B39*C39,0)+IF(G40="●",B40*C40,0)</f>
-        <v/>
-      </c>
-      <c r="H41" s="130">
-        <f>IF(OR(H38="●"),B38*C38,0)+IF(H39="●",B39*C39,0)+IF(H40="●",B40*C40,0)</f>
-        <v/>
-      </c>
-      <c r="I41" s="130">
-        <f>IF(OR(I38="●"),B38*C38,0)+IF(I39="●",B39*C39,0)+IF(I40="●",B40*C40,0)</f>
-        <v/>
-      </c>
-      <c r="J41" s="88">
+      <c r="B42" s="114" t="inlineStr"/>
+      <c r="C42" s="114" t="inlineStr"/>
+      <c r="D42" s="114" t="inlineStr"/>
+      <c r="E42" s="114" t="inlineStr"/>
+      <c r="F42" s="130">
+        <f>SUMPRODUCT((F38:F40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="G42" s="130">
+        <f>SUMPRODUCT((G38:G40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="H42" s="130">
+        <f>SUMPRODUCT((H38:H40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="I42" s="130">
+        <f>SUMPRODUCT((I38:I40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="J42" s="88">
         <f>SUM(J38:J40)</f>
         <v/>
       </c>
-      <c r="K41" s="88">
+      <c r="K42" s="88">
         <f>SUM(K38:K40)</f>
         <v/>
       </c>
-      <c r="L41" s="130">
-        <f>IF(OR(L38="●"),B38*C38,0)+IF(L39="●",B39*C39,0)+IF(L40="●",B40*C40,0)</f>
-        <v/>
-      </c>
-      <c r="M41" s="130">
-        <f>IF(OR(M38="●"),B38*C38,0)+IF(M39="●",B39*C39,0)+IF(M40="●",B40*C40,0)</f>
-        <v/>
-      </c>
-      <c r="N41" s="130">
-        <f>IF(OR(N38="●"),B38*C38,0)+IF(N39="●",B39*C39,0)+IF(N40="●",B40*C40,0)</f>
-        <v/>
-      </c>
-      <c r="O41" s="130">
-        <f>IF(OR(O38="●"),B38*C38,0)+IF(O39="●",B39*C39,0)+IF(O40="●",B40*C40,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="128" t="inlineStr">
+      <c r="L42" s="130">
+        <f>SUMPRODUCT((L38:L40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="M42" s="130">
+        <f>SUMPRODUCT((M38:M40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="N42" s="130">
+        <f>SUMPRODUCT((N38:N40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+      <c r="O42" s="130">
+        <f>SUMPRODUCT((O38:O40="●")*1,B38:B40,C38:C40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" s="128" t="inlineStr">
         <is>
           <t>🎯 ACTIVITIES</t>
         </is>
       </c>
-      <c r="B43" s="150" t="n"/>
-      <c r="C43" s="150" t="n"/>
-      <c r="D43" s="150" t="n"/>
-      <c r="E43" s="150" t="n"/>
-      <c r="F43" s="150" t="n"/>
-      <c r="G43" s="150" t="n"/>
-      <c r="H43" s="150" t="n"/>
-      <c r="I43" s="150" t="n"/>
-      <c r="J43" s="150" t="n"/>
-      <c r="K43" s="92" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="109" t="inlineStr">
+      <c r="B44" s="150" t="n"/>
+      <c r="C44" s="150" t="n"/>
+      <c r="D44" s="150" t="n"/>
+      <c r="E44" s="150" t="n"/>
+      <c r="F44" s="150" t="n"/>
+      <c r="G44" s="150" t="n"/>
+      <c r="H44" s="150" t="n"/>
+      <c r="I44" s="150" t="n"/>
+      <c r="J44" s="150" t="n"/>
+      <c r="K44" s="92" t="n"/>
+      <c r="L44" s="159" t="inlineStr">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="109" t="inlineStr">
         <is>
           <t>Beach/Surf Lesson</t>
-        </is>
-      </c>
-      <c r="B44" s="83" t="n">
-        <v>1</v>
-      </c>
-      <c r="C44" s="84">
-        <f>IF(A44="","",VLOOKUP(A44,'Master Data'!$A$86:$C$94,2,FALSE))</f>
-        <v/>
-      </c>
-      <c r="D44" s="84">
-        <f>IF(A44="","",VLOOKUP(A44,'Master Data'!$A$86:$C$94,3,FALSE))</f>
-        <v/>
-      </c>
-      <c r="E44" s="137">
-        <f>IF(D44&gt;0,(D44-C44)/D44,0)</f>
-        <v/>
-      </c>
-      <c r="F44" s="145" t="inlineStr"/>
-      <c r="G44" s="145" t="inlineStr"/>
-      <c r="H44" s="145" t="inlineStr"/>
-      <c r="I44" s="145" t="inlineStr"/>
-      <c r="J44" s="84">
-        <f>IF(A44="","",(COUNTIF(F44,"●")+COUNTIF(G44,"●")+COUNTIF(H44,"●")+COUNTIF(I44,"●")+COUNTIF(L44,"●")+COUNTIF(M44,"●")+COUNTIF(N44,"●")+COUNTIF(O44,"●"))*B44*C44)</f>
-        <v/>
-      </c>
-      <c r="K44" s="84">
-        <f>IF(A44="","",(COUNTIF(F44,"●")+COUNTIF(G44,"●")+COUNTIF(H44,"●")+COUNTIF(I44,"●")+COUNTIF(L44,"●")+COUNTIF(M44,"●")+COUNTIF(N44,"●")+COUNTIF(O44,"●"))*B44*D44)</f>
-        <v/>
-      </c>
-      <c r="L44" s="145" t="inlineStr"/>
-      <c r="M44" s="145" t="inlineStr"/>
-      <c r="N44" s="145" t="inlineStr"/>
-      <c r="O44" s="145" t="inlineStr"/>
-      <c r="Q44" s="81">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="R44" s="81" t="inlineStr">
-        <is>
-          <t>pp</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="108" t="inlineStr">
-        <is>
-          <t>Local Hiking (Griffith/Runyon)</t>
         </is>
       </c>
       <c r="B45" s="83" t="n">
         <v>1</v>
       </c>
       <c r="C45" s="84">
-        <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A44="","",VLOOKUP(A44,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D45" s="84">
-        <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A44="","",VLOOKUP(A44,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E45" s="137">
-        <f>IF(D45&gt;0,(D45-C45)/D45,0)</f>
+        <f>IF(D44&gt;0,(D44-C44)/D44,0)</f>
         <v/>
       </c>
       <c r="F45" s="145" t="inlineStr"/>
@@ -5267,46 +5000,41 @@
       <c r="H45" s="145" t="inlineStr"/>
       <c r="I45" s="145" t="inlineStr"/>
       <c r="J45" s="84">
-        <f>IF(A45="","",(COUNTIF(F45,"●")+COUNTIF(G45,"●")+COUNTIF(H45,"●")+COUNTIF(I45,"●")+COUNTIF(L45,"●")+COUNTIF(M45,"●")+COUNTIF(N45,"●")+COUNTIF(O45,"●"))*B45*C45)</f>
+        <f>IF(A44="","",(COUNTIF(F44,"●")+COUNTIF(G44,"●")+COUNTIF(H44,"●")+COUNTIF(I44,"●")+COUNTIF(L44,"●")+COUNTIF(M44,"●")+COUNTIF(N44,"●")+COUNTIF(O44,"●"))*B44*C44)</f>
         <v/>
       </c>
       <c r="K45" s="84">
-        <f>IF(A45="","",(COUNTIF(F45,"●")+COUNTIF(G45,"●")+COUNTIF(H45,"●")+COUNTIF(I45,"●")+COUNTIF(L45,"●")+COUNTIF(M45,"●")+COUNTIF(N45,"●")+COUNTIF(O45,"●"))*B45*D45)</f>
+        <f>IF(A44="","",(COUNTIF(F44,"●")+COUNTIF(G44,"●")+COUNTIF(H44,"●")+COUNTIF(I44,"●")+COUNTIF(L44,"●")+COUNTIF(M44,"●")+COUNTIF(N44,"●")+COUNTIF(O44,"●"))*B44*D44)</f>
         <v/>
       </c>
       <c r="L45" s="145" t="inlineStr"/>
       <c r="M45" s="145" t="inlineStr"/>
       <c r="N45" s="145" t="inlineStr"/>
       <c r="O45" s="145" t="inlineStr"/>
-      <c r="Q45" s="81">
-        <f>IF(A45="",0,COUNTIF(A$44:A44,A45))</f>
-        <v/>
-      </c>
-      <c r="R45" s="81" t="inlineStr">
-        <is>
-          <t>pp</t>
-        </is>
+      <c r="P45" s="81">
+        <f>0</f>
+        <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="109" t="inlineStr">
-        <is>
-          <t>NBA/MLB Game (Ticket)</t>
+      <c r="A46" s="108" t="inlineStr">
+        <is>
+          <t>Local Hiking (Griffith/Runyon)</t>
         </is>
       </c>
       <c r="B46" s="83" t="n">
         <v>1</v>
       </c>
       <c r="C46" s="84">
-        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D46" s="84">
-        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E46" s="137">
-        <f>IF(D46&gt;0,(D46-C46)/D46,0)</f>
+        <f>IF(D45&gt;0,(D45-C45)/D45,0)</f>
         <v/>
       </c>
       <c r="F46" s="145" t="inlineStr"/>
@@ -5314,46 +5042,41 @@
       <c r="H46" s="145" t="inlineStr"/>
       <c r="I46" s="145" t="inlineStr"/>
       <c r="J46" s="84">
-        <f>IF(A46="","",(COUNTIF(F46,"●")+COUNTIF(G46,"●")+COUNTIF(H46,"●")+COUNTIF(I46,"●")+COUNTIF(L46,"●")+COUNTIF(M46,"●")+COUNTIF(N46,"●")+COUNTIF(O46,"●"))*B46*C46)</f>
+        <f>IF(A45="","",(COUNTIF(F45,"●")+COUNTIF(G45,"●")+COUNTIF(H45,"●")+COUNTIF(I45,"●")+COUNTIF(L45,"●")+COUNTIF(M45,"●")+COUNTIF(N45,"●")+COUNTIF(O45,"●"))*B45*C45)</f>
         <v/>
       </c>
       <c r="K46" s="84">
-        <f>IF(A46="","",(COUNTIF(F46,"●")+COUNTIF(G46,"●")+COUNTIF(H46,"●")+COUNTIF(I46,"●")+COUNTIF(L46,"●")+COUNTIF(M46,"●")+COUNTIF(N46,"●")+COUNTIF(O46,"●"))*B46*D46)</f>
+        <f>IF(A45="","",(COUNTIF(F45,"●")+COUNTIF(G45,"●")+COUNTIF(H45,"●")+COUNTIF(I45,"●")+COUNTIF(L45,"●")+COUNTIF(M45,"●")+COUNTIF(N45,"●")+COUNTIF(O45,"●"))*B45*D45)</f>
         <v/>
       </c>
       <c r="L46" s="145" t="inlineStr"/>
       <c r="M46" s="145" t="inlineStr"/>
       <c r="N46" s="145" t="inlineStr"/>
       <c r="O46" s="145" t="inlineStr"/>
-      <c r="Q46" s="81">
-        <f>IF(A46="",0,COUNTIF(A$44:A45,A46))</f>
-        <v/>
-      </c>
-      <c r="R46" s="81" t="inlineStr">
-        <is>
-          <t>pp</t>
-        </is>
+      <c r="P46" s="81">
+        <f>IF(A45="",0,COUNTIF(A$44:A44,A45))</f>
+        <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="108" t="inlineStr">
-        <is>
-          <t>Sports Bar Experience</t>
+      <c r="A47" s="109" t="inlineStr">
+        <is>
+          <t>NBA/MLB Game (Ticket)</t>
         </is>
       </c>
       <c r="B47" s="83" t="n">
         <v>1</v>
       </c>
       <c r="C47" s="84">
-        <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D47" s="84">
-        <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E47" s="137">
-        <f>IF(D47&gt;0,(D47-C47)/D47,0)</f>
+        <f>IF(D46&gt;0,(D46-C46)/D46,0)</f>
         <v/>
       </c>
       <c r="F47" s="145" t="inlineStr"/>
@@ -5361,40 +5084,41 @@
       <c r="H47" s="145" t="inlineStr"/>
       <c r="I47" s="145" t="inlineStr"/>
       <c r="J47" s="84">
-        <f>IF(A47="","",(COUNTIF(F47,"●")+COUNTIF(G47,"●")+COUNTIF(H47,"●")+COUNTIF(I47,"●")+COUNTIF(L47,"●")+COUNTIF(M47,"●")+COUNTIF(N47,"●")+COUNTIF(O47,"●"))*B47*C47)</f>
+        <f>IF(A46="","",(COUNTIF(F46,"●")+COUNTIF(G46,"●")+COUNTIF(H46,"●")+COUNTIF(I46,"●")+COUNTIF(L46,"●")+COUNTIF(M46,"●")+COUNTIF(N46,"●")+COUNTIF(O46,"●"))*B46*C46)</f>
         <v/>
       </c>
       <c r="K47" s="84">
-        <f>IF(A47="","",(COUNTIF(F47,"●")+COUNTIF(G47,"●")+COUNTIF(H47,"●")+COUNTIF(I47,"●")+COUNTIF(L47,"●")+COUNTIF(M47,"●")+COUNTIF(N47,"●")+COUNTIF(O47,"●"))*B47*D47)</f>
+        <f>IF(A46="","",(COUNTIF(F46,"●")+COUNTIF(G46,"●")+COUNTIF(H46,"●")+COUNTIF(I46,"●")+COUNTIF(L46,"●")+COUNTIF(M46,"●")+COUNTIF(N46,"●")+COUNTIF(O46,"●"))*B46*D46)</f>
         <v/>
       </c>
       <c r="L47" s="145" t="inlineStr"/>
       <c r="M47" s="145" t="inlineStr"/>
       <c r="N47" s="145" t="inlineStr"/>
       <c r="O47" s="145" t="inlineStr"/>
-      <c r="Q47" s="81">
-        <f>IF(A47="",0,COUNTIF(A$44:A46,A47))</f>
-        <v/>
-      </c>
-      <c r="R47" s="81" t="inlineStr">
-        <is>
-          <t>pp</t>
-        </is>
+      <c r="P47" s="81">
+        <f>IF(A46="",0,COUNTIF(A$44:A45,A46))</f>
+        <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="129" t="inlineStr"/>
-      <c r="B48" s="83" t="inlineStr"/>
+      <c r="A48" s="108" t="inlineStr">
+        <is>
+          <t>Sports Bar Experience</t>
+        </is>
+      </c>
+      <c r="B48" s="83" t="n">
+        <v>1</v>
+      </c>
       <c r="C48" s="84">
-        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D48" s="84">
-        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E48" s="137">
-        <f>IF(D48&gt;0,(D48-C48)/D48,0)</f>
+        <f>IF(D47&gt;0,(D47-C47)/D47,0)</f>
         <v/>
       </c>
       <c r="F48" s="145" t="inlineStr"/>
@@ -5402,36 +5126,35 @@
       <c r="H48" s="145" t="inlineStr"/>
       <c r="I48" s="145" t="inlineStr"/>
       <c r="J48" s="84">
-        <f>IF(A48="","",(COUNTIF(F48,"●")+COUNTIF(G48,"●")+COUNTIF(H48,"●")+COUNTIF(I48,"●")+COUNTIF(L48,"●")+COUNTIF(M48,"●")+COUNTIF(N48,"●")+COUNTIF(O48,"●"))*B48*C48)</f>
+        <f>IF(A47="","",(COUNTIF(F47,"●")+COUNTIF(G47,"●")+COUNTIF(H47,"●")+COUNTIF(I47,"●")+COUNTIF(L47,"●")+COUNTIF(M47,"●")+COUNTIF(N47,"●")+COUNTIF(O47,"●"))*B47*C47)</f>
         <v/>
       </c>
       <c r="K48" s="84">
-        <f>IF(A48="","",(COUNTIF(F48,"●")+COUNTIF(G48,"●")+COUNTIF(H48,"●")+COUNTIF(I48,"●")+COUNTIF(L48,"●")+COUNTIF(M48,"●")+COUNTIF(N48,"●")+COUNTIF(O48,"●"))*B48*D48)</f>
+        <f>IF(A47="","",(COUNTIF(F47,"●")+COUNTIF(G47,"●")+COUNTIF(H47,"●")+COUNTIF(I47,"●")+COUNTIF(L47,"●")+COUNTIF(M47,"●")+COUNTIF(N47,"●")+COUNTIF(O47,"●"))*B47*D47)</f>
         <v/>
       </c>
       <c r="L48" s="145" t="inlineStr"/>
       <c r="M48" s="145" t="inlineStr"/>
       <c r="N48" s="145" t="inlineStr"/>
       <c r="O48" s="145" t="inlineStr"/>
-      <c r="Q48" s="81">
-        <f>IF(A48="",0,COUNTIF(A$44:A47,A48))</f>
-        <v/>
-      </c>
-      <c r="R48" s="81" t="inlineStr"/>
+      <c r="P48" s="81">
+        <f>IF(A47="",0,COUNTIF(A$44:A46,A47))</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="129" t="inlineStr"/>
       <c r="B49" s="83" t="inlineStr"/>
       <c r="C49" s="84">
-        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D49" s="84">
-        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E49" s="137">
-        <f>IF(D49&gt;0,(D49-C49)/D49,0)</f>
+        <f>IF(D48&gt;0,(D48-C48)/D48,0)</f>
         <v/>
       </c>
       <c r="F49" s="145" t="inlineStr"/>
@@ -5439,36 +5162,35 @@
       <c r="H49" s="145" t="inlineStr"/>
       <c r="I49" s="145" t="inlineStr"/>
       <c r="J49" s="84">
-        <f>IF(A49="","",(COUNTIF(F49,"●")+COUNTIF(G49,"●")+COUNTIF(H49,"●")+COUNTIF(I49,"●")+COUNTIF(L49,"●")+COUNTIF(M49,"●")+COUNTIF(N49,"●")+COUNTIF(O49,"●"))*B49*C49)</f>
+        <f>IF(A48="","",(COUNTIF(F48,"●")+COUNTIF(G48,"●")+COUNTIF(H48,"●")+COUNTIF(I48,"●")+COUNTIF(L48,"●")+COUNTIF(M48,"●")+COUNTIF(N48,"●")+COUNTIF(O48,"●"))*B48*C48)</f>
         <v/>
       </c>
       <c r="K49" s="84">
-        <f>IF(A49="","",(COUNTIF(F49,"●")+COUNTIF(G49,"●")+COUNTIF(H49,"●")+COUNTIF(I49,"●")+COUNTIF(L49,"●")+COUNTIF(M49,"●")+COUNTIF(N49,"●")+COUNTIF(O49,"●"))*B49*D49)</f>
+        <f>IF(A48="","",(COUNTIF(F48,"●")+COUNTIF(G48,"●")+COUNTIF(H48,"●")+COUNTIF(I48,"●")+COUNTIF(L48,"●")+COUNTIF(M48,"●")+COUNTIF(N48,"●")+COUNTIF(O48,"●"))*B48*D48)</f>
         <v/>
       </c>
       <c r="L49" s="145" t="inlineStr"/>
       <c r="M49" s="145" t="inlineStr"/>
       <c r="N49" s="145" t="inlineStr"/>
       <c r="O49" s="145" t="inlineStr"/>
-      <c r="Q49" s="81">
-        <f>IF(A49="",0,COUNTIF(A$44:A48,A49))</f>
-        <v/>
-      </c>
-      <c r="R49" s="81" t="inlineStr"/>
+      <c r="P49" s="81">
+        <f>IF(A48="",0,COUNTIF(A$44:A47,A48))</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="129" t="inlineStr"/>
       <c r="B50" s="83" t="inlineStr"/>
       <c r="C50" s="84">
-        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D50" s="84">
-        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E50" s="137">
-        <f>IF(D50&gt;0,(D50-C50)/D50,0)</f>
+        <f>IF(D49&gt;0,(D49-C49)/D49,0)</f>
         <v/>
       </c>
       <c r="F50" s="145" t="inlineStr"/>
@@ -5476,36 +5198,35 @@
       <c r="H50" s="145" t="inlineStr"/>
       <c r="I50" s="145" t="inlineStr"/>
       <c r="J50" s="84">
-        <f>IF(A50="","",(COUNTIF(F50,"●")+COUNTIF(G50,"●")+COUNTIF(H50,"●")+COUNTIF(I50,"●")+COUNTIF(L50,"●")+COUNTIF(M50,"●")+COUNTIF(N50,"●")+COUNTIF(O50,"●"))*B50*C50)</f>
+        <f>IF(A49="","",(COUNTIF(F49,"●")+COUNTIF(G49,"●")+COUNTIF(H49,"●")+COUNTIF(I49,"●")+COUNTIF(L49,"●")+COUNTIF(M49,"●")+COUNTIF(N49,"●")+COUNTIF(O49,"●"))*B49*C49)</f>
         <v/>
       </c>
       <c r="K50" s="84">
-        <f>IF(A50="","",(COUNTIF(F50,"●")+COUNTIF(G50,"●")+COUNTIF(H50,"●")+COUNTIF(I50,"●")+COUNTIF(L50,"●")+COUNTIF(M50,"●")+COUNTIF(N50,"●")+COUNTIF(O50,"●"))*B50*D50)</f>
+        <f>IF(A49="","",(COUNTIF(F49,"●")+COUNTIF(G49,"●")+COUNTIF(H49,"●")+COUNTIF(I49,"●")+COUNTIF(L49,"●")+COUNTIF(M49,"●")+COUNTIF(N49,"●")+COUNTIF(O49,"●"))*B49*D49)</f>
         <v/>
       </c>
       <c r="L50" s="145" t="inlineStr"/>
       <c r="M50" s="145" t="inlineStr"/>
       <c r="N50" s="145" t="inlineStr"/>
       <c r="O50" s="145" t="inlineStr"/>
-      <c r="Q50" s="81">
-        <f>IF(A50="",0,COUNTIF(A$44:A49,A50))</f>
-        <v/>
-      </c>
-      <c r="R50" s="81" t="inlineStr"/>
+      <c r="P50" s="81">
+        <f>IF(A49="",0,COUNTIF(A$44:A48,A49))</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="129" t="inlineStr"/>
       <c r="B51" s="83" t="inlineStr"/>
       <c r="C51" s="84">
-        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D51" s="84">
-        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E51" s="137">
-        <f>IF(D51&gt;0,(D51-C51)/D51,0)</f>
+        <f>IF(D50&gt;0,(D50-C50)/D50,0)</f>
         <v/>
       </c>
       <c r="F51" s="145" t="inlineStr"/>
@@ -5513,36 +5234,35 @@
       <c r="H51" s="145" t="inlineStr"/>
       <c r="I51" s="145" t="inlineStr"/>
       <c r="J51" s="84">
-        <f>IF(A51="","",(COUNTIF(F51,"●")+COUNTIF(G51,"●")+COUNTIF(H51,"●")+COUNTIF(I51,"●")+COUNTIF(L51,"●")+COUNTIF(M51,"●")+COUNTIF(N51,"●")+COUNTIF(O51,"●"))*B51*C51)</f>
+        <f>IF(A50="","",(COUNTIF(F50,"●")+COUNTIF(G50,"●")+COUNTIF(H50,"●")+COUNTIF(I50,"●")+COUNTIF(L50,"●")+COUNTIF(M50,"●")+COUNTIF(N50,"●")+COUNTIF(O50,"●"))*B50*C50)</f>
         <v/>
       </c>
       <c r="K51" s="84">
-        <f>IF(A51="","",(COUNTIF(F51,"●")+COUNTIF(G51,"●")+COUNTIF(H51,"●")+COUNTIF(I51,"●")+COUNTIF(L51,"●")+COUNTIF(M51,"●")+COUNTIF(N51,"●")+COUNTIF(O51,"●"))*B51*D51)</f>
+        <f>IF(A50="","",(COUNTIF(F50,"●")+COUNTIF(G50,"●")+COUNTIF(H50,"●")+COUNTIF(I50,"●")+COUNTIF(L50,"●")+COUNTIF(M50,"●")+COUNTIF(N50,"●")+COUNTIF(O50,"●"))*B50*D50)</f>
         <v/>
       </c>
       <c r="L51" s="145" t="inlineStr"/>
       <c r="M51" s="145" t="inlineStr"/>
       <c r="N51" s="145" t="inlineStr"/>
       <c r="O51" s="145" t="inlineStr"/>
-      <c r="Q51" s="81">
-        <f>IF(A51="",0,COUNTIF(A$44:A50,A51))</f>
-        <v/>
-      </c>
-      <c r="R51" s="81" t="inlineStr"/>
+      <c r="P51" s="81">
+        <f>IF(A50="",0,COUNTIF(A$44:A49,A50))</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="129" t="inlineStr"/>
       <c r="B52" s="83" t="inlineStr"/>
       <c r="C52" s="84">
-        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D52" s="84">
-        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E52" s="137">
-        <f>IF(D52&gt;0,(D52-C52)/D52,0)</f>
+        <f>IF(D51&gt;0,(D51-C51)/D51,0)</f>
         <v/>
       </c>
       <c r="F52" s="145" t="inlineStr"/>
@@ -5550,399 +5270,461 @@
       <c r="H52" s="145" t="inlineStr"/>
       <c r="I52" s="145" t="inlineStr"/>
       <c r="J52" s="84">
-        <f>IF(A52="","",(COUNTIF(F52,"●")+COUNTIF(G52,"●")+COUNTIF(H52,"●")+COUNTIF(I52,"●")+COUNTIF(L52,"●")+COUNTIF(M52,"●")+COUNTIF(N52,"●")+COUNTIF(O52,"●"))*B52*C52)</f>
+        <f>IF(A51="","",(COUNTIF(F51,"●")+COUNTIF(G51,"●")+COUNTIF(H51,"●")+COUNTIF(I51,"●")+COUNTIF(L51,"●")+COUNTIF(M51,"●")+COUNTIF(N51,"●")+COUNTIF(O51,"●"))*B51*C51)</f>
         <v/>
       </c>
       <c r="K52" s="84">
-        <f>IF(A52="","",(COUNTIF(F52,"●")+COUNTIF(G52,"●")+COUNTIF(H52,"●")+COUNTIF(I52,"●")+COUNTIF(L52,"●")+COUNTIF(M52,"●")+COUNTIF(N52,"●")+COUNTIF(O52,"●"))*B52*D52)</f>
+        <f>IF(A51="","",(COUNTIF(F51,"●")+COUNTIF(G51,"●")+COUNTIF(H51,"●")+COUNTIF(I51,"●")+COUNTIF(L51,"●")+COUNTIF(M51,"●")+COUNTIF(N51,"●")+COUNTIF(O51,"●"))*B51*D51)</f>
         <v/>
       </c>
       <c r="L52" s="145" t="inlineStr"/>
       <c r="M52" s="145" t="inlineStr"/>
       <c r="N52" s="145" t="inlineStr"/>
       <c r="O52" s="145" t="inlineStr"/>
-      <c r="Q52" s="81">
+      <c r="P52" s="81">
+        <f>IF(A51="",0,COUNTIF(A$44:A50,A51))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="129" t="inlineStr"/>
+      <c r="B53" s="83" t="inlineStr"/>
+      <c r="C53" s="84">
+        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D53" s="84">
+        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <v/>
+      </c>
+      <c r="E53" s="137">
+        <f>IF(D52&gt;0,(D52-C52)/D52,0)</f>
+        <v/>
+      </c>
+      <c r="F53" s="145" t="inlineStr"/>
+      <c r="G53" s="145" t="inlineStr"/>
+      <c r="H53" s="145" t="inlineStr"/>
+      <c r="I53" s="145" t="inlineStr"/>
+      <c r="J53" s="84">
+        <f>IF(A52="","",(COUNTIF(F52,"●")+COUNTIF(G52,"●")+COUNTIF(H52,"●")+COUNTIF(I52,"●")+COUNTIF(L52,"●")+COUNTIF(M52,"●")+COUNTIF(N52,"●")+COUNTIF(O52,"●"))*B52*C52)</f>
+        <v/>
+      </c>
+      <c r="K53" s="84">
+        <f>IF(A52="","",(COUNTIF(F52,"●")+COUNTIF(G52,"●")+COUNTIF(H52,"●")+COUNTIF(I52,"●")+COUNTIF(L52,"●")+COUNTIF(M52,"●")+COUNTIF(N52,"●")+COUNTIF(O52,"●"))*B52*D52)</f>
+        <v/>
+      </c>
+      <c r="L53" s="145" t="inlineStr"/>
+      <c r="M53" s="145" t="inlineStr"/>
+      <c r="N53" s="145" t="inlineStr"/>
+      <c r="O53" s="145" t="inlineStr"/>
+      <c r="P53" s="81">
         <f>IF(A52="",0,COUNTIF(A$44:A51,A52))</f>
         <v/>
       </c>
-      <c r="R52" s="81" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="123" t="inlineStr">
+    </row>
+    <row r="54">
+      <c r="A54" s="123" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B53" s="114" t="inlineStr"/>
-      <c r="C53" s="114" t="inlineStr"/>
-      <c r="D53" s="114" t="inlineStr"/>
-      <c r="E53" s="114" t="inlineStr"/>
-      <c r="F53" s="130">
-        <f>IF(F44="●",B44*C44,0)+IF(F45="●",B45*C45,0)+IF(F46="●",B46*C46,0)+IF(F47="●",B47*C47,0)+IF(F48="●",B48*C48,0)+IF(F49="●",B49*C49,0)+IF(F50="●",B50*C50,0)+IF(F51="●",B51*C51,0)+IF(F52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="G53" s="130">
-        <f>IF(G44="●",B44*C44,0)+IF(G45="●",B45*C45,0)+IF(G46="●",B46*C46,0)+IF(G47="●",B47*C47,0)+IF(G48="●",B48*C48,0)+IF(G49="●",B49*C49,0)+IF(G50="●",B50*C50,0)+IF(G51="●",B51*C51,0)+IF(G52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="H53" s="130">
-        <f>IF(H44="●",B44*C44,0)+IF(H45="●",B45*C45,0)+IF(H46="●",B46*C46,0)+IF(H47="●",B47*C47,0)+IF(H48="●",B48*C48,0)+IF(H49="●",B49*C49,0)+IF(H50="●",B50*C50,0)+IF(H51="●",B51*C51,0)+IF(H52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="I53" s="130">
-        <f>IF(I44="●",B44*C44,0)+IF(I45="●",B45*C45,0)+IF(I46="●",B46*C46,0)+IF(I47="●",B47*C47,0)+IF(I48="●",B48*C48,0)+IF(I49="●",B49*C49,0)+IF(I50="●",B50*C50,0)+IF(I51="●",B51*C51,0)+IF(I52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="J53" s="88">
+      <c r="B54" s="114" t="inlineStr"/>
+      <c r="C54" s="114" t="inlineStr"/>
+      <c r="D54" s="114" t="inlineStr"/>
+      <c r="E54" s="114" t="inlineStr"/>
+      <c r="F54" s="130">
+        <f>SUMPRODUCT((F44:F52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="G54" s="130">
+        <f>SUMPRODUCT((G44:G52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="H54" s="130">
+        <f>SUMPRODUCT((H44:H52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="I54" s="130">
+        <f>SUMPRODUCT((I44:I52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="J54" s="88">
         <f>SUM(J44:J52)</f>
         <v/>
       </c>
-      <c r="K53" s="88">
+      <c r="K54" s="88">
         <f>SUM(K44:K52)</f>
         <v/>
       </c>
-      <c r="L53" s="130">
-        <f>IF(L44="●",B44*C44,0)+IF(L45="●",B45*C45,0)+IF(L46="●",B46*C46,0)+IF(L47="●",B47*C47,0)+IF(L48="●",B48*C48,0)+IF(L49="●",B49*C49,0)+IF(L50="●",B50*C50,0)+IF(L51="●",B51*C51,0)+IF(L52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="M53" s="130">
-        <f>IF(M44="●",B44*C44,0)+IF(M45="●",B45*C45,0)+IF(M46="●",B46*C46,0)+IF(M47="●",B47*C47,0)+IF(M48="●",B48*C48,0)+IF(M49="●",B49*C49,0)+IF(M50="●",B50*C50,0)+IF(M51="●",B51*C51,0)+IF(M52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="N53" s="130">
-        <f>IF(N44="●",B44*C44,0)+IF(N45="●",B45*C45,0)+IF(N46="●",B46*C46,0)+IF(N47="●",B47*C47,0)+IF(N48="●",B48*C48,0)+IF(N49="●",B49*C49,0)+IF(N50="●",B50*C50,0)+IF(N51="●",B51*C51,0)+IF(N52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="O53" s="130">
-        <f>IF(O44="●",B44*C44,0)+IF(O45="●",B45*C45,0)+IF(O46="●",B46*C46,0)+IF(O47="●",B47*C47,0)+IF(O48="●",B48*C48,0)+IF(O49="●",B49*C49,0)+IF(O50="●",B50*C50,0)+IF(O51="●",B51*C51,0)+IF(O52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="103" t="inlineStr">
+      <c r="L54" s="130">
+        <f>SUMPRODUCT((L44:L52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="M54" s="130">
+        <f>SUMPRODUCT((M44:M52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="N54" s="130">
+        <f>SUMPRODUCT((N44:N52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="O54" s="130">
+        <f>SUMPRODUCT((O44:O52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57">
+      <c r="A57" s="103" t="inlineStr">
         <is>
           <t>🏆 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B56" s="150" t="n"/>
-      <c r="C56" s="150" t="n"/>
-      <c r="D56" s="150" t="n"/>
-      <c r="E56" s="150" t="n"/>
-      <c r="F56" s="150" t="n"/>
-      <c r="G56" s="150" t="n"/>
-      <c r="H56" s="150" t="n"/>
-      <c r="I56" s="150" t="n"/>
-      <c r="J56" s="150" t="n"/>
-      <c r="K56" s="92" t="n"/>
-    </row>
-    <row r="57">
-      <c r="C57" s="104" t="n"/>
+      <c r="B57" s="150" t="n"/>
+      <c r="C57" s="150" t="n"/>
+      <c r="D57" s="150" t="n"/>
+      <c r="E57" s="150" t="n"/>
+      <c r="F57" s="150" t="n"/>
+      <c r="G57" s="150" t="n"/>
+      <c r="H57" s="150" t="n"/>
+      <c r="I57" s="150" t="n"/>
+      <c r="J57" s="150" t="n"/>
+      <c r="K57" s="92" t="n"/>
     </row>
     <row r="58">
-      <c r="D58" s="104" t="n"/>
+      <c r="A58" s="108" t="inlineStr">
+        <is>
+          <t>GOLF</t>
+        </is>
+      </c>
+      <c r="J58" s="84">
+        <f>J15</f>
+        <v/>
+      </c>
+      <c r="K58" s="84">
+        <f>K15</f>
+        <v/>
+      </c>
+      <c r="L58" s="159" t="inlineStr">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="E59" s="104" t="n"/>
+      <c r="A59" s="108" t="inlineStr">
+        <is>
+          <t>HOTEL</t>
+        </is>
+      </c>
+      <c r="J59" s="84">
+        <f>J21</f>
+        <v/>
+      </c>
+      <c r="K59" s="84">
+        <f>K21</f>
+        <v/>
+      </c>
+      <c r="L59" s="159" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="F60" s="104" t="n"/>
+      <c r="A60" s="108" t="inlineStr">
+        <is>
+          <t>TRANSPORT</t>
+        </is>
+      </c>
+      <c r="J60" s="84">
+        <f>J27</f>
+        <v/>
+      </c>
+      <c r="K60" s="84">
+        <f>K27</f>
+        <v/>
+      </c>
+      <c r="L60" s="159" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="G61" s="104" t="n"/>
+      <c r="A61" s="108" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> MEALS</t>
+        </is>
+      </c>
+      <c r="J61" s="84">
+        <f>J35</f>
+        <v/>
+      </c>
+      <c r="K61" s="84">
+        <f>K35</f>
+        <v/>
+      </c>
+      <c r="L61" s="159" t="inlineStr">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="H62" s="104" t="n"/>
+      <c r="A62" s="108" t="inlineStr">
+        <is>
+          <t>OTHER</t>
+        </is>
+      </c>
+      <c r="J62" s="84">
+        <f>J41</f>
+        <v/>
+      </c>
+      <c r="K62" s="84">
+        <f>K41</f>
+        <v/>
+      </c>
+      <c r="L62" s="159" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="I63" s="104" t="n"/>
+      <c r="A63" s="108" t="inlineStr">
+        <is>
+          <t>ACTIVITIES</t>
+        </is>
+      </c>
+      <c r="J63" s="84">
+        <f>J53</f>
+        <v/>
+      </c>
+      <c r="K63" s="84">
+        <f>K53</f>
+        <v/>
+      </c>
+      <c r="L63" s="159" t="inlineStr">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="J64" s="104" t="n"/>
-    </row>
-    <row r="65">
-      <c r="K65" s="104" t="n"/>
-    </row>
+      <c r="A64" s="115" t="inlineStr">
+        <is>
+          <t>📌 GRAND TOTAL</t>
+        </is>
+      </c>
+      <c r="C64" s="106" t="inlineStr">
+        <is>
+          <t>Margin:</t>
+        </is>
+      </c>
+      <c r="D64" s="91">
+        <f>IF(K63&gt;0,(K63-J63)/K63,0)</f>
+        <v/>
+      </c>
+      <c r="J64" s="88">
+        <f>SUM(J57:J62)</f>
+        <v/>
+      </c>
+      <c r="K64" s="88">
+        <f>SUM(K57:K62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65"/>
     <row r="66">
-      <c r="A66" s="108" t="inlineStr">
-        <is>
-          <t>GOLF</t>
-        </is>
-      </c>
-      <c r="J66" s="84">
-        <f>J15</f>
-        <v/>
-      </c>
-      <c r="K66" s="84">
-        <f>K15</f>
-        <v/>
-      </c>
+      <c r="A66" s="103" t="inlineStr">
+        <is>
+          <t>👤 PER PERSON</t>
+        </is>
+      </c>
+      <c r="B66" s="150" t="n"/>
+      <c r="C66" s="150" t="n"/>
+      <c r="D66" s="150" t="n"/>
+      <c r="E66" s="150" t="n"/>
+      <c r="F66" s="150" t="n"/>
+      <c r="G66" s="150" t="n"/>
+      <c r="H66" s="150" t="n"/>
+      <c r="I66" s="150" t="n"/>
+      <c r="J66" s="150" t="n"/>
+      <c r="K66" s="92" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="108" t="inlineStr">
-        <is>
-          <t>HOTEL</t>
-        </is>
-      </c>
-      <c r="J67" s="84">
-        <f>J21</f>
-        <v/>
-      </c>
-      <c r="K67" s="84">
-        <f>K21</f>
-        <v/>
+      <c r="A67" s="98" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="B67" s="98" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="C67" s="98" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="D67" s="98" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="E67" s="98" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F67" s="98" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="108" t="inlineStr">
-        <is>
-          <t>TRANSPORT</t>
-        </is>
-      </c>
-      <c r="J68" s="84">
-        <f>J27</f>
-        <v/>
-      </c>
-      <c r="K68" s="84">
-        <f>K27</f>
+      <c r="A68" s="108">
+        <f>F2</f>
+        <v/>
+      </c>
+      <c r="B68" s="131">
+        <f>SUMPRODUCT((F10:F14="●")*1,B10:B14,C10:C14)+SUMPRODUCT((F18:F20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((F24:F26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((F30:F34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((F38:F40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((F44:F52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="C68" s="131">
+        <f>SUMPRODUCT((F10:F14="●")*1,B10:B14,D10:D14)+SUMPRODUCT((F18:F20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((F24:F26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((F30:F34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((F38:F40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((F44:F52="●")*1,B44:B52,D44:D52)</f>
+        <v/>
+      </c>
+      <c r="D68" s="110">
+        <f>C67-B67</f>
+        <v/>
+      </c>
+      <c r="E68" s="132">
+        <f>IF(C67&gt;0,D67/C67,0)</f>
+        <v/>
+      </c>
+      <c r="F68" s="139">
+        <f>COUNTIF(F10:F14,"●")+COUNTIF(F18:F20,"●")+COUNTIF(F24:F26,"●")+COUNTIF(F30:F34,"●")+COUNTIF(F38:F40,"●")+COUNTIF(F44:F52,"●")</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="108" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> MEALS</t>
-        </is>
-      </c>
-      <c r="J69" s="84">
-        <f>J35</f>
-        <v/>
-      </c>
-      <c r="K69" s="84">
-        <f>K35</f>
+      <c r="A69" s="108">
+        <f>G2</f>
+        <v/>
+      </c>
+      <c r="B69" s="131">
+        <f>SUMPRODUCT((G10:G14="●")*1,B10:B14,C10:C14)+SUMPRODUCT((G18:G20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((G24:G26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((G30:G34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((G38:G40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((G44:G52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="C69" s="131">
+        <f>SUMPRODUCT((G10:G14="●")*1,B10:B14,D10:D14)+SUMPRODUCT((G18:G20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((G24:G26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((G30:G34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((G38:G40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((G44:G52="●")*1,B44:B52,D44:D52)</f>
+        <v/>
+      </c>
+      <c r="D69" s="110">
+        <f>C68-B68</f>
+        <v/>
+      </c>
+      <c r="E69" s="132">
+        <f>IF(C68&gt;0,D68/C68,0)</f>
+        <v/>
+      </c>
+      <c r="F69" s="139">
+        <f>COUNTIF(G10:G14,"●")+COUNTIF(G18:G20,"●")+COUNTIF(G24:G26,"●")+COUNTIF(G30:G34,"●")+COUNTIF(G38:G40,"●")+COUNTIF(G44:G52,"●")</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="108" t="inlineStr">
-        <is>
-          <t>OTHER</t>
-        </is>
-      </c>
-      <c r="J70" s="84">
-        <f>J41</f>
-        <v/>
-      </c>
-      <c r="K70" s="84">
-        <f>K41</f>
+      <c r="A70" s="108">
+        <f>H2</f>
+        <v/>
+      </c>
+      <c r="B70" s="131">
+        <f>SUMPRODUCT((H10:H14="●")*1,B10:B14,C10:C14)+SUMPRODUCT((H18:H20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((H24:H26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((H30:H34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((H38:H40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((H44:H52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="C70" s="131">
+        <f>SUMPRODUCT((H10:H14="●")*1,B10:B14,D10:D14)+SUMPRODUCT((H18:H20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((H24:H26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((H30:H34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((H38:H40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((H44:H52="●")*1,B44:B52,D44:D52)</f>
+        <v/>
+      </c>
+      <c r="D70" s="110">
+        <f>C69-B69</f>
+        <v/>
+      </c>
+      <c r="E70" s="132">
+        <f>IF(C69&gt;0,D69/C69,0)</f>
+        <v/>
+      </c>
+      <c r="F70" s="139">
+        <f>COUNTIF(H10:H14,"●")+COUNTIF(H18:H20,"●")+COUNTIF(H24:H26,"●")+COUNTIF(H30:H34,"●")+COUNTIF(H38:H40,"●")+COUNTIF(H44:H52,"●")</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="108" t="inlineStr">
-        <is>
-          <t>ACTIVITIES</t>
-        </is>
-      </c>
-      <c r="J71" s="84">
-        <f>J53</f>
-        <v/>
-      </c>
-      <c r="K71" s="84">
-        <f>K53</f>
+      <c r="A71" s="108">
+        <f>I2</f>
+        <v/>
+      </c>
+      <c r="B71" s="131">
+        <f>SUMPRODUCT((I10:I14="●")*1,B10:B14,C10:C14)+SUMPRODUCT((I18:I20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((I24:I26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((I30:I34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((I38:I40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((I44:I52="●")*1,B44:B52,C44:C52)</f>
+        <v/>
+      </c>
+      <c r="C71" s="131">
+        <f>SUMPRODUCT((I10:I14="●")*1,B10:B14,D10:D14)+SUMPRODUCT((I18:I20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((I24:I26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((I30:I34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((I38:I40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((I44:I52="●")*1,B44:B52,D44:D52)</f>
+        <v/>
+      </c>
+      <c r="D71" s="110">
+        <f>C70-B70</f>
+        <v/>
+      </c>
+      <c r="E71" s="132">
+        <f>IF(C70&gt;0,D70/C70,0)</f>
+        <v/>
+      </c>
+      <c r="F71" s="139">
+        <f>COUNTIF(I10:I14,"●")+COUNTIF(I18:I20,"●")+COUNTIF(I24:I26,"●")+COUNTIF(I30:I34,"●")+COUNTIF(I38:I40,"●")+COUNTIF(I44:I52,"●")</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="115" t="inlineStr">
         <is>
-          <t>📌 GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="C72" s="106" t="inlineStr">
-        <is>
-          <t>Margin:</t>
-        </is>
-      </c>
-      <c r="D72" s="91">
-        <f>IF(K72&gt;0,(K72-J72)/K72,0)</f>
-        <v/>
-      </c>
-      <c r="J72" s="88">
-        <f>SUM(J66:J71)</f>
-        <v/>
-      </c>
-      <c r="K72" s="88">
-        <f>SUM(K66:K71)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="103" t="inlineStr">
-        <is>
-          <t>👤 PER PERSON</t>
-        </is>
-      </c>
-      <c r="B74" s="150" t="n"/>
-      <c r="C74" s="150" t="n"/>
-      <c r="D74" s="150" t="n"/>
-      <c r="E74" s="150" t="n"/>
-      <c r="F74" s="150" t="n"/>
-      <c r="G74" s="150" t="n"/>
-      <c r="H74" s="150" t="n"/>
-      <c r="I74" s="150" t="n"/>
-      <c r="J74" s="150" t="n"/>
-      <c r="K74" s="92" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="98" t="inlineStr">
-        <is>
-          <t>Person</t>
-        </is>
-      </c>
-      <c r="B75" s="98" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="C75" s="98" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="D75" s="98" t="inlineStr">
-        <is>
-          <t>Margin</t>
-        </is>
-      </c>
-      <c r="E75" s="98" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="108">
-        <f>F2</f>
-        <v/>
-      </c>
-      <c r="B76" s="131">
-        <f>IF(F10="●",B10*C10,0)+IF(F11="●",B11*C11,0)+IF(F12="●",B12*C12,0)+IF(F13="●",B13*C13,0)+IF(F14="●",B14*C14,0)+IF(F18="●",B18*C18,0)+IF(F19="●",B19*C19,0)+IF(F20="●",B20*C20,0)+IF(F24="●",B24*C24,0)+IF(F25="●",B25*C25,0)+IF(F26="●",B26*C26,0)+IF(F30="●",B30*C30,0)+IF(F31="●",B31*C31,0)+IF(F32="●",B32*C32,0)+IF(F33="●",B33*C33,0)+IF(F34="●",B34*C34,0)+IF(F38="●",B38*C38,0)+IF(F39="●",B39*C39,0)+IF(F40="●",B40*C40,0)+IF(F44="●",B44*C44,0)+IF(F45="●",B45*C45,0)+IF(F46="●",B46*C46,0)+IF(F47="●",B47*C47,0)+IF(F48="●",B48*C48,0)+IF(F49="●",B49*C49,0)+IF(F50="●",B50*C50,0)+IF(F51="●",B51*C51,0)+IF(F52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="C76" s="131">
-        <f>IF(F10="●",B10*D10,0)+IF(F11="●",B11*D11,0)+IF(F12="●",B12*D12,0)+IF(F13="●",B13*D13,0)+IF(F14="●",B14*D14,0)+IF(F18="●",B18*D18,0)+IF(F19="●",B19*D19,0)+IF(F20="●",B20*D20,0)+IF(F24="●",B24*D24,0)+IF(F25="●",B25*D25,0)+IF(F26="●",B26*D26,0)+IF(F30="●",B30*D30,0)+IF(F31="●",B31*D31,0)+IF(F32="●",B32*D32,0)+IF(F33="●",B33*D33,0)+IF(F34="●",B34*D34,0)+IF(F38="●",B38*D38,0)+IF(F39="●",B39*D39,0)+IF(F40="●",B40*D40,0)+IF(F44="●",B44*D44,0)+IF(F45="●",B45*D45,0)+IF(F46="●",B46*D46,0)+IF(F47="●",B47*D47,0)+IF(F48="●",B48*D48,0)+IF(F49="●",B49*D49,0)+IF(F50="●",B50*D50,0)+IF(F51="●",B51*D51,0)+IF(F52="●",B52*D52,0)</f>
-        <v/>
-      </c>
-      <c r="D76" s="110">
-        <f>C85-B85</f>
-        <v/>
-      </c>
-      <c r="E76" s="132">
-        <f>IF(C85&gt;0,D85/C85,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="108">
-        <f>G2</f>
-        <v/>
-      </c>
-      <c r="B77" s="131">
-        <f>IF(G10="●",B10*C10,0)+IF(G11="●",B11*C11,0)+IF(G12="●",B12*C12,0)+IF(G13="●",B13*C13,0)+IF(G14="●",B14*C14,0)+IF(G18="●",B18*C18,0)+IF(G19="●",B19*C19,0)+IF(G20="●",B20*C20,0)+IF(G24="●",B24*C24,0)+IF(G25="●",B25*C25,0)+IF(G26="●",B26*C26,0)+IF(G30="●",B30*C30,0)+IF(G31="●",B31*C31,0)+IF(G32="●",B32*C32,0)+IF(G33="●",B33*C33,0)+IF(G34="●",B34*C34,0)+IF(G38="●",B38*C38,0)+IF(G39="●",B39*C39,0)+IF(G40="●",B40*C40,0)+IF(G44="●",B44*C44,0)+IF(G45="●",B45*C45,0)+IF(G46="●",B46*C46,0)+IF(G47="●",B47*C47,0)+IF(G48="●",B48*C48,0)+IF(G49="●",B49*C49,0)+IF(G50="●",B50*C50,0)+IF(G51="●",B51*C51,0)+IF(G52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="C77" s="131">
-        <f>IF(G10="●",B10*D10,0)+IF(G11="●",B11*D11,0)+IF(G12="●",B12*D12,0)+IF(G13="●",B13*D13,0)+IF(G14="●",B14*D14,0)+IF(G18="●",B18*D18,0)+IF(G19="●",B19*D19,0)+IF(G20="●",B20*D20,0)+IF(G24="●",B24*D24,0)+IF(G25="●",B25*D25,0)+IF(G26="●",B26*D26,0)+IF(G30="●",B30*D30,0)+IF(G31="●",B31*D31,0)+IF(G32="●",B32*D32,0)+IF(G33="●",B33*D33,0)+IF(G34="●",B34*D34,0)+IF(G38="●",B38*D38,0)+IF(G39="●",B39*D39,0)+IF(G40="●",B40*D40,0)+IF(G44="●",B44*D44,0)+IF(G45="●",B45*D45,0)+IF(G46="●",B46*D46,0)+IF(G47="●",B47*D47,0)+IF(G48="●",B48*D48,0)+IF(G49="●",B49*D49,0)+IF(G50="●",B50*D50,0)+IF(G51="●",B51*D51,0)+IF(G52="●",B52*D52,0)</f>
-        <v/>
-      </c>
-      <c r="D77" s="110">
-        <f>C86-B86</f>
-        <v/>
-      </c>
-      <c r="E77" s="132">
-        <f>IF(C86&gt;0,D86/C86,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="108">
-        <f>H2</f>
-        <v/>
-      </c>
-      <c r="B78" s="131">
-        <f>IF(H10="●",B10*C10,0)+IF(H11="●",B11*C11,0)+IF(H12="●",B12*C12,0)+IF(H13="●",B13*C13,0)+IF(H14="●",B14*C14,0)+IF(H18="●",B18*C18,0)+IF(H19="●",B19*C19,0)+IF(H20="●",B20*C20,0)+IF(H24="●",B24*C24,0)+IF(H25="●",B25*C25,0)+IF(H26="●",B26*C26,0)+IF(H30="●",B30*C30,0)+IF(H31="●",B31*C31,0)+IF(H32="●",B32*C32,0)+IF(H33="●",B33*C33,0)+IF(H34="●",B34*C34,0)+IF(H38="●",B38*C38,0)+IF(H39="●",B39*C39,0)+IF(H40="●",B40*C40,0)+IF(H44="●",B44*C44,0)+IF(H45="●",B45*C45,0)+IF(H46="●",B46*C46,0)+IF(H47="●",B47*C47,0)+IF(H48="●",B48*C48,0)+IF(H49="●",B49*C49,0)+IF(H50="●",B50*C50,0)+IF(H51="●",B51*C51,0)+IF(H52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="C78" s="131">
-        <f>IF(H10="●",B10*D10,0)+IF(H11="●",B11*D11,0)+IF(H12="●",B12*D12,0)+IF(H13="●",B13*D13,0)+IF(H14="●",B14*D14,0)+IF(H18="●",B18*D18,0)+IF(H19="●",B19*D19,0)+IF(H20="●",B20*D20,0)+IF(H24="●",B24*D24,0)+IF(H25="●",B25*D25,0)+IF(H26="●",B26*D26,0)+IF(H30="●",B30*D30,0)+IF(H31="●",B31*D31,0)+IF(H32="●",B32*D32,0)+IF(H33="●",B33*D33,0)+IF(H34="●",B34*D34,0)+IF(H38="●",B38*D38,0)+IF(H39="●",B39*D39,0)+IF(H40="●",B40*D40,0)+IF(H44="●",B44*D44,0)+IF(H45="●",B45*D45,0)+IF(H46="●",B46*D46,0)+IF(H47="●",B47*D47,0)+IF(H48="●",B48*D48,0)+IF(H49="●",B49*D49,0)+IF(H50="●",B50*D50,0)+IF(H51="●",B51*D51,0)+IF(H52="●",B52*D52,0)</f>
-        <v/>
-      </c>
-      <c r="D78" s="110">
-        <f>C87-B87</f>
-        <v/>
-      </c>
-      <c r="E78" s="132">
-        <f>IF(C87&gt;0,D87/C87,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="108">
-        <f>I2</f>
-        <v/>
-      </c>
-      <c r="B79" s="131">
-        <f>IF(I10="●",B10*C10,0)+IF(I11="●",B11*C11,0)+IF(I12="●",B12*C12,0)+IF(I13="●",B13*C13,0)+IF(I14="●",B14*C14,0)+IF(I18="●",B18*C18,0)+IF(I19="●",B19*C19,0)+IF(I20="●",B20*C20,0)+IF(I24="●",B24*C24,0)+IF(I25="●",B25*C25,0)+IF(I26="●",B26*C26,0)+IF(I30="●",B30*C30,0)+IF(I31="●",B31*C31,0)+IF(I32="●",B32*C32,0)+IF(I33="●",B33*C33,0)+IF(I34="●",B34*C34,0)+IF(I38="●",B38*C38,0)+IF(I39="●",B39*C39,0)+IF(I40="●",B40*C40,0)+IF(I44="●",B44*C44,0)+IF(I45="●",B45*C45,0)+IF(I46="●",B46*C46,0)+IF(I47="●",B47*C47,0)+IF(I48="●",B48*C48,0)+IF(I49="●",B49*C49,0)+IF(I50="●",B50*C50,0)+IF(I51="●",B51*C51,0)+IF(I52="●",B52*C52,0)</f>
-        <v/>
-      </c>
-      <c r="C79" s="131">
-        <f>IF(I10="●",B10*D10,0)+IF(I11="●",B11*D11,0)+IF(I12="●",B12*D12,0)+IF(I13="●",B13*D13,0)+IF(I14="●",B14*D14,0)+IF(I18="●",B18*D18,0)+IF(I19="●",B19*D19,0)+IF(I20="●",B20*D20,0)+IF(I24="●",B24*D24,0)+IF(I25="●",B25*D25,0)+IF(I26="●",B26*D26,0)+IF(I30="●",B30*D30,0)+IF(I31="●",B31*D31,0)+IF(I32="●",B32*D32,0)+IF(I33="●",B33*D33,0)+IF(I34="●",B34*D34,0)+IF(I38="●",B38*D38,0)+IF(I39="●",B39*D39,0)+IF(I40="●",B40*D40,0)+IF(I44="●",B44*D44,0)+IF(I45="●",B45*D45,0)+IF(I46="●",B46*D46,0)+IF(I47="●",B47*D47,0)+IF(I48="●",B48*D48,0)+IF(I49="●",B49*D49,0)+IF(I50="●",B50*D50,0)+IF(I51="●",B51*D51,0)+IF(I52="●",B52*D52,0)</f>
-        <v/>
-      </c>
-      <c r="D79" s="110">
-        <f>C88-B88</f>
-        <v/>
-      </c>
-      <c r="E79" s="132">
-        <f>IF(C88&gt;0,D88/C88,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="115" t="inlineStr">
-        <is>
           <t>📌 TOTAL</t>
         </is>
       </c>
-      <c r="B80" s="88">
-        <f>SUM(B85:B88)</f>
-        <v/>
-      </c>
-      <c r="C80" s="88">
-        <f>SUM(C85:C88)</f>
-        <v/>
-      </c>
-      <c r="D80" s="88">
-        <f>SUM(D85:D88)</f>
+      <c r="B72" s="88">
+        <f>SUM(B67:B70)</f>
+        <v/>
+      </c>
+      <c r="C72" s="88">
+        <f>SUM(C67:C70)</f>
+        <v/>
+      </c>
+      <c r="D72" s="88">
+        <f>SUM(D67:D70)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A74:K74"/>
     <mergeCell ref="A56:K56"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="A37:K37"/>
     <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A23:K23"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="A29:K29"/>
     <mergeCell ref="E4:H4"/>
     <mergeCell ref="A43:K43"/>
     <mergeCell ref="E6:H6"/>
+    <mergeCell ref="A65:K65"/>
     <mergeCell ref="A17:K17"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A23:K23"/>
+    <mergeCell ref="A37:K37"/>
     <mergeCell ref="A9:K9"/>
   </mergeCells>
   <conditionalFormatting sqref="F10">
@@ -5965,7 +5747,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q10">
+  <conditionalFormatting sqref="P10">
     <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -5990,7 +5772,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q11">
+  <conditionalFormatting sqref="P11">
     <cfRule type="cellIs" priority="10" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6015,7 +5797,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q12">
+  <conditionalFormatting sqref="P12">
     <cfRule type="cellIs" priority="15" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6040,7 +5822,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q13">
+  <conditionalFormatting sqref="P13">
     <cfRule type="cellIs" priority="20" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6065,7 +5847,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q14">
+  <conditionalFormatting sqref="P14">
     <cfRule type="cellIs" priority="25" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6090,7 +5872,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q18">
+  <conditionalFormatting sqref="P18">
     <cfRule type="cellIs" priority="30" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6115,7 +5897,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q19">
+  <conditionalFormatting sqref="P19">
     <cfRule type="cellIs" priority="35" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6140,7 +5922,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q20">
+  <conditionalFormatting sqref="P20">
     <cfRule type="cellIs" priority="40" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6165,7 +5947,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q24">
+  <conditionalFormatting sqref="P24">
     <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6190,7 +5972,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q25">
+  <conditionalFormatting sqref="P25">
     <cfRule type="cellIs" priority="50" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6215,7 +5997,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q26">
+  <conditionalFormatting sqref="P26">
     <cfRule type="cellIs" priority="55" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6240,7 +6022,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q30">
+  <conditionalFormatting sqref="P30">
     <cfRule type="cellIs" priority="60" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6265,7 +6047,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q31">
+  <conditionalFormatting sqref="P31">
     <cfRule type="cellIs" priority="65" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6290,7 +6072,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q32">
+  <conditionalFormatting sqref="P32">
     <cfRule type="cellIs" priority="70" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6315,7 +6097,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q33">
+  <conditionalFormatting sqref="P33">
     <cfRule type="cellIs" priority="75" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6340,7 +6122,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q34">
+  <conditionalFormatting sqref="P34">
     <cfRule type="cellIs" priority="80" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6365,7 +6147,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q38">
+  <conditionalFormatting sqref="P38">
     <cfRule type="cellIs" priority="85" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6390,7 +6172,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q39">
+  <conditionalFormatting sqref="P39">
     <cfRule type="cellIs" priority="90" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6415,7 +6197,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q40">
+  <conditionalFormatting sqref="P40">
     <cfRule type="cellIs" priority="95" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6440,7 +6222,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q44">
+  <conditionalFormatting sqref="P44">
     <cfRule type="cellIs" priority="100" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6465,7 +6247,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q45">
+  <conditionalFormatting sqref="P45">
     <cfRule type="cellIs" priority="105" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6490,7 +6272,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q46">
+  <conditionalFormatting sqref="P46">
     <cfRule type="cellIs" priority="110" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6515,7 +6297,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q47">
+  <conditionalFormatting sqref="P47">
     <cfRule type="cellIs" priority="115" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6540,7 +6322,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q48">
+  <conditionalFormatting sqref="P48">
     <cfRule type="cellIs" priority="120" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6565,7 +6347,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q49">
+  <conditionalFormatting sqref="P49">
     <cfRule type="cellIs" priority="125" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6590,7 +6372,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q50">
+  <conditionalFormatting sqref="P50">
     <cfRule type="cellIs" priority="130" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6615,7 +6397,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q51">
+  <conditionalFormatting sqref="P51">
     <cfRule type="cellIs" priority="135" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6640,7 +6422,7 @@
       <formula>"●"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q52">
+  <conditionalFormatting sqref="P52">
     <cfRule type="cellIs" priority="140" operator="greaterThan" dxfId="3">
       <formula>0</formula>
     </cfRule>
@@ -6663,7 +6445,7 @@
     <dataValidation sqref="D6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>'Master Data'!$A$74:$A$77</formula1>
     </dataValidation>
-    <dataValidation sqref="F10 F11 F12 F13 F14 F18 F19 F20 F24 F25 F26 F30 F31 F32 F33 F34 F38 F39 F40 F44 F45 F46 F47 F48 F49 F50 F51 F52 G10 G11 G12 G13 G14 G18 G19 G20 G24 G25 G26 G30 G31 G32 G33 G34 G38 G39 G40 G44 G45 G46 G47 G48 G49 G50 G51 G52 H10 H11 H12 H13 H14 H18 H19 H20 H24 H25 H26 H30 H31 H32 H33 H34 H38 H39 H40 H44 H45 H46 H47 H48 H49 H50 H51 H52 I10 I11 I12 I13 I14 I18 I19 I20 I24 I25 I26 I30 I31 I32 I33 I34 I38 I39 I40 I44 I45 I46 I47 I48 I49 I50 I51 I52 L10 L11 L12 L13 L14 L18 L19 L20 L24 L25 L26 L30 L31 L32 L33 L34 L38 L39 L40 L44 L45 L46 L47 L48 L49 L50 L51 L52 M10 M11 M12 M13 M14 M18 M19 M20 M24 M25 M26 M30 M31 M32 M33 M34 M38 M39 M40 M44 M45 M46 M47 M48 M49 M50 M51 M52 N10 N11 N12 N13 N14 N18 N19 N20 N24 N25 N26 N30 N31 N32 N33 N34 N38 N39 N40 N44 N45 N46 N47 N48 N49 N50 N51 N52 O10 O11 O12 O13 O14 O18 O19 O20 O24 O25 O26 O30 O31 O32 O33 O34 O38 O39 O40 O44 O45 O46 O47 O48 O49 O50 O51 O52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="● = ON, blank = OFF" type="list">
+    <dataValidation sqref="F10 F11 F12 F13 F14 F18 F19 F20 F24 F25 F26 F30 F31 F32 F33 F34 F38 F39 F40 F44 F45 F46 F47 F48 F49 F50 F51 F52 G10 G11 G12 G13 G14 G18 G19 G20 G24 G25 G26 G30 G31 G32 G33 G34 G38 G39 G40 G44 G45 G46 G47 G48 G49 G50 G51 G52 H10 H11 H12 H13 H14 H18 H19 H20 H24 H25 H26 H30 H31 H32 H33 H34 H38 H39 H40 H44 H45 H46 H47 H48 H49 H50 H51 H52 I10 I11 I12 I13 I14 I18 I19 I20 I24 I25 I26 I30 I31 I32 I33 I34 I38 I39 I40 I44 I45 I46 I47 I48 I49 I50 I51 I52 L10 L11 L12 L13 L14 L18 L19 L20 L24 L25 L26 L30 L31 L32 L33 L34 L38 L39 L40 L44 L45 L46 L47 L48 L49 L50 L51 L52 M10 M11 M12 M13 M14 M18 M19 M20 M24 M25 M26 M30 M31 M32 M33 M34 M38 M39 M40 M44 M45 M46 M47 M48 M49 M50 M51 M52 N10 N11 N12 N13 N14 N18 N19 N20 N24 N25 N26 N30 N31 N32 N33 N34 N38 N39 N40 N44 N45 N46 N47 N48 N49 N50 N51 N52 O10 O11 O12 O13 O14 O18 O19 O20 O24 O25 O26 O30 O31 O32 O33 O34 O38 O39 O40 O44 O45 O46 O47 O48 O49 O50 O51 O52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Toggle" error="● = ON, blank = OFF" type="list">
       <formula1>"●"</formula1>
     </dataValidation>
     <dataValidation sqref="A10 A11 A12 A13 A14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -6709,7 +6491,7 @@
     <row r="1">
       <c r="A1" s="103" t="inlineStr">
         <is>
-          <t>📊 PACKAGE SUMMARY</t>
+          <t>📊 PACKAGE SUMMARY — Current Selection</t>
         </is>
       </c>
       <c r="B1" s="150" t="n"/>
@@ -6928,6 +6710,14 @@
       </c>
       <c r="D11" s="88">
         <f>SUM(D5:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="91">
+        <f>IF(C11&gt;0,D11/C11,0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="88">
+        <f>IF(E2&gt;0,B11/E2,0)</f>
         <v/>
       </c>
     </row>
@@ -6945,7 +6735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="42" min="1" max="1"/>
@@ -6957,13 +6747,14 @@
     <row r="1">
       <c r="A1" s="103" t="inlineStr">
         <is>
-          <t>🎫 GUEST PACKAGE</t>
+          <t>🎫 GUEST PACKAGE — Client Summary</t>
         </is>
       </c>
       <c r="B1" s="150" t="n"/>
       <c r="C1" s="150" t="n"/>
       <c r="D1" s="92" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="106" t="inlineStr">
         <is>
@@ -6987,6 +6778,11 @@
         <f>'Package Selector'!E2</f>
         <v/>
       </c>
+      <c r="C4" s="108" t="inlineStr">
+        <is>
+          <t>persons</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="106" t="inlineStr">
@@ -7001,28 +6797,27 @@
       <c r="C5" s="86" t="n"/>
       <c r="D5" s="87" t="n"/>
     </row>
+    <row r="6"/>
     <row r="7">
-      <c r="A7" s="140" t="inlineStr">
-        <is>
-          <t>⛳ Golf</t>
-        </is>
-      </c>
-      <c r="B7" s="108">
-        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F9:I14,"●")+COUNTIF(L9:O14,"●"))&gt;0,A9:A14,""))</f>
-        <v/>
-      </c>
-      <c r="C7" s="86" t="n"/>
-      <c r="D7" s="87" t="n"/>
+      <c r="A7" s="124" t="inlineStr">
+        <is>
+          <t>📋 PACKAGE INCLUDES</t>
+        </is>
+      </c>
+      <c r="B7" s="150" t="n"/>
+      <c r="C7" s="150" t="n"/>
+      <c r="D7" s="92" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="140" t="inlineStr">
         <is>
-          <t>🏨 Hotel</t>
-        </is>
-      </c>
-      <c r="B8" s="108">
-        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F17:I21,"●")+COUNTIF(L17:O21,"●"))&gt;0,A17:A21,""))</f>
-        <v/>
+          <t>⛳ Golf</t>
+        </is>
+      </c>
+      <c r="B8" s="108" t="inlineStr">
+        <is>
+          <t>(see Package Selector for details)</t>
+        </is>
       </c>
       <c r="C8" s="86" t="n"/>
       <c r="D8" s="87" t="n"/>
@@ -7030,12 +6825,13 @@
     <row r="9">
       <c r="A9" s="140" t="inlineStr">
         <is>
-          <t>🚐 Transport</t>
-        </is>
-      </c>
-      <c r="B9" s="108">
-        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F23:I27,"●")+COUNTIF(L23:O27,"●"))&gt;0,A23:A27,""))</f>
-        <v/>
+          <t>🏨 Hotel</t>
+        </is>
+      </c>
+      <c r="B9" s="108" t="inlineStr">
+        <is>
+          <t>(see Package Selector for details)</t>
+        </is>
       </c>
       <c r="C9" s="86" t="n"/>
       <c r="D9" s="87" t="n"/>
@@ -7043,12 +6839,13 @@
     <row r="10">
       <c r="A10" s="140" t="inlineStr">
         <is>
-          <t>🍽️ Meals</t>
-        </is>
-      </c>
-      <c r="B10" s="108">
-        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F29:I35,"●")+COUNTIF(L29:O35,"●"))&gt;0,A29:A35,""))</f>
-        <v/>
+          <t>🚐 Transport</t>
+        </is>
+      </c>
+      <c r="B10" s="108" t="inlineStr">
+        <is>
+          <t>(see Package Selector for details)</t>
+        </is>
       </c>
       <c r="C10" s="86" t="n"/>
       <c r="D10" s="87" t="n"/>
@@ -7056,12 +6853,13 @@
     <row r="11">
       <c r="A11" s="140" t="inlineStr">
         <is>
-          <t>📦 Other</t>
-        </is>
-      </c>
-      <c r="B11" s="108">
-        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F37:I41,"●")+COUNTIF(L37:O41,"●"))&gt;0,A37:A41,""))</f>
-        <v/>
+          <t>🍽️ Meals</t>
+        </is>
+      </c>
+      <c r="B11" s="108" t="inlineStr">
+        <is>
+          <t>(see Package Selector for details)</t>
+        </is>
       </c>
       <c r="C11" s="86" t="n"/>
       <c r="D11" s="87" t="n"/>
@@ -7069,52 +6867,102 @@
     <row r="12">
       <c r="A12" s="140" t="inlineStr">
         <is>
-          <t>🎯 Activities</t>
-        </is>
-      </c>
-      <c r="B12" s="108">
-        <f>TEXTJOIN(", ",TRUE,IF((COUNTIF(F43:I53,"●")+COUNTIF(L43:O53,"●"))&gt;0,A43:A53,""))</f>
-        <v/>
+          <t>📦 Other</t>
+        </is>
+      </c>
+      <c r="B12" s="108" t="inlineStr">
+        <is>
+          <t>(see Package Selector for details)</t>
+        </is>
       </c>
       <c r="C12" s="86" t="n"/>
       <c r="D12" s="87" t="n"/>
     </row>
-    <row r="14">
-      <c r="A14" s="124" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="140" t="inlineStr">
+        <is>
+          <t>🎯 Activities</t>
+        </is>
+      </c>
+      <c r="B13" s="108" t="inlineStr">
+        <is>
+          <t>(see Package Selector for details)</t>
+        </is>
+      </c>
+      <c r="C13" s="86" t="n"/>
+      <c r="D13" s="87" t="n"/>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="104" t="inlineStr"/>
+      <c r="B15" s="150" t="n"/>
+      <c r="C15" s="150" t="n"/>
+      <c r="D15" s="92" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="124" t="inlineStr">
         <is>
           <t>💰 ALL-INCLUSIVE PRICE</t>
         </is>
       </c>
-      <c r="B14" s="150" t="n"/>
-      <c r="C14" s="150" t="n"/>
-      <c r="D14" s="92" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="106" t="inlineStr">
-        <is>
-          <t>Total:</t>
-        </is>
-      </c>
-      <c r="B15" s="153">
-        <f>'Package Selector'!K72</f>
-        <v/>
-      </c>
-      <c r="C15" s="86" t="n"/>
-      <c r="D15" s="87" t="n"/>
+      <c r="B16" s="150" t="n"/>
+      <c r="C16" s="150" t="n"/>
+      <c r="D16" s="92" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="106" t="inlineStr">
+        <is>
+          <t>Total Package Price:</t>
+        </is>
+      </c>
+      <c r="B17" s="153">
+        <f>'Package Selector'!K63</f>
+        <v/>
+      </c>
+      <c r="C17" s="86" t="n"/>
+      <c r="D17" s="87" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="106" t="inlineStr">
+        <is>
+          <t>Per Person:</t>
+        </is>
+      </c>
+      <c r="B18" s="154">
+        <f>IF(B4&gt;0,B11/B4,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="106" t="inlineStr">
+        <is>
+          <t>Margin:</t>
+        </is>
+      </c>
+      <c r="B19" s="155">
+        <f>B11-B14</f>
+        <v/>
+      </c>
+      <c r="C19" s="156">
+        <f>IF(B11&gt;0,B13/B11,0)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="13">
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B15:D15"/>
     <mergeCell ref="B8:D8"/>
+    <mergeCell ref="B17:D17"/>
     <mergeCell ref="B9:D9"/>
+    <mergeCell ref="A7:D7"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A16:D16"/>
     <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
sync: v3 canonical — remove Package Types, fix 84 off-by-one formulas, fix Guest Package margin
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -7,10 +7,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Types" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Selector" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guest Package" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Selector" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Package Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guest Package" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -3002,523 +3001,10 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FFD4AF37"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" style="42" min="1" max="1"/>
-    <col width="3.7109375" bestFit="1" customWidth="1" style="42" min="2" max="2"/>
-    <col width="5.7109375" bestFit="1" customWidth="1" style="42" min="3" max="3"/>
-    <col width="12" customWidth="1" style="42" min="4" max="4"/>
-    <col width="3" bestFit="1" customWidth="1" style="42" min="5" max="6"/>
-    <col width="4" bestFit="1" customWidth="1" style="42" min="7" max="7"/>
-    <col width="14" customWidth="1" style="42" min="8" max="8"/>
-    <col width="6.28515625" bestFit="1" customWidth="1" style="42" min="9" max="9"/>
-    <col width="6.140625" bestFit="1" customWidth="1" style="42" min="10" max="10"/>
-    <col width="6.28515625" bestFit="1" customWidth="1" style="42" min="11" max="11"/>
-    <col width="6.140625" bestFit="1" customWidth="1" style="42" min="12" max="12"/>
-    <col width="5.140625" bestFit="1" customWidth="1" style="42" min="13" max="13"/>
-    <col width="7.28515625" bestFit="1" customWidth="1" style="42" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="38.25" customHeight="1" s="42">
-      <c r="A1" s="32" t="inlineStr">
-        <is>
-          <t>🎯 결 TOUR — 대표 패키지 (1인 기준, USD | 중복코스 없음)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="37" t="inlineStr">
-        <is>
-          <t>⚠️ 참고용 대표패키지 → 'Package Selector' 시트에서 자유롭게 커스터마이징</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16.5" customHeight="1" s="42">
-      <c r="A4" s="76" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B4" s="76" t="inlineStr">
-        <is>
-          <t>일정</t>
-        </is>
-      </c>
-      <c r="C4" s="76" t="inlineStr">
-        <is>
-          <t>패키지명</t>
-        </is>
-      </c>
-      <c r="D4" s="76" t="inlineStr">
-        <is>
-          <t>박</t>
-        </is>
-      </c>
-      <c r="E4" s="76" t="inlineStr">
-        <is>
-          <t>일</t>
-        </is>
-      </c>
-      <c r="F4" s="76" t="inlineStr">
-        <is>
-          <t>Rds</t>
-        </is>
-      </c>
-      <c r="G4" s="76" t="inlineStr">
-        <is>
-          <t>패키지 구성</t>
-        </is>
-      </c>
-      <c r="H4" s="77" t="inlineStr">
-        <is>
-          <t>⛳ 골프</t>
-        </is>
-      </c>
-      <c r="I4" s="92" t="n"/>
-      <c r="J4" s="92" t="n"/>
-      <c r="K4" s="92" t="n"/>
-      <c r="L4" s="92" t="n"/>
-      <c r="M4" s="92" t="n"/>
-      <c r="N4" s="92" t="n"/>
-      <c r="O4" s="92" t="n"/>
-      <c r="P4" s="77" t="inlineStr">
-        <is>
-          <t>🍽️ 식사</t>
-        </is>
-      </c>
-      <c r="Q4" s="92" t="n"/>
-      <c r="R4" s="77" t="inlineStr">
-        <is>
-          <t>📦 기타</t>
-        </is>
-      </c>
-      <c r="S4" s="92" t="n"/>
-      <c r="T4" s="76" t="inlineStr">
-        <is>
-          <t>마진</t>
-        </is>
-      </c>
-      <c r="U4" s="76" t="inlineStr">
-        <is>
-          <t>마진율</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="51" customHeight="1" s="42">
-      <c r="A5" s="78" t="n"/>
-      <c r="B5" s="78" t="n"/>
-      <c r="C5" s="78" t="n"/>
-      <c r="D5" s="78" t="n"/>
-      <c r="E5" s="78" t="n"/>
-      <c r="F5" s="78" t="n"/>
-      <c r="G5" s="78" t="n"/>
-      <c r="H5" s="148" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="I5" s="148" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="J5" s="148" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="K5" s="148" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="L5" s="148" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="M5" s="148" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="N5" s="148" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="O5" s="148" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="P5" s="148" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="Q5" s="148" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="R5" s="148" t="inlineStr">
-        <is>
-          <t>Cost</t>
-        </is>
-      </c>
-      <c r="S5" s="148" t="inlineStr">
-        <is>
-          <t>Sell</t>
-        </is>
-      </c>
-      <c r="T5" s="148" t="inlineStr"/>
-      <c r="U5" s="148" t="inlineStr"/>
-    </row>
-    <row r="6" ht="51" customHeight="1" s="42">
-      <c r="A6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>3N4D</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>트럼프 + 샌드파이퍼 오션뷰</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Trump×1 + Sand×1</t>
-        </is>
-      </c>
-      <c r="H6" s="149" t="inlineStr">
-        <is>
-          <t>G2·H3·T3·M3B3L3D2Ex·I4</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>745</v>
-      </c>
-      <c r="J6" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="79" t="n">
-        <v>120</v>
-      </c>
-      <c r="L6" s="5" t="n">
-        <v>825</v>
-      </c>
-      <c r="M6" s="5" t="n">
-        <v>1125</v>
-      </c>
-      <c r="N6" s="79" t="n">
-        <v>375</v>
-      </c>
-      <c r="O6" s="79" t="n">
-        <v>525</v>
-      </c>
-      <c r="P6" s="79" t="n">
-        <v>810</v>
-      </c>
-      <c r="Q6" s="79" t="n">
-        <v>1215</v>
-      </c>
-      <c r="R6" s="79" t="n">
-        <v>200</v>
-      </c>
-      <c r="S6" s="79" t="n">
-        <v>300</v>
-      </c>
-      <c r="T6" s="79">
-        <f>(J6+L6+N6+P6+R6+T6)-(I6+K6+M6+O6+Q6+S6)</f>
-        <v/>
-      </c>
-      <c r="U6" s="80">
-        <f>IF(J6+L6+N6+P6+R6+T6&gt;0,((J6+L6+N6+P6+R6+T6)-(I6+K6+M6+O6+Q6+S6))/(J6+L6+N6+P6+R6+T6),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="34.5" customHeight="1" s="42">
-      <c r="A7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>3N4D</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>트럼프 + 히든밸리 밸리뷰</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Trump×1 + HV×1</t>
-        </is>
-      </c>
-      <c r="H7" s="149" t="inlineStr">
-        <is>
-          <t>G2·H3·T3·M3B3L3D2Ex·I4</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>609</v>
-      </c>
-      <c r="J7" s="79" t="n">
-        <v>45</v>
-      </c>
-      <c r="K7" s="79" t="n">
-        <v>45</v>
-      </c>
-      <c r="L7" s="5" t="n">
-        <v>825</v>
-      </c>
-      <c r="M7" s="5" t="n">
-        <v>1125</v>
-      </c>
-      <c r="N7" s="79" t="n">
-        <v>375</v>
-      </c>
-      <c r="O7" s="79" t="n">
-        <v>525</v>
-      </c>
-      <c r="P7" s="79" t="n">
-        <v>810</v>
-      </c>
-      <c r="Q7" s="79" t="n">
-        <v>1215</v>
-      </c>
-      <c r="R7" s="79" t="n">
-        <v>200</v>
-      </c>
-      <c r="S7" s="79" t="n">
-        <v>300</v>
-      </c>
-      <c r="T7" s="79">
-        <f>(J7+L7+N7+P7+R7+T7)-(I7+K7+M7+O7+Q7+S7)</f>
-        <v/>
-      </c>
-      <c r="U7" s="80">
-        <f>IF(J7+L7+N7+P7+R7+T7&gt;0,((J7+L7+N7+P7+R7+T7)-(I7+K7+M7+O7+Q7+S7))/(J7+L7+N7+P7+R7+T7),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>3N4D</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>샌드파이퍼 + 히든밸리</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Sand×1 + HV×1</t>
-        </is>
-      </c>
-      <c r="H8" s="149" t="inlineStr">
-        <is>
-          <t>G2·H3·T3·M3B3L3D2Ex·I4</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>354</v>
-      </c>
-      <c r="J8" s="79" t="n">
-        <v>45</v>
-      </c>
-      <c r="K8" s="79" t="n">
-        <v>45</v>
-      </c>
-      <c r="L8" s="5" t="n">
-        <v>825</v>
-      </c>
-      <c r="M8" s="5" t="n">
-        <v>1125</v>
-      </c>
-      <c r="N8" s="79" t="n">
-        <v>375</v>
-      </c>
-      <c r="O8" s="79" t="n">
-        <v>525</v>
-      </c>
-      <c r="P8" s="79" t="n">
-        <v>810</v>
-      </c>
-      <c r="Q8" s="79" t="n">
-        <v>1215</v>
-      </c>
-      <c r="R8" s="79" t="n">
-        <v>200</v>
-      </c>
-      <c r="S8" s="79" t="n">
-        <v>300</v>
-      </c>
-      <c r="T8" s="79">
-        <f>(J8+L8+N8+P8+R8+T8)-(I8+K8+M8+O8+Q8+S8)</f>
-        <v/>
-      </c>
-      <c r="U8" s="80">
-        <f>IF(J8+L8+N8+P8+R8+T8&gt;0,((J8+L8+N8+P8+R8+T8)-(I8+K8+M8+O8+Q8+S8))/(J8+L8+N8+P8+R8+T8),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="51" customHeight="1" s="42">
-      <c r="A9" s="10" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
-      <c r="H9" s="10" t="n"/>
-      <c r="I9" s="10" t="n"/>
-      <c r="L9" s="10" t="n"/>
-      <c r="M9" s="10" t="n"/>
-      <c r="T9" s="10" t="n"/>
-      <c r="U9" s="10" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>5N7D</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>트럼프+샌드+히든 3色 시그니처</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Trump×1+Sand×1+HV×1</t>
-        </is>
-      </c>
-      <c r="H10" s="149" t="inlineStr">
-        <is>
-          <t>G3·H5·T5·M5B5L5D2Ex·I5</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>854</v>
-      </c>
-      <c r="J10" s="79" t="n">
-        <v>45</v>
-      </c>
-      <c r="K10" s="79" t="n">
-        <v>165</v>
-      </c>
-      <c r="L10" s="5" t="n">
-        <v>1375</v>
-      </c>
-      <c r="M10" s="5" t="n">
-        <v>1875</v>
-      </c>
-      <c r="N10" s="79" t="n">
-        <v>625</v>
-      </c>
-      <c r="O10" s="79" t="n">
-        <v>875</v>
-      </c>
-      <c r="P10" s="79" t="n">
-        <v>1350</v>
-      </c>
-      <c r="Q10" s="79" t="n">
-        <v>2025</v>
-      </c>
-      <c r="R10" s="79" t="n">
-        <v>250</v>
-      </c>
-      <c r="S10" s="79" t="n">
-        <v>375</v>
-      </c>
-      <c r="T10" s="79">
-        <f>(J10+L10+N10+P10+R10+T10)-(I10+K10+M10+O10+Q10+S10)</f>
-        <v/>
-      </c>
-      <c r="U10" s="80">
-        <f>IF(J10+L10+N10+P10+R10+T10&gt;0,((J10+L10+N10+P10+R10+T10)-(I10+K10+M10+O10+Q10+S10))/(J10+L10+N10+P10+R10+T10),0)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="A1:U1"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="R4:S4"/>
-    <mergeCell ref="N4:O4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:R72"/>
+  <dimension ref="A1:P72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="42" min="1" max="1"/>
@@ -3599,16 +3085,16 @@
           <t>💰 CHARGE LEGEND:  PP=Per Person  |  PG=Per Group(1회청구)  |  P2=2인1실  |  P4=4인1조</t>
         </is>
       </c>
-      <c r="B3" s="158" t="n"/>
-      <c r="C3" s="158" t="n"/>
-      <c r="D3" s="158" t="n"/>
-      <c r="E3" s="158" t="n"/>
-      <c r="F3" s="158" t="n"/>
-      <c r="G3" s="158" t="n"/>
-      <c r="H3" s="158" t="n"/>
-      <c r="I3" s="158" t="n"/>
-      <c r="J3" s="158" t="n"/>
-      <c r="K3" s="158" t="n"/>
+      <c r="B3" s="86" t="n"/>
+      <c r="C3" s="86" t="n"/>
+      <c r="D3" s="86" t="n"/>
+      <c r="E3" s="86" t="n"/>
+      <c r="F3" s="86" t="n"/>
+      <c r="G3" s="86" t="n"/>
+      <c r="H3" s="86" t="n"/>
+      <c r="I3" s="86" t="n"/>
+      <c r="J3" s="86" t="n"/>
+      <c r="K3" s="87" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="128" t="inlineStr">
@@ -3633,38 +3119,16 @@
           <t>Date:</t>
         </is>
       </c>
-      <c r="B5" s="82" t="inlineStr">
-        <is>
-          <t>2026-05-25</t>
-        </is>
-      </c>
-      <c r="C5" s="106" t="inlineStr">
-        <is>
-          <t>Flight:</t>
-        </is>
-      </c>
-      <c r="D5" s="82" t="inlineStr">
-        <is>
-          <t>KE011</t>
-        </is>
-      </c>
-      <c r="E5" s="144">
-        <f>IF(D4="","",VLOOKUP(D4,'Master Data'!$A$60:$D$63,3,FALSE))&amp;" → "&amp;IF(D4="","",VLOOKUP(D4,'Master Data'!$A$60:$D$63,4,FALSE))</f>
-        <v/>
-      </c>
+      <c r="B5" s="86" t="n"/>
+      <c r="C5" s="86" t="n"/>
+      <c r="D5" s="86" t="n"/>
+      <c r="E5" s="86" t="n"/>
       <c r="F5" s="86" t="n"/>
       <c r="G5" s="86" t="n"/>
-      <c r="H5" s="87" t="n"/>
-      <c r="I5" s="106" t="inlineStr">
-        <is>
-          <t>Seat:</t>
-        </is>
-      </c>
-      <c r="J5" s="82" t="inlineStr">
-        <is>
-          <t>Economy</t>
-        </is>
-      </c>
+      <c r="H5" s="86" t="n"/>
+      <c r="I5" s="86" t="n"/>
+      <c r="J5" s="86" t="n"/>
+      <c r="K5" s="87" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="128" t="inlineStr">
@@ -3680,7 +3144,7 @@
       <c r="G6" s="150" t="n"/>
       <c r="H6" s="150" t="n"/>
       <c r="I6" s="150" t="n"/>
-      <c r="J6" s="150" t="n"/>
+      <c r="J6" s="92" t="n"/>
       <c r="K6" s="92" t="n"/>
     </row>
     <row r="7">
@@ -3766,52 +3230,16 @@
           <t>Item ▼</t>
         </is>
       </c>
-      <c r="B9" s="98" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="C9" s="98" t="inlineStr">
-        <is>
-          <t>Cost/P</t>
-        </is>
-      </c>
-      <c r="D9" s="98" t="inlineStr">
-        <is>
-          <t>Sell/P</t>
-        </is>
-      </c>
-      <c r="E9" s="98" t="inlineStr">
-        <is>
-          <t>M%</t>
-        </is>
-      </c>
-      <c r="F9" s="98">
-        <f>F2</f>
-        <v/>
-      </c>
-      <c r="G9" s="98">
-        <f>G2</f>
-        <v/>
-      </c>
-      <c r="H9" s="98">
-        <f>H2</f>
-        <v/>
-      </c>
-      <c r="I9" s="98">
-        <f>I2</f>
-        <v/>
-      </c>
-      <c r="J9" s="98" t="inlineStr">
-        <is>
-          <t>TotCost</t>
-        </is>
-      </c>
-      <c r="K9" s="98" t="inlineStr">
-        <is>
-          <t>TotSell</t>
-        </is>
-      </c>
+      <c r="B9" s="86" t="n"/>
+      <c r="C9" s="86" t="n"/>
+      <c r="D9" s="86" t="n"/>
+      <c r="E9" s="86" t="n"/>
+      <c r="F9" s="86" t="n"/>
+      <c r="G9" s="86" t="n"/>
+      <c r="H9" s="86" t="n"/>
+      <c r="I9" s="86" t="n"/>
+      <c r="J9" s="86" t="n"/>
+      <c r="K9" s="87" t="n"/>
       <c r="L9" s="98" t="inlineStr">
         <is>
           <t>P5</t>
@@ -3870,15 +3298,15 @@
         <v>1</v>
       </c>
       <c r="C11" s="84">
-        <f>IF(A10="","",VLOOKUP(A10,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D11" s="84">
-        <f>IF(A10="","",VLOOKUP(A10,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E11" s="137">
-        <f>IF(D10&gt;0,(D10-C10)/D10,0)</f>
+        <f>IF(D11&gt;0,(D11-C11)/D11,0)</f>
         <v/>
       </c>
       <c r="F11" s="145" t="inlineStr"/>
@@ -3912,15 +3340,15 @@
         <v>2</v>
       </c>
       <c r="C12" s="84">
-        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D12" s="84">
-        <f>IF(A11="","",VLOOKUP(A11,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E12" s="137">
-        <f>IF(D11&gt;0,(D11-C11)/D11,0)</f>
+        <f>IF(D12&gt;0,(D12-C12)/D12,0)</f>
         <v/>
       </c>
       <c r="F12" s="145" t="inlineStr"/>
@@ -3954,15 +3382,15 @@
         <v>2</v>
       </c>
       <c r="C13" s="84">
-        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D13" s="84">
-        <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E13" s="137">
-        <f>IF(D12&gt;0,(D12-C12)/D12,0)</f>
+        <f>IF(D13&gt;0,(D13-C13)/D13,0)</f>
         <v/>
       </c>
       <c r="F13" s="145" t="inlineStr"/>
@@ -3990,15 +3418,15 @@
       <c r="A14" s="129" t="inlineStr"/>
       <c r="B14" s="83" t="inlineStr"/>
       <c r="C14" s="84">
-        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D14" s="84">
-        <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E14" s="137">
-        <f>IF(D13&gt;0,(D13-C13)/D13,0)</f>
+        <f>IF(D14&gt;0,(D14-C14)/D14,0)</f>
         <v/>
       </c>
       <c r="F14" s="145" t="inlineStr"/>
@@ -4026,15 +3454,15 @@
       <c r="A15" s="129" t="inlineStr"/>
       <c r="B15" s="83" t="inlineStr"/>
       <c r="C15" s="84">
-        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,2,FALSE))</f>
+        <f>IF(A15="","",VLOOKUP(A15,'Master Data'!$A$7:$C$14,2,FALSE))</f>
         <v/>
       </c>
       <c r="D15" s="84">
-        <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$7:$C$14,3,FALSE))</f>
+        <f>IF(A15="","",VLOOKUP(A15,'Master Data'!$A$7:$C$14,3,FALSE))</f>
         <v/>
       </c>
       <c r="E15" s="137">
-        <f>IF(D14&gt;0,(D14-C14)/D14,0)</f>
+        <f>IF(D15&gt;0,(D15-C15)/D15,0)</f>
         <v/>
       </c>
       <c r="F15" s="145" t="inlineStr"/>
@@ -4142,15 +3570,15 @@
         <v>3</v>
       </c>
       <c r="C19" s="84">
-        <f>IF(A18="","",VLOOKUP(A18,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,2,FALSE))</f>
         <v/>
       </c>
       <c r="D19" s="84">
-        <f>IF(A18="","",VLOOKUP(A18,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
       <c r="E19" s="137">
-        <f>IF(D18&gt;0,(D18-C18)/D18,0)</f>
+        <f>IF(D19&gt;0,(D19-C19)/D19,0)</f>
         <v/>
       </c>
       <c r="F19" s="145" t="inlineStr"/>
@@ -4178,15 +3606,15 @@
       <c r="A20" s="129" t="inlineStr"/>
       <c r="B20" s="83" t="inlineStr"/>
       <c r="C20" s="84">
-        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,2,FALSE))</f>
         <v/>
       </c>
       <c r="D20" s="84">
-        <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
       <c r="E20" s="137">
-        <f>IF(D19&gt;0,(D19-C19)/D19,0)</f>
+        <f>IF(D20&gt;0,(D20-C20)/D20,0)</f>
         <v/>
       </c>
       <c r="F20" s="145" t="inlineStr"/>
@@ -4214,15 +3642,15 @@
       <c r="A21" s="129" t="inlineStr"/>
       <c r="B21" s="83" t="inlineStr"/>
       <c r="C21" s="84">
-        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,2,FALSE))</f>
+        <f>IF(A21="","",VLOOKUP(A21,'Master Data'!$A$19:$C$24,2,FALSE))</f>
         <v/>
       </c>
       <c r="D21" s="84">
-        <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$19:$C$24,3,FALSE))</f>
+        <f>IF(A21="","",VLOOKUP(A21,'Master Data'!$A$19:$C$24,3,FALSE))</f>
         <v/>
       </c>
       <c r="E21" s="137">
-        <f>IF(D20&gt;0,(D20-C20)/D20,0)</f>
+        <f>IF(D21&gt;0,(D21-C21)/D21,0)</f>
         <v/>
       </c>
       <c r="F21" s="145" t="inlineStr"/>
@@ -4330,15 +3758,15 @@
         <v>3</v>
       </c>
       <c r="C25" s="84">
-        <f>IF(A24="","",VLOOKUP(A24,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,2,FALSE))</f>
         <v/>
       </c>
       <c r="D25" s="84">
-        <f>IF(A24="","",VLOOKUP(A24,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
       <c r="E25" s="137">
-        <f>IF(D24&gt;0,(D24-C24)/D24,0)</f>
+        <f>IF(D25&gt;0,(D25-C25)/D25,0)</f>
         <v/>
       </c>
       <c r="F25" s="145" t="inlineStr"/>
@@ -4366,15 +3794,15 @@
       <c r="A26" s="129" t="inlineStr"/>
       <c r="B26" s="83" t="inlineStr"/>
       <c r="C26" s="84">
-        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,2,FALSE))</f>
         <v/>
       </c>
       <c r="D26" s="84">
-        <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
       <c r="E26" s="137">
-        <f>IF(D25&gt;0,(D25-C25)/D25,0)</f>
+        <f>IF(D26&gt;0,(D26-C26)/D26,0)</f>
         <v/>
       </c>
       <c r="F26" s="145" t="inlineStr"/>
@@ -4402,15 +3830,15 @@
       <c r="A27" s="129" t="inlineStr"/>
       <c r="B27" s="83" t="inlineStr"/>
       <c r="C27" s="84">
-        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,2,FALSE))</f>
+        <f>IF(A27="","",VLOOKUP(A27,'Master Data'!$A$28:$C$34,2,FALSE))</f>
         <v/>
       </c>
       <c r="D27" s="84">
-        <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$28:$C$34,3,FALSE))</f>
+        <f>IF(A27="","",VLOOKUP(A27,'Master Data'!$A$28:$C$34,3,FALSE))</f>
         <v/>
       </c>
       <c r="E27" s="137">
-        <f>IF(D26&gt;0,(D26-C26)/D26,0)</f>
+        <f>IF(D27&gt;0,(D27-C27)/D27,0)</f>
         <v/>
       </c>
       <c r="F27" s="145" t="inlineStr"/>
@@ -4518,15 +3946,15 @@
         <v>3</v>
       </c>
       <c r="C31" s="84">
-        <f>IF(A30="","",VLOOKUP(A30,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D31" s="84">
-        <f>IF(A30="","",VLOOKUP(A30,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E31" s="137">
-        <f>IF(D30&gt;0,(D30-C30)/D30,0)</f>
+        <f>IF(D31&gt;0,(D31-C31)/D31,0)</f>
         <v/>
       </c>
       <c r="F31" s="145" t="inlineStr"/>
@@ -4560,15 +3988,15 @@
         <v>3</v>
       </c>
       <c r="C32" s="84">
-        <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D32" s="84">
-        <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E32" s="137">
-        <f>IF(D31&gt;0,(D31-C31)/D31,0)</f>
+        <f>IF(D32&gt;0,(D32-C32)/D32,0)</f>
         <v/>
       </c>
       <c r="F32" s="145" t="inlineStr"/>
@@ -4602,15 +4030,15 @@
         <v>2</v>
       </c>
       <c r="C33" s="84">
-        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D33" s="84">
-        <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E33" s="137">
-        <f>IF(D32&gt;0,(D32-C32)/D32,0)</f>
+        <f>IF(D33&gt;0,(D33-C33)/D33,0)</f>
         <v/>
       </c>
       <c r="F33" s="145" t="inlineStr"/>
@@ -4644,15 +4072,15 @@
         <v>3</v>
       </c>
       <c r="C34" s="84">
-        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D34" s="84">
-        <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E34" s="137">
-        <f>IF(D33&gt;0,(D33-C33)/D33,0)</f>
+        <f>IF(D34&gt;0,(D34-C34)/D34,0)</f>
         <v/>
       </c>
       <c r="F34" s="145" t="inlineStr"/>
@@ -4680,15 +4108,15 @@
       <c r="A35" s="129" t="inlineStr"/>
       <c r="B35" s="83" t="inlineStr"/>
       <c r="C35" s="84">
-        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,2,FALSE))</f>
+        <f>IF(A35="","",VLOOKUP(A35,'Master Data'!$A$38:$C$46,2,FALSE))</f>
         <v/>
       </c>
       <c r="D35" s="84">
-        <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$38:$C$46,3,FALSE))</f>
+        <f>IF(A35="","",VLOOKUP(A35,'Master Data'!$A$38:$C$46,3,FALSE))</f>
         <v/>
       </c>
       <c r="E35" s="137">
-        <f>IF(D34&gt;0,(D34-C34)/D34,0)</f>
+        <f>IF(D35&gt;0,(D35-C35)/D35,0)</f>
         <v/>
       </c>
       <c r="F35" s="145" t="inlineStr"/>
@@ -4796,15 +4224,15 @@
         <v>4</v>
       </c>
       <c r="C39" s="84">
-        <f>IF(A38="","",VLOOKUP(A38,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,2,FALSE))</f>
         <v/>
       </c>
       <c r="D39" s="84">
-        <f>IF(A38="","",VLOOKUP(A38,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
       <c r="E39" s="137">
-        <f>IF(D38&gt;0,(D38-C38)/D38,0)</f>
+        <f>IF(D39&gt;0,(D39-C39)/D39,0)</f>
         <v/>
       </c>
       <c r="F39" s="145" t="inlineStr"/>
@@ -4832,15 +4260,15 @@
       <c r="A40" s="129" t="inlineStr"/>
       <c r="B40" s="83" t="inlineStr"/>
       <c r="C40" s="84">
-        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,2,FALSE))</f>
         <v/>
       </c>
       <c r="D40" s="84">
-        <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
       <c r="E40" s="137">
-        <f>IF(D39&gt;0,(D39-C39)/D39,0)</f>
+        <f>IF(D40&gt;0,(D40-C40)/D40,0)</f>
         <v/>
       </c>
       <c r="F40" s="145" t="inlineStr"/>
@@ -4868,15 +4296,15 @@
       <c r="A41" s="129" t="inlineStr"/>
       <c r="B41" s="83" t="inlineStr"/>
       <c r="C41" s="84">
-        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,2,FALSE))</f>
+        <f>IF(A41="","",VLOOKUP(A41,'Master Data'!$A$50:$C$56,2,FALSE))</f>
         <v/>
       </c>
       <c r="D41" s="84">
-        <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$50:$C$56,3,FALSE))</f>
+        <f>IF(A41="","",VLOOKUP(A41,'Master Data'!$A$50:$C$56,3,FALSE))</f>
         <v/>
       </c>
       <c r="E41" s="137">
-        <f>IF(D40&gt;0,(D40-C40)/D40,0)</f>
+        <f>IF(D41&gt;0,(D41-C41)/D41,0)</f>
         <v/>
       </c>
       <c r="F41" s="145" t="inlineStr"/>
@@ -4984,15 +4412,15 @@
         <v>1</v>
       </c>
       <c r="C45" s="84">
-        <f>IF(A44="","",VLOOKUP(A44,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D45" s="84">
-        <f>IF(A44="","",VLOOKUP(A44,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E45" s="137">
-        <f>IF(D44&gt;0,(D44-C44)/D44,0)</f>
+        <f>IF(D45&gt;0,(D45-C45)/D45,0)</f>
         <v/>
       </c>
       <c r="F45" s="145" t="inlineStr"/>
@@ -5026,15 +4454,15 @@
         <v>1</v>
       </c>
       <c r="C46" s="84">
-        <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D46" s="84">
-        <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E46" s="137">
-        <f>IF(D45&gt;0,(D45-C45)/D45,0)</f>
+        <f>IF(D46&gt;0,(D46-C46)/D46,0)</f>
         <v/>
       </c>
       <c r="F46" s="145" t="inlineStr"/>
@@ -5068,15 +4496,15 @@
         <v>1</v>
       </c>
       <c r="C47" s="84">
-        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D47" s="84">
-        <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E47" s="137">
-        <f>IF(D46&gt;0,(D46-C46)/D46,0)</f>
+        <f>IF(D47&gt;0,(D47-C47)/D47,0)</f>
         <v/>
       </c>
       <c r="F47" s="145" t="inlineStr"/>
@@ -5110,15 +4538,15 @@
         <v>1</v>
       </c>
       <c r="C48" s="84">
-        <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D48" s="84">
-        <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E48" s="137">
-        <f>IF(D47&gt;0,(D47-C47)/D47,0)</f>
+        <f>IF(D48&gt;0,(D48-C48)/D48,0)</f>
         <v/>
       </c>
       <c r="F48" s="145" t="inlineStr"/>
@@ -5146,15 +4574,15 @@
       <c r="A49" s="129" t="inlineStr"/>
       <c r="B49" s="83" t="inlineStr"/>
       <c r="C49" s="84">
-        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D49" s="84">
-        <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E49" s="137">
-        <f>IF(D48&gt;0,(D48-C48)/D48,0)</f>
+        <f>IF(D49&gt;0,(D49-C49)/D49,0)</f>
         <v/>
       </c>
       <c r="F49" s="145" t="inlineStr"/>
@@ -5182,15 +4610,15 @@
       <c r="A50" s="129" t="inlineStr"/>
       <c r="B50" s="83" t="inlineStr"/>
       <c r="C50" s="84">
-        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D50" s="84">
-        <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E50" s="137">
-        <f>IF(D49&gt;0,(D49-C49)/D49,0)</f>
+        <f>IF(D50&gt;0,(D50-C50)/D50,0)</f>
         <v/>
       </c>
       <c r="F50" s="145" t="inlineStr"/>
@@ -5218,15 +4646,15 @@
       <c r="A51" s="129" t="inlineStr"/>
       <c r="B51" s="83" t="inlineStr"/>
       <c r="C51" s="84">
-        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D51" s="84">
-        <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E51" s="137">
-        <f>IF(D50&gt;0,(D50-C50)/D50,0)</f>
+        <f>IF(D51&gt;0,(D51-C51)/D51,0)</f>
         <v/>
       </c>
       <c r="F51" s="145" t="inlineStr"/>
@@ -5254,15 +4682,15 @@
       <c r="A52" s="129" t="inlineStr"/>
       <c r="B52" s="83" t="inlineStr"/>
       <c r="C52" s="84">
-        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D52" s="84">
-        <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E52" s="137">
-        <f>IF(D51&gt;0,(D51-C51)/D51,0)</f>
+        <f>IF(D52&gt;0,(D52-C52)/D52,0)</f>
         <v/>
       </c>
       <c r="F52" s="145" t="inlineStr"/>
@@ -5290,15 +4718,15 @@
       <c r="A53" s="129" t="inlineStr"/>
       <c r="B53" s="83" t="inlineStr"/>
       <c r="C53" s="84">
-        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,2,FALSE))</f>
+        <f>IF(A53="","",VLOOKUP(A53,'Master Data'!$A$86:$C$94,2,FALSE))</f>
         <v/>
       </c>
       <c r="D53" s="84">
-        <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$86:$C$94,3,FALSE))</f>
+        <f>IF(A53="","",VLOOKUP(A53,'Master Data'!$A$86:$C$94,3,FALSE))</f>
         <v/>
       </c>
       <c r="E53" s="137">
-        <f>IF(D52&gt;0,(D52-C52)/D52,0)</f>
+        <f>IF(D53&gt;0,(D53-C53)/D53,0)</f>
         <v/>
       </c>
       <c r="F53" s="145" t="inlineStr"/>
@@ -6471,7 +5899,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6729,13 +6157,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="42" min="1" max="1"/>
@@ -6754,7 +6182,6 @@
       <c r="C1" s="150" t="n"/>
       <c r="D1" s="92" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="106" t="inlineStr">
         <is>
@@ -6797,7 +6224,6 @@
       <c r="C5" s="86" t="n"/>
       <c r="D5" s="87" t="n"/>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="124" t="inlineStr">
         <is>
@@ -6892,7 +6318,6 @@
       <c r="C13" s="86" t="n"/>
       <c r="D13" s="87" t="n"/>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="104" t="inlineStr"/>
       <c r="B15" s="150" t="n"/>
@@ -6929,22 +6354,7 @@
         </is>
       </c>
       <c r="B18" s="154">
-        <f>IF(B4&gt;0,B11/B4,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="106" t="inlineStr">
-        <is>
-          <t>Margin:</t>
-        </is>
-      </c>
-      <c r="B19" s="155">
-        <f>B11-B14</f>
-        <v/>
-      </c>
-      <c r="C19" s="156">
-        <f>IF(B11&gt;0,B13/B11,0)</f>
+        <f>IF(B4&gt;0,B17/B4,0)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
v3 fix: restore Guest1-4 editing, golf dropdown A-only, FlightAware visible, Master Data values preserved
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -528,7 +528,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -749,15 +749,21 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="9" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="18" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -783,9 +789,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="21" fillId="11" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -3284,20 +3287,39 @@
           <t>Package:</t>
         </is>
       </c>
-      <c r="B2" s="48" t="n"/>
-      <c r="C2" s="48" t="n"/>
-      <c r="D2" s="48" t="n"/>
-      <c r="E2" s="48" t="n"/>
-      <c r="F2" s="48" t="n"/>
-      <c r="G2" s="48" t="n"/>
-      <c r="H2" s="48" t="n"/>
-      <c r="I2" s="48" t="n"/>
-      <c r="J2" s="48" t="n"/>
-      <c r="K2" s="48" t="n"/>
-      <c r="L2" s="46" t="n"/>
+      <c r="B2" s="84" t="n"/>
+      <c r="C2" s="46" t="n"/>
+      <c r="D2" s="85" t="inlineStr">
+        <is>
+          <t>Golfers:</t>
+        </is>
+      </c>
+      <c r="E2" s="86" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="86" t="inlineStr">
+        <is>
+          <t>Guest1</t>
+        </is>
+      </c>
+      <c r="G2" s="86" t="inlineStr">
+        <is>
+          <t>Guest2</t>
+        </is>
+      </c>
+      <c r="H2" s="86" t="inlineStr">
+        <is>
+          <t>Guest3</t>
+        </is>
+      </c>
+      <c r="I2" s="86" t="inlineStr">
+        <is>
+          <t>Guest4</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="84" t="inlineStr">
+      <c r="A3" s="87" t="inlineStr">
         <is>
           <t>💰 CHARGE LEGEND:  PG=Per Group(1회청구) | P1=Per Person(1인) | P2=2인1실 | P3=3인1조 | ... P20=20인까지 | 각 카테고리 ▼ 드롭다운으로 선택</t>
         </is>
@@ -3333,69 +3355,69 @@
       <c r="L4" s="46" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="85" t="inlineStr">
+      <c r="A5" s="88" t="inlineStr">
         <is>
           <t>Date:</t>
         </is>
       </c>
       <c r="B5" s="86" t="n"/>
-      <c r="C5" s="87">
-        <f>IF(D5="","Flight# ▼",HYPERLINK("https://flightaware.com/live/flight/"&amp;LEFT(D5,2)&amp;VALUE(MID(D5,3,10)),"✈ "&amp;D5))</f>
+      <c r="C5" s="89">
+        <f>IF(D5="","✈ Select flight ▼",HYPERLINK("https://flightaware.com/live/flight/"&amp;LEFT(D5,2)&amp;VALUE(MID(D5,3,10)),"✈ "&amp;D5&amp;" 🔗"))</f>
         <v/>
       </c>
       <c r="D5" s="86" t="n"/>
-      <c r="E5" s="85" t="inlineStr">
+      <c r="E5" s="88" t="inlineStr">
         <is>
           <t>Airline:</t>
         </is>
       </c>
-      <c r="F5" s="88">
+      <c r="F5" s="90">
         <f>IF(D5="","",VLOOKUP(D5,'Master Data'!$A$77:$B$80,2,FALSE))</f>
         <v/>
       </c>
-      <c r="G5" s="85" t="inlineStr">
+      <c r="G5" s="88" t="inlineStr">
         <is>
           <t>Departure:</t>
         </is>
       </c>
-      <c r="H5" s="88">
+      <c r="H5" s="90">
         <f>IF(D5="","",VLOOKUP(D5,'Master Data'!$A$77:$D$80,3,FALSE))</f>
         <v/>
       </c>
-      <c r="I5" s="85" t="inlineStr">
+      <c r="I5" s="88" t="inlineStr">
         <is>
           <t>Arrival:</t>
         </is>
       </c>
-      <c r="J5" s="88">
+      <c r="J5" s="90">
         <f>IF(D5="","",VLOOKUP(D5,'Master Data'!$A$77:$D$80,4,FALSE))</f>
         <v/>
       </c>
-      <c r="K5" s="85" t="inlineStr">
+      <c r="K5" s="88" t="inlineStr">
         <is>
           <t>Seat:</t>
         </is>
       </c>
       <c r="L5" s="86" t="n"/>
-      <c r="M5" s="88">
+      <c r="M5" s="90">
         <f>IF(D5="","",VLOOKUP(D5,'Master Data'!$A$77:$I$80,9,FALSE)&amp;" hrs")</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="89" t="n"/>
-      <c r="B6" s="89" t="n"/>
-      <c r="C6" s="89" t="n"/>
-      <c r="D6" s="89" t="n"/>
-      <c r="E6" s="89" t="n"/>
-      <c r="F6" s="89" t="n"/>
-      <c r="G6" s="89" t="n"/>
-      <c r="H6" s="89" t="n"/>
-      <c r="I6" s="89" t="n"/>
-      <c r="J6" s="89" t="n"/>
-      <c r="K6" s="89" t="n"/>
-      <c r="L6" s="89" t="n"/>
-      <c r="M6" s="89" t="n"/>
+      <c r="A6" s="91" t="n"/>
+      <c r="B6" s="91" t="n"/>
+      <c r="C6" s="91" t="n"/>
+      <c r="D6" s="91" t="n"/>
+      <c r="E6" s="91" t="n"/>
+      <c r="F6" s="91" t="n"/>
+      <c r="G6" s="91" t="n"/>
+      <c r="H6" s="91" t="n"/>
+      <c r="I6" s="91" t="n"/>
+      <c r="J6" s="91" t="n"/>
+      <c r="K6" s="91" t="n"/>
+      <c r="L6" s="91" t="n"/>
+      <c r="M6" s="91" t="n"/>
     </row>
     <row r="7" ht="27.6" customHeight="1" s="44">
       <c r="A7" s="82" t="inlineStr">
@@ -3416,94 +3438,94 @@
       <c r="L7" s="46" t="n"/>
     </row>
     <row r="8" ht="27.6" customHeight="1" s="44">
-      <c r="A8" s="85" t="inlineStr">
+      <c r="A8" s="88" t="inlineStr">
         <is>
           <t>Date:</t>
         </is>
       </c>
       <c r="B8" s="86" t="n"/>
-      <c r="C8" s="87">
-        <f>IF(D8="","Flight# ▼",HYPERLINK("https://flightaware.com/live/flight/"&amp;LEFT(D8,2)&amp;VALUE(MID(D8,3,10)),"✈ "&amp;D8))</f>
+      <c r="C8" s="89">
+        <f>IF(D8="","✈ Select flight ▼",HYPERLINK("https://flightaware.com/live/flight/"&amp;LEFT(D8,2)&amp;VALUE(MID(D8,3,10)),"✈ "&amp;D8&amp;" 🔗"))</f>
         <v/>
       </c>
       <c r="D8" s="86" t="n"/>
-      <c r="E8" s="90" t="inlineStr">
+      <c r="E8" s="92" t="inlineStr">
         <is>
           <t>Airline:</t>
         </is>
       </c>
-      <c r="F8" s="88">
+      <c r="F8" s="90">
         <f>IF(D8="","",VLOOKUP(D8,'Master Data'!$A$91:$B$94,2,FALSE))</f>
         <v/>
       </c>
-      <c r="G8" s="90" t="inlineStr">
+      <c r="G8" s="92" t="inlineStr">
         <is>
           <t>Departure:</t>
         </is>
       </c>
-      <c r="H8" s="88">
+      <c r="H8" s="90">
         <f>IF(D8="","",VLOOKUP(D8,'Master Data'!$A$91:$D$94,3,FALSE))</f>
         <v/>
       </c>
-      <c r="I8" s="85" t="inlineStr">
+      <c r="I8" s="88" t="inlineStr">
         <is>
           <t>Arrival:</t>
         </is>
       </c>
-      <c r="J8" s="88">
+      <c r="J8" s="90">
         <f>IF(D8="","",VLOOKUP(D8,'Master Data'!$A$91:$D$94,4,FALSE))</f>
         <v/>
       </c>
-      <c r="K8" s="85" t="inlineStr">
+      <c r="K8" s="88" t="inlineStr">
         <is>
           <t>Seat:</t>
         </is>
       </c>
       <c r="L8" s="86" t="n"/>
-      <c r="M8" s="88">
+      <c r="M8" s="90">
         <f>IF(D8="","",VLOOKUP(D8,'Master Data'!$A$91:$I$94,9,FALSE)&amp;" hrs")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="91" t="inlineStr">
+      <c r="A9" s="93" t="inlineStr">
         <is>
           <t>📅 Trip:</t>
         </is>
       </c>
-      <c r="B9" s="91">
+      <c r="B9" s="93">
         <f>IF(AND(B5&lt;&gt;"",B8&lt;&gt;""),B8-B5&amp;"N "&amp;B8-B5+1&amp;"D","")</f>
         <v/>
       </c>
       <c r="C9" s="46" t="n"/>
-      <c r="D9" s="85" t="inlineStr">
+      <c r="D9" s="88" t="inlineStr">
         <is>
           <t>Status:</t>
         </is>
       </c>
-      <c r="E9" s="87">
+      <c r="E9" s="89">
         <f>IF(SUM(P11:P52)&gt;0,"❌"&amp;SUM(P11:P52)&amp;" dup","✅")</f>
         <v/>
       </c>
-      <c r="F9" s="85" t="inlineStr">
+      <c r="F9" s="88" t="inlineStr">
         <is>
           <t>X-Check:</t>
         </is>
       </c>
-      <c r="G9" s="92">
+      <c r="G9" s="94">
         <f>J64</f>
         <v/>
       </c>
-      <c r="H9" s="87" t="inlineStr">
+      <c r="H9" s="89" t="inlineStr">
         <is>
           <t>vs</t>
         </is>
       </c>
-      <c r="I9" s="92">
+      <c r="I9" s="94">
         <f>B72</f>
         <v/>
       </c>
-      <c r="J9" s="93">
+      <c r="J9" s="95">
         <f>IF(G9-I9=0,"✅MATCH","❌MISMATCH")</f>
         <v/>
       </c>
@@ -3534,94 +3556,94 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="94" t="inlineStr">
+      <c r="A10" s="96" t="inlineStr">
         <is>
           <t>Item ▼</t>
         </is>
       </c>
-      <c r="B10" s="94" t="inlineStr">
+      <c r="B10" s="96" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="C10" s="94" t="inlineStr">
+      <c r="C10" s="96" t="inlineStr">
         <is>
           <t>Cost/P</t>
         </is>
       </c>
-      <c r="D10" s="94" t="inlineStr">
+      <c r="D10" s="96" t="inlineStr">
         <is>
           <t>Sell/P</t>
         </is>
       </c>
-      <c r="E10" s="94" t="inlineStr">
+      <c r="E10" s="96" t="inlineStr">
         <is>
           <t>Margin%</t>
         </is>
       </c>
-      <c r="F10" s="94" t="inlineStr">
+      <c r="F10" s="96" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="G10" s="94" t="inlineStr">
+      <c r="G10" s="96" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="H10" s="94" t="inlineStr">
+      <c r="H10" s="96" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="I10" s="94" t="inlineStr">
+      <c r="I10" s="96" t="inlineStr">
         <is>
           <t>P4</t>
         </is>
       </c>
-      <c r="J10" s="94" t="inlineStr">
+      <c r="J10" s="96" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K10" s="94" t="inlineStr">
+      <c r="K10" s="96" t="inlineStr">
         <is>
           <t>Tot Cost</t>
         </is>
       </c>
-      <c r="L10" s="94" t="inlineStr">
+      <c r="L10" s="96" t="inlineStr">
         <is>
           <t>Tot Sell</t>
         </is>
       </c>
-      <c r="M10" s="94" t="inlineStr">
+      <c r="M10" s="96" t="inlineStr">
         <is>
           <t>P5</t>
         </is>
       </c>
-      <c r="N10" s="94" t="inlineStr">
+      <c r="N10" s="96" t="inlineStr">
         <is>
           <t>P6</t>
         </is>
       </c>
-      <c r="O10" s="94" t="inlineStr">
+      <c r="O10" s="96" t="inlineStr">
         <is>
           <t>P7</t>
         </is>
       </c>
-      <c r="P10" s="94" t="inlineStr">
+      <c r="P10" s="96" t="inlineStr">
         <is>
           <t>P8</t>
         </is>
       </c>
-      <c r="Q10" s="94" t="inlineStr">
+      <c r="Q10" s="96" t="inlineStr">
         <is>
           <t>Dup</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" s="44">
-      <c r="A11" s="95" t="inlineStr">
+      <c r="A11" s="97" t="inlineStr">
         <is>
           <t>⛳ GOLF</t>
         </is>
@@ -3636,267 +3658,267 @@
       <c r="I11" s="48" t="n"/>
       <c r="J11" s="48" t="n"/>
       <c r="K11" s="46" t="n"/>
-      <c r="L11" s="91" t="inlineStr">
+      <c r="L11" s="93" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="M11" s="94" t="n"/>
-      <c r="N11" s="94" t="n"/>
-      <c r="O11" s="94" t="n"/>
-      <c r="P11" s="94" t="n"/>
-      <c r="Q11" s="94" t="n"/>
+      <c r="M11" s="96" t="n"/>
+      <c r="N11" s="96" t="n"/>
+      <c r="O11" s="96" t="n"/>
+      <c r="P11" s="96" t="n"/>
+      <c r="Q11" s="96" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1" s="44">
-      <c r="A12" s="96" t="inlineStr">
+      <c r="A12" s="84" t="inlineStr">
         <is>
           <t>Sandpiper GC</t>
         </is>
       </c>
-      <c r="B12" s="97" t="n">
+      <c r="B12" s="98" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="98">
+      <c r="C12" s="99">
         <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$8:$C$15,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D12" s="98">
+      <c r="D12" s="99">
         <f>IF(A12="","",VLOOKUP(A12,'Master Data'!$A$8:$C$15,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E12" s="99">
+      <c r="E12" s="100">
         <f>IF(D12&gt;0,(D12-C12)/D12,0)</f>
         <v/>
       </c>
-      <c r="F12" s="87" t="n"/>
-      <c r="G12" s="87" t="n"/>
-      <c r="H12" s="87" t="n"/>
-      <c r="I12" s="87" t="n"/>
-      <c r="J12" s="100" t="inlineStr">
+      <c r="F12" s="89" t="n"/>
+      <c r="G12" s="89" t="n"/>
+      <c r="H12" s="89" t="n"/>
+      <c r="I12" s="89" t="n"/>
+      <c r="J12" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K12" s="98">
+      <c r="K12" s="99">
         <f>IF(A12="","",IF(L11="PG",IF((F12="●")+(G12="●")+(H12="●")+(I12="●")+(L12="●")+(M12="●")+(N12="●")+(O12="●")&gt;0,B12*C12,0),ROUNDUP((F12="●")+(G12="●")+(H12="●")+(I12="●")+(L12="●")+(M12="●")+(N12="●")+(O12="●")/VALUE(MID(L11,2,2)),0)*B12*C12))</f>
         <v/>
       </c>
-      <c r="L12" s="98">
+      <c r="L12" s="99">
         <f>IF(A12="","",IF(L11="PG",IF((F12="●")+(G12="●")+(H12="●")+(I12="●")+(L12="●")+(M12="●")+(N12="●")+(O12="●")&gt;0,B12*D12,0),ROUNDUP((F12="●")+(G12="●")+(H12="●")+(I12="●")+(L12="●")+(M12="●")+(N12="●")+(O12="●")/VALUE(MID(L11,2,2)),0)*B12*D12))</f>
         <v/>
       </c>
-      <c r="M12" s="87" t="n"/>
-      <c r="N12" s="87" t="n"/>
-      <c r="O12" s="87" t="n"/>
+      <c r="M12" s="89" t="n"/>
+      <c r="N12" s="89" t="n"/>
+      <c r="O12" s="89" t="n"/>
       <c r="P12" s="5">
         <f>IF(A12="",0,COUNTIF(A$11:A11,A12))</f>
         <v/>
       </c>
-      <c r="Q12" s="87" t="n"/>
+      <c r="Q12" s="89" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1" s="44">
-      <c r="A13" s="96" t="inlineStr">
+      <c r="A13" s="84" t="inlineStr">
         <is>
           <t>Trump National LA</t>
         </is>
       </c>
-      <c r="B13" s="97" t="n">
+      <c r="B13" s="98" t="n">
         <v>1</v>
       </c>
-      <c r="C13" s="98">
+      <c r="C13" s="99">
         <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$8:$C$15,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D13" s="98">
+      <c r="D13" s="99">
         <f>IF(A13="","",VLOOKUP(A13,'Master Data'!$A$8:$C$15,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E13" s="99">
+      <c r="E13" s="100">
         <f>IF(D13&gt;0,(D13-C13)/D13,0)</f>
         <v/>
       </c>
-      <c r="F13" s="87" t="n"/>
-      <c r="G13" s="87" t="n"/>
-      <c r="H13" s="87" t="n"/>
-      <c r="I13" s="87" t="n"/>
-      <c r="J13" s="100" t="inlineStr">
+      <c r="F13" s="89" t="n"/>
+      <c r="G13" s="89" t="n"/>
+      <c r="H13" s="89" t="n"/>
+      <c r="I13" s="89" t="n"/>
+      <c r="J13" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K13" s="98">
+      <c r="K13" s="99">
         <f>IF(A13="","",IF(L11="PG",IF((F13="●")+(G13="●")+(H13="●")+(I13="●")+(L13="●")+(M13="●")+(N13="●")+(O13="●")&gt;0,B13*C13,0),ROUNDUP((F13="●")+(G13="●")+(H13="●")+(I13="●")+(L13="●")+(M13="●")+(N13="●")+(O13="●")/VALUE(MID(L11,2,2)),0)*B13*C13))</f>
         <v/>
       </c>
-      <c r="L13" s="98">
+      <c r="L13" s="99">
         <f>IF(A13="","",IF(L11="PG",IF((F13="●")+(G13="●")+(H13="●")+(I13="●")+(L13="●")+(M13="●")+(N13="●")+(O13="●")&gt;0,B13*D13,0),ROUNDUP((F13="●")+(G13="●")+(H13="●")+(I13="●")+(L13="●")+(M13="●")+(N13="●")+(O13="●")/VALUE(MID(L11,2,2)),0)*B13*D13))</f>
         <v/>
       </c>
-      <c r="M13" s="87" t="n"/>
-      <c r="N13" s="87" t="n"/>
-      <c r="O13" s="87" t="n"/>
+      <c r="M13" s="89" t="n"/>
+      <c r="N13" s="89" t="n"/>
+      <c r="O13" s="89" t="n"/>
       <c r="P13" s="5">
         <f>IF(A13="",0,COUNTIF(A$11:A12,A13))</f>
         <v/>
       </c>
-      <c r="Q13" s="87" t="n"/>
+      <c r="Q13" s="89" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1" s="44">
-      <c r="A14" s="101" t="n"/>
-      <c r="B14" s="100" t="n"/>
-      <c r="C14" s="98">
+      <c r="A14" s="102" t="n"/>
+      <c r="B14" s="101" t="n"/>
+      <c r="C14" s="99">
         <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$8:$C$15,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D14" s="98">
+      <c r="D14" s="99">
         <f>IF(A14="","",VLOOKUP(A14,'Master Data'!$A$8:$C$15,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E14" s="99">
+      <c r="E14" s="100">
         <f>IF(D14&gt;0,(D14-C14)/D14,0)</f>
         <v/>
       </c>
-      <c r="F14" s="87" t="n"/>
-      <c r="G14" s="87" t="n"/>
-      <c r="H14" s="87" t="n"/>
-      <c r="I14" s="87" t="n"/>
-      <c r="J14" s="100" t="inlineStr">
+      <c r="F14" s="89" t="n"/>
+      <c r="G14" s="89" t="n"/>
+      <c r="H14" s="89" t="n"/>
+      <c r="I14" s="89" t="n"/>
+      <c r="J14" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K14" s="98">
+      <c r="K14" s="99">
         <f>IF(A14="","",IF(L11="PG",IF((F14="●")+(G14="●")+(H14="●")+(I14="●")+(L14="●")+(M14="●")+(N14="●")+(O14="●")&gt;0,B14*C14,0),ROUNDUP((F14="●")+(G14="●")+(H14="●")+(I14="●")+(L14="●")+(M14="●")+(N14="●")+(O14="●")/VALUE(MID(L11,2,2)),0)*B14*C14))</f>
         <v/>
       </c>
-      <c r="L14" s="98">
+      <c r="L14" s="99">
         <f>IF(A14="","",IF(L11="PG",IF((F14="●")+(G14="●")+(H14="●")+(I14="●")+(L14="●")+(M14="●")+(N14="●")+(O14="●")&gt;0,B14*D14,0),ROUNDUP((F14="●")+(G14="●")+(H14="●")+(I14="●")+(L14="●")+(M14="●")+(N14="●")+(O14="●")/VALUE(MID(L11,2,2)),0)*B14*D14))</f>
         <v/>
       </c>
-      <c r="M14" s="87" t="n"/>
-      <c r="N14" s="87" t="n"/>
-      <c r="O14" s="87" t="n"/>
+      <c r="M14" s="89" t="n"/>
+      <c r="N14" s="89" t="n"/>
+      <c r="O14" s="89" t="n"/>
       <c r="P14" s="5">
         <f>IF(A14="",0,COUNTIF(A$11:A13,A14))</f>
         <v/>
       </c>
-      <c r="Q14" s="87" t="n"/>
+      <c r="Q14" s="89" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1" s="44">
-      <c r="A15" s="101" t="n"/>
-      <c r="B15" s="100" t="n"/>
-      <c r="C15" s="98">
+      <c r="A15" s="102" t="n"/>
+      <c r="B15" s="101" t="n"/>
+      <c r="C15" s="99">
         <f>IF(A15="","",VLOOKUP(A15,'Master Data'!$A$8:$C$15,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D15" s="98">
+      <c r="D15" s="99">
         <f>IF(A15="","",VLOOKUP(A15,'Master Data'!$A$8:$C$15,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E15" s="99">
+      <c r="E15" s="100">
         <f>IF(D15&gt;0,(D15-C15)/D15,0)</f>
         <v/>
       </c>
-      <c r="F15" s="87" t="n"/>
-      <c r="G15" s="87" t="n"/>
-      <c r="H15" s="87" t="n"/>
-      <c r="I15" s="87" t="n"/>
-      <c r="J15" s="100" t="inlineStr">
+      <c r="F15" s="89" t="n"/>
+      <c r="G15" s="89" t="n"/>
+      <c r="H15" s="89" t="n"/>
+      <c r="I15" s="89" t="n"/>
+      <c r="J15" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K15" s="98">
+      <c r="K15" s="99">
         <f>IF(A15="","",IF(L11="PG",IF((F15="●")+(G15="●")+(H15="●")+(I15="●")+(L15="●")+(M15="●")+(N15="●")+(O15="●")&gt;0,B15*C15,0),ROUNDUP((F15="●")+(G15="●")+(H15="●")+(I15="●")+(L15="●")+(M15="●")+(N15="●")+(O15="●")/VALUE(MID(L11,2,2)),0)*B15*C15))</f>
         <v/>
       </c>
-      <c r="L15" s="98">
+      <c r="L15" s="99">
         <f>IF(A15="","",IF(L11="PG",IF((F15="●")+(G15="●")+(H15="●")+(I15="●")+(L15="●")+(M15="●")+(N15="●")+(O15="●")&gt;0,B15*D15,0),ROUNDUP((F15="●")+(G15="●")+(H15="●")+(I15="●")+(L15="●")+(M15="●")+(N15="●")+(O15="●")/VALUE(MID(L11,2,2)),0)*B15*D15))</f>
         <v/>
       </c>
-      <c r="M15" s="87" t="n"/>
-      <c r="N15" s="87" t="n"/>
-      <c r="O15" s="87" t="n"/>
+      <c r="M15" s="89" t="n"/>
+      <c r="N15" s="89" t="n"/>
+      <c r="O15" s="89" t="n"/>
       <c r="P15" s="5">
         <f>IF(A15="",0,COUNTIF(A$11:A14,A15))</f>
         <v/>
       </c>
-      <c r="Q15" s="87" t="n"/>
+      <c r="Q15" s="89" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="102" t="inlineStr">
+      <c r="A16" s="103" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B16" s="91" t="n"/>
-      <c r="C16" s="91" t="n"/>
-      <c r="D16" s="91" t="n"/>
-      <c r="E16" s="91" t="n"/>
-      <c r="F16" s="103">
+      <c r="B16" s="93" t="n"/>
+      <c r="C16" s="93" t="n"/>
+      <c r="D16" s="93" t="n"/>
+      <c r="E16" s="93" t="n"/>
+      <c r="F16" s="104">
         <f>SUMPRODUCT((F11:F15="●")*1,B11:B15,C11:C15)</f>
         <v/>
       </c>
-      <c r="G16" s="103">
+      <c r="G16" s="104">
         <f>SUMPRODUCT((G11:G15="●")*1,B11:B15,C11:C15)</f>
         <v/>
       </c>
-      <c r="H16" s="103">
+      <c r="H16" s="104">
         <f>SUMPRODUCT((H11:H15="●")*1,B11:B15,C11:C15)</f>
         <v/>
       </c>
-      <c r="I16" s="103">
+      <c r="I16" s="104">
         <f>SUMPRODUCT((I11:I15="●")*1,B11:B15,C11:C15)</f>
         <v/>
       </c>
-      <c r="J16" s="104" t="n"/>
-      <c r="K16" s="103">
+      <c r="J16" s="105" t="n"/>
+      <c r="K16" s="104">
         <f>SUM(K11:K15)</f>
         <v/>
       </c>
-      <c r="L16" s="103">
+      <c r="L16" s="104">
         <f>SUM(L11:L15)</f>
         <v/>
       </c>
-      <c r="M16" s="103">
+      <c r="M16" s="104">
         <f>SUMPRODUCT((M11:M15="●")*1,B11:B15,C11:C15)</f>
         <v/>
       </c>
-      <c r="N16" s="103">
+      <c r="N16" s="104">
         <f>SUMPRODUCT((N11:N15="●")*1,B11:B15,C11:C15)</f>
         <v/>
       </c>
-      <c r="O16" s="103">
+      <c r="O16" s="104">
         <f>SUMPRODUCT((O11:O15="●")*1,B11:B15,C11:C15)</f>
         <v/>
       </c>
-      <c r="P16" s="91">
+      <c r="P16" s="93">
         <f>SUM(P11:P15)</f>
         <v/>
       </c>
-      <c r="Q16" s="91" t="n"/>
+      <c r="Q16" s="93" t="n"/>
     </row>
     <row r="17" ht="6" customHeight="1" s="44">
-      <c r="A17" s="89" t="n"/>
-      <c r="B17" s="89" t="n"/>
-      <c r="C17" s="89" t="n"/>
-      <c r="D17" s="89" t="n"/>
-      <c r="E17" s="89" t="n"/>
-      <c r="F17" s="89" t="n"/>
-      <c r="G17" s="89" t="n"/>
-      <c r="H17" s="89" t="n"/>
-      <c r="I17" s="89" t="n"/>
-      <c r="J17" s="89" t="n"/>
-      <c r="K17" s="89" t="n"/>
-      <c r="L17" s="89" t="n"/>
-      <c r="M17" s="89" t="n"/>
-      <c r="N17" s="89" t="n"/>
-      <c r="O17" s="89" t="n"/>
-      <c r="P17" s="89" t="n"/>
-      <c r="Q17" s="89" t="n"/>
+      <c r="A17" s="91" t="n"/>
+      <c r="B17" s="91" t="n"/>
+      <c r="C17" s="91" t="n"/>
+      <c r="D17" s="91" t="n"/>
+      <c r="E17" s="91" t="n"/>
+      <c r="F17" s="91" t="n"/>
+      <c r="G17" s="91" t="n"/>
+      <c r="H17" s="91" t="n"/>
+      <c r="I17" s="91" t="n"/>
+      <c r="J17" s="91" t="n"/>
+      <c r="K17" s="91" t="n"/>
+      <c r="L17" s="91" t="n"/>
+      <c r="M17" s="91" t="n"/>
+      <c r="N17" s="91" t="n"/>
+      <c r="O17" s="91" t="n"/>
+      <c r="P17" s="91" t="n"/>
+      <c r="Q17" s="91" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="95" t="inlineStr">
+      <c r="A18" s="97" t="inlineStr">
         <is>
           <t>🏨 HOTEL</t>
         </is>
@@ -3911,174 +3933,174 @@
       <c r="I18" s="48" t="n"/>
       <c r="J18" s="48" t="n"/>
       <c r="K18" s="46" t="n"/>
-      <c r="L18" s="91" t="inlineStr">
+      <c r="L18" s="93" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="M18" s="94" t="n"/>
-      <c r="N18" s="94" t="n"/>
-      <c r="O18" s="94" t="n"/>
-      <c r="P18" s="94" t="n"/>
-      <c r="Q18" s="94" t="n"/>
+      <c r="M18" s="96" t="n"/>
+      <c r="N18" s="96" t="n"/>
+      <c r="O18" s="96" t="n"/>
+      <c r="P18" s="96" t="n"/>
+      <c r="Q18" s="96" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1" s="44">
-      <c r="A19" s="101" t="n"/>
-      <c r="B19" s="100" t="n"/>
-      <c r="C19" s="98">
+      <c r="A19" s="102" t="n"/>
+      <c r="B19" s="101" t="n"/>
+      <c r="C19" s="99">
         <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$21:$C$26,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D19" s="98">
+      <c r="D19" s="99">
         <f>IF(A19="","",VLOOKUP(A19,'Master Data'!$A$21:$C$26,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E19" s="99">
+      <c r="E19" s="100">
         <f>IF(D19&gt;0,(D19-C19)/D19,0)</f>
         <v/>
       </c>
-      <c r="F19" s="87" t="n"/>
-      <c r="G19" s="87" t="n"/>
-      <c r="H19" s="87" t="n"/>
-      <c r="I19" s="87" t="n"/>
-      <c r="J19" s="100" t="inlineStr">
+      <c r="F19" s="89" t="n"/>
+      <c r="G19" s="89" t="n"/>
+      <c r="H19" s="89" t="n"/>
+      <c r="I19" s="89" t="n"/>
+      <c r="J19" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K19" s="98">
+      <c r="K19" s="99">
         <f>IF(A19="","",IF(L18="PG",IF((F19="●")+(G19="●")+(H19="●")+(I19="●")+(L19="●")+(M19="●")+(N19="●")+(O19="●")&gt;0,B19*C19,0),ROUNDUP((F19="●")+(G19="●")+(H19="●")+(I19="●")+(L19="●")+(M19="●")+(N19="●")+(O19="●")/VALUE(MID(L18,2,2)),0)*B19*C19))</f>
         <v/>
       </c>
-      <c r="L19" s="98">
+      <c r="L19" s="99">
         <f>IF(A19="","",IF(L18="PG",IF((F19="●")+(G19="●")+(H19="●")+(I19="●")+(L19="●")+(M19="●")+(N19="●")+(O19="●")&gt;0,B19*D19,0),ROUNDUP((F19="●")+(G19="●")+(H19="●")+(I19="●")+(L19="●")+(M19="●")+(N19="●")+(O19="●")/VALUE(MID(L18,2,2)),0)*B19*D19))</f>
         <v/>
       </c>
-      <c r="M19" s="87" t="n"/>
-      <c r="N19" s="87" t="n"/>
-      <c r="O19" s="87" t="n"/>
+      <c r="M19" s="89" t="n"/>
+      <c r="N19" s="89" t="n"/>
+      <c r="O19" s="89" t="n"/>
       <c r="P19" s="5">
         <f>IF(A19="",0,COUNTIF(A$18:A18,A19))</f>
         <v/>
       </c>
-      <c r="Q19" s="87" t="n"/>
+      <c r="Q19" s="89" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1" s="44">
-      <c r="A20" s="101" t="n"/>
-      <c r="B20" s="100" t="n"/>
-      <c r="C20" s="98">
+      <c r="A20" s="102" t="n"/>
+      <c r="B20" s="101" t="n"/>
+      <c r="C20" s="99">
         <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$21:$C$26,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D20" s="98">
+      <c r="D20" s="99">
         <f>IF(A20="","",VLOOKUP(A20,'Master Data'!$A$21:$C$26,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E20" s="99">
+      <c r="E20" s="100">
         <f>IF(D20&gt;0,(D20-C20)/D20,0)</f>
         <v/>
       </c>
-      <c r="F20" s="87" t="n"/>
-      <c r="G20" s="87" t="n"/>
-      <c r="H20" s="87" t="n"/>
-      <c r="I20" s="87" t="n"/>
-      <c r="J20" s="100" t="inlineStr">
+      <c r="F20" s="89" t="n"/>
+      <c r="G20" s="89" t="n"/>
+      <c r="H20" s="89" t="n"/>
+      <c r="I20" s="89" t="n"/>
+      <c r="J20" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K20" s="98">
+      <c r="K20" s="99">
         <f>IF(A20="","",IF(L18="PG",IF((F20="●")+(G20="●")+(H20="●")+(I20="●")+(L20="●")+(M20="●")+(N20="●")+(O20="●")&gt;0,B20*C20,0),ROUNDUP((F20="●")+(G20="●")+(H20="●")+(I20="●")+(L20="●")+(M20="●")+(N20="●")+(O20="●")/VALUE(MID(L18,2,2)),0)*B20*C20))</f>
         <v/>
       </c>
-      <c r="L20" s="98">
+      <c r="L20" s="99">
         <f>IF(A20="","",IF(L18="PG",IF((F20="●")+(G20="●")+(H20="●")+(I20="●")+(L20="●")+(M20="●")+(N20="●")+(O20="●")&gt;0,B20*D20,0),ROUNDUP((F20="●")+(G20="●")+(H20="●")+(I20="●")+(L20="●")+(M20="●")+(N20="●")+(O20="●")/VALUE(MID(L18,2,2)),0)*B20*D20))</f>
         <v/>
       </c>
-      <c r="M20" s="87" t="n"/>
-      <c r="N20" s="87" t="n"/>
-      <c r="O20" s="87" t="n"/>
+      <c r="M20" s="89" t="n"/>
+      <c r="N20" s="89" t="n"/>
+      <c r="O20" s="89" t="n"/>
       <c r="P20" s="5">
         <f>IF(A20="",0,COUNTIF(A$18:A19,A20))</f>
         <v/>
       </c>
-      <c r="Q20" s="87" t="n"/>
+      <c r="Q20" s="89" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1" s="44">
-      <c r="A21" s="102" t="inlineStr">
+      <c r="A21" s="103" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B21" s="104" t="n"/>
-      <c r="C21" s="104" t="n"/>
-      <c r="D21" s="104" t="n"/>
-      <c r="E21" s="105" t="n"/>
-      <c r="F21" s="103">
+      <c r="B21" s="105" t="n"/>
+      <c r="C21" s="105" t="n"/>
+      <c r="D21" s="105" t="n"/>
+      <c r="E21" s="106" t="n"/>
+      <c r="F21" s="104">
         <f>SUMPRODUCT((F18:F20="●")*1,B18:B20,C18:C20)</f>
         <v/>
       </c>
-      <c r="G21" s="103">
+      <c r="G21" s="104">
         <f>SUMPRODUCT((G18:G20="●")*1,B18:B20,C18:C20)</f>
         <v/>
       </c>
-      <c r="H21" s="103">
+      <c r="H21" s="104">
         <f>SUMPRODUCT((H18:H20="●")*1,B18:B20,C18:C20)</f>
         <v/>
       </c>
-      <c r="I21" s="103">
+      <c r="I21" s="104">
         <f>SUMPRODUCT((I18:I20="●")*1,B18:B20,C18:C20)</f>
         <v/>
       </c>
-      <c r="J21" s="104" t="n"/>
-      <c r="K21" s="103">
+      <c r="J21" s="105" t="n"/>
+      <c r="K21" s="104">
         <f>SUM(K18:K20)</f>
         <v/>
       </c>
-      <c r="L21" s="103">
+      <c r="L21" s="104">
         <f>SUM(L18:L20)</f>
         <v/>
       </c>
-      <c r="M21" s="103">
+      <c r="M21" s="104">
         <f>SUMPRODUCT((M18:M20="●")*1,B18:B20,C18:C20)</f>
         <v/>
       </c>
-      <c r="N21" s="103">
+      <c r="N21" s="104">
         <f>SUMPRODUCT((N18:N20="●")*1,B18:B20,C18:C20)</f>
         <v/>
       </c>
-      <c r="O21" s="103">
+      <c r="O21" s="104">
         <f>SUMPRODUCT((O18:O20="●")*1,B18:B20,C18:C20)</f>
         <v/>
       </c>
-      <c r="P21" s="91">
+      <c r="P21" s="93">
         <f>SUM(P18:P20)</f>
         <v/>
       </c>
-      <c r="Q21" s="91" t="n"/>
+      <c r="Q21" s="93" t="n"/>
     </row>
     <row r="22" ht="6" customHeight="1" s="44">
-      <c r="A22" s="89" t="n"/>
-      <c r="B22" s="89" t="n"/>
-      <c r="C22" s="89" t="n"/>
-      <c r="D22" s="89" t="n"/>
-      <c r="E22" s="89" t="n"/>
-      <c r="F22" s="106" t="n"/>
-      <c r="G22" s="106" t="n"/>
-      <c r="H22" s="106" t="n"/>
-      <c r="I22" s="106" t="n"/>
-      <c r="J22" s="106" t="n"/>
-      <c r="K22" s="106" t="n"/>
-      <c r="L22" s="106" t="n"/>
-      <c r="M22" s="106" t="n"/>
-      <c r="N22" s="106" t="n"/>
-      <c r="O22" s="106" t="n"/>
-      <c r="P22" s="89" t="n"/>
-      <c r="Q22" s="89" t="n"/>
+      <c r="A22" s="91" t="n"/>
+      <c r="B22" s="91" t="n"/>
+      <c r="C22" s="91" t="n"/>
+      <c r="D22" s="91" t="n"/>
+      <c r="E22" s="91" t="n"/>
+      <c r="F22" s="107" t="n"/>
+      <c r="G22" s="107" t="n"/>
+      <c r="H22" s="107" t="n"/>
+      <c r="I22" s="107" t="n"/>
+      <c r="J22" s="107" t="n"/>
+      <c r="K22" s="107" t="n"/>
+      <c r="L22" s="107" t="n"/>
+      <c r="M22" s="107" t="n"/>
+      <c r="N22" s="107" t="n"/>
+      <c r="O22" s="107" t="n"/>
+      <c r="P22" s="91" t="n"/>
+      <c r="Q22" s="91" t="n"/>
     </row>
     <row r="23"/>
     <row r="24">
-      <c r="A24" s="95" t="inlineStr">
+      <c r="A24" s="97" t="inlineStr">
         <is>
           <t>🚐 TRANSPORT</t>
         </is>
@@ -4093,174 +4115,174 @@
       <c r="I24" s="48" t="n"/>
       <c r="J24" s="48" t="n"/>
       <c r="K24" s="46" t="n"/>
-      <c r="L24" s="91" t="inlineStr">
+      <c r="L24" s="93" t="inlineStr">
         <is>
           <t>PG</t>
         </is>
       </c>
-      <c r="M24" s="94" t="n"/>
-      <c r="N24" s="94" t="n"/>
-      <c r="O24" s="94" t="n"/>
-      <c r="P24" s="94" t="n"/>
-      <c r="Q24" s="94" t="n"/>
+      <c r="M24" s="96" t="n"/>
+      <c r="N24" s="96" t="n"/>
+      <c r="O24" s="96" t="n"/>
+      <c r="P24" s="96" t="n"/>
+      <c r="Q24" s="96" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1" s="44">
-      <c r="A25" s="101" t="n"/>
-      <c r="B25" s="100" t="n"/>
-      <c r="C25" s="98">
+      <c r="A25" s="102" t="n"/>
+      <c r="B25" s="101" t="n"/>
+      <c r="C25" s="99">
         <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$31:$C$37,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D25" s="98">
+      <c r="D25" s="99">
         <f>IF(A25="","",VLOOKUP(A25,'Master Data'!$A$31:$C$37,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E25" s="99">
+      <c r="E25" s="100">
         <f>IF(D25&gt;0,(D25-C25)/D25,0)</f>
         <v/>
       </c>
-      <c r="F25" s="87" t="n"/>
-      <c r="G25" s="87" t="n"/>
-      <c r="H25" s="87" t="n"/>
-      <c r="I25" s="87" t="n"/>
-      <c r="J25" s="100" t="inlineStr">
+      <c r="F25" s="89" t="n"/>
+      <c r="G25" s="89" t="n"/>
+      <c r="H25" s="89" t="n"/>
+      <c r="I25" s="89" t="n"/>
+      <c r="J25" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K25" s="98">
+      <c r="K25" s="99">
         <f>IF(A25="","",IF(L24="PG",IF((F25="●")+(G25="●")+(H25="●")+(I25="●")+(L25="●")+(M25="●")+(N25="●")+(O25="●")&gt;0,B25*C25,0),ROUNDUP((F25="●")+(G25="●")+(H25="●")+(I25="●")+(L25="●")+(M25="●")+(N25="●")+(O25="●")/VALUE(MID(L24,2,2)),0)*B25*C25))</f>
         <v/>
       </c>
-      <c r="L25" s="98">
+      <c r="L25" s="99">
         <f>IF(A25="","",IF(L24="PG",IF((F25="●")+(G25="●")+(H25="●")+(I25="●")+(L25="●")+(M25="●")+(N25="●")+(O25="●")&gt;0,B25*D25,0),ROUNDUP((F25="●")+(G25="●")+(H25="●")+(I25="●")+(L25="●")+(M25="●")+(N25="●")+(O25="●")/VALUE(MID(L24,2,2)),0)*B25*D25))</f>
         <v/>
       </c>
-      <c r="M25" s="87" t="n"/>
-      <c r="N25" s="87" t="n"/>
-      <c r="O25" s="87" t="n"/>
+      <c r="M25" s="89" t="n"/>
+      <c r="N25" s="89" t="n"/>
+      <c r="O25" s="89" t="n"/>
       <c r="P25" s="5">
         <f>IF(A25="",0,COUNTIF(A$24:A24,A25))</f>
         <v/>
       </c>
-      <c r="Q25" s="87" t="n"/>
+      <c r="Q25" s="89" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1" s="44">
-      <c r="A26" s="101" t="n"/>
-      <c r="B26" s="100" t="n"/>
-      <c r="C26" s="98">
+      <c r="A26" s="102" t="n"/>
+      <c r="B26" s="101" t="n"/>
+      <c r="C26" s="99">
         <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$31:$C$37,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D26" s="98">
+      <c r="D26" s="99">
         <f>IF(A26="","",VLOOKUP(A26,'Master Data'!$A$31:$C$37,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E26" s="99">
+      <c r="E26" s="100">
         <f>IF(D26&gt;0,(D26-C26)/D26,0)</f>
         <v/>
       </c>
-      <c r="F26" s="87" t="n"/>
-      <c r="G26" s="87" t="n"/>
-      <c r="H26" s="87" t="n"/>
-      <c r="I26" s="87" t="n"/>
-      <c r="J26" s="100" t="inlineStr">
+      <c r="F26" s="89" t="n"/>
+      <c r="G26" s="89" t="n"/>
+      <c r="H26" s="89" t="n"/>
+      <c r="I26" s="89" t="n"/>
+      <c r="J26" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K26" s="98">
+      <c r="K26" s="99">
         <f>IF(A26="","",IF(L24="PG",IF((F26="●")+(G26="●")+(H26="●")+(I26="●")+(L26="●")+(M26="●")+(N26="●")+(O26="●")&gt;0,B26*C26,0),ROUNDUP((F26="●")+(G26="●")+(H26="●")+(I26="●")+(L26="●")+(M26="●")+(N26="●")+(O26="●")/VALUE(MID(L24,2,2)),0)*B26*C26))</f>
         <v/>
       </c>
-      <c r="L26" s="98">
+      <c r="L26" s="99">
         <f>IF(A26="","",IF(L24="PG",IF((F26="●")+(G26="●")+(H26="●")+(I26="●")+(L26="●")+(M26="●")+(N26="●")+(O26="●")&gt;0,B26*D26,0),ROUNDUP((F26="●")+(G26="●")+(H26="●")+(I26="●")+(L26="●")+(M26="●")+(N26="●")+(O26="●")/VALUE(MID(L24,2,2)),0)*B26*D26))</f>
         <v/>
       </c>
-      <c r="M26" s="87" t="n"/>
-      <c r="N26" s="87" t="n"/>
-      <c r="O26" s="87" t="n"/>
+      <c r="M26" s="89" t="n"/>
+      <c r="N26" s="89" t="n"/>
+      <c r="O26" s="89" t="n"/>
       <c r="P26" s="5">
         <f>IF(A26="",0,COUNTIF(A$24:A25,A26))</f>
         <v/>
       </c>
-      <c r="Q26" s="87" t="n"/>
+      <c r="Q26" s="89" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1" s="44">
-      <c r="A27" s="102" t="inlineStr">
+      <c r="A27" s="103" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B27" s="104" t="n"/>
-      <c r="C27" s="104" t="n"/>
-      <c r="D27" s="104" t="n"/>
-      <c r="E27" s="105" t="n"/>
-      <c r="F27" s="103">
+      <c r="B27" s="105" t="n"/>
+      <c r="C27" s="105" t="n"/>
+      <c r="D27" s="105" t="n"/>
+      <c r="E27" s="106" t="n"/>
+      <c r="F27" s="104">
         <f>SUMPRODUCT((F24:F26="●")*1,B24:B26,C24:C26)</f>
         <v/>
       </c>
-      <c r="G27" s="103">
+      <c r="G27" s="104">
         <f>SUMPRODUCT((G24:G26="●")*1,B24:B26,C24:C26)</f>
         <v/>
       </c>
-      <c r="H27" s="103">
+      <c r="H27" s="104">
         <f>SUMPRODUCT((H24:H26="●")*1,B24:B26,C24:C26)</f>
         <v/>
       </c>
-      <c r="I27" s="103">
+      <c r="I27" s="104">
         <f>SUMPRODUCT((I24:I26="●")*1,B24:B26,C24:C26)</f>
         <v/>
       </c>
-      <c r="J27" s="104" t="n"/>
-      <c r="K27" s="103">
+      <c r="J27" s="105" t="n"/>
+      <c r="K27" s="104">
         <f>SUM(K24:K26)</f>
         <v/>
       </c>
-      <c r="L27" s="103">
+      <c r="L27" s="104">
         <f>SUM(L24:L26)</f>
         <v/>
       </c>
-      <c r="M27" s="103">
+      <c r="M27" s="104">
         <f>SUMPRODUCT((M24:M26="●")*1,B24:B26,C24:C26)</f>
         <v/>
       </c>
-      <c r="N27" s="103">
+      <c r="N27" s="104">
         <f>SUMPRODUCT((N24:N26="●")*1,B24:B26,C24:C26)</f>
         <v/>
       </c>
-      <c r="O27" s="103">
+      <c r="O27" s="104">
         <f>SUMPRODUCT((O24:O26="●")*1,B24:B26,C24:C26)</f>
         <v/>
       </c>
-      <c r="P27" s="91">
+      <c r="P27" s="93">
         <f>SUM(P24:P26)</f>
         <v/>
       </c>
-      <c r="Q27" s="91" t="n"/>
+      <c r="Q27" s="93" t="n"/>
     </row>
     <row r="28" ht="6" customHeight="1" s="44">
-      <c r="A28" s="89" t="n"/>
-      <c r="B28" s="89" t="n"/>
-      <c r="C28" s="89" t="n"/>
-      <c r="D28" s="89" t="n"/>
-      <c r="E28" s="89" t="n"/>
-      <c r="F28" s="106" t="n"/>
-      <c r="G28" s="106" t="n"/>
-      <c r="H28" s="106" t="n"/>
-      <c r="I28" s="106" t="n"/>
-      <c r="J28" s="106" t="n"/>
-      <c r="K28" s="106" t="n"/>
-      <c r="L28" s="106" t="n"/>
-      <c r="M28" s="106" t="n"/>
-      <c r="N28" s="106" t="n"/>
-      <c r="O28" s="106" t="n"/>
-      <c r="P28" s="89" t="n"/>
-      <c r="Q28" s="89" t="n"/>
+      <c r="A28" s="91" t="n"/>
+      <c r="B28" s="91" t="n"/>
+      <c r="C28" s="91" t="n"/>
+      <c r="D28" s="91" t="n"/>
+      <c r="E28" s="91" t="n"/>
+      <c r="F28" s="107" t="n"/>
+      <c r="G28" s="107" t="n"/>
+      <c r="H28" s="107" t="n"/>
+      <c r="I28" s="107" t="n"/>
+      <c r="J28" s="107" t="n"/>
+      <c r="K28" s="107" t="n"/>
+      <c r="L28" s="107" t="n"/>
+      <c r="M28" s="107" t="n"/>
+      <c r="N28" s="107" t="n"/>
+      <c r="O28" s="107" t="n"/>
+      <c r="P28" s="91" t="n"/>
+      <c r="Q28" s="91" t="n"/>
     </row>
     <row r="29"/>
     <row r="30">
-      <c r="A30" s="95" t="inlineStr">
+      <c r="A30" s="97" t="inlineStr">
         <is>
           <t>🍽️ MEALS</t>
         </is>
@@ -4275,274 +4297,274 @@
       <c r="I30" s="48" t="n"/>
       <c r="J30" s="48" t="n"/>
       <c r="K30" s="46" t="n"/>
-      <c r="L30" s="91" t="inlineStr">
+      <c r="L30" s="93" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="M30" s="94" t="n"/>
-      <c r="N30" s="94" t="n"/>
-      <c r="O30" s="94" t="n"/>
-      <c r="P30" s="94" t="n"/>
-      <c r="Q30" s="94" t="n"/>
+      <c r="M30" s="96" t="n"/>
+      <c r="N30" s="96" t="n"/>
+      <c r="O30" s="96" t="n"/>
+      <c r="P30" s="96" t="n"/>
+      <c r="Q30" s="96" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1" s="44">
-      <c r="A31" s="96" t="inlineStr">
+      <c r="A31" s="84" t="inlineStr">
         <is>
           <t>Dinner (Regular)</t>
         </is>
       </c>
-      <c r="B31" s="97" t="n">
+      <c r="B31" s="98" t="n">
         <v>3</v>
       </c>
-      <c r="C31" s="98">
+      <c r="C31" s="99">
         <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$42:$C$50,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D31" s="98">
+      <c r="D31" s="99">
         <f>IF(A31="","",VLOOKUP(A31,'Master Data'!$A$42:$C$50,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E31" s="99">
+      <c r="E31" s="100">
         <f>IF(D31&gt;0,(D31-C31)/D31,0)</f>
         <v/>
       </c>
-      <c r="F31" s="87" t="n"/>
-      <c r="G31" s="87" t="n"/>
-      <c r="H31" s="87" t="n"/>
-      <c r="I31" s="87" t="n"/>
-      <c r="J31" s="100" t="inlineStr">
+      <c r="F31" s="89" t="n"/>
+      <c r="G31" s="89" t="n"/>
+      <c r="H31" s="89" t="n"/>
+      <c r="I31" s="89" t="n"/>
+      <c r="J31" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K31" s="98">
+      <c r="K31" s="99">
         <f>IF(A31="","",IF(L30="PG",IF((F31="●")+(G31="●")+(H31="●")+(I31="●")+(L31="●")+(M31="●")+(N31="●")+(O31="●")&gt;0,B31*C31,0),ROUNDUP((F31="●")+(G31="●")+(H31="●")+(I31="●")+(L31="●")+(M31="●")+(N31="●")+(O31="●")/VALUE(MID(L30,2,2)),0)*B31*C31))</f>
         <v/>
       </c>
-      <c r="L31" s="98">
+      <c r="L31" s="99">
         <f>IF(A31="","",IF(L30="PG",IF((F31="●")+(G31="●")+(H31="●")+(I31="●")+(L31="●")+(M31="●")+(N31="●")+(O31="●")&gt;0,B31*D31,0),ROUNDUP((F31="●")+(G31="●")+(H31="●")+(I31="●")+(L31="●")+(M31="●")+(N31="●")+(O31="●")/VALUE(MID(L30,2,2)),0)*B31*D31))</f>
         <v/>
       </c>
-      <c r="M31" s="87" t="n"/>
-      <c r="N31" s="87" t="n"/>
-      <c r="O31" s="87" t="n"/>
+      <c r="M31" s="89" t="n"/>
+      <c r="N31" s="89" t="n"/>
+      <c r="O31" s="89" t="n"/>
       <c r="P31" s="5">
         <f>IF(A31="",0,COUNTIF(A$30:A30,A31))</f>
         <v/>
       </c>
-      <c r="Q31" s="87" t="n"/>
+      <c r="Q31" s="89" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1" s="44">
-      <c r="A32" s="96" t="inlineStr">
+      <c r="A32" s="84" t="inlineStr">
         <is>
           <t>Exclusive Dinner (Michelin/Fine)</t>
         </is>
       </c>
-      <c r="B32" s="97" t="n">
+      <c r="B32" s="98" t="n">
         <v>2</v>
       </c>
-      <c r="C32" s="98">
+      <c r="C32" s="99">
         <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$42:$C$50,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D32" s="98">
+      <c r="D32" s="99">
         <f>IF(A32="","",VLOOKUP(A32,'Master Data'!$A$42:$C$50,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E32" s="99">
+      <c r="E32" s="100">
         <f>IF(D32&gt;0,(D32-C32)/D32,0)</f>
         <v/>
       </c>
-      <c r="F32" s="87" t="n"/>
-      <c r="G32" s="87" t="n"/>
-      <c r="H32" s="87" t="n"/>
-      <c r="I32" s="87" t="n"/>
-      <c r="J32" s="100" t="inlineStr">
+      <c r="F32" s="89" t="n"/>
+      <c r="G32" s="89" t="n"/>
+      <c r="H32" s="89" t="n"/>
+      <c r="I32" s="89" t="n"/>
+      <c r="J32" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K32" s="98">
+      <c r="K32" s="99">
         <f>IF(A32="","",IF(L30="PG",IF((F32="●")+(G32="●")+(H32="●")+(I32="●")+(L32="●")+(M32="●")+(N32="●")+(O32="●")&gt;0,B32*C32,0),ROUNDUP((F32="●")+(G32="●")+(H32="●")+(I32="●")+(L32="●")+(M32="●")+(N32="●")+(O32="●")/VALUE(MID(L30,2,2)),0)*B32*C32))</f>
         <v/>
       </c>
-      <c r="L32" s="98">
+      <c r="L32" s="99">
         <f>IF(A32="","",IF(L30="PG",IF((F32="●")+(G32="●")+(H32="●")+(I32="●")+(L32="●")+(M32="●")+(N32="●")+(O32="●")&gt;0,B32*D32,0),ROUNDUP((F32="●")+(G32="●")+(H32="●")+(I32="●")+(L32="●")+(M32="●")+(N32="●")+(O32="●")/VALUE(MID(L30,2,2)),0)*B32*D32))</f>
         <v/>
       </c>
-      <c r="M32" s="87" t="n"/>
-      <c r="N32" s="87" t="n"/>
-      <c r="O32" s="87" t="n"/>
+      <c r="M32" s="89" t="n"/>
+      <c r="N32" s="89" t="n"/>
+      <c r="O32" s="89" t="n"/>
       <c r="P32" s="5">
         <f>IF(A32="",0,COUNTIF(A$30:A31,A32))</f>
         <v/>
       </c>
-      <c r="Q32" s="87" t="n"/>
+      <c r="Q32" s="89" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1" s="44">
-      <c r="A33" s="96" t="inlineStr">
+      <c r="A33" s="84" t="inlineStr">
         <is>
           <t>Lunch</t>
         </is>
       </c>
-      <c r="B33" s="97" t="n">
+      <c r="B33" s="98" t="n">
         <v>3</v>
       </c>
-      <c r="C33" s="98">
+      <c r="C33" s="99">
         <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$42:$C$50,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D33" s="98">
+      <c r="D33" s="99">
         <f>IF(A33="","",VLOOKUP(A33,'Master Data'!$A$42:$C$50,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E33" s="99">
+      <c r="E33" s="100">
         <f>IF(D33&gt;0,(D33-C33)/D33,0)</f>
         <v/>
       </c>
-      <c r="F33" s="87" t="n"/>
-      <c r="G33" s="87" t="n"/>
-      <c r="H33" s="87" t="n"/>
-      <c r="I33" s="87" t="n"/>
-      <c r="J33" s="100" t="inlineStr">
+      <c r="F33" s="89" t="n"/>
+      <c r="G33" s="89" t="n"/>
+      <c r="H33" s="89" t="n"/>
+      <c r="I33" s="89" t="n"/>
+      <c r="J33" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K33" s="98">
+      <c r="K33" s="99">
         <f>IF(A33="","",IF(L30="PG",IF((F33="●")+(G33="●")+(H33="●")+(I33="●")+(L33="●")+(M33="●")+(N33="●")+(O33="●")&gt;0,B33*C33,0),ROUNDUP((F33="●")+(G33="●")+(H33="●")+(I33="●")+(L33="●")+(M33="●")+(N33="●")+(O33="●")/VALUE(MID(L30,2,2)),0)*B33*C33))</f>
         <v/>
       </c>
-      <c r="L33" s="98">
+      <c r="L33" s="99">
         <f>IF(A33="","",IF(L30="PG",IF((F33="●")+(G33="●")+(H33="●")+(I33="●")+(L33="●")+(M33="●")+(N33="●")+(O33="●")&gt;0,B33*D33,0),ROUNDUP((F33="●")+(G33="●")+(H33="●")+(I33="●")+(L33="●")+(M33="●")+(N33="●")+(O33="●")/VALUE(MID(L30,2,2)),0)*B33*D33))</f>
         <v/>
       </c>
-      <c r="M33" s="87" t="n"/>
-      <c r="N33" s="87" t="n"/>
-      <c r="O33" s="87" t="n"/>
+      <c r="M33" s="89" t="n"/>
+      <c r="N33" s="89" t="n"/>
+      <c r="O33" s="89" t="n"/>
       <c r="P33" s="5">
         <f>IF(A33="",0,COUNTIF(A$30:A32,A33))</f>
         <v/>
       </c>
-      <c r="Q33" s="87" t="n"/>
+      <c r="Q33" s="89" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1" s="44">
-      <c r="A34" s="101" t="n"/>
-      <c r="B34" s="100" t="n"/>
-      <c r="C34" s="98">
+      <c r="A34" s="102" t="n"/>
+      <c r="B34" s="101" t="n"/>
+      <c r="C34" s="99">
         <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$42:$C$50,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D34" s="98">
+      <c r="D34" s="99">
         <f>IF(A34="","",VLOOKUP(A34,'Master Data'!$A$42:$C$50,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E34" s="99">
+      <c r="E34" s="100">
         <f>IF(D34&gt;0,(D34-C34)/D34,0)</f>
         <v/>
       </c>
-      <c r="F34" s="87" t="n"/>
-      <c r="G34" s="87" t="n"/>
-      <c r="H34" s="87" t="n"/>
-      <c r="I34" s="87" t="n"/>
-      <c r="J34" s="100" t="inlineStr">
+      <c r="F34" s="89" t="n"/>
+      <c r="G34" s="89" t="n"/>
+      <c r="H34" s="89" t="n"/>
+      <c r="I34" s="89" t="n"/>
+      <c r="J34" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K34" s="98">
+      <c r="K34" s="99">
         <f>IF(A34="","",IF(L30="PG",IF((F34="●")+(G34="●")+(H34="●")+(I34="●")+(L34="●")+(M34="●")+(N34="●")+(O34="●")&gt;0,B34*C34,0),ROUNDUP((F34="●")+(G34="●")+(H34="●")+(I34="●")+(L34="●")+(M34="●")+(N34="●")+(O34="●")/VALUE(MID(L30,2,2)),0)*B34*C34))</f>
         <v/>
       </c>
-      <c r="L34" s="98">
+      <c r="L34" s="99">
         <f>IF(A34="","",IF(L30="PG",IF((F34="●")+(G34="●")+(H34="●")+(I34="●")+(L34="●")+(M34="●")+(N34="●")+(O34="●")&gt;0,B34*D34,0),ROUNDUP((F34="●")+(G34="●")+(H34="●")+(I34="●")+(L34="●")+(M34="●")+(N34="●")+(O34="●")/VALUE(MID(L30,2,2)),0)*B34*D34))</f>
         <v/>
       </c>
-      <c r="M34" s="87" t="n"/>
-      <c r="N34" s="87" t="n"/>
-      <c r="O34" s="87" t="n"/>
+      <c r="M34" s="89" t="n"/>
+      <c r="N34" s="89" t="n"/>
+      <c r="O34" s="89" t="n"/>
       <c r="P34" s="5">
         <f>IF(A34="",0,COUNTIF(A$30:A33,A34))</f>
         <v/>
       </c>
-      <c r="Q34" s="87" t="n"/>
+      <c r="Q34" s="89" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1" s="44">
-      <c r="A35" s="102" t="inlineStr">
+      <c r="A35" s="103" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B35" s="104" t="n"/>
-      <c r="C35" s="104" t="n"/>
-      <c r="D35" s="104" t="n"/>
-      <c r="E35" s="105" t="n"/>
-      <c r="F35" s="103">
+      <c r="B35" s="105" t="n"/>
+      <c r="C35" s="105" t="n"/>
+      <c r="D35" s="105" t="n"/>
+      <c r="E35" s="106" t="n"/>
+      <c r="F35" s="104">
         <f>SUMPRODUCT((F30:F34="●")*1,B30:B34,C30:C34)</f>
         <v/>
       </c>
-      <c r="G35" s="103">
+      <c r="G35" s="104">
         <f>SUMPRODUCT((G30:G34="●")*1,B30:B34,C30:C34)</f>
         <v/>
       </c>
-      <c r="H35" s="103">
+      <c r="H35" s="104">
         <f>SUMPRODUCT((H30:H34="●")*1,B30:B34,C30:C34)</f>
         <v/>
       </c>
-      <c r="I35" s="103">
+      <c r="I35" s="104">
         <f>SUMPRODUCT((I30:I34="●")*1,B30:B34,C30:C34)</f>
         <v/>
       </c>
-      <c r="J35" s="104" t="n"/>
-      <c r="K35" s="103">
+      <c r="J35" s="105" t="n"/>
+      <c r="K35" s="104">
         <f>SUM(K30:K34)</f>
         <v/>
       </c>
-      <c r="L35" s="103">
+      <c r="L35" s="104">
         <f>SUM(L30:L34)</f>
         <v/>
       </c>
-      <c r="M35" s="103">
+      <c r="M35" s="104">
         <f>SUMPRODUCT((M30:M34="●")*1,B30:B34,C30:C34)</f>
         <v/>
       </c>
-      <c r="N35" s="103">
+      <c r="N35" s="104">
         <f>SUMPRODUCT((N30:N34="●")*1,B30:B34,C30:C34)</f>
         <v/>
       </c>
-      <c r="O35" s="103">
+      <c r="O35" s="104">
         <f>SUMPRODUCT((O30:O34="●")*1,B30:B34,C30:C34)</f>
         <v/>
       </c>
-      <c r="P35" s="91">
+      <c r="P35" s="93">
         <f>SUM(P30:P34)</f>
         <v/>
       </c>
-      <c r="Q35" s="91" t="n"/>
+      <c r="Q35" s="93" t="n"/>
     </row>
     <row r="36" ht="6" customHeight="1" s="44">
-      <c r="A36" s="89" t="n"/>
-      <c r="B36" s="89" t="n"/>
-      <c r="C36" s="89" t="n"/>
-      <c r="D36" s="89" t="n"/>
-      <c r="E36" s="89" t="n"/>
-      <c r="F36" s="106" t="n"/>
-      <c r="G36" s="106" t="n"/>
-      <c r="H36" s="106" t="n"/>
-      <c r="I36" s="106" t="n"/>
-      <c r="J36" s="106" t="n"/>
-      <c r="K36" s="106" t="n"/>
-      <c r="L36" s="106" t="n"/>
-      <c r="M36" s="106" t="n"/>
-      <c r="N36" s="106" t="n"/>
-      <c r="O36" s="106" t="n"/>
-      <c r="P36" s="89" t="n"/>
-      <c r="Q36" s="89" t="n"/>
+      <c r="A36" s="91" t="n"/>
+      <c r="B36" s="91" t="n"/>
+      <c r="C36" s="91" t="n"/>
+      <c r="D36" s="91" t="n"/>
+      <c r="E36" s="91" t="n"/>
+      <c r="F36" s="107" t="n"/>
+      <c r="G36" s="107" t="n"/>
+      <c r="H36" s="107" t="n"/>
+      <c r="I36" s="107" t="n"/>
+      <c r="J36" s="107" t="n"/>
+      <c r="K36" s="107" t="n"/>
+      <c r="L36" s="107" t="n"/>
+      <c r="M36" s="107" t="n"/>
+      <c r="N36" s="107" t="n"/>
+      <c r="O36" s="107" t="n"/>
+      <c r="P36" s="91" t="n"/>
+      <c r="Q36" s="91" t="n"/>
     </row>
     <row r="37"/>
     <row r="38">
-      <c r="A38" s="95" t="inlineStr">
+      <c r="A38" s="97" t="inlineStr">
         <is>
           <t>📦 OTHER</t>
         </is>
@@ -4557,174 +4579,174 @@
       <c r="I38" s="48" t="n"/>
       <c r="J38" s="48" t="n"/>
       <c r="K38" s="46" t="n"/>
-      <c r="L38" s="91" t="inlineStr">
+      <c r="L38" s="93" t="inlineStr">
         <is>
           <t>PG</t>
         </is>
       </c>
-      <c r="M38" s="94" t="n"/>
-      <c r="N38" s="94" t="n"/>
-      <c r="O38" s="94" t="n"/>
-      <c r="P38" s="94" t="n"/>
-      <c r="Q38" s="94" t="n"/>
+      <c r="M38" s="96" t="n"/>
+      <c r="N38" s="96" t="n"/>
+      <c r="O38" s="96" t="n"/>
+      <c r="P38" s="96" t="n"/>
+      <c r="Q38" s="96" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1" s="44">
-      <c r="A39" s="101" t="n"/>
-      <c r="B39" s="100" t="n"/>
-      <c r="C39" s="98">
+      <c r="A39" s="102" t="n"/>
+      <c r="B39" s="101" t="n"/>
+      <c r="C39" s="99">
         <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$55:$C$61,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D39" s="98">
+      <c r="D39" s="99">
         <f>IF(A39="","",VLOOKUP(A39,'Master Data'!$A$55:$C$61,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E39" s="99">
+      <c r="E39" s="100">
         <f>IF(D39&gt;0,(D39-C39)/D39,0)</f>
         <v/>
       </c>
-      <c r="F39" s="87" t="n"/>
-      <c r="G39" s="87" t="n"/>
-      <c r="H39" s="87" t="n"/>
-      <c r="I39" s="87" t="n"/>
-      <c r="J39" s="100" t="inlineStr">
+      <c r="F39" s="89" t="n"/>
+      <c r="G39" s="89" t="n"/>
+      <c r="H39" s="89" t="n"/>
+      <c r="I39" s="89" t="n"/>
+      <c r="J39" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K39" s="98">
+      <c r="K39" s="99">
         <f>IF(A39="","",IF(L38="PG",IF((F39="●")+(G39="●")+(H39="●")+(I39="●")+(L39="●")+(M39="●")+(N39="●")+(O39="●")&gt;0,B39*C39,0),ROUNDUP((F39="●")+(G39="●")+(H39="●")+(I39="●")+(L39="●")+(M39="●")+(N39="●")+(O39="●")/VALUE(MID(L38,2,2)),0)*B39*C39))</f>
         <v/>
       </c>
-      <c r="L39" s="98">
+      <c r="L39" s="99">
         <f>IF(A39="","",IF(L38="PG",IF((F39="●")+(G39="●")+(H39="●")+(I39="●")+(L39="●")+(M39="●")+(N39="●")+(O39="●")&gt;0,B39*D39,0),ROUNDUP((F39="●")+(G39="●")+(H39="●")+(I39="●")+(L39="●")+(M39="●")+(N39="●")+(O39="●")/VALUE(MID(L38,2,2)),0)*B39*D39))</f>
         <v/>
       </c>
-      <c r="M39" s="87" t="n"/>
-      <c r="N39" s="87" t="n"/>
-      <c r="O39" s="87" t="n"/>
+      <c r="M39" s="89" t="n"/>
+      <c r="N39" s="89" t="n"/>
+      <c r="O39" s="89" t="n"/>
       <c r="P39" s="5">
         <f>IF(A39="",0,COUNTIF(A$38:A38,A39))</f>
         <v/>
       </c>
-      <c r="Q39" s="87" t="n"/>
+      <c r="Q39" s="89" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1" s="44">
-      <c r="A40" s="101" t="n"/>
-      <c r="B40" s="100" t="n"/>
-      <c r="C40" s="98">
+      <c r="A40" s="102" t="n"/>
+      <c r="B40" s="101" t="n"/>
+      <c r="C40" s="99">
         <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$55:$C$61,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D40" s="98">
+      <c r="D40" s="99">
         <f>IF(A40="","",VLOOKUP(A40,'Master Data'!$A$55:$C$61,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E40" s="99">
+      <c r="E40" s="100">
         <f>IF(D40&gt;0,(D40-C40)/D40,0)</f>
         <v/>
       </c>
-      <c r="F40" s="87" t="n"/>
-      <c r="G40" s="87" t="n"/>
-      <c r="H40" s="87" t="n"/>
-      <c r="I40" s="87" t="n"/>
-      <c r="J40" s="100" t="inlineStr">
+      <c r="F40" s="89" t="n"/>
+      <c r="G40" s="89" t="n"/>
+      <c r="H40" s="89" t="n"/>
+      <c r="I40" s="89" t="n"/>
+      <c r="J40" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K40" s="98">
+      <c r="K40" s="99">
         <f>IF(A40="","",IF(L38="PG",IF((F40="●")+(G40="●")+(H40="●")+(I40="●")+(L40="●")+(M40="●")+(N40="●")+(O40="●")&gt;0,B40*C40,0),ROUNDUP((F40="●")+(G40="●")+(H40="●")+(I40="●")+(L40="●")+(M40="●")+(N40="●")+(O40="●")/VALUE(MID(L38,2,2)),0)*B40*C40))</f>
         <v/>
       </c>
-      <c r="L40" s="98">
+      <c r="L40" s="99">
         <f>IF(A40="","",IF(L38="PG",IF((F40="●")+(G40="●")+(H40="●")+(I40="●")+(L40="●")+(M40="●")+(N40="●")+(O40="●")&gt;0,B40*D40,0),ROUNDUP((F40="●")+(G40="●")+(H40="●")+(I40="●")+(L40="●")+(M40="●")+(N40="●")+(O40="●")/VALUE(MID(L38,2,2)),0)*B40*D40))</f>
         <v/>
       </c>
-      <c r="M40" s="87" t="n"/>
-      <c r="N40" s="87" t="n"/>
-      <c r="O40" s="87" t="n"/>
+      <c r="M40" s="89" t="n"/>
+      <c r="N40" s="89" t="n"/>
+      <c r="O40" s="89" t="n"/>
       <c r="P40" s="5">
         <f>IF(A40="",0,COUNTIF(A$38:A39,A40))</f>
         <v/>
       </c>
-      <c r="Q40" s="87" t="n"/>
+      <c r="Q40" s="89" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1" s="44">
-      <c r="A41" s="102" t="inlineStr">
+      <c r="A41" s="103" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B41" s="104" t="n"/>
-      <c r="C41" s="104" t="n"/>
-      <c r="D41" s="104" t="n"/>
-      <c r="E41" s="105" t="n"/>
-      <c r="F41" s="103">
+      <c r="B41" s="105" t="n"/>
+      <c r="C41" s="105" t="n"/>
+      <c r="D41" s="105" t="n"/>
+      <c r="E41" s="106" t="n"/>
+      <c r="F41" s="104">
         <f>SUMPRODUCT((F38:F40="●")*1,B38:B40,C38:C40)</f>
         <v/>
       </c>
-      <c r="G41" s="103">
+      <c r="G41" s="104">
         <f>SUMPRODUCT((G38:G40="●")*1,B38:B40,C38:C40)</f>
         <v/>
       </c>
-      <c r="H41" s="103">
+      <c r="H41" s="104">
         <f>SUMPRODUCT((H38:H40="●")*1,B38:B40,C38:C40)</f>
         <v/>
       </c>
-      <c r="I41" s="103">
+      <c r="I41" s="104">
         <f>SUMPRODUCT((I38:I40="●")*1,B38:B40,C38:C40)</f>
         <v/>
       </c>
-      <c r="J41" s="104" t="n"/>
-      <c r="K41" s="103">
+      <c r="J41" s="105" t="n"/>
+      <c r="K41" s="104">
         <f>SUM(K38:K40)</f>
         <v/>
       </c>
-      <c r="L41" s="103">
+      <c r="L41" s="104">
         <f>SUM(L38:L40)</f>
         <v/>
       </c>
-      <c r="M41" s="103">
+      <c r="M41" s="104">
         <f>SUMPRODUCT((M38:M40="●")*1,B38:B40,C38:C40)</f>
         <v/>
       </c>
-      <c r="N41" s="103">
+      <c r="N41" s="104">
         <f>SUMPRODUCT((N38:N40="●")*1,B38:B40,C38:C40)</f>
         <v/>
       </c>
-      <c r="O41" s="103">
+      <c r="O41" s="104">
         <f>SUMPRODUCT((O38:O40="●")*1,B38:B40,C38:C40)</f>
         <v/>
       </c>
-      <c r="P41" s="91">
+      <c r="P41" s="93">
         <f>SUM(P38:P40)</f>
         <v/>
       </c>
-      <c r="Q41" s="91" t="n"/>
+      <c r="Q41" s="93" t="n"/>
     </row>
     <row r="42" ht="6" customHeight="1" s="44">
-      <c r="A42" s="89" t="n"/>
-      <c r="B42" s="89" t="n"/>
-      <c r="C42" s="89" t="n"/>
-      <c r="D42" s="89" t="n"/>
-      <c r="E42" s="89" t="n"/>
-      <c r="F42" s="106" t="n"/>
-      <c r="G42" s="106" t="n"/>
-      <c r="H42" s="106" t="n"/>
-      <c r="I42" s="106" t="n"/>
-      <c r="J42" s="106" t="n"/>
-      <c r="K42" s="106" t="n"/>
-      <c r="L42" s="106" t="n"/>
-      <c r="M42" s="106" t="n"/>
-      <c r="N42" s="106" t="n"/>
-      <c r="O42" s="106" t="n"/>
-      <c r="P42" s="89" t="n"/>
-      <c r="Q42" s="89" t="n"/>
+      <c r="A42" s="91" t="n"/>
+      <c r="B42" s="91" t="n"/>
+      <c r="C42" s="91" t="n"/>
+      <c r="D42" s="91" t="n"/>
+      <c r="E42" s="91" t="n"/>
+      <c r="F42" s="107" t="n"/>
+      <c r="G42" s="107" t="n"/>
+      <c r="H42" s="107" t="n"/>
+      <c r="I42" s="107" t="n"/>
+      <c r="J42" s="107" t="n"/>
+      <c r="K42" s="107" t="n"/>
+      <c r="L42" s="107" t="n"/>
+      <c r="M42" s="107" t="n"/>
+      <c r="N42" s="107" t="n"/>
+      <c r="O42" s="107" t="n"/>
+      <c r="P42" s="91" t="n"/>
+      <c r="Q42" s="91" t="n"/>
     </row>
     <row r="43"/>
     <row r="44">
-      <c r="A44" s="95" t="inlineStr">
+      <c r="A44" s="97" t="inlineStr">
         <is>
           <t>🎯 ACTIVITIES</t>
         </is>
@@ -4739,438 +4761,438 @@
       <c r="I44" s="48" t="n"/>
       <c r="J44" s="48" t="n"/>
       <c r="K44" s="46" t="n"/>
-      <c r="L44" s="91" t="inlineStr">
+      <c r="L44" s="93" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="M44" s="94" t="n"/>
-      <c r="N44" s="94" t="n"/>
-      <c r="O44" s="94" t="n"/>
-      <c r="P44" s="94" t="n"/>
-      <c r="Q44" s="94" t="n"/>
+      <c r="M44" s="96" t="n"/>
+      <c r="N44" s="96" t="n"/>
+      <c r="O44" s="96" t="n"/>
+      <c r="P44" s="96" t="n"/>
+      <c r="Q44" s="96" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1" s="44">
-      <c r="A45" s="96" t="inlineStr">
+      <c r="A45" s="84" t="inlineStr">
         <is>
           <t>Local Hiking (Griffith/Runyon)</t>
         </is>
       </c>
-      <c r="B45" s="97" t="n">
+      <c r="B45" s="98" t="n">
         <v>1</v>
       </c>
-      <c r="C45" s="98">
+      <c r="C45" s="99">
         <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$65:$C$73,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D45" s="98">
+      <c r="D45" s="99">
         <f>IF(A45="","",VLOOKUP(A45,'Master Data'!$A$65:$C$73,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E45" s="99">
+      <c r="E45" s="100">
         <f>IF(D45&gt;0,(D45-C45)/D45,0)</f>
         <v/>
       </c>
-      <c r="F45" s="87" t="n"/>
-      <c r="G45" s="87" t="n"/>
-      <c r="H45" s="87" t="n"/>
-      <c r="I45" s="87" t="n"/>
-      <c r="J45" s="100" t="inlineStr">
+      <c r="F45" s="89" t="n"/>
+      <c r="G45" s="89" t="n"/>
+      <c r="H45" s="89" t="n"/>
+      <c r="I45" s="89" t="n"/>
+      <c r="J45" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K45" s="98">
+      <c r="K45" s="99">
         <f>IF(A45="","",IF(L44="PG",IF((F45="●")+(G45="●")+(H45="●")+(I45="●")+(L45="●")+(M45="●")+(N45="●")+(O45="●")&gt;0,B45*C45,0),ROUNDUP((F45="●")+(G45="●")+(H45="●")+(I45="●")+(L45="●")+(M45="●")+(N45="●")+(O45="●")/VALUE(MID(L44,2,2)),0)*B45*C45))</f>
         <v/>
       </c>
-      <c r="L45" s="98">
+      <c r="L45" s="99">
         <f>IF(A45="","",IF(L44="PG",IF((F45="●")+(G45="●")+(H45="●")+(I45="●")+(L45="●")+(M45="●")+(N45="●")+(O45="●")&gt;0,B45*D45,0),ROUNDUP((F45="●")+(G45="●")+(H45="●")+(I45="●")+(L45="●")+(M45="●")+(N45="●")+(O45="●")/VALUE(MID(L44,2,2)),0)*B45*D45))</f>
         <v/>
       </c>
-      <c r="M45" s="87" t="n"/>
-      <c r="N45" s="87" t="n"/>
-      <c r="O45" s="87" t="n"/>
+      <c r="M45" s="89" t="n"/>
+      <c r="N45" s="89" t="n"/>
+      <c r="O45" s="89" t="n"/>
       <c r="P45" s="5">
         <f>IF(A45="",0,COUNTIF(A$44:A44,A45))</f>
         <v/>
       </c>
-      <c r="Q45" s="87" t="n"/>
+      <c r="Q45" s="89" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1" s="44">
-      <c r="A46" s="96" t="inlineStr">
+      <c r="A46" s="84" t="inlineStr">
         <is>
           <t>NBA/MLB Game (Ticket)</t>
         </is>
       </c>
-      <c r="B46" s="97" t="n">
+      <c r="B46" s="98" t="n">
         <v>1</v>
       </c>
-      <c r="C46" s="98">
+      <c r="C46" s="99">
         <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$65:$C$73,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D46" s="98">
+      <c r="D46" s="99">
         <f>IF(A46="","",VLOOKUP(A46,'Master Data'!$A$65:$C$73,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E46" s="99">
+      <c r="E46" s="100">
         <f>IF(D46&gt;0,(D46-C46)/D46,0)</f>
         <v/>
       </c>
-      <c r="F46" s="87" t="n"/>
-      <c r="G46" s="87" t="n"/>
-      <c r="H46" s="87" t="n"/>
-      <c r="I46" s="87" t="n"/>
-      <c r="J46" s="100" t="inlineStr">
+      <c r="F46" s="89" t="n"/>
+      <c r="G46" s="89" t="n"/>
+      <c r="H46" s="89" t="n"/>
+      <c r="I46" s="89" t="n"/>
+      <c r="J46" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K46" s="98">
+      <c r="K46" s="99">
         <f>IF(A46="","",IF(L44="PG",IF((F46="●")+(G46="●")+(H46="●")+(I46="●")+(L46="●")+(M46="●")+(N46="●")+(O46="●")&gt;0,B46*C46,0),ROUNDUP((F46="●")+(G46="●")+(H46="●")+(I46="●")+(L46="●")+(M46="●")+(N46="●")+(O46="●")/VALUE(MID(L44,2,2)),0)*B46*C46))</f>
         <v/>
       </c>
-      <c r="L46" s="98">
+      <c r="L46" s="99">
         <f>IF(A46="","",IF(L44="PG",IF((F46="●")+(G46="●")+(H46="●")+(I46="●")+(L46="●")+(M46="●")+(N46="●")+(O46="●")&gt;0,B46*D46,0),ROUNDUP((F46="●")+(G46="●")+(H46="●")+(I46="●")+(L46="●")+(M46="●")+(N46="●")+(O46="●")/VALUE(MID(L44,2,2)),0)*B46*D46))</f>
         <v/>
       </c>
-      <c r="M46" s="87" t="n"/>
-      <c r="N46" s="87" t="n"/>
-      <c r="O46" s="87" t="n"/>
+      <c r="M46" s="89" t="n"/>
+      <c r="N46" s="89" t="n"/>
+      <c r="O46" s="89" t="n"/>
       <c r="P46" s="5">
         <f>IF(A46="",0,COUNTIF(A$44:A45,A46))</f>
         <v/>
       </c>
-      <c r="Q46" s="87" t="n"/>
+      <c r="Q46" s="89" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1" s="44">
-      <c r="A47" s="96" t="inlineStr">
+      <c r="A47" s="84" t="inlineStr">
         <is>
           <t>Sports Bar Experience</t>
         </is>
       </c>
-      <c r="B47" s="97" t="n">
+      <c r="B47" s="98" t="n">
         <v>1</v>
       </c>
-      <c r="C47" s="98">
+      <c r="C47" s="99">
         <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$65:$C$73,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D47" s="98">
+      <c r="D47" s="99">
         <f>IF(A47="","",VLOOKUP(A47,'Master Data'!$A$65:$C$73,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E47" s="99">
+      <c r="E47" s="100">
         <f>IF(D47&gt;0,(D47-C47)/D47,0)</f>
         <v/>
       </c>
-      <c r="F47" s="87" t="n"/>
-      <c r="G47" s="87" t="n"/>
-      <c r="H47" s="87" t="n"/>
-      <c r="I47" s="87" t="n"/>
-      <c r="J47" s="100" t="inlineStr">
+      <c r="F47" s="89" t="n"/>
+      <c r="G47" s="89" t="n"/>
+      <c r="H47" s="89" t="n"/>
+      <c r="I47" s="89" t="n"/>
+      <c r="J47" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K47" s="98">
+      <c r="K47" s="99">
         <f>IF(A47="","",IF(L44="PG",IF((F47="●")+(G47="●")+(H47="●")+(I47="●")+(L47="●")+(M47="●")+(N47="●")+(O47="●")&gt;0,B47*C47,0),ROUNDUP((F47="●")+(G47="●")+(H47="●")+(I47="●")+(L47="●")+(M47="●")+(N47="●")+(O47="●")/VALUE(MID(L44,2,2)),0)*B47*C47))</f>
         <v/>
       </c>
-      <c r="L47" s="98">
+      <c r="L47" s="99">
         <f>IF(A47="","",IF(L44="PG",IF((F47="●")+(G47="●")+(H47="●")+(I47="●")+(L47="●")+(M47="●")+(N47="●")+(O47="●")&gt;0,B47*D47,0),ROUNDUP((F47="●")+(G47="●")+(H47="●")+(I47="●")+(L47="●")+(M47="●")+(N47="●")+(O47="●")/VALUE(MID(L44,2,2)),0)*B47*D47))</f>
         <v/>
       </c>
-      <c r="M47" s="87" t="n"/>
-      <c r="N47" s="87" t="n"/>
-      <c r="O47" s="87" t="n"/>
+      <c r="M47" s="89" t="n"/>
+      <c r="N47" s="89" t="n"/>
+      <c r="O47" s="89" t="n"/>
       <c r="P47" s="5">
         <f>IF(A47="",0,COUNTIF(A$44:A46,A47))</f>
         <v/>
       </c>
-      <c r="Q47" s="87" t="n"/>
+      <c r="Q47" s="89" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1" s="44">
-      <c r="A48" s="101" t="n"/>
-      <c r="B48" s="100" t="n"/>
-      <c r="C48" s="98">
+      <c r="A48" s="102" t="n"/>
+      <c r="B48" s="101" t="n"/>
+      <c r="C48" s="99">
         <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$65:$C$73,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D48" s="98">
+      <c r="D48" s="99">
         <f>IF(A48="","",VLOOKUP(A48,'Master Data'!$A$65:$C$73,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E48" s="99">
+      <c r="E48" s="100">
         <f>IF(D48&gt;0,(D48-C48)/D48,0)</f>
         <v/>
       </c>
-      <c r="F48" s="87" t="n"/>
-      <c r="G48" s="87" t="n"/>
-      <c r="H48" s="87" t="n"/>
-      <c r="I48" s="87" t="n"/>
-      <c r="J48" s="100" t="inlineStr">
+      <c r="F48" s="89" t="n"/>
+      <c r="G48" s="89" t="n"/>
+      <c r="H48" s="89" t="n"/>
+      <c r="I48" s="89" t="n"/>
+      <c r="J48" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K48" s="98">
+      <c r="K48" s="99">
         <f>IF(A48="","",IF(L44="PG",IF((F48="●")+(G48="●")+(H48="●")+(I48="●")+(L48="●")+(M48="●")+(N48="●")+(O48="●")&gt;0,B48*C48,0),ROUNDUP((F48="●")+(G48="●")+(H48="●")+(I48="●")+(L48="●")+(M48="●")+(N48="●")+(O48="●")/VALUE(MID(L44,2,2)),0)*B48*C48))</f>
         <v/>
       </c>
-      <c r="L48" s="98">
+      <c r="L48" s="99">
         <f>IF(A48="","",IF(L44="PG",IF((F48="●")+(G48="●")+(H48="●")+(I48="●")+(L48="●")+(M48="●")+(N48="●")+(O48="●")&gt;0,B48*D48,0),ROUNDUP((F48="●")+(G48="●")+(H48="●")+(I48="●")+(L48="●")+(M48="●")+(N48="●")+(O48="●")/VALUE(MID(L44,2,2)),0)*B48*D48))</f>
         <v/>
       </c>
-      <c r="M48" s="87" t="n"/>
-      <c r="N48" s="87" t="n"/>
-      <c r="O48" s="87" t="n"/>
+      <c r="M48" s="89" t="n"/>
+      <c r="N48" s="89" t="n"/>
+      <c r="O48" s="89" t="n"/>
       <c r="P48" s="5">
         <f>IF(A48="",0,COUNTIF(A$44:A47,A48))</f>
         <v/>
       </c>
-      <c r="Q48" s="87" t="n"/>
+      <c r="Q48" s="89" t="n"/>
     </row>
     <row r="49" ht="18" customHeight="1" s="44">
-      <c r="A49" s="101" t="n"/>
-      <c r="B49" s="100" t="n"/>
-      <c r="C49" s="98">
+      <c r="A49" s="102" t="n"/>
+      <c r="B49" s="101" t="n"/>
+      <c r="C49" s="99">
         <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$65:$C$73,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D49" s="98">
+      <c r="D49" s="99">
         <f>IF(A49="","",VLOOKUP(A49,'Master Data'!$A$65:$C$73,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E49" s="99">
+      <c r="E49" s="100">
         <f>IF(D49&gt;0,(D49-C49)/D49,0)</f>
         <v/>
       </c>
-      <c r="F49" s="87" t="n"/>
-      <c r="G49" s="87" t="n"/>
-      <c r="H49" s="87" t="n"/>
-      <c r="I49" s="87" t="n"/>
-      <c r="J49" s="100" t="inlineStr">
+      <c r="F49" s="89" t="n"/>
+      <c r="G49" s="89" t="n"/>
+      <c r="H49" s="89" t="n"/>
+      <c r="I49" s="89" t="n"/>
+      <c r="J49" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K49" s="98">
+      <c r="K49" s="99">
         <f>IF(A49="","",IF(L44="PG",IF((F49="●")+(G49="●")+(H49="●")+(I49="●")+(L49="●")+(M49="●")+(N49="●")+(O49="●")&gt;0,B49*C49,0),ROUNDUP((F49="●")+(G49="●")+(H49="●")+(I49="●")+(L49="●")+(M49="●")+(N49="●")+(O49="●")/VALUE(MID(L44,2,2)),0)*B49*C49))</f>
         <v/>
       </c>
-      <c r="L49" s="98">
+      <c r="L49" s="99">
         <f>IF(A49="","",IF(L44="PG",IF((F49="●")+(G49="●")+(H49="●")+(I49="●")+(L49="●")+(M49="●")+(N49="●")+(O49="●")&gt;0,B49*D49,0),ROUNDUP((F49="●")+(G49="●")+(H49="●")+(I49="●")+(L49="●")+(M49="●")+(N49="●")+(O49="●")/VALUE(MID(L44,2,2)),0)*B49*D49))</f>
         <v/>
       </c>
-      <c r="M49" s="87" t="n"/>
-      <c r="N49" s="87" t="n"/>
-      <c r="O49" s="87" t="n"/>
+      <c r="M49" s="89" t="n"/>
+      <c r="N49" s="89" t="n"/>
+      <c r="O49" s="89" t="n"/>
       <c r="P49" s="5">
         <f>IF(A49="",0,COUNTIF(A$44:A48,A49))</f>
         <v/>
       </c>
-      <c r="Q49" s="87" t="n"/>
+      <c r="Q49" s="89" t="n"/>
     </row>
     <row r="50" ht="18" customHeight="1" s="44">
-      <c r="A50" s="101" t="n"/>
-      <c r="B50" s="100" t="n"/>
-      <c r="C50" s="98">
+      <c r="A50" s="102" t="n"/>
+      <c r="B50" s="101" t="n"/>
+      <c r="C50" s="99">
         <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$65:$C$73,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D50" s="98">
+      <c r="D50" s="99">
         <f>IF(A50="","",VLOOKUP(A50,'Master Data'!$A$65:$C$73,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E50" s="99">
+      <c r="E50" s="100">
         <f>IF(D50&gt;0,(D50-C50)/D50,0)</f>
         <v/>
       </c>
-      <c r="F50" s="87" t="n"/>
-      <c r="G50" s="87" t="n"/>
-      <c r="H50" s="87" t="n"/>
-      <c r="I50" s="87" t="n"/>
-      <c r="J50" s="100" t="inlineStr">
+      <c r="F50" s="89" t="n"/>
+      <c r="G50" s="89" t="n"/>
+      <c r="H50" s="89" t="n"/>
+      <c r="I50" s="89" t="n"/>
+      <c r="J50" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K50" s="98">
+      <c r="K50" s="99">
         <f>IF(A50="","",IF(L44="PG",IF((F50="●")+(G50="●")+(H50="●")+(I50="●")+(L50="●")+(M50="●")+(N50="●")+(O50="●")&gt;0,B50*C50,0),ROUNDUP((F50="●")+(G50="●")+(H50="●")+(I50="●")+(L50="●")+(M50="●")+(N50="●")+(O50="●")/VALUE(MID(L44,2,2)),0)*B50*C50))</f>
         <v/>
       </c>
-      <c r="L50" s="98">
+      <c r="L50" s="99">
         <f>IF(A50="","",IF(L44="PG",IF((F50="●")+(G50="●")+(H50="●")+(I50="●")+(L50="●")+(M50="●")+(N50="●")+(O50="●")&gt;0,B50*D50,0),ROUNDUP((F50="●")+(G50="●")+(H50="●")+(I50="●")+(L50="●")+(M50="●")+(N50="●")+(O50="●")/VALUE(MID(L44,2,2)),0)*B50*D50))</f>
         <v/>
       </c>
-      <c r="M50" s="87" t="n"/>
-      <c r="N50" s="87" t="n"/>
-      <c r="O50" s="87" t="n"/>
+      <c r="M50" s="89" t="n"/>
+      <c r="N50" s="89" t="n"/>
+      <c r="O50" s="89" t="n"/>
       <c r="P50" s="5">
         <f>IF(A50="",0,COUNTIF(A$44:A49,A50))</f>
         <v/>
       </c>
-      <c r="Q50" s="87" t="n"/>
+      <c r="Q50" s="89" t="n"/>
     </row>
     <row r="51" ht="18" customHeight="1" s="44">
-      <c r="A51" s="101" t="n"/>
-      <c r="B51" s="100" t="n"/>
-      <c r="C51" s="98">
+      <c r="A51" s="102" t="n"/>
+      <c r="B51" s="101" t="n"/>
+      <c r="C51" s="99">
         <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$65:$C$73,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D51" s="98">
+      <c r="D51" s="99">
         <f>IF(A51="","",VLOOKUP(A51,'Master Data'!$A$65:$C$73,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E51" s="99">
+      <c r="E51" s="100">
         <f>IF(D51&gt;0,(D51-C51)/D51,0)</f>
         <v/>
       </c>
-      <c r="F51" s="87" t="n"/>
-      <c r="G51" s="87" t="n"/>
-      <c r="H51" s="87" t="n"/>
-      <c r="I51" s="87" t="n"/>
-      <c r="J51" s="100" t="inlineStr">
+      <c r="F51" s="89" t="n"/>
+      <c r="G51" s="89" t="n"/>
+      <c r="H51" s="89" t="n"/>
+      <c r="I51" s="89" t="n"/>
+      <c r="J51" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K51" s="98">
+      <c r="K51" s="99">
         <f>IF(A51="","",IF(L44="PG",IF((F51="●")+(G51="●")+(H51="●")+(I51="●")+(L51="●")+(M51="●")+(N51="●")+(O51="●")&gt;0,B51*C51,0),ROUNDUP((F51="●")+(G51="●")+(H51="●")+(I51="●")+(L51="●")+(M51="●")+(N51="●")+(O51="●")/VALUE(MID(L44,2,2)),0)*B51*C51))</f>
         <v/>
       </c>
-      <c r="L51" s="98">
+      <c r="L51" s="99">
         <f>IF(A51="","",IF(L44="PG",IF((F51="●")+(G51="●")+(H51="●")+(I51="●")+(L51="●")+(M51="●")+(N51="●")+(O51="●")&gt;0,B51*D51,0),ROUNDUP((F51="●")+(G51="●")+(H51="●")+(I51="●")+(L51="●")+(M51="●")+(N51="●")+(O51="●")/VALUE(MID(L44,2,2)),0)*B51*D51))</f>
         <v/>
       </c>
-      <c r="M51" s="87" t="n"/>
-      <c r="N51" s="87" t="n"/>
-      <c r="O51" s="87" t="n"/>
+      <c r="M51" s="89" t="n"/>
+      <c r="N51" s="89" t="n"/>
+      <c r="O51" s="89" t="n"/>
       <c r="P51" s="5">
         <f>IF(A51="",0,COUNTIF(A$44:A50,A51))</f>
         <v/>
       </c>
-      <c r="Q51" s="87" t="n"/>
+      <c r="Q51" s="89" t="n"/>
     </row>
     <row r="52" ht="18" customHeight="1" s="44">
-      <c r="A52" s="101" t="n"/>
-      <c r="B52" s="100" t="n"/>
-      <c r="C52" s="98">
+      <c r="A52" s="102" t="n"/>
+      <c r="B52" s="101" t="n"/>
+      <c r="C52" s="99">
         <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$65:$C$73,2,FALSE))</f>
         <v/>
       </c>
-      <c r="D52" s="98">
+      <c r="D52" s="99">
         <f>IF(A52="","",VLOOKUP(A52,'Master Data'!$A$65:$C$73,3,FALSE))</f>
         <v/>
       </c>
-      <c r="E52" s="99">
+      <c r="E52" s="100">
         <f>IF(D52&gt;0,(D52-C52)/D52,0)</f>
         <v/>
       </c>
-      <c r="F52" s="87" t="n"/>
-      <c r="G52" s="87" t="n"/>
-      <c r="H52" s="87" t="n"/>
-      <c r="I52" s="87" t="n"/>
-      <c r="J52" s="100" t="inlineStr">
+      <c r="F52" s="89" t="n"/>
+      <c r="G52" s="89" t="n"/>
+      <c r="H52" s="89" t="n"/>
+      <c r="I52" s="89" t="n"/>
+      <c r="J52" s="101" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="K52" s="98">
+      <c r="K52" s="99">
         <f>IF(A52="","",IF(L44="PG",IF((F52="●")+(G52="●")+(H52="●")+(I52="●")+(L52="●")+(M52="●")+(N52="●")+(O52="●")&gt;0,B52*C52,0),ROUNDUP((F52="●")+(G52="●")+(H52="●")+(I52="●")+(L52="●")+(M52="●")+(N52="●")+(O52="●")/VALUE(MID(L44,2,2)),0)*B52*C52))</f>
         <v/>
       </c>
-      <c r="L52" s="98">
+      <c r="L52" s="99">
         <f>IF(A52="","",IF(L44="PG",IF((F52="●")+(G52="●")+(H52="●")+(I52="●")+(L52="●")+(M52="●")+(N52="●")+(O52="●")&gt;0,B52*D52,0),ROUNDUP((F52="●")+(G52="●")+(H52="●")+(I52="●")+(L52="●")+(M52="●")+(N52="●")+(O52="●")/VALUE(MID(L44,2,2)),0)*B52*D52))</f>
         <v/>
       </c>
-      <c r="M52" s="87" t="n"/>
-      <c r="N52" s="87" t="n"/>
-      <c r="O52" s="87" t="n"/>
+      <c r="M52" s="89" t="n"/>
+      <c r="N52" s="89" t="n"/>
+      <c r="O52" s="89" t="n"/>
       <c r="P52" s="5">
         <f>IF(A52="",0,COUNTIF(A$44:A51,A52))</f>
         <v/>
       </c>
-      <c r="Q52" s="87" t="n"/>
+      <c r="Q52" s="89" t="n"/>
     </row>
     <row r="53" ht="18" customHeight="1" s="44">
-      <c r="A53" s="102" t="inlineStr">
+      <c r="A53" s="103" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B53" s="104" t="n"/>
-      <c r="C53" s="104" t="n"/>
-      <c r="D53" s="104" t="n"/>
-      <c r="E53" s="105" t="n"/>
-      <c r="F53" s="103">
+      <c r="B53" s="105" t="n"/>
+      <c r="C53" s="105" t="n"/>
+      <c r="D53" s="105" t="n"/>
+      <c r="E53" s="106" t="n"/>
+      <c r="F53" s="104">
         <f>SUMPRODUCT((F44:F52="●")*1,B44:B52,C44:C52)</f>
         <v/>
       </c>
-      <c r="G53" s="103">
+      <c r="G53" s="104">
         <f>SUMPRODUCT((G44:G52="●")*1,B44:B52,C44:C52)</f>
         <v/>
       </c>
-      <c r="H53" s="103">
+      <c r="H53" s="104">
         <f>SUMPRODUCT((H44:H52="●")*1,B44:B52,C44:C52)</f>
         <v/>
       </c>
-      <c r="I53" s="103">
+      <c r="I53" s="104">
         <f>SUMPRODUCT((I44:I52="●")*1,B44:B52,C44:C52)</f>
         <v/>
       </c>
-      <c r="J53" s="104" t="n"/>
-      <c r="K53" s="103">
+      <c r="J53" s="105" t="n"/>
+      <c r="K53" s="104">
         <f>SUM(K44:K52)</f>
         <v/>
       </c>
-      <c r="L53" s="103">
+      <c r="L53" s="104">
         <f>SUM(L44:L52)</f>
         <v/>
       </c>
-      <c r="M53" s="103">
+      <c r="M53" s="104">
         <f>SUMPRODUCT((M44:M52="●")*1,B44:B52,C44:C52)</f>
         <v/>
       </c>
-      <c r="N53" s="103">
+      <c r="N53" s="104">
         <f>SUMPRODUCT((N44:N52="●")*1,B44:B52,C44:C52)</f>
         <v/>
       </c>
-      <c r="O53" s="103">
+      <c r="O53" s="104">
         <f>SUMPRODUCT((O44:O52="●")*1,B44:B52,C44:C52)</f>
         <v/>
       </c>
-      <c r="P53" s="91">
+      <c r="P53" s="93">
         <f>SUM(P44:P52)</f>
         <v/>
       </c>
-      <c r="Q53" s="91" t="n"/>
+      <c r="Q53" s="93" t="n"/>
     </row>
     <row r="54" ht="6" customHeight="1" s="44">
-      <c r="A54" s="89" t="n"/>
-      <c r="B54" s="89" t="n"/>
-      <c r="C54" s="89" t="n"/>
-      <c r="D54" s="89" t="n"/>
-      <c r="E54" s="89" t="n"/>
-      <c r="F54" s="106" t="n"/>
-      <c r="G54" s="106" t="n"/>
-      <c r="H54" s="106" t="n"/>
-      <c r="I54" s="106" t="n"/>
-      <c r="J54" s="106" t="n"/>
-      <c r="K54" s="106" t="n"/>
-      <c r="L54" s="106" t="n"/>
-      <c r="M54" s="106" t="n"/>
-      <c r="N54" s="106" t="n"/>
-      <c r="O54" s="106" t="n"/>
-      <c r="P54" s="89" t="n"/>
-      <c r="Q54" s="89" t="n"/>
+      <c r="A54" s="91" t="n"/>
+      <c r="B54" s="91" t="n"/>
+      <c r="C54" s="91" t="n"/>
+      <c r="D54" s="91" t="n"/>
+      <c r="E54" s="91" t="n"/>
+      <c r="F54" s="107" t="n"/>
+      <c r="G54" s="107" t="n"/>
+      <c r="H54" s="107" t="n"/>
+      <c r="I54" s="107" t="n"/>
+      <c r="J54" s="107" t="n"/>
+      <c r="K54" s="107" t="n"/>
+      <c r="L54" s="107" t="n"/>
+      <c r="M54" s="107" t="n"/>
+      <c r="N54" s="107" t="n"/>
+      <c r="O54" s="107" t="n"/>
+      <c r="P54" s="91" t="n"/>
+      <c r="Q54" s="91" t="n"/>
     </row>
     <row r="56"/>
     <row r="57">
-      <c r="A57" s="95" t="inlineStr">
+      <c r="A57" s="97" t="inlineStr">
         <is>
           <t>🏆 GRAND TOTAL</t>
         </is>
@@ -5188,207 +5210,207 @@
       <c r="L57" s="46" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="107" t="inlineStr">
+      <c r="A58" s="108" t="inlineStr">
         <is>
           <t>GOLF</t>
         </is>
       </c>
-      <c r="B58" s="108" t="n"/>
-      <c r="C58" s="108" t="n"/>
-      <c r="D58" s="108" t="n"/>
-      <c r="E58" s="108" t="n"/>
-      <c r="F58" s="108" t="n"/>
-      <c r="G58" s="108" t="n"/>
-      <c r="H58" s="108" t="n"/>
-      <c r="I58" s="108" t="n"/>
-      <c r="J58" s="109">
+      <c r="B58" s="109" t="n"/>
+      <c r="C58" s="109" t="n"/>
+      <c r="D58" s="109" t="n"/>
+      <c r="E58" s="109" t="n"/>
+      <c r="F58" s="109" t="n"/>
+      <c r="G58" s="109" t="n"/>
+      <c r="H58" s="109" t="n"/>
+      <c r="I58" s="109" t="n"/>
+      <c r="J58" s="110">
         <f>K16</f>
         <v/>
       </c>
-      <c r="K58" s="109">
+      <c r="K58" s="110">
         <f>L16</f>
         <v/>
       </c>
-      <c r="L58" s="87" t="inlineStr">
+      <c r="L58" s="89" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="107" t="inlineStr">
+      <c r="A59" s="108" t="inlineStr">
         <is>
           <t>HOTEL</t>
         </is>
       </c>
-      <c r="B59" s="108" t="n"/>
-      <c r="C59" s="108" t="n"/>
-      <c r="D59" s="108" t="n"/>
-      <c r="E59" s="108" t="n"/>
-      <c r="F59" s="108" t="n"/>
-      <c r="G59" s="108" t="n"/>
-      <c r="H59" s="108" t="n"/>
-      <c r="I59" s="108" t="n"/>
-      <c r="J59" s="109">
+      <c r="B59" s="109" t="n"/>
+      <c r="C59" s="109" t="n"/>
+      <c r="D59" s="109" t="n"/>
+      <c r="E59" s="109" t="n"/>
+      <c r="F59" s="109" t="n"/>
+      <c r="G59" s="109" t="n"/>
+      <c r="H59" s="109" t="n"/>
+      <c r="I59" s="109" t="n"/>
+      <c r="J59" s="110">
         <f>K21</f>
         <v/>
       </c>
-      <c r="K59" s="109">
+      <c r="K59" s="110">
         <f>L21</f>
         <v/>
       </c>
-      <c r="L59" s="87" t="inlineStr">
+      <c r="L59" s="89" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="107" t="inlineStr">
+      <c r="A60" s="108" t="inlineStr">
         <is>
           <t>TRANSPORT</t>
         </is>
       </c>
-      <c r="B60" s="108" t="n"/>
-      <c r="C60" s="108" t="n"/>
-      <c r="D60" s="108" t="n"/>
-      <c r="E60" s="108" t="n"/>
-      <c r="F60" s="108" t="n"/>
-      <c r="G60" s="108" t="n"/>
-      <c r="H60" s="108" t="n"/>
-      <c r="I60" s="108" t="n"/>
-      <c r="J60" s="109">
+      <c r="B60" s="109" t="n"/>
+      <c r="C60" s="109" t="n"/>
+      <c r="D60" s="109" t="n"/>
+      <c r="E60" s="109" t="n"/>
+      <c r="F60" s="109" t="n"/>
+      <c r="G60" s="109" t="n"/>
+      <c r="H60" s="109" t="n"/>
+      <c r="I60" s="109" t="n"/>
+      <c r="J60" s="110">
         <f>K27</f>
         <v/>
       </c>
-      <c r="K60" s="109">
+      <c r="K60" s="110">
         <f>L27</f>
         <v/>
       </c>
-      <c r="L60" s="87" t="inlineStr">
+      <c r="L60" s="89" t="inlineStr">
         <is>
           <t>PG</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="107" t="inlineStr">
+      <c r="A61" s="108" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
       </c>
-      <c r="B61" s="108" t="n"/>
-      <c r="C61" s="108" t="n"/>
-      <c r="D61" s="108" t="n"/>
-      <c r="E61" s="108" t="n"/>
-      <c r="F61" s="108" t="n"/>
-      <c r="G61" s="108" t="n"/>
-      <c r="H61" s="108" t="n"/>
-      <c r="I61" s="108" t="n"/>
-      <c r="J61" s="109">
+      <c r="B61" s="109" t="n"/>
+      <c r="C61" s="109" t="n"/>
+      <c r="D61" s="109" t="n"/>
+      <c r="E61" s="109" t="n"/>
+      <c r="F61" s="109" t="n"/>
+      <c r="G61" s="109" t="n"/>
+      <c r="H61" s="109" t="n"/>
+      <c r="I61" s="109" t="n"/>
+      <c r="J61" s="110">
         <f>K35</f>
         <v/>
       </c>
-      <c r="K61" s="109">
+      <c r="K61" s="110">
         <f>L35</f>
         <v/>
       </c>
-      <c r="L61" s="87" t="inlineStr">
+      <c r="L61" s="89" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="107" t="inlineStr">
+      <c r="A62" s="108" t="inlineStr">
         <is>
           <t>OTHER</t>
         </is>
       </c>
-      <c r="B62" s="108" t="n"/>
-      <c r="C62" s="108" t="n"/>
-      <c r="D62" s="108" t="n"/>
-      <c r="E62" s="108" t="n"/>
-      <c r="F62" s="108" t="n"/>
-      <c r="G62" s="108" t="n"/>
-      <c r="H62" s="108" t="n"/>
-      <c r="I62" s="108" t="n"/>
-      <c r="J62" s="109">
+      <c r="B62" s="109" t="n"/>
+      <c r="C62" s="109" t="n"/>
+      <c r="D62" s="109" t="n"/>
+      <c r="E62" s="109" t="n"/>
+      <c r="F62" s="109" t="n"/>
+      <c r="G62" s="109" t="n"/>
+      <c r="H62" s="109" t="n"/>
+      <c r="I62" s="109" t="n"/>
+      <c r="J62" s="110">
         <f>K41</f>
         <v/>
       </c>
-      <c r="K62" s="109">
+      <c r="K62" s="110">
         <f>L41</f>
         <v/>
       </c>
-      <c r="L62" s="87" t="inlineStr">
+      <c r="L62" s="89" t="inlineStr">
         <is>
           <t>PG</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="107" t="inlineStr">
+      <c r="A63" s="108" t="inlineStr">
         <is>
           <t>ACTIVITIES</t>
         </is>
       </c>
-      <c r="B63" s="108" t="n"/>
-      <c r="C63" s="108" t="n"/>
-      <c r="D63" s="108" t="n"/>
-      <c r="E63" s="108" t="n"/>
-      <c r="F63" s="108" t="n"/>
-      <c r="G63" s="108" t="n"/>
-      <c r="H63" s="108" t="n"/>
-      <c r="I63" s="108" t="n"/>
-      <c r="J63" s="109">
+      <c r="B63" s="109" t="n"/>
+      <c r="C63" s="109" t="n"/>
+      <c r="D63" s="109" t="n"/>
+      <c r="E63" s="109" t="n"/>
+      <c r="F63" s="109" t="n"/>
+      <c r="G63" s="109" t="n"/>
+      <c r="H63" s="109" t="n"/>
+      <c r="I63" s="109" t="n"/>
+      <c r="J63" s="110">
         <f>K53</f>
         <v/>
       </c>
-      <c r="K63" s="109">
+      <c r="K63" s="110">
         <f>L53</f>
         <v/>
       </c>
-      <c r="L63" s="87" t="inlineStr">
+      <c r="L63" s="89" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="102" t="inlineStr">
+      <c r="A64" s="103" t="inlineStr">
         <is>
           <t>📌 GRAND TOTAL</t>
         </is>
       </c>
-      <c r="B64" s="91" t="n"/>
-      <c r="C64" s="110" t="inlineStr">
+      <c r="B64" s="93" t="n"/>
+      <c r="C64" s="111" t="inlineStr">
         <is>
           <t>Margin:</t>
         </is>
       </c>
-      <c r="D64" s="105">
+      <c r="D64" s="106">
         <f>IF(K64&gt;0,(K64-J64)/K64,0)</f>
         <v/>
       </c>
-      <c r="E64" s="91" t="n"/>
-      <c r="F64" s="91" t="n"/>
-      <c r="G64" s="91" t="n"/>
-      <c r="H64" s="91" t="n"/>
-      <c r="I64" s="91" t="n"/>
-      <c r="J64" s="103">
+      <c r="E64" s="93" t="n"/>
+      <c r="F64" s="93" t="n"/>
+      <c r="G64" s="93" t="n"/>
+      <c r="H64" s="93" t="n"/>
+      <c r="I64" s="93" t="n"/>
+      <c r="J64" s="104">
         <f>SUM(J58:J63)</f>
         <v/>
       </c>
-      <c r="K64" s="103">
+      <c r="K64" s="104">
         <f>SUM(K58:K63)</f>
         <v/>
       </c>
-      <c r="L64" s="91" t="n"/>
+      <c r="L64" s="93" t="n"/>
     </row>
     <row r="65"/>
     <row r="66">
-      <c r="A66" s="95" t="inlineStr">
+      <c r="A66" s="97" t="inlineStr">
         <is>
           <t>👤 PER PERSON</t>
         </is>
@@ -5406,32 +5428,32 @@
       <c r="L66" s="46" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="85" t="inlineStr">
+      <c r="A67" s="88" t="inlineStr">
         <is>
           <t>Person</t>
         </is>
       </c>
-      <c r="B67" s="85" t="inlineStr">
+      <c r="B67" s="88" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="C67" s="85" t="inlineStr">
+      <c r="C67" s="88" t="inlineStr">
         <is>
           <t>Sell</t>
         </is>
       </c>
-      <c r="D67" s="85" t="inlineStr">
+      <c r="D67" s="88" t="inlineStr">
         <is>
           <t>Margin</t>
         </is>
       </c>
-      <c r="E67" s="85" t="inlineStr">
+      <c r="E67" s="88" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F67" s="85" t="inlineStr">
+      <c r="F67" s="88" t="inlineStr">
         <is>
           <t>#</t>
         </is>
@@ -5442,23 +5464,23 @@
         <f>F2</f>
         <v/>
       </c>
-      <c r="B68" s="98">
+      <c r="B68" s="99">
         <f>SUMPRODUCT((F11:F15="●")*1,B11:B15,C11:C15)+SUMPRODUCT((F18:F20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((F24:F26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((F30:F34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((F38:F40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((F44:F52="●")*1,B44:B52,C44:C52)</f>
         <v/>
       </c>
-      <c r="C68" s="98">
+      <c r="C68" s="99">
         <f>SUMPRODUCT((F11:F15="●")*1,B11:B15,D11:D15)+SUMPRODUCT((F18:F20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((F24:F26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((F30:F34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((F38:F40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((F44:F52="●")*1,B44:B52,D44:D52)</f>
         <v/>
       </c>
-      <c r="D68" s="98">
+      <c r="D68" s="99">
         <f>C68-B68</f>
         <v/>
       </c>
-      <c r="E68" s="99">
+      <c r="E68" s="100">
         <f>IF(C68&gt;0,D68/C68,0)</f>
         <v/>
       </c>
-      <c r="F68" s="87">
+      <c r="F68" s="89">
         <f>COUNTIF(F11:F15,"●")+COUNTIF(F18:F20,"●")+COUNTIF(F24:F26,"●")+COUNTIF(F30:F34,"●")+COUNTIF(F38:F40,"●")+COUNTIF(F44:F52,"●")</f>
         <v/>
       </c>
@@ -5468,23 +5490,23 @@
         <f>G2</f>
         <v/>
       </c>
-      <c r="B69" s="98">
+      <c r="B69" s="99">
         <f>SUMPRODUCT((G11:G15="●")*1,B11:B15,C11:C15)+SUMPRODUCT((G18:G20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((G24:G26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((G30:G34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((G38:G40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((G44:G52="●")*1,B44:B52,C44:C52)</f>
         <v/>
       </c>
-      <c r="C69" s="98">
+      <c r="C69" s="99">
         <f>SUMPRODUCT((G11:G15="●")*1,B11:B15,D11:D15)+SUMPRODUCT((G18:G20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((G24:G26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((G30:G34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((G38:G40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((G44:G52="●")*1,B44:B52,D44:D52)</f>
         <v/>
       </c>
-      <c r="D69" s="98">
+      <c r="D69" s="99">
         <f>C69-B69</f>
         <v/>
       </c>
-      <c r="E69" s="99">
+      <c r="E69" s="100">
         <f>IF(C69&gt;0,D69/C69,0)</f>
         <v/>
       </c>
-      <c r="F69" s="87">
+      <c r="F69" s="89">
         <f>COUNTIF(G11:G15,"●")+COUNTIF(G18:G20,"●")+COUNTIF(G24:G26,"●")+COUNTIF(G30:G34,"●")+COUNTIF(G38:G40,"●")+COUNTIF(G44:G52,"●")</f>
         <v/>
       </c>
@@ -5494,23 +5516,23 @@
         <f>H2</f>
         <v/>
       </c>
-      <c r="B70" s="98">
+      <c r="B70" s="99">
         <f>SUMPRODUCT((H11:H15="●")*1,B11:B15,C11:C15)+SUMPRODUCT((H18:H20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((H24:H26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((H30:H34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((H38:H40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((H44:H52="●")*1,B44:B52,C44:C52)</f>
         <v/>
       </c>
-      <c r="C70" s="98">
+      <c r="C70" s="99">
         <f>SUMPRODUCT((H11:H15="●")*1,B11:B15,D11:D15)+SUMPRODUCT((H18:H20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((H24:H26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((H30:H34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((H38:H40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((H44:H52="●")*1,B44:B52,D44:D52)</f>
         <v/>
       </c>
-      <c r="D70" s="98">
+      <c r="D70" s="99">
         <f>C70-B70</f>
         <v/>
       </c>
-      <c r="E70" s="99">
+      <c r="E70" s="100">
         <f>IF(C70&gt;0,D70/C70,0)</f>
         <v/>
       </c>
-      <c r="F70" s="87">
+      <c r="F70" s="89">
         <f>COUNTIF(H11:H15,"●")+COUNTIF(H18:H20,"●")+COUNTIF(H24:H26,"●")+COUNTIF(H30:H34,"●")+COUNTIF(H38:H40,"●")+COUNTIF(H44:H52,"●")</f>
         <v/>
       </c>
@@ -5520,64 +5542,64 @@
         <f>I2</f>
         <v/>
       </c>
-      <c r="B71" s="98">
+      <c r="B71" s="99">
         <f>SUMPRODUCT((I11:I15="●")*1,B11:B15,C11:C15)+SUMPRODUCT((I18:I20="●")*1,B18:B20,C18:C20)+SUMPRODUCT((I24:I26="●")*1,B24:B26,C24:C26)+SUMPRODUCT((I30:I34="●")*1,B30:B34,C30:C34)+SUMPRODUCT((I38:I40="●")*1,B38:B40,C38:C40)+SUMPRODUCT((I44:I52="●")*1,B44:B52,C44:C52)</f>
         <v/>
       </c>
-      <c r="C71" s="98">
+      <c r="C71" s="99">
         <f>SUMPRODUCT((I11:I15="●")*1,B11:B15,D11:D15)+SUMPRODUCT((I18:I20="●")*1,B18:B20,D18:D20)+SUMPRODUCT((I24:I26="●")*1,B24:B26,D24:D26)+SUMPRODUCT((I30:I34="●")*1,B30:B34,D30:D34)+SUMPRODUCT((I38:I40="●")*1,B38:B40,D38:D40)+SUMPRODUCT((I44:I52="●")*1,B44:B52,D44:D52)</f>
         <v/>
       </c>
-      <c r="D71" s="98">
+      <c r="D71" s="99">
         <f>C71-B71</f>
         <v/>
       </c>
-      <c r="E71" s="99">
+      <c r="E71" s="100">
         <f>IF(C71&gt;0,D71/C71,0)</f>
         <v/>
       </c>
-      <c r="F71" s="87">
+      <c r="F71" s="89">
         <f>COUNTIF(I11:I15,"●")+COUNTIF(I18:I20,"●")+COUNTIF(I24:I26,"●")+COUNTIF(I30:I34,"●")+COUNTIF(I38:I40,"●")+COUNTIF(I44:I52,"●")</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="102" t="inlineStr">
+      <c r="A72" s="103" t="inlineStr">
         <is>
           <t>📌 TOTAL</t>
         </is>
       </c>
-      <c r="B72" s="103" t="n"/>
-      <c r="C72" s="103" t="n"/>
-      <c r="D72" s="103" t="n"/>
-      <c r="E72" s="91" t="n"/>
-      <c r="F72" s="91" t="n"/>
+      <c r="B72" s="104" t="n"/>
+      <c r="C72" s="104" t="n"/>
+      <c r="D72" s="104" t="n"/>
+      <c r="E72" s="93" t="n"/>
+      <c r="F72" s="93" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="89" t="n"/>
-      <c r="B73" s="89" t="n"/>
-      <c r="C73" s="89" t="n"/>
-      <c r="D73" s="89" t="n"/>
-      <c r="E73" s="89" t="n"/>
-      <c r="F73" s="89" t="n"/>
-      <c r="G73" s="89" t="n"/>
-      <c r="H73" s="89" t="n"/>
-      <c r="I73" s="89" t="n"/>
-      <c r="J73" s="89" t="n"/>
-      <c r="K73" s="89" t="n"/>
-      <c r="L73" s="89" t="n"/>
-      <c r="M73" s="89" t="n"/>
-      <c r="N73" s="89" t="n"/>
-      <c r="O73" s="89" t="n"/>
-      <c r="P73" s="89" t="n"/>
-      <c r="Q73" s="89" t="n"/>
+      <c r="A73" s="91" t="n"/>
+      <c r="B73" s="91" t="n"/>
+      <c r="C73" s="91" t="n"/>
+      <c r="D73" s="91" t="n"/>
+      <c r="E73" s="91" t="n"/>
+      <c r="F73" s="91" t="n"/>
+      <c r="G73" s="91" t="n"/>
+      <c r="H73" s="91" t="n"/>
+      <c r="I73" s="91" t="n"/>
+      <c r="J73" s="91" t="n"/>
+      <c r="K73" s="91" t="n"/>
+      <c r="L73" s="91" t="n"/>
+      <c r="M73" s="91" t="n"/>
+      <c r="N73" s="91" t="n"/>
+      <c r="O73" s="91" t="n"/>
+      <c r="P73" s="91" t="n"/>
+      <c r="Q73" s="91" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="A57:L57"/>
-    <mergeCell ref="A2:L2"/>
     <mergeCell ref="A18:K18"/>
     <mergeCell ref="A7:L7"/>
+    <mergeCell ref="B2:C2"/>
     <mergeCell ref="A30:K30"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A24:K24"/>
@@ -5941,22 +5963,22 @@
       <formula1>"PG,P1,P2,P3,P4,P5,P6,P7,P8,P9,P10,P11,P12,P13,P14,P15,P16,P17,P18,P19,P20"</formula1>
     </dataValidation>
     <dataValidation sqref="A12 A13 A14 A15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Master Data'!$A$8:$C$15</formula1>
+      <formula1>'Master Data'!$A$8:$A$15</formula1>
     </dataValidation>
     <dataValidation sqref="A19 A20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Master Data'!$A$21:$C$26</formula1>
+      <formula1>'Master Data'!$A$21:$A$26</formula1>
     </dataValidation>
     <dataValidation sqref="A25 A26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Master Data'!$A$31:$C$37</formula1>
+      <formula1>'Master Data'!$A$31:$A$37</formula1>
     </dataValidation>
     <dataValidation sqref="A31 A32 A33 A34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Master Data'!$A$42:$C$50</formula1>
+      <formula1>'Master Data'!$A$42:$A$50</formula1>
     </dataValidation>
     <dataValidation sqref="A39 A40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Master Data'!$A$55:$C$61</formula1>
+      <formula1>'Master Data'!$A$55:$A$61</formula1>
     </dataValidation>
     <dataValidation sqref="A45 A46 A47 A48 A49 A50 A51 A52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'Master Data'!$A$65:$C$73</formula1>
+      <formula1>'Master Data'!$A$65:$A$73</formula1>
     </dataValidation>
     <dataValidation sqref="F12 F13 F14 F15 F19 F20 F25 F26 F31 F32 F33 F34 F39 F40 F45 F46 F47 F48 F49 F50 F51 F52 G12 G13 G14 G15 G19 G20 G25 G26 G31 G32 G33 G34 G39 G40 G45 G46 G47 G48 G49 G50 G51 G52 H12 H13 H14 H15 H19 H20 H25 H26 H31 H32 H33 H34 H39 H40 H45 H46 H47 H48 H49 H50 H51 H52 I12 I13 I14 I15 I19 I20 I25 I26 I31 I32 I33 I34 I39 I40 I45 I46 I47 I48 I49 I50 I51 I52 L12 L13 L14 L15 L19 L20 L25 L26 L31 L32 L33 L34 L39 L40 L45 L46 L47 L48 L49 L50 L51 L52 M12 M13 M14 M15 M19 M20 M25 M26 M31 M32 M33 M34 M39 M40 M45 M46 M47 M48 M49 M50 M51 M52 N12 N13 N14 N15 N19 N20 N25 N26 N31 N32 N33 N34 N39 N40 N45 N46 N47 N48 N49 N50 N51 N52 O12 O13 O14 O15 O19 O20 O25 O26 O31 O32 O33 O34 O39 O40 O45 O46 O47 O48 O49 O50 O51 O52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Toggle" error="● = ON, blank = OFF" type="list">
       <formula1>"●"</formula1>
@@ -5994,139 +6016,139 @@
       <c r="F1" s="46" t="n"/>
     </row>
     <row r="2">
-      <c r="E2" s="89">
+      <c r="E2" s="91">
         <f>'Package Selector'!E2</f>
         <v/>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="94" t="inlineStr">
+      <c r="A4" s="96" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B4" s="94" t="inlineStr">
+      <c r="B4" s="96" t="inlineStr">
         <is>
           <t>Total Cost</t>
         </is>
       </c>
-      <c r="C4" s="94" t="inlineStr">
+      <c r="C4" s="96" t="inlineStr">
         <is>
           <t>Total Sell</t>
         </is>
       </c>
-      <c r="D4" s="94" t="inlineStr">
+      <c r="D4" s="96" t="inlineStr">
         <is>
           <t>Margin</t>
         </is>
       </c>
-      <c r="E4" s="94" t="inlineStr">
+      <c r="E4" s="96" t="inlineStr">
         <is>
           <t>Margin%</t>
         </is>
       </c>
-      <c r="F4" s="94" t="inlineStr">
+      <c r="F4" s="96" t="inlineStr">
         <is>
           <t>Per Person</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="101" t="inlineStr">
+      <c r="A5" s="102" t="inlineStr">
         <is>
           <t>GOLF</t>
         </is>
       </c>
-      <c r="B5" s="109" t="n"/>
-      <c r="C5" s="109" t="n"/>
-      <c r="D5" s="100" t="n"/>
-      <c r="E5" s="111" t="n"/>
-      <c r="F5" s="100" t="n"/>
+      <c r="B5" s="110" t="n"/>
+      <c r="C5" s="110" t="n"/>
+      <c r="D5" s="101" t="n"/>
+      <c r="E5" s="112" t="n"/>
+      <c r="F5" s="101" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="101" t="inlineStr">
+      <c r="A6" s="102" t="inlineStr">
         <is>
           <t>HOTEL</t>
         </is>
       </c>
-      <c r="B6" s="109" t="n"/>
-      <c r="C6" s="109" t="n"/>
-      <c r="D6" s="100" t="n"/>
-      <c r="E6" s="111" t="n"/>
-      <c r="F6" s="100" t="n"/>
+      <c r="B6" s="110" t="n"/>
+      <c r="C6" s="110" t="n"/>
+      <c r="D6" s="101" t="n"/>
+      <c r="E6" s="112" t="n"/>
+      <c r="F6" s="101" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="101" t="inlineStr">
+      <c r="A7" s="102" t="inlineStr">
         <is>
           <t>TRANSPORT</t>
         </is>
       </c>
-      <c r="B7" s="109" t="n"/>
-      <c r="C7" s="109" t="n"/>
-      <c r="D7" s="100" t="n"/>
-      <c r="E7" s="111" t="n"/>
-      <c r="F7" s="100" t="n"/>
+      <c r="B7" s="110" t="n"/>
+      <c r="C7" s="110" t="n"/>
+      <c r="D7" s="101" t="n"/>
+      <c r="E7" s="112" t="n"/>
+      <c r="F7" s="101" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="101" t="inlineStr">
+      <c r="A8" s="102" t="inlineStr">
         <is>
           <t>MEALS</t>
         </is>
       </c>
-      <c r="B8" s="109" t="n"/>
-      <c r="C8" s="109" t="n"/>
-      <c r="D8" s="100" t="n"/>
-      <c r="E8" s="111" t="n"/>
-      <c r="F8" s="100" t="n"/>
+      <c r="B8" s="110" t="n"/>
+      <c r="C8" s="110" t="n"/>
+      <c r="D8" s="101" t="n"/>
+      <c r="E8" s="112" t="n"/>
+      <c r="F8" s="101" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="101" t="inlineStr">
+      <c r="A9" s="102" t="inlineStr">
         <is>
           <t>OTHER</t>
         </is>
       </c>
-      <c r="B9" s="109" t="n"/>
-      <c r="C9" s="109" t="n"/>
-      <c r="D9" s="100" t="n"/>
-      <c r="E9" s="111" t="n"/>
-      <c r="F9" s="100" t="n"/>
+      <c r="B9" s="110" t="n"/>
+      <c r="C9" s="110" t="n"/>
+      <c r="D9" s="101" t="n"/>
+      <c r="E9" s="112" t="n"/>
+      <c r="F9" s="101" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="101" t="inlineStr">
+      <c r="A10" s="102" t="inlineStr">
         <is>
           <t>ACTIVITIES</t>
         </is>
       </c>
-      <c r="B10" s="109" t="n"/>
-      <c r="C10" s="109" t="n"/>
-      <c r="D10" s="100" t="n"/>
-      <c r="E10" s="111" t="n"/>
-      <c r="F10" s="100" t="n"/>
+      <c r="B10" s="110" t="n"/>
+      <c r="C10" s="110" t="n"/>
+      <c r="D10" s="101" t="n"/>
+      <c r="E10" s="112" t="n"/>
+      <c r="F10" s="101" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="102" t="inlineStr">
+      <c r="A11" s="103" t="inlineStr">
         <is>
           <t>📌 TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="104">
+      <c r="B11" s="105">
         <f>SUM(B5:B10)</f>
         <v/>
       </c>
-      <c r="C11" s="104">
+      <c r="C11" s="105">
         <f>SUM(C5:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="104">
+      <c r="D11" s="105">
         <f>SUM(D5:D10)</f>
         <v/>
       </c>
-      <c r="E11" s="105">
+      <c r="E11" s="106">
         <f>IF(C11&gt;0,D11/C11,0)</f>
         <v/>
       </c>
-      <c r="F11" s="104">
+      <c r="F11" s="105">
         <f>IF(E2&gt;0,B11/E2,0)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
v3: remove kj title, fix FlightAware ICAO codes (KE→KAL/OZ→AAR), hide column P
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -3259,14 +3259,14 @@
     <col hidden="1" width="6" customWidth="1" style="44" min="13" max="13"/>
     <col hidden="1" width="6" customWidth="1" style="44" min="14" max="14"/>
     <col hidden="1" width="6" customWidth="1" style="44" min="15" max="15"/>
-    <col width="6" customWidth="1" style="44" min="16" max="16"/>
+    <col hidden="1" width="6" customWidth="1" style="44" min="16" max="16"/>
     <col hidden="1" width="6" customWidth="1" style="44" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="82" t="inlineStr">
         <is>
-          <t>kj'</t>
+          <t>🏌️ LA GOLF PACKAGE SELECTOR</t>
         </is>
       </c>
       <c r="B1" s="42" t="n"/>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="B5" s="86" t="n"/>
       <c r="C5" s="89">
-        <f>IF(D5="","✈ Select flight ▼",HYPERLINK("https://flightaware.com/live/flight/"&amp;LEFT(D5,2)&amp;VALUE(MID(D5,3,10)),"✈ "&amp;D5&amp;" 🔗"))</f>
+        <f>IF(D5="","✈ Select flight ▼",HYPERLINK("https://flightaware.com/live/flight/"&amp;IF(LEFT(D5,2)="KE","KAL","AAR")&amp;VALUE(MID(D5,3,10)),"✈ "&amp;D5&amp;" 🔗"))</f>
         <v/>
       </c>
       <c r="D5" s="86" t="n"/>
@@ -3445,7 +3445,7 @@
       </c>
       <c r="B8" s="86" t="n"/>
       <c r="C8" s="89">
-        <f>IF(D8="","✈ Select flight ▼",HYPERLINK("https://flightaware.com/live/flight/"&amp;LEFT(D8,2)&amp;VALUE(MID(D8,3,10)),"✈ "&amp;D8&amp;" 🔗"))</f>
+        <f>IF(D8="","✈ Select flight ▼",HYPERLINK("https://flightaware.com/live/flight/"&amp;IF(LEFT(D8,2)="KE","KAL","AAR")&amp;VALUE(MID(D8,3,10)),"✈ "&amp;D8&amp;" 🔗"))</f>
         <v/>
       </c>
       <c r="D8" s="86" t="n"/>

</xml_diff>

<commit_message>
FlightAware links → /history page
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -3362,7 +3362,7 @@
       </c>
       <c r="B5" s="86" t="n"/>
       <c r="C5" s="89">
-        <f>IF(D5="","✈ Select flight ▼",HYPERLINK("https://flightaware.com/live/flight/"&amp;IF(LEFT(D5,2)="KE","KAL","AAR")&amp;VALUE(MID(D5,3,10)),"✈ "&amp;D5&amp;" 🔗"))</f>
+        <f>IF(D5="","✈ Select flight ▼",HYPERLINK("https://www.flightaware.com/live/flight/"&amp;IF(LEFT(D5,2)="KE","KAL","AAR")&amp;VALUE(MID(D5,3,10))&amp;"/history","✈ "&amp;D5&amp;" 🔗"))</f>
         <v/>
       </c>
       <c r="D5" s="86" t="n"/>
@@ -3445,7 +3445,7 @@
       </c>
       <c r="B8" s="86" t="n"/>
       <c r="C8" s="89">
-        <f>IF(D8="","✈ Select flight ▼",HYPERLINK("https://flightaware.com/live/flight/"&amp;IF(LEFT(D8,2)="KE","KAL","AAR")&amp;VALUE(MID(D8,3,10)),"✈ "&amp;D8&amp;" 🔗"))</f>
+        <f>IF(D8="","✈ Select flight ▼",HYPERLINK("https://www.flightaware.com/live/flight/"&amp;IF(LEFT(D8,2)="KE","KAL","AAR")&amp;VALUE(MID(D8,3,10))&amp;"/history","✈ "&amp;D8&amp;" 🔗"))</f>
         <v/>
       </c>
       <c r="D8" s="86" t="n"/>

</xml_diff>

<commit_message>
Fix K/L columns: move charge type to hidden col R, remove self-references
</commit_message>
<xml_diff>
--- a/files/LA_Golf_Package_Selector_v3.xlsx
+++ b/files/LA_Golf_Package_Selector_v3.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="\$#,##0"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -148,6 +148,11 @@
     <font>
       <name val="Calibri"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00888888"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="20">
@@ -528,7 +533,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -836,6 +841,8 @@
     <xf numFmtId="164" fontId="21" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1446,7 +1453,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="65" t="inlineStr">
         <is>
@@ -1845,7 +1851,6 @@
       </c>
       <c r="G26" s="68" t="n"/>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="65" t="inlineStr">
         <is>
@@ -2022,7 +2027,6 @@
       </c>
       <c r="G37" s="68" t="n"/>
     </row>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="65" t="inlineStr">
         <is>
@@ -2243,7 +2247,6 @@
       </c>
       <c r="G50" s="68" t="n"/>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="A52" s="65" t="inlineStr">
         <is>
@@ -2383,7 +2386,6 @@
       <c r="E60" s="76" t="n"/>
       <c r="G60" s="68" t="n"/>
     </row>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="70" t="inlineStr">
         <is>
@@ -2586,7 +2588,6 @@
         <v/>
       </c>
     </row>
-    <row r="74"/>
     <row r="75">
       <c r="A75" s="65" t="inlineStr">
         <is>
@@ -2886,9 +2887,6 @@
       <c r="F85" s="68" t="n"/>
       <c r="G85" s="68" t="n"/>
     </row>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
     <row r="89">
       <c r="A89" s="65" t="inlineStr">
         <is>
@@ -3241,7 +3239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q73"/>
+  <dimension ref="A1:R73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" customWidth="1" style="44" min="1" max="1"/>
@@ -3261,6 +3259,7 @@
     <col hidden="1" width="6" customWidth="1" style="44" min="15" max="15"/>
     <col hidden="1" width="6" customWidth="1" style="44" min="16" max="16"/>
     <col hidden="1" width="6" customWidth="1" style="44" min="17" max="17"/>
+    <col hidden="1" width="13" customWidth="1" style="44" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3269,17 +3268,17 @@
           <t>🏌️ LA GOLF PACKAGE SELECTOR</t>
         </is>
       </c>
-      <c r="B1" s="42" t="n"/>
-      <c r="C1" s="42" t="n"/>
-      <c r="D1" s="42" t="n"/>
-      <c r="E1" s="42" t="n"/>
-      <c r="F1" s="42" t="n"/>
-      <c r="G1" s="42" t="n"/>
-      <c r="H1" s="42" t="n"/>
-      <c r="I1" s="42" t="n"/>
-      <c r="J1" s="42" t="n"/>
-      <c r="K1" s="42" t="n"/>
-      <c r="L1" s="43" t="n"/>
+      <c r="B1" s="48" t="n"/>
+      <c r="C1" s="48" t="n"/>
+      <c r="D1" s="48" t="n"/>
+      <c r="E1" s="48" t="n"/>
+      <c r="F1" s="48" t="n"/>
+      <c r="G1" s="48" t="n"/>
+      <c r="H1" s="48" t="n"/>
+      <c r="I1" s="48" t="n"/>
+      <c r="J1" s="48" t="n"/>
+      <c r="K1" s="48" t="n"/>
+      <c r="L1" s="46" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="83" t="inlineStr">
@@ -3641,6 +3640,11 @@
           <t>Dup</t>
         </is>
       </c>
+      <c r="R10" s="113" t="inlineStr">
+        <is>
+          <t>Chg</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1" s="44">
       <c r="A11" s="97" t="inlineStr">
@@ -3658,16 +3662,17 @@
       <c r="I11" s="48" t="n"/>
       <c r="J11" s="48" t="n"/>
       <c r="K11" s="46" t="n"/>
-      <c r="L11" s="93" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
+      <c r="L11" s="93" t="n"/>
       <c r="M11" s="96" t="n"/>
       <c r="N11" s="96" t="n"/>
       <c r="O11" s="96" t="n"/>
       <c r="P11" s="96" t="n"/>
       <c r="Q11" s="96" t="n"/>
+      <c r="R11" s="114" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="44">
       <c r="A12" s="84" t="inlineStr">
@@ -3700,11 +3705,11 @@
         </is>
       </c>
       <c r="K12" s="99">
-        <f>IF(A12="","",IF(L11="PG",IF((F12="●")+(G12="●")+(H12="●")+(I12="●")+(L12="●")+(M12="●")+(N12="●")+(O12="●")&gt;0,B12*C12,0),ROUNDUP((F12="●")+(G12="●")+(H12="●")+(I12="●")+(L12="●")+(M12="●")+(N12="●")+(O12="●")/VALUE(MID(L11,2,2)),0)*B12*C12))</f>
+        <f>IF(A12="","",IF(R11="PG",IF((F12="●")+(G12="●")+(H12="●")+(I12="●")+(M12="●")+(N12="●")+(O12="●")&gt;0,B12*C12,0),ROUNDUP((F12="●")+(G12="●")+(H12="●")+(I12="●")+(M12="●")+(N12="●")+(O12="●")/VALUE(MID(R11,2,2)),0)*B12*C12))</f>
         <v/>
       </c>
       <c r="L12" s="99">
-        <f>IF(A12="","",IF(L11="PG",IF((F12="●")+(G12="●")+(H12="●")+(I12="●")+(L12="●")+(M12="●")+(N12="●")+(O12="●")&gt;0,B12*D12,0),ROUNDUP((F12="●")+(G12="●")+(H12="●")+(I12="●")+(L12="●")+(M12="●")+(N12="●")+(O12="●")/VALUE(MID(L11,2,2)),0)*B12*D12))</f>
+        <f>IF(A12="","",IF(R11="PG",IF((F12="●")+(G12="●")+(H12="●")+(I12="●")+(M12="●")+(N12="●")+(O12="●")&gt;0,B12*D12,0),ROUNDUP((F12="●")+(G12="●")+(H12="●")+(I12="●")+(M12="●")+(N12="●")+(O12="●")/VALUE(MID(R11,2,2)),0)*B12*D12))</f>
         <v/>
       </c>
       <c r="M12" s="89" t="n"/>
@@ -3747,11 +3752,11 @@
         </is>
       </c>
       <c r="K13" s="99">
-        <f>IF(A13="","",IF(L11="PG",IF((F13="●")+(G13="●")+(H13="●")+(I13="●")+(L13="●")+(M13="●")+(N13="●")+(O13="●")&gt;0,B13*C13,0),ROUNDUP((F13="●")+(G13="●")+(H13="●")+(I13="●")+(L13="●")+(M13="●")+(N13="●")+(O13="●")/VALUE(MID(L11,2,2)),0)*B13*C13))</f>
+        <f>IF(A13="","",IF(R11="PG",IF((F13="●")+(G13="●")+(H13="●")+(I13="●")+(M13="●")+(N13="●")+(O13="●")&gt;0,B13*C13,0),ROUNDUP((F13="●")+(G13="●")+(H13="●")+(I13="●")+(M13="●")+(N13="●")+(O13="●")/VALUE(MID(R11,2,2)),0)*B13*C13))</f>
         <v/>
       </c>
       <c r="L13" s="99">
-        <f>IF(A13="","",IF(L11="PG",IF((F13="●")+(G13="●")+(H13="●")+(I13="●")+(L13="●")+(M13="●")+(N13="●")+(O13="●")&gt;0,B13*D13,0),ROUNDUP((F13="●")+(G13="●")+(H13="●")+(I13="●")+(L13="●")+(M13="●")+(N13="●")+(O13="●")/VALUE(MID(L11,2,2)),0)*B13*D13))</f>
+        <f>IF(A13="","",IF(R11="PG",IF((F13="●")+(G13="●")+(H13="●")+(I13="●")+(M13="●")+(N13="●")+(O13="●")&gt;0,B13*D13,0),ROUNDUP((F13="●")+(G13="●")+(H13="●")+(I13="●")+(M13="●")+(N13="●")+(O13="●")/VALUE(MID(R11,2,2)),0)*B13*D13))</f>
         <v/>
       </c>
       <c r="M13" s="89" t="n"/>
@@ -3788,11 +3793,11 @@
         </is>
       </c>
       <c r="K14" s="99">
-        <f>IF(A14="","",IF(L11="PG",IF((F14="●")+(G14="●")+(H14="●")+(I14="●")+(L14="●")+(M14="●")+(N14="●")+(O14="●")&gt;0,B14*C14,0),ROUNDUP((F14="●")+(G14="●")+(H14="●")+(I14="●")+(L14="●")+(M14="●")+(N14="●")+(O14="●")/VALUE(MID(L11,2,2)),0)*B14*C14))</f>
+        <f>IF(A14="","",IF(R11="PG",IF((F14="●")+(G14="●")+(H14="●")+(I14="●")+(M14="●")+(N14="●")+(O14="●")&gt;0,B14*C14,0),ROUNDUP((F14="●")+(G14="●")+(H14="●")+(I14="●")+(M14="●")+(N14="●")+(O14="●")/VALUE(MID(R11,2,2)),0)*B14*C14))</f>
         <v/>
       </c>
       <c r="L14" s="99">
-        <f>IF(A14="","",IF(L11="PG",IF((F14="●")+(G14="●")+(H14="●")+(I14="●")+(L14="●")+(M14="●")+(N14="●")+(O14="●")&gt;0,B14*D14,0),ROUNDUP((F14="●")+(G14="●")+(H14="●")+(I14="●")+(L14="●")+(M14="●")+(N14="●")+(O14="●")/VALUE(MID(L11,2,2)),0)*B14*D14))</f>
+        <f>IF(A14="","",IF(R11="PG",IF((F14="●")+(G14="●")+(H14="●")+(I14="●")+(M14="●")+(N14="●")+(O14="●")&gt;0,B14*D14,0),ROUNDUP((F14="●")+(G14="●")+(H14="●")+(I14="●")+(M14="●")+(N14="●")+(O14="●")/VALUE(MID(R11,2,2)),0)*B14*D14))</f>
         <v/>
       </c>
       <c r="M14" s="89" t="n"/>
@@ -3829,11 +3834,11 @@
         </is>
       </c>
       <c r="K15" s="99">
-        <f>IF(A15="","",IF(L11="PG",IF((F15="●")+(G15="●")+(H15="●")+(I15="●")+(L15="●")+(M15="●")+(N15="●")+(O15="●")&gt;0,B15*C15,0),ROUNDUP((F15="●")+(G15="●")+(H15="●")+(I15="●")+(L15="●")+(M15="●")+(N15="●")+(O15="●")/VALUE(MID(L11,2,2)),0)*B15*C15))</f>
+        <f>IF(A15="","",IF(R11="PG",IF((F15="●")+(G15="●")+(H15="●")+(I15="●")+(M15="●")+(N15="●")+(O15="●")&gt;0,B15*C15,0),ROUNDUP((F15="●")+(G15="●")+(H15="●")+(I15="●")+(M15="●")+(N15="●")+(O15="●")/VALUE(MID(R11,2,2)),0)*B15*C15))</f>
         <v/>
       </c>
       <c r="L15" s="99">
-        <f>IF(A15="","",IF(L11="PG",IF((F15="●")+(G15="●")+(H15="●")+(I15="●")+(L15="●")+(M15="●")+(N15="●")+(O15="●")&gt;0,B15*D15,0),ROUNDUP((F15="●")+(G15="●")+(H15="●")+(I15="●")+(L15="●")+(M15="●")+(N15="●")+(O15="●")/VALUE(MID(L11,2,2)),0)*B15*D15))</f>
+        <f>IF(A15="","",IF(R11="PG",IF((F15="●")+(G15="●")+(H15="●")+(I15="●")+(M15="●")+(N15="●")+(O15="●")&gt;0,B15*D15,0),ROUNDUP((F15="●")+(G15="●")+(H15="●")+(I15="●")+(M15="●")+(N15="●")+(O15="●")/VALUE(MID(R11,2,2)),0)*B15*D15))</f>
         <v/>
       </c>
       <c r="M15" s="89" t="n"/>
@@ -3933,16 +3938,17 @@
       <c r="I18" s="48" t="n"/>
       <c r="J18" s="48" t="n"/>
       <c r="K18" s="46" t="n"/>
-      <c r="L18" s="93" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
+      <c r="L18" s="93" t="n"/>
       <c r="M18" s="96" t="n"/>
       <c r="N18" s="96" t="n"/>
       <c r="O18" s="96" t="n"/>
       <c r="P18" s="96" t="n"/>
       <c r="Q18" s="96" t="n"/>
+      <c r="R18" s="114" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1" s="44">
       <c r="A19" s="102" t="n"/>
@@ -3969,11 +3975,11 @@
         </is>
       </c>
       <c r="K19" s="99">
-        <f>IF(A19="","",IF(L18="PG",IF((F19="●")+(G19="●")+(H19="●")+(I19="●")+(L19="●")+(M19="●")+(N19="●")+(O19="●")&gt;0,B19*C19,0),ROUNDUP((F19="●")+(G19="●")+(H19="●")+(I19="●")+(L19="●")+(M19="●")+(N19="●")+(O19="●")/VALUE(MID(L18,2,2)),0)*B19*C19))</f>
+        <f>IF(A19="","",IF(R18="PG",IF((F19="●")+(G19="●")+(H19="●")+(I19="●")+(M19="●")+(N19="●")+(O19="●")&gt;0,B19*C19,0),ROUNDUP((F19="●")+(G19="●")+(H19="●")+(I19="●")+(M19="●")+(N19="●")+(O19="●")/VALUE(MID(R18,2,2)),0)*B19*C19))</f>
         <v/>
       </c>
       <c r="L19" s="99">
-        <f>IF(A19="","",IF(L18="PG",IF((F19="●")+(G19="●")+(H19="●")+(I19="●")+(L19="●")+(M19="●")+(N19="●")+(O19="●")&gt;0,B19*D19,0),ROUNDUP((F19="●")+(G19="●")+(H19="●")+(I19="●")+(L19="●")+(M19="●")+(N19="●")+(O19="●")/VALUE(MID(L18,2,2)),0)*B19*D19))</f>
+        <f>IF(A19="","",IF(R18="PG",IF((F19="●")+(G19="●")+(H19="●")+(I19="●")+(M19="●")+(N19="●")+(O19="●")&gt;0,B19*D19,0),ROUNDUP((F19="●")+(G19="●")+(H19="●")+(I19="●")+(M19="●")+(N19="●")+(O19="●")/VALUE(MID(R18,2,2)),0)*B19*D19))</f>
         <v/>
       </c>
       <c r="M19" s="89" t="n"/>
@@ -4010,11 +4016,11 @@
         </is>
       </c>
       <c r="K20" s="99">
-        <f>IF(A20="","",IF(L18="PG",IF((F20="●")+(G20="●")+(H20="●")+(I20="●")+(L20="●")+(M20="●")+(N20="●")+(O20="●")&gt;0,B20*C20,0),ROUNDUP((F20="●")+(G20="●")+(H20="●")+(I20="●")+(L20="●")+(M20="●")+(N20="●")+(O20="●")/VALUE(MID(L18,2,2)),0)*B20*C20))</f>
+        <f>IF(A20="","",IF(R18="PG",IF((F20="●")+(G20="●")+(H20="●")+(I20="●")+(M20="●")+(N20="●")+(O20="●")&gt;0,B20*C20,0),ROUNDUP((F20="●")+(G20="●")+(H20="●")+(I20="●")+(M20="●")+(N20="●")+(O20="●")/VALUE(MID(R18,2,2)),0)*B20*C20))</f>
         <v/>
       </c>
       <c r="L20" s="99">
-        <f>IF(A20="","",IF(L18="PG",IF((F20="●")+(G20="●")+(H20="●")+(I20="●")+(L20="●")+(M20="●")+(N20="●")+(O20="●")&gt;0,B20*D20,0),ROUNDUP((F20="●")+(G20="●")+(H20="●")+(I20="●")+(L20="●")+(M20="●")+(N20="●")+(O20="●")/VALUE(MID(L18,2,2)),0)*B20*D20))</f>
+        <f>IF(A20="","",IF(R18="PG",IF((F20="●")+(G20="●")+(H20="●")+(I20="●")+(M20="●")+(N20="●")+(O20="●")&gt;0,B20*D20,0),ROUNDUP((F20="●")+(G20="●")+(H20="●")+(I20="●")+(M20="●")+(N20="●")+(O20="●")/VALUE(MID(R18,2,2)),0)*B20*D20))</f>
         <v/>
       </c>
       <c r="M20" s="89" t="n"/>
@@ -4115,16 +4121,17 @@
       <c r="I24" s="48" t="n"/>
       <c r="J24" s="48" t="n"/>
       <c r="K24" s="46" t="n"/>
-      <c r="L24" s="93" t="inlineStr">
-        <is>
-          <t>PG</t>
-        </is>
-      </c>
+      <c r="L24" s="93" t="n"/>
       <c r="M24" s="96" t="n"/>
       <c r="N24" s="96" t="n"/>
       <c r="O24" s="96" t="n"/>
       <c r="P24" s="96" t="n"/>
       <c r="Q24" s="96" t="n"/>
+      <c r="R24" s="114" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1" s="44">
       <c r="A25" s="102" t="n"/>
@@ -4151,11 +4158,11 @@
         </is>
       </c>
       <c r="K25" s="99">
-        <f>IF(A25="","",IF(L24="PG",IF((F25="●")+(G25="●")+(H25="●")+(I25="●")+(L25="●")+(M25="●")+(N25="●")+(O25="●")&gt;0,B25*C25,0),ROUNDUP((F25="●")+(G25="●")+(H25="●")+(I25="●")+(L25="●")+(M25="●")+(N25="●")+(O25="●")/VALUE(MID(L24,2,2)),0)*B25*C25))</f>
+        <f>IF(A25="","",IF(R24="PG",IF((F25="●")+(G25="●")+(H25="●")+(I25="●")+(M25="●")+(N25="●")+(O25="●")&gt;0,B25*C25,0),ROUNDUP((F25="●")+(G25="●")+(H25="●")+(I25="●")+(M25="●")+(N25="●")+(O25="●")/VALUE(MID(R24,2,2)),0)*B25*C25))</f>
         <v/>
       </c>
       <c r="L25" s="99">
-        <f>IF(A25="","",IF(L24="PG",IF((F25="●")+(G25="●")+(H25="●")+(I25="●")+(L25="●")+(M25="●")+(N25="●")+(O25="●")&gt;0,B25*D25,0),ROUNDUP((F25="●")+(G25="●")+(H25="●")+(I25="●")+(L25="●")+(M25="●")+(N25="●")+(O25="●")/VALUE(MID(L24,2,2)),0)*B25*D25))</f>
+        <f>IF(A25="","",IF(R24="PG",IF((F25="●")+(G25="●")+(H25="●")+(I25="●")+(M25="●")+(N25="●")+(O25="●")&gt;0,B25*D25,0),ROUNDUP((F25="●")+(G25="●")+(H25="●")+(I25="●")+(M25="●")+(N25="●")+(O25="●")/VALUE(MID(R24,2,2)),0)*B25*D25))</f>
         <v/>
       </c>
       <c r="M25" s="89" t="n"/>
@@ -4192,11 +4199,11 @@
         </is>
       </c>
       <c r="K26" s="99">
-        <f>IF(A26="","",IF(L24="PG",IF((F26="●")+(G26="●")+(H26="●")+(I26="●")+(L26="●")+(M26="●")+(N26="●")+(O26="●")&gt;0,B26*C26,0),ROUNDUP((F26="●")+(G26="●")+(H26="●")+(I26="●")+(L26="●")+(M26="●")+(N26="●")+(O26="●")/VALUE(MID(L24,2,2)),0)*B26*C26))</f>
+        <f>IF(A26="","",IF(R24="PG",IF((F26="●")+(G26="●")+(H26="●")+(I26="●")+(M26="●")+(N26="●")+(O26="●")&gt;0,B26*C26,0),ROUNDUP((F26="●")+(G26="●")+(H26="●")+(I26="●")+(M26="●")+(N26="●")+(O26="●")/VALUE(MID(R24,2,2)),0)*B26*C26))</f>
         <v/>
       </c>
       <c r="L26" s="99">
-        <f>IF(A26="","",IF(L24="PG",IF((F26="●")+(G26="●")+(H26="●")+(I26="●")+(L26="●")+(M26="●")+(N26="●")+(O26="●")&gt;0,B26*D26,0),ROUNDUP((F26="●")+(G26="●")+(H26="●")+(I26="●")+(L26="●")+(M26="●")+(N26="●")+(O26="●")/VALUE(MID(L24,2,2)),0)*B26*D26))</f>
+        <f>IF(A26="","",IF(R24="PG",IF((F26="●")+(G26="●")+(H26="●")+(I26="●")+(M26="●")+(N26="●")+(O26="●")&gt;0,B26*D26,0),ROUNDUP((F26="●")+(G26="●")+(H26="●")+(I26="●")+(M26="●")+(N26="●")+(O26="●")/VALUE(MID(R24,2,2)),0)*B26*D26))</f>
         <v/>
       </c>
       <c r="M26" s="89" t="n"/>
@@ -4297,16 +4304,17 @@
       <c r="I30" s="48" t="n"/>
       <c r="J30" s="48" t="n"/>
       <c r="K30" s="46" t="n"/>
-      <c r="L30" s="93" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
+      <c r="L30" s="93" t="n"/>
       <c r="M30" s="96" t="n"/>
       <c r="N30" s="96" t="n"/>
       <c r="O30" s="96" t="n"/>
       <c r="P30" s="96" t="n"/>
       <c r="Q30" s="96" t="n"/>
+      <c r="R30" s="114" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1" s="44">
       <c r="A31" s="84" t="inlineStr">
@@ -4339,11 +4347,11 @@
         </is>
       </c>
       <c r="K31" s="99">
-        <f>IF(A31="","",IF(L30="PG",IF((F31="●")+(G31="●")+(H31="●")+(I31="●")+(L31="●")+(M31="●")+(N31="●")+(O31="●")&gt;0,B31*C31,0),ROUNDUP((F31="●")+(G31="●")+(H31="●")+(I31="●")+(L31="●")+(M31="●")+(N31="●")+(O31="●")/VALUE(MID(L30,2,2)),0)*B31*C31))</f>
+        <f>IF(A31="","",IF(R30="PG",IF((F31="●")+(G31="●")+(H31="●")+(I31="●")+(M31="●")+(N31="●")+(O31="●")&gt;0,B31*C31,0),ROUNDUP((F31="●")+(G31="●")+(H31="●")+(I31="●")+(M31="●")+(N31="●")+(O31="●")/VALUE(MID(R30,2,2)),0)*B31*C31))</f>
         <v/>
       </c>
       <c r="L31" s="99">
-        <f>IF(A31="","",IF(L30="PG",IF((F31="●")+(G31="●")+(H31="●")+(I31="●")+(L31="●")+(M31="●")+(N31="●")+(O31="●")&gt;0,B31*D31,0),ROUNDUP((F31="●")+(G31="●")+(H31="●")+(I31="●")+(L31="●")+(M31="●")+(N31="●")+(O31="●")/VALUE(MID(L30,2,2)),0)*B31*D31))</f>
+        <f>IF(A31="","",IF(R30="PG",IF((F31="●")+(G31="●")+(H31="●")+(I31="●")+(M31="●")+(N31="●")+(O31="●")&gt;0,B31*D31,0),ROUNDUP((F31="●")+(G31="●")+(H31="●")+(I31="●")+(M31="●")+(N31="●")+(O31="●")/VALUE(MID(R30,2,2)),0)*B31*D31))</f>
         <v/>
       </c>
       <c r="M31" s="89" t="n"/>
@@ -4386,11 +4394,11 @@
         </is>
       </c>
       <c r="K32" s="99">
-        <f>IF(A32="","",IF(L30="PG",IF((F32="●")+(G32="●")+(H32="●")+(I32="●")+(L32="●")+(M32="●")+(N32="●")+(O32="●")&gt;0,B32*C32,0),ROUNDUP((F32="●")+(G32="●")+(H32="●")+(I32="●")+(L32="●")+(M32="●")+(N32="●")+(O32="●")/VALUE(MID(L30,2,2)),0)*B32*C32))</f>
+        <f>IF(A32="","",IF(R30="PG",IF((F32="●")+(G32="●")+(H32="●")+(I32="●")+(M32="●")+(N32="●")+(O32="●")&gt;0,B32*C32,0),ROUNDUP((F32="●")+(G32="●")+(H32="●")+(I32="●")+(M32="●")+(N32="●")+(O32="●")/VALUE(MID(R30,2,2)),0)*B32*C32))</f>
         <v/>
       </c>
       <c r="L32" s="99">
-        <f>IF(A32="","",IF(L30="PG",IF((F32="●")+(G32="●")+(H32="●")+(I32="●")+(L32="●")+(M32="●")+(N32="●")+(O32="●")&gt;0,B32*D32,0),ROUNDUP((F32="●")+(G32="●")+(H32="●")+(I32="●")+(L32="●")+(M32="●")+(N32="●")+(O32="●")/VALUE(MID(L30,2,2)),0)*B32*D32))</f>
+        <f>IF(A32="","",IF(R30="PG",IF((F32="●")+(G32="●")+(H32="●")+(I32="●")+(M32="●")+(N32="●")+(O32="●")&gt;0,B32*D32,0),ROUNDUP((F32="●")+(G32="●")+(H32="●")+(I32="●")+(M32="●")+(N32="●")+(O32="●")/VALUE(MID(R30,2,2)),0)*B32*D32))</f>
         <v/>
       </c>
       <c r="M32" s="89" t="n"/>
@@ -4433,11 +4441,11 @@
         </is>
       </c>
       <c r="K33" s="99">
-        <f>IF(A33="","",IF(L30="PG",IF((F33="●")+(G33="●")+(H33="●")+(I33="●")+(L33="●")+(M33="●")+(N33="●")+(O33="●")&gt;0,B33*C33,0),ROUNDUP((F33="●")+(G33="●")+(H33="●")+(I33="●")+(L33="●")+(M33="●")+(N33="●")+(O33="●")/VALUE(MID(L30,2,2)),0)*B33*C33))</f>
+        <f>IF(A33="","",IF(R30="PG",IF((F33="●")+(G33="●")+(H33="●")+(I33="●")+(M33="●")+(N33="●")+(O33="●")&gt;0,B33*C33,0),ROUNDUP((F33="●")+(G33="●")+(H33="●")+(I33="●")+(M33="●")+(N33="●")+(O33="●")/VALUE(MID(R30,2,2)),0)*B33*C33))</f>
         <v/>
       </c>
       <c r="L33" s="99">
-        <f>IF(A33="","",IF(L30="PG",IF((F33="●")+(G33="●")+(H33="●")+(I33="●")+(L33="●")+(M33="●")+(N33="●")+(O33="●")&gt;0,B33*D33,0),ROUNDUP((F33="●")+(G33="●")+(H33="●")+(I33="●")+(L33="●")+(M33="●")+(N33="●")+(O33="●")/VALUE(MID(L30,2,2)),0)*B33*D33))</f>
+        <f>IF(A33="","",IF(R30="PG",IF((F33="●")+(G33="●")+(H33="●")+(I33="●")+(M33="●")+(N33="●")+(O33="●")&gt;0,B33*D33,0),ROUNDUP((F33="●")+(G33="●")+(H33="●")+(I33="●")+(M33="●")+(N33="●")+(O33="●")/VALUE(MID(R30,2,2)),0)*B33*D33))</f>
         <v/>
       </c>
       <c r="M33" s="89" t="n"/>
@@ -4474,11 +4482,11 @@
         </is>
       </c>
       <c r="K34" s="99">
-        <f>IF(A34="","",IF(L30="PG",IF((F34="●")+(G34="●")+(H34="●")+(I34="●")+(L34="●")+(M34="●")+(N34="●")+(O34="●")&gt;0,B34*C34,0),ROUNDUP((F34="●")+(G34="●")+(H34="●")+(I34="●")+(L34="●")+(M34="●")+(N34="●")+(O34="●")/VALUE(MID(L30,2,2)),0)*B34*C34))</f>
+        <f>IF(A34="","",IF(R30="PG",IF((F34="●")+(G34="●")+(H34="●")+(I34="●")+(M34="●")+(N34="●")+(O34="●")&gt;0,B34*C34,0),ROUNDUP((F34="●")+(G34="●")+(H34="●")+(I34="●")+(M34="●")+(N34="●")+(O34="●")/VALUE(MID(R30,2,2)),0)*B34*C34))</f>
         <v/>
       </c>
       <c r="L34" s="99">
-        <f>IF(A34="","",IF(L30="PG",IF((F34="●")+(G34="●")+(H34="●")+(I34="●")+(L34="●")+(M34="●")+(N34="●")+(O34="●")&gt;0,B34*D34,0),ROUNDUP((F34="●")+(G34="●")+(H34="●")+(I34="●")+(L34="●")+(M34="●")+(N34="●")+(O34="●")/VALUE(MID(L30,2,2)),0)*B34*D34))</f>
+        <f>IF(A34="","",IF(R30="PG",IF((F34="●")+(G34="●")+(H34="●")+(I34="●")+(M34="●")+(N34="●")+(O34="●")&gt;0,B34*D34,0),ROUNDUP((F34="●")+(G34="●")+(H34="●")+(I34="●")+(M34="●")+(N34="●")+(O34="●")/VALUE(MID(R30,2,2)),0)*B34*D34))</f>
         <v/>
       </c>
       <c r="M34" s="89" t="n"/>
@@ -4579,16 +4587,17 @@
       <c r="I38" s="48" t="n"/>
       <c r="J38" s="48" t="n"/>
       <c r="K38" s="46" t="n"/>
-      <c r="L38" s="93" t="inlineStr">
-        <is>
-          <t>PG</t>
-        </is>
-      </c>
+      <c r="L38" s="93" t="n"/>
       <c r="M38" s="96" t="n"/>
       <c r="N38" s="96" t="n"/>
       <c r="O38" s="96" t="n"/>
       <c r="P38" s="96" t="n"/>
       <c r="Q38" s="96" t="n"/>
+      <c r="R38" s="114" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1" s="44">
       <c r="A39" s="102" t="n"/>
@@ -4615,11 +4624,11 @@
         </is>
       </c>
       <c r="K39" s="99">
-        <f>IF(A39="","",IF(L38="PG",IF((F39="●")+(G39="●")+(H39="●")+(I39="●")+(L39="●")+(M39="●")+(N39="●")+(O39="●")&gt;0,B39*C39,0),ROUNDUP((F39="●")+(G39="●")+(H39="●")+(I39="●")+(L39="●")+(M39="●")+(N39="●")+(O39="●")/VALUE(MID(L38,2,2)),0)*B39*C39))</f>
+        <f>IF(A39="","",IF(R38="PG",IF((F39="●")+(G39="●")+(H39="●")+(I39="●")+(M39="●")+(N39="●")+(O39="●")&gt;0,B39*C39,0),ROUNDUP((F39="●")+(G39="●")+(H39="●")+(I39="●")+(M39="●")+(N39="●")+(O39="●")/VALUE(MID(R38,2,2)),0)*B39*C39))</f>
         <v/>
       </c>
       <c r="L39" s="99">
-        <f>IF(A39="","",IF(L38="PG",IF((F39="●")+(G39="●")+(H39="●")+(I39="●")+(L39="●")+(M39="●")+(N39="●")+(O39="●")&gt;0,B39*D39,0),ROUNDUP((F39="●")+(G39="●")+(H39="●")+(I39="●")+(L39="●")+(M39="●")+(N39="●")+(O39="●")/VALUE(MID(L38,2,2)),0)*B39*D39))</f>
+        <f>IF(A39="","",IF(R38="PG",IF((F39="●")+(G39="●")+(H39="●")+(I39="●")+(M39="●")+(N39="●")+(O39="●")&gt;0,B39*D39,0),ROUNDUP((F39="●")+(G39="●")+(H39="●")+(I39="●")+(M39="●")+(N39="●")+(O39="●")/VALUE(MID(R38,2,2)),0)*B39*D39))</f>
         <v/>
       </c>
       <c r="M39" s="89" t="n"/>
@@ -4656,11 +4665,11 @@
         </is>
       </c>
       <c r="K40" s="99">
-        <f>IF(A40="","",IF(L38="PG",IF((F40="●")+(G40="●")+(H40="●")+(I40="●")+(L40="●")+(M40="●")+(N40="●")+(O40="●")&gt;0,B40*C40,0),ROUNDUP((F40="●")+(G40="●")+(H40="●")+(I40="●")+(L40="●")+(M40="●")+(N40="●")+(O40="●")/VALUE(MID(L38,2,2)),0)*B40*C40))</f>
+        <f>IF(A40="","",IF(R38="PG",IF((F40="●")+(G40="●")+(H40="●")+(I40="●")+(M40="●")+(N40="●")+(O40="●")&gt;0,B40*C40,0),ROUNDUP((F40="●")+(G40="●")+(H40="●")+(I40="●")+(M40="●")+(N40="●")+(O40="●")/VALUE(MID(R38,2,2)),0)*B40*C40))</f>
         <v/>
       </c>
       <c r="L40" s="99">
-        <f>IF(A40="","",IF(L38="PG",IF((F40="●")+(G40="●")+(H40="●")+(I40="●")+(L40="●")+(M40="●")+(N40="●")+(O40="●")&gt;0,B40*D40,0),ROUNDUP((F40="●")+(G40="●")+(H40="●")+(I40="●")+(L40="●")+(M40="●")+(N40="●")+(O40="●")/VALUE(MID(L38,2,2)),0)*B40*D40))</f>
+        <f>IF(A40="","",IF(R38="PG",IF((F40="●")+(G40="●")+(H40="●")+(I40="●")+(M40="●")+(N40="●")+(O40="●")&gt;0,B40*D40,0),ROUNDUP((F40="●")+(G40="●")+(H40="●")+(I40="●")+(M40="●")+(N40="●")+(O40="●")/VALUE(MID(R38,2,2)),0)*B40*D40))</f>
         <v/>
       </c>
       <c r="M40" s="89" t="n"/>
@@ -4761,16 +4770,17 @@
       <c r="I44" s="48" t="n"/>
       <c r="J44" s="48" t="n"/>
       <c r="K44" s="46" t="n"/>
-      <c r="L44" s="93" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
+      <c r="L44" s="93" t="n"/>
       <c r="M44" s="96" t="n"/>
       <c r="N44" s="96" t="n"/>
       <c r="O44" s="96" t="n"/>
       <c r="P44" s="96" t="n"/>
       <c r="Q44" s="96" t="n"/>
+      <c r="R44" s="114" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1" s="44">
       <c r="A45" s="84" t="inlineStr">
@@ -4803,11 +4813,11 @@
         </is>
       </c>
       <c r="K45" s="99">
-        <f>IF(A45="","",IF(L44="PG",IF((F45="●")+(G45="●")+(H45="●")+(I45="●")+(L45="●")+(M45="●")+(N45="●")+(O45="●")&gt;0,B45*C45,0),ROUNDUP((F45="●")+(G45="●")+(H45="●")+(I45="●")+(L45="●")+(M45="●")+(N45="●")+(O45="●")/VALUE(MID(L44,2,2)),0)*B45*C45))</f>
+        <f>IF(A45="","",IF(R44="PG",IF((F45="●")+(G45="●")+(H45="●")+(I45="●")+(M45="●")+(N45="●")+(O45="●")&gt;0,B45*C45,0),ROUNDUP((F45="●")+(G45="●")+(H45="●")+(I45="●")+(M45="●")+(N45="●")+(O45="●")/VALUE(MID(R44,2,2)),0)*B45*C45))</f>
         <v/>
       </c>
       <c r="L45" s="99">
-        <f>IF(A45="","",IF(L44="PG",IF((F45="●")+(G45="●")+(H45="●")+(I45="●")+(L45="●")+(M45="●")+(N45="●")+(O45="●")&gt;0,B45*D45,0),ROUNDUP((F45="●")+(G45="●")+(H45="●")+(I45="●")+(L45="●")+(M45="●")+(N45="●")+(O45="●")/VALUE(MID(L44,2,2)),0)*B45*D45))</f>
+        <f>IF(A45="","",IF(R44="PG",IF((F45="●")+(G45="●")+(H45="●")+(I45="●")+(M45="●")+(N45="●")+(O45="●")&gt;0,B45*D45,0),ROUNDUP((F45="●")+(G45="●")+(H45="●")+(I45="●")+(M45="●")+(N45="●")+(O45="●")/VALUE(MID(R44,2,2)),0)*B45*D45))</f>
         <v/>
       </c>
       <c r="M45" s="89" t="n"/>
@@ -4850,11 +4860,11 @@
         </is>
       </c>
       <c r="K46" s="99">
-        <f>IF(A46="","",IF(L44="PG",IF((F46="●")+(G46="●")+(H46="●")+(I46="●")+(L46="●")+(M46="●")+(N46="●")+(O46="●")&gt;0,B46*C46,0),ROUNDUP((F46="●")+(G46="●")+(H46="●")+(I46="●")+(L46="●")+(M46="●")+(N46="●")+(O46="●")/VALUE(MID(L44,2,2)),0)*B46*C46))</f>
+        <f>IF(A46="","",IF(R44="PG",IF((F46="●")+(G46="●")+(H46="●")+(I46="●")+(M46="●")+(N46="●")+(O46="●")&gt;0,B46*C46,0),ROUNDUP((F46="●")+(G46="●")+(H46="●")+(I46="●")+(M46="●")+(N46="●")+(O46="●")/VALUE(MID(R44,2,2)),0)*B46*C46))</f>
         <v/>
       </c>
       <c r="L46" s="99">
-        <f>IF(A46="","",IF(L44="PG",IF((F46="●")+(G46="●")+(H46="●")+(I46="●")+(L46="●")+(M46="●")+(N46="●")+(O46="●")&gt;0,B46*D46,0),ROUNDUP((F46="●")+(G46="●")+(H46="●")+(I46="●")+(L46="●")+(M46="●")+(N46="●")+(O46="●")/VALUE(MID(L44,2,2)),0)*B46*D46))</f>
+        <f>IF(A46="","",IF(R44="PG",IF((F46="●")+(G46="●")+(H46="●")+(I46="●")+(M46="●")+(N46="●")+(O46="●")&gt;0,B46*D46,0),ROUNDUP((F46="●")+(G46="●")+(H46="●")+(I46="●")+(M46="●")+(N46="●")+(O46="●")/VALUE(MID(R44,2,2)),0)*B46*D46))</f>
         <v/>
       </c>
       <c r="M46" s="89" t="n"/>
@@ -4897,11 +4907,11 @@
         </is>
       </c>
       <c r="K47" s="99">
-        <f>IF(A47="","",IF(L44="PG",IF((F47="●")+(G47="●")+(H47="●")+(I47="●")+(L47="●")+(M47="●")+(N47="●")+(O47="●")&gt;0,B47*C47,0),ROUNDUP((F47="●")+(G47="●")+(H47="●")+(I47="●")+(L47="●")+(M47="●")+(N47="●")+(O47="●")/VALUE(MID(L44,2,2)),0)*B47*C47))</f>
+        <f>IF(A47="","",IF(R44="PG",IF((F47="●")+(G47="●")+(H47="●")+(I47="●")+(M47="●")+(N47="●")+(O47="●")&gt;0,B47*C47,0),ROUNDUP((F47="●")+(G47="●")+(H47="●")+(I47="●")+(M47="●")+(N47="●")+(O47="●")/VALUE(MID(R44,2,2)),0)*B47*C47))</f>
         <v/>
       </c>
       <c r="L47" s="99">
-        <f>IF(A47="","",IF(L44="PG",IF((F47="●")+(G47="●")+(H47="●")+(I47="●")+(L47="●")+(M47="●")+(N47="●")+(O47="●")&gt;0,B47*D47,0),ROUNDUP((F47="●")+(G47="●")+(H47="●")+(I47="●")+(L47="●")+(M47="●")+(N47="●")+(O47="●")/VALUE(MID(L44,2,2)),0)*B47*D47))</f>
+        <f>IF(A47="","",IF(R44="PG",IF((F47="●")+(G47="●")+(H47="●")+(I47="●")+(M47="●")+(N47="●")+(O47="●")&gt;0,B47*D47,0),ROUNDUP((F47="●")+(G47="●")+(H47="●")+(I47="●")+(M47="●")+(N47="●")+(O47="●")/VALUE(MID(R44,2,2)),0)*B47*D47))</f>
         <v/>
       </c>
       <c r="M47" s="89" t="n"/>
@@ -4938,11 +4948,11 @@
         </is>
       </c>
       <c r="K48" s="99">
-        <f>IF(A48="","",IF(L44="PG",IF((F48="●")+(G48="●")+(H48="●")+(I48="●")+(L48="●")+(M48="●")+(N48="●")+(O48="●")&gt;0,B48*C48,0),ROUNDUP((F48="●")+(G48="●")+(H48="●")+(I48="●")+(L48="●")+(M48="●")+(N48="●")+(O48="●")/VALUE(MID(L44,2,2)),0)*B48*C48))</f>
+        <f>IF(A48="","",IF(R44="PG",IF((F48="●")+(G48="●")+(H48="●")+(I48="●")+(M48="●")+(N48="●")+(O48="●")&gt;0,B48*C48,0),ROUNDUP((F48="●")+(G48="●")+(H48="●")+(I48="●")+(M48="●")+(N48="●")+(O48="●")/VALUE(MID(R44,2,2)),0)*B48*C48))</f>
         <v/>
       </c>
       <c r="L48" s="99">
-        <f>IF(A48="","",IF(L44="PG",IF((F48="●")+(G48="●")+(H48="●")+(I48="●")+(L48="●")+(M48="●")+(N48="●")+(O48="●")&gt;0,B48*D48,0),ROUNDUP((F48="●")+(G48="●")+(H48="●")+(I48="●")+(L48="●")+(M48="●")+(N48="●")+(O48="●")/VALUE(MID(L44,2,2)),0)*B48*D48))</f>
+        <f>IF(A48="","",IF(R44="PG",IF((F48="●")+(G48="●")+(H48="●")+(I48="●")+(M48="●")+(N48="●")+(O48="●")&gt;0,B48*D48,0),ROUNDUP((F48="●")+(G48="●")+(H48="●")+(I48="●")+(M48="●")+(N48="●")+(O48="●")/VALUE(MID(R44,2,2)),0)*B48*D48))</f>
         <v/>
       </c>
       <c r="M48" s="89" t="n"/>
@@ -4979,11 +4989,11 @@
         </is>
       </c>
       <c r="K49" s="99">
-        <f>IF(A49="","",IF(L44="PG",IF((F49="●")+(G49="●")+(H49="●")+(I49="●")+(L49="●")+(M49="●")+(N49="●")+(O49="●")&gt;0,B49*C49,0),ROUNDUP((F49="●")+(G49="●")+(H49="●")+(I49="●")+(L49="●")+(M49="●")+(N49="●")+(O49="●")/VALUE(MID(L44,2,2)),0)*B49*C49))</f>
+        <f>IF(A49="","",IF(R44="PG",IF((F49="●")+(G49="●")+(H49="●")+(I49="●")+(M49="●")+(N49="●")+(O49="●")&gt;0,B49*C49,0),ROUNDUP((F49="●")+(G49="●")+(H49="●")+(I49="●")+(M49="●")+(N49="●")+(O49="●")/VALUE(MID(R44,2,2)),0)*B49*C49))</f>
         <v/>
       </c>
       <c r="L49" s="99">
-        <f>IF(A49="","",IF(L44="PG",IF((F49="●")+(G49="●")+(H49="●")+(I49="●")+(L49="●")+(M49="●")+(N49="●")+(O49="●")&gt;0,B49*D49,0),ROUNDUP((F49="●")+(G49="●")+(H49="●")+(I49="●")+(L49="●")+(M49="●")+(N49="●")+(O49="●")/VALUE(MID(L44,2,2)),0)*B49*D49))</f>
+        <f>IF(A49="","",IF(R44="PG",IF((F49="●")+(G49="●")+(H49="●")+(I49="●")+(M49="●")+(N49="●")+(O49="●")&gt;0,B49*D49,0),ROUNDUP((F49="●")+(G49="●")+(H49="●")+(I49="●")+(M49="●")+(N49="●")+(O49="●")/VALUE(MID(R44,2,2)),0)*B49*D49))</f>
         <v/>
       </c>
       <c r="M49" s="89" t="n"/>
@@ -5020,11 +5030,11 @@
         </is>
       </c>
       <c r="K50" s="99">
-        <f>IF(A50="","",IF(L44="PG",IF((F50="●")+(G50="●")+(H50="●")+(I50="●")+(L50="●")+(M50="●")+(N50="●")+(O50="●")&gt;0,B50*C50,0),ROUNDUP((F50="●")+(G50="●")+(H50="●")+(I50="●")+(L50="●")+(M50="●")+(N50="●")+(O50="●")/VALUE(MID(L44,2,2)),0)*B50*C50))</f>
+        <f>IF(A50="","",IF(R44="PG",IF((F50="●")+(G50="●")+(H50="●")+(I50="●")+(M50="●")+(N50="●")+(O50="●")&gt;0,B50*C50,0),ROUNDUP((F50="●")+(G50="●")+(H50="●")+(I50="●")+(M50="●")+(N50="●")+(O50="●")/VALUE(MID(R44,2,2)),0)*B50*C50))</f>
         <v/>
       </c>
       <c r="L50" s="99">
-        <f>IF(A50="","",IF(L44="PG",IF((F50="●")+(G50="●")+(H50="●")+(I50="●")+(L50="●")+(M50="●")+(N50="●")+(O50="●")&gt;0,B50*D50,0),ROUNDUP((F50="●")+(G50="●")+(H50="●")+(I50="●")+(L50="●")+(M50="●")+(N50="●")+(O50="●")/VALUE(MID(L44,2,2)),0)*B50*D50))</f>
+        <f>IF(A50="","",IF(R44="PG",IF((F50="●")+(G50="●")+(H50="●")+(I50="●")+(M50="●")+(N50="●")+(O50="●")&gt;0,B50*D50,0),ROUNDUP((F50="●")+(G50="●")+(H50="●")+(I50="●")+(M50="●")+(N50="●")+(O50="●")/VALUE(MID(R44,2,2)),0)*B50*D50))</f>
         <v/>
       </c>
       <c r="M50" s="89" t="n"/>
@@ -5061,11 +5071,11 @@
         </is>
       </c>
       <c r="K51" s="99">
-        <f>IF(A51="","",IF(L44="PG",IF((F51="●")+(G51="●")+(H51="●")+(I51="●")+(L51="●")+(M51="●")+(N51="●")+(O51="●")&gt;0,B51*C51,0),ROUNDUP((F51="●")+(G51="●")+(H51="●")+(I51="●")+(L51="●")+(M51="●")+(N51="●")+(O51="●")/VALUE(MID(L44,2,2)),0)*B51*C51))</f>
+        <f>IF(A51="","",IF(R44="PG",IF((F51="●")+(G51="●")+(H51="●")+(I51="●")+(M51="●")+(N51="●")+(O51="●")&gt;0,B51*C51,0),ROUNDUP((F51="●")+(G51="●")+(H51="●")+(I51="●")+(M51="●")+(N51="●")+(O51="●")/VALUE(MID(R44,2,2)),0)*B51*C51))</f>
         <v/>
       </c>
       <c r="L51" s="99">
-        <f>IF(A51="","",IF(L44="PG",IF((F51="●")+(G51="●")+(H51="●")+(I51="●")+(L51="●")+(M51="●")+(N51="●")+(O51="●")&gt;0,B51*D51,0),ROUNDUP((F51="●")+(G51="●")+(H51="●")+(I51="●")+(L51="●")+(M51="●")+(N51="●")+(O51="●")/VALUE(MID(L44,2,2)),0)*B51*D51))</f>
+        <f>IF(A51="","",IF(R44="PG",IF((F51="●")+(G51="●")+(H51="●")+(I51="●")+(M51="●")+(N51="●")+(O51="●")&gt;0,B51*D51,0),ROUNDUP((F51="●")+(G51="●")+(H51="●")+(I51="●")+(M51="●")+(N51="●")+(O51="●")/VALUE(MID(R44,2,2)),0)*B51*D51))</f>
         <v/>
       </c>
       <c r="M51" s="89" t="n"/>
@@ -5102,11 +5112,11 @@
         </is>
       </c>
       <c r="K52" s="99">
-        <f>IF(A52="","",IF(L44="PG",IF((F52="●")+(G52="●")+(H52="●")+(I52="●")+(L52="●")+(M52="●")+(N52="●")+(O52="●")&gt;0,B52*C52,0),ROUNDUP((F52="●")+(G52="●")+(H52="●")+(I52="●")+(L52="●")+(M52="●")+(N52="●")+(O52="●")/VALUE(MID(L44,2,2)),0)*B52*C52))</f>
+        <f>IF(A52="","",IF(R44="PG",IF((F52="●")+(G52="●")+(H52="●")+(I52="●")+(M52="●")+(N52="●")+(O52="●")&gt;0,B52*C52,0),ROUNDUP((F52="●")+(G52="●")+(H52="●")+(I52="●")+(M52="●")+(N52="●")+(O52="●")/VALUE(MID(R44,2,2)),0)*B52*C52))</f>
         <v/>
       </c>
       <c r="L52" s="99">
-        <f>IF(A52="","",IF(L44="PG",IF((F52="●")+(G52="●")+(H52="●")+(I52="●")+(L52="●")+(M52="●")+(N52="●")+(O52="●")&gt;0,B52*D52,0),ROUNDUP((F52="●")+(G52="●")+(H52="●")+(I52="●")+(L52="●")+(M52="●")+(N52="●")+(O52="●")/VALUE(MID(L44,2,2)),0)*B52*D52))</f>
+        <f>IF(A52="","",IF(R44="PG",IF((F52="●")+(G52="●")+(H52="●")+(I52="●")+(M52="●")+(N52="●")+(O52="●")&gt;0,B52*D52,0),ROUNDUP((F52="●")+(G52="●")+(H52="●")+(I52="●")+(M52="●")+(N52="●")+(O52="●")/VALUE(MID(R44,2,2)),0)*B52*D52))</f>
         <v/>
       </c>
       <c r="M52" s="89" t="n"/>
@@ -5190,6 +5200,7 @@
       <c r="P54" s="91" t="n"/>
       <c r="Q54" s="91" t="n"/>
     </row>
+    <row r="55"/>
     <row r="56"/>
     <row r="57">
       <c r="A57" s="97" t="inlineStr">
@@ -5597,17 +5608,17 @@
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="A57:L57"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A7:L7"/>
     <mergeCell ref="A18:K18"/>
-    <mergeCell ref="A7:L7"/>
-    <mergeCell ref="B2:C2"/>
     <mergeCell ref="A30:K30"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A24:K24"/>
     <mergeCell ref="A38:K38"/>
     <mergeCell ref="A66:L66"/>
     <mergeCell ref="A11:K11"/>
+    <mergeCell ref="B9:C9"/>
     <mergeCell ref="A3:L3"/>
-    <mergeCell ref="B9:C9"/>
     <mergeCell ref="A44:K44"/>
     <mergeCell ref="A4:L4"/>
   </mergeCells>
@@ -5946,7 +5957,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="12">
+  <dataValidations count="13">
     <dataValidation sqref="E2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"2,4,6,8"</formula1>
     </dataValidation>
@@ -5983,6 +5994,9 @@
     <dataValidation sqref="F12 F13 F14 F15 F19 F20 F25 F26 F31 F32 F33 F34 F39 F40 F45 F46 F47 F48 F49 F50 F51 F52 G12 G13 G14 G15 G19 G20 G25 G26 G31 G32 G33 G34 G39 G40 G45 G46 G47 G48 G49 G50 G51 G52 H12 H13 H14 H15 H19 H20 H25 H26 H31 H32 H33 H34 H39 H40 H45 H46 H47 H48 H49 H50 H51 H52 I12 I13 I14 I15 I19 I20 I25 I26 I31 I32 I33 I34 I39 I40 I45 I46 I47 I48 I49 I50 I51 I52 L12 L13 L14 L15 L19 L20 L25 L26 L31 L32 L33 L34 L39 L40 L45 L46 L47 L48 L49 L50 L51 L52 M12 M13 M14 M15 M19 M20 M25 M26 M31 M32 M33 M34 M39 M40 M45 M46 M47 M48 M49 M50 M51 M52 N12 N13 N14 N15 N19 N20 N25 N26 N31 N32 N33 N34 N39 N40 N45 N46 N47 N48 N49 N50 N51 N52 O12 O13 O14 O15 O19 O20 O25 O26 O31 O32 O33 O34 O39 O40 O45 O46 O47 O48 O49 O50 O51 O52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Toggle" error="● = ON, blank = OFF" type="list">
       <formula1>"●"</formula1>
     </dataValidation>
+    <dataValidation sqref="R11 R18 R24 R30 R38 R44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Charge Type" error="Valid: PG, P1-P20" type="list">
+      <formula1>"PG,P1,P2,P3,P4,P5,P6,P7,P8,P9,P10,P11,P12,P13,P14,P15,P16,P17,P18,P19,P20"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6021,7 +6035,6 @@
         <v/>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="96" t="inlineStr">
         <is>

</xml_diff>